<commit_message>
Atualização automática: emergencias (06/07/2026 11:20)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA18"/>
+  <dimension ref="A1:AA17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -631,10 +631,10 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="n">
-        <v>-9</v>
+        <v>-6</v>
       </c>
       <c r="R2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -726,10 +726,10 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="R3" t="n">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -819,14 +819,14 @@
         <v>46184</v>
       </c>
       <c r="O4" s="2" t="n">
-        <v>46148</v>
+        <v>46178</v>
       </c>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="R4" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -930,10 +930,10 @@
       </c>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="R5" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -1031,10 +1031,10 @@
       </c>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="R6" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1132,10 +1132,10 @@
       </c>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="R7" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1233,10 +1233,10 @@
       </c>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="n">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="R8" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1332,10 +1332,10 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="R9" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -1429,10 +1429,10 @@
       </c>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="n">
-        <v>-10</v>
+        <v>-7</v>
       </c>
       <c r="R10" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
@@ -1447,7 +1447,7 @@
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr">
         <is>
-          <t>DPE de 01 ea para 25/06/2026 (REZ- 15/06/2026).Nova DPE 02/07/2026</t>
+          <t>ENVIADO PARA O OPERADDOR DIA 02/0726, AWB 127-4481 4663- (REZ-02/07/26)</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
@@ -1526,10 +1526,10 @@
       </c>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="n">
-        <v>-10</v>
+        <v>-7</v>
       </c>
       <c r="R11" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="R12" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -1656,26 +1656,26 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>419</v>
+        <v>313</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CLA</t>
+          <t>BAMN</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>419260000555</t>
+          <t>313260018646</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>3244897-4</t>
+          <t>011-00883-20</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>FUEL CONTROL UNIT</t>
+          <t>RADAR GWX 68 WEATHER</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1684,7 +1684,7 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>2723</v>
+        <v>2734</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1697,10 +1697,10 @@
         </is>
       </c>
       <c r="J13" s="2" t="n">
-        <v>46195</v>
+        <v>46199</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>46196</v>
+        <v>46203</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1711,17 +1711,15 @@
         </is>
       </c>
       <c r="N13" s="2" t="n">
-        <v>46207</v>
-      </c>
-      <c r="O13" s="2" t="n">
-        <v>46207</v>
-      </c>
+        <v>46214</v>
+      </c>
+      <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="n">
-        <v>-1</v>
+        <v>-5</v>
       </c>
       <c r="R13" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
@@ -1730,13 +1728,17 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr"/>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Retirado para atender a Anv 2740 - Godoy 30/06/26.</t>
+        </is>
+      </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>MATERIAL EM BANCADA COM DPE INICIAL NA V1 DIA 01/07/26 - SOLICITAÇÃO EPM A26619 - PO 726/JPA/2026 de 30/6/2026 ATZ Marcio 30/6 - MATERIAL EM TRANSITO - RECIBO 532/FAB/26 AWB 12744595530 DPE 04/07/2026</t>
+          <t>Efetuada a Compra em SP na Jet Avionics, aguardando confirmar unidade em estoque para liberação do item para a Veeone 01/7/2026 14:15 Marcio - DECLINADO pela JET AVIONICS, colocado Pedido TEXTRON Confirmation Number: WB0003077522 de 01/7/2026 Invoice IJ17546081 as 15:08PM Previsao DPE AGS Miami 02/7/2026 - ATZ Marcio 1/7/26 15:09</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
@@ -1762,26 +1764,26 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>313260018646</t>
+          <t>313260018651</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>011-00883-20</t>
+          <t>AS5174D1210</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>RADAR GWX 68 WEATHER</t>
+          <t>REDUCER, TUBE</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>2734</v>
+        <v>2732</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -1794,10 +1796,10 @@
         </is>
       </c>
       <c r="J14" s="2" t="n">
-        <v>46199</v>
+        <v>46204</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>46203</v>
+        <v>46205</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
@@ -1808,34 +1810,30 @@
         </is>
       </c>
       <c r="N14" s="2" t="n">
-        <v>46214</v>
+        <v>46216</v>
       </c>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="n">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="R14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="T14" t="inlineStr">
-        <is>
           <t>Sim</t>
         </is>
       </c>
+      <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr">
         <is>
-          <t>Retirado para atender a Anv 2740 - Godoy 30/06/26.</t>
+          <t>Cedeu o item para o C-98 2738</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>Efetuada a Compra em SP na Jet Avionics, aguardando confirmar unidade em estoque para liberação do item para a Veeone 01/7/2026 14:15 Marcio - DECLINADO pela JET AVIONICS, colocado Pedido TEXTRON Confirmation Number: WB0003077522 de 01/7/2026 Invoice IJ17546081 as 15:08PM Previsao DPE AGS Miami 02/7/2026 - ATZ Marcio 1/7/26 15:09</t>
+          <t>PEDIDO NO EPM - FOI SOLICITADO ATENDIMENTO COM ESTOUE FAB - CLA-02-07</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
@@ -1861,17 +1859,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>313260018651</t>
+          <t>313260018652</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>AS5174D1210</t>
+          <t>24540-100</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>REDUCER, TUBE</t>
+          <t>COUPLING,CLAMP,GROOV</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1884,7 +1882,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Aguardando solução</t>
+          <t>Providência tomada</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1912,14 +1910,14 @@
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="n">
-        <v>-10</v>
+        <v>-7</v>
       </c>
       <c r="R15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="T15" t="inlineStr"/>
@@ -1928,7 +1926,11 @@
           <t>Cedeu o item para o C-98 2738</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr"/>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>Colocado pedido fornecedor nacional. Previsão de entrega V1 Campinas 03/07</t>
+        </is>
+      </c>
       <c r="W15" t="inlineStr">
         <is>
           <t>VEE ONE</t>
@@ -1952,17 +1954,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>313260018652</t>
+          <t>313260018653</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>24540-100</t>
+          <t>MS24392-10</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>COUPLING,CLAMP,GROOV</t>
+          <t>NIPPLE,TUBE</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1975,7 +1977,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Aguardando solução</t>
+          <t>Providência tomada</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -2003,14 +2005,14 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="n">
-        <v>-10</v>
+        <v>-7</v>
       </c>
       <c r="R16" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="T16" t="inlineStr"/>
@@ -2019,7 +2021,11 @@
           <t>Cedeu o item para o C-98 2738</t>
         </is>
       </c>
-      <c r="V16" t="inlineStr"/>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>PEDIDO NO EPM - FOI SOLICITADO ATENDIMENTO COM ESTOUE FAB - CLA-02-07</t>
+        </is>
+      </c>
       <c r="W16" t="inlineStr">
         <is>
           <t>VEE ONE</t>
@@ -2034,51 +2040,51 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>BAMN</t>
+          <t>BABR</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>313260018653</t>
+          <t>329260019179</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>MS24392-10</t>
+          <t>066-3046-07</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>NIPPLE,TUBE</t>
+          <t>CONTROL,INDICATOR</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>R</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>2732</v>
+        <v>2721</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Aguardando solução</t>
+          <t>Providência tomada</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>IPLR</t>
+          <t>AIFP</t>
         </is>
       </c>
       <c r="J17" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
       <c r="L17" t="n">
         <v>1</v>
@@ -2089,27 +2095,23 @@
         </is>
       </c>
       <c r="N17" s="2" t="n">
-        <v>46216</v>
+        <v>46213</v>
       </c>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="n">
-        <v>-10</v>
+        <v>-4</v>
       </c>
       <c r="R17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>Cedeu o item para o C-98 2738</t>
-        </is>
-      </c>
+      <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr">
         <is>
@@ -2120,93 +2122,6 @@
       <c r="Y17" t="inlineStr"/>
       <c r="Z17" t="inlineStr"/>
       <c r="AA17" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>329</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>BABR</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>329260019179</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>066-3046-07</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>CONTROL,INDICATOR</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="G18" t="n">
-        <v>2721</v>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Aguardando solução</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>AIFP</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="n">
-        <v>46205</v>
-      </c>
-      <c r="K18" s="2" t="n">
-        <v>46206</v>
-      </c>
-      <c r="L18" t="n">
-        <v>1</v>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>EA</t>
-        </is>
-      </c>
-      <c r="N18" s="2" t="n">
-        <v>46213</v>
-      </c>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="n">
-        <v>-7</v>
-      </c>
-      <c r="R18" t="n">
-        <v>0</v>
-      </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr"/>
-      <c r="W18" t="inlineStr">
-        <is>
-          <t>VEE ONE</t>
-        </is>
-      </c>
-      <c r="X18" t="inlineStr"/>
-      <c r="Y18" t="inlineStr"/>
-      <c r="Z18" t="inlineStr"/>
-      <c r="AA18" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (06/07/2026 15:33)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,137 +421,137 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>om_emg</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>om</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>numero_emergencia</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>categoria</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>matricula_aeronave</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>tpemg</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>data_abertura</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>data_info</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>quantidade</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>unidade_medida</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>prazo_entrega</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>dpe</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>atendido_cancelado</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>dias_atraso</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>dias_corridos</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>estoque</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>retirado_empresa_recibo_obrigatorio</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>obs_coordenadoria_fiscal</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>obs_vee_one</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>provedor</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>awb</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>prev_entrega</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>mensagem_operador</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>em_aberto</t>
         </is>
@@ -611,10 +599,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J2" s="2" t="n">
+      <c r="J2" s="1" t="n">
         <v>46057</v>
       </c>
-      <c r="K2" s="2" t="n">
+      <c r="K2" s="1" t="n">
         <v>46204</v>
       </c>
       <c r="L2" t="n">
@@ -625,7 +613,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N2" s="2" t="n">
+      <c r="N2" s="1" t="n">
         <v>46215</v>
       </c>
       <c r="O2" t="inlineStr"/>
@@ -706,10 +694,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J3" s="2" t="n">
+      <c r="J3" s="1" t="n">
         <v>46076</v>
       </c>
-      <c r="K3" s="2" t="n">
+      <c r="K3" s="1" t="n">
         <v>46080</v>
       </c>
       <c r="L3" t="n">
@@ -720,7 +708,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N3" s="2" t="n">
+      <c r="N3" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="O3" t="inlineStr"/>
@@ -801,10 +789,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J4" s="2" t="n">
+      <c r="J4" s="1" t="n">
         <v>46150</v>
       </c>
-      <c r="K4" s="2" t="n">
+      <c r="K4" s="1" t="n">
         <v>46153</v>
       </c>
       <c r="L4" t="n">
@@ -815,10 +803,10 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N4" s="2" t="n">
+      <c r="N4" s="1" t="n">
         <v>46184</v>
       </c>
-      <c r="O4" s="2" t="n">
+      <c r="O4" s="1" t="n">
         <v>46178</v>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -908,10 +896,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J5" s="2" t="n">
+      <c r="J5" s="1" t="n">
         <v>46160</v>
       </c>
-      <c r="K5" s="2" t="n">
+      <c r="K5" s="1" t="n">
         <v>46161</v>
       </c>
       <c r="L5" t="n">
@@ -922,10 +910,10 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N5" s="2" t="n">
+      <c r="N5" s="1" t="n">
         <v>46192</v>
       </c>
-      <c r="O5" s="2" t="n">
+      <c r="O5" s="1" t="n">
         <v>-620019</v>
       </c>
       <c r="P5" t="inlineStr"/>
@@ -1009,10 +997,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J6" s="2" t="n">
+      <c r="J6" s="1" t="n">
         <v>46168</v>
       </c>
-      <c r="K6" s="2" t="n">
+      <c r="K6" s="1" t="n">
         <v>46168</v>
       </c>
       <c r="L6" t="n">
@@ -1023,10 +1011,10 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N6" s="2" t="n">
+      <c r="N6" s="1" t="n">
         <v>46199</v>
       </c>
-      <c r="O6" s="2" t="n">
+      <c r="O6" s="1" t="n">
         <v>46203</v>
       </c>
       <c r="P6" t="inlineStr"/>
@@ -1110,10 +1098,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="J7" s="1" t="n">
         <v>46167</v>
       </c>
-      <c r="K7" s="2" t="n">
+      <c r="K7" s="1" t="n">
         <v>46168</v>
       </c>
       <c r="L7" t="n">
@@ -1124,10 +1112,10 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N7" s="2" t="n">
+      <c r="N7" s="1" t="n">
         <v>46199</v>
       </c>
-      <c r="O7" s="2" t="n">
+      <c r="O7" s="1" t="n">
         <v>46203</v>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1211,10 +1199,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J8" s="2" t="n">
+      <c r="J8" s="1" t="n">
         <v>46176</v>
       </c>
-      <c r="K8" s="2" t="n">
+      <c r="K8" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="L8" t="n">
@@ -1225,10 +1213,10 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N8" s="2" t="n">
+      <c r="N8" s="1" t="n">
         <v>46207</v>
       </c>
-      <c r="O8" s="2" t="n">
+      <c r="O8" s="1" t="n">
         <v>46196</v>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1312,10 +1300,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J9" s="2" t="n">
+      <c r="J9" s="1" t="n">
         <v>46184</v>
       </c>
-      <c r="K9" s="2" t="n">
+      <c r="K9" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="L9" t="n">
@@ -1326,7 +1314,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N9" s="2" t="n">
+      <c r="N9" s="1" t="n">
         <v>46196</v>
       </c>
       <c r="O9" t="inlineStr"/>
@@ -1407,10 +1395,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J10" s="2" t="n">
+      <c r="J10" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="K10" s="2" t="n">
+      <c r="K10" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="L10" t="n">
@@ -1421,10 +1409,10 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N10" s="2" t="n">
+      <c r="N10" s="1" t="n">
         <v>46216</v>
       </c>
-      <c r="O10" s="2" t="n">
+      <c r="O10" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1504,10 +1492,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J11" s="2" t="n">
+      <c r="J11" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="K11" s="2" t="n">
+      <c r="K11" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="L11" t="n">
@@ -1518,10 +1506,10 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N11" s="2" t="n">
+      <c r="N11" s="1" t="n">
         <v>46216</v>
       </c>
-      <c r="O11" s="2" t="n">
+      <c r="O11" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="P11" t="inlineStr"/>
@@ -1601,10 +1589,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J12" s="2" t="n">
+      <c r="J12" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="K12" s="2" t="n">
+      <c r="K12" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="L12" t="n">
@@ -1615,7 +1603,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N12" s="2" t="n">
+      <c r="N12" s="1" t="n">
         <v>46192</v>
       </c>
       <c r="O12" t="inlineStr"/>
@@ -1696,10 +1684,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J13" s="2" t="n">
+      <c r="J13" s="1" t="n">
         <v>46199</v>
       </c>
-      <c r="K13" s="2" t="n">
+      <c r="K13" s="1" t="n">
         <v>46203</v>
       </c>
       <c r="L13" t="n">
@@ -1710,7 +1698,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N13" s="2" t="n">
+      <c r="N13" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="O13" t="inlineStr"/>
@@ -1795,10 +1783,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J14" s="2" t="n">
+      <c r="J14" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="K14" s="2" t="n">
+      <c r="K14" s="1" t="n">
         <v>46205</v>
       </c>
       <c r="L14" t="n">
@@ -1809,7 +1797,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N14" s="2" t="n">
+      <c r="N14" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="O14" t="inlineStr"/>
@@ -1890,10 +1878,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J15" s="2" t="n">
+      <c r="J15" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="K15" s="2" t="n">
+      <c r="K15" s="1" t="n">
         <v>46205</v>
       </c>
       <c r="L15" t="n">
@@ -1904,7 +1892,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N15" s="2" t="n">
+      <c r="N15" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="O15" t="inlineStr"/>
@@ -1985,10 +1973,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J16" s="2" t="n">
+      <c r="J16" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="K16" s="2" t="n">
+      <c r="K16" s="1" t="n">
         <v>46205</v>
       </c>
       <c r="L16" t="n">
@@ -1999,7 +1987,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N16" s="2" t="n">
+      <c r="N16" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="O16" t="inlineStr"/>
@@ -2080,10 +2068,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J17" s="2" t="n">
+      <c r="J17" s="1" t="n">
         <v>46205</v>
       </c>
-      <c r="K17" s="2" t="n">
+      <c r="K17" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="L17" t="n">
@@ -2094,7 +2082,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N17" s="2" t="n">
+      <c r="N17" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="O17" t="inlineStr"/>

</xml_diff>

<commit_message>
Emergências: tabela completa da planilha + novidades desde ontem
Adiciona data de abertura, data da última informação e as 2 observações de
texto livre (coordenadoria/fiscal e VEE ONE) na tabela de Emergências
Abertas, junto com o restante das colunas da planilha original.

Também passa a registrar um snapshot diário das emergências em aberto
(historico_emergencias.csv, mesmo padrão do RAC) pra alimentar a nova seção
"Novidades desde a última atualização" — o que entrou e o que saiu da lista
desde o snapshot anterior.
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -417,141 +429,141 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA17"/>
+  <dimension ref="A1:AA14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>om_emg</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>om</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>numero_emergencia</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>categoria</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>matricula_aeronave</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>tpemg</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>data_abertura</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>data_info</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>quantidade</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>unidade_medida</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>prazo_entrega</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>dpe</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>atendido_cancelado</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>dias_atraso</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>dias_corridos</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>estoque</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>retirado_empresa_recibo_obrigatorio</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>obs_coordenadoria_fiscal</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>obs_vee_one</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>provedor</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>awb</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>prev_entrega</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>mensagem_operador</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>em_aberto</t>
         </is>
@@ -599,10 +611,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J2" s="1" t="n">
+      <c r="J2" s="2" t="n">
         <v>46057</v>
       </c>
-      <c r="K2" s="1" t="n">
+      <c r="K2" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="L2" t="n">
@@ -613,7 +625,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N2" s="1" t="n">
+      <c r="N2" s="2" t="n">
         <v>46215</v>
       </c>
       <c r="O2" t="inlineStr"/>
@@ -694,10 +706,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J3" s="1" t="n">
+      <c r="J3" s="2" t="n">
         <v>46076</v>
       </c>
-      <c r="K3" s="1" t="n">
+      <c r="K3" s="2" t="n">
         <v>46080</v>
       </c>
       <c r="L3" t="n">
@@ -708,7 +720,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N3" s="1" t="n">
+      <c r="N3" s="2" t="n">
         <v>46111</v>
       </c>
       <c r="O3" t="inlineStr"/>
@@ -789,10 +801,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J4" s="1" t="n">
+      <c r="J4" s="2" t="n">
         <v>46150</v>
       </c>
-      <c r="K4" s="1" t="n">
+      <c r="K4" s="2" t="n">
         <v>46153</v>
       </c>
       <c r="L4" t="n">
@@ -803,10 +815,10 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N4" s="1" t="n">
+      <c r="N4" s="2" t="n">
         <v>46184</v>
       </c>
-      <c r="O4" s="1" t="n">
+      <c r="O4" s="2" t="n">
         <v>46178</v>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -896,10 +908,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J5" s="1" t="n">
+      <c r="J5" s="2" t="n">
         <v>46160</v>
       </c>
-      <c r="K5" s="1" t="n">
+      <c r="K5" s="2" t="n">
         <v>46161</v>
       </c>
       <c r="L5" t="n">
@@ -910,10 +922,10 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N5" s="1" t="n">
+      <c r="N5" s="2" t="n">
         <v>46192</v>
       </c>
-      <c r="O5" s="1" t="n">
+      <c r="O5" s="2" t="n">
         <v>-620019</v>
       </c>
       <c r="P5" t="inlineStr"/>
@@ -966,26 +978,26 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>313260018281</t>
+          <t>313260018412</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>S3105-8</t>
+          <t>011-01105-01</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>RESISTOR</t>
+          <t>INTEGRATED AVIONICS</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>R</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>2736</v>
+        <v>2734</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -994,54 +1006,48 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>ANCE</t>
-        </is>
-      </c>
-      <c r="J6" s="1" t="n">
-        <v>46168</v>
-      </c>
-      <c r="K6" s="1" t="n">
-        <v>46168</v>
+          <t>IPLR</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>46184</v>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>46185</v>
       </c>
       <c r="L6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
           <t>EA</t>
         </is>
       </c>
-      <c r="N6" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="O6" s="1" t="n">
-        <v>46203</v>
-      </c>
+      <c r="N6" s="2" t="n">
+        <v>46196</v>
+      </c>
+      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="R6" t="n">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
+      <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr">
         <is>
-          <t>AWB 12743528074 -  volume retirado na loja GOLLOG - QMA por kleyton. Godoy 30/06/2026.</t>
+          <t>Retirado para atender a Anv 2737 - Godoy 12/06/26.</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Colocado pedido Textron IJ17463339. Entregue em Miami 29/05. Chegada em VCP 04/06 (voo 3906). Canal amarelo dia 10/06. Carga liberada para entrega em Campinas 25/06 - MATERIAL EM TRANSITO 0 DIA 25/05/2026 VIA AWB 12743528074 RECIBO 507/FAB/26 - DPE 01/07/2026 ATZ RC 14:21 26/06/2026</t>
+          <t>Material Liberado Canal Verde em 01/7/2026 - HAWB: 00125552354 00004021 , Invoice PPSPI01534 PO 696/JPA/2026, aguardando ICMS GIGRJ. ATZ Marcio 01/7/2026 16:13</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
@@ -1058,35 +1064,35 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>384</v>
+        <v>313</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>DACTA II</t>
+          <t>BAMN</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>384260009381</t>
+          <t>313260018414</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>9514A-1</t>
+          <t>011-00916-10</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>PUMP ASSY</t>
+          <t>DISPLAY UNIT,FLIGHT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>R</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>2742</v>
+        <v>2740</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -1098,11 +1104,11 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J7" s="1" t="n">
-        <v>46167</v>
-      </c>
-      <c r="K7" s="1" t="n">
-        <v>46168</v>
+      <c r="J7" s="2" t="n">
+        <v>46185</v>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>46185</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
@@ -1112,18 +1118,18 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N7" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="O7" s="1" t="n">
-        <v>46203</v>
+      <c r="N7" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>46216</v>
       </c>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="n">
-        <v>10</v>
+        <v>-7</v>
       </c>
       <c r="R7" t="n">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1135,14 +1141,10 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>AWB 12743092324 - volume retirado na loja GOLLOG - CWB por Brendon. Godoy 30/06/2026.</t>
-        </is>
-      </c>
+      <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Colocado pedido no fornecedor I807209 dia 03/06. Previsão de entrega Miami 16/06. Previsão de chegada em GIG 18/06 - MATERIAL EM PROCESSO DE RECEBIMENTO STK V1 23/06/2026 - MATERIAL ENVIADO VIA RECIBO 501/FAB/26 AWB 12743092324 - MATERIAL DISPONIVEL PARA RETIRADA, CONTATO REALIZADO PARA RETIRADA 25/06/2026 - MATERIAL ENTREGUE DIA 25/06/2026 NOTA FISCAL ENVIADA DIA 25/06/2026 RC ATZ RC 14:21 26/06/2026</t>
+          <t>ENVIADO PARA O OPERADDOR DIA 02/0726, AWB 127-4481 4663- (REZ-02/07/26)</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
@@ -1159,35 +1161,35 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BAMN</t>
+          <t>BABR</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>313260018294</t>
+          <t>329260019153</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>011-00916-10</t>
+          <t>TWINA0502</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>DISPLAY UNIT,FLIGHT</t>
+          <t>PROBE TEMPERATURE</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>2741</v>
+        <v>2721</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -1199,11 +1201,11 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J8" s="1" t="n">
-        <v>46176</v>
-      </c>
-      <c r="K8" s="1" t="n">
-        <v>46176</v>
+      <c r="J8" s="2" t="n">
+        <v>46185</v>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>46185</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
@@ -1213,18 +1215,18 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N8" s="1" t="n">
-        <v>46207</v>
-      </c>
-      <c r="O8" s="1" t="n">
-        <v>46196</v>
+      <c r="N8" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="O8" s="2" t="n">
+        <v>46216</v>
       </c>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="n">
-        <v>2</v>
+        <v>-7</v>
       </c>
       <c r="R8" t="n">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1236,14 +1238,10 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>AWB 12742260142 volume retirado na loja GOLLOG - MAO por José silva em 23/06/2026 - Godoy 23/06/2026.</t>
-        </is>
-      </c>
+      <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
-          <t>CHECADO O ESTOQUE FAB QUE CONSTAVA NO SISTEMA O ESTOQUE, PORÉM É VIRTUAL. SOLICITADO APRESSAMENTO PARA A OFICINA REPARADORA ATZ 09/06/2026 - DPE de 01 ea para 18/06/2026 (REZ- 11/06/2026). - AWB 127-4226 0142 CLA 19-06 - MATERIAL DISPONIVEL PARA RETIRADA, DPE 23/06/2026 - RECIBO NO DRIVE E ENVIADO AO FISCAL</t>
+          <t>Colocado pedido na Textron IJ17507011. Previsão de entrega em Miami 17/06. Carga recepcionada no GIG 24/06. Canal verde dia 26/06. DPE V1 29/06. Verificar entrega do item. ATZ 30/06 - MATERIAL EM RECEBIMENTO V1 30-06-2026 - MATERIAL EM PROCESSO DE ENVIO RECIBO 524/FAB/26 ATZ RC 30-06-2026 - MATERIAL EM TRANSITO - AWB 12744330731 DPE 03/07/2026</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
@@ -1260,35 +1258,35 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>313</v>
+        <v>396</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>BAMN</t>
+          <t>BABE</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>313260018412</t>
+          <t>396260016520</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>011-01105-01</t>
+          <t>1H75-21</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>INTEGRATED AVIONICS</t>
+          <t>PRESSURE REGULATOR</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>T</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>2734</v>
+        <v>2726</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -1297,15 +1295,15 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>IPLR</t>
-        </is>
-      </c>
-      <c r="J9" s="1" t="n">
-        <v>46184</v>
-      </c>
-      <c r="K9" s="1" t="n">
+          <t>AIFP</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="n">
         <v>46185</v>
       </c>
+      <c r="K9" s="2" t="n">
+        <v>46185</v>
+      </c>
       <c r="L9" t="n">
         <v>1</v>
       </c>
@@ -1314,13 +1312,13 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N9" s="1" t="n">
-        <v>46196</v>
+      <c r="N9" s="2" t="n">
+        <v>46192</v>
       </c>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="R9" t="n">
         <v>24</v>
@@ -1333,12 +1331,12 @@
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr">
         <is>
-          <t>Retirado para atender a Anv 2737 - Godoy 12/06/26.</t>
+          <t>Item retirado para atender o C-98 2731. Ramon 15/06/26.</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Material Liberado Canal Verde em 01/7/2026 - HAWB: 00125552354 00004021 , Invoice PPSPI01534 PO 696/JPA/2026, aguardando ICMS GIGRJ. ATZ Marcio 01/7/2026 16:13</t>
+          <t>04 ea recolhidos para a V1, chegada dos itens dia 23/06/2026. Itens não tem oficina no Brasil, terá que ser feito Exchange rc 23/06 - MATERIAL ADQUIRIDO FORNECEDOR TEXTRON -WB0003073549 DPE AGS Miami 29/6/2026 ate 10 30AM - ATZ Marcio 26/6/26 17 23PM</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
@@ -1364,17 +1362,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>313260018414</t>
+          <t>313260018646</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>011-00916-10</t>
+          <t>011-00883-20</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>DISPLAY UNIT,FLIGHT</t>
+          <t>RADAR GWX 68 WEATHER</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1383,7 +1381,7 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>2740</v>
+        <v>2734</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -1392,14 +1390,14 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>ANCE</t>
-        </is>
-      </c>
-      <c r="J10" s="1" t="n">
-        <v>46185</v>
-      </c>
-      <c r="K10" s="1" t="n">
-        <v>46185</v>
+          <t>IPLR</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>46203</v>
       </c>
       <c r="L10" t="n">
         <v>1</v>
@@ -1409,18 +1407,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N10" s="1" t="n">
-        <v>46216</v>
-      </c>
-      <c r="O10" s="1" t="n">
-        <v>46216</v>
-      </c>
+      <c r="N10" s="2" t="n">
+        <v>46214</v>
+      </c>
+      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="n">
-        <v>-7</v>
+        <v>-5</v>
       </c>
       <c r="R10" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
@@ -1432,10 +1428,14 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr"/>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Retirado para atender a Anv 2740 - Godoy 30/06/26.</t>
+        </is>
+      </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>ENVIADO PARA O OPERADDOR DIA 02/0726, AWB 127-4481 4663- (REZ-02/07/26)</t>
+          <t>Efetuada a Compra em SP na Jet Avionics, aguardando confirmar unidade em estoque para liberação do item para a Veeone 01/7/2026 14:15 Marcio - DECLINADO pela JET AVIONICS, colocado Pedido TEXTRON Confirmation Number: WB0003077522 de 01/7/2026 Invoice IJ17546081 as 15:08PM Previsao DPE AGS Miami 02/7/2026 - ATZ Marcio 1/7/26 15:09</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
@@ -1452,26 +1452,26 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>329</v>
+        <v>313</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BABR</t>
+          <t>BAMN</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>329260019153</t>
+          <t>313260018651</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>TWINA0502</t>
+          <t>AS5174D1210</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>PROBE TEMPERATURE</t>
+          <t>REDUCER, TUBE</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1480,7 +1480,7 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>2721</v>
+        <v>2732</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -1489,14 +1489,14 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>ANCE</t>
-        </is>
-      </c>
-      <c r="J11" s="1" t="n">
-        <v>46185</v>
-      </c>
-      <c r="K11" s="1" t="n">
-        <v>46185</v>
+          <t>IPLR</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>46204</v>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>46205</v>
       </c>
       <c r="L11" t="n">
         <v>1</v>
@@ -1506,33 +1506,31 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N11" s="1" t="n">
+      <c r="N11" s="2" t="n">
         <v>46216</v>
       </c>
-      <c r="O11" s="1" t="n">
-        <v>46216</v>
-      </c>
+      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="n">
         <v>-7</v>
       </c>
       <c r="R11" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr"/>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Cedeu o item para o C-98 2738</t>
+        </is>
+      </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Colocado pedido na Textron IJ17507011. Previsão de entrega em Miami 17/06. Carga recepcionada no GIG 24/06. Canal verde dia 26/06. DPE V1 29/06. Verificar entrega do item. ATZ 30/06 - MATERIAL EM RECEBIMENTO V1 30-06-2026 - MATERIAL EM PROCESSO DE ENVIO RECIBO 524/FAB/26 ATZ RC 30-06-2026 - MATERIAL EM TRANSITO - AWB 12744330731 DPE 03/07/2026</t>
+          <t>PEDIDO NO EPM - FOI SOLICITADO ATENDIMENTO COM ESTOUE FAB - CLA-02-07</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
@@ -1549,35 +1547,35 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>396</v>
+        <v>313</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>BABE</t>
+          <t>BAMN</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>396260016520</t>
+          <t>313260018652</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1H75-21</t>
+          <t>24540-100</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>PRESSURE REGULATOR</t>
+          <t>COUPLING,CLAMP,GROOV</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>2726</v>
+        <v>2732</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -1586,14 +1584,14 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>AIFP</t>
-        </is>
-      </c>
-      <c r="J12" s="1" t="n">
-        <v>46185</v>
-      </c>
-      <c r="K12" s="1" t="n">
-        <v>46185</v>
+          <t>IPLR</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>46204</v>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>46205</v>
       </c>
       <c r="L12" t="n">
         <v>1</v>
@@ -1603,16 +1601,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N12" s="1" t="n">
-        <v>46192</v>
+      <c r="N12" s="2" t="n">
+        <v>46216</v>
       </c>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="n">
-        <v>17</v>
+        <v>-7</v>
       </c>
       <c r="R12" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -1622,12 +1620,12 @@
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr">
         <is>
-          <t>Item retirado para atender o C-98 2731. Ramon 15/06/26.</t>
+          <t>Cedeu o item para o C-98 2738</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>04 ea recolhidos para a V1, chegada dos itens dia 23/06/2026. Itens não tem oficina no Brasil, terá que ser feito Exchange rc 23/06 - MATERIAL ADQUIRIDO FORNECEDOR TEXTRON -WB0003073549 DPE AGS Miami 29/6/2026 ate 10 30AM - ATZ Marcio 26/6/26 17 23PM</t>
+          <t>Colocado pedido fornecedor nacional. Previsão de entrega V1 Campinas 03/07</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
@@ -1653,26 +1651,26 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>313260018646</t>
+          <t>313260018653</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>011-00883-20</t>
+          <t>MS24392-10</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>RADAR GWX 68 WEATHER</t>
+          <t>NIPPLE,TUBE</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>2734</v>
+        <v>2732</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1684,11 +1682,11 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J13" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="K13" s="1" t="n">
-        <v>46203</v>
+      <c r="J13" s="2" t="n">
+        <v>46204</v>
+      </c>
+      <c r="K13" s="2" t="n">
+        <v>46205</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1698,35 +1696,31 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N13" s="1" t="n">
-        <v>46214</v>
+      <c r="N13" s="2" t="n">
+        <v>46216</v>
       </c>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="n">
-        <v>-5</v>
+        <v>-7</v>
       </c>
       <c r="R13" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr">
-        <is>
           <t>Sim</t>
         </is>
       </c>
+      <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr">
         <is>
-          <t>Retirado para atender a Anv 2740 - Godoy 30/06/26.</t>
+          <t>Cedeu o item para o C-98 2738</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>Efetuada a Compra em SP na Jet Avionics, aguardando confirmar unidade em estoque para liberação do item para a Veeone 01/7/2026 14:15 Marcio - DECLINADO pela JET AVIONICS, colocado Pedido TEXTRON Confirmation Number: WB0003077522 de 01/7/2026 Invoice IJ17546081 as 15:08PM Previsao DPE AGS Miami 02/7/2026 - ATZ Marcio 1/7/26 15:09</t>
+          <t>PEDIDO NO EPM - FOI SOLICITADO ATENDIMENTO COM ESTOUE FAB - CLA-02-07</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
@@ -1743,35 +1737,35 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BAMN</t>
+          <t>BABR</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>313260018651</t>
+          <t>329260019179</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>AS5174D1210</t>
+          <t>066-3046-07</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>REDUCER, TUBE</t>
+          <t>CONTROL,INDICATOR</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>R</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>2732</v>
+        <v>2721</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -1780,15 +1774,15 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>IPLR</t>
-        </is>
-      </c>
-      <c r="J14" s="1" t="n">
-        <v>46204</v>
-      </c>
-      <c r="K14" s="1" t="n">
+          <t>AIFP</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="n">
         <v>46205</v>
       </c>
+      <c r="K14" s="2" t="n">
+        <v>46206</v>
+      </c>
       <c r="L14" t="n">
         <v>1</v>
       </c>
@@ -1797,33 +1791,25 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N14" s="1" t="n">
-        <v>46216</v>
+      <c r="N14" s="2" t="n">
+        <v>46213</v>
       </c>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="n">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="R14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>Cedeu o item para o C-98 2738</t>
-        </is>
-      </c>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>PEDIDO NO EPM - FOI SOLICITADO ATENDIMENTO COM ESTOUE FAB - CLA-02-07</t>
-        </is>
-      </c>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr">
         <is>
           <t>VEE ONE</t>
@@ -1833,283 +1819,6 @@
       <c r="Y14" t="inlineStr"/>
       <c r="Z14" t="inlineStr"/>
       <c r="AA14" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>313</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>BAMN</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>313260018652</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>24540-100</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>COUPLING,CLAMP,GROOV</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G15" t="n">
-        <v>2732</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Providência tomada</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>IPLR</t>
-        </is>
-      </c>
-      <c r="J15" s="1" t="n">
-        <v>46204</v>
-      </c>
-      <c r="K15" s="1" t="n">
-        <v>46205</v>
-      </c>
-      <c r="L15" t="n">
-        <v>1</v>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>EA</t>
-        </is>
-      </c>
-      <c r="N15" s="1" t="n">
-        <v>46216</v>
-      </c>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="n">
-        <v>-7</v>
-      </c>
-      <c r="R15" t="n">
-        <v>4</v>
-      </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>Cedeu o item para o C-98 2738</t>
-        </is>
-      </c>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>Colocado pedido fornecedor nacional. Previsão de entrega V1 Campinas 03/07</t>
-        </is>
-      </c>
-      <c r="W15" t="inlineStr">
-        <is>
-          <t>VEE ONE</t>
-        </is>
-      </c>
-      <c r="X15" t="inlineStr"/>
-      <c r="Y15" t="inlineStr"/>
-      <c r="Z15" t="inlineStr"/>
-      <c r="AA15" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>313</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>BAMN</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>313260018653</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>MS24392-10</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>NIPPLE,TUBE</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G16" t="n">
-        <v>2732</v>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Providência tomada</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>IPLR</t>
-        </is>
-      </c>
-      <c r="J16" s="1" t="n">
-        <v>46204</v>
-      </c>
-      <c r="K16" s="1" t="n">
-        <v>46205</v>
-      </c>
-      <c r="L16" t="n">
-        <v>1</v>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>EA</t>
-        </is>
-      </c>
-      <c r="N16" s="1" t="n">
-        <v>46216</v>
-      </c>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="n">
-        <v>-7</v>
-      </c>
-      <c r="R16" t="n">
-        <v>4</v>
-      </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>Cedeu o item para o C-98 2738</t>
-        </is>
-      </c>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>PEDIDO NO EPM - FOI SOLICITADO ATENDIMENTO COM ESTOUE FAB - CLA-02-07</t>
-        </is>
-      </c>
-      <c r="W16" t="inlineStr">
-        <is>
-          <t>VEE ONE</t>
-        </is>
-      </c>
-      <c r="X16" t="inlineStr"/>
-      <c r="Y16" t="inlineStr"/>
-      <c r="Z16" t="inlineStr"/>
-      <c r="AA16" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>329</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>BABR</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>329260019179</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>066-3046-07</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>CONTROL,INDICATOR</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="G17" t="n">
-        <v>2721</v>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Providência tomada</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>AIFP</t>
-        </is>
-      </c>
-      <c r="J17" s="1" t="n">
-        <v>46205</v>
-      </c>
-      <c r="K17" s="1" t="n">
-        <v>46206</v>
-      </c>
-      <c r="L17" t="n">
-        <v>1</v>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>EA</t>
-        </is>
-      </c>
-      <c r="N17" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="n">
-        <v>-4</v>
-      </c>
-      <c r="R17" t="n">
-        <v>3</v>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr">
-        <is>
-          <t>VEE ONE</t>
-        </is>
-      </c>
-      <c r="X17" t="inlineStr"/>
-      <c r="Y17" t="inlineStr"/>
-      <c r="Z17" t="inlineStr"/>
-      <c r="AA17" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auditoria: confirma RAC/Emergências/Pagamentos imunes ao bug do BOM
Rodei atualizar_do_drive() de verdade nas 3 fontes que faltavam auditar
depois do bug da Disponibilidade Diária — todas usam exportação binária
(.xlsx), não texto puro, então não têm o mesmo risco de BOM quebrando o
parser. Sem erros nas 3; dados do dia (07/07) atualizados como consequência.
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA14"/>
+  <dimension ref="A1:AA17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -631,10 +631,10 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="n">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -726,10 +726,10 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="R3" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -819,14 +819,14 @@
         <v>46184</v>
       </c>
       <c r="O4" s="2" t="n">
-        <v>46178</v>
+        <v>46148</v>
       </c>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="R4" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -840,7 +840,7 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>O item em estoque na BANT foi enviado pela própria Vee One em 08/05. A intenção realmente é pegar o item de volta?</t>
+          <t>O item em estoque na BANT foi enviado pela própria Vee One em 08/05. A intenção realmente é pegar o item de volta? Recibo 432/FAB/26 é referente a atendimento de emergência do 2741 em Manaus. Ramon 07/07/26.</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -930,10 +930,10 @@
       </c>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="R5" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R6" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1047,7 +1047,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Material Liberado Canal Verde em 01/7/2026 - HAWB: 00125552354 00004021 , Invoice PPSPI01534 PO 696/JPA/2026, aguardando ICMS GIGRJ. ATZ Marcio 01/7/2026 16:13</t>
+          <t>Material Liberado Canal Verde em 01/7/2026 - HAWB: 00125552354 00004021 , Invoice PPSPI01534 PO 696/JPA/2026, aguardando ICMS GIGRJ. ATZ Marcio 01/7/2026 16:13 - material em processo de envio 06/07/2026</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
@@ -1126,10 +1126,10 @@
       </c>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R7" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1223,10 +1223,10 @@
       </c>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R8" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1241,7 +1241,7 @@
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Colocado pedido na Textron IJ17507011. Previsão de entrega em Miami 17/06. Carga recepcionada no GIG 24/06. Canal verde dia 26/06. DPE V1 29/06. Verificar entrega do item. ATZ 30/06 - MATERIAL EM RECEBIMENTO V1 30-06-2026 - MATERIAL EM PROCESSO DE ENVIO RECIBO 524/FAB/26 ATZ RC 30-06-2026 - MATERIAL EM TRANSITO - AWB 12744330731 DPE 03/07/2026</t>
+          <t>Material Liberado Canal Verde em 01/7/2026 - HAWB: 00125552354 00004021 , Invoice PPSPI01534 PO 696/JPA/2026, aguardando ICMS GIGRJ. ATZ Marcio 01/7/2026 16:13 - material em processo de envio 06/07/2026</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
@@ -1318,10 +1318,10 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="R9" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -1336,7 +1336,7 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>04 ea recolhidos para a V1, chegada dos itens dia 23/06/2026. Itens não tem oficina no Brasil, terá que ser feito Exchange rc 23/06 - MATERIAL ADQUIRIDO FORNECEDOR TEXTRON -WB0003073549 DPE AGS Miami 29/6/2026 ate 10 30AM - ATZ Marcio 26/6/26 17 23PM</t>
+          <t>04 ea recolhidos para a V1, chegada dos itens dia 23/06/2026. Itens não tem oficina no Brasil, terá que ser feito Exchange rc 23/06 - MATERIAL ADQUIRIDO FORNECEDOR TEXTRON -WB0003073549 Inovice IJ17534800 DPE AGS Miami 29/6/2026 ate 10 30AM - AIR EXPORT HOUSE: 00004046 de 30/6/2026 Chegou no GIGRJ em 01/7/26 para Desembaraço - ATZ Marcio 3/7/2614:35</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
@@ -1413,10 +1413,10 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="n">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
@@ -1435,7 +1435,7 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Efetuada a Compra em SP na Jet Avionics, aguardando confirmar unidade em estoque para liberação do item para a Veeone 01/7/2026 14:15 Marcio - DECLINADO pela JET AVIONICS, colocado Pedido TEXTRON Confirmation Number: WB0003077522 de 01/7/2026 Invoice IJ17546081 as 15:08PM Previsao DPE AGS Miami 02/7/2026 - ATZ Marcio 1/7/26 15:09</t>
+          <t>Efetuada a Compra em SP na Jet Avionics, aguardando confirmar unidade em estoque para liberação do item para a Veeone 01/7/2026 14:15 Marcio - DECLINADO pela JET AVIONICS, colocado Pedido TEXTRON Confirmation Number: WB0003077522 de 01/7/2026 Invoice IJ17546081 as 15:08PM Previsao DPE AGS Miami 02/7/2026 - PRE ALERTA do VOO de 3/7/2026 aguardando chegada no GIGRJ - ATZ Marcio 3/7/26 14:31</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
@@ -1512,10 +1512,10 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
@@ -1525,7 +1525,7 @@
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr">
         <is>
-          <t>Cedeu o item para o C-98 2738</t>
+          <t>Cedeu o item para o C-98 2738. Pedido será atendido pelo estoque FAB pedido n° 17874678 - Godoy 07/07/2026.</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
@@ -1607,10 +1607,10 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -1702,10 +1702,10 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
@@ -1715,7 +1715,7 @@
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr">
         <is>
-          <t>Cedeu o item para o C-98 2738</t>
+          <t>Cedeu o item para o C-98 2738. Pedido será atendido pelo estoque FAB pedido n° 17875036 - Godoy 07/07/2026.</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
@@ -1797,10 +1797,10 @@
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
@@ -1809,7 +1809,11 @@
       </c>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr"/>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>Item estara disponivel no RJ na oficina para coleta dia 6/7 apos as 14 horas ATZ Marcio 3/7/ 14:25PM</t>
+        </is>
+      </c>
       <c r="W14" t="inlineStr">
         <is>
           <t>VEE ONE</t>
@@ -1819,6 +1823,267 @@
       <c r="Y14" t="inlineStr"/>
       <c r="Z14" t="inlineStr"/>
       <c r="AA14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>329</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>BABR</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>329260019180</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>C145-00-46</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>TRANSMISSION ASSY</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>2709</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Aguardando solução</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>AIFP</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="K15" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="L15" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="n">
+        <v>-7</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>VEE ONE</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr"/>
+      <c r="Y15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr"/>
+      <c r="AA15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>329</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>BABR</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>329260019181</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>C145-00-46</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>TRANSMISSION ASSY</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>2721</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Aguardando solução</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>AIFP</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="K16" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="L16" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="n">
+        <v>-7</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>VEE ONE</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr"/>
+      <c r="Y16" t="inlineStr"/>
+      <c r="Z16" t="inlineStr"/>
+      <c r="AA16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>685</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>BANT</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>685260012303</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>065-0065-01</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>SELECTOR ALT</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>2719</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Aguardando solução</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>ANCE</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="K17" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="L17" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="n">
+        <v>-31</v>
+      </c>
+      <c r="R17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>VEE ONE</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr"/>
+      <c r="Y17" t="inlineStr"/>
+      <c r="Z17" t="inlineStr"/>
+      <c r="AA17" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (07/07/2026 21:06)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,137 +421,137 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>om_emg</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>om</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>numero_emergencia</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>categoria</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>matricula_aeronave</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>tpemg</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>data_abertura</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>data_info</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>quantidade</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>unidade_medida</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>prazo_entrega</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>dpe</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>atendido_cancelado</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>dias_atraso</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>dias_corridos</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>estoque</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>retirado_empresa_recibo_obrigatorio</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>obs_coordenadoria_fiscal</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>obs_vee_one</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>provedor</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>awb</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>prev_entrega</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>mensagem_operador</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>em_aberto</t>
         </is>
@@ -611,10 +599,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J2" s="2" t="n">
+      <c r="J2" s="1" t="n">
         <v>46057</v>
       </c>
-      <c r="K2" s="2" t="n">
+      <c r="K2" s="1" t="n">
         <v>46204</v>
       </c>
       <c r="L2" t="n">
@@ -625,7 +613,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N2" s="2" t="n">
+      <c r="N2" s="1" t="n">
         <v>46215</v>
       </c>
       <c r="O2" t="inlineStr"/>
@@ -706,10 +694,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J3" s="2" t="n">
+      <c r="J3" s="1" t="n">
         <v>46076</v>
       </c>
-      <c r="K3" s="2" t="n">
+      <c r="K3" s="1" t="n">
         <v>46080</v>
       </c>
       <c r="L3" t="n">
@@ -720,7 +708,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N3" s="2" t="n">
+      <c r="N3" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="O3" t="inlineStr"/>
@@ -801,10 +789,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J4" s="2" t="n">
+      <c r="J4" s="1" t="n">
         <v>46150</v>
       </c>
-      <c r="K4" s="2" t="n">
+      <c r="K4" s="1" t="n">
         <v>46153</v>
       </c>
       <c r="L4" t="n">
@@ -815,10 +803,10 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N4" s="2" t="n">
+      <c r="N4" s="1" t="n">
         <v>46184</v>
       </c>
-      <c r="O4" s="2" t="n">
+      <c r="O4" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -908,10 +896,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J5" s="2" t="n">
+      <c r="J5" s="1" t="n">
         <v>46160</v>
       </c>
-      <c r="K5" s="2" t="n">
+      <c r="K5" s="1" t="n">
         <v>46161</v>
       </c>
       <c r="L5" t="n">
@@ -922,10 +910,10 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N5" s="2" t="n">
+      <c r="N5" s="1" t="n">
         <v>46192</v>
       </c>
-      <c r="O5" s="2" t="n">
+      <c r="O5" s="1" t="n">
         <v>-620019</v>
       </c>
       <c r="P5" t="inlineStr"/>
@@ -1009,10 +997,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J6" s="2" t="n">
+      <c r="J6" s="1" t="n">
         <v>46184</v>
       </c>
-      <c r="K6" s="2" t="n">
+      <c r="K6" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="L6" t="n">
@@ -1023,7 +1011,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N6" s="2" t="n">
+      <c r="N6" s="1" t="n">
         <v>46196</v>
       </c>
       <c r="O6" t="inlineStr"/>
@@ -1104,10 +1092,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="J7" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="K7" s="2" t="n">
+      <c r="K7" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="L7" t="n">
@@ -1118,10 +1106,10 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N7" s="2" t="n">
+      <c r="N7" s="1" t="n">
         <v>46216</v>
       </c>
-      <c r="O7" s="2" t="n">
+      <c r="O7" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1201,10 +1189,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J8" s="2" t="n">
+      <c r="J8" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="K8" s="2" t="n">
+      <c r="K8" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="L8" t="n">
@@ -1215,10 +1203,10 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N8" s="2" t="n">
+      <c r="N8" s="1" t="n">
         <v>46216</v>
       </c>
-      <c r="O8" s="2" t="n">
+      <c r="O8" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1298,10 +1286,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J9" s="2" t="n">
+      <c r="J9" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="K9" s="2" t="n">
+      <c r="K9" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="L9" t="n">
@@ -1312,7 +1300,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N9" s="2" t="n">
+      <c r="N9" s="1" t="n">
         <v>46192</v>
       </c>
       <c r="O9" t="inlineStr"/>
@@ -1393,10 +1381,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J10" s="2" t="n">
+      <c r="J10" s="1" t="n">
         <v>46199</v>
       </c>
-      <c r="K10" s="2" t="n">
+      <c r="K10" s="1" t="n">
         <v>46203</v>
       </c>
       <c r="L10" t="n">
@@ -1407,7 +1395,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N10" s="2" t="n">
+      <c r="N10" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="O10" t="inlineStr"/>
@@ -1492,10 +1480,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J11" s="2" t="n">
+      <c r="J11" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="K11" s="2" t="n">
+      <c r="K11" s="1" t="n">
         <v>46205</v>
       </c>
       <c r="L11" t="n">
@@ -1506,7 +1494,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N11" s="2" t="n">
+      <c r="N11" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="O11" t="inlineStr"/>
@@ -1587,10 +1575,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J12" s="2" t="n">
+      <c r="J12" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="K12" s="2" t="n">
+      <c r="K12" s="1" t="n">
         <v>46205</v>
       </c>
       <c r="L12" t="n">
@@ -1601,7 +1589,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N12" s="2" t="n">
+      <c r="N12" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="O12" t="inlineStr"/>
@@ -1682,10 +1670,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J13" s="2" t="n">
+      <c r="J13" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="K13" s="2" t="n">
+      <c r="K13" s="1" t="n">
         <v>46205</v>
       </c>
       <c r="L13" t="n">
@@ -1696,7 +1684,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N13" s="2" t="n">
+      <c r="N13" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="O13" t="inlineStr"/>
@@ -1777,10 +1765,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J14" s="2" t="n">
+      <c r="J14" s="1" t="n">
         <v>46205</v>
       </c>
-      <c r="K14" s="2" t="n">
+      <c r="K14" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="L14" t="n">
@@ -1791,7 +1779,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N14" s="2" t="n">
+      <c r="N14" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="O14" t="inlineStr"/>
@@ -1868,10 +1856,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J15" s="2" t="n">
+      <c r="J15" s="1" t="n">
         <v>46209</v>
       </c>
-      <c r="K15" s="2" t="n">
+      <c r="K15" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="L15" t="n">
@@ -1882,7 +1870,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N15" s="2" t="n">
+      <c r="N15" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="O15" t="inlineStr"/>
@@ -1955,10 +1943,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J16" s="2" t="n">
+      <c r="J16" s="1" t="n">
         <v>46209</v>
       </c>
-      <c r="K16" s="2" t="n">
+      <c r="K16" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="L16" t="n">
@@ -1969,7 +1957,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N16" s="2" t="n">
+      <c r="N16" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="O16" t="inlineStr"/>
@@ -2042,10 +2030,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J17" s="2" t="n">
+      <c r="J17" s="1" t="n">
         <v>46210</v>
       </c>
-      <c r="K17" s="2" t="n">
+      <c r="K17" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="L17" t="n">
@@ -2056,7 +2044,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N17" s="2" t="n">
+      <c r="N17" s="1" t="n">
         <v>46241</v>
       </c>
       <c r="O17" t="inlineStr"/>

</xml_diff>

<commit_message>
Atualização automática: emergencias (08/07/2026 14:33)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -417,141 +429,141 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA17"/>
+  <dimension ref="A1:AA16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>om_emg</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>om</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>numero_emergencia</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>categoria</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>matricula_aeronave</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>tpemg</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>data_abertura</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>data_info</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>quantidade</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>unidade_medida</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>prazo_entrega</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>dpe</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>atendido_cancelado</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>dias_atraso</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>dias_corridos</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>estoque</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>retirado_empresa_recibo_obrigatorio</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>obs_coordenadoria_fiscal</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>obs_vee_one</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>provedor</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>awb</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>prev_entrega</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>mensagem_operador</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>em_aberto</t>
         </is>
@@ -568,26 +580,26 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>313260017680</t>
+          <t>313260017747</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>030-18200</t>
+          <t>1214134-1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>MAIN WHEEL BRAKE</t>
+          <t>BELLCRANK ASSY</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>2732</v>
+        <v>2730</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -596,48 +608,48 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>IPLR</t>
-        </is>
-      </c>
-      <c r="J2" s="1" t="n">
-        <v>46057</v>
-      </c>
-      <c r="K2" s="1" t="n">
-        <v>46204</v>
+          <t>ANCE</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>46076</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>46080</v>
       </c>
       <c r="L2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
           <t>EA</t>
         </is>
       </c>
-      <c r="N2" s="1" t="n">
-        <v>46215</v>
+      <c r="N2" s="2" t="n">
+        <v>46111</v>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="n">
-        <v>-5</v>
+        <v>100</v>
       </c>
       <c r="R2" t="n">
-        <v>6</v>
+        <v>131</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Cedeu conjunto de freio para o 2738 em 19/07/2025. Ramon 30/06/26.</t>
+          <t>Foram cedidos para o C-98 2733. / De acordo com o manual da aeronave, o QPA é 02 EA por cadeira. Sendo o total para a aeronave 04 EA.A demanda aberta foi de  4EA, o SO Bispo que intermediou . Wallace 29.05</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>MATERIAL EM PROCESSO DE EXPEDIÇÃO DIA 01/07/2026 - SERIAL 02LS - MATERIAL EM TRANSITO RECIBO 529/FAB/26 AWB 12744560622 DPE 07/07/2026</t>
+          <t>Foi solicitado via email no dia 02-03-2 o atendimento do item com estoque FAB. Claudio -02-03-26 - Em resposta, a coordenadoria disse que o estque seria insuficiente. Foi verificado que na T.O da ANV o QPA para esse item são 2 EA, solicitei confirmação. - Cláudio -02-03-2026. Solicitado o cancelamento da emergência em função da quantidade cedida ao 2733 ter sido de 01ea. Considerando o QPA 02 ea. Encontra-se em tratativa junto a fiscalização e o gestor do contrato conforme mensagem de e-mail de 05/03. - SOLICITAÇÃO E-C98-26047.Colocado pedido AOG Textron WB0003068789 - previsão de entrega 60 dias em média. Os demais fornecedores informaram não ter em estoque ou não possuírem a certificação necessária da peça.</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
@@ -654,35 +666,35 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BAMN</t>
+          <t>BABR</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>313260017747</t>
+          <t>329260019106</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1214134-1</t>
+          <t>066-3084-32</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BELLCRANK ASSY</t>
+          <t>IND RDR 2000 IN-182A</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>R</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>2730</v>
+        <v>2721</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -694,45 +706,51 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J3" s="1" t="n">
-        <v>46076</v>
-      </c>
-      <c r="K3" s="1" t="n">
-        <v>46080</v>
+      <c r="J3" s="2" t="n">
+        <v>46150</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>46153</v>
       </c>
       <c r="L3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
           <t>EA</t>
         </is>
       </c>
-      <c r="N3" s="1" t="n">
-        <v>46111</v>
-      </c>
-      <c r="O3" t="inlineStr"/>
+      <c r="N3" s="2" t="n">
+        <v>46184</v>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>46148</v>
+      </c>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="n">
-        <v>99</v>
+        <v>27</v>
       </c>
       <c r="R3" t="n">
-        <v>130</v>
+        <v>58</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Foram cedidos para o C-98 2733. / De acordo com o manual da aeronave, o QPA é 02 EA por cadeira. Sendo o total para a aeronave 04 EA.A demanda aberta foi de  4EA, o SO Bispo que intermediou . Wallace 29.05</t>
+          <t>O item em estoque na BANT foi enviado pela própria Vee One em 08/05. A intenção realmente é pegar o item de volta? Recibo 432/FAB/26 é referente a atendimento de emergência do 2741 em Manaus. Ramon 07/07/26.</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Foi solicitado via email no dia 02-03-2 o atendimento do item com estoque FAB. Claudio -02-03-26 - Em resposta, a coordenadoria disse que o estque seria insuficiente. Foi verificado que na T.O da ANV o QPA para esse item são 2 EA, solicitei confirmação. - Cláudio -02-03-2026. Solicitado o cancelamento da emergência em função da quantidade cedida ao 2733 ter sido de 01ea. Considerando o QPA 02 ea. Encontra-se em tratativa junto a fiscalização e o gestor do contrato conforme mensagem de e-mail de 05/03. - SOLICITAÇÃO E-C98-26047.Colocado pedido AOG Textron WB0003068789 - previsão de entrega 60 dias em média. Os demais fornecedores informaram não ter em estoque ou não possuírem a certificação necessária da peça.</t>
+          <t>Colocado pedido junto ao fornecedor I800035 dia 30/04. ENTREGUE EM MIAMI 14/05. Carga recepcionada VCP dia 23/05. Em processo de desembaraço aduaneiro. ATZ 28/05 - MATERIAL EM RECEBIMENTO V1 AMA 29/05/2026 RC 12:06 - MATERIAL ENVIADO PELA AWB 12738616480 - DPE 02/06/2026 - MATERIAL RECEBIDO DIA 02/06/2026 3S SARA RECIBO ASSINADO 432-fab-26 EM 313260018247 313260018248 ATZ RC 03/06/2026 14:18 - RECIBO NO DRIVE COMPARTILHADO - 432-fab-26 EM 313260018247 313260018248</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
@@ -740,44 +758,50 @@
           <t>VEE ONE</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr"/>
+      <c r="X3" t="n">
+        <v>12738926716</v>
+      </c>
       <c r="Y3" t="inlineStr"/>
-      <c r="Z3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>Informo o envio de 1 EA do IND RDR 2000 IN-182A (PN 066-3084-32) para atender ANCE 329260019106 do C-98 2721 (BABR) através do AWB 12738926716 com previsão de entrega em .</t>
+        </is>
+      </c>
       <c r="AA3" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>329</v>
+        <v>304</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BABR</t>
+          <t>PAMA-LS</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>329260019106</t>
+          <t>304260076049</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>066-3084-32</t>
+          <t>C596504-0102</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>IND RDR 2000 IN-182A</t>
+          <t>OVERHEAD SPEAKER</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>2721</v>
+        <v>2704</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -789,11 +813,11 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J4" s="1" t="n">
-        <v>46150</v>
-      </c>
-      <c r="K4" s="1" t="n">
-        <v>46153</v>
+      <c r="J4" s="2" t="n">
+        <v>46160</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>46161</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
@@ -803,18 +827,18 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N4" s="1" t="n">
-        <v>46184</v>
-      </c>
-      <c r="O4" s="1" t="n">
-        <v>46148</v>
+      <c r="N4" s="2" t="n">
+        <v>46192</v>
+      </c>
+      <c r="O4" s="2" t="n">
+        <v>-620019</v>
       </c>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="R4" t="n">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -823,17 +847,17 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>O item em estoque na BANT foi enviado pela própria Vee One em 08/05. A intenção realmente é pegar o item de volta? Recibo 432/FAB/26 é referente a atendimento de emergência do 2741 em Manaus. Ramon 07/07/26.</t>
+          <t>Recibo não se encontra na Pasta do DRIVE. Godoy 30/06/2026.Como não tem AWB vou cobrar o recibo Wallace 30/06/2026</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Colocado pedido junto ao fornecedor I800035 dia 30/04. ENTREGUE EM MIAMI 14/05. Carga recepcionada VCP dia 23/05. Em processo de desembaraço aduaneiro. ATZ 28/05 - MATERIAL EM RECEBIMENTO V1 AMA 29/05/2026 RC 12:06 - MATERIAL ENVIADO PELA AWB 12738616480 - DPE 02/06/2026 - MATERIAL RECEBIDO DIA 02/06/2026 3S SARA RECIBO ASSINADO 432-fab-26 EM 313260018247 313260018248 ATZ RC 03/06/2026 14:18 - RECIBO NO DRIVE COMPARTILHADO - 432-fab-26 EM 313260018247 313260018248</t>
+          <t>Colocado pedido I803776 no fornecedor dia 18/05. Chegada em VCP dia 04/06 (voo 3906). Canal amarelo dia 10/06. Carga liberada para entrega em Campinas 25/06 - MATERIAL EM TRANSITO - DIA 25/06/2026 - RECIBO 511/FAB/26 DPE 29/06/2026 ATZ RC 14:21 26/06/2026</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
@@ -841,50 +865,44 @@
           <t>VEE ONE</t>
         </is>
       </c>
-      <c r="X4" t="n">
-        <v>12738926716</v>
-      </c>
+      <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>Informo o envio de 1 EA do IND RDR 2000 IN-182A (PN 066-3084-32) para atender ANCE 329260019106 do C-98 2721 (BABR) através do AWB 12738926716 com previsão de entrega em .</t>
-        </is>
-      </c>
+      <c r="Z4" t="inlineStr"/>
       <c r="AA4" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>304</v>
+        <v>313</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>PAMA-LS</t>
+          <t>BAMN</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>304260076049</t>
+          <t>313260018412</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>C596504-0102</t>
+          <t>011-01105-01</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>OVERHEAD SPEAKER</t>
+          <t>INTEGRATED AVIONICS</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>R</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>2704</v>
+        <v>2734</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -893,14 +911,14 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>ANCE</t>
-        </is>
-      </c>
-      <c r="J5" s="1" t="n">
-        <v>46160</v>
-      </c>
-      <c r="K5" s="1" t="n">
-        <v>46161</v>
+          <t>IPLR</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>46184</v>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>46185</v>
       </c>
       <c r="L5" t="n">
         <v>1</v>
@@ -910,37 +928,31 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N5" s="1" t="n">
-        <v>46192</v>
-      </c>
-      <c r="O5" s="1" t="n">
-        <v>-620019</v>
-      </c>
+      <c r="N5" s="2" t="n">
+        <v>46196</v>
+      </c>
+      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="R5" t="n">
-        <v>49</v>
+        <v>26</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
+      <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Recibo não se encontra na Pasta do DRIVE. Godoy 30/06/2026.Como não tem AWB vou cobrar o recibo Wallace 30/06/2026</t>
+          <t>Retirado para atender a Anv 2737 - Godoy 12/06/26.</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Colocado pedido I803776 no fornecedor dia 18/05. Chegada em VCP dia 04/06 (voo 3906). Canal amarelo dia 10/06. Carga liberada para entrega em Campinas 25/06 - MATERIAL EM TRANSITO - DIA 25/06/2026 - RECIBO 511/FAB/26 DPE 29/06/2026 ATZ RC 14:21 26/06/2026</t>
+          <t>Material Liberado Canal Verde em 01/7/2026 - HAWB: 00125552354 00004021 , Invoice PPSPI01534 PO 696/JPA/2026, aguardando ICMS GIGRJ. ATZ Marcio 01/7/2026 16:13 - material em processo de envio 06/07/2026 - AWB 12744955875 dpe 10/07/2026</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
@@ -957,35 +969,35 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BAMN</t>
+          <t>BABR</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>313260018412</t>
+          <t>329260019153</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>011-01105-01</t>
+          <t>TWINA0502</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>INTEGRATED AVIONICS</t>
+          <t>PROBE TEMPERATURE</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>2734</v>
+        <v>2721</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -994,15 +1006,15 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>IPLR</t>
-        </is>
-      </c>
-      <c r="J6" s="1" t="n">
-        <v>46184</v>
-      </c>
-      <c r="K6" s="1" t="n">
+          <t>ANCE</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n">
         <v>46185</v>
       </c>
+      <c r="K6" s="2" t="n">
+        <v>46185</v>
+      </c>
       <c r="L6" t="n">
         <v>1</v>
       </c>
@@ -1011,31 +1023,37 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N6" s="1" t="n">
-        <v>46196</v>
-      </c>
-      <c r="O6" t="inlineStr"/>
+      <c r="N6" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="O6" s="2" t="n">
+        <v>46216</v>
+      </c>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="n">
-        <v>14</v>
+        <v>-5</v>
       </c>
       <c r="R6" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr"/>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Retirado para atender a Anv 2737 - Godoy 12/06/26.</t>
+          <t>Volume retirado na loja GOLLOG - BSB por tanise Assis em 03/07/2026 - Godoy 08/07/2026. Recibo não se encontra na Pasta do DRIVE. Godoy 08/07/2026.</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Material Liberado Canal Verde em 01/7/2026 - HAWB: 00125552354 00004021 , Invoice PPSPI01534 PO 696/JPA/2026, aguardando ICMS GIGRJ. ATZ Marcio 01/7/2026 16:13 - material em processo de envio 06/07/2026</t>
+          <t>Colocado pedido na Textron IJ17507011. Previsão de entrega em Miami 17/06. Carga recepcionada no GIG 24/06. Canal verde dia 26/06. DPE V1 29/06. Verificar entrega do item. ATZ 30/06 - MATERIAL EM RECEBIMENTO V1 30-06-2026 - MATERIAL EM PROCESSO DE ENVIO RECIBO 524/FAB/26 ATZ RC 30-06-2026 - MATERIAL EM TRANSITO - AWB 12744330731 DPE 03/07/2026 - MATERIAL RECEBIDO POR tanise Assis RG 14807641751 DIA 03/07/2026</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
@@ -1052,35 +1070,35 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>313</v>
+        <v>396</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BAMN</t>
+          <t>BABE</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>313260018414</t>
+          <t>396260016520</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>011-00916-10</t>
+          <t>1H75-21</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>DISPLAY UNIT,FLIGHT</t>
+          <t>PRESSURE REGULATOR</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>T</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>2740</v>
+        <v>2726</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -1089,13 +1107,13 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>ANCE</t>
-        </is>
-      </c>
-      <c r="J7" s="1" t="n">
+          <t>AIFP</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="n">
         <v>46185</v>
       </c>
-      <c r="K7" s="1" t="n">
+      <c r="K7" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="L7" t="n">
@@ -1106,33 +1124,31 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N7" s="1" t="n">
-        <v>46216</v>
-      </c>
-      <c r="O7" s="1" t="n">
-        <v>46216</v>
-      </c>
+      <c r="N7" s="2" t="n">
+        <v>46192</v>
+      </c>
+      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="n">
-        <v>-6</v>
+        <v>19</v>
       </c>
       <c r="R7" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Item retirado para atender o C-98 2731. Ramon 15/06/26.</t>
+        </is>
+      </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>ENVIADO PARA O OPERADDOR DIA 02/0726, AWB 127-4481 4663- (REZ-02/07/26)</t>
+          <t>04 ea recolhidos para a V1, chegada dos itens dia 23/06/2026. Itens não tem oficina no Brasil, terá que ser feito Exchange rc 23/06 - MATERIAL ADQUIRIDO FORNECEDOR TEXTRON -WB0003073549 Inovice IJ17534800 DPE AGS Miami 29/6/2026 ate 10 30AM - AIR EXPORT HOUSE: 00004046 de 30/6/2026 Chegou no GIGRJ em 01/7/26 para Desembaraço - ATZ Marcio 3/7/2614:35</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
@@ -1149,35 +1165,35 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>329</v>
+        <v>313</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BABR</t>
+          <t>BAMN</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>329260019153</t>
+          <t>313260018646</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>TWINA0502</t>
+          <t>011-00883-20</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>PROBE TEMPERATURE</t>
+          <t>RADAR GWX 68 WEATHER</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>R</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>2721</v>
+        <v>2734</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -1186,14 +1202,14 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>ANCE</t>
-        </is>
-      </c>
-      <c r="J8" s="1" t="n">
-        <v>46185</v>
-      </c>
-      <c r="K8" s="1" t="n">
-        <v>46185</v>
+          <t>IPLR</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>46203</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
@@ -1203,18 +1219,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N8" s="1" t="n">
-        <v>46216</v>
-      </c>
-      <c r="O8" s="1" t="n">
-        <v>46216</v>
-      </c>
+      <c r="N8" s="2" t="n">
+        <v>46214</v>
+      </c>
+      <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="n">
-        <v>-6</v>
+        <v>-3</v>
       </c>
       <c r="R8" t="n">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1223,13 +1237,17 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr"/>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Retirado para atender a Anv 2740 - Godoy 30/06/26.</t>
+        </is>
+      </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Material Liberado Canal Verde em 01/7/2026 - HAWB: 00125552354 00004021 , Invoice PPSPI01534 PO 696/JPA/2026, aguardando ICMS GIGRJ. ATZ Marcio 01/7/2026 16:13 - material em processo de envio 06/07/2026</t>
+          <t>Efetuada a Compra em SP na Jet Avionics, aguardando confirmar unidade em estoque para liberação do item para a Veeone 01/7/2026 14:15 Marcio - DECLINADO pela JET AVIONICS, colocado Pedido TEXTRON Confirmation Number: WB0003077522 de 01/7/2026 Invoice IJ17546081 as 15:08PM Previsao DPE AGS Miami 02/7/2026 - PRE ALERTA do VOO de 3/7/2026 HAWB4065 - CANAL VERDE - ATZ Mayara 7/7/26 14:34</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
@@ -1246,35 +1264,35 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>396</v>
+        <v>313</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>BABE</t>
+          <t>BAMN</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>396260016520</t>
+          <t>313260018651</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1H75-21</t>
+          <t>AS5174D1210</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>PRESSURE REGULATOR</t>
+          <t>REDUCER, TUBE</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>2726</v>
+        <v>2732</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -1283,14 +1301,14 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>AIFP</t>
-        </is>
-      </c>
-      <c r="J9" s="1" t="n">
-        <v>46185</v>
-      </c>
-      <c r="K9" s="1" t="n">
-        <v>46185</v>
+          <t>IPLR</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>46204</v>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>46205</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -1300,31 +1318,31 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N9" s="1" t="n">
-        <v>46192</v>
+      <c r="N9" s="2" t="n">
+        <v>46216</v>
       </c>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="n">
-        <v>18</v>
+        <v>-5</v>
       </c>
       <c r="R9" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr">
         <is>
-          <t>Item retirado para atender o C-98 2731. Ramon 15/06/26.</t>
+          <t>Cedeu o item para o C-98 2738. Pedido será atendido pelo estoque FAB pedido n° 17874678 - Godoy 07/07/2026.</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>04 ea recolhidos para a V1, chegada dos itens dia 23/06/2026. Itens não tem oficina no Brasil, terá que ser feito Exchange rc 23/06 - MATERIAL ADQUIRIDO FORNECEDOR TEXTRON -WB0003073549 Inovice IJ17534800 DPE AGS Miami 29/6/2026 ate 10 30AM - AIR EXPORT HOUSE: 00004046 de 30/6/2026 Chegou no GIGRJ em 01/7/26 para Desembaraço - ATZ Marcio 3/7/2614:35</t>
+          <t>PEDIDO NO EPM - FOI SOLICITADO ATENDIMENTO COM ESTOUE FAB - CLA-02-07 - AWB 12744814663 DPE 07/07/2026</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
@@ -1350,26 +1368,26 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>313260018646</t>
+          <t>313260018653</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>011-00883-20</t>
+          <t>MS24392-10</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>RADAR GWX 68 WEATHER</t>
+          <t>NIPPLE,TUBE</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>2734</v>
+        <v>2732</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -1381,11 +1399,11 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J10" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="K10" s="1" t="n">
-        <v>46203</v>
+      <c r="J10" s="2" t="n">
+        <v>46204</v>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>46205</v>
       </c>
       <c r="L10" t="n">
         <v>1</v>
@@ -1395,35 +1413,31 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N10" s="1" t="n">
-        <v>46214</v>
+      <c r="N10" s="2" t="n">
+        <v>46216</v>
       </c>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="n">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="R10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="T10" t="inlineStr">
-        <is>
           <t>Sim</t>
         </is>
       </c>
+      <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr">
         <is>
-          <t>Retirado para atender a Anv 2740 - Godoy 30/06/26.</t>
+          <t>Cedeu o item para o C-98 2738. Pedido será atendido pelo estoque FAB pedido n° 17875036 - Godoy 07/07/2026.</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Efetuada a Compra em SP na Jet Avionics, aguardando confirmar unidade em estoque para liberação do item para a Veeone 01/7/2026 14:15 Marcio - DECLINADO pela JET AVIONICS, colocado Pedido TEXTRON Confirmation Number: WB0003077522 de 01/7/2026 Invoice IJ17546081 as 15:08PM Previsao DPE AGS Miami 02/7/2026 - PRE ALERTA do VOO de 3/7/2026 aguardando chegada no GIGRJ - ATZ Marcio 3/7/26 14:31</t>
+          <t>PEDIDO NO EPM - FOI SOLICITADO ATENDIMENTO COM ESTOUE FAB - CLA-02-07 - AWB 12744814663 DPE 07/07/2026</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
@@ -1440,35 +1454,35 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BAMN</t>
+          <t>BABR</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>313260018651</t>
+          <t>329260019179</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>AS5174D1210</t>
+          <t>066-3046-07</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>REDUCER, TUBE</t>
+          <t>CONTROL,INDICATOR</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>R</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>2732</v>
+        <v>2721</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -1477,15 +1491,15 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>IPLR</t>
-        </is>
-      </c>
-      <c r="J11" s="1" t="n">
-        <v>46204</v>
-      </c>
-      <c r="K11" s="1" t="n">
+          <t>AIFP</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="n">
         <v>46205</v>
       </c>
+      <c r="K11" s="2" t="n">
+        <v>46206</v>
+      </c>
       <c r="L11" t="n">
         <v>1</v>
       </c>
@@ -1494,31 +1508,31 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N11" s="1" t="n">
-        <v>46216</v>
+      <c r="N11" s="2" t="n">
+        <v>46213</v>
       </c>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="n">
-        <v>-6</v>
+        <v>-2</v>
       </c>
       <c r="R11" t="n">
         <v>5</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr">
         <is>
-          <t>Cedeu o item para o C-98 2738. Pedido será atendido pelo estoque FAB pedido n° 17874678 - Godoy 07/07/2026.</t>
+          <t>Recibo não se encontra na Pasta do DRIVE. Godoy 08/07/2026.</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>PEDIDO NO EPM - FOI SOLICITADO ATENDIMENTO COM ESTOUE FAB - CLA-02-07</t>
+          <t>Item estara disponivel no RJ na oficina para coleta dia 6/7 apos as 14 horas ATZ Marcio 3/7/ 14:25PM/ MATERIAL EM TRANSITO- RECIBO 548/FAB/26- AWB 12745474752 DPE 08/07 - Atlz Lucas- JPA (07/07)</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
@@ -1535,26 +1549,26 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>BAMN</t>
+          <t>BABR</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>313260018652</t>
+          <t>329260019180</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>24540-100</t>
+          <t>C145-00-46</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>COUPLING,CLAMP,GROOV</t>
+          <t>TRANSMISSION ASSY</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1563,23 +1577,23 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>2732</v>
+        <v>2709</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Providência tomada</t>
+          <t>Aguardando solução</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>IPLR</t>
-        </is>
-      </c>
-      <c r="J12" s="1" t="n">
-        <v>46204</v>
-      </c>
-      <c r="K12" s="1" t="n">
-        <v>46205</v>
+          <t>AIFP</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>46210</v>
       </c>
       <c r="L12" t="n">
         <v>1</v>
@@ -1589,8 +1603,8 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N12" s="1" t="n">
-        <v>46216</v>
+      <c r="N12" s="2" t="n">
+        <v>46217</v>
       </c>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
@@ -1598,7 +1612,7 @@
         <v>-6</v>
       </c>
       <c r="R12" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -1606,14 +1620,10 @@
         </is>
       </c>
       <c r="T12" t="inlineStr"/>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>Cedeu o item para o C-98 2738</t>
-        </is>
-      </c>
+      <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Colocado pedido fornecedor nacional. Previsão de entrega V1 Campinas 03/07</t>
+          <t>Colocado pedido AOG Textron WB0003081885 - previsão de entrega em Miami 08/07</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
@@ -1630,26 +1640,26 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BAMN</t>
+          <t>BABR</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>313260018653</t>
+          <t>329260019181</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>MS24392-10</t>
+          <t>C145-00-46</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>NIPPLE,TUBE</t>
+          <t>TRANSMISSION ASSY</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1658,23 +1668,23 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>2732</v>
+        <v>2721</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Providência tomada</t>
+          <t>Aguardando solução</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>IPLR</t>
-        </is>
-      </c>
-      <c r="J13" s="1" t="n">
-        <v>46204</v>
-      </c>
-      <c r="K13" s="1" t="n">
-        <v>46205</v>
+          <t>AIFP</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="K13" s="2" t="n">
+        <v>46210</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1684,8 +1694,8 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N13" s="1" t="n">
-        <v>46216</v>
+      <c r="N13" s="2" t="n">
+        <v>46217</v>
       </c>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
@@ -1693,22 +1703,18 @@
         <v>-6</v>
       </c>
       <c r="R13" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="T13" t="inlineStr"/>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>Cedeu o item para o C-98 2738. Pedido será atendido pelo estoque FAB pedido n° 17875036 - Godoy 07/07/2026.</t>
-        </is>
-      </c>
+      <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr">
         <is>
-          <t>PEDIDO NO EPM - FOI SOLICITADO ATENDIMENTO COM ESTOUE FAB - CLA-02-07</t>
+          <t>Colocado pedido AOG Textron WB0003081885 - previsão de entrega em Miami 08/07</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
@@ -1725,51 +1731,51 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BABR</t>
+          <t>BANT</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>329260019179</t>
+          <t>685260012303</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>066-3046-07</t>
+          <t>065-0065-01</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CONTROL,INDICATOR</t>
+          <t>SELECTOR ALT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>T</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>2721</v>
+        <v>2719</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Providência tomada</t>
+          <t>Aguardando solução</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>AIFP</t>
-        </is>
-      </c>
-      <c r="J14" s="1" t="n">
-        <v>46205</v>
-      </c>
-      <c r="K14" s="1" t="n">
-        <v>46206</v>
+          <t>ANCE</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="K14" s="2" t="n">
+        <v>46210</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
@@ -1779,16 +1785,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N14" s="1" t="n">
-        <v>46213</v>
+      <c r="N14" s="2" t="n">
+        <v>46241</v>
       </c>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="n">
-        <v>-3</v>
+        <v>-30</v>
       </c>
       <c r="R14" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
@@ -1797,11 +1803,7 @@
       </c>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>Item estara disponivel no RJ na oficina para coleta dia 6/7 apos as 14 horas ATZ Marcio 3/7/ 14:25PM</t>
-        </is>
-      </c>
+      <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr">
         <is>
           <t>VEE ONE</t>
@@ -1816,35 +1818,35 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>329</v>
+        <v>419</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>BABR</t>
+          <t>CLA</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>329260019180</t>
+          <t>419260000556</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>C145-00-46</t>
+          <t>066-3046-07</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>TRANSMISSION ASSY</t>
+          <t>CONTROL,INDICATOR</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>R</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>2709</v>
+        <v>2723</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1856,12 +1858,12 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J15" s="1" t="n">
-        <v>46209</v>
-      </c>
-      <c r="K15" s="1" t="n">
+      <c r="J15" s="2" t="n">
         <v>46210</v>
       </c>
+      <c r="K15" s="2" t="n">
+        <v>46211</v>
+      </c>
       <c r="L15" t="n">
         <v>1</v>
       </c>
@@ -1870,8 +1872,8 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N15" s="1" t="n">
-        <v>46217</v>
+      <c r="N15" s="2" t="n">
+        <v>46218</v>
       </c>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
@@ -1903,35 +1905,35 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>329</v>
+        <v>396</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>BABR</t>
+          <t>BABE</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>329260019181</t>
+          <t>396260016563</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>C145-00-46</t>
+          <t>3244809-4</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>TRANSMISSION ASSY</t>
+          <t>FUEL CONTROL,MAIN,TU</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>R</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>2721</v>
+        <v>2733</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1940,14 +1942,14 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>AIFP</t>
-        </is>
-      </c>
-      <c r="J16" s="1" t="n">
-        <v>46209</v>
-      </c>
-      <c r="K16" s="1" t="n">
-        <v>46210</v>
+          <t>IPLR</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="K16" s="2" t="n">
+        <v>46211</v>
       </c>
       <c r="L16" t="n">
         <v>1</v>
@@ -1957,13 +1959,13 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N16" s="1" t="n">
-        <v>46217</v>
+      <c r="N16" s="2" t="n">
+        <v>46222</v>
       </c>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="n">
-        <v>-7</v>
+        <v>-11</v>
       </c>
       <c r="R16" t="n">
         <v>0</v>
@@ -1985,93 +1987,6 @@
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="inlineStr"/>
       <c r="AA16" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>685</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>BANT</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>685260012303</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>065-0065-01</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>SELECTOR ALT</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="G17" t="n">
-        <v>2719</v>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Aguardando solução</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>ANCE</t>
-        </is>
-      </c>
-      <c r="J17" s="1" t="n">
-        <v>46210</v>
-      </c>
-      <c r="K17" s="1" t="n">
-        <v>46210</v>
-      </c>
-      <c r="L17" t="n">
-        <v>1</v>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>EA</t>
-        </is>
-      </c>
-      <c r="N17" s="1" t="n">
-        <v>46241</v>
-      </c>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="n">
-        <v>-31</v>
-      </c>
-      <c r="R17" t="n">
-        <v>0</v>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr">
-        <is>
-          <t>VEE ONE</t>
-        </is>
-      </c>
-      <c r="X17" t="inlineStr"/>
-      <c r="Y17" t="inlineStr"/>
-      <c r="Z17" t="inlineStr"/>
-      <c r="AA17" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Cômputo Mensal recalcula sozinho junto com Emergências
A pedido do Wallace: extrair_emergencias.atualizar_do_drive() agora também
chama calcular_computo_mensal.calcular_mes() pro mês atual, logo depois de
regenerar o histórico completo — a matriz da Pré-RNA (aba 1.2) fica sempre
em dia sem precisar clicar em "Recalcular" (o botão continua existindo
pra rodar na hora, se quiser). Mesma cadência de sempre (seg-sex ~12h,
GitHub e Mac).

Reparáveis fica manual por decisão do Wallace (tem atualizar_do_drive()
pronto, mas sem agendamento — não mexido nessa sessão).
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -631,10 +631,10 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="R2" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -726,10 +726,10 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="R3" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -823,10 +823,10 @@
       </c>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="n">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R4" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -922,10 +922,10 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="R5" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -1017,10 +1017,10 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1116,10 +1116,10 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="n">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1211,10 +1211,10 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="n">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1306,10 +1306,10 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -1401,10 +1401,10 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="n">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
@@ -1492,10 +1492,10 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="n">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
@@ -1583,10 +1583,10 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="n">
-        <v>-30</v>
+        <v>-29</v>
       </c>
       <c r="R12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -1670,10 +1670,10 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
@@ -1761,10 +1761,10 @@
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática: emergencias (09/07/2026 15:31)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA14"/>
+  <dimension ref="A1:AA15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1056,35 +1056,35 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BAMN</t>
+          <t>BABR</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>313260018651</t>
+          <t>329260019179</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>AS5174D1210</t>
+          <t>066-3046-07</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>REDUCER, TUBE</t>
+          <t>CONTROL,INDICATOR</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>R</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>2732</v>
+        <v>2721</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -1093,14 +1093,14 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>IPLR</t>
+          <t>AIFP</t>
         </is>
       </c>
       <c r="J7" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
@@ -1111,30 +1111,30 @@
         </is>
       </c>
       <c r="N7" s="2" t="n">
-        <v>46216</v>
+        <v>46213</v>
       </c>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="n">
-        <v>-4</v>
+        <v>-1</v>
       </c>
       <c r="R7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr">
         <is>
-          <t>Cedeu o item para o C-98 2738. Pedido será atendido pelo estoque FAB pedido n° 17874678 - Godoy 07/07/2026.</t>
+          <t>Recibo não se encontra na Pasta do DRIVE. Godoy 08/07/2026.</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>PEDIDO NO EPM - FOI SOLICITADO ATENDIMENTO COM ESTOUE FAB - CLA-02-07 - AWB 12744814663 DPE 07/07/2026</t>
+          <t>Item estara disponivel no RJ na oficina para coleta dia 6/7 apos as 14 horas ATZ Marcio 3/7/ 14:25PM/ MATERIAL EM TRANSITO- RECIBO 548/FAB/26- AWB 12745474752 DPE 08/07 - Atlz Lucas- JPA (07/07)</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
@@ -1151,26 +1151,26 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BAMN</t>
+          <t>BABR</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>313260018653</t>
+          <t>329260019180</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MS24392-10</t>
+          <t>C145-00-46</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>NIPPLE,TUBE</t>
+          <t>TRANSMISSION ASSY</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1179,7 +1179,7 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>2732</v>
+        <v>2709</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -1188,14 +1188,14 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>IPLR</t>
+          <t>AIFP</t>
         </is>
       </c>
       <c r="J8" s="2" t="n">
-        <v>46204</v>
+        <v>46209</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>46205</v>
+        <v>46210</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
@@ -1206,30 +1206,26 @@
         </is>
       </c>
       <c r="N8" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="n">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="R8" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>Cedeu o item para o C-98 2738. Pedido será atendido pelo estoque FAB pedido n° 17875036 - Godoy 07/07/2026.</t>
-        </is>
-      </c>
+      <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
-          <t>PEDIDO NO EPM - FOI SOLICITADO ATENDIMENTO COM ESTOUE FAB - CLA-02-07 - AWB 12744814663 DPE 07/07/2026</t>
+          <t>Colocado pedido AOG Textron WB0003081885 - previsão de entrega em Miami 08/07</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
@@ -1255,22 +1251,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>329260019179</t>
+          <t>329260019181</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>066-3046-07</t>
+          <t>C145-00-46</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CONTROL,INDICATOR</t>
+          <t>TRANSMISSION ASSY</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -1287,10 +1283,10 @@
         </is>
       </c>
       <c r="J9" s="2" t="n">
-        <v>46205</v>
+        <v>46209</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>46206</v>
+        <v>46210</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -1301,15 +1297,15 @@
         </is>
       </c>
       <c r="N9" s="2" t="n">
-        <v>46213</v>
+        <v>46217</v>
       </c>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="n">
-        <v>-1</v>
+        <v>-5</v>
       </c>
       <c r="R9" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -1317,14 +1313,10 @@
         </is>
       </c>
       <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>Recibo não se encontra na Pasta do DRIVE. Godoy 08/07/2026.</t>
-        </is>
-      </c>
+      <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Item estara disponivel no RJ na oficina para coleta dia 6/7 apos as 14 horas ATZ Marcio 3/7/ 14:25PM/ MATERIAL EM TRANSITO- RECIBO 548/FAB/26- AWB 12745474752 DPE 08/07 - Atlz Lucas- JPA (07/07)</t>
+          <t>Colocado pedido AOG Textron WB0003081885 - previsão de entrega em Miami 08/07</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
@@ -1341,48 +1333,48 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>BABR</t>
+          <t>BANT</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>329260019180</t>
+          <t>685260012303</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>C145-00-46</t>
+          <t>065-0065-01</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>TRANSMISSION ASSY</t>
+          <t>SELECTOR ALT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>T</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>2709</v>
+        <v>2719</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Aguardando solução</t>
+          <t>Providência tomada</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>AIFP</t>
+          <t>ANCE</t>
         </is>
       </c>
       <c r="J10" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="K10" s="2" t="n">
         <v>46210</v>
@@ -1396,12 +1388,12 @@
         </is>
       </c>
       <c r="N10" s="2" t="n">
-        <v>46217</v>
+        <v>46241</v>
       </c>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="n">
-        <v>-5</v>
+        <v>-29</v>
       </c>
       <c r="R10" t="n">
         <v>2</v>
@@ -1413,11 +1405,7 @@
       </c>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>Colocado pedido AOG Textron WB0003081885 - previsão de entrega em Miami 08/07</t>
-        </is>
-      </c>
+      <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr">
         <is>
           <t>VEE ONE</t>
@@ -1432,39 +1420,39 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>329</v>
+        <v>419</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BABR</t>
+          <t>CLA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>329260019181</t>
+          <t>419260000556</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>C145-00-46</t>
+          <t>066-3046-07</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>TRANSMISSION ASSY</t>
+          <t>CONTROL,INDICATOR</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>R</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>2721</v>
+        <v>2723</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Aguardando solução</t>
+          <t>Providência tomada</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1473,10 +1461,10 @@
         </is>
       </c>
       <c r="J11" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="L11" t="n">
         <v>1</v>
@@ -1487,15 +1475,15 @@
         </is>
       </c>
       <c r="N11" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="n">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="R11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
@@ -1506,7 +1494,7 @@
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Colocado pedido AOG Textron WB0003081885 - previsão de entrega em Miami 08/07</t>
+          <t>MATERIAL EM TRANSITO - AWB 12745918331 dpe 11/07/2026 - atz rc 08/07/2026</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
@@ -1523,51 +1511,51 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>685</v>
+        <v>396</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>BANT</t>
+          <t>BABE</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>685260012303</t>
+          <t>396260016563</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>065-0065-01</t>
+          <t>3244809-4</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SELECTOR ALT</t>
+          <t>FUEL CONTROL,MAIN,TU</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>R</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>2719</v>
+        <v>2733</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Aguardando solução</t>
+          <t>Providência tomada</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>ANCE</t>
+          <t>IPLR</t>
         </is>
       </c>
       <c r="J12" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="L12" t="n">
         <v>1</v>
@@ -1578,15 +1566,15 @@
         </is>
       </c>
       <c r="N12" s="2" t="n">
-        <v>46241</v>
+        <v>46222</v>
       </c>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="n">
-        <v>-29</v>
+        <v>-10</v>
       </c>
       <c r="R12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -1610,26 +1598,26 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>419</v>
+        <v>396</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CLA</t>
+          <t>BABE</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>419260000556</t>
+          <t>396260016566</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>066-3046-07</t>
+          <t>060-0015-00</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CONTROL,INDICATOR</t>
+          <t>CONTROL,DIRECTIONAL,</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1638,7 +1626,7 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>2723</v>
+        <v>2726</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1651,10 +1639,10 @@
         </is>
       </c>
       <c r="J13" s="2" t="n">
-        <v>46210</v>
+        <v>46212</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1665,28 +1653,28 @@
         </is>
       </c>
       <c r="N13" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="n">
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="R13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="T13" t="inlineStr"/>
-      <c r="U13" t="inlineStr"/>
-      <c r="V13" t="inlineStr">
-        <is>
-          <t>MATERIAL EM TRANSITO - AWB 12745918331 dpe 11/07/2026 - atz rc 08/07/2026</t>
-        </is>
-      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Cedeu o item para o C-98 2721. Ramon 09/07/26.</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr">
         <is>
           <t>VEE ONE</t>
@@ -1701,26 +1689,26 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>396</v>
+        <v>419</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BABE</t>
+          <t>CLA</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>396260016563</t>
+          <t>419260000557</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>3244809-4</t>
+          <t>3244897-4</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>FUEL CONTROL,MAIN,TU</t>
+          <t>FUEL CONTROL UNIT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1729,7 +1717,7 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>2733</v>
+        <v>2723</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -1738,14 +1726,14 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>IPLR</t>
+          <t>AIFP</t>
         </is>
       </c>
       <c r="J14" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
@@ -1756,15 +1744,15 @@
         </is>
       </c>
       <c r="N14" s="2" t="n">
-        <v>46222</v>
+        <v>46219</v>
       </c>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="n">
-        <v>-10</v>
+        <v>-7</v>
       </c>
       <c r="R14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
@@ -1783,6 +1771,93 @@
       <c r="Y14" t="inlineStr"/>
       <c r="Z14" t="inlineStr"/>
       <c r="AA14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>685</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>BANT</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>685260012350</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>030-1094-58</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>CONNECTOR</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>2702</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Aguardando solução</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>ANCE</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="K15" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="L15" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="n">
+        <v>46243</v>
+      </c>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="n">
+        <v>-31</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>VEE ONE</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr"/>
+      <c r="Y15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr"/>
+      <c r="AA15" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (09/07/2026 23:47)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,137 +421,137 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>om_emg</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>om</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>numero_emergencia</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>categoria</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>matricula_aeronave</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>tpemg</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>data_abertura</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>data_info</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>quantidade</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>unidade_medida</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>prazo_entrega</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>dpe</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>atendido_cancelado</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>dias_atraso</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>dias_corridos</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>estoque</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>retirado_empresa_recibo_obrigatorio</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>obs_coordenadoria_fiscal</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>obs_vee_one</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>provedor</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>awb</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>prev_entrega</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>mensagem_operador</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>em_aberto</t>
         </is>
@@ -611,10 +599,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J2" s="2" t="n">
+      <c r="J2" s="1" t="n">
         <v>46076</v>
       </c>
-      <c r="K2" s="2" t="n">
+      <c r="K2" s="1" t="n">
         <v>46080</v>
       </c>
       <c r="L2" t="n">
@@ -625,7 +613,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N2" s="2" t="n">
+      <c r="N2" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="O2" t="inlineStr"/>
@@ -706,10 +694,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J3" s="2" t="n">
+      <c r="J3" s="1" t="n">
         <v>46184</v>
       </c>
-      <c r="K3" s="2" t="n">
+      <c r="K3" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="L3" t="n">
@@ -720,7 +708,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N3" s="2" t="n">
+      <c r="N3" s="1" t="n">
         <v>46196</v>
       </c>
       <c r="O3" t="inlineStr"/>
@@ -801,10 +789,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J4" s="2" t="n">
+      <c r="J4" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="K4" s="2" t="n">
+      <c r="K4" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="L4" t="n">
@@ -815,10 +803,10 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N4" s="2" t="n">
+      <c r="N4" s="1" t="n">
         <v>46216</v>
       </c>
-      <c r="O4" s="2" t="n">
+      <c r="O4" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -902,10 +890,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J5" s="2" t="n">
+      <c r="J5" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="K5" s="2" t="n">
+      <c r="K5" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="L5" t="n">
@@ -916,7 +904,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N5" s="2" t="n">
+      <c r="N5" s="1" t="n">
         <v>46192</v>
       </c>
       <c r="O5" t="inlineStr"/>
@@ -997,10 +985,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J6" s="2" t="n">
+      <c r="J6" s="1" t="n">
         <v>46199</v>
       </c>
-      <c r="K6" s="2" t="n">
+      <c r="K6" s="1" t="n">
         <v>46203</v>
       </c>
       <c r="L6" t="n">
@@ -1011,7 +999,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N6" s="2" t="n">
+      <c r="N6" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="O6" t="inlineStr"/>
@@ -1096,10 +1084,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="J7" s="1" t="n">
         <v>46205</v>
       </c>
-      <c r="K7" s="2" t="n">
+      <c r="K7" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="L7" t="n">
@@ -1110,7 +1098,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N7" s="2" t="n">
+      <c r="N7" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="O7" t="inlineStr"/>
@@ -1191,10 +1179,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J8" s="2" t="n">
+      <c r="J8" s="1" t="n">
         <v>46209</v>
       </c>
-      <c r="K8" s="2" t="n">
+      <c r="K8" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="L8" t="n">
@@ -1205,7 +1193,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N8" s="2" t="n">
+      <c r="N8" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="O8" t="inlineStr"/>
@@ -1282,10 +1270,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J9" s="2" t="n">
+      <c r="J9" s="1" t="n">
         <v>46209</v>
       </c>
-      <c r="K9" s="2" t="n">
+      <c r="K9" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="L9" t="n">
@@ -1296,7 +1284,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N9" s="2" t="n">
+      <c r="N9" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="O9" t="inlineStr"/>
@@ -1373,10 +1361,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J10" s="2" t="n">
+      <c r="J10" s="1" t="n">
         <v>46210</v>
       </c>
-      <c r="K10" s="2" t="n">
+      <c r="K10" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="L10" t="n">
@@ -1387,7 +1375,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N10" s="2" t="n">
+      <c r="N10" s="1" t="n">
         <v>46241</v>
       </c>
       <c r="O10" t="inlineStr"/>
@@ -1460,10 +1448,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J11" s="2" t="n">
+      <c r="J11" s="1" t="n">
         <v>46210</v>
       </c>
-      <c r="K11" s="2" t="n">
+      <c r="K11" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="L11" t="n">
@@ -1474,7 +1462,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N11" s="2" t="n">
+      <c r="N11" s="1" t="n">
         <v>46218</v>
       </c>
       <c r="O11" t="inlineStr"/>
@@ -1551,10 +1539,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J12" s="2" t="n">
+      <c r="J12" s="1" t="n">
         <v>46211</v>
       </c>
-      <c r="K12" s="2" t="n">
+      <c r="K12" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="L12" t="n">
@@ -1565,7 +1553,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N12" s="2" t="n">
+      <c r="N12" s="1" t="n">
         <v>46222</v>
       </c>
       <c r="O12" t="inlineStr"/>
@@ -1638,10 +1626,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J13" s="2" t="n">
+      <c r="J13" s="1" t="n">
         <v>46212</v>
       </c>
-      <c r="K13" s="2" t="n">
+      <c r="K13" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="L13" t="n">
@@ -1652,7 +1640,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N13" s="2" t="n">
+      <c r="N13" s="1" t="n">
         <v>46219</v>
       </c>
       <c r="O13" t="inlineStr"/>
@@ -1729,10 +1717,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J14" s="2" t="n">
+      <c r="J14" s="1" t="n">
         <v>46211</v>
       </c>
-      <c r="K14" s="2" t="n">
+      <c r="K14" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="L14" t="n">
@@ -1743,7 +1731,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N14" s="2" t="n">
+      <c r="N14" s="1" t="n">
         <v>46219</v>
       </c>
       <c r="O14" t="inlineStr"/>
@@ -1816,10 +1804,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J15" s="2" t="n">
+      <c r="J15" s="1" t="n">
         <v>46212</v>
       </c>
-      <c r="K15" s="2" t="n">
+      <c r="K15" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="L15" t="n">
@@ -1830,7 +1818,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N15" s="2" t="n">
+      <c r="N15" s="1" t="n">
         <v>46243</v>
       </c>
       <c r="O15" t="inlineStr"/>

</xml_diff>

<commit_message>
Atualização automática: emergencias (10/07/2026 10:10)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -421,137 +433,137 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>om_emg</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>om</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>numero_emergencia</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>categoria</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>matricula_aeronave</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>tpemg</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>data_abertura</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>data_info</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>quantidade</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>unidade_medida</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>prazo_entrega</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>dpe</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>atendido_cancelado</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>dias_atraso</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>dias_corridos</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>estoque</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>retirado_empresa_recibo_obrigatorio</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>obs_coordenadoria_fiscal</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>obs_vee_one</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>provedor</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>awb</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>prev_entrega</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>mensagem_operador</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>em_aberto</t>
         </is>
@@ -599,10 +611,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J2" s="1" t="n">
+      <c r="J2" s="2" t="n">
         <v>46076</v>
       </c>
-      <c r="K2" s="1" t="n">
+      <c r="K2" s="2" t="n">
         <v>46080</v>
       </c>
       <c r="L2" t="n">
@@ -613,16 +625,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N2" s="1" t="n">
+      <c r="N2" s="2" t="n">
         <v>46111</v>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="R2" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -694,10 +706,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J3" s="1" t="n">
+      <c r="J3" s="2" t="n">
         <v>46184</v>
       </c>
-      <c r="K3" s="1" t="n">
+      <c r="K3" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="L3" t="n">
@@ -708,16 +720,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N3" s="1" t="n">
+      <c r="N3" s="2" t="n">
         <v>46196</v>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="R3" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -789,10 +801,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J4" s="1" t="n">
+      <c r="J4" s="2" t="n">
         <v>46185</v>
       </c>
-      <c r="K4" s="1" t="n">
+      <c r="K4" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="L4" t="n">
@@ -803,18 +815,18 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N4" s="1" t="n">
+      <c r="N4" s="2" t="n">
         <v>46216</v>
       </c>
-      <c r="O4" s="1" t="n">
+      <c r="O4" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R4" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -890,10 +902,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J5" s="1" t="n">
+      <c r="J5" s="2" t="n">
         <v>46185</v>
       </c>
-      <c r="K5" s="1" t="n">
+      <c r="K5" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="L5" t="n">
@@ -904,16 +916,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N5" s="1" t="n">
+      <c r="N5" s="2" t="n">
         <v>46192</v>
       </c>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="R5" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -928,7 +940,7 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>04 ea recolhidos para a V1, chegada dos itens dia 23/06/2026. Itens não tem oficina no Brasil, terá que ser feito Exchange rc 23/06 - MATERIAL ADQUIRIDO FORNECEDOR TEXTRON -WB0003073549 Inovice IJ17534800 DPE AGS Miami 29/6/2026 ate 10 30AM - AIR EXPORT HOUSE: 00004046 de 30/6/2026 Chegou no GIGRJ em 01/7/26 para Desembaraço - ATZ Marcio 3/7/2614:35</t>
+          <t>"04 ea recolhidos para a V1, chegada dos itens dia 23/06/2026. Itens não tem oficina no Brasil, terá que ser feito Exchange rc 23/06 - MATERIAL ADQUIRIDO FORNECEDOR TEXTRON -WB0003073549 Inovice IJ17534800 DPE AGS Miami 29/6/2026 ate 10 30AM - AIR EXPORT HOUSE: 00004046 de 30/6/2026 Chegou no GIGRJ em 01/7/26 para Desembaraço - ATZ Marcio 3/7/26 CANAL VERDE EM 7/7/26 entregue V1 em 8/7/26 ATZ Marcio 9/7/26"</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
@@ -985,10 +997,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J6" s="1" t="n">
+      <c r="J6" s="2" t="n">
         <v>46199</v>
       </c>
-      <c r="K6" s="1" t="n">
+      <c r="K6" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="L6" t="n">
@@ -999,16 +1011,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N6" s="1" t="n">
+      <c r="N6" s="2" t="n">
         <v>46214</v>
       </c>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1027,7 +1039,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Efetuada a Compra em SP na Jet Avionics, aguardando confirmar unidade em estoque para liberação do item para a Veeone 01/7/2026 14:15 Marcio - DECLINADO pela JET AVIONICS, colocado Pedido TEXTRON Confirmation Number: WB0003077522 de 01/7/2026 Invoice IJ17546081 as 15:08PM Previsao DPE AGS Miami 02/7/2026 - PRE ALERTA do VOO de 3/7/2026 HAWB4065 - CANAL VERDE - ATZ Mayara 7/7/26 14:34 (MATERIAL EM SEPARAÇÃO - SUP V1 JPA) Atlz Lucas 08/07 14:01</t>
+          <t>Efetuada a Compra em SP na Jet Avionics, aguardando confirmar unidade em estoque para liberação do item para a Veeone 01/7/2026 14:15 Marcio - DECLINADO pela JET AVIONICS, colocado Pedido TEXTRON Confirmation Number: WB0003077522 de 01/7/2026 Invoice IJ17546081 as 15:08PM Previsao DPE AGS Miami 02/7/2026 - PRE ALERTA do VOO de 3/7/2026 HAWB4065 - CANAL VERDE - ATZ Mayara 7/7/26 14:34 (MATERIAL EM SEPARAÇÃO - SUP V1 JPA) Atlz Lucas 08/07 14:01 - MATERIAL EM TRANSITO - RECIBO 556/FAB/26 - AWB 12745953832 DPE 14/07/2026</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
@@ -1084,10 +1096,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J7" s="1" t="n">
+      <c r="J7" s="2" t="n">
         <v>46205</v>
       </c>
-      <c r="K7" s="1" t="n">
+      <c r="K7" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="L7" t="n">
@@ -1098,16 +1110,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N7" s="1" t="n">
+      <c r="N7" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1122,7 +1134,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Item estara disponivel no RJ na oficina para coleta dia 6/7 apos as 14 horas ATZ Marcio 3/7/ 14:25PM/ MATERIAL EM TRANSITO- RECIBO 548/FAB/26- AWB 12745474752 DPE 08/07 - Atlz Lucas- JPA (07/07)</t>
+          <t>Item estara disponivel no RJ na oficina para coleta dia 6/7 apos as 14 horas ATZ Marcio 3/7/ 14:25PM/ MATERIAL EM TRANSITO- RECIBO 548/FAB/26- AWB 12745474752 DPE 08/07 - Atlz Lucas- JPA (07/07) - MATERIAL DISPONIVEL PRA RETIRADA DIA 09/07/2026 ATZ RC</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
@@ -1179,10 +1191,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J8" s="1" t="n">
+      <c r="J8" s="2" t="n">
         <v>46209</v>
       </c>
-      <c r="K8" s="1" t="n">
+      <c r="K8" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="L8" t="n">
@@ -1193,16 +1205,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N8" s="1" t="n">
+      <c r="N8" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="n">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1213,7 +1225,7 @@
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Colocado pedido AOG Textron WB0003081885 - previsão de entrega em Miami 08/07</t>
+          <t>Colocado pedido AOG Textron IJ17557538 - previsão de entrega em Miami 08/07. Previsão de chegada GIG 09/07 - MATERIAL EM TRANSITO - RECIBO 551/FAB/26 - ENVIADO PN COMPLETO PARA SANAR A EMERGENCIA DO 2709, ENVIADO MODAL TERRESTRE, DPE 09/07/2026</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
@@ -1270,10 +1282,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J9" s="1" t="n">
+      <c r="J9" s="2" t="n">
         <v>46209</v>
       </c>
-      <c r="K9" s="1" t="n">
+      <c r="K9" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="L9" t="n">
@@ -1284,16 +1296,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N9" s="1" t="n">
+      <c r="N9" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="n">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -1304,7 +1316,7 @@
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Colocado pedido AOG Textron WB0003081885 - previsão de entrega em Miami 08/07</t>
+          <t>Colocado pedido AOG Textron IJ17557538 - previsão de entrega em Miami 08/07. Previsão de chegada GIG 09/07 (voo 4093)</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
@@ -1361,10 +1373,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J10" s="1" t="n">
+      <c r="J10" s="2" t="n">
         <v>46210</v>
       </c>
-      <c r="K10" s="1" t="n">
+      <c r="K10" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="L10" t="n">
@@ -1375,16 +1387,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N10" s="1" t="n">
+      <c r="N10" s="2" t="n">
         <v>46241</v>
       </c>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="n">
-        <v>-29</v>
+        <v>-28</v>
       </c>
       <c r="R10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
@@ -1393,7 +1405,11 @@
       </c>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr"/>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Aguardando orçamento oficina BH ATZ Marcio 9/7/26 - DPE 17/07/2026(REZ 09/07/26)</t>
+        </is>
+      </c>
       <c r="W10" t="inlineStr">
         <is>
           <t>VEE ONE</t>
@@ -1448,10 +1464,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J11" s="1" t="n">
+      <c r="J11" s="2" t="n">
         <v>46210</v>
       </c>
-      <c r="K11" s="1" t="n">
+      <c r="K11" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="L11" t="n">
@@ -1462,16 +1478,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N11" s="1" t="n">
+      <c r="N11" s="2" t="n">
         <v>46218</v>
       </c>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="n">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
@@ -1539,10 +1555,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J12" s="1" t="n">
+      <c r="J12" s="2" t="n">
         <v>46211</v>
       </c>
-      <c r="K12" s="1" t="n">
+      <c r="K12" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="L12" t="n">
@@ -1553,16 +1569,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N12" s="1" t="n">
+      <c r="N12" s="2" t="n">
         <v>46222</v>
       </c>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="n">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="R12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -1571,7 +1587,11 @@
       </c>
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr"/>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>Aguardando APROVAÇÃO PO 793/JPA/2026 em referencia ao orçamento 0274/26 - Prazo ofocina 15 dias após aprovação. ATZ Marcio 9/7/26 14:50</t>
+        </is>
+      </c>
       <c r="W12" t="inlineStr">
         <is>
           <t>VEE ONE</t>
@@ -1626,10 +1646,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J13" s="1" t="n">
+      <c r="J13" s="2" t="n">
         <v>46212</v>
       </c>
-      <c r="K13" s="1" t="n">
+      <c r="K13" s="2" t="n">
         <v>46212</v>
       </c>
       <c r="L13" t="n">
@@ -1640,16 +1660,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N13" s="1" t="n">
+      <c r="N13" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
@@ -1662,7 +1682,11 @@
           <t>Cedeu o item para o C-98 2721. Ramon 09/07/26.</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr"/>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>Foi solicitado, via Email, o atendimento com estoque FAB - CLA -09-07-26</t>
+        </is>
+      </c>
       <c r="W13" t="inlineStr">
         <is>
           <t>VEE ONE</t>
@@ -1717,10 +1741,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J14" s="1" t="n">
+      <c r="J14" s="2" t="n">
         <v>46211</v>
       </c>
-      <c r="K14" s="1" t="n">
+      <c r="K14" s="2" t="n">
         <v>46212</v>
       </c>
       <c r="L14" t="n">
@@ -1731,16 +1755,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N14" s="1" t="n">
+      <c r="N14" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
@@ -1749,7 +1773,11 @@
       </c>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr"/>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>Aguardando o retorno dos subcomponentes removidos da unidade para ser enviado a oficiana para aplicação na unidade Prazo apos aprovação 10 dias ATZ Marcio 9/7/26 14 53</t>
+        </is>
+      </c>
       <c r="W14" t="inlineStr">
         <is>
           <t>VEE ONE</t>
@@ -1804,10 +1832,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J15" s="1" t="n">
+      <c r="J15" s="2" t="n">
         <v>46212</v>
       </c>
-      <c r="K15" s="1" t="n">
+      <c r="K15" s="2" t="n">
         <v>46212</v>
       </c>
       <c r="L15" t="n">
@@ -1818,16 +1846,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N15" s="1" t="n">
+      <c r="N15" s="2" t="n">
         <v>46243</v>
       </c>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="n">
-        <v>-31</v>
+        <v>-30</v>
       </c>
       <c r="R15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
@@ -1836,7 +1864,11 @@
       </c>
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr"/>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>Pedido no EPm nº E-C98-26056 - CLA -09-07-26</t>
+        </is>
+      </c>
       <c r="W15" t="inlineStr">
         <is>
           <t>VEE ONE</t>

</xml_diff>

<commit_message>
Atualização automática: emergencias (10/07/2026 14:00)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -1638,7 +1638,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Aguardando solução</t>
+          <t>Providência tomada</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Aguardando solução</t>
+          <t>Providência tomada</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1824,7 +1824,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Aguardando solução</t>
+          <t>Providência tomada</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">

</xml_diff>

<commit_message>
Atualização automática: emergencias (10/07/2026 17:31)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,137 +421,137 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>om_emg</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>om</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>numero_emergencia</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>categoria</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>matricula_aeronave</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>tpemg</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>data_abertura</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>data_info</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>quantidade</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>unidade_medida</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>prazo_entrega</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>dpe</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>atendido_cancelado</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>dias_atraso</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>dias_corridos</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>estoque</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>retirado_empresa_recibo_obrigatorio</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>obs_coordenadoria_fiscal</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>obs_vee_one</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>provedor</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>awb</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>prev_entrega</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>mensagem_operador</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>em_aberto</t>
         </is>
@@ -611,10 +599,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J2" s="2" t="n">
+      <c r="J2" s="1" t="n">
         <v>46076</v>
       </c>
-      <c r="K2" s="2" t="n">
+      <c r="K2" s="1" t="n">
         <v>46080</v>
       </c>
       <c r="L2" t="n">
@@ -625,7 +613,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N2" s="2" t="n">
+      <c r="N2" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="O2" t="inlineStr"/>
@@ -706,10 +694,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J3" s="2" t="n">
+      <c r="J3" s="1" t="n">
         <v>46184</v>
       </c>
-      <c r="K3" s="2" t="n">
+      <c r="K3" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="L3" t="n">
@@ -720,7 +708,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N3" s="2" t="n">
+      <c r="N3" s="1" t="n">
         <v>46196</v>
       </c>
       <c r="O3" t="inlineStr"/>
@@ -801,10 +789,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J4" s="2" t="n">
+      <c r="J4" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="K4" s="2" t="n">
+      <c r="K4" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="L4" t="n">
@@ -815,10 +803,10 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N4" s="2" t="n">
+      <c r="N4" s="1" t="n">
         <v>46216</v>
       </c>
-      <c r="O4" s="2" t="n">
+      <c r="O4" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -902,10 +890,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J5" s="2" t="n">
+      <c r="J5" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="K5" s="2" t="n">
+      <c r="K5" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="L5" t="n">
@@ -916,7 +904,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N5" s="2" t="n">
+      <c r="N5" s="1" t="n">
         <v>46192</v>
       </c>
       <c r="O5" t="inlineStr"/>
@@ -997,10 +985,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J6" s="2" t="n">
+      <c r="J6" s="1" t="n">
         <v>46199</v>
       </c>
-      <c r="K6" s="2" t="n">
+      <c r="K6" s="1" t="n">
         <v>46203</v>
       </c>
       <c r="L6" t="n">
@@ -1011,7 +999,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N6" s="2" t="n">
+      <c r="N6" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="O6" t="inlineStr"/>
@@ -1096,10 +1084,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="J7" s="1" t="n">
         <v>46205</v>
       </c>
-      <c r="K7" s="2" t="n">
+      <c r="K7" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="L7" t="n">
@@ -1110,7 +1098,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N7" s="2" t="n">
+      <c r="N7" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="O7" t="inlineStr"/>
@@ -1191,10 +1179,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J8" s="2" t="n">
+      <c r="J8" s="1" t="n">
         <v>46209</v>
       </c>
-      <c r="K8" s="2" t="n">
+      <c r="K8" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="L8" t="n">
@@ -1205,7 +1193,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N8" s="2" t="n">
+      <c r="N8" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="O8" t="inlineStr"/>
@@ -1282,10 +1270,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J9" s="2" t="n">
+      <c r="J9" s="1" t="n">
         <v>46209</v>
       </c>
-      <c r="K9" s="2" t="n">
+      <c r="K9" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="L9" t="n">
@@ -1296,7 +1284,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N9" s="2" t="n">
+      <c r="N9" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="O9" t="inlineStr"/>
@@ -1373,10 +1361,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J10" s="2" t="n">
+      <c r="J10" s="1" t="n">
         <v>46210</v>
       </c>
-      <c r="K10" s="2" t="n">
+      <c r="K10" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="L10" t="n">
@@ -1387,7 +1375,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N10" s="2" t="n">
+      <c r="N10" s="1" t="n">
         <v>46241</v>
       </c>
       <c r="O10" t="inlineStr"/>
@@ -1464,10 +1452,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J11" s="2" t="n">
+      <c r="J11" s="1" t="n">
         <v>46210</v>
       </c>
-      <c r="K11" s="2" t="n">
+      <c r="K11" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="L11" t="n">
@@ -1478,7 +1466,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N11" s="2" t="n">
+      <c r="N11" s="1" t="n">
         <v>46218</v>
       </c>
       <c r="O11" t="inlineStr"/>
@@ -1555,10 +1543,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J12" s="2" t="n">
+      <c r="J12" s="1" t="n">
         <v>46211</v>
       </c>
-      <c r="K12" s="2" t="n">
+      <c r="K12" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="L12" t="n">
@@ -1569,7 +1557,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N12" s="2" t="n">
+      <c r="N12" s="1" t="n">
         <v>46222</v>
       </c>
       <c r="O12" t="inlineStr"/>
@@ -1646,10 +1634,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J13" s="2" t="n">
+      <c r="J13" s="1" t="n">
         <v>46212</v>
       </c>
-      <c r="K13" s="2" t="n">
+      <c r="K13" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="L13" t="n">
@@ -1660,7 +1648,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N13" s="2" t="n">
+      <c r="N13" s="1" t="n">
         <v>46219</v>
       </c>
       <c r="O13" t="inlineStr"/>
@@ -1741,10 +1729,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J14" s="2" t="n">
+      <c r="J14" s="1" t="n">
         <v>46211</v>
       </c>
-      <c r="K14" s="2" t="n">
+      <c r="K14" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="L14" t="n">
@@ -1755,7 +1743,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N14" s="2" t="n">
+      <c r="N14" s="1" t="n">
         <v>46219</v>
       </c>
       <c r="O14" t="inlineStr"/>
@@ -1832,10 +1820,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J15" s="2" t="n">
+      <c r="J15" s="1" t="n">
         <v>46212</v>
       </c>
-      <c r="K15" s="2" t="n">
+      <c r="K15" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="L15" t="n">
@@ -1846,7 +1834,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N15" s="2" t="n">
+      <c r="N15" s="1" t="n">
         <v>46243</v>
       </c>
       <c r="O15" t="inlineStr"/>

</xml_diff>

<commit_message>
Atualização automática: emergencias (10/07/2026 16:00)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -421,137 +433,137 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>om_emg</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>om</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>numero_emergencia</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>categoria</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>matricula_aeronave</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>tpemg</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>data_abertura</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>data_info</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>quantidade</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>unidade_medida</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>prazo_entrega</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>dpe</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>atendido_cancelado</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>dias_atraso</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>dias_corridos</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>estoque</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>retirado_empresa_recibo_obrigatorio</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>obs_coordenadoria_fiscal</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>obs_vee_one</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>provedor</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>awb</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>prev_entrega</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>mensagem_operador</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>em_aberto</t>
         </is>
@@ -599,10 +611,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J2" s="1" t="n">
+      <c r="J2" s="2" t="n">
         <v>46076</v>
       </c>
-      <c r="K2" s="1" t="n">
+      <c r="K2" s="2" t="n">
         <v>46080</v>
       </c>
       <c r="L2" t="n">
@@ -613,7 +625,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N2" s="1" t="n">
+      <c r="N2" s="2" t="n">
         <v>46111</v>
       </c>
       <c r="O2" t="inlineStr"/>
@@ -694,10 +706,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J3" s="1" t="n">
+      <c r="J3" s="2" t="n">
         <v>46184</v>
       </c>
-      <c r="K3" s="1" t="n">
+      <c r="K3" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="L3" t="n">
@@ -708,7 +720,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N3" s="1" t="n">
+      <c r="N3" s="2" t="n">
         <v>46196</v>
       </c>
       <c r="O3" t="inlineStr"/>
@@ -789,10 +801,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J4" s="1" t="n">
+      <c r="J4" s="2" t="n">
         <v>46185</v>
       </c>
-      <c r="K4" s="1" t="n">
+      <c r="K4" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="L4" t="n">
@@ -803,10 +815,10 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N4" s="1" t="n">
+      <c r="N4" s="2" t="n">
         <v>46216</v>
       </c>
-      <c r="O4" s="1" t="n">
+      <c r="O4" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -890,10 +902,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J5" s="1" t="n">
+      <c r="J5" s="2" t="n">
         <v>46185</v>
       </c>
-      <c r="K5" s="1" t="n">
+      <c r="K5" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="L5" t="n">
@@ -904,7 +916,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N5" s="1" t="n">
+      <c r="N5" s="2" t="n">
         <v>46192</v>
       </c>
       <c r="O5" t="inlineStr"/>
@@ -985,10 +997,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J6" s="1" t="n">
+      <c r="J6" s="2" t="n">
         <v>46199</v>
       </c>
-      <c r="K6" s="1" t="n">
+      <c r="K6" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="L6" t="n">
@@ -999,7 +1011,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N6" s="1" t="n">
+      <c r="N6" s="2" t="n">
         <v>46214</v>
       </c>
       <c r="O6" t="inlineStr"/>
@@ -1084,10 +1096,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J7" s="1" t="n">
+      <c r="J7" s="2" t="n">
         <v>46205</v>
       </c>
-      <c r="K7" s="1" t="n">
+      <c r="K7" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="L7" t="n">
@@ -1098,7 +1110,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N7" s="1" t="n">
+      <c r="N7" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="O7" t="inlineStr"/>
@@ -1179,10 +1191,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J8" s="1" t="n">
+      <c r="J8" s="2" t="n">
         <v>46209</v>
       </c>
-      <c r="K8" s="1" t="n">
+      <c r="K8" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="L8" t="n">
@@ -1193,7 +1205,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N8" s="1" t="n">
+      <c r="N8" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="O8" t="inlineStr"/>
@@ -1270,10 +1282,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J9" s="1" t="n">
+      <c r="J9" s="2" t="n">
         <v>46209</v>
       </c>
-      <c r="K9" s="1" t="n">
+      <c r="K9" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="L9" t="n">
@@ -1284,7 +1296,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N9" s="1" t="n">
+      <c r="N9" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="O9" t="inlineStr"/>
@@ -1361,10 +1373,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J10" s="1" t="n">
+      <c r="J10" s="2" t="n">
         <v>46210</v>
       </c>
-      <c r="K10" s="1" t="n">
+      <c r="K10" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="L10" t="n">
@@ -1375,7 +1387,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N10" s="1" t="n">
+      <c r="N10" s="2" t="n">
         <v>46241</v>
       </c>
       <c r="O10" t="inlineStr"/>
@@ -1452,10 +1464,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J11" s="1" t="n">
+      <c r="J11" s="2" t="n">
         <v>46210</v>
       </c>
-      <c r="K11" s="1" t="n">
+      <c r="K11" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="L11" t="n">
@@ -1466,7 +1478,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N11" s="1" t="n">
+      <c r="N11" s="2" t="n">
         <v>46218</v>
       </c>
       <c r="O11" t="inlineStr"/>
@@ -1543,10 +1555,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J12" s="1" t="n">
+      <c r="J12" s="2" t="n">
         <v>46211</v>
       </c>
-      <c r="K12" s="1" t="n">
+      <c r="K12" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="L12" t="n">
@@ -1557,7 +1569,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N12" s="1" t="n">
+      <c r="N12" s="2" t="n">
         <v>46222</v>
       </c>
       <c r="O12" t="inlineStr"/>
@@ -1634,10 +1646,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J13" s="1" t="n">
+      <c r="J13" s="2" t="n">
         <v>46212</v>
       </c>
-      <c r="K13" s="1" t="n">
+      <c r="K13" s="2" t="n">
         <v>46212</v>
       </c>
       <c r="L13" t="n">
@@ -1648,7 +1660,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N13" s="1" t="n">
+      <c r="N13" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="O13" t="inlineStr"/>
@@ -1729,10 +1741,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J14" s="1" t="n">
+      <c r="J14" s="2" t="n">
         <v>46211</v>
       </c>
-      <c r="K14" s="1" t="n">
+      <c r="K14" s="2" t="n">
         <v>46212</v>
       </c>
       <c r="L14" t="n">
@@ -1743,7 +1755,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N14" s="1" t="n">
+      <c r="N14" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="O14" t="inlineStr"/>
@@ -1820,10 +1832,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J15" s="1" t="n">
+      <c r="J15" s="2" t="n">
         <v>46212</v>
       </c>
-      <c r="K15" s="1" t="n">
+      <c r="K15" s="2" t="n">
         <v>46212</v>
       </c>
       <c r="L15" t="n">
@@ -1834,7 +1846,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N15" s="1" t="n">
+      <c r="N15" s="2" t="n">
         <v>46243</v>
       </c>
       <c r="O15" t="inlineStr"/>

</xml_diff>

<commit_message>
Atualização automática: emergencias (10/07/2026 22:38)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,137 +421,137 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>om_emg</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>om</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>numero_emergencia</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>categoria</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>matricula_aeronave</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>tpemg</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>data_abertura</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>data_info</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>quantidade</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>unidade_medida</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>prazo_entrega</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>dpe</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>atendido_cancelado</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>dias_atraso</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>dias_corridos</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>estoque</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>retirado_empresa_recibo_obrigatorio</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>obs_coordenadoria_fiscal</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>obs_vee_one</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>provedor</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>awb</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>prev_entrega</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>mensagem_operador</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>em_aberto</t>
         </is>
@@ -611,10 +599,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J2" s="2" t="n">
+      <c r="J2" s="1" t="n">
         <v>46076</v>
       </c>
-      <c r="K2" s="2" t="n">
+      <c r="K2" s="1" t="n">
         <v>46080</v>
       </c>
       <c r="L2" t="n">
@@ -625,7 +613,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N2" s="2" t="n">
+      <c r="N2" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="O2" t="inlineStr"/>
@@ -706,10 +694,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J3" s="2" t="n">
+      <c r="J3" s="1" t="n">
         <v>46184</v>
       </c>
-      <c r="K3" s="2" t="n">
+      <c r="K3" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="L3" t="n">
@@ -720,7 +708,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N3" s="2" t="n">
+      <c r="N3" s="1" t="n">
         <v>46196</v>
       </c>
       <c r="O3" t="inlineStr"/>
@@ -801,10 +789,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J4" s="2" t="n">
+      <c r="J4" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="K4" s="2" t="n">
+      <c r="K4" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="L4" t="n">
@@ -815,10 +803,10 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N4" s="2" t="n">
+      <c r="N4" s="1" t="n">
         <v>46216</v>
       </c>
-      <c r="O4" s="2" t="n">
+      <c r="O4" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -902,10 +890,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J5" s="2" t="n">
+      <c r="J5" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="K5" s="2" t="n">
+      <c r="K5" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="L5" t="n">
@@ -916,7 +904,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N5" s="2" t="n">
+      <c r="N5" s="1" t="n">
         <v>46192</v>
       </c>
       <c r="O5" t="inlineStr"/>
@@ -997,10 +985,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J6" s="2" t="n">
+      <c r="J6" s="1" t="n">
         <v>46199</v>
       </c>
-      <c r="K6" s="2" t="n">
+      <c r="K6" s="1" t="n">
         <v>46203</v>
       </c>
       <c r="L6" t="n">
@@ -1011,7 +999,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N6" s="2" t="n">
+      <c r="N6" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="O6" t="inlineStr"/>
@@ -1096,10 +1084,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="J7" s="1" t="n">
         <v>46205</v>
       </c>
-      <c r="K7" s="2" t="n">
+      <c r="K7" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="L7" t="n">
@@ -1110,7 +1098,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N7" s="2" t="n">
+      <c r="N7" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="O7" t="inlineStr"/>
@@ -1191,10 +1179,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J8" s="2" t="n">
+      <c r="J8" s="1" t="n">
         <v>46209</v>
       </c>
-      <c r="K8" s="2" t="n">
+      <c r="K8" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="L8" t="n">
@@ -1205,7 +1193,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N8" s="2" t="n">
+      <c r="N8" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="O8" t="inlineStr"/>
@@ -1282,10 +1270,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J9" s="2" t="n">
+      <c r="J9" s="1" t="n">
         <v>46209</v>
       </c>
-      <c r="K9" s="2" t="n">
+      <c r="K9" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="L9" t="n">
@@ -1296,7 +1284,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N9" s="2" t="n">
+      <c r="N9" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="O9" t="inlineStr"/>
@@ -1373,10 +1361,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J10" s="2" t="n">
+      <c r="J10" s="1" t="n">
         <v>46210</v>
       </c>
-      <c r="K10" s="2" t="n">
+      <c r="K10" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="L10" t="n">
@@ -1387,7 +1375,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N10" s="2" t="n">
+      <c r="N10" s="1" t="n">
         <v>46241</v>
       </c>
       <c r="O10" t="inlineStr"/>
@@ -1464,10 +1452,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J11" s="2" t="n">
+      <c r="J11" s="1" t="n">
         <v>46210</v>
       </c>
-      <c r="K11" s="2" t="n">
+      <c r="K11" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="L11" t="n">
@@ -1478,7 +1466,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N11" s="2" t="n">
+      <c r="N11" s="1" t="n">
         <v>46218</v>
       </c>
       <c r="O11" t="inlineStr"/>
@@ -1555,10 +1543,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J12" s="2" t="n">
+      <c r="J12" s="1" t="n">
         <v>46211</v>
       </c>
-      <c r="K12" s="2" t="n">
+      <c r="K12" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="L12" t="n">
@@ -1569,7 +1557,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N12" s="2" t="n">
+      <c r="N12" s="1" t="n">
         <v>46222</v>
       </c>
       <c r="O12" t="inlineStr"/>
@@ -1646,10 +1634,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J13" s="2" t="n">
+      <c r="J13" s="1" t="n">
         <v>46212</v>
       </c>
-      <c r="K13" s="2" t="n">
+      <c r="K13" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="L13" t="n">
@@ -1660,7 +1648,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N13" s="2" t="n">
+      <c r="N13" s="1" t="n">
         <v>46219</v>
       </c>
       <c r="O13" t="inlineStr"/>
@@ -1741,10 +1729,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J14" s="2" t="n">
+      <c r="J14" s="1" t="n">
         <v>46211</v>
       </c>
-      <c r="K14" s="2" t="n">
+      <c r="K14" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="L14" t="n">
@@ -1755,7 +1743,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N14" s="2" t="n">
+      <c r="N14" s="1" t="n">
         <v>46219</v>
       </c>
       <c r="O14" t="inlineStr"/>
@@ -1832,10 +1820,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J15" s="2" t="n">
+      <c r="J15" s="1" t="n">
         <v>46212</v>
       </c>
-      <c r="K15" s="2" t="n">
+      <c r="K15" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="L15" t="n">
@@ -1846,7 +1834,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N15" s="2" t="n">
+      <c r="N15" s="1" t="n">
         <v>46243</v>
       </c>
       <c r="O15" t="inlineStr"/>

</xml_diff>

<commit_message>
Atualização automática: emergencias (10/07/2026 20:00)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -421,137 +433,137 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>om_emg</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>om</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>numero_emergencia</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>categoria</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>matricula_aeronave</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>tpemg</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>data_abertura</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>data_info</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>quantidade</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>unidade_medida</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>prazo_entrega</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>dpe</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>atendido_cancelado</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>dias_atraso</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>dias_corridos</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>estoque</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>retirado_empresa_recibo_obrigatorio</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>obs_coordenadoria_fiscal</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>obs_vee_one</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>provedor</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>awb</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>prev_entrega</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>mensagem_operador</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>em_aberto</t>
         </is>
@@ -599,10 +611,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J2" s="1" t="n">
+      <c r="J2" s="2" t="n">
         <v>46076</v>
       </c>
-      <c r="K2" s="1" t="n">
+      <c r="K2" s="2" t="n">
         <v>46080</v>
       </c>
       <c r="L2" t="n">
@@ -613,7 +625,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N2" s="1" t="n">
+      <c r="N2" s="2" t="n">
         <v>46111</v>
       </c>
       <c r="O2" t="inlineStr"/>
@@ -694,10 +706,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J3" s="1" t="n">
+      <c r="J3" s="2" t="n">
         <v>46184</v>
       </c>
-      <c r="K3" s="1" t="n">
+      <c r="K3" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="L3" t="n">
@@ -708,7 +720,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N3" s="1" t="n">
+      <c r="N3" s="2" t="n">
         <v>46196</v>
       </c>
       <c r="O3" t="inlineStr"/>
@@ -789,10 +801,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J4" s="1" t="n">
+      <c r="J4" s="2" t="n">
         <v>46185</v>
       </c>
-      <c r="K4" s="1" t="n">
+      <c r="K4" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="L4" t="n">
@@ -803,10 +815,10 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N4" s="1" t="n">
+      <c r="N4" s="2" t="n">
         <v>46216</v>
       </c>
-      <c r="O4" s="1" t="n">
+      <c r="O4" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -890,10 +902,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J5" s="1" t="n">
+      <c r="J5" s="2" t="n">
         <v>46185</v>
       </c>
-      <c r="K5" s="1" t="n">
+      <c r="K5" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="L5" t="n">
@@ -904,7 +916,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N5" s="1" t="n">
+      <c r="N5" s="2" t="n">
         <v>46192</v>
       </c>
       <c r="O5" t="inlineStr"/>
@@ -985,10 +997,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J6" s="1" t="n">
+      <c r="J6" s="2" t="n">
         <v>46199</v>
       </c>
-      <c r="K6" s="1" t="n">
+      <c r="K6" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="L6" t="n">
@@ -999,7 +1011,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N6" s="1" t="n">
+      <c r="N6" s="2" t="n">
         <v>46214</v>
       </c>
       <c r="O6" t="inlineStr"/>
@@ -1084,10 +1096,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J7" s="1" t="n">
+      <c r="J7" s="2" t="n">
         <v>46205</v>
       </c>
-      <c r="K7" s="1" t="n">
+      <c r="K7" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="L7" t="n">
@@ -1098,7 +1110,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N7" s="1" t="n">
+      <c r="N7" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="O7" t="inlineStr"/>
@@ -1179,10 +1191,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J8" s="1" t="n">
+      <c r="J8" s="2" t="n">
         <v>46209</v>
       </c>
-      <c r="K8" s="1" t="n">
+      <c r="K8" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="L8" t="n">
@@ -1193,7 +1205,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N8" s="1" t="n">
+      <c r="N8" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="O8" t="inlineStr"/>
@@ -1270,10 +1282,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J9" s="1" t="n">
+      <c r="J9" s="2" t="n">
         <v>46209</v>
       </c>
-      <c r="K9" s="1" t="n">
+      <c r="K9" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="L9" t="n">
@@ -1284,7 +1296,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N9" s="1" t="n">
+      <c r="N9" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="O9" t="inlineStr"/>
@@ -1361,10 +1373,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J10" s="1" t="n">
+      <c r="J10" s="2" t="n">
         <v>46210</v>
       </c>
-      <c r="K10" s="1" t="n">
+      <c r="K10" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="L10" t="n">
@@ -1375,7 +1387,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N10" s="1" t="n">
+      <c r="N10" s="2" t="n">
         <v>46241</v>
       </c>
       <c r="O10" t="inlineStr"/>
@@ -1452,10 +1464,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J11" s="1" t="n">
+      <c r="J11" s="2" t="n">
         <v>46210</v>
       </c>
-      <c r="K11" s="1" t="n">
+      <c r="K11" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="L11" t="n">
@@ -1466,7 +1478,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N11" s="1" t="n">
+      <c r="N11" s="2" t="n">
         <v>46218</v>
       </c>
       <c r="O11" t="inlineStr"/>
@@ -1543,10 +1555,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J12" s="1" t="n">
+      <c r="J12" s="2" t="n">
         <v>46211</v>
       </c>
-      <c r="K12" s="1" t="n">
+      <c r="K12" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="L12" t="n">
@@ -1557,7 +1569,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N12" s="1" t="n">
+      <c r="N12" s="2" t="n">
         <v>46222</v>
       </c>
       <c r="O12" t="inlineStr"/>
@@ -1634,10 +1646,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J13" s="1" t="n">
+      <c r="J13" s="2" t="n">
         <v>46212</v>
       </c>
-      <c r="K13" s="1" t="n">
+      <c r="K13" s="2" t="n">
         <v>46212</v>
       </c>
       <c r="L13" t="n">
@@ -1648,7 +1660,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N13" s="1" t="n">
+      <c r="N13" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="O13" t="inlineStr"/>
@@ -1729,10 +1741,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J14" s="1" t="n">
+      <c r="J14" s="2" t="n">
         <v>46211</v>
       </c>
-      <c r="K14" s="1" t="n">
+      <c r="K14" s="2" t="n">
         <v>46212</v>
       </c>
       <c r="L14" t="n">
@@ -1743,7 +1755,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N14" s="1" t="n">
+      <c r="N14" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="O14" t="inlineStr"/>
@@ -1820,10 +1832,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J15" s="1" t="n">
+      <c r="J15" s="2" t="n">
         <v>46212</v>
       </c>
-      <c r="K15" s="1" t="n">
+      <c r="K15" s="2" t="n">
         <v>46212</v>
       </c>
       <c r="L15" t="n">
@@ -1834,7 +1846,7 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N15" s="1" t="n">
+      <c r="N15" s="2" t="n">
         <v>46243</v>
       </c>
       <c r="O15" t="inlineStr"/>

</xml_diff>

<commit_message>
Atualização automática: emergencias (11/07/2026 07:19)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,137 +421,137 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>om_emg</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>om</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>numero_emergencia</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>categoria</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>matricula_aeronave</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>tpemg</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>data_abertura</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>data_info</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>quantidade</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>unidade_medida</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>prazo_entrega</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>dpe</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>atendido_cancelado</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>dias_atraso</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>dias_corridos</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>estoque</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>retirado_empresa_recibo_obrigatorio</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>obs_coordenadoria_fiscal</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>obs_vee_one</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>provedor</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>awb</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>prev_entrega</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>mensagem_operador</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>em_aberto</t>
         </is>
@@ -611,10 +599,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J2" s="2" t="n">
+      <c r="J2" s="1" t="n">
         <v>46076</v>
       </c>
-      <c r="K2" s="2" t="n">
+      <c r="K2" s="1" t="n">
         <v>46080</v>
       </c>
       <c r="L2" t="n">
@@ -625,16 +613,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N2" s="2" t="n">
+      <c r="N2" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="R2" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -706,10 +694,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J3" s="2" t="n">
+      <c r="J3" s="1" t="n">
         <v>46184</v>
       </c>
-      <c r="K3" s="2" t="n">
+      <c r="K3" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="L3" t="n">
@@ -720,16 +708,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N3" s="2" t="n">
+      <c r="N3" s="1" t="n">
         <v>46196</v>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="R3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -801,10 +789,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J4" s="2" t="n">
+      <c r="J4" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="K4" s="2" t="n">
+      <c r="K4" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="L4" t="n">
@@ -815,18 +803,18 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N4" s="2" t="n">
+      <c r="N4" s="1" t="n">
         <v>46216</v>
       </c>
-      <c r="O4" s="2" t="n">
+      <c r="O4" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R4" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -902,10 +890,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J5" s="2" t="n">
+      <c r="J5" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="K5" s="2" t="n">
+      <c r="K5" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="L5" t="n">
@@ -916,16 +904,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N5" s="2" t="n">
+      <c r="N5" s="1" t="n">
         <v>46192</v>
       </c>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="R5" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -997,10 +985,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J6" s="2" t="n">
+      <c r="J6" s="1" t="n">
         <v>46199</v>
       </c>
-      <c r="K6" s="2" t="n">
+      <c r="K6" s="1" t="n">
         <v>46203</v>
       </c>
       <c r="L6" t="n">
@@ -1011,16 +999,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N6" s="2" t="n">
+      <c r="N6" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1096,10 +1084,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="J7" s="1" t="n">
         <v>46205</v>
       </c>
-      <c r="K7" s="2" t="n">
+      <c r="K7" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="L7" t="n">
@@ -1110,16 +1098,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N7" s="2" t="n">
+      <c r="N7" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1191,10 +1179,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J8" s="2" t="n">
+      <c r="J8" s="1" t="n">
         <v>46209</v>
       </c>
-      <c r="K8" s="2" t="n">
+      <c r="K8" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="L8" t="n">
@@ -1205,16 +1193,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N8" s="2" t="n">
+      <c r="N8" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1282,10 +1270,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J9" s="2" t="n">
+      <c r="J9" s="1" t="n">
         <v>46209</v>
       </c>
-      <c r="K9" s="2" t="n">
+      <c r="K9" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="L9" t="n">
@@ -1296,16 +1284,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N9" s="2" t="n">
+      <c r="N9" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -1373,10 +1361,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J10" s="2" t="n">
+      <c r="J10" s="1" t="n">
         <v>46210</v>
       </c>
-      <c r="K10" s="2" t="n">
+      <c r="K10" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="L10" t="n">
@@ -1387,16 +1375,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N10" s="2" t="n">
+      <c r="N10" s="1" t="n">
         <v>46241</v>
       </c>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="n">
-        <v>-28</v>
+        <v>-27</v>
       </c>
       <c r="R10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
@@ -1464,10 +1452,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J11" s="2" t="n">
+      <c r="J11" s="1" t="n">
         <v>46210</v>
       </c>
-      <c r="K11" s="2" t="n">
+      <c r="K11" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="L11" t="n">
@@ -1478,16 +1466,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N11" s="2" t="n">
+      <c r="N11" s="1" t="n">
         <v>46218</v>
       </c>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="n">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
@@ -1555,10 +1543,10 @@
           <t>IPLR</t>
         </is>
       </c>
-      <c r="J12" s="2" t="n">
+      <c r="J12" s="1" t="n">
         <v>46211</v>
       </c>
-      <c r="K12" s="2" t="n">
+      <c r="K12" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="L12" t="n">
@@ -1569,16 +1557,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N12" s="2" t="n">
+      <c r="N12" s="1" t="n">
         <v>46222</v>
       </c>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="n">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="R12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -1646,10 +1634,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J13" s="2" t="n">
+      <c r="J13" s="1" t="n">
         <v>46212</v>
       </c>
-      <c r="K13" s="2" t="n">
+      <c r="K13" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="L13" t="n">
@@ -1660,16 +1648,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N13" s="2" t="n">
+      <c r="N13" s="1" t="n">
         <v>46219</v>
       </c>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="n">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
@@ -1741,10 +1729,10 @@
           <t>AIFP</t>
         </is>
       </c>
-      <c r="J14" s="2" t="n">
+      <c r="J14" s="1" t="n">
         <v>46211</v>
       </c>
-      <c r="K14" s="2" t="n">
+      <c r="K14" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="L14" t="n">
@@ -1755,16 +1743,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N14" s="2" t="n">
+      <c r="N14" s="1" t="n">
         <v>46219</v>
       </c>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="n">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
@@ -1832,10 +1820,10 @@
           <t>ANCE</t>
         </is>
       </c>
-      <c r="J15" s="2" t="n">
+      <c r="J15" s="1" t="n">
         <v>46212</v>
       </c>
-      <c r="K15" s="2" t="n">
+      <c r="K15" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="L15" t="n">
@@ -1846,16 +1834,16 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="N15" s="2" t="n">
+      <c r="N15" s="1" t="n">
         <v>46243</v>
       </c>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="n">
-        <v>-30</v>
+        <v>-29</v>
       </c>
       <c r="R15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Corrige crash em produção: PN com tipo misto (int/str) quebrava sorted()
Depois da atualização de Reparáveis, uma OS nova tinha PN só numérico,
que o openpyxl lê como int em vez de str — a coluna "pn" ficou com
tipos mistos, e sorted(df["pn"].dropna().unique()) quebrava com
TypeError direto no Streamlit Cloud. Mesma causa quebrava a conversão
pra Arrow do st.dataframe.

Correção em duas camadas: (1) normaliza PN pra string na extração
(extrair_reparaveis.py, extrair_emergencias.py — parse_texto_pn), raiz
do problema; (2) troca todo `sorted(df[col].dropna().unique())` por um
helper novo (components/utils.py::ordenar_unicos, ordena por
representação em string) nas 7 telas que tinham o mesmo padrão frágil,
defensivo contra o mesmo tipo de dado sujo em qualquer coluna.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="108">
   <si>
     <t>om_emg</t>
   </si>
@@ -154,6 +154,9 @@
     <t>685260012350</t>
   </si>
   <si>
+    <t>313260018670</t>
+  </si>
+  <si>
     <t>1214134-1</t>
   </si>
   <si>
@@ -190,6 +193,9 @@
     <t>030-1094-58</t>
   </si>
   <si>
+    <t>S2655-1</t>
+  </si>
+  <si>
     <t>BELLCRANK ASSY</t>
   </si>
   <si>
@@ -226,6 +232,9 @@
     <t>CONNECTOR</t>
   </si>
   <si>
+    <t>DUCT-FLEX</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -238,6 +247,9 @@
     <t>Providência tomada</t>
   </si>
   <si>
+    <t>Aguardando solução</t>
+  </si>
+  <si>
     <t>ANCE</t>
   </si>
   <si>
@@ -274,7 +286,13 @@
     <t>Recibo não se encontra na Pasta do DRIVE. Godoy 08/07/2026.</t>
   </si>
   <si>
+    <t>AWB 12745918331 volume retirado na loja GOLLOG - BEL por bispo em 10/07/2026 - Godoy 13/07/2026.</t>
+  </si>
+  <si>
     <t>Cedeu o item para o C-98 2721. Ramon 09/07/26.</t>
+  </si>
+  <si>
+    <t>Cedeu o item para o C-98 2738. Godoy 13/07/26</t>
   </si>
   <si>
     <t>Foi solicitado via email no dia 02-03-2 o atendimento do item com estoque FAB. Claudio -02-03-26 - Em resposta, a coordenadoria disse que o estque seria insuficiente. Foi verificado que na T.O da ANV o QPA para esse item são 2 EA, solicitei confirmação. - Cláudio -02-03-2026. Solicitado o cancelamento da emergência em função da quantidade cedida ao 2733 ter sido de 01ea. Considerando o QPA 02 ea. Encontra-se em tratativa junto a fiscalização e o gestor do contrato conforme mensagem de e-mail de 05/03. - SOLICITAÇÃO E-C98-26047.Colocado pedido AOG Textron WB0003068789 - previsão de entrega 60 dias em média. Os demais fornecedores informaram não ter em estoque ou não possuírem a certificação necessária da peça.</t>
@@ -681,7 +699,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA15"/>
+  <dimension ref="A1:AA16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -778,22 +796,22 @@
         <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F2" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G2">
         <v>2730</v>
       </c>
       <c r="H2" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I2" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="J2" s="2">
         <v>46076</v>
@@ -805,7 +823,7 @@
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="N2" s="2">
         <v>46111</v>
@@ -817,16 +835,16 @@
         <v>136</v>
       </c>
       <c r="S2" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="U2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="V2" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="W2" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -843,22 +861,22 @@
         <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="G3">
         <v>2734</v>
       </c>
       <c r="H3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I3" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="J3" s="2">
         <v>46184</v>
@@ -870,7 +888,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="N3" s="2">
         <v>46196</v>
@@ -882,16 +900,16 @@
         <v>31</v>
       </c>
       <c r="S3" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="U3" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="V3" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="W3" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -908,22 +926,22 @@
         <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F4" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G4">
         <v>2721</v>
       </c>
       <c r="H4" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I4" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="J4" s="2">
         <v>46185</v>
@@ -935,7 +953,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="N4" s="2">
         <v>46216</v>
@@ -950,19 +968,19 @@
         <v>31</v>
       </c>
       <c r="S4" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="T4" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="U4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="V4" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="W4" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -979,22 +997,22 @@
         <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F5" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="G5">
         <v>2726</v>
       </c>
       <c r="H5" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I5" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="J5" s="2">
         <v>46185</v>
@@ -1006,7 +1024,7 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="N5" s="2">
         <v>46192</v>
@@ -1018,16 +1036,16 @@
         <v>31</v>
       </c>
       <c r="S5" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="U5" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="V5" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="W5" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1044,22 +1062,22 @@
         <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E6" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F6" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="G6">
         <v>2734</v>
       </c>
       <c r="H6" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I6" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="J6" s="2">
         <v>46199</v>
@@ -1071,7 +1089,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="N6" s="2">
         <v>46214</v>
@@ -1083,19 +1101,19 @@
         <v>13</v>
       </c>
       <c r="S6" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="T6" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="U6" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="V6" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="W6" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1112,22 +1130,22 @@
         <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E7" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F7" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="G7">
         <v>2721</v>
       </c>
       <c r="H7" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I7" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="J7" s="2">
         <v>46205</v>
@@ -1139,7 +1157,7 @@
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="N7" s="2">
         <v>46213</v>
@@ -1151,16 +1169,16 @@
         <v>10</v>
       </c>
       <c r="S7" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="U7" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="V7" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="W7" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1177,22 +1195,22 @@
         <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F8" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G8">
         <v>2709</v>
       </c>
       <c r="H8" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I8" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="J8" s="2">
         <v>46209</v>
@@ -1204,7 +1222,7 @@
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="N8" s="2">
         <v>46217</v>
@@ -1216,13 +1234,13 @@
         <v>6</v>
       </c>
       <c r="S8" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="V8" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="W8" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1239,22 +1257,22 @@
         <v>39</v>
       </c>
       <c r="D9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F9" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G9">
         <v>2721</v>
       </c>
       <c r="H9" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I9" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="J9" s="2">
         <v>46209</v>
@@ -1266,7 +1284,7 @@
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="N9" s="2">
         <v>46217</v>
@@ -1278,13 +1296,13 @@
         <v>6</v>
       </c>
       <c r="S9" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="V9" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="W9" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1301,22 +1319,22 @@
         <v>40</v>
       </c>
       <c r="D10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E10" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F10" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="G10">
         <v>2719</v>
       </c>
       <c r="H10" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I10" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="J10" s="2">
         <v>46210</v>
@@ -1328,7 +1346,7 @@
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="N10" s="2">
         <v>46241</v>
@@ -1340,13 +1358,13 @@
         <v>6</v>
       </c>
       <c r="S10" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="V10" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="W10" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1363,22 +1381,22 @@
         <v>41</v>
       </c>
       <c r="D11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E11" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F11" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="G11">
         <v>2723</v>
       </c>
       <c r="H11" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I11" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="J11" s="2">
         <v>46210</v>
@@ -1390,7 +1408,7 @@
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="N11" s="2">
         <v>46218</v>
@@ -1402,13 +1420,16 @@
         <v>5</v>
       </c>
       <c r="S11" t="s">
-        <v>78</v>
+        <v>82</v>
+      </c>
+      <c r="U11" t="s">
+        <v>90</v>
       </c>
       <c r="V11" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="W11" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1425,22 +1446,22 @@
         <v>42</v>
       </c>
       <c r="D12" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E12" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F12" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="G12">
         <v>2733</v>
       </c>
       <c r="H12" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I12" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="J12" s="2">
         <v>46211</v>
@@ -1452,7 +1473,7 @@
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="N12" s="2">
         <v>46222</v>
@@ -1464,13 +1485,13 @@
         <v>5</v>
       </c>
       <c r="S12" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="V12" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="W12" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1487,22 +1508,22 @@
         <v>43</v>
       </c>
       <c r="D13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F13" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="G13">
         <v>2726</v>
       </c>
       <c r="H13" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I13" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="J13" s="2">
         <v>46212</v>
@@ -1514,7 +1535,7 @@
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="N13" s="2">
         <v>46219</v>
@@ -1526,16 +1547,16 @@
         <v>4</v>
       </c>
       <c r="S13" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="U13" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="V13" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="W13" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1552,22 +1573,22 @@
         <v>44</v>
       </c>
       <c r="D14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E14" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F14" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="G14">
         <v>2723</v>
       </c>
       <c r="H14" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I14" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="J14" s="2">
         <v>46211</v>
@@ -1579,7 +1600,7 @@
         <v>1</v>
       </c>
       <c r="M14" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="N14" s="2">
         <v>46219</v>
@@ -1591,13 +1612,13 @@
         <v>4</v>
       </c>
       <c r="S14" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="V14" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="W14" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
@@ -1614,22 +1635,22 @@
         <v>45</v>
       </c>
       <c r="D15" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E15" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F15" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G15">
         <v>2702</v>
       </c>
       <c r="H15" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I15" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="J15" s="2">
         <v>46212</v>
@@ -1641,7 +1662,7 @@
         <v>1</v>
       </c>
       <c r="M15" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="N15" s="2">
         <v>46243</v>
@@ -1653,15 +1674,77 @@
         <v>4</v>
       </c>
       <c r="S15" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="V15" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="W15" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="AA15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27">
+      <c r="A16">
+        <v>313</v>
+      </c>
+      <c r="B16" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" t="s">
+        <v>46</v>
+      </c>
+      <c r="D16" t="s">
+        <v>59</v>
+      </c>
+      <c r="E16" t="s">
+        <v>72</v>
+      </c>
+      <c r="F16" t="s">
+        <v>73</v>
+      </c>
+      <c r="G16">
+        <v>2734</v>
+      </c>
+      <c r="H16" t="s">
+        <v>77</v>
+      </c>
+      <c r="I16" t="s">
+        <v>79</v>
+      </c>
+      <c r="J16" s="2">
+        <v>46213</v>
+      </c>
+      <c r="K16" s="2">
+        <v>46213</v>
+      </c>
+      <c r="L16">
+        <v>1</v>
+      </c>
+      <c r="M16" t="s">
+        <v>81</v>
+      </c>
+      <c r="N16" s="2">
+        <v>46224</v>
+      </c>
+      <c r="Q16">
+        <v>-8</v>
+      </c>
+      <c r="R16">
+        <v>3</v>
+      </c>
+      <c r="S16" t="s">
+        <v>82</v>
+      </c>
+      <c r="U16" t="s">
+        <v>92</v>
+      </c>
+      <c r="W16" t="s">
+        <v>107</v>
+      </c>
+      <c r="AA16" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (14/07/2026 06:38)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -619,10 +619,10 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="R2" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -714,10 +714,10 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="R3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -811,10 +811,10 @@
       </c>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R4" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -910,10 +910,10 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="R5" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -1005,10 +1005,10 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1104,10 +1104,10 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1199,10 +1199,10 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1290,10 +1290,10 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -1381,10 +1381,10 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="n">
-        <v>-25</v>
+        <v>-24</v>
       </c>
       <c r="R10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
@@ -1472,10 +1472,10 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
@@ -1567,10 +1567,10 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="n">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -1658,10 +1658,10 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
@@ -1753,10 +1753,10 @@
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
@@ -1844,10 +1844,10 @@
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="n">
-        <v>-27</v>
+        <v>-26</v>
       </c>
       <c r="R15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
@@ -1935,10 +1935,10 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="n">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="R16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática: emergencias (14/07/2026 16:03)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA16"/>
+  <dimension ref="A1:AA19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -928,7 +928,7 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>"04 ea recolhidos para a V1, chegada dos itens dia 23/06/2026. Itens não tem oficina no Brasil, terá que ser feito  Exchange rc 23/06 - MATERIAL ADQUIRIDO FORNECEDOR TEXTRON -WB0003073549 Inovice IJ17534800 DPE AGS  Miami 29/6/2026 ate 10 30AM - AIR EXPORT HOUSE: 00004046 de 30/6/2026 Chegou no GIGRJ em 01/7/26 para  Desembaraço - ATZ Marcio 3/7/26 CANAL VERDE EM 7/7/26 entregue V1 em 8/7/26 ATZ Marcio 9/7/26"</t>
+          <t>04 ea recolhidos para a V1, chegada dos itens dia 23/06/2026. Itens não tem oficina no Brasil, terá que ser feito Exchange rc 23/06 - MATERIAL ADQUIRIDO FORNECEDOR TEXTRON -WB0003073549 Inovice IJ17534800 DPE AGS Miami 29/6/2026 ate 10 30AM - AIR EXPORT HOUSE: 00004046 de 30/6/2026 Chegou no GIGRJ em 01/7/26 para Desembaraço - ATZ Marcio 3/7/26 CANAL VERDE EM 7/7/26 entregue V1 em 8/7/26 ATZ Marcio 9/7/26 - MATERIAL EM TRANSITO - RECIBO 560/FAB/26 AWB - 12746187256 DPE 13/07/2026</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
@@ -1122,7 +1122,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Item estara disponivel no RJ na oficina para coleta dia 6/7 apos as 14 horas ATZ Marcio 3/7/ 14:25PM/ MATERIAL EM TRANSITO- RECIBO 548/FAB/26- AWB 12745474752 DPE 08/07 - Atlz Lucas- JPA (07/07) - MATERIAL DISPONIVEL PRA RETIRADA DIA 09/07/2026 ATZ RC</t>
+          <t>Item estara disponivel no RJ na oficina para coleta dia 6/7 apos as 14 horas ATZ Marcio 3/7/ 14:25PM/ MATERIAL EM TRANSITO- RECIBO 548/FAB/26- AWB 12745474752 DPE 08/07 - Atlz Lucas- JPA (07/07) - MATERIAL DISPONIVEL PRA RETIRADA DIA 09/07/2026 ATZ RC - MATERIAL RETIRADO DIA 09/07/2026 POR KÉSIA SANTOS</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
@@ -1176,7 +1176,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>AIFP</t>
+          <t>ANCE</t>
         </is>
       </c>
       <c r="J8" s="1" t="n">
@@ -1194,12 +1194,12 @@
         </is>
       </c>
       <c r="N8" s="1" t="n">
-        <v>46217</v>
+        <v>46241</v>
       </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="n">
-        <v>0</v>
+        <v>-24</v>
       </c>
       <c r="R8" t="n">
         <v>7</v>
@@ -1213,7 +1213,7 @@
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Colocado pedido AOG Textron IJ17557538 - previsão de entrega em Miami 08/07. Previsão de chegada GIG 09/07 - MATERIAL EM TRANSITO - RECIBO 551/FAB/26 - ENVIADO PN COMPLETO PARA SANAR A EMERGENCIA DO 2709, ENVIADO MODAL TERRESTRE, DPE 09/07/2026</t>
+          <t>Colocado pedido AOG Textron IJ17557538 - previsão de entrega em Miami 08/07. Previsão de chegada GIG 09/07 - MATERIAL EM TRANSITO - RECIBO 551/FAB/26 - ENVIADO PN COMPLETO PARA SANAR A EMERGENCIA DO 2709, ENVIADO MODAL TERRESTRE, DPE 13/07/2026</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
@@ -1304,7 +1304,7 @@
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Colocado pedido AOG Textron IJ17557538 - previsão de entrega em Miami 08/07. Previsão de chegada GIG 09/07 (voo 4093)</t>
+          <t>Colocado pedido AOG Textron IJ17557538 - previsão de entrega em Miami 08/07. HAWB4093 - CANAL VERDE - ENTREGUE NA VEE ONE 13/07. ATZ MAYARA 13/07/26</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
@@ -1907,7 +1907,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Aguardando solução</t>
+          <t>Providência tomada</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1961,6 +1961,267 @@
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="inlineStr"/>
       <c r="AA16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>313</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>BAMN</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>313260018674</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>205842-1</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>CONNECTOR</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>2736</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Aguardando solução</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>ANCE</t>
+        </is>
+      </c>
+      <c r="J17" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="K17" s="1" t="n">
+        <v>46217</v>
+      </c>
+      <c r="L17" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="N17" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="n">
+        <v>-31</v>
+      </c>
+      <c r="R17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>VEE ONE</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr"/>
+      <c r="Y17" t="inlineStr"/>
+      <c r="Z17" t="inlineStr"/>
+      <c r="AA17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>685</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>BANT</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>685260012368</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>C611008-0101</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>ALTERNATOR CONTROL U</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>2729</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Aguardando solução</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>ANCE</t>
+        </is>
+      </c>
+      <c r="J18" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="K18" s="1" t="n">
+        <v>46217</v>
+      </c>
+      <c r="L18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="N18" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="n">
+        <v>-31</v>
+      </c>
+      <c r="R18" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>VEE ONE</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr"/>
+      <c r="Y18" t="inlineStr"/>
+      <c r="Z18" t="inlineStr"/>
+      <c r="AA18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>386</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>BACO</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>386260013445</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>C611008-0101</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>ALTERNATOR CONTROL U</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>2743</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Aguardando solução</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>IPLR</t>
+        </is>
+      </c>
+      <c r="J19" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="K19" s="1" t="n">
+        <v>46217</v>
+      </c>
+      <c r="L19" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="N19" s="1" t="n">
+        <v>46228</v>
+      </c>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="n">
+        <v>-11</v>
+      </c>
+      <c r="R19" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr"/>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>VEE ONE</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr"/>
+      <c r="Y19" t="inlineStr"/>
+      <c r="Z19" t="inlineStr"/>
+      <c r="AA19" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (15/07/2026 16:10)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="110">
   <si>
     <t>om_emg</t>
   </si>
@@ -118,9 +118,6 @@
     <t>313260017747</t>
   </si>
   <si>
-    <t>313260018412</t>
-  </si>
-  <si>
     <t>329260019153</t>
   </si>
   <si>
@@ -169,12 +166,12 @@
     <t>386260013445</t>
   </si>
   <si>
+    <t>685260012377</t>
+  </si>
+  <si>
     <t>1214134-1</t>
   </si>
   <si>
-    <t>011-01105-01</t>
-  </si>
-  <si>
     <t>TWINA0502</t>
   </si>
   <si>
@@ -217,9 +214,6 @@
     <t>BELLCRANK ASSY</t>
   </si>
   <si>
-    <t>INTEGRATED AVIONICS</t>
-  </si>
-  <si>
     <t>PROBE TEMPERATURE</t>
   </si>
   <si>
@@ -259,12 +253,12 @@
     <t>C</t>
   </si>
   <si>
+    <t>T</t>
+  </si>
+  <si>
     <t>R</t>
   </si>
   <si>
-    <t>T</t>
-  </si>
-  <si>
     <t>Providência tomada</t>
   </si>
   <si>
@@ -274,12 +268,12 @@
     <t>ANCE</t>
   </si>
   <si>
+    <t>AIFP</t>
+  </si>
+  <si>
     <t>IPLR</t>
   </si>
   <si>
-    <t>AIFP</t>
-  </si>
-  <si>
     <t>EA</t>
   </si>
   <si>
@@ -292,16 +286,13 @@
     <t>Foram cedidos para o C-98 2733. / De acordo com o manual da aeronave, o QPA é 02 EA por cadeira. Sendo o total para a aeronave 04 EA.A demanda aberta foi de  4EA, o SO Bispo que intermediou . Wallace 29.05</t>
   </si>
   <si>
-    <t>Retirado para atender a Anv 2737 - Godoy 12/06/26.</t>
-  </si>
-  <si>
     <t>Volume retirado na loja GOLLOG - BSB por tanise Assis em 03/07/2026 - Godoy 08/07/2026. Recibo não se encontra na Pasta do DRIVE. Godoy 08/07/2026.</t>
   </si>
   <si>
     <t>Item retirado para atender o C-98 2731. Ramon 15/06/26.</t>
   </si>
   <si>
-    <t>Retirado para atender a Anv 2740 - Godoy 30/06/26.</t>
+    <t>Retirado para atender a Anv 2740 - Godoy 30/06/26. AWB 12745953832 - Volume retirado na loja GOLLOG - QMA por Kleyton em 13/07/26. Godoy 15/07/26.</t>
   </si>
   <si>
     <t>Recibo não se encontra na Pasta do DRIVE. Godoy 08/07/2026.</t>
@@ -310,16 +301,13 @@
     <t>AWB 12745918331 volume retirado na loja GOLLOG - BEL por bispo em 10/07/2026 - Godoy 13/07/2026.</t>
   </si>
   <si>
-    <t>Cedeu o item para o C-98 2721. Ramon 09/07/26.</t>
+    <t>Cedeu o item para o C-98 2721. Ramon 09/07/26. AWB 12746175415 - 2 volumes retirados na loja GOLLOG - BEL por bispo em 13/07/26. Godoy 15/07/26.</t>
   </si>
   <si>
     <t>Cedeu o item para o C-98 2738. Godoy 13/07/26</t>
   </si>
   <si>
     <t>Foi solicitado via email no dia 02-03-2 o atendimento do item com estoque FAB. Claudio -02-03-26 - Em resposta, a coordenadoria disse que o estque seria insuficiente. Foi verificado que na T.O da ANV o QPA para esse item são 2 EA, solicitei confirmação. - Cláudio -02-03-2026. Solicitado o cancelamento da emergência em função da quantidade cedida ao 2733 ter sido de 01ea. Considerando o QPA 02 ea. Encontra-se em tratativa junto a fiscalização e o gestor do contrato conforme mensagem de e-mail de 05/03. - SOLICITAÇÃO E-C98-26047.Colocado pedido AOG Textron WB0003068789 - previsão de entrega 60 dias em média. Os demais fornecedores informaram não ter em estoque ou não possuírem a certificação necessária da peça.</t>
-  </si>
-  <si>
-    <t>Material Liberado Canal Verde em 01/7/2026 - HAWB: 00125552354 00004021 , Invoice PPSPI01534 PO 696/JPA/2026, aguardando ICMS GIGRJ. ATZ Marcio 01/7/2026 16:13 - material em processo de envio 06/07/2026 - AWB 12744955875 dpe 10/07/2026</t>
   </si>
   <si>
     <t>Colocado pedido na Textron IJ17507011. Previsão de entrega em Miami 17/06. Carga recepcionada no GIG 24/06. Canal verde dia 26/06. DPE V1 29/06. Verificar entrega do item. ATZ 30/06 - MATERIAL EM RECEBIMENTO V1 30-06-2026 - MATERIAL EM PROCESSO DE ENVIO RECIBO 524/FAB/26 ATZ RC 30-06-2026 - MATERIAL EM TRANSITO - AWB 12744330731 DPE 03/07/2026 - MATERIAL RECEBIDO POR tanise Assis RG 14807641751 DIA 03/07/2026</t>
@@ -791,19 +779,19 @@
         <v>51</v>
       </c>
       <c r="E2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G2">
         <v>2730</v>
       </c>
       <c r="H2" t="s">
+        <v>81</v>
+      </c>
+      <c r="I2" t="s">
         <v>83</v>
-      </c>
-      <c r="I2" t="s">
-        <v>85</v>
       </c>
       <c r="J2" s="1">
         <v>46076</v>
@@ -815,28 +803,28 @@
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N2" s="1">
         <v>46111</v>
       </c>
       <c r="Q2">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="R2">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="S2" t="s">
+        <v>87</v>
+      </c>
+      <c r="U2" t="s">
         <v>89</v>
       </c>
-      <c r="U2" t="s">
-        <v>91</v>
-      </c>
       <c r="V2" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="W2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -844,10 +832,10 @@
     </row>
     <row r="3" spans="1:27">
       <c r="A3">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
         <v>34</v>
@@ -856,22 +844,22 @@
         <v>52</v>
       </c>
       <c r="E3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F3" t="s">
+        <v>78</v>
+      </c>
+      <c r="G3">
+        <v>2721</v>
+      </c>
+      <c r="H3" t="s">
         <v>81</v>
       </c>
-      <c r="G3">
-        <v>2734</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>83</v>
       </c>
-      <c r="I3" t="s">
-        <v>86</v>
-      </c>
       <c r="J3" s="1">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="K3" s="1">
         <v>46185</v>
@@ -880,28 +868,34 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N3" s="1">
-        <v>46196</v>
+        <v>46216</v>
+      </c>
+      <c r="O3" s="1">
+        <v>46216</v>
       </c>
       <c r="Q3">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="R3">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S3" t="s">
-        <v>89</v>
+        <v>87</v>
+      </c>
+      <c r="T3" t="s">
+        <v>87</v>
       </c>
       <c r="U3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="V3" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="W3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -909,10 +903,10 @@
     </row>
     <row r="4" spans="1:27">
       <c r="A4">
-        <v>329</v>
+        <v>396</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C4" t="s">
         <v>35</v>
@@ -921,19 +915,19 @@
         <v>53</v>
       </c>
       <c r="E4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G4">
-        <v>2721</v>
+        <v>2726</v>
       </c>
       <c r="H4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J4" s="1">
         <v>46185</v>
@@ -945,34 +939,28 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N4" s="1">
-        <v>46216</v>
-      </c>
-      <c r="O4" s="1">
-        <v>46216</v>
+        <v>46192</v>
       </c>
       <c r="Q4">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="R4">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S4" t="s">
-        <v>89</v>
-      </c>
-      <c r="T4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="U4" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="V4" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="W4" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -980,10 +968,10 @@
     </row>
     <row r="5" spans="1:27">
       <c r="A5">
-        <v>396</v>
+        <v>313</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C5" t="s">
         <v>36</v>
@@ -992,52 +980,55 @@
         <v>54</v>
       </c>
       <c r="E5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G5">
-        <v>2726</v>
+        <v>2734</v>
       </c>
       <c r="H5" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J5" s="1">
+        <v>46199</v>
+      </c>
+      <c r="K5" s="1">
+        <v>46203</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5" t="s">
+        <v>86</v>
+      </c>
+      <c r="N5" s="1">
+        <v>46214</v>
+      </c>
+      <c r="Q5">
+        <v>4</v>
+      </c>
+      <c r="R5">
+        <v>15</v>
+      </c>
+      <c r="S5" t="s">
         <v>87</v>
       </c>
-      <c r="J5" s="1">
-        <v>46185</v>
-      </c>
-      <c r="K5" s="1">
-        <v>46185</v>
-      </c>
-      <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5" t="s">
+      <c r="T5" t="s">
         <v>88</v>
       </c>
-      <c r="N5" s="1">
-        <v>46192</v>
-      </c>
-      <c r="Q5">
-        <v>25</v>
-      </c>
-      <c r="R5">
-        <v>32</v>
-      </c>
-      <c r="S5" t="s">
-        <v>89</v>
-      </c>
       <c r="U5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="V5" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="W5" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1045,10 +1036,10 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C6" t="s">
         <v>37</v>
@@ -1057,55 +1048,52 @@
         <v>55</v>
       </c>
       <c r="E6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G6">
+        <v>2721</v>
+      </c>
+      <c r="H6" t="s">
         <v>81</v>
       </c>
-      <c r="G6">
-        <v>2734</v>
-      </c>
-      <c r="H6" t="s">
-        <v>83</v>
-      </c>
       <c r="I6" t="s">
+        <v>84</v>
+      </c>
+      <c r="J6" s="1">
+        <v>46205</v>
+      </c>
+      <c r="K6" s="1">
+        <v>46206</v>
+      </c>
+      <c r="L6">
+        <v>1</v>
+      </c>
+      <c r="M6" t="s">
         <v>86</v>
       </c>
-      <c r="J6" s="1">
-        <v>46199</v>
-      </c>
-      <c r="K6" s="1">
-        <v>46203</v>
-      </c>
-      <c r="L6">
-        <v>1</v>
-      </c>
-      <c r="M6" t="s">
-        <v>88</v>
-      </c>
       <c r="N6" s="1">
-        <v>46214</v>
+        <v>46213</v>
       </c>
       <c r="Q6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R6">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="S6" t="s">
-        <v>89</v>
-      </c>
-      <c r="T6" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="U6" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="V6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="W6" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1125,52 +1113,49 @@
         <v>56</v>
       </c>
       <c r="E7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F7" t="s">
+        <v>78</v>
+      </c>
+      <c r="G7">
+        <v>2709</v>
+      </c>
+      <c r="H7" t="s">
         <v>81</v>
       </c>
-      <c r="G7">
-        <v>2721</v>
-      </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>83</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" s="1">
+        <v>46209</v>
+      </c>
+      <c r="K7" s="1">
+        <v>46210</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7" t="s">
+        <v>86</v>
+      </c>
+      <c r="N7" s="1">
+        <v>46241</v>
+      </c>
+      <c r="Q7">
+        <v>-23</v>
+      </c>
+      <c r="R7">
+        <v>8</v>
+      </c>
+      <c r="S7" t="s">
         <v>87</v>
       </c>
-      <c r="J7" s="1">
-        <v>46205</v>
-      </c>
-      <c r="K7" s="1">
-        <v>46206</v>
-      </c>
-      <c r="L7">
-        <v>1</v>
-      </c>
-      <c r="M7" t="s">
-        <v>88</v>
-      </c>
-      <c r="N7" s="1">
-        <v>46213</v>
-      </c>
-      <c r="Q7">
-        <v>4</v>
-      </c>
-      <c r="R7">
-        <v>11</v>
-      </c>
-      <c r="S7" t="s">
-        <v>89</v>
-      </c>
-      <c r="U7" t="s">
-        <v>96</v>
-      </c>
       <c r="V7" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="W7" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1187,22 +1172,22 @@
         <v>39</v>
       </c>
       <c r="D8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E8" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G8">
-        <v>2709</v>
+        <v>2721</v>
       </c>
       <c r="H8" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J8" s="1">
         <v>46209</v>
@@ -1214,25 +1199,25 @@
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N8" s="1">
-        <v>46241</v>
+        <v>46217</v>
       </c>
       <c r="Q8">
-        <v>-24</v>
+        <v>1</v>
       </c>
       <c r="R8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S8" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="V8" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="W8" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1240,10 +1225,10 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C9" t="s">
         <v>40</v>
@@ -1252,22 +1237,22 @@
         <v>57</v>
       </c>
       <c r="E9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G9">
-        <v>2721</v>
+        <v>2719</v>
       </c>
       <c r="H9" t="s">
+        <v>81</v>
+      </c>
+      <c r="I9" t="s">
         <v>83</v>
       </c>
-      <c r="I9" t="s">
-        <v>87</v>
-      </c>
       <c r="J9" s="1">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="K9" s="1">
         <v>46210</v>
@@ -1276,25 +1261,25 @@
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N9" s="1">
-        <v>46217</v>
+        <v>46241</v>
       </c>
       <c r="Q9">
-        <v>0</v>
+        <v>-23</v>
       </c>
       <c r="R9">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S9" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="V9" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="W9" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1302,61 +1287,64 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>685</v>
+        <v>419</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C10" t="s">
         <v>41</v>
       </c>
       <c r="D10" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F10" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G10">
-        <v>2719</v>
+        <v>2723</v>
       </c>
       <c r="H10" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J10" s="1">
         <v>46210</v>
       </c>
       <c r="K10" s="1">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="L10">
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N10" s="1">
-        <v>46241</v>
+        <v>46218</v>
       </c>
       <c r="Q10">
-        <v>-24</v>
+        <v>0</v>
       </c>
       <c r="R10">
         <v>7</v>
       </c>
       <c r="S10" t="s">
-        <v>89</v>
+        <v>87</v>
+      </c>
+      <c r="U10" t="s">
+        <v>94</v>
       </c>
       <c r="V10" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="W10" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1364,34 +1352,34 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>419</v>
+        <v>396</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C11" t="s">
         <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F11" t="s">
+        <v>80</v>
+      </c>
+      <c r="G11">
+        <v>2733</v>
+      </c>
+      <c r="H11" t="s">
         <v>81</v>
       </c>
-      <c r="G11">
-        <v>2723</v>
-      </c>
-      <c r="H11" t="s">
-        <v>83</v>
-      </c>
       <c r="I11" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="J11" s="1">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="K11" s="1">
         <v>46211</v>
@@ -1400,28 +1388,25 @@
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N11" s="1">
-        <v>46218</v>
+        <v>46222</v>
       </c>
       <c r="Q11">
-        <v>-1</v>
+        <v>-4</v>
       </c>
       <c r="R11">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S11" t="s">
-        <v>89</v>
-      </c>
-      <c r="U11" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="V11" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="W11" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1441,49 +1426,52 @@
         <v>59</v>
       </c>
       <c r="E12" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F12" t="s">
+        <v>80</v>
+      </c>
+      <c r="G12">
+        <v>2726</v>
+      </c>
+      <c r="H12" t="s">
         <v>81</v>
       </c>
-      <c r="G12">
-        <v>2733</v>
-      </c>
-      <c r="H12" t="s">
-        <v>83</v>
-      </c>
       <c r="I12" t="s">
+        <v>84</v>
+      </c>
+      <c r="J12" s="1">
+        <v>46212</v>
+      </c>
+      <c r="K12" s="1">
+        <v>46212</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12" t="s">
         <v>86</v>
       </c>
-      <c r="J12" s="1">
-        <v>46211</v>
-      </c>
-      <c r="K12" s="1">
-        <v>46211</v>
-      </c>
-      <c r="L12">
-        <v>1</v>
-      </c>
-      <c r="M12" t="s">
-        <v>88</v>
-      </c>
       <c r="N12" s="1">
-        <v>46222</v>
+        <v>46219</v>
       </c>
       <c r="Q12">
-        <v>-5</v>
+        <v>-1</v>
       </c>
       <c r="R12">
         <v>6</v>
       </c>
       <c r="S12" t="s">
-        <v>89</v>
+        <v>88</v>
+      </c>
+      <c r="U12" t="s">
+        <v>95</v>
       </c>
       <c r="V12" t="s">
+        <v>106</v>
+      </c>
+      <c r="W12" t="s">
         <v>109</v>
-      </c>
-      <c r="W12" t="s">
-        <v>113</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1491,10 +1479,10 @@
     </row>
     <row r="13" spans="1:27">
       <c r="A13">
-        <v>396</v>
+        <v>419</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C13" t="s">
         <v>44</v>
@@ -1503,22 +1491,22 @@
         <v>60</v>
       </c>
       <c r="E13" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F13" t="s">
+        <v>80</v>
+      </c>
+      <c r="G13">
+        <v>2723</v>
+      </c>
+      <c r="H13" t="s">
         <v>81</v>
       </c>
-      <c r="G13">
-        <v>2726</v>
-      </c>
-      <c r="H13" t="s">
-        <v>83</v>
-      </c>
       <c r="I13" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="J13" s="1">
-        <v>46212</v>
+        <v>46211</v>
       </c>
       <c r="K13" s="1">
         <v>46212</v>
@@ -1527,28 +1515,25 @@
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N13" s="1">
         <v>46219</v>
       </c>
       <c r="Q13">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S13" t="s">
-        <v>90</v>
-      </c>
-      <c r="U13" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="V13" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="W13" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1556,10 +1541,10 @@
     </row>
     <row r="14" spans="1:27">
       <c r="A14">
-        <v>419</v>
+        <v>685</v>
       </c>
       <c r="B14" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C14" t="s">
         <v>45</v>
@@ -1568,22 +1553,22 @@
         <v>61</v>
       </c>
       <c r="E14" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F14" t="s">
+        <v>78</v>
+      </c>
+      <c r="G14">
+        <v>2702</v>
+      </c>
+      <c r="H14" t="s">
         <v>81</v>
       </c>
-      <c r="G14">
-        <v>2723</v>
-      </c>
-      <c r="H14" t="s">
+      <c r="I14" t="s">
         <v>83</v>
       </c>
-      <c r="I14" t="s">
-        <v>87</v>
-      </c>
       <c r="J14" s="1">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="K14" s="1">
         <v>46212</v>
@@ -1592,25 +1577,22 @@
         <v>1</v>
       </c>
       <c r="M14" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N14" s="1">
-        <v>46219</v>
+        <v>46243</v>
       </c>
       <c r="Q14">
-        <v>-2</v>
+        <v>-25</v>
       </c>
       <c r="R14">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S14" t="s">
-        <v>89</v>
-      </c>
-      <c r="V14" t="s">
-        <v>111</v>
+        <v>87</v>
       </c>
       <c r="W14" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
@@ -1618,10 +1600,10 @@
     </row>
     <row r="15" spans="1:27">
       <c r="A15">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B15" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C15" t="s">
         <v>46</v>
@@ -1630,46 +1612,52 @@
         <v>62</v>
       </c>
       <c r="E15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F15" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G15">
-        <v>2702</v>
+        <v>2734</v>
       </c>
       <c r="H15" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I15" t="s">
         <v>85</v>
       </c>
       <c r="J15" s="1">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="K15" s="1">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="L15">
         <v>1</v>
       </c>
       <c r="M15" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N15" s="1">
-        <v>46243</v>
+        <v>46224</v>
       </c>
       <c r="Q15">
-        <v>-26</v>
+        <v>-6</v>
       </c>
       <c r="R15">
         <v>5</v>
       </c>
       <c r="S15" t="s">
-        <v>89</v>
+        <v>87</v>
+      </c>
+      <c r="U15" t="s">
+        <v>96</v>
+      </c>
+      <c r="V15" t="s">
+        <v>108</v>
       </c>
       <c r="W15" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
@@ -1689,52 +1677,46 @@
         <v>63</v>
       </c>
       <c r="E16" t="s">
+        <v>75</v>
+      </c>
+      <c r="F16" t="s">
         <v>78</v>
       </c>
-      <c r="F16" t="s">
-        <v>80</v>
-      </c>
       <c r="G16">
-        <v>2734</v>
+        <v>2736</v>
       </c>
       <c r="H16" t="s">
+        <v>82</v>
+      </c>
+      <c r="I16" t="s">
         <v>83</v>
       </c>
-      <c r="I16" t="s">
+      <c r="J16" s="1">
+        <v>46216</v>
+      </c>
+      <c r="K16" s="1">
+        <v>46217</v>
+      </c>
+      <c r="L16">
+        <v>1</v>
+      </c>
+      <c r="M16" t="s">
         <v>86</v>
       </c>
-      <c r="J16" s="1">
-        <v>46213</v>
-      </c>
-      <c r="K16" s="1">
-        <v>46213</v>
-      </c>
-      <c r="L16">
-        <v>1</v>
-      </c>
-      <c r="M16" t="s">
-        <v>88</v>
-      </c>
       <c r="N16" s="1">
-        <v>46224</v>
+        <v>46248</v>
       </c>
       <c r="Q16">
-        <v>-7</v>
+        <v>-30</v>
       </c>
       <c r="R16">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="S16" t="s">
-        <v>89</v>
-      </c>
-      <c r="U16" t="s">
-        <v>99</v>
-      </c>
-      <c r="V16" t="s">
-        <v>112</v>
+        <v>87</v>
       </c>
       <c r="W16" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="AA16" t="b">
         <v>1</v>
@@ -1742,10 +1724,10 @@
     </row>
     <row r="17" spans="1:27">
       <c r="A17">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B17" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C17" t="s">
         <v>48</v>
@@ -1757,16 +1739,16 @@
         <v>77</v>
       </c>
       <c r="F17" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G17">
-        <v>2736</v>
+        <v>2729</v>
       </c>
       <c r="H17" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="I17" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="J17" s="1">
         <v>46216</v>
@@ -1778,22 +1760,22 @@
         <v>1</v>
       </c>
       <c r="M17" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N17" s="1">
         <v>46248</v>
       </c>
       <c r="Q17">
-        <v>-31</v>
+        <v>-30</v>
       </c>
       <c r="R17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S17" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="W17" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="AA17" t="b">
         <v>1</v>
@@ -1801,34 +1783,34 @@
     </row>
     <row r="18" spans="1:27">
       <c r="A18">
-        <v>685</v>
+        <v>386</v>
       </c>
       <c r="B18" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C18" t="s">
         <v>49</v>
       </c>
       <c r="D18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E18" t="s">
+        <v>77</v>
+      </c>
+      <c r="F18" t="s">
         <v>79</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18">
+        <v>2743</v>
+      </c>
+      <c r="H18" t="s">
         <v>82</v>
-      </c>
-      <c r="G18">
-        <v>2729</v>
-      </c>
-      <c r="H18" t="s">
-        <v>84</v>
       </c>
       <c r="I18" t="s">
         <v>85</v>
       </c>
       <c r="J18" s="1">
-        <v>46216</v>
+        <v>46213</v>
       </c>
       <c r="K18" s="1">
         <v>46217</v>
@@ -1837,22 +1819,22 @@
         <v>1</v>
       </c>
       <c r="M18" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N18" s="1">
-        <v>46248</v>
+        <v>46228</v>
       </c>
       <c r="Q18">
-        <v>-31</v>
+        <v>-10</v>
       </c>
       <c r="R18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S18" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="W18" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="AA18" t="b">
         <v>1</v>
@@ -1860,46 +1842,46 @@
     </row>
     <row r="19" spans="1:27">
       <c r="A19">
-        <v>386</v>
+        <v>685</v>
       </c>
       <c r="B19" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C19" t="s">
         <v>50</v>
       </c>
       <c r="D19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E19" t="s">
+        <v>77</v>
+      </c>
+      <c r="F19" t="s">
         <v>79</v>
       </c>
-      <c r="F19" t="s">
+      <c r="G19">
+        <v>2722</v>
+      </c>
+      <c r="H19" t="s">
         <v>82</v>
       </c>
-      <c r="G19">
-        <v>2743</v>
-      </c>
-      <c r="H19" t="s">
-        <v>84</v>
-      </c>
       <c r="I19" t="s">
+        <v>85</v>
+      </c>
+      <c r="J19" s="1">
+        <v>46217</v>
+      </c>
+      <c r="K19" s="1">
+        <v>46218</v>
+      </c>
+      <c r="L19">
+        <v>1</v>
+      </c>
+      <c r="M19" t="s">
         <v>86</v>
       </c>
-      <c r="J19" s="1">
-        <v>46213</v>
-      </c>
-      <c r="K19" s="1">
-        <v>46217</v>
-      </c>
-      <c r="L19">
-        <v>1</v>
-      </c>
-      <c r="M19" t="s">
-        <v>88</v>
-      </c>
       <c r="N19" s="1">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="Q19">
         <v>-11</v>
@@ -1908,10 +1890,10 @@
         <v>0</v>
       </c>
       <c r="S19" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="W19" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="AA19" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (16/07/2026 16:03)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="124">
   <si>
     <t>om_emg</t>
   </si>
@@ -115,6 +115,9 @@
     <t>BACO</t>
   </si>
   <si>
+    <t>BACG</t>
+  </si>
+  <si>
     <t>313260017747</t>
   </si>
   <si>
@@ -130,9 +133,6 @@
     <t>329260019179</t>
   </si>
   <si>
-    <t>329260019180</t>
-  </si>
-  <si>
     <t>329260019181</t>
   </si>
   <si>
@@ -169,6 +169,18 @@
     <t>685260012377</t>
   </si>
   <si>
+    <t>685260012387</t>
+  </si>
+  <si>
+    <t>685260012394</t>
+  </si>
+  <si>
+    <t>685260012395</t>
+  </si>
+  <si>
+    <t>690260002487</t>
+  </si>
+  <si>
     <t>1214134-1</t>
   </si>
   <si>
@@ -211,6 +223,18 @@
     <t>C611008-0101</t>
   </si>
   <si>
+    <t>066-3084-32</t>
+  </si>
+  <si>
+    <t>3011755</t>
+  </si>
+  <si>
+    <t>2611024-1</t>
+  </si>
+  <si>
+    <t>850C86-2</t>
+  </si>
+  <si>
     <t>BELLCRANK ASSY</t>
   </si>
   <si>
@@ -250,6 +274,18 @@
     <t>ALTERNATOR CONTROL U</t>
   </si>
   <si>
+    <t>IND RDR 2000 IN-182A</t>
+  </si>
+  <si>
+    <t>INSULATION BLANKET,T</t>
+  </si>
+  <si>
+    <t>WINDOW</t>
+  </si>
+  <si>
+    <t>TIRE,PNEUMATIC,AIRC</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -289,7 +325,7 @@
     <t>Volume retirado na loja GOLLOG - BSB por tanise Assis em 03/07/2026 - Godoy 08/07/2026. Recibo não se encontra na Pasta do DRIVE. Godoy 08/07/2026.</t>
   </si>
   <si>
-    <t>Item retirado para atender o C-98 2731. Ramon 15/06/26.</t>
+    <t>Item retirado para atender o C-98 2731. Ramon 15/06/26. AWB 12746187256 - volume retirado na loja GOLLOG - BEL por bispo em 13/07. Godoy 16/07/26.</t>
   </si>
   <si>
     <t>Retirado para atender a Anv 2740 - Godoy 30/06/26. AWB 12745953832 - Volume retirado na loja GOLLOG - QMA por Kleyton em 13/07/26. Godoy 15/07/26.</t>
@@ -301,12 +337,15 @@
     <t>AWB 12745918331 volume retirado na loja GOLLOG - BEL por bispo em 10/07/2026 - Godoy 13/07/2026.</t>
   </si>
   <si>
-    <t>Cedeu o item para o C-98 2721. Ramon 09/07/26. AWB 12746175415 - 2 volumes retirados na loja GOLLOG - BEL por bispo em 13/07/26. Godoy 15/07/26.</t>
+    <t>Cedeu o item para o C-98 2721. Ramon 09/07/26. AWB 12746175415 - 2 volumes retirados na loja GOLLOG - BEL por bispo em 13/07/26. Godoy 15/07/26. Vee One, não temos o recibo assinado. Godoy 16/07/26.</t>
   </si>
   <si>
     <t>Cedeu o item para o C-98 2738. Godoy 13/07/26</t>
   </si>
   <si>
+    <t>Vee One preferiu atender a demanda com estoque da empresa. Godoy 16/07/26.</t>
+  </si>
+  <si>
     <t>Foi solicitado via email no dia 02-03-2 o atendimento do item com estoque FAB. Claudio -02-03-26 - Em resposta, a coordenadoria disse que o estque seria insuficiente. Foi verificado que na T.O da ANV o QPA para esse item são 2 EA, solicitei confirmação. - Cláudio -02-03-2026. Solicitado o cancelamento da emergência em função da quantidade cedida ao 2733 ter sido de 01ea. Considerando o QPA 02 ea. Encontra-se em tratativa junto a fiscalização e o gestor do contrato conforme mensagem de e-mail de 05/03. - SOLICITAÇÃO E-C98-26047.Colocado pedido AOG Textron WB0003068789 - previsão de entrega 60 dias em média. Os demais fornecedores informaram não ter em estoque ou não possuírem a certificação necessária da peça.</t>
   </si>
   <si>
@@ -341,6 +380,9 @@
   </si>
   <si>
     <t>Será atendido via estoque V1. ATZ 13/07 - material em transito recibo 568/FAB/26 AWB 12746855476 DPE 17/07/2026</t>
+  </si>
+  <si>
+    <t>Colocado pedido Textron WB0003089604 - previsão de entrega Miami 15/07</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -679,7 +721,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA19"/>
+  <dimension ref="A1:AA22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -773,25 +815,25 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="E2" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="F2" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="G2">
         <v>2730</v>
       </c>
       <c r="H2" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="I2" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="J2" s="1">
         <v>46076</v>
@@ -803,28 +845,28 @@
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="N2" s="1">
         <v>46111</v>
       </c>
       <c r="Q2">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="R2">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="S2" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="U2" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="V2" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="W2" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -838,25 +880,25 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E3" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="F3" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="G3">
         <v>2721</v>
       </c>
       <c r="H3" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="I3" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="J3" s="1">
         <v>46185</v>
@@ -868,7 +910,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="N3" s="1">
         <v>46216</v>
@@ -877,25 +919,25 @@
         <v>46216</v>
       </c>
       <c r="Q3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R3">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="S3" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="T3" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="U3" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="V3" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="W3" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -909,25 +951,25 @@
         <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E4" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="F4" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="G4">
         <v>2726</v>
       </c>
       <c r="H4" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="I4" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="J4" s="1">
         <v>46185</v>
@@ -939,28 +981,31 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="N4" s="1">
         <v>46192</v>
       </c>
+      <c r="O4" s="1">
+        <v>46216</v>
+      </c>
       <c r="Q4">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="R4">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="S4" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="U4" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="V4" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="W4" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -974,25 +1019,25 @@
         <v>27</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="E5" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="F5" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="G5">
         <v>2734</v>
       </c>
       <c r="H5" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="I5" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="J5" s="1">
         <v>46199</v>
@@ -1004,31 +1049,31 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="N5" s="1">
         <v>46214</v>
       </c>
       <c r="Q5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R5">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S5" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="T5" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="U5" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="V5" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="W5" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1042,25 +1087,25 @@
         <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D6" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="E6" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="F6" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="G6">
         <v>2721</v>
       </c>
       <c r="H6" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="I6" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="J6" s="1">
         <v>46205</v>
@@ -1072,28 +1117,31 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="N6" s="1">
         <v>46213</v>
       </c>
+      <c r="O6" s="1">
+        <v>46212</v>
+      </c>
       <c r="Q6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R6">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S6" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="U6" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="V6" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
       <c r="W6" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1107,25 +1155,25 @@
         <v>28</v>
       </c>
       <c r="C7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D7" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="E7" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="F7" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="G7">
-        <v>2709</v>
+        <v>2721</v>
       </c>
       <c r="H7" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="I7" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="J7" s="1">
         <v>46209</v>
@@ -1137,25 +1185,28 @@
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="N7" s="1">
-        <v>46241</v>
+        <v>46217</v>
+      </c>
+      <c r="O7" s="1">
+        <v>46216</v>
       </c>
       <c r="Q7">
-        <v>-23</v>
+        <v>2</v>
       </c>
       <c r="R7">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S7" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="V7" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="W7" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1163,34 +1214,34 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D8" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="E8" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="F8" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="G8">
-        <v>2721</v>
+        <v>2719</v>
       </c>
       <c r="H8" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="I8" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="J8" s="1">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="K8" s="1">
         <v>46210</v>
@@ -1199,25 +1250,28 @@
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="N8" s="1">
-        <v>46217</v>
+        <v>46241</v>
+      </c>
+      <c r="O8" s="1">
+        <v>46238</v>
       </c>
       <c r="Q8">
-        <v>1</v>
+        <v>-22</v>
       </c>
       <c r="R8">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S8" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="V8" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="W8" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1225,61 +1279,67 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9">
-        <v>685</v>
+        <v>419</v>
       </c>
       <c r="B9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E9" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="F9" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="G9">
-        <v>2719</v>
+        <v>2723</v>
       </c>
       <c r="H9" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="I9" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="J9" s="1">
         <v>46210</v>
       </c>
       <c r="K9" s="1">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="L9">
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="N9" s="1">
-        <v>46241</v>
+        <v>46218</v>
+      </c>
+      <c r="O9" s="1">
+        <v>46213</v>
       </c>
       <c r="Q9">
-        <v>-23</v>
+        <v>1</v>
       </c>
       <c r="R9">
         <v>8</v>
       </c>
       <c r="S9" t="s">
-        <v>87</v>
+        <v>99</v>
+      </c>
+      <c r="U9" t="s">
+        <v>106</v>
       </c>
       <c r="V9" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="W9" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1287,34 +1347,34 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>419</v>
+        <v>396</v>
       </c>
       <c r="B10" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="E10" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="F10" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="G10">
-        <v>2723</v>
+        <v>2733</v>
       </c>
       <c r="H10" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="I10" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="J10" s="1">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="K10" s="1">
         <v>46211</v>
@@ -1323,28 +1383,28 @@
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="N10" s="1">
-        <v>46218</v>
+        <v>46222</v>
+      </c>
+      <c r="O10" s="1">
+        <v>46237</v>
       </c>
       <c r="Q10">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="R10">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S10" t="s">
-        <v>87</v>
-      </c>
-      <c r="U10" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="V10" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="W10" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1358,55 +1418,61 @@
         <v>29</v>
       </c>
       <c r="C11" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D11" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="E11" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="F11" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="G11">
-        <v>2733</v>
+        <v>2726</v>
       </c>
       <c r="H11" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="I11" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="J11" s="1">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="K11" s="1">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="L11">
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="N11" s="1">
-        <v>46222</v>
+        <v>46219</v>
+      </c>
+      <c r="O11" s="1">
+        <v>46216</v>
       </c>
       <c r="Q11">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="R11">
         <v>7</v>
       </c>
       <c r="S11" t="s">
-        <v>87</v>
+        <v>100</v>
+      </c>
+      <c r="U11" t="s">
+        <v>107</v>
       </c>
       <c r="V11" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="W11" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1414,34 +1480,34 @@
     </row>
     <row r="12" spans="1:27">
       <c r="A12">
-        <v>396</v>
+        <v>419</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C12" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D12" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="E12" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="F12" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="G12">
-        <v>2726</v>
+        <v>2723</v>
       </c>
       <c r="H12" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="I12" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="J12" s="1">
-        <v>46212</v>
+        <v>46211</v>
       </c>
       <c r="K12" s="1">
         <v>46212</v>
@@ -1450,28 +1516,28 @@
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="N12" s="1">
         <v>46219</v>
       </c>
+      <c r="O12" s="1">
+        <v>46237</v>
+      </c>
       <c r="Q12">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R12">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S12" t="s">
-        <v>88</v>
-      </c>
-      <c r="U12" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="V12" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="W12" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1479,34 +1545,34 @@
     </row>
     <row r="13" spans="1:27">
       <c r="A13">
-        <v>419</v>
+        <v>685</v>
       </c>
       <c r="B13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D13" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="E13" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="F13" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G13">
-        <v>2723</v>
+        <v>2702</v>
       </c>
       <c r="H13" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="I13" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="J13" s="1">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="K13" s="1">
         <v>46212</v>
@@ -1515,25 +1581,22 @@
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="N13" s="1">
-        <v>46219</v>
+        <v>46243</v>
       </c>
       <c r="Q13">
-        <v>-1</v>
+        <v>-24</v>
       </c>
       <c r="R13">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S13" t="s">
-        <v>87</v>
-      </c>
-      <c r="V13" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="W13" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1541,58 +1604,64 @@
     </row>
     <row r="14" spans="1:27">
       <c r="A14">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B14" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D14" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="E14" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="F14" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="G14">
-        <v>2702</v>
+        <v>2734</v>
       </c>
       <c r="H14" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="I14" t="s">
-        <v>83</v>
+        <v>97</v>
       </c>
       <c r="J14" s="1">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="K14" s="1">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="L14">
         <v>1</v>
       </c>
       <c r="M14" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="N14" s="1">
-        <v>46243</v>
+        <v>46224</v>
       </c>
       <c r="Q14">
-        <v>-25</v>
+        <v>-5</v>
       </c>
       <c r="R14">
         <v>6</v>
       </c>
       <c r="S14" t="s">
-        <v>87</v>
+        <v>99</v>
+      </c>
+      <c r="U14" t="s">
+        <v>108</v>
+      </c>
+      <c r="V14" t="s">
+        <v>121</v>
       </c>
       <c r="W14" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
@@ -1606,58 +1675,52 @@
         <v>27</v>
       </c>
       <c r="C15" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D15" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="E15" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="F15" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="G15">
-        <v>2734</v>
+        <v>2736</v>
       </c>
       <c r="H15" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="I15" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="J15" s="1">
-        <v>46213</v>
+        <v>46216</v>
       </c>
       <c r="K15" s="1">
-        <v>46213</v>
+        <v>46217</v>
       </c>
       <c r="L15">
         <v>1</v>
       </c>
       <c r="M15" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="N15" s="1">
-        <v>46224</v>
+        <v>46248</v>
       </c>
       <c r="Q15">
-        <v>-6</v>
+        <v>-29</v>
       </c>
       <c r="R15">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="S15" t="s">
-        <v>87</v>
-      </c>
-      <c r="U15" t="s">
-        <v>96</v>
-      </c>
-      <c r="V15" t="s">
-        <v>108</v>
+        <v>99</v>
       </c>
       <c r="W15" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
@@ -1665,31 +1728,31 @@
     </row>
     <row r="16" spans="1:27">
       <c r="A16">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B16" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C16" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D16" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="E16" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="F16" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="G16">
-        <v>2736</v>
+        <v>2729</v>
       </c>
       <c r="H16" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="I16" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="J16" s="1">
         <v>46216</v>
@@ -1701,22 +1764,22 @@
         <v>1</v>
       </c>
       <c r="M16" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="N16" s="1">
         <v>46248</v>
       </c>
       <c r="Q16">
-        <v>-30</v>
+        <v>-29</v>
       </c>
       <c r="R16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S16" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="W16" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="AA16" t="b">
         <v>1</v>
@@ -1724,34 +1787,34 @@
     </row>
     <row r="17" spans="1:27">
       <c r="A17">
-        <v>685</v>
+        <v>386</v>
       </c>
       <c r="B17" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C17" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D17" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E17" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="F17" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="G17">
-        <v>2729</v>
+        <v>2743</v>
       </c>
       <c r="H17" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="I17" t="s">
-        <v>83</v>
+        <v>97</v>
       </c>
       <c r="J17" s="1">
-        <v>46216</v>
+        <v>46213</v>
       </c>
       <c r="K17" s="1">
         <v>46217</v>
@@ -1760,22 +1823,25 @@
         <v>1</v>
       </c>
       <c r="M17" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="N17" s="1">
-        <v>46248</v>
+        <v>46228</v>
       </c>
       <c r="Q17">
-        <v>-30</v>
+        <v>-9</v>
       </c>
       <c r="R17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S17" t="s">
-        <v>87</v>
+        <v>99</v>
+      </c>
+      <c r="V17" t="s">
+        <v>122</v>
       </c>
       <c r="W17" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="AA17" t="b">
         <v>1</v>
@@ -1783,46 +1849,46 @@
     </row>
     <row r="18" spans="1:27">
       <c r="A18">
-        <v>386</v>
+        <v>685</v>
       </c>
       <c r="B18" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C18" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D18" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E18" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="F18" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="G18">
-        <v>2743</v>
+        <v>2722</v>
       </c>
       <c r="H18" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="I18" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="J18" s="1">
-        <v>46213</v>
+        <v>46217</v>
       </c>
       <c r="K18" s="1">
-        <v>46217</v>
+        <v>46218</v>
       </c>
       <c r="L18">
         <v>1</v>
       </c>
       <c r="M18" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="N18" s="1">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="Q18">
         <v>-10</v>
@@ -1831,10 +1897,10 @@
         <v>1</v>
       </c>
       <c r="S18" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="W18" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="AA18" t="b">
         <v>1</v>
@@ -1848,28 +1914,28 @@
         <v>30</v>
       </c>
       <c r="C19" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D19" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="E19" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="F19" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="G19">
         <v>2722</v>
       </c>
       <c r="H19" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="I19" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="J19" s="1">
-        <v>46217</v>
+        <v>46219</v>
       </c>
       <c r="K19" s="1">
         <v>46218</v>
@@ -1878,24 +1944,204 @@
         <v>1</v>
       </c>
       <c r="M19" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="N19" s="1">
-        <v>46229</v>
+        <v>46249</v>
       </c>
       <c r="Q19">
+        <v>-30</v>
+      </c>
+      <c r="R19">
+        <v>1</v>
+      </c>
+      <c r="S19" t="s">
+        <v>99</v>
+      </c>
+      <c r="W19" t="s">
+        <v>123</v>
+      </c>
+      <c r="AA19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:27">
+      <c r="A20">
+        <v>685</v>
+      </c>
+      <c r="B20" t="s">
+        <v>30</v>
+      </c>
+      <c r="C20" t="s">
+        <v>52</v>
+      </c>
+      <c r="D20" t="s">
+        <v>70</v>
+      </c>
+      <c r="E20" t="s">
+        <v>87</v>
+      </c>
+      <c r="F20" t="s">
+        <v>91</v>
+      </c>
+      <c r="G20">
+        <v>2729</v>
+      </c>
+      <c r="H20" t="s">
+        <v>94</v>
+      </c>
+      <c r="I20" t="s">
+        <v>97</v>
+      </c>
+      <c r="J20" s="1">
+        <v>46219</v>
+      </c>
+      <c r="K20" s="1">
+        <v>46219</v>
+      </c>
+      <c r="L20">
+        <v>1</v>
+      </c>
+      <c r="M20" t="s">
+        <v>98</v>
+      </c>
+      <c r="N20" s="1">
+        <v>46230</v>
+      </c>
+      <c r="Q20">
         <v>-11</v>
       </c>
-      <c r="R19">
+      <c r="R20">
         <v>0</v>
       </c>
-      <c r="S19" t="s">
-        <v>87</v>
-      </c>
-      <c r="W19" t="s">
+      <c r="S20" t="s">
+        <v>99</v>
+      </c>
+      <c r="W20" t="s">
+        <v>123</v>
+      </c>
+      <c r="AA20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:27">
+      <c r="A21">
+        <v>685</v>
+      </c>
+      <c r="B21" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21" t="s">
+        <v>53</v>
+      </c>
+      <c r="D21" t="s">
+        <v>71</v>
+      </c>
+      <c r="E21" t="s">
+        <v>88</v>
+      </c>
+      <c r="F21" t="s">
+        <v>90</v>
+      </c>
+      <c r="G21">
+        <v>2703</v>
+      </c>
+      <c r="H21" t="s">
+        <v>94</v>
+      </c>
+      <c r="I21" t="s">
+        <v>95</v>
+      </c>
+      <c r="J21" s="1">
+        <v>46219</v>
+      </c>
+      <c r="K21" s="1">
+        <v>46220</v>
+      </c>
+      <c r="L21">
+        <v>2</v>
+      </c>
+      <c r="M21" t="s">
+        <v>98</v>
+      </c>
+      <c r="N21" s="1">
+        <v>46251</v>
+      </c>
+      <c r="Q21">
+        <v>-32</v>
+      </c>
+      <c r="R21">
+        <v>-1</v>
+      </c>
+      <c r="S21" t="s">
+        <v>100</v>
+      </c>
+      <c r="W21" t="s">
+        <v>123</v>
+      </c>
+      <c r="AA21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:27">
+      <c r="A22">
+        <v>690</v>
+      </c>
+      <c r="B22" t="s">
+        <v>33</v>
+      </c>
+      <c r="C22" t="s">
+        <v>54</v>
+      </c>
+      <c r="D22" t="s">
+        <v>72</v>
+      </c>
+      <c r="E22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F22" t="s">
+        <v>90</v>
+      </c>
+      <c r="G22">
+        <v>2727</v>
+      </c>
+      <c r="H22" t="s">
+        <v>94</v>
+      </c>
+      <c r="I22" t="s">
+        <v>96</v>
+      </c>
+      <c r="J22" s="1">
+        <v>46219</v>
+      </c>
+      <c r="K22" s="1">
+        <v>46221</v>
+      </c>
+      <c r="L22">
+        <v>1</v>
+      </c>
+      <c r="M22" t="s">
+        <v>98</v>
+      </c>
+      <c r="N22" s="1">
+        <v>46228</v>
+      </c>
+      <c r="Q22">
+        <v>-9</v>
+      </c>
+      <c r="R22">
+        <v>-2</v>
+      </c>
+      <c r="S22" t="s">
+        <v>100</v>
+      </c>
+      <c r="U22" t="s">
         <v>109</v>
       </c>
-      <c r="AA19" t="b">
+      <c r="W22" t="s">
+        <v>123</v>
+      </c>
+      <c r="AA22" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (17/07/2026 16:02)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="129">
   <si>
     <t>om_emg</t>
   </si>
@@ -181,6 +181,9 @@
     <t>690260002487</t>
   </si>
   <si>
+    <t>685260012396</t>
+  </si>
+  <si>
     <t>1214134-1</t>
   </si>
   <si>
@@ -235,6 +238,9 @@
     <t>850C86-2</t>
   </si>
   <si>
+    <t>540-1407-4</t>
+  </si>
+  <si>
     <t>BELLCRANK ASSY</t>
   </si>
   <si>
@@ -286,6 +292,9 @@
     <t>TIRE,PNEUMATIC,AIRC</t>
   </si>
   <si>
+    <t>VALVE,BLEED,TURBINEE</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -298,18 +307,21 @@
     <t>Providência tomada</t>
   </si>
   <si>
+    <t>Expedido total</t>
+  </si>
+  <si>
     <t>Aguardando solução</t>
   </si>
   <si>
+    <t>IPLR</t>
+  </si>
+  <si>
     <t>ANCE</t>
   </si>
   <si>
     <t>AIFP</t>
   </si>
   <si>
-    <t>IPLR</t>
-  </si>
-  <si>
     <t>EA</t>
   </si>
   <si>
@@ -325,7 +337,7 @@
     <t>Volume retirado na loja GOLLOG - BSB por tanise Assis em 03/07/2026 - Godoy 08/07/2026. Recibo não se encontra na Pasta do DRIVE. Godoy 08/07/2026.</t>
   </si>
   <si>
-    <t>Item retirado para atender o C-98 2731. Ramon 15/06/26. AWB 12746187256 - volume retirado na loja GOLLOG - BEL por bispo em 13/07. Godoy 16/07/26.</t>
+    <t>Item retirado para atender o C-98 2731. Ramon 15/06/26. AWB 12746187256 - volume retirado na loja GOLLOG - BEL por bispo em 13/07. Godoy 16/07/26. Recibo não se encontra na Pasta do DRIVE. Godoy 17/07/2026.</t>
   </si>
   <si>
     <t>Retirado para atender a Anv 2740 - Godoy 30/06/26. AWB 12745953832 - Volume retirado na loja GOLLOG - QMA por Kleyton em 13/07/26. Godoy 15/07/26.</t>
@@ -334,7 +346,7 @@
     <t>Recibo não se encontra na Pasta do DRIVE. Godoy 08/07/2026.</t>
   </si>
   <si>
-    <t>AWB 12745918331 volume retirado na loja GOLLOG - BEL por bispo em 10/07/2026 - Godoy 13/07/2026.</t>
+    <t>AWB 12745918331 volume retirado na loja GOLLOG - BEL por bispo em 10/07/2026 - Godoy 13/07/2026. Recibo não se encontra na Pasta do DRIVE. Godoy 17/07/2026.</t>
   </si>
   <si>
     <t>Cedeu o item para o C-98 2721. Ramon 09/07/26. AWB 12746175415 - 2 volumes retirados na loja GOLLOG - BEL por bispo em 13/07/26. Godoy 15/07/26. Vee One, não temos o recibo assinado. Godoy 16/07/26.</t>
@@ -352,7 +364,7 @@
     <t>Colocado pedido na Textron IJ17507011. Previsão de entrega em Miami 17/06. Carga recepcionada no GIG 24/06. Canal verde dia 26/06. DPE V1 29/06. Verificar entrega do item. ATZ 30/06 - MATERIAL EM RECEBIMENTO V1 30-06-2026 - MATERIAL EM PROCESSO DE ENVIO RECIBO 524/FAB/26 ATZ RC 30-06-2026 - MATERIAL EM TRANSITO - AWB 12744330731 DPE 03/07/2026 - MATERIAL RECEBIDO POR tanise Assis RG 14807641751 DIA 03/07/2026</t>
   </si>
   <si>
-    <t>04 ea recolhidos para a V1, chegada dos itens dia 23/06/2026. Itens não tem oficina no Brasil, terá que ser feito Exchange rc 23/06 - MATERIAL ADQUIRIDO FORNECEDOR TEXTRON -WB0003073549 Inovice IJ17534800 DPE AGS Miami 29/6/2026 ate 10 30AM - AIR EXPORT HOUSE: 00004046 de 30/6/2026 Chegou no GIGRJ em 01/7/26 para Desembaraço - ATZ Marcio 3/7/26 CANAL VERDE EM 7/7/26 entregue V1 em 8/7/26 ATZ Marcio 9/7/26 - MATERIAL EM TRANSITO - RECIBO 560/FAB/26 AWB - 12746187256 DPE 13/07/2026</t>
+    <t>04 ea recolhidos para a V1, chegada dos itens dia 23/06/2026. Itens não tem oficina no Brasil, terá que ser feito  Exchange rc 23/06 - MATERIAL ADQUIRIDO FORNECEDOR TEXTRON -WB0003073549 Inovice IJ17534800 DPE AGS  Miami 29/6/2026 ate 10 30AM - AIR EXPORT HOUSE: 00004046 de 30/6/2026 Chegou no GIGRJ em 01/7/26 para  Desembaraço - ATZ Marcio 3/7/26 CANAL VERDE EM 7/7/26 entregue V1 em 8/7/26 ATZ Marcio 9/7/26 - MATERIAL EM TRANSITO - RECIBO 560/FAB/26 AWB - 12746187256 DPE 13/07/2026</t>
   </si>
   <si>
     <t>Efetuada a Compra em SP na Jet Avionics, aguardando confirmar unidade em estoque para liberação do item para a Veeone 01/7/2026 14:15 Marcio - DECLINADO pela JET AVIONICS, colocado Pedido TEXTRON Confirmation Number: WB0003077522 de 01/7/2026 Invoice IJ17546081 as 15:08PM Previsao DPE AGS Miami 02/7/2026 - PRE ALERTA do VOO de 3/7/2026 HAWB4065 - CANAL VERDE - ATZ Mayara 7/7/26 14:34 (MATERIAL EM SEPARAÇÃO - SUP V1 JPA) Atlz Lucas 08/07 14:01 - MATERIAL EM TRANSITO - RECIBO 556/FAB/26 - AWB 12745953832 DPE 14/07/2026</t>
@@ -379,10 +391,13 @@
     <t>Aguardando o retorno dos subcomponentes removidos da unidade para ser enviado a oficiana para aplicação na unidade Prazo apos aprovação 10 dias ATZ Marcio 9/7/26 14 53</t>
   </si>
   <si>
-    <t>Será atendido via estoque V1. ATZ 13/07 - material em transito recibo 568/FAB/26 AWB 12746855476 DPE 17/07/2026</t>
-  </si>
-  <si>
-    <t>Colocado pedido Textron WB0003089604 - previsão de entrega Miami 15/07</t>
+    <t>Colocado pedido junto ao fornecedor AEROBASE, aguardando pagamento proforma. ATZ 16/07</t>
+  </si>
+  <si>
+    <t>Será atendido via estoque V1. ATZ 13/07 - material em transito recibo 568/FAB/26 AWB 12746855476 DPE 17/07/2026 - DPE ATT 16/07/2026 - Recibo enviado dia 16/07/2026</t>
+  </si>
+  <si>
+    <t>ENVIADO NO DIA 10-07-26 AWB 127-4640 3125 - material recebido dia 15/07/2026 - nota fiscal enviada dia 15/07/2026</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -721,7 +736,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA22"/>
+  <dimension ref="A1:AA23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -818,22 +833,22 @@
         <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="G2">
         <v>2730</v>
       </c>
       <c r="H2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="I2" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="J2" s="1">
         <v>46076</v>
@@ -845,28 +860,28 @@
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="N2" s="1">
-        <v>46111</v>
+        <v>46091</v>
       </c>
       <c r="Q2">
-        <v>108</v>
+        <v>129</v>
       </c>
       <c r="R2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="S2" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="U2" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="V2" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="W2" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -883,22 +898,22 @@
         <v>35</v>
       </c>
       <c r="D3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="G3">
         <v>2721</v>
       </c>
       <c r="H3" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="I3" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="J3" s="1">
         <v>46185</v>
@@ -910,7 +925,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="N3" s="1">
         <v>46216</v>
@@ -919,25 +934,25 @@
         <v>46216</v>
       </c>
       <c r="Q3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R3">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S3" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="T3" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="U3" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="V3" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="W3" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -954,22 +969,22 @@
         <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F4" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G4">
         <v>2726</v>
       </c>
       <c r="H4" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="I4" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="J4" s="1">
         <v>46185</v>
@@ -981,7 +996,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="N4" s="1">
         <v>46192</v>
@@ -990,22 +1005,22 @@
         <v>46216</v>
       </c>
       <c r="Q4">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R4">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S4" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="U4" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="V4" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="W4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -1022,22 +1037,22 @@
         <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F5" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="G5">
         <v>2734</v>
       </c>
       <c r="H5" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="I5" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="J5" s="1">
         <v>46199</v>
@@ -1049,31 +1064,31 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="N5" s="1">
         <v>46214</v>
       </c>
       <c r="Q5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R5">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="S5" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="T5" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="U5" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="V5" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="W5" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1090,22 +1105,22 @@
         <v>38</v>
       </c>
       <c r="D6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E6" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F6" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="G6">
         <v>2721</v>
       </c>
       <c r="H6" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="I6" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="J6" s="1">
         <v>46205</v>
@@ -1117,7 +1132,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="N6" s="1">
         <v>46213</v>
@@ -1126,22 +1141,22 @@
         <v>46212</v>
       </c>
       <c r="Q6">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R6">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S6" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="U6" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="V6" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="W6" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1158,22 +1173,22 @@
         <v>39</v>
       </c>
       <c r="D7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E7" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F7" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="G7">
         <v>2721</v>
       </c>
       <c r="H7" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="I7" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="J7" s="1">
         <v>46209</v>
@@ -1185,7 +1200,7 @@
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="N7" s="1">
         <v>46217</v>
@@ -1194,19 +1209,19 @@
         <v>46216</v>
       </c>
       <c r="Q7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R7">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="S7" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="V7" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="W7" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1223,22 +1238,22 @@
         <v>40</v>
       </c>
       <c r="D8" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E8" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="F8" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G8">
         <v>2719</v>
       </c>
       <c r="H8" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="I8" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="J8" s="1">
         <v>46210</v>
@@ -1250,7 +1265,7 @@
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="N8" s="1">
         <v>46241</v>
@@ -1259,19 +1274,19 @@
         <v>46238</v>
       </c>
       <c r="Q8">
-        <v>-22</v>
+        <v>-21</v>
       </c>
       <c r="R8">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="S8" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="V8" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="W8" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1288,22 +1303,22 @@
         <v>41</v>
       </c>
       <c r="D9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E9" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F9" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="G9">
         <v>2723</v>
       </c>
       <c r="H9" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="I9" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="J9" s="1">
         <v>46210</v>
@@ -1315,7 +1330,7 @@
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="N9" s="1">
         <v>46218</v>
@@ -1324,22 +1339,22 @@
         <v>46213</v>
       </c>
       <c r="Q9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S9" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="U9" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="V9" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="W9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1356,22 +1371,22 @@
         <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E10" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F10" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="G10">
         <v>2733</v>
       </c>
       <c r="H10" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="I10" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="J10" s="1">
         <v>46211</v>
@@ -1383,7 +1398,7 @@
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="N10" s="1">
         <v>46222</v>
@@ -1392,19 +1407,19 @@
         <v>46237</v>
       </c>
       <c r="Q10">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R10">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S10" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="V10" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="W10" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1421,22 +1436,22 @@
         <v>43</v>
       </c>
       <c r="D11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E11" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F11" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="G11">
         <v>2726</v>
       </c>
       <c r="H11" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="I11" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="J11" s="1">
         <v>46212</v>
@@ -1448,7 +1463,7 @@
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="N11" s="1">
         <v>46219</v>
@@ -1457,22 +1472,22 @@
         <v>46216</v>
       </c>
       <c r="Q11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R11">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S11" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="U11" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="V11" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="W11" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1489,22 +1504,22 @@
         <v>44</v>
       </c>
       <c r="D12" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E12" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F12" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="G12">
         <v>2723</v>
       </c>
       <c r="H12" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="I12" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="J12" s="1">
         <v>46211</v>
@@ -1516,7 +1531,7 @@
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="N12" s="1">
         <v>46219</v>
@@ -1525,19 +1540,19 @@
         <v>46237</v>
       </c>
       <c r="Q12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R12">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S12" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="V12" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="W12" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1554,22 +1569,22 @@
         <v>45</v>
       </c>
       <c r="D13" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E13" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F13" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="G13">
         <v>2702</v>
       </c>
       <c r="H13" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="I13" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="J13" s="1">
         <v>46212</v>
@@ -1581,22 +1596,25 @@
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="N13" s="1">
         <v>46243</v>
       </c>
       <c r="Q13">
-        <v>-24</v>
+        <v>-23</v>
       </c>
       <c r="R13">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S13" t="s">
-        <v>99</v>
+        <v>103</v>
+      </c>
+      <c r="V13" t="s">
+        <v>125</v>
       </c>
       <c r="W13" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1613,22 +1631,22 @@
         <v>46</v>
       </c>
       <c r="D14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E14" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F14" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="G14">
         <v>2734</v>
       </c>
       <c r="H14" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="I14" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="J14" s="1">
         <v>46213</v>
@@ -1640,28 +1658,31 @@
         <v>1</v>
       </c>
       <c r="M14" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="N14" s="1">
         <v>46224</v>
       </c>
+      <c r="O14" s="1">
+        <v>46219</v>
+      </c>
       <c r="Q14">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R14">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S14" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="U14" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="V14" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="W14" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
@@ -1678,22 +1699,22 @@
         <v>47</v>
       </c>
       <c r="D15" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E15" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F15" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="G15">
         <v>2736</v>
       </c>
       <c r="H15" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I15" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="J15" s="1">
         <v>46216</v>
@@ -1705,22 +1726,22 @@
         <v>1</v>
       </c>
       <c r="M15" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="N15" s="1">
         <v>46248</v>
       </c>
       <c r="Q15">
-        <v>-29</v>
+        <v>-28</v>
       </c>
       <c r="R15">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S15" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="W15" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
@@ -1737,22 +1758,22 @@
         <v>48</v>
       </c>
       <c r="D16" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E16" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F16" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G16">
         <v>2729</v>
       </c>
       <c r="H16" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I16" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="J16" s="1">
         <v>46216</v>
@@ -1764,22 +1785,22 @@
         <v>1</v>
       </c>
       <c r="M16" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="N16" s="1">
-        <v>46248</v>
+        <v>46228</v>
       </c>
       <c r="Q16">
-        <v>-29</v>
+        <v>-8</v>
       </c>
       <c r="R16">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S16" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="W16" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="AA16" t="b">
         <v>1</v>
@@ -1796,22 +1817,22 @@
         <v>49</v>
       </c>
       <c r="D17" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E17" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F17" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G17">
         <v>2743</v>
       </c>
       <c r="H17" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="I17" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="J17" s="1">
         <v>46213</v>
@@ -1823,25 +1844,28 @@
         <v>1</v>
       </c>
       <c r="M17" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="N17" s="1">
         <v>46228</v>
       </c>
+      <c r="O17" s="1">
+        <v>46218</v>
+      </c>
       <c r="Q17">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="R17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S17" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="V17" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="W17" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="AA17" t="b">
         <v>1</v>
@@ -1858,22 +1882,22 @@
         <v>50</v>
       </c>
       <c r="D18" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E18" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F18" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G18">
         <v>2722</v>
       </c>
       <c r="H18" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="I18" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="J18" s="1">
         <v>46217</v>
@@ -1885,22 +1909,22 @@
         <v>1</v>
       </c>
       <c r="M18" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="N18" s="1">
         <v>46229</v>
       </c>
       <c r="Q18">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="R18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S18" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="W18" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="AA18" t="b">
         <v>1</v>
@@ -1917,22 +1941,22 @@
         <v>51</v>
       </c>
       <c r="D19" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E19" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F19" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="G19">
         <v>2722</v>
       </c>
       <c r="H19" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I19" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="J19" s="1">
         <v>46219</v>
@@ -1944,22 +1968,22 @@
         <v>1</v>
       </c>
       <c r="M19" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="N19" s="1">
-        <v>46249</v>
+        <v>46229</v>
       </c>
       <c r="Q19">
-        <v>-30</v>
+        <v>-9</v>
       </c>
       <c r="R19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S19" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="W19" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="AA19" t="b">
         <v>1</v>
@@ -1976,22 +2000,22 @@
         <v>52</v>
       </c>
       <c r="D20" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E20" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F20" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G20">
         <v>2729</v>
       </c>
       <c r="H20" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I20" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="J20" s="1">
         <v>46219</v>
@@ -2003,22 +2027,22 @@
         <v>1</v>
       </c>
       <c r="M20" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="N20" s="1">
         <v>46230</v>
       </c>
       <c r="Q20">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S20" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="W20" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="AA20" t="b">
         <v>1</v>
@@ -2035,22 +2059,22 @@
         <v>53</v>
       </c>
       <c r="D21" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E21" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F21" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="G21">
         <v>2703</v>
       </c>
       <c r="H21" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I21" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="J21" s="1">
         <v>46219</v>
@@ -2062,22 +2086,22 @@
         <v>2</v>
       </c>
       <c r="M21" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="N21" s="1">
         <v>46251</v>
       </c>
       <c r="Q21">
-        <v>-32</v>
+        <v>-31</v>
       </c>
       <c r="R21">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="S21" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="W21" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="AA21" t="b">
         <v>1</v>
@@ -2094,22 +2118,22 @@
         <v>54</v>
       </c>
       <c r="D22" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E22" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F22" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="G22">
         <v>2727</v>
       </c>
       <c r="H22" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I22" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="J22" s="1">
         <v>46219</v>
@@ -2121,27 +2145,86 @@
         <v>1</v>
       </c>
       <c r="M22" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="N22" s="1">
         <v>46228</v>
       </c>
       <c r="Q22">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="R22">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="S22" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="U22" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W22" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="AA22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:27">
+      <c r="A23">
+        <v>685</v>
+      </c>
+      <c r="B23" t="s">
+        <v>30</v>
+      </c>
+      <c r="C23" t="s">
+        <v>55</v>
+      </c>
+      <c r="D23" t="s">
+        <v>74</v>
+      </c>
+      <c r="E23" t="s">
+        <v>92</v>
+      </c>
+      <c r="F23" t="s">
+        <v>95</v>
+      </c>
+      <c r="G23">
+        <v>2729</v>
+      </c>
+      <c r="H23" t="s">
+        <v>98</v>
+      </c>
+      <c r="I23" t="s">
+        <v>99</v>
+      </c>
+      <c r="J23" s="1">
+        <v>46219</v>
+      </c>
+      <c r="K23" s="1">
+        <v>46221</v>
+      </c>
+      <c r="L23">
+        <v>1</v>
+      </c>
+      <c r="M23" t="s">
+        <v>102</v>
+      </c>
+      <c r="N23" s="1">
+        <v>46232</v>
+      </c>
+      <c r="Q23">
+        <v>-12</v>
+      </c>
+      <c r="R23">
+        <v>-1</v>
+      </c>
+      <c r="S23" t="s">
+        <v>103</v>
+      </c>
+      <c r="W23" t="s">
+        <v>128</v>
+      </c>
+      <c r="AA23" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (20/07/2026 16:19)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -866,10 +866,10 @@
         <v>46091</v>
       </c>
       <c r="Q2">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="R2">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="S2" t="s">
         <v>103</v>
@@ -934,10 +934,10 @@
         <v>46216</v>
       </c>
       <c r="Q3">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="R3">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="S3" t="s">
         <v>103</v>
@@ -1005,10 +1005,10 @@
         <v>46216</v>
       </c>
       <c r="Q4">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="R4">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="S4" t="s">
         <v>103</v>
@@ -1070,10 +1070,10 @@
         <v>46214</v>
       </c>
       <c r="Q5">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="R5">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="S5" t="s">
         <v>103</v>
@@ -1141,10 +1141,10 @@
         <v>46212</v>
       </c>
       <c r="Q6">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="R6">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="S6" t="s">
         <v>103</v>
@@ -1209,10 +1209,10 @@
         <v>46216</v>
       </c>
       <c r="Q7">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="R7">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="S7" t="s">
         <v>103</v>
@@ -1274,10 +1274,10 @@
         <v>46238</v>
       </c>
       <c r="Q8">
-        <v>-21</v>
+        <v>-18</v>
       </c>
       <c r="R8">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="S8" t="s">
         <v>103</v>
@@ -1339,10 +1339,10 @@
         <v>46213</v>
       </c>
       <c r="Q9">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R9">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="S9" t="s">
         <v>103</v>
@@ -1407,10 +1407,10 @@
         <v>46237</v>
       </c>
       <c r="Q10">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="R10">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="S10" t="s">
         <v>103</v>
@@ -1472,10 +1472,10 @@
         <v>46216</v>
       </c>
       <c r="Q11">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="R11">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="S11" t="s">
         <v>104</v>
@@ -1540,10 +1540,10 @@
         <v>46237</v>
       </c>
       <c r="Q12">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="R12">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="S12" t="s">
         <v>103</v>
@@ -1602,10 +1602,10 @@
         <v>46243</v>
       </c>
       <c r="Q13">
-        <v>-23</v>
+        <v>-20</v>
       </c>
       <c r="R13">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="S13" t="s">
         <v>103</v>
@@ -1667,10 +1667,10 @@
         <v>46219</v>
       </c>
       <c r="Q14">
-        <v>-4</v>
+        <v>-1</v>
       </c>
       <c r="R14">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S14" t="s">
         <v>103</v>
@@ -1732,10 +1732,10 @@
         <v>46248</v>
       </c>
       <c r="Q15">
-        <v>-28</v>
+        <v>-25</v>
       </c>
       <c r="R15">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="S15" t="s">
         <v>103</v>
@@ -1791,10 +1791,10 @@
         <v>46228</v>
       </c>
       <c r="Q16">
-        <v>-8</v>
+        <v>-5</v>
       </c>
       <c r="R16">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="S16" t="s">
         <v>103</v>
@@ -1853,10 +1853,10 @@
         <v>46218</v>
       </c>
       <c r="Q17">
-        <v>-8</v>
+        <v>-5</v>
       </c>
       <c r="R17">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="S17" t="s">
         <v>103</v>
@@ -1915,10 +1915,10 @@
         <v>46229</v>
       </c>
       <c r="Q18">
-        <v>-9</v>
+        <v>-6</v>
       </c>
       <c r="R18">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S18" t="s">
         <v>103</v>
@@ -1974,10 +1974,10 @@
         <v>46229</v>
       </c>
       <c r="Q19">
-        <v>-9</v>
+        <v>-6</v>
       </c>
       <c r="R19">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S19" t="s">
         <v>103</v>
@@ -2033,10 +2033,10 @@
         <v>46230</v>
       </c>
       <c r="Q20">
-        <v>-10</v>
+        <v>-7</v>
       </c>
       <c r="R20">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S20" t="s">
         <v>103</v>
@@ -2092,10 +2092,10 @@
         <v>46251</v>
       </c>
       <c r="Q21">
-        <v>-31</v>
+        <v>-28</v>
       </c>
       <c r="R21">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S21" t="s">
         <v>104</v>
@@ -2151,10 +2151,10 @@
         <v>46228</v>
       </c>
       <c r="Q22">
-        <v>-8</v>
+        <v>-5</v>
       </c>
       <c r="R22">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="S22" t="s">
         <v>104</v>
@@ -2213,10 +2213,10 @@
         <v>46232</v>
       </c>
       <c r="Q23">
-        <v>-12</v>
+        <v>-9</v>
       </c>
       <c r="R23">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="S23" t="s">
         <v>103</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (21/07/2026 16:08)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="134">
   <si>
     <t>om_emg</t>
   </si>
@@ -112,9 +112,6 @@
     <t>CLA</t>
   </si>
   <si>
-    <t>BACO</t>
-  </si>
-  <si>
     <t>BACG</t>
   </si>
   <si>
@@ -127,12 +124,6 @@
     <t>396260016520</t>
   </si>
   <si>
-    <t>313260018646</t>
-  </si>
-  <si>
-    <t>329260019179</t>
-  </si>
-  <si>
     <t>329260019181</t>
   </si>
   <si>
@@ -154,18 +145,12 @@
     <t>685260012350</t>
   </si>
   <si>
-    <t>313260018670</t>
-  </si>
-  <si>
     <t>313260018674</t>
   </si>
   <si>
     <t>685260012368</t>
   </si>
   <si>
-    <t>386260013445</t>
-  </si>
-  <si>
     <t>685260012377</t>
   </si>
   <si>
@@ -184,6 +169,21 @@
     <t>685260012396</t>
   </si>
   <si>
+    <t>313260018675</t>
+  </si>
+  <si>
+    <t>313260018676</t>
+  </si>
+  <si>
+    <t>329260019225</t>
+  </si>
+  <si>
+    <t>329260019226</t>
+  </si>
+  <si>
+    <t>329260019227</t>
+  </si>
+  <si>
     <t>1214134-1</t>
   </si>
   <si>
@@ -193,18 +193,15 @@
     <t>1H75-21</t>
   </si>
   <si>
-    <t>011-00883-20</t>
+    <t>C145-00-46</t>
+  </si>
+  <si>
+    <t>065-0065-01</t>
   </si>
   <si>
     <t>066-3046-07</t>
   </si>
   <si>
-    <t>C145-00-46</t>
-  </si>
-  <si>
-    <t>065-0065-01</t>
-  </si>
-  <si>
     <t>3244809-4</t>
   </si>
   <si>
@@ -217,9 +214,6 @@
     <t>030-1094-58</t>
   </si>
   <si>
-    <t>S2655-1</t>
-  </si>
-  <si>
     <t>205842-1</t>
   </si>
   <si>
@@ -241,6 +235,21 @@
     <t>540-1407-4</t>
   </si>
   <si>
+    <t>011-00870-00</t>
+  </si>
+  <si>
+    <t>ASG12000-2</t>
+  </si>
+  <si>
+    <t>MS21442-121</t>
+  </si>
+  <si>
+    <t>2625014-10</t>
+  </si>
+  <si>
+    <t>2625014-9</t>
+  </si>
+  <si>
     <t>BELLCRANK ASSY</t>
   </si>
   <si>
@@ -250,18 +259,15 @@
     <t>PRESSURE REGULATOR</t>
   </si>
   <si>
-    <t>RADAR GWX 68 WEATHER</t>
+    <t>TRANSMISSION ASSY</t>
+  </si>
+  <si>
+    <t>SELECTOR ALT</t>
   </si>
   <si>
     <t>CONTROL,INDICATOR</t>
   </si>
   <si>
-    <t>TRANSMISSION ASSY</t>
-  </si>
-  <si>
-    <t>SELECTOR ALT</t>
-  </si>
-  <si>
     <t>FUEL CONTROL,MAIN,TU</t>
   </si>
   <si>
@@ -274,9 +280,6 @@
     <t>CONNECTOR</t>
   </si>
   <si>
-    <t>DUCT-FLEX</t>
-  </si>
-  <si>
     <t>ALTERNATOR CONTROL U</t>
   </si>
   <si>
@@ -295,6 +298,18 @@
     <t>VALVE,BLEED,TURBINEE</t>
   </si>
   <si>
+    <t>MAGNETOMETER GMU 44</t>
+  </si>
+  <si>
+    <t>ALTERNATOR</t>
+  </si>
+  <si>
+    <t>BEARING,ROLLER,NEEDL</t>
+  </si>
+  <si>
+    <t>SPACER</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -340,22 +355,16 @@
     <t>Item retirado para atender o C-98 2731. Ramon 15/06/26. AWB 12746187256 - volume retirado na loja GOLLOG - BEL por bispo em 13/07. Godoy 16/07/26. Recibo não se encontra na Pasta do DRIVE. Godoy 17/07/2026.</t>
   </si>
   <si>
-    <t>Retirado para atender a Anv 2740 - Godoy 30/06/26. AWB 12745953832 - Volume retirado na loja GOLLOG - QMA por Kleyton em 13/07/26. Godoy 15/07/26.</t>
-  </si>
-  <si>
-    <t>Recibo não se encontra na Pasta do DRIVE. Godoy 08/07/2026.</t>
-  </si>
-  <si>
     <t>AWB 12745918331 volume retirado na loja GOLLOG - BEL por bispo em 10/07/2026 - Godoy 13/07/2026. Recibo não se encontra na Pasta do DRIVE. Godoy 17/07/2026.</t>
   </si>
   <si>
     <t>Cedeu o item para o C-98 2721. Ramon 09/07/26. AWB 12746175415 - 2 volumes retirados na loja GOLLOG - BEL por bispo em 13/07/26. Godoy 15/07/26. Vee One, não temos o recibo assinado. Godoy 16/07/26.</t>
   </si>
   <si>
-    <t>Cedeu o item para o C-98 2738. Godoy 13/07/26</t>
-  </si>
-  <si>
-    <t>Vee One preferiu atender a demanda com estoque da empresa. Godoy 16/07/26.</t>
+    <t>Vee One preferiu atender a demanda com estoque da empresa. Godoy 16/07/26. AWB 12747645135 - volume retirados na loja GOLLOG - CGR por givanildo em 20/07. Godoy 21/07/26.</t>
+  </si>
+  <si>
+    <t>Cedeu o item para o C-98 2737. Godoy 21/07/26.</t>
   </si>
   <si>
     <t>Foi solicitado via email no dia 02-03-2 o atendimento do item com estoque FAB. Claudio -02-03-26 - Em resposta, a coordenadoria disse que o estque seria insuficiente. Foi verificado que na T.O da ANV o QPA para esse item são 2 EA, solicitei confirmação. - Cláudio -02-03-2026. Solicitado o cancelamento da emergência em função da quantidade cedida ao 2733 ter sido de 01ea. Considerando o QPA 02 ea. Encontra-se em tratativa junto a fiscalização e o gestor do contrato conforme mensagem de e-mail de 05/03. - SOLICITAÇÃO E-C98-26047.Colocado pedido AOG Textron WB0003068789 - previsão de entrega 60 dias em média. Os demais fornecedores informaram não ter em estoque ou não possuírem a certificação necessária da peça.</t>
@@ -364,13 +373,7 @@
     <t>Colocado pedido na Textron IJ17507011. Previsão de entrega em Miami 17/06. Carga recepcionada no GIG 24/06. Canal verde dia 26/06. DPE V1 29/06. Verificar entrega do item. ATZ 30/06 - MATERIAL EM RECEBIMENTO V1 30-06-2026 - MATERIAL EM PROCESSO DE ENVIO RECIBO 524/FAB/26 ATZ RC 30-06-2026 - MATERIAL EM TRANSITO - AWB 12744330731 DPE 03/07/2026 - MATERIAL RECEBIDO POR tanise Assis RG 14807641751 DIA 03/07/2026</t>
   </si>
   <si>
-    <t>04 ea recolhidos para a V1, chegada dos itens dia 23/06/2026. Itens não tem oficina no Brasil, terá que ser feito  Exchange rc 23/06 - MATERIAL ADQUIRIDO FORNECEDOR TEXTRON -WB0003073549 Inovice IJ17534800 DPE AGS  Miami 29/6/2026 ate 10 30AM - AIR EXPORT HOUSE: 00004046 de 30/6/2026 Chegou no GIGRJ em 01/7/26 para  Desembaraço - ATZ Marcio 3/7/26 CANAL VERDE EM 7/7/26 entregue V1 em 8/7/26 ATZ Marcio 9/7/26 - MATERIAL EM TRANSITO - RECIBO 560/FAB/26 AWB - 12746187256 DPE 13/07/2026</t>
-  </si>
-  <si>
-    <t>Efetuada a Compra em SP na Jet Avionics, aguardando confirmar unidade em estoque para liberação do item para a Veeone 01/7/2026 14:15 Marcio - DECLINADO pela JET AVIONICS, colocado Pedido TEXTRON Confirmation Number: WB0003077522 de 01/7/2026 Invoice IJ17546081 as 15:08PM Previsao DPE AGS Miami 02/7/2026 - PRE ALERTA do VOO de 3/7/2026 HAWB4065 - CANAL VERDE - ATZ Mayara 7/7/26 14:34 (MATERIAL EM SEPARAÇÃO - SUP V1 JPA) Atlz Lucas 08/07 14:01 - MATERIAL EM TRANSITO - RECIBO 556/FAB/26 - AWB 12745953832 DPE 14/07/2026</t>
-  </si>
-  <si>
-    <t>Item estara disponivel no RJ na oficina para coleta dia 6/7 apos as 14 horas ATZ Marcio 3/7/ 14:25PM/ MATERIAL EM TRANSITO- RECIBO 548/FAB/26- AWB 12745474752 DPE 08/07 - Atlz Lucas- JPA (07/07) - MATERIAL DISPONIVEL PRA RETIRADA DIA 09/07/2026 ATZ RC - MATERIAL RETIRADO DIA 09/07/2026 POR KÉSIA SANTOS</t>
+    <t>04 ea recolhidos para a V1, chegada dos itens dia 23/06/2026. Itens não tem oficina no Brasil, terá que ser feito Exchange rc 23/06 - MATERIAL ADQUIRIDO FORNECEDOR TEXTRON -WB0003073549 Inovice IJ17534800 DPE AGS Miami 29/6/2026 ate 10 30AM - AIR EXPORT HOUSE: 00004046 de 30/6/2026 Chegou no GIGRJ em 01/7/26 para Desembaraço - ATZ Marcio 3/7/26 CANAL VERDE EM 7/7/26 entregue V1 em 8/7/26 ATZ Marcio 9/7/26 - MATERIAL EM TRANSITO - RECIBO 560/FAB/26 AWB - 12746187256 DPE 13/07/2026</t>
   </si>
   <si>
     <t>Colocado pedido AOG Textron IJ17557538 - previsão de entrega em Miami 08/07. Previsão de chegada GIG 09/07 - MATERIAL EM TRANSITO - RECIBO 551/FAB/26 - ENVIADO PN COMPLETO PARA SANAR A EMERGENCIA DO 2709, ENVIADO MODAL TERRESTRE, DPE 13/07/2026</t>
@@ -394,10 +397,22 @@
     <t>Colocado pedido junto ao fornecedor AEROBASE, aguardando pagamento proforma. ATZ 16/07</t>
   </si>
   <si>
-    <t>Será atendido via estoque V1. ATZ 13/07 - material em transito recibo 568/FAB/26 AWB 12746855476 DPE 17/07/2026 - DPE ATT 16/07/2026 - Recibo enviado dia 16/07/2026</t>
-  </si>
-  <si>
-    <t>ENVIADO NO DIA 10-07-26 AWB 127-4640 3125 - material recebido dia 15/07/2026 - nota fiscal enviada dia 15/07/2026</t>
+    <t>Colocado pedido Textron IJ17575583 - entregue em Miami 15/07. Será consolidado próximo voo GIG</t>
+  </si>
+  <si>
+    <t>Previsão 17/07 da oficina de BH - material em transito - recibo 582/FAB/26 AWB A SER GERADA PELA GOLLOG ATZ 17/07/2026</t>
+  </si>
+  <si>
+    <t>Item em bancada porem em pessimo estado, foi solicitado recolhimento de mais unidades para envio a oficina para tentativa de reparo ATZ Marcio 17/7/26</t>
+  </si>
+  <si>
+    <t>Nao temos oficina no Brasil para reparo desse item, temos que iniciar processo de aquisiçáo do material para atendimento a essa necessidade ATZ Marcio 17/7/26</t>
+  </si>
+  <si>
+    <t>Material em transito - recibo 576/FAB/26 AWB a ser gerada pela Gollog - Atz Rc 16/07/2026 - awb 12747645135</t>
+  </si>
+  <si>
+    <t>Enviado 1 unidade (CORE) para reparo na oficina no RJ em 17/7, aguardando orçamento com prazo de entrega, ATZ Marcio 17/7</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -736,7 +751,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA23"/>
+  <dimension ref="A1:AA24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -830,25 +845,25 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D2" t="s">
         <v>56</v>
       </c>
       <c r="E2" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F2" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="G2">
         <v>2730</v>
       </c>
       <c r="H2" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="I2" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="J2" s="1">
         <v>46076</v>
@@ -860,28 +875,28 @@
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N2" s="1">
         <v>46091</v>
       </c>
       <c r="Q2">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="R2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="S2" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="U2" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="V2" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="W2" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -895,25 +910,25 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D3" t="s">
         <v>57</v>
       </c>
       <c r="E3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="F3" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="G3">
         <v>2721</v>
       </c>
       <c r="H3" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="I3" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="J3" s="1">
         <v>46185</v>
@@ -925,7 +940,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N3" s="1">
         <v>46216</v>
@@ -934,25 +949,25 @@
         <v>46216</v>
       </c>
       <c r="Q3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R3">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="S3" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="T3" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="U3" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="V3" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="W3" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -966,25 +981,25 @@
         <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s">
         <v>58</v>
       </c>
       <c r="E4" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="F4" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="G4">
         <v>2726</v>
       </c>
       <c r="H4" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="I4" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="J4" s="1">
         <v>46185</v>
@@ -996,7 +1011,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N4" s="1">
         <v>46192</v>
@@ -1005,22 +1020,22 @@
         <v>46216</v>
       </c>
       <c r="Q4">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R4">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="S4" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="U4" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="V4" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="W4" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -1028,67 +1043,67 @@
     </row>
     <row r="5" spans="1:27">
       <c r="A5">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D5" t="s">
         <v>59</v>
       </c>
       <c r="E5" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="F5" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="G5">
-        <v>2734</v>
+        <v>2721</v>
       </c>
       <c r="H5" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="I5" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="J5" s="1">
-        <v>46199</v>
+        <v>46209</v>
       </c>
       <c r="K5" s="1">
-        <v>46203</v>
+        <v>46210</v>
       </c>
       <c r="L5">
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N5" s="1">
-        <v>46214</v>
+        <v>46217</v>
+      </c>
+      <c r="O5" s="1">
+        <v>46216</v>
       </c>
       <c r="Q5">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="R5">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="S5" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="T5" t="s">
-        <v>104</v>
-      </c>
-      <c r="U5" t="s">
         <v>108</v>
       </c>
       <c r="V5" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="W5" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1096,67 +1111,64 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D6" t="s">
         <v>60</v>
       </c>
       <c r="E6" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="F6" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="G6">
-        <v>2721</v>
+        <v>2719</v>
       </c>
       <c r="H6" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="I6" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="J6" s="1">
-        <v>46205</v>
+        <v>46210</v>
       </c>
       <c r="K6" s="1">
-        <v>46206</v>
+        <v>46210</v>
       </c>
       <c r="L6">
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N6" s="1">
-        <v>46213</v>
+        <v>46241</v>
       </c>
       <c r="O6" s="1">
-        <v>46212</v>
+        <v>46238</v>
       </c>
       <c r="Q6">
-        <v>10</v>
+        <v>-17</v>
       </c>
       <c r="R6">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="S6" t="s">
-        <v>103</v>
-      </c>
-      <c r="U6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="V6" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="W6" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1164,49 +1176,49 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>329</v>
+        <v>419</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D7" t="s">
         <v>61</v>
       </c>
       <c r="E7" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F7" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="G7">
-        <v>2721</v>
+        <v>2723</v>
       </c>
       <c r="H7" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="I7" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="J7" s="1">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="K7" s="1">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="L7">
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N7" s="1">
-        <v>46217</v>
+        <v>46218</v>
       </c>
       <c r="O7" s="1">
-        <v>46216</v>
+        <v>46213</v>
       </c>
       <c r="Q7">
         <v>6</v>
@@ -1215,13 +1227,19 @@
         <v>13</v>
       </c>
       <c r="S7" t="s">
-        <v>103</v>
+        <v>108</v>
+      </c>
+      <c r="T7" t="s">
+        <v>109</v>
+      </c>
+      <c r="U7" t="s">
+        <v>113</v>
       </c>
       <c r="V7" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="W7" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1229,64 +1247,67 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>685</v>
+        <v>396</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D8" t="s">
         <v>62</v>
       </c>
       <c r="E8" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="F8" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G8">
-        <v>2719</v>
+        <v>2733</v>
       </c>
       <c r="H8" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="I8" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J8" s="1">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="K8" s="1">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="L8">
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N8" s="1">
-        <v>46241</v>
+        <v>46222</v>
       </c>
       <c r="O8" s="1">
-        <v>46238</v>
+        <v>46237</v>
       </c>
       <c r="Q8">
-        <v>-18</v>
+        <v>2</v>
       </c>
       <c r="R8">
         <v>13</v>
       </c>
       <c r="S8" t="s">
-        <v>103</v>
+        <v>108</v>
+      </c>
+      <c r="T8" t="s">
+        <v>109</v>
       </c>
       <c r="V8" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="W8" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1294,49 +1315,49 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9">
-        <v>419</v>
+        <v>396</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D9" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E9" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="F9" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="G9">
-        <v>2723</v>
+        <v>2726</v>
       </c>
       <c r="H9" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="I9" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="J9" s="1">
-        <v>46210</v>
+        <v>46212</v>
       </c>
       <c r="K9" s="1">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="L9">
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N9" s="1">
-        <v>46218</v>
+        <v>46219</v>
       </c>
       <c r="O9" s="1">
-        <v>46213</v>
+        <v>46216</v>
       </c>
       <c r="Q9">
         <v>5</v>
@@ -1345,16 +1366,16 @@
         <v>12</v>
       </c>
       <c r="S9" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="U9" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="V9" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="W9" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1362,64 +1383,67 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>396</v>
+        <v>419</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D10" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E10" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="F10" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="G10">
-        <v>2733</v>
+        <v>2723</v>
       </c>
       <c r="H10" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="I10" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="J10" s="1">
         <v>46211</v>
       </c>
       <c r="K10" s="1">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="L10">
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N10" s="1">
-        <v>46222</v>
+        <v>46219</v>
       </c>
       <c r="O10" s="1">
         <v>46237</v>
       </c>
       <c r="Q10">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="R10">
         <v>12</v>
       </c>
       <c r="S10" t="s">
-        <v>103</v>
+        <v>108</v>
+      </c>
+      <c r="T10" t="s">
+        <v>108</v>
       </c>
       <c r="V10" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="W10" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1427,31 +1451,31 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>396</v>
+        <v>685</v>
       </c>
       <c r="B11" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E11" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="F11" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="G11">
-        <v>2726</v>
+        <v>2702</v>
       </c>
       <c r="H11" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="I11" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="J11" s="1">
         <v>46212</v>
@@ -1463,31 +1487,25 @@
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N11" s="1">
-        <v>46219</v>
-      </c>
-      <c r="O11" s="1">
-        <v>46216</v>
+        <v>46243</v>
       </c>
       <c r="Q11">
-        <v>4</v>
+        <v>-19</v>
       </c>
       <c r="R11">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="S11" t="s">
-        <v>104</v>
-      </c>
-      <c r="U11" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="V11" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="W11" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1495,64 +1513,61 @@
     </row>
     <row r="12" spans="1:27">
       <c r="A12">
-        <v>419</v>
+        <v>313</v>
       </c>
       <c r="B12" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D12" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E12" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F12" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="G12">
-        <v>2723</v>
+        <v>2736</v>
       </c>
       <c r="H12" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I12" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="J12" s="1">
-        <v>46211</v>
+        <v>46216</v>
       </c>
       <c r="K12" s="1">
-        <v>46212</v>
+        <v>46217</v>
       </c>
       <c r="L12">
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N12" s="1">
-        <v>46219</v>
-      </c>
-      <c r="O12" s="1">
-        <v>46237</v>
+        <v>46248</v>
       </c>
       <c r="Q12">
-        <v>4</v>
+        <v>-24</v>
       </c>
       <c r="R12">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="S12" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="V12" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="W12" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1566,55 +1581,55 @@
         <v>30</v>
       </c>
       <c r="C13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D13" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E13" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="F13" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="G13">
-        <v>2702</v>
+        <v>2729</v>
       </c>
       <c r="H13" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="I13" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J13" s="1">
-        <v>46212</v>
+        <v>46216</v>
       </c>
       <c r="K13" s="1">
-        <v>46212</v>
+        <v>46217</v>
       </c>
       <c r="L13">
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N13" s="1">
-        <v>46243</v>
+        <v>46228</v>
       </c>
       <c r="Q13">
-        <v>-20</v>
+        <v>-4</v>
       </c>
       <c r="R13">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="S13" t="s">
-        <v>103</v>
-      </c>
-      <c r="V13" t="s">
-        <v>125</v>
+        <v>108</v>
+      </c>
+      <c r="T13" t="s">
+        <v>109</v>
       </c>
       <c r="W13" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1622,67 +1637,67 @@
     </row>
     <row r="14" spans="1:27">
       <c r="A14">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B14" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D14" t="s">
         <v>67</v>
       </c>
       <c r="E14" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F14" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="G14">
-        <v>2734</v>
+        <v>2722</v>
       </c>
       <c r="H14" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="I14" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="J14" s="1">
-        <v>46213</v>
+        <v>46217</v>
       </c>
       <c r="K14" s="1">
-        <v>46213</v>
+        <v>46218</v>
       </c>
       <c r="L14">
         <v>1</v>
       </c>
       <c r="M14" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N14" s="1">
-        <v>46224</v>
+        <v>46229</v>
       </c>
       <c r="O14" s="1">
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="Q14">
-        <v>-1</v>
+        <v>-5</v>
       </c>
       <c r="R14">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="S14" t="s">
-        <v>103</v>
-      </c>
-      <c r="U14" t="s">
-        <v>112</v>
+        <v>108</v>
+      </c>
+      <c r="T14" t="s">
+        <v>109</v>
       </c>
       <c r="V14" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="W14" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
@@ -1690,58 +1705,64 @@
     </row>
     <row r="15" spans="1:27">
       <c r="A15">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B15" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D15" t="s">
         <v>68</v>
       </c>
       <c r="E15" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F15" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="G15">
-        <v>2736</v>
+        <v>2722</v>
       </c>
       <c r="H15" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="I15" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J15" s="1">
-        <v>46216</v>
+        <v>46219</v>
       </c>
       <c r="K15" s="1">
-        <v>46217</v>
+        <v>46218</v>
       </c>
       <c r="L15">
         <v>1</v>
       </c>
       <c r="M15" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N15" s="1">
-        <v>46248</v>
+        <v>46229</v>
       </c>
       <c r="Q15">
-        <v>-25</v>
+        <v>-5</v>
       </c>
       <c r="R15">
         <v>6</v>
       </c>
       <c r="S15" t="s">
-        <v>103</v>
+        <v>108</v>
+      </c>
+      <c r="T15" t="s">
+        <v>109</v>
+      </c>
+      <c r="V15" t="s">
+        <v>129</v>
       </c>
       <c r="W15" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
@@ -1755,52 +1776,58 @@
         <v>30</v>
       </c>
       <c r="C16" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D16" t="s">
         <v>69</v>
       </c>
       <c r="E16" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="F16" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="G16">
         <v>2729</v>
       </c>
       <c r="H16" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="I16" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="J16" s="1">
-        <v>46216</v>
+        <v>46219</v>
       </c>
       <c r="K16" s="1">
-        <v>46217</v>
+        <v>46219</v>
       </c>
       <c r="L16">
         <v>1</v>
       </c>
       <c r="M16" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N16" s="1">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="Q16">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="R16">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S16" t="s">
-        <v>103</v>
+        <v>108</v>
+      </c>
+      <c r="T16" t="s">
+        <v>109</v>
+      </c>
+      <c r="V16" t="s">
+        <v>130</v>
       </c>
       <c r="W16" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="AA16" t="b">
         <v>1</v>
@@ -1808,64 +1835,58 @@
     </row>
     <row r="17" spans="1:27">
       <c r="A17">
-        <v>386</v>
+        <v>685</v>
       </c>
       <c r="B17" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D17" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E17" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F17" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="G17">
-        <v>2743</v>
+        <v>2703</v>
       </c>
       <c r="H17" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="I17" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="J17" s="1">
-        <v>46213</v>
+        <v>46219</v>
       </c>
       <c r="K17" s="1">
-        <v>46217</v>
+        <v>46220</v>
       </c>
       <c r="L17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M17" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N17" s="1">
-        <v>46228</v>
-      </c>
-      <c r="O17" s="1">
-        <v>46218</v>
+        <v>46251</v>
       </c>
       <c r="Q17">
-        <v>-5</v>
+        <v>-27</v>
       </c>
       <c r="R17">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="S17" t="s">
-        <v>103</v>
-      </c>
-      <c r="V17" t="s">
-        <v>127</v>
+        <v>109</v>
       </c>
       <c r="W17" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="AA17" t="b">
         <v>1</v>
@@ -1873,58 +1894,67 @@
     </row>
     <row r="18" spans="1:27">
       <c r="A18">
-        <v>685</v>
+        <v>690</v>
       </c>
       <c r="B18" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C18" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D18" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E18" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="F18" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="G18">
-        <v>2722</v>
+        <v>2727</v>
       </c>
       <c r="H18" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="I18" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="J18" s="1">
-        <v>46217</v>
+        <v>46219</v>
       </c>
       <c r="K18" s="1">
-        <v>46218</v>
+        <v>46221</v>
       </c>
       <c r="L18">
         <v>1</v>
       </c>
       <c r="M18" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N18" s="1">
-        <v>46229</v>
+        <v>46228</v>
+      </c>
+      <c r="O18" s="1">
+        <v>46223</v>
       </c>
       <c r="Q18">
-        <v>-6</v>
+        <v>-4</v>
       </c>
       <c r="R18">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="S18" t="s">
-        <v>103</v>
+        <v>109</v>
+      </c>
+      <c r="U18" t="s">
+        <v>115</v>
+      </c>
+      <c r="V18" t="s">
+        <v>131</v>
       </c>
       <c r="W18" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="AA18" t="b">
         <v>1</v>
@@ -1938,52 +1968,58 @@
         <v>30</v>
       </c>
       <c r="C19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D19" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E19" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="F19" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="G19">
-        <v>2722</v>
+        <v>2729</v>
       </c>
       <c r="H19" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="I19" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="J19" s="1">
         <v>46219</v>
       </c>
       <c r="K19" s="1">
-        <v>46218</v>
+        <v>46221</v>
       </c>
       <c r="L19">
         <v>1</v>
       </c>
       <c r="M19" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N19" s="1">
-        <v>46229</v>
+        <v>46232</v>
       </c>
       <c r="Q19">
-        <v>-6</v>
+        <v>-8</v>
       </c>
       <c r="R19">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="S19" t="s">
-        <v>103</v>
+        <v>108</v>
+      </c>
+      <c r="T19" t="s">
+        <v>109</v>
+      </c>
+      <c r="V19" t="s">
+        <v>132</v>
       </c>
       <c r="W19" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="AA19" t="b">
         <v>1</v>
@@ -1991,58 +2027,64 @@
     </row>
     <row r="20" spans="1:27">
       <c r="A20">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B20" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D20" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E20" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="F20" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G20">
-        <v>2729</v>
+        <v>2730</v>
       </c>
       <c r="H20" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="I20" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="J20" s="1">
-        <v>46219</v>
+        <v>46220</v>
       </c>
       <c r="K20" s="1">
-        <v>46219</v>
+        <v>46221</v>
       </c>
       <c r="L20">
         <v>1</v>
       </c>
       <c r="M20" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N20" s="1">
-        <v>46230</v>
+        <v>46228</v>
       </c>
       <c r="Q20">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="R20">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S20" t="s">
-        <v>103</v>
+        <v>108</v>
+      </c>
+      <c r="T20" t="s">
+        <v>109</v>
+      </c>
+      <c r="U20" t="s">
+        <v>116</v>
       </c>
       <c r="W20" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="AA20" t="b">
         <v>1</v>
@@ -2050,58 +2092,61 @@
     </row>
     <row r="21" spans="1:27">
       <c r="A21">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B21" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C21" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D21" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E21" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="F21" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="G21">
-        <v>2703</v>
+        <v>2741</v>
       </c>
       <c r="H21" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="I21" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="J21" s="1">
-        <v>46219</v>
+        <v>46224</v>
       </c>
       <c r="K21" s="1">
-        <v>46220</v>
+        <v>46222</v>
       </c>
       <c r="L21">
+        <v>1</v>
+      </c>
+      <c r="M21" t="s">
+        <v>107</v>
+      </c>
+      <c r="N21" s="1">
+        <v>46229</v>
+      </c>
+      <c r="Q21">
+        <v>-5</v>
+      </c>
+      <c r="R21">
         <v>2</v>
       </c>
-      <c r="M21" t="s">
-        <v>102</v>
-      </c>
-      <c r="N21" s="1">
-        <v>46251</v>
-      </c>
-      <c r="Q21">
-        <v>-28</v>
-      </c>
-      <c r="R21">
-        <v>3</v>
-      </c>
       <c r="S21" t="s">
-        <v>104</v>
+        <v>108</v>
+      </c>
+      <c r="T21" t="s">
+        <v>109</v>
       </c>
       <c r="W21" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="AA21" t="b">
         <v>1</v>
@@ -2109,61 +2154,61 @@
     </row>
     <row r="22" spans="1:27">
       <c r="A22">
-        <v>690</v>
+        <v>329</v>
       </c>
       <c r="B22" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C22" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D22" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E22" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="F22" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="G22">
-        <v>2727</v>
+        <v>2720</v>
       </c>
       <c r="H22" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="I22" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="J22" s="1">
-        <v>46219</v>
+        <v>46220</v>
       </c>
       <c r="K22" s="1">
-        <v>46221</v>
+        <v>46223</v>
       </c>
       <c r="L22">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="M22" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N22" s="1">
-        <v>46228</v>
+        <v>46254</v>
       </c>
       <c r="Q22">
-        <v>-5</v>
+        <v>-30</v>
       </c>
       <c r="R22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S22" t="s">
-        <v>104</v>
-      </c>
-      <c r="U22" t="s">
-        <v>113</v>
+        <v>108</v>
+      </c>
+      <c r="T22" t="s">
+        <v>108</v>
       </c>
       <c r="W22" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="AA22" t="b">
         <v>1</v>
@@ -2171,60 +2216,125 @@
     </row>
     <row r="23" spans="1:27">
       <c r="A23">
-        <v>685</v>
+        <v>329</v>
       </c>
       <c r="B23" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C23" t="s">
+        <v>54</v>
+      </c>
+      <c r="D23" t="s">
+        <v>76</v>
+      </c>
+      <c r="E23" t="s">
+        <v>97</v>
+      </c>
+      <c r="F23" t="s">
+        <v>98</v>
+      </c>
+      <c r="G23">
+        <v>2720</v>
+      </c>
+      <c r="H23" t="s">
+        <v>103</v>
+      </c>
+      <c r="I23" t="s">
+        <v>105</v>
+      </c>
+      <c r="J23" s="1">
+        <v>46220</v>
+      </c>
+      <c r="K23" s="1">
+        <v>46224</v>
+      </c>
+      <c r="L23">
+        <v>6</v>
+      </c>
+      <c r="M23" t="s">
+        <v>107</v>
+      </c>
+      <c r="N23" s="1">
+        <v>46255</v>
+      </c>
+      <c r="Q23">
+        <v>-31</v>
+      </c>
+      <c r="R23">
+        <v>0</v>
+      </c>
+      <c r="S23" t="s">
+        <v>108</v>
+      </c>
+      <c r="T23" t="s">
+        <v>108</v>
+      </c>
+      <c r="W23" t="s">
+        <v>133</v>
+      </c>
+      <c r="AA23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:27">
+      <c r="A24">
+        <v>329</v>
+      </c>
+      <c r="B24" t="s">
+        <v>28</v>
+      </c>
+      <c r="C24" t="s">
         <v>55</v>
       </c>
-      <c r="D23" t="s">
-        <v>74</v>
-      </c>
-      <c r="E23" t="s">
-        <v>92</v>
-      </c>
-      <c r="F23" t="s">
-        <v>95</v>
-      </c>
-      <c r="G23">
-        <v>2729</v>
-      </c>
-      <c r="H23" t="s">
+      <c r="D24" t="s">
+        <v>77</v>
+      </c>
+      <c r="E24" t="s">
+        <v>97</v>
+      </c>
+      <c r="F24" t="s">
         <v>98</v>
       </c>
-      <c r="I23" t="s">
-        <v>99</v>
-      </c>
-      <c r="J23" s="1">
-        <v>46219</v>
-      </c>
-      <c r="K23" s="1">
-        <v>46221</v>
-      </c>
-      <c r="L23">
-        <v>1</v>
-      </c>
-      <c r="M23" t="s">
-        <v>102</v>
-      </c>
-      <c r="N23" s="1">
-        <v>46232</v>
-      </c>
-      <c r="Q23">
-        <v>-9</v>
-      </c>
-      <c r="R23">
-        <v>2</v>
-      </c>
-      <c r="S23" t="s">
+      <c r="G24">
+        <v>2720</v>
+      </c>
+      <c r="H24" t="s">
         <v>103</v>
       </c>
-      <c r="W23" t="s">
-        <v>128</v>
-      </c>
-      <c r="AA23" t="b">
+      <c r="I24" t="s">
+        <v>105</v>
+      </c>
+      <c r="J24" s="1">
+        <v>46220</v>
+      </c>
+      <c r="K24" s="1">
+        <v>46225</v>
+      </c>
+      <c r="L24">
+        <v>6</v>
+      </c>
+      <c r="M24" t="s">
+        <v>107</v>
+      </c>
+      <c r="N24" s="1">
+        <v>46256</v>
+      </c>
+      <c r="Q24">
+        <v>-32</v>
+      </c>
+      <c r="R24">
+        <v>-1</v>
+      </c>
+      <c r="S24" t="s">
+        <v>109</v>
+      </c>
+      <c r="T24" t="s">
+        <v>108</v>
+      </c>
+      <c r="W24" t="s">
+        <v>133</v>
+      </c>
+      <c r="AA24" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (21/07/2026 20:52)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="128">
   <si>
     <t>om_emg</t>
   </si>
@@ -112,9 +112,6 @@
     <t>CLA</t>
   </si>
   <si>
-    <t>BACG</t>
-  </si>
-  <si>
     <t>313260017747</t>
   </si>
   <si>
@@ -163,9 +160,6 @@
     <t>685260012395</t>
   </si>
   <si>
-    <t>690260002487</t>
-  </si>
-  <si>
     <t>685260012396</t>
   </si>
   <si>
@@ -229,9 +223,6 @@
     <t>2611024-1</t>
   </si>
   <si>
-    <t>850C86-2</t>
-  </si>
-  <si>
     <t>540-1407-4</t>
   </si>
   <si>
@@ -292,9 +283,6 @@
     <t>WINDOW</t>
   </si>
   <si>
-    <t>TIRE,PNEUMATIC,AIRC</t>
-  </si>
-  <si>
     <t>VALVE,BLEED,TURBINEE</t>
   </si>
   <si>
@@ -361,9 +349,6 @@
     <t>Cedeu o item para o C-98 2721. Ramon 09/07/26. AWB 12746175415 - 2 volumes retirados na loja GOLLOG - BEL por bispo em 13/07/26. Godoy 15/07/26. Vee One, não temos o recibo assinado. Godoy 16/07/26.</t>
   </si>
   <si>
-    <t>Vee One preferiu atender a demanda com estoque da empresa. Godoy 16/07/26. AWB 12747645135 - volume retirados na loja GOLLOG - CGR por givanildo em 20/07. Godoy 21/07/26.</t>
-  </si>
-  <si>
     <t>Cedeu o item para o C-98 2737. Godoy 21/07/26.</t>
   </si>
   <si>
@@ -407,9 +392,6 @@
   </si>
   <si>
     <t>Nao temos oficina no Brasil para reparo desse item, temos que iniciar processo de aquisiçáo do material para atendimento a essa necessidade ATZ Marcio 17/7/26</t>
-  </si>
-  <si>
-    <t>Material em transito - recibo 576/FAB/26 AWB a ser gerada pela Gollog - Atz Rc 16/07/2026 - awb 12747645135</t>
   </si>
   <si>
     <t>Enviado 1 unidade (CORE) para reparo na oficina no RJ em 17/7, aguardando orçamento com prazo de entrega, ATZ Marcio 17/7</t>
@@ -751,7 +733,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA24"/>
+  <dimension ref="A1:AA23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -845,25 +827,25 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="F2" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="G2">
         <v>2730</v>
       </c>
       <c r="H2" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I2" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="J2" s="1">
         <v>46076</v>
@@ -875,7 +857,7 @@
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="N2" s="1">
         <v>46091</v>
@@ -887,16 +869,16 @@
         <v>144</v>
       </c>
       <c r="S2" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="U2" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="V2" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="W2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -910,25 +892,25 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E3" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="F3" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="G3">
         <v>2721</v>
       </c>
       <c r="H3" t="s">
+        <v>97</v>
+      </c>
+      <c r="I3" t="s">
         <v>101</v>
-      </c>
-      <c r="I3" t="s">
-        <v>105</v>
       </c>
       <c r="J3" s="1">
         <v>46185</v>
@@ -940,7 +922,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="N3" s="1">
         <v>46216</v>
@@ -955,19 +937,19 @@
         <v>39</v>
       </c>
       <c r="S3" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="T3" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="U3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="V3" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="W3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -981,25 +963,25 @@
         <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E4" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="F4" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="G4">
         <v>2726</v>
       </c>
       <c r="H4" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I4" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="J4" s="1">
         <v>46185</v>
@@ -1011,7 +993,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="N4" s="1">
         <v>46192</v>
@@ -1026,16 +1008,16 @@
         <v>39</v>
       </c>
       <c r="S4" t="s">
+        <v>104</v>
+      </c>
+      <c r="U4" t="s">
         <v>108</v>
       </c>
-      <c r="U4" t="s">
-        <v>112</v>
-      </c>
       <c r="V4" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="W4" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -1049,25 +1031,25 @@
         <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E5" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="F5" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="G5">
         <v>2721</v>
       </c>
       <c r="H5" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I5" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="J5" s="1">
         <v>46209</v>
@@ -1079,7 +1061,7 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="N5" s="1">
         <v>46217</v>
@@ -1094,16 +1076,16 @@
         <v>14</v>
       </c>
       <c r="S5" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="T5" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="V5" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="W5" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1117,25 +1099,25 @@
         <v>30</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E6" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F6" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="G6">
         <v>2719</v>
       </c>
       <c r="H6" t="s">
+        <v>97</v>
+      </c>
+      <c r="I6" t="s">
         <v>101</v>
-      </c>
-      <c r="I6" t="s">
-        <v>105</v>
       </c>
       <c r="J6" s="1">
         <v>46210</v>
@@ -1147,7 +1129,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="N6" s="1">
         <v>46241</v>
@@ -1162,13 +1144,13 @@
         <v>14</v>
       </c>
       <c r="S6" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="V6" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="W6" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1182,25 +1164,25 @@
         <v>31</v>
       </c>
       <c r="C7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E7" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F7" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="G7">
         <v>2723</v>
       </c>
       <c r="H7" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I7" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="J7" s="1">
         <v>46210</v>
@@ -1212,7 +1194,7 @@
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="N7" s="1">
         <v>46218</v>
@@ -1227,19 +1209,19 @@
         <v>13</v>
       </c>
       <c r="S7" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="T7" t="s">
+        <v>105</v>
+      </c>
+      <c r="U7" t="s">
         <v>109</v>
       </c>
-      <c r="U7" t="s">
-        <v>113</v>
-      </c>
       <c r="V7" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="W7" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1253,25 +1235,25 @@
         <v>29</v>
       </c>
       <c r="C8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="F8" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="G8">
         <v>2733</v>
       </c>
       <c r="H8" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I8" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="J8" s="1">
         <v>46211</v>
@@ -1283,7 +1265,7 @@
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="N8" s="1">
         <v>46222</v>
@@ -1298,16 +1280,16 @@
         <v>13</v>
       </c>
       <c r="S8" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="T8" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="V8" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="W8" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1321,25 +1303,25 @@
         <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D9" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E9" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="F9" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="G9">
         <v>2726</v>
       </c>
       <c r="H9" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I9" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="J9" s="1">
         <v>46212</v>
@@ -1351,7 +1333,7 @@
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="N9" s="1">
         <v>46219</v>
@@ -1366,16 +1348,16 @@
         <v>12</v>
       </c>
       <c r="S9" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="U9" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="V9" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="W9" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1389,25 +1371,25 @@
         <v>31</v>
       </c>
       <c r="C10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D10" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E10" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="F10" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="G10">
         <v>2723</v>
       </c>
       <c r="H10" t="s">
+        <v>98</v>
+      </c>
+      <c r="I10" t="s">
         <v>102</v>
-      </c>
-      <c r="I10" t="s">
-        <v>106</v>
       </c>
       <c r="J10" s="1">
         <v>46211</v>
@@ -1419,7 +1401,7 @@
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="N10" s="1">
         <v>46219</v>
@@ -1434,16 +1416,16 @@
         <v>12</v>
       </c>
       <c r="S10" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="T10" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="V10" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="W10" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1457,25 +1439,25 @@
         <v>30</v>
       </c>
       <c r="C11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D11" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E11" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="F11" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="G11">
         <v>2702</v>
       </c>
       <c r="H11" t="s">
+        <v>97</v>
+      </c>
+      <c r="I11" t="s">
         <v>101</v>
-      </c>
-      <c r="I11" t="s">
-        <v>105</v>
       </c>
       <c r="J11" s="1">
         <v>46212</v>
@@ -1487,7 +1469,7 @@
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="N11" s="1">
         <v>46243</v>
@@ -1499,13 +1481,13 @@
         <v>12</v>
       </c>
       <c r="S11" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="V11" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="W11" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1519,25 +1501,25 @@
         <v>27</v>
       </c>
       <c r="C12" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D12" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E12" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="F12" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="G12">
         <v>2736</v>
       </c>
       <c r="H12" t="s">
+        <v>97</v>
+      </c>
+      <c r="I12" t="s">
         <v>101</v>
-      </c>
-      <c r="I12" t="s">
-        <v>105</v>
       </c>
       <c r="J12" s="1">
         <v>46216</v>
@@ -1549,7 +1531,7 @@
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="N12" s="1">
         <v>46248</v>
@@ -1561,13 +1543,13 @@
         <v>7</v>
       </c>
       <c r="S12" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="V12" t="s">
+        <v>122</v>
+      </c>
+      <c r="W12" t="s">
         <v>127</v>
-      </c>
-      <c r="W12" t="s">
-        <v>133</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1581,25 +1563,25 @@
         <v>30</v>
       </c>
       <c r="C13" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D13" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E13" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="F13" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="G13">
         <v>2729</v>
       </c>
       <c r="H13" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I13" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="J13" s="1">
         <v>46216</v>
@@ -1611,7 +1593,7 @@
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="N13" s="1">
         <v>46228</v>
@@ -1623,13 +1605,13 @@
         <v>7</v>
       </c>
       <c r="S13" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="T13" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="W13" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1643,25 +1625,25 @@
         <v>30</v>
       </c>
       <c r="C14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D14" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E14" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="F14" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="G14">
         <v>2722</v>
       </c>
       <c r="H14" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I14" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="J14" s="1">
         <v>46217</v>
@@ -1673,7 +1655,7 @@
         <v>1</v>
       </c>
       <c r="M14" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="N14" s="1">
         <v>46229</v>
@@ -1688,16 +1670,16 @@
         <v>6</v>
       </c>
       <c r="S14" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="T14" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="V14" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="W14" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
@@ -1711,25 +1693,25 @@
         <v>30</v>
       </c>
       <c r="C15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D15" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E15" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="F15" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="G15">
         <v>2722</v>
       </c>
       <c r="H15" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I15" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="J15" s="1">
         <v>46219</v>
@@ -1741,7 +1723,7 @@
         <v>1</v>
       </c>
       <c r="M15" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="N15" s="1">
         <v>46229</v>
@@ -1753,16 +1735,16 @@
         <v>6</v>
       </c>
       <c r="S15" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="T15" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="V15" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="W15" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
@@ -1776,25 +1758,25 @@
         <v>30</v>
       </c>
       <c r="C16" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E16" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="F16" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="G16">
         <v>2729</v>
       </c>
       <c r="H16" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I16" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="J16" s="1">
         <v>46219</v>
@@ -1806,7 +1788,7 @@
         <v>1</v>
       </c>
       <c r="M16" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="N16" s="1">
         <v>46230</v>
@@ -1818,16 +1800,16 @@
         <v>5</v>
       </c>
       <c r="S16" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="T16" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="V16" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="W16" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="AA16" t="b">
         <v>1</v>
@@ -1841,25 +1823,25 @@
         <v>30</v>
       </c>
       <c r="C17" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D17" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E17" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="F17" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="G17">
         <v>2703</v>
       </c>
       <c r="H17" t="s">
+        <v>97</v>
+      </c>
+      <c r="I17" t="s">
         <v>101</v>
-      </c>
-      <c r="I17" t="s">
-        <v>105</v>
       </c>
       <c r="J17" s="1">
         <v>46219</v>
@@ -1871,7 +1853,7 @@
         <v>2</v>
       </c>
       <c r="M17" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="N17" s="1">
         <v>46251</v>
@@ -1883,10 +1865,10 @@
         <v>4</v>
       </c>
       <c r="S17" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="W17" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="AA17" t="b">
         <v>1</v>
@@ -1894,31 +1876,31 @@
     </row>
     <row r="18" spans="1:27">
       <c r="A18">
-        <v>690</v>
+        <v>685</v>
       </c>
       <c r="B18" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C18" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D18" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E18" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="F18" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G18">
-        <v>2727</v>
+        <v>2729</v>
       </c>
       <c r="H18" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I18" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="J18" s="1">
         <v>46219</v>
@@ -1930,31 +1912,28 @@
         <v>1</v>
       </c>
       <c r="M18" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="N18" s="1">
-        <v>46228</v>
-      </c>
-      <c r="O18" s="1">
-        <v>46223</v>
+        <v>46232</v>
       </c>
       <c r="Q18">
-        <v>-4</v>
+        <v>-8</v>
       </c>
       <c r="R18">
         <v>3</v>
       </c>
       <c r="S18" t="s">
-        <v>109</v>
-      </c>
-      <c r="U18" t="s">
-        <v>115</v>
+        <v>104</v>
+      </c>
+      <c r="T18" t="s">
+        <v>105</v>
       </c>
       <c r="V18" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="W18" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="AA18" t="b">
         <v>1</v>
@@ -1962,34 +1941,34 @@
     </row>
     <row r="19" spans="1:27">
       <c r="A19">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B19" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C19" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D19" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E19" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="F19" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="G19">
-        <v>2729</v>
+        <v>2730</v>
       </c>
       <c r="H19" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="I19" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="J19" s="1">
-        <v>46219</v>
+        <v>46220</v>
       </c>
       <c r="K19" s="1">
         <v>46221</v>
@@ -1998,28 +1977,28 @@
         <v>1</v>
       </c>
       <c r="M19" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="N19" s="1">
-        <v>46232</v>
+        <v>46228</v>
       </c>
       <c r="Q19">
-        <v>-8</v>
+        <v>-4</v>
       </c>
       <c r="R19">
         <v>3</v>
       </c>
       <c r="S19" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="T19" t="s">
-        <v>109</v>
-      </c>
-      <c r="V19" t="s">
-        <v>132</v>
+        <v>105</v>
+      </c>
+      <c r="U19" t="s">
+        <v>111</v>
       </c>
       <c r="W19" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="AA19" t="b">
         <v>1</v>
@@ -2033,58 +2012,55 @@
         <v>27</v>
       </c>
       <c r="C20" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D20" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E20" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="F20" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="G20">
-        <v>2730</v>
+        <v>2741</v>
       </c>
       <c r="H20" t="s">
+        <v>99</v>
+      </c>
+      <c r="I20" t="s">
+        <v>102</v>
+      </c>
+      <c r="J20" s="1">
+        <v>46224</v>
+      </c>
+      <c r="K20" s="1">
+        <v>46222</v>
+      </c>
+      <c r="L20">
+        <v>1</v>
+      </c>
+      <c r="M20" t="s">
         <v>103</v>
       </c>
-      <c r="I20" t="s">
-        <v>106</v>
-      </c>
-      <c r="J20" s="1">
-        <v>46220</v>
-      </c>
-      <c r="K20" s="1">
-        <v>46221</v>
-      </c>
-      <c r="L20">
-        <v>1</v>
-      </c>
-      <c r="M20" t="s">
-        <v>107</v>
-      </c>
       <c r="N20" s="1">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="Q20">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="R20">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S20" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="T20" t="s">
-        <v>109</v>
-      </c>
-      <c r="U20" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="W20" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="AA20" t="b">
         <v>1</v>
@@ -2092,61 +2068,61 @@
     </row>
     <row r="21" spans="1:27">
       <c r="A21">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B21" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D21" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E21" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="F21" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="G21">
-        <v>2741</v>
+        <v>2720</v>
       </c>
       <c r="H21" t="s">
+        <v>99</v>
+      </c>
+      <c r="I21" t="s">
+        <v>101</v>
+      </c>
+      <c r="J21" s="1">
+        <v>46220</v>
+      </c>
+      <c r="K21" s="1">
+        <v>46223</v>
+      </c>
+      <c r="L21">
+        <v>10</v>
+      </c>
+      <c r="M21" t="s">
         <v>103</v>
       </c>
-      <c r="I21" t="s">
-        <v>106</v>
-      </c>
-      <c r="J21" s="1">
-        <v>46224</v>
-      </c>
-      <c r="K21" s="1">
-        <v>46222</v>
-      </c>
-      <c r="L21">
-        <v>1</v>
-      </c>
-      <c r="M21" t="s">
-        <v>107</v>
-      </c>
       <c r="N21" s="1">
-        <v>46229</v>
+        <v>46254</v>
       </c>
       <c r="Q21">
-        <v>-5</v>
+        <v>-30</v>
       </c>
       <c r="R21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S21" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="T21" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="W21" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="AA21" t="b">
         <v>1</v>
@@ -2160,55 +2136,55 @@
         <v>28</v>
       </c>
       <c r="C22" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D22" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E22" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="F22" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="G22">
         <v>2720</v>
       </c>
       <c r="H22" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="I22" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="J22" s="1">
         <v>46220</v>
       </c>
       <c r="K22" s="1">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="L22">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="M22" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="N22" s="1">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="Q22">
-        <v>-30</v>
+        <v>-31</v>
       </c>
       <c r="R22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S22" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="T22" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="W22" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="AA22" t="b">
         <v>1</v>
@@ -2222,119 +2198,57 @@
         <v>28</v>
       </c>
       <c r="C23" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D23" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E23" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="F23" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="G23">
         <v>2720</v>
       </c>
       <c r="H23" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="I23" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="J23" s="1">
         <v>46220</v>
       </c>
       <c r="K23" s="1">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="L23">
         <v>6</v>
       </c>
       <c r="M23" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="N23" s="1">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="Q23">
-        <v>-31</v>
+        <v>-32</v>
       </c>
       <c r="R23">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="S23" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="T23" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="W23" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="AA23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:27">
-      <c r="A24">
-        <v>329</v>
-      </c>
-      <c r="B24" t="s">
-        <v>28</v>
-      </c>
-      <c r="C24" t="s">
-        <v>55</v>
-      </c>
-      <c r="D24" t="s">
-        <v>77</v>
-      </c>
-      <c r="E24" t="s">
-        <v>97</v>
-      </c>
-      <c r="F24" t="s">
-        <v>98</v>
-      </c>
-      <c r="G24">
-        <v>2720</v>
-      </c>
-      <c r="H24" t="s">
-        <v>103</v>
-      </c>
-      <c r="I24" t="s">
-        <v>105</v>
-      </c>
-      <c r="J24" s="1">
-        <v>46220</v>
-      </c>
-      <c r="K24" s="1">
-        <v>46225</v>
-      </c>
-      <c r="L24">
-        <v>6</v>
-      </c>
-      <c r="M24" t="s">
-        <v>107</v>
-      </c>
-      <c r="N24" s="1">
-        <v>46256</v>
-      </c>
-      <c r="Q24">
-        <v>-32</v>
-      </c>
-      <c r="R24">
-        <v>-1</v>
-      </c>
-      <c r="S24" t="s">
-        <v>109</v>
-      </c>
-      <c r="T24" t="s">
-        <v>108</v>
-      </c>
-      <c r="W24" t="s">
-        <v>133</v>
-      </c>
-      <c r="AA24" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (22/07/2026 12:01)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="130">
   <si>
     <t>om_emg</t>
   </si>
@@ -103,24 +103,21 @@
     <t>BABR</t>
   </si>
   <si>
+    <t>BANT</t>
+  </si>
+  <si>
+    <t>CLA</t>
+  </si>
+  <si>
     <t>BABE</t>
   </si>
   <si>
-    <t>BANT</t>
-  </si>
-  <si>
-    <t>CLA</t>
-  </si>
-  <si>
     <t>313260017747</t>
   </si>
   <si>
     <t>329260019153</t>
   </si>
   <si>
-    <t>396260016520</t>
-  </si>
-  <si>
     <t>329260019181</t>
   </si>
   <si>
@@ -148,9 +145,6 @@
     <t>685260012368</t>
   </si>
   <si>
-    <t>685260012377</t>
-  </si>
-  <si>
     <t>685260012387</t>
   </si>
   <si>
@@ -178,15 +172,15 @@
     <t>329260019227</t>
   </si>
   <si>
+    <t>329260019241</t>
+  </si>
+  <si>
     <t>1214134-1</t>
   </si>
   <si>
     <t>TWINA0502</t>
   </si>
   <si>
-    <t>1H75-21</t>
-  </si>
-  <si>
     <t>C145-00-46</t>
   </si>
   <si>
@@ -241,15 +235,15 @@
     <t>2625014-9</t>
   </si>
   <si>
+    <t>9910592-2</t>
+  </si>
+  <si>
     <t>BELLCRANK ASSY</t>
   </si>
   <si>
     <t>PROBE TEMPERATURE</t>
   </si>
   <si>
-    <t>PRESSURE REGULATOR</t>
-  </si>
-  <si>
     <t>TRANSMISSION ASSY</t>
   </si>
   <si>
@@ -298,6 +292,9 @@
     <t>SPACER</t>
   </si>
   <si>
+    <t>ALTERNADOR</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -340,15 +337,18 @@
     <t>Volume retirado na loja GOLLOG - BSB por tanise Assis em 03/07/2026 - Godoy 08/07/2026. Recibo não se encontra na Pasta do DRIVE. Godoy 08/07/2026.</t>
   </si>
   <si>
-    <t>Item retirado para atender o C-98 2731. Ramon 15/06/26. AWB 12746187256 - volume retirado na loja GOLLOG - BEL por bispo em 13/07. Godoy 16/07/26. Recibo não se encontra na Pasta do DRIVE. Godoy 17/07/2026.</t>
-  </si>
-  <si>
     <t>AWB 12745918331 volume retirado na loja GOLLOG - BEL por bispo em 10/07/2026 - Godoy 13/07/2026. Recibo não se encontra na Pasta do DRIVE. Godoy 17/07/2026.</t>
   </si>
   <si>
     <t>Cedeu o item para o C-98 2721. Ramon 09/07/26. AWB 12746175415 - 2 volumes retirados na loja GOLLOG - BEL por bispo em 13/07/26. Godoy 15/07/26. Vee One, não temos o recibo assinado. Godoy 16/07/26.</t>
   </si>
   <si>
+    <t>AWB 12747899051 volume retirado na loja GOLLOG - BEL por marlos em 20/07. Godoy 22/07/2026.</t>
+  </si>
+  <si>
+    <t>Alterado o tipo da emerg. de IPLR para ANCE. Godoy 22/07/26</t>
+  </si>
+  <si>
     <t>Cedeu o item para o C-98 2737. Godoy 21/07/26.</t>
   </si>
   <si>
@@ -358,43 +358,49 @@
     <t>Colocado pedido na Textron IJ17507011. Previsão de entrega em Miami 17/06. Carga recepcionada no GIG 24/06. Canal verde dia 26/06. DPE V1 29/06. Verificar entrega do item. ATZ 30/06 - MATERIAL EM RECEBIMENTO V1 30-06-2026 - MATERIAL EM PROCESSO DE ENVIO RECIBO 524/FAB/26 ATZ RC 30-06-2026 - MATERIAL EM TRANSITO - AWB 12744330731 DPE 03/07/2026 - MATERIAL RECEBIDO POR tanise Assis RG 14807641751 DIA 03/07/2026</t>
   </si>
   <si>
-    <t>04 ea recolhidos para a V1, chegada dos itens dia 23/06/2026. Itens não tem oficina no Brasil, terá que ser feito Exchange rc 23/06 - MATERIAL ADQUIRIDO FORNECEDOR TEXTRON -WB0003073549 Inovice IJ17534800 DPE AGS Miami 29/6/2026 ate 10 30AM - AIR EXPORT HOUSE: 00004046 de 30/6/2026 Chegou no GIGRJ em 01/7/26 para Desembaraço - ATZ Marcio 3/7/26 CANAL VERDE EM 7/7/26 entregue V1 em 8/7/26 ATZ Marcio 9/7/26 - MATERIAL EM TRANSITO - RECIBO 560/FAB/26 AWB - 12746187256 DPE 13/07/2026</t>
-  </si>
-  <si>
     <t>Colocado pedido AOG Textron IJ17557538 - previsão de entrega em Miami 08/07. Previsão de chegada GIG 09/07 - MATERIAL EM TRANSITO - RECIBO 551/FAB/26 - ENVIADO PN COMPLETO PARA SANAR A EMERGENCIA DO 2709, ENVIADO MODAL TERRESTRE, DPE 13/07/2026</t>
   </si>
   <si>
-    <t>DPE 17/07/2026(REZ 09/07/26)</t>
+    <t>confirmado entrega 01 ea hj(21/07/26) pela William - REZ</t>
   </si>
   <si>
     <t>MATERIAL EM TRANSITO - AWB 12745918331 dpe 11/07/2026 - atz rc 08/07/2026</t>
   </si>
   <si>
-    <t>Aguardando APROVAÇÃO PO 793/JPA/2026 em referencia ao orçamento 0274/26 - Prazo oficina 15 dias após aprovação. ATZ Marcio 9/7/26 14:50</t>
+    <t>Aguardando APROVAÇÃO PO 793/JPA/2026 em referencia ao orçamento 0274/26 - Prazo oficina 15 dias após aprovação. ATZ Marcio 9/7/26 14:50 ( MATERIAL EM SEPAÇÃO EM JPA - V1 ) 20/07 15:40.</t>
   </si>
   <si>
     <t>Atendido em 09/07/26 AWB 12746175415 - CLA (09/07/26)</t>
   </si>
   <si>
-    <t>Aguardando o retorno dos subcomponentes removidos da unidade para ser enviado a oficiana para aplicação na unidade Prazo apos aprovação 10 dias ATZ Marcio 9/7/26 14 53</t>
-  </si>
-  <si>
-    <t>Colocado pedido junto ao fornecedor AEROBASE, aguardando pagamento proforma. ATZ 16/07</t>
-  </si>
-  <si>
-    <t>Colocado pedido Textron IJ17575583 - entregue em Miami 15/07. Será consolidado próximo voo GIG</t>
-  </si>
-  <si>
-    <t>Previsão 17/07 da oficina de BH - material em transito - recibo 582/FAB/26 AWB A SER GERADA PELA GOLLOG ATZ 17/07/2026</t>
-  </si>
-  <si>
-    <t>Item em bancada porem em pessimo estado, foi solicitado recolhimento de mais unidades para envio a oficina para tentativa de reparo ATZ Marcio 17/7/26</t>
-  </si>
-  <si>
-    <t>Nao temos oficina no Brasil para reparo desse item, temos que iniciar processo de aquisiçáo do material para atendimento a essa necessidade ATZ Marcio 17/7/26</t>
+    <t>Aguardando o retorno dos subcomponentes removidos da unidade para ser enviado a oficiana para aplicação na unidade Prazo apos aprovação 10 dias ATZ Marcio 9/7/26 14 53 - Enviado uma FCU em 17/7 fornecida pela FAB , ATZ Macio, Aguardando a atualização com o recibo e AWB ATZ Marcio 20/7 - FCU ENVIADA FOI RECUSADA PELA INSPETORIA DE RECEBIMENTO DA BABE - 20/07/2026 RC - ITEM ATENDIDO COM ESTOQUE FAB AWB 127-4789 9051</t>
+  </si>
+  <si>
+    <t>Colocado pedido junto ao fornecedor AEROBASE, aguardando pagamento proforma. ATZ 21/07</t>
+  </si>
+  <si>
+    <t>Colocado pedido Textron IJ17575583 - entregue em Miami 15/07. Carga rercepcionada GIG 19/07 - Aguardando liberação do SEFAZ. ATZ 21/07</t>
+  </si>
+  <si>
+    <t>Checando se consegue priorizar 20/7 com a oficina em BH se consegue entregar mais 1 unidade (William) , o item que esta na Av aeronautica tem a probabilidade de estar SCRAP (nao pegar reparo e voltar no estado msg de 20/7 do Sr. Ricardo da AV.) - Atz Marcio 20/7 11:13hs - confirmado entrega 01 ea hj(21/07/26) pela William - REZ</t>
+  </si>
+  <si>
+    <t>Item em bancada porem em pessimo estado, foi solicitado recolhimento de mais unidades para envio a oficina para tentativa de reparo ATZ Marcio 17/7/26. Solicitado abertura de O.S. para 3EA do item no dia 16-07-26 via Email para a Coordenadoria - CLA-21-07-26</t>
+  </si>
+  <si>
+    <t>Nao temos oficina no Brasil para reparo desse item, temos que iniciar processo de aquisiçáo do material para atendimento a essa necessidade ATZ Marcio 17/7/26 - Efetuada compra em AOG , aguardando o AWB de envio para Natal, peça saindo do Espirito Santo ATZ Marcio 20/7 15:54</t>
+  </si>
+  <si>
+    <t>Validando atendimento via estoque FAB. ATZ 20/07</t>
   </si>
   <si>
     <t>Enviado 1 unidade (CORE) para reparo na oficina no RJ em 17/7, aguardando orçamento com prazo de entrega, ATZ Marcio 17/7</t>
+  </si>
+  <si>
+    <t>TEMOS EM ESTOQUE NA BASE PAMALS, SERÁ ENVIADO. CLA-21-07</t>
+  </si>
+  <si>
+    <t>PEDIDO NO EPM E-C98-26059 - CLA-21-07</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -407,8 +413,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -424,7 +438,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -432,12 +446,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -733,89 +765,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA23"/>
+  <dimension ref="A1:AA22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -830,55 +862,55 @@
         <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G2">
         <v>2730</v>
       </c>
       <c r="H2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I2" t="s">
-        <v>100</v>
-      </c>
-      <c r="J2" s="1">
+        <v>99</v>
+      </c>
+      <c r="J2" s="2">
         <v>46076</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46080</v>
       </c>
       <c r="L2">
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>103</v>
-      </c>
-      <c r="N2" s="1">
+        <v>102</v>
+      </c>
+      <c r="N2" s="2">
         <v>46091</v>
       </c>
       <c r="Q2">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="R2">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="S2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="U2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="V2" t="s">
         <v>112</v>
       </c>
       <c r="W2" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -895,61 +927,61 @@
         <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G3">
         <v>2721</v>
       </c>
       <c r="H3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I3" t="s">
-        <v>101</v>
-      </c>
-      <c r="J3" s="1">
+        <v>100</v>
+      </c>
+      <c r="J3" s="2">
         <v>46185</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46185</v>
       </c>
       <c r="L3">
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>103</v>
-      </c>
-      <c r="N3" s="1">
+        <v>102</v>
+      </c>
+      <c r="N3" s="2">
         <v>46216</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46216</v>
       </c>
       <c r="Q3">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R3">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="S3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="U3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="V3" t="s">
         <v>113</v>
       </c>
       <c r="W3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -957,67 +989,67 @@
     </row>
     <row r="4" spans="1:27">
       <c r="A4">
-        <v>396</v>
+        <v>329</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s">
         <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="G4">
-        <v>2726</v>
+        <v>2721</v>
       </c>
       <c r="H4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I4" t="s">
+        <v>101</v>
+      </c>
+      <c r="J4" s="2">
+        <v>46209</v>
+      </c>
+      <c r="K4" s="2">
+        <v>46210</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4" t="s">
         <v>102</v>
       </c>
-      <c r="J4" s="1">
-        <v>46185</v>
-      </c>
-      <c r="K4" s="1">
-        <v>46185</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4" t="s">
-        <v>103</v>
-      </c>
-      <c r="N4" s="1">
-        <v>46192</v>
-      </c>
-      <c r="O4" s="1">
+      <c r="N4" s="2">
+        <v>46217</v>
+      </c>
+      <c r="O4" s="2">
         <v>46216</v>
       </c>
       <c r="Q4">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="R4">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="S4" t="s">
-        <v>104</v>
-      </c>
-      <c r="U4" t="s">
-        <v>108</v>
+        <v>103</v>
+      </c>
+      <c r="T4" t="s">
+        <v>103</v>
       </c>
       <c r="V4" t="s">
         <v>114</v>
       </c>
       <c r="W4" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -1025,67 +1057,64 @@
     </row>
     <row r="5" spans="1:27">
       <c r="A5">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C5" t="s">
         <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F5" t="s">
         <v>94</v>
       </c>
       <c r="G5">
-        <v>2721</v>
+        <v>2719</v>
       </c>
       <c r="H5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I5" t="s">
+        <v>100</v>
+      </c>
+      <c r="J5" s="2">
+        <v>46210</v>
+      </c>
+      <c r="K5" s="2">
+        <v>46210</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5" t="s">
         <v>102</v>
       </c>
-      <c r="J5" s="1">
-        <v>46209</v>
-      </c>
-      <c r="K5" s="1">
-        <v>46210</v>
-      </c>
-      <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5" t="s">
-        <v>103</v>
-      </c>
-      <c r="N5" s="1">
-        <v>46217</v>
-      </c>
-      <c r="O5" s="1">
-        <v>46216</v>
+      <c r="N5" s="2">
+        <v>46241</v>
+      </c>
+      <c r="O5" s="2">
+        <v>46238</v>
       </c>
       <c r="Q5">
-        <v>7</v>
+        <v>-16</v>
       </c>
       <c r="R5">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S5" t="s">
-        <v>104</v>
-      </c>
-      <c r="T5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="V5" t="s">
         <v>115</v>
       </c>
       <c r="W5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1093,7 +1122,7 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6">
-        <v>685</v>
+        <v>419</v>
       </c>
       <c r="B6" t="s">
         <v>30</v>
@@ -1102,55 +1131,61 @@
         <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F6" t="s">
         <v>95</v>
       </c>
       <c r="G6">
-        <v>2719</v>
+        <v>2723</v>
       </c>
       <c r="H6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I6" t="s">
         <v>101</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>46210</v>
       </c>
-      <c r="K6" s="1">
-        <v>46210</v>
+      <c r="K6" s="2">
+        <v>46211</v>
       </c>
       <c r="L6">
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>103</v>
-      </c>
-      <c r="N6" s="1">
-        <v>46241</v>
-      </c>
-      <c r="O6" s="1">
-        <v>46238</v>
+        <v>102</v>
+      </c>
+      <c r="N6" s="2">
+        <v>46218</v>
+      </c>
+      <c r="O6" s="2">
+        <v>46213</v>
       </c>
       <c r="Q6">
-        <v>-17</v>
+        <v>7</v>
       </c>
       <c r="R6">
         <v>14</v>
       </c>
       <c r="S6" t="s">
+        <v>103</v>
+      </c>
+      <c r="T6" t="s">
         <v>104</v>
+      </c>
+      <c r="U6" t="s">
+        <v>107</v>
       </c>
       <c r="V6" t="s">
         <v>116</v>
       </c>
       <c r="W6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1158,7 +1193,7 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>419</v>
+        <v>396</v>
       </c>
       <c r="B7" t="s">
         <v>31</v>
@@ -1167,61 +1202,58 @@
         <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F7" t="s">
+        <v>95</v>
+      </c>
+      <c r="G7">
+        <v>2733</v>
+      </c>
+      <c r="H7" t="s">
         <v>96</v>
       </c>
-      <c r="G7">
-        <v>2723</v>
-      </c>
-      <c r="H7" t="s">
-        <v>97</v>
-      </c>
       <c r="I7" t="s">
+        <v>99</v>
+      </c>
+      <c r="J7" s="2">
+        <v>46211</v>
+      </c>
+      <c r="K7" s="2">
+        <v>46211</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7" t="s">
         <v>102</v>
       </c>
-      <c r="J7" s="1">
-        <v>46210</v>
-      </c>
-      <c r="K7" s="1">
-        <v>46211</v>
-      </c>
-      <c r="L7">
-        <v>1</v>
-      </c>
-      <c r="M7" t="s">
-        <v>103</v>
-      </c>
-      <c r="N7" s="1">
-        <v>46218</v>
-      </c>
-      <c r="O7" s="1">
-        <v>46213</v>
+      <c r="N7" s="2">
+        <v>46222</v>
+      </c>
+      <c r="O7" s="2">
+        <v>46237</v>
       </c>
       <c r="Q7">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R7">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S7" t="s">
+        <v>103</v>
+      </c>
+      <c r="T7" t="s">
         <v>104</v>
-      </c>
-      <c r="T7" t="s">
-        <v>105</v>
-      </c>
-      <c r="U7" t="s">
-        <v>109</v>
       </c>
       <c r="V7" t="s">
         <v>117</v>
       </c>
       <c r="W7" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1232,49 +1264,49 @@
         <v>396</v>
       </c>
       <c r="B8" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C8" t="s">
         <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F8" t="s">
+        <v>95</v>
+      </c>
+      <c r="G8">
+        <v>2726</v>
+      </c>
+      <c r="H8" t="s">
         <v>96</v>
       </c>
-      <c r="G8">
-        <v>2733</v>
-      </c>
-      <c r="H8" t="s">
-        <v>97</v>
-      </c>
       <c r="I8" t="s">
-        <v>100</v>
-      </c>
-      <c r="J8" s="1">
-        <v>46211</v>
-      </c>
-      <c r="K8" s="1">
-        <v>46211</v>
+        <v>101</v>
+      </c>
+      <c r="J8" s="2">
+        <v>46212</v>
+      </c>
+      <c r="K8" s="2">
+        <v>46212</v>
       </c>
       <c r="L8">
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>103</v>
-      </c>
-      <c r="N8" s="1">
-        <v>46222</v>
-      </c>
-      <c r="O8" s="1">
-        <v>46237</v>
+        <v>102</v>
+      </c>
+      <c r="N8" s="2">
+        <v>46219</v>
+      </c>
+      <c r="O8" s="2">
+        <v>46216</v>
       </c>
       <c r="Q8">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="R8">
         <v>13</v>
@@ -1282,14 +1314,14 @@
       <c r="S8" t="s">
         <v>104</v>
       </c>
-      <c r="T8" t="s">
-        <v>105</v>
+      <c r="U8" t="s">
+        <v>108</v>
       </c>
       <c r="V8" t="s">
         <v>118</v>
       </c>
       <c r="W8" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1297,67 +1329,70 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9">
-        <v>396</v>
+        <v>419</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C9" t="s">
         <v>39</v>
       </c>
       <c r="D9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G9">
-        <v>2726</v>
+        <v>2723</v>
       </c>
       <c r="H9" t="s">
         <v>97</v>
       </c>
       <c r="I9" t="s">
+        <v>101</v>
+      </c>
+      <c r="J9" s="2">
+        <v>46211</v>
+      </c>
+      <c r="K9" s="2">
+        <v>46212</v>
+      </c>
+      <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9" t="s">
         <v>102</v>
       </c>
-      <c r="J9" s="1">
-        <v>46212</v>
-      </c>
-      <c r="K9" s="1">
-        <v>46212</v>
-      </c>
-      <c r="L9">
-        <v>1</v>
-      </c>
-      <c r="M9" t="s">
-        <v>103</v>
-      </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>46219</v>
       </c>
-      <c r="O9" s="1">
-        <v>46216</v>
+      <c r="O9" s="2">
+        <v>46237</v>
       </c>
       <c r="Q9">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R9">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S9" t="s">
-        <v>105</v>
+        <v>103</v>
+      </c>
+      <c r="T9" t="s">
+        <v>103</v>
       </c>
       <c r="U9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="V9" t="s">
         <v>119</v>
       </c>
       <c r="W9" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1365,67 +1400,61 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>419</v>
+        <v>685</v>
       </c>
       <c r="B10" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C10" t="s">
         <v>40</v>
       </c>
       <c r="D10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F10" t="s">
+        <v>93</v>
+      </c>
+      <c r="G10">
+        <v>2702</v>
+      </c>
+      <c r="H10" t="s">
         <v>96</v>
       </c>
-      <c r="G10">
-        <v>2723</v>
-      </c>
-      <c r="H10" t="s">
-        <v>98</v>
-      </c>
       <c r="I10" t="s">
+        <v>100</v>
+      </c>
+      <c r="J10" s="2">
+        <v>46212</v>
+      </c>
+      <c r="K10" s="2">
+        <v>46212</v>
+      </c>
+      <c r="L10">
+        <v>1</v>
+      </c>
+      <c r="M10" t="s">
         <v>102</v>
       </c>
-      <c r="J10" s="1">
-        <v>46211</v>
-      </c>
-      <c r="K10" s="1">
-        <v>46212</v>
-      </c>
-      <c r="L10">
-        <v>1</v>
-      </c>
-      <c r="M10" t="s">
-        <v>103</v>
-      </c>
-      <c r="N10" s="1">
-        <v>46219</v>
-      </c>
-      <c r="O10" s="1">
-        <v>46237</v>
+      <c r="N10" s="2">
+        <v>46243</v>
       </c>
       <c r="Q10">
-        <v>5</v>
+        <v>-18</v>
       </c>
       <c r="R10">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S10" t="s">
-        <v>104</v>
-      </c>
-      <c r="T10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="V10" t="s">
         <v>120</v>
       </c>
       <c r="W10" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1433,61 +1462,64 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C11" t="s">
         <v>41</v>
       </c>
       <c r="D11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E11" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G11">
-        <v>2702</v>
+        <v>2736</v>
       </c>
       <c r="H11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I11" t="s">
-        <v>101</v>
-      </c>
-      <c r="J11" s="1">
-        <v>46212</v>
-      </c>
-      <c r="K11" s="1">
-        <v>46212</v>
+        <v>100</v>
+      </c>
+      <c r="J11" s="2">
+        <v>46216</v>
+      </c>
+      <c r="K11" s="2">
+        <v>46217</v>
       </c>
       <c r="L11">
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>103</v>
-      </c>
-      <c r="N11" s="1">
-        <v>46243</v>
+        <v>102</v>
+      </c>
+      <c r="N11" s="2">
+        <v>46248</v>
+      </c>
+      <c r="O11" s="2">
+        <v>46248</v>
       </c>
       <c r="Q11">
-        <v>-19</v>
+        <v>-23</v>
       </c>
       <c r="R11">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="S11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="V11" t="s">
         <v>121</v>
       </c>
       <c r="W11" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1495,61 +1527,64 @@
     </row>
     <row r="12" spans="1:27">
       <c r="A12">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C12" t="s">
         <v>42</v>
       </c>
       <c r="D12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E12" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F12" t="s">
         <v>94</v>
       </c>
       <c r="G12">
-        <v>2736</v>
+        <v>2729</v>
       </c>
       <c r="H12" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I12" t="s">
-        <v>101</v>
-      </c>
-      <c r="J12" s="1">
+        <v>99</v>
+      </c>
+      <c r="J12" s="2">
         <v>46216</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>46217</v>
       </c>
       <c r="L12">
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>103</v>
-      </c>
-      <c r="N12" s="1">
-        <v>46248</v>
+        <v>102</v>
+      </c>
+      <c r="N12" s="2">
+        <v>46228</v>
       </c>
       <c r="Q12">
-        <v>-24</v>
+        <v>-3</v>
       </c>
       <c r="R12">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S12" t="s">
+        <v>103</v>
+      </c>
+      <c r="T12" t="s">
         <v>104</v>
       </c>
       <c r="V12" t="s">
         <v>122</v>
       </c>
       <c r="W12" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1560,58 +1595,64 @@
         <v>685</v>
       </c>
       <c r="B13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C13" t="s">
         <v>43</v>
       </c>
       <c r="D13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E13" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F13" t="s">
         <v>95</v>
       </c>
       <c r="G13">
-        <v>2729</v>
+        <v>2722</v>
       </c>
       <c r="H13" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I13" t="s">
         <v>100</v>
       </c>
-      <c r="J13" s="1">
-        <v>46216</v>
-      </c>
-      <c r="K13" s="1">
-        <v>46217</v>
+      <c r="J13" s="2">
+        <v>46219</v>
+      </c>
+      <c r="K13" s="2">
+        <v>46218</v>
       </c>
       <c r="L13">
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>103</v>
-      </c>
-      <c r="N13" s="1">
-        <v>46228</v>
+        <v>102</v>
+      </c>
+      <c r="N13" s="2">
+        <v>46249</v>
       </c>
       <c r="Q13">
-        <v>-4</v>
+        <v>-24</v>
       </c>
       <c r="R13">
         <v>7</v>
       </c>
       <c r="S13" t="s">
+        <v>103</v>
+      </c>
+      <c r="T13" t="s">
         <v>104</v>
       </c>
-      <c r="T13" t="s">
-        <v>105</v>
+      <c r="U13" t="s">
+        <v>110</v>
+      </c>
+      <c r="V13" t="s">
+        <v>123</v>
       </c>
       <c r="W13" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1622,7 +1663,7 @@
         <v>685</v>
       </c>
       <c r="B14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C14" t="s">
         <v>44</v>
@@ -1634,34 +1675,31 @@
         <v>85</v>
       </c>
       <c r="F14" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G14">
-        <v>2722</v>
+        <v>2729</v>
       </c>
       <c r="H14" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I14" t="s">
-        <v>100</v>
-      </c>
-      <c r="J14" s="1">
-        <v>46217</v>
-      </c>
-      <c r="K14" s="1">
-        <v>46218</v>
+        <v>99</v>
+      </c>
+      <c r="J14" s="2">
+        <v>46219</v>
+      </c>
+      <c r="K14" s="2">
+        <v>46219</v>
       </c>
       <c r="L14">
         <v>1</v>
       </c>
       <c r="M14" t="s">
-        <v>103</v>
-      </c>
-      <c r="N14" s="1">
-        <v>46229</v>
-      </c>
-      <c r="O14" s="1">
-        <v>46223</v>
+        <v>102</v>
+      </c>
+      <c r="N14" s="2">
+        <v>46230</v>
       </c>
       <c r="Q14">
         <v>-5</v>
@@ -1670,16 +1708,16 @@
         <v>6</v>
       </c>
       <c r="S14" t="s">
+        <v>103</v>
+      </c>
+      <c r="T14" t="s">
         <v>104</v>
       </c>
-      <c r="T14" t="s">
-        <v>105</v>
-      </c>
       <c r="V14" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="W14" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
@@ -1690,7 +1728,7 @@
         <v>685</v>
       </c>
       <c r="B15" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C15" t="s">
         <v>45</v>
@@ -1702,49 +1740,46 @@
         <v>86</v>
       </c>
       <c r="F15" t="s">
+        <v>93</v>
+      </c>
+      <c r="G15">
+        <v>2703</v>
+      </c>
+      <c r="H15" t="s">
         <v>96</v>
-      </c>
-      <c r="G15">
-        <v>2722</v>
-      </c>
-      <c r="H15" t="s">
-        <v>97</v>
       </c>
       <c r="I15" t="s">
         <v>100</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46219</v>
       </c>
-      <c r="K15" s="1">
-        <v>46218</v>
+      <c r="K15" s="2">
+        <v>46220</v>
       </c>
       <c r="L15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M15" t="s">
-        <v>103</v>
-      </c>
-      <c r="N15" s="1">
-        <v>46229</v>
+        <v>102</v>
+      </c>
+      <c r="N15" s="2">
+        <v>46251</v>
       </c>
       <c r="Q15">
-        <v>-5</v>
+        <v>-26</v>
       </c>
       <c r="R15">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S15" t="s">
         <v>104</v>
       </c>
-      <c r="T15" t="s">
-        <v>105</v>
-      </c>
       <c r="V15" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="W15" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
@@ -1755,7 +1790,7 @@
         <v>685</v>
       </c>
       <c r="B16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C16" t="s">
         <v>46</v>
@@ -1773,43 +1808,43 @@
         <v>2729</v>
       </c>
       <c r="H16" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I16" t="s">
-        <v>100</v>
-      </c>
-      <c r="J16" s="1">
+        <v>99</v>
+      </c>
+      <c r="J16" s="2">
         <v>46219</v>
       </c>
-      <c r="K16" s="1">
-        <v>46219</v>
+      <c r="K16" s="2">
+        <v>46221</v>
       </c>
       <c r="L16">
         <v>1</v>
       </c>
       <c r="M16" t="s">
-        <v>103</v>
-      </c>
-      <c r="N16" s="1">
-        <v>46230</v>
+        <v>102</v>
+      </c>
+      <c r="N16" s="2">
+        <v>46232</v>
       </c>
       <c r="Q16">
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="R16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S16" t="s">
+        <v>103</v>
+      </c>
+      <c r="T16" t="s">
         <v>104</v>
       </c>
-      <c r="T16" t="s">
-        <v>105</v>
-      </c>
       <c r="V16" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="W16" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="AA16" t="b">
         <v>1</v>
@@ -1817,10 +1852,10 @@
     </row>
     <row r="17" spans="1:27">
       <c r="A17">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B17" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C17" t="s">
         <v>47</v>
@@ -1832,10 +1867,10 @@
         <v>88</v>
       </c>
       <c r="F17" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G17">
-        <v>2703</v>
+        <v>2730</v>
       </c>
       <c r="H17" t="s">
         <v>97</v>
@@ -1843,32 +1878,38 @@
       <c r="I17" t="s">
         <v>101</v>
       </c>
-      <c r="J17" s="1">
-        <v>46219</v>
-      </c>
-      <c r="K17" s="1">
+      <c r="J17" s="2">
         <v>46220</v>
       </c>
+      <c r="K17" s="2">
+        <v>46221</v>
+      </c>
       <c r="L17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M17" t="s">
-        <v>103</v>
-      </c>
-      <c r="N17" s="1">
-        <v>46251</v>
+        <v>102</v>
+      </c>
+      <c r="N17" s="2">
+        <v>46228</v>
       </c>
       <c r="Q17">
-        <v>-27</v>
+        <v>-3</v>
       </c>
       <c r="R17">
         <v>4</v>
       </c>
       <c r="S17" t="s">
-        <v>105</v>
+        <v>103</v>
+      </c>
+      <c r="T17" t="s">
+        <v>104</v>
+      </c>
+      <c r="U17" t="s">
+        <v>111</v>
       </c>
       <c r="W17" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="AA17" t="b">
         <v>1</v>
@@ -1876,10 +1917,10 @@
     </row>
     <row r="18" spans="1:27">
       <c r="A18">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B18" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C18" t="s">
         <v>48</v>
@@ -1891,49 +1932,49 @@
         <v>89</v>
       </c>
       <c r="F18" t="s">
+        <v>95</v>
+      </c>
+      <c r="G18">
+        <v>2741</v>
+      </c>
+      <c r="H18" t="s">
         <v>96</v>
       </c>
-      <c r="G18">
-        <v>2729</v>
-      </c>
-      <c r="H18" t="s">
-        <v>97</v>
-      </c>
       <c r="I18" t="s">
-        <v>100</v>
-      </c>
-      <c r="J18" s="1">
-        <v>46219</v>
-      </c>
-      <c r="K18" s="1">
-        <v>46221</v>
+        <v>101</v>
+      </c>
+      <c r="J18" s="2">
+        <v>46224</v>
+      </c>
+      <c r="K18" s="2">
+        <v>46222</v>
       </c>
       <c r="L18">
         <v>1</v>
       </c>
       <c r="M18" t="s">
-        <v>103</v>
-      </c>
-      <c r="N18" s="1">
-        <v>46232</v>
+        <v>102</v>
+      </c>
+      <c r="N18" s="2">
+        <v>46229</v>
       </c>
       <c r="Q18">
-        <v>-8</v>
+        <v>-4</v>
       </c>
       <c r="R18">
         <v>3</v>
       </c>
       <c r="S18" t="s">
+        <v>103</v>
+      </c>
+      <c r="T18" t="s">
         <v>104</v>
       </c>
-      <c r="T18" t="s">
-        <v>105</v>
-      </c>
       <c r="V18" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="W18" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="AA18" t="b">
         <v>1</v>
@@ -1941,10 +1982,10 @@
     </row>
     <row r="19" spans="1:27">
       <c r="A19">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B19" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C19" t="s">
         <v>49</v>
@@ -1956,49 +1997,49 @@
         <v>90</v>
       </c>
       <c r="F19" t="s">
+        <v>93</v>
+      </c>
+      <c r="G19">
+        <v>2720</v>
+      </c>
+      <c r="H19" t="s">
         <v>96</v>
       </c>
-      <c r="G19">
-        <v>2730</v>
-      </c>
-      <c r="H19" t="s">
-        <v>99</v>
-      </c>
       <c r="I19" t="s">
+        <v>100</v>
+      </c>
+      <c r="J19" s="2">
+        <v>46220</v>
+      </c>
+      <c r="K19" s="2">
+        <v>46223</v>
+      </c>
+      <c r="L19">
+        <v>10</v>
+      </c>
+      <c r="M19" t="s">
         <v>102</v>
       </c>
-      <c r="J19" s="1">
-        <v>46220</v>
-      </c>
-      <c r="K19" s="1">
-        <v>46221</v>
-      </c>
-      <c r="L19">
-        <v>1</v>
-      </c>
-      <c r="M19" t="s">
-        <v>103</v>
-      </c>
-      <c r="N19" s="1">
-        <v>46228</v>
+      <c r="N19" s="2">
+        <v>46254</v>
       </c>
       <c r="Q19">
-        <v>-4</v>
+        <v>-29</v>
       </c>
       <c r="R19">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S19" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T19" t="s">
-        <v>105</v>
-      </c>
-      <c r="U19" t="s">
-        <v>111</v>
+        <v>103</v>
+      </c>
+      <c r="V19" t="s">
+        <v>128</v>
       </c>
       <c r="W19" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="AA19" t="b">
         <v>1</v>
@@ -2006,10 +2047,10 @@
     </row>
     <row r="20" spans="1:27">
       <c r="A20">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B20" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C20" t="s">
         <v>50</v>
@@ -2021,46 +2062,46 @@
         <v>91</v>
       </c>
       <c r="F20" t="s">
+        <v>93</v>
+      </c>
+      <c r="G20">
+        <v>2720</v>
+      </c>
+      <c r="H20" t="s">
         <v>96</v>
       </c>
-      <c r="G20">
-        <v>2741</v>
-      </c>
-      <c r="H20" t="s">
-        <v>99</v>
-      </c>
       <c r="I20" t="s">
+        <v>100</v>
+      </c>
+      <c r="J20" s="2">
+        <v>46220</v>
+      </c>
+      <c r="K20" s="2">
+        <v>46224</v>
+      </c>
+      <c r="L20">
+        <v>6</v>
+      </c>
+      <c r="M20" t="s">
         <v>102</v>
       </c>
-      <c r="J20" s="1">
-        <v>46224</v>
-      </c>
-      <c r="K20" s="1">
-        <v>46222</v>
-      </c>
-      <c r="L20">
-        <v>1</v>
-      </c>
-      <c r="M20" t="s">
-        <v>103</v>
-      </c>
-      <c r="N20" s="1">
-        <v>46229</v>
+      <c r="N20" s="2">
+        <v>46255</v>
       </c>
       <c r="Q20">
-        <v>-5</v>
+        <v>-30</v>
       </c>
       <c r="R20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S20" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T20" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="W20" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="AA20" t="b">
         <v>1</v>
@@ -2080,49 +2121,49 @@
         <v>72</v>
       </c>
       <c r="E21" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F21" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G21">
         <v>2720</v>
       </c>
       <c r="H21" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="I21" t="s">
-        <v>101</v>
-      </c>
-      <c r="J21" s="1">
+        <v>100</v>
+      </c>
+      <c r="J21" s="2">
         <v>46220</v>
       </c>
-      <c r="K21" s="1">
-        <v>46223</v>
+      <c r="K21" s="2">
+        <v>46225</v>
       </c>
       <c r="L21">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="M21" t="s">
-        <v>103</v>
-      </c>
-      <c r="N21" s="1">
-        <v>46254</v>
+        <v>102</v>
+      </c>
+      <c r="N21" s="2">
+        <v>46256</v>
       </c>
       <c r="Q21">
-        <v>-30</v>
+        <v>-31</v>
       </c>
       <c r="R21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S21" t="s">
         <v>104</v>
       </c>
       <c r="T21" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="W21" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="AA21" t="b">
         <v>1</v>
@@ -2142,113 +2183,51 @@
         <v>73</v>
       </c>
       <c r="E22" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F22" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G22">
-        <v>2720</v>
+        <v>2721</v>
       </c>
       <c r="H22" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I22" t="s">
         <v>101</v>
       </c>
-      <c r="J22" s="1">
-        <v>46220</v>
-      </c>
-      <c r="K22" s="1">
-        <v>46224</v>
+      <c r="J22" s="2">
+        <v>46225</v>
+      </c>
+      <c r="K22" s="2">
+        <v>46226</v>
       </c>
       <c r="L22">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M22" t="s">
-        <v>103</v>
-      </c>
-      <c r="N22" s="1">
-        <v>46255</v>
+        <v>102</v>
+      </c>
+      <c r="N22" s="2">
+        <v>46233</v>
       </c>
       <c r="Q22">
-        <v>-31</v>
+        <v>-8</v>
       </c>
       <c r="R22">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="S22" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="T22" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="W22" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="AA22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:27">
-      <c r="A23">
-        <v>329</v>
-      </c>
-      <c r="B23" t="s">
-        <v>28</v>
-      </c>
-      <c r="C23" t="s">
-        <v>53</v>
-      </c>
-      <c r="D23" t="s">
-        <v>74</v>
-      </c>
-      <c r="E23" t="s">
-        <v>93</v>
-      </c>
-      <c r="F23" t="s">
-        <v>94</v>
-      </c>
-      <c r="G23">
-        <v>2720</v>
-      </c>
-      <c r="H23" t="s">
-        <v>99</v>
-      </c>
-      <c r="I23" t="s">
-        <v>101</v>
-      </c>
-      <c r="J23" s="1">
-        <v>46220</v>
-      </c>
-      <c r="K23" s="1">
-        <v>46225</v>
-      </c>
-      <c r="L23">
-        <v>6</v>
-      </c>
-      <c r="M23" t="s">
-        <v>103</v>
-      </c>
-      <c r="N23" s="1">
-        <v>46256</v>
-      </c>
-      <c r="Q23">
-        <v>-32</v>
-      </c>
-      <c r="R23">
-        <v>-1</v>
-      </c>
-      <c r="S23" t="s">
-        <v>105</v>
-      </c>
-      <c r="T23" t="s">
-        <v>104</v>
-      </c>
-      <c r="W23" t="s">
-        <v>127</v>
-      </c>
-      <c r="AA23" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (22/07/2026 16:09)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -413,16 +413,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -438,7 +430,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -446,30 +438,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -769,85 +743,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -879,10 +853,10 @@
       <c r="I2" t="s">
         <v>99</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>46076</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46080</v>
       </c>
       <c r="L2">
@@ -891,7 +865,7 @@
       <c r="M2" t="s">
         <v>102</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="1">
         <v>46091</v>
       </c>
       <c r="Q2">
@@ -944,10 +918,10 @@
       <c r="I3" t="s">
         <v>100</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>46185</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46185</v>
       </c>
       <c r="L3">
@@ -956,10 +930,10 @@
       <c r="M3" t="s">
         <v>102</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="1">
         <v>46216</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46216</v>
       </c>
       <c r="Q3">
@@ -1015,10 +989,10 @@
       <c r="I4" t="s">
         <v>101</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>46209</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46210</v>
       </c>
       <c r="L4">
@@ -1027,10 +1001,10 @@
       <c r="M4" t="s">
         <v>102</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="1">
         <v>46217</v>
       </c>
-      <c r="O4" s="2">
+      <c r="O4" s="1">
         <v>46216</v>
       </c>
       <c r="Q4">
@@ -1083,10 +1057,10 @@
       <c r="I5" t="s">
         <v>100</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>46210</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46210</v>
       </c>
       <c r="L5">
@@ -1095,10 +1069,10 @@
       <c r="M5" t="s">
         <v>102</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="1">
         <v>46241</v>
       </c>
-      <c r="O5" s="2">
+      <c r="O5" s="1">
         <v>46238</v>
       </c>
       <c r="Q5">
@@ -1148,10 +1122,10 @@
       <c r="I6" t="s">
         <v>101</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>46210</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46211</v>
       </c>
       <c r="L6">
@@ -1160,10 +1134,10 @@
       <c r="M6" t="s">
         <v>102</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="1">
         <v>46218</v>
       </c>
-      <c r="O6" s="2">
+      <c r="O6" s="1">
         <v>46213</v>
       </c>
       <c r="Q6">
@@ -1219,10 +1193,10 @@
       <c r="I7" t="s">
         <v>99</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46211</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>46211</v>
       </c>
       <c r="L7">
@@ -1231,10 +1205,10 @@
       <c r="M7" t="s">
         <v>102</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="1">
         <v>46222</v>
       </c>
-      <c r="O7" s="2">
+      <c r="O7" s="1">
         <v>46237</v>
       </c>
       <c r="Q7">
@@ -1287,10 +1261,10 @@
       <c r="I8" t="s">
         <v>101</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46212</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>46212</v>
       </c>
       <c r="L8">
@@ -1299,10 +1273,10 @@
       <c r="M8" t="s">
         <v>102</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="1">
         <v>46219</v>
       </c>
-      <c r="O8" s="2">
+      <c r="O8" s="1">
         <v>46216</v>
       </c>
       <c r="Q8">
@@ -1355,10 +1329,10 @@
       <c r="I9" t="s">
         <v>101</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46211</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>46212</v>
       </c>
       <c r="L9">
@@ -1367,10 +1341,10 @@
       <c r="M9" t="s">
         <v>102</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="1">
         <v>46219</v>
       </c>
-      <c r="O9" s="2">
+      <c r="O9" s="1">
         <v>46237</v>
       </c>
       <c r="Q9">
@@ -1426,10 +1400,10 @@
       <c r="I10" t="s">
         <v>100</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>46212</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>46212</v>
       </c>
       <c r="L10">
@@ -1438,7 +1412,7 @@
       <c r="M10" t="s">
         <v>102</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="1">
         <v>46243</v>
       </c>
       <c r="Q10">
@@ -1488,10 +1462,10 @@
       <c r="I11" t="s">
         <v>100</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46216</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>46217</v>
       </c>
       <c r="L11">
@@ -1500,10 +1474,10 @@
       <c r="M11" t="s">
         <v>102</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11" s="1">
         <v>46248</v>
       </c>
-      <c r="O11" s="2">
+      <c r="O11" s="1">
         <v>46248</v>
       </c>
       <c r="Q11">
@@ -1553,10 +1527,10 @@
       <c r="I12" t="s">
         <v>99</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>46216</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>46217</v>
       </c>
       <c r="L12">
@@ -1565,7 +1539,7 @@
       <c r="M12" t="s">
         <v>102</v>
       </c>
-      <c r="N12" s="2">
+      <c r="N12" s="1">
         <v>46228</v>
       </c>
       <c r="Q12">
@@ -1618,10 +1592,10 @@
       <c r="I13" t="s">
         <v>100</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46219</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>46218</v>
       </c>
       <c r="L13">
@@ -1630,7 +1604,7 @@
       <c r="M13" t="s">
         <v>102</v>
       </c>
-      <c r="N13" s="2">
+      <c r="N13" s="1">
         <v>46249</v>
       </c>
       <c r="Q13">
@@ -1686,10 +1660,10 @@
       <c r="I14" t="s">
         <v>99</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46219</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>46219</v>
       </c>
       <c r="L14">
@@ -1698,7 +1672,7 @@
       <c r="M14" t="s">
         <v>102</v>
       </c>
-      <c r="N14" s="2">
+      <c r="N14" s="1">
         <v>46230</v>
       </c>
       <c r="Q14">
@@ -1751,10 +1725,10 @@
       <c r="I15" t="s">
         <v>100</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46219</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46220</v>
       </c>
       <c r="L15">
@@ -1763,7 +1737,7 @@
       <c r="M15" t="s">
         <v>102</v>
       </c>
-      <c r="N15" s="2">
+      <c r="N15" s="1">
         <v>46251</v>
       </c>
       <c r="Q15">
@@ -1813,10 +1787,10 @@
       <c r="I16" t="s">
         <v>99</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46219</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46221</v>
       </c>
       <c r="L16">
@@ -1825,7 +1799,7 @@
       <c r="M16" t="s">
         <v>102</v>
       </c>
-      <c r="N16" s="2">
+      <c r="N16" s="1">
         <v>46232</v>
       </c>
       <c r="Q16">
@@ -1878,10 +1852,10 @@
       <c r="I17" t="s">
         <v>101</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46220</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46221</v>
       </c>
       <c r="L17">
@@ -1890,7 +1864,7 @@
       <c r="M17" t="s">
         <v>102</v>
       </c>
-      <c r="N17" s="2">
+      <c r="N17" s="1">
         <v>46228</v>
       </c>
       <c r="Q17">
@@ -1943,10 +1917,10 @@
       <c r="I18" t="s">
         <v>101</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46224</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>46222</v>
       </c>
       <c r="L18">
@@ -1955,7 +1929,7 @@
       <c r="M18" t="s">
         <v>102</v>
       </c>
-      <c r="N18" s="2">
+      <c r="N18" s="1">
         <v>46229</v>
       </c>
       <c r="Q18">
@@ -2008,10 +1982,10 @@
       <c r="I19" t="s">
         <v>100</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>46220</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>46223</v>
       </c>
       <c r="L19">
@@ -2020,7 +1994,7 @@
       <c r="M19" t="s">
         <v>102</v>
       </c>
-      <c r="N19" s="2">
+      <c r="N19" s="1">
         <v>46254</v>
       </c>
       <c r="Q19">
@@ -2073,10 +2047,10 @@
       <c r="I20" t="s">
         <v>100</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>46220</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>46224</v>
       </c>
       <c r="L20">
@@ -2085,7 +2059,7 @@
       <c r="M20" t="s">
         <v>102</v>
       </c>
-      <c r="N20" s="2">
+      <c r="N20" s="1">
         <v>46255</v>
       </c>
       <c r="Q20">
@@ -2135,10 +2109,10 @@
       <c r="I21" t="s">
         <v>100</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46220</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>46225</v>
       </c>
       <c r="L21">
@@ -2147,7 +2121,7 @@
       <c r="M21" t="s">
         <v>102</v>
       </c>
-      <c r="N21" s="2">
+      <c r="N21" s="1">
         <v>46256</v>
       </c>
       <c r="Q21">
@@ -2197,10 +2171,10 @@
       <c r="I22" t="s">
         <v>101</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46225</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>46226</v>
       </c>
       <c r="L22">
@@ -2209,7 +2183,7 @@
       <c r="M22" t="s">
         <v>102</v>
       </c>
-      <c r="N22" s="2">
+      <c r="N22" s="1">
         <v>46233</v>
       </c>
       <c r="Q22">

</xml_diff>

<commit_message>
Atualização automática: emergencias (23/07/2026 06:39)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -869,10 +869,10 @@
         <v>46091</v>
       </c>
       <c r="Q2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="R2">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="S2" t="s">
         <v>103</v>
@@ -937,10 +937,10 @@
         <v>46216</v>
       </c>
       <c r="Q3">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R3">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="S3" t="s">
         <v>103</v>
@@ -1008,10 +1008,10 @@
         <v>46216</v>
       </c>
       <c r="Q4">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R4">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S4" t="s">
         <v>103</v>
@@ -1076,10 +1076,10 @@
         <v>46238</v>
       </c>
       <c r="Q5">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="R5">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S5" t="s">
         <v>103</v>
@@ -1141,10 +1141,10 @@
         <v>46213</v>
       </c>
       <c r="Q6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R6">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S6" t="s">
         <v>103</v>
@@ -1212,10 +1212,10 @@
         <v>46237</v>
       </c>
       <c r="Q7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R7">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S7" t="s">
         <v>103</v>
@@ -1280,10 +1280,10 @@
         <v>46216</v>
       </c>
       <c r="Q8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R8">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S8" t="s">
         <v>104</v>
@@ -1348,10 +1348,10 @@
         <v>46237</v>
       </c>
       <c r="Q9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R9">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S9" t="s">
         <v>103</v>
@@ -1416,10 +1416,10 @@
         <v>46243</v>
       </c>
       <c r="Q10">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="R10">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S10" t="s">
         <v>103</v>
@@ -1481,10 +1481,10 @@
         <v>46248</v>
       </c>
       <c r="Q11">
-        <v>-23</v>
+        <v>-22</v>
       </c>
       <c r="R11">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S11" t="s">
         <v>103</v>
@@ -1543,10 +1543,10 @@
         <v>46228</v>
       </c>
       <c r="Q12">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R12">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S12" t="s">
         <v>103</v>
@@ -1608,10 +1608,10 @@
         <v>46249</v>
       </c>
       <c r="Q13">
-        <v>-24</v>
+        <v>-23</v>
       </c>
       <c r="R13">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S13" t="s">
         <v>103</v>
@@ -1676,10 +1676,10 @@
         <v>46230</v>
       </c>
       <c r="Q14">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R14">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S14" t="s">
         <v>103</v>
@@ -1741,10 +1741,10 @@
         <v>46251</v>
       </c>
       <c r="Q15">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="R15">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S15" t="s">
         <v>104</v>
@@ -1803,10 +1803,10 @@
         <v>46232</v>
       </c>
       <c r="Q16">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R16">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S16" t="s">
         <v>103</v>
@@ -1868,10 +1868,10 @@
         <v>46228</v>
       </c>
       <c r="Q17">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R17">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S17" t="s">
         <v>103</v>
@@ -1933,10 +1933,10 @@
         <v>46229</v>
       </c>
       <c r="Q18">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R18">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S18" t="s">
         <v>103</v>
@@ -1998,10 +1998,10 @@
         <v>46254</v>
       </c>
       <c r="Q19">
-        <v>-29</v>
+        <v>-28</v>
       </c>
       <c r="R19">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S19" t="s">
         <v>103</v>
@@ -2063,10 +2063,10 @@
         <v>46255</v>
       </c>
       <c r="Q20">
-        <v>-30</v>
+        <v>-29</v>
       </c>
       <c r="R20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S20" t="s">
         <v>103</v>
@@ -2125,10 +2125,10 @@
         <v>46256</v>
       </c>
       <c r="Q21">
-        <v>-31</v>
+        <v>-30</v>
       </c>
       <c r="R21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S21" t="s">
         <v>104</v>
@@ -2187,10 +2187,10 @@
         <v>46233</v>
       </c>
       <c r="Q22">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="R22">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="S22" t="s">
         <v>103</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (23/07/2026 11:41)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="130">
   <si>
     <t>om_emg</t>
   </si>
@@ -142,9 +142,6 @@
     <t>313260018674</t>
   </si>
   <si>
-    <t>685260012368</t>
-  </si>
-  <si>
     <t>685260012387</t>
   </si>
   <si>
@@ -205,9 +202,6 @@
     <t>205842-1</t>
   </si>
   <si>
-    <t>C611008-0101</t>
-  </si>
-  <si>
     <t>066-3084-32</t>
   </si>
   <si>
@@ -265,9 +259,6 @@
     <t>CONNECTOR</t>
   </si>
   <si>
-    <t>ALTERNATOR CONTROL U</t>
-  </si>
-  <si>
     <t>IND RDR 2000 IN-182A</t>
   </si>
   <si>
@@ -310,9 +301,6 @@
     <t>Expedido total</t>
   </si>
   <si>
-    <t>Aguardando solução</t>
-  </si>
-  <si>
     <t>IPLR</t>
   </si>
   <si>
@@ -337,9 +325,15 @@
     <t>Volume retirado na loja GOLLOG - BSB por tanise Assis em 03/07/2026 - Godoy 08/07/2026. Recibo não se encontra na Pasta do DRIVE. Godoy 08/07/2026.</t>
   </si>
   <si>
+    <t>Vee One tem alguma atualização do DPE ?. Godoy 23/07/26</t>
+  </si>
+  <si>
     <t>AWB 12745918331 volume retirado na loja GOLLOG - BEL por bispo em 10/07/2026 - Godoy 13/07/2026. Recibo não se encontra na Pasta do DRIVE. Godoy 17/07/2026.</t>
   </si>
   <si>
+    <t>AWB 12748346281 -  volume retirado na loja GOLLOG - BEL por bispo em 23/07. Godoy 23/07/26.</t>
+  </si>
+  <si>
     <t>Cedeu o item para o C-98 2721. Ramon 09/07/26. AWB 12746175415 - 2 volumes retirados na loja GOLLOG - BEL por bispo em 13/07/26. Godoy 15/07/26. Vee One, não temos o recibo assinado. Godoy 16/07/26.</t>
   </si>
   <si>
@@ -352,6 +346,9 @@
     <t>Cedeu o item para o C-98 2737. Godoy 21/07/26.</t>
   </si>
   <si>
+    <t>AWB 12748301050 - volume retirado na loja GOLLOG - BSB por MARIO JORGE BARRIOLi em 21/07. Godoy 23/07/26</t>
+  </si>
+  <si>
     <t>Foi solicitado via email no dia 02-03-2 o atendimento do item com estoque FAB. Claudio -02-03-26 - Em resposta, a coordenadoria disse que o estque seria insuficiente. Foi verificado que na T.O da ANV o QPA para esse item são 2 EA, solicitei confirmação. - Cláudio -02-03-2026. Solicitado o cancelamento da emergência em função da quantidade cedida ao 2733 ter sido de 01ea. Considerando o QPA 02 ea. Encontra-se em tratativa junto a fiscalização e o gestor do contrato conforme mensagem de e-mail de 05/03. - SOLICITAÇÃO E-C98-26047.Colocado pedido AOG Textron WB0003068789 - previsão de entrega 60 dias em média. Os demais fornecedores informaram não ter em estoque ou não possuírem a certificação necessária da peça.</t>
   </si>
   <si>
@@ -367,7 +364,7 @@
     <t>MATERIAL EM TRANSITO - AWB 12745918331 dpe 11/07/2026 - atz rc 08/07/2026</t>
   </si>
   <si>
-    <t>Aguardando APROVAÇÃO PO 793/JPA/2026 em referencia ao orçamento 0274/26 - Prazo oficina 15 dias após aprovação. ATZ Marcio 9/7/26 14:50 ( MATERIAL EM SEPAÇÃO EM JPA - V1 ) 20/07 15:40.</t>
+    <t>Aguardando APROVAÇÃO PO 793/JPA/2026 em referencia ao orçamento 0274/26 - Prazo oficina 15 dias após aprovação. ATZ Marcio 9/7/26 14:50 ( MATERIAL EM SEPAÇÃO EM JPA - V1 ) 20/07 15:40. - AWB 12748346281 DPE 24/07/2026 - ATZ RC 22/07/2026</t>
   </si>
   <si>
     <t>Atendido em 09/07/26 AWB 12746175415 - CLA (09/07/26)</t>
@@ -382,9 +379,6 @@
     <t>Colocado pedido Textron IJ17575583 - entregue em Miami 15/07. Carga rercepcionada GIG 19/07 - Aguardando liberação do SEFAZ. ATZ 21/07</t>
   </si>
   <si>
-    <t>Checando se consegue priorizar 20/7 com a oficina em BH se consegue entregar mais 1 unidade (William) , o item que esta na Av aeronautica tem a probabilidade de estar SCRAP (nao pegar reparo e voltar no estado msg de 20/7 do Sr. Ricardo da AV.) - Atz Marcio 20/7 11:13hs - confirmado entrega 01 ea hj(21/07/26) pela William - REZ</t>
-  </si>
-  <si>
     <t>Item em bancada porem em pessimo estado, foi solicitado recolhimento de mais unidades para envio a oficina para tentativa de reparo ATZ Marcio 17/7/26. Solicitado abertura de O.S. para 3EA do item no dia 16-07-26 via Email para a Coordenadoria - CLA-21-07-26</t>
   </si>
   <si>
@@ -394,13 +388,19 @@
     <t>Validando atendimento via estoque FAB. ATZ 20/07</t>
   </si>
   <si>
-    <t>Enviado 1 unidade (CORE) para reparo na oficina no RJ em 17/7, aguardando orçamento com prazo de entrega, ATZ Marcio 17/7</t>
-  </si>
-  <si>
-    <t>TEMOS EM ESTOQUE NA BASE PAMALS, SERÁ ENVIADO. CLA-21-07</t>
+    <t>Consta 1 each em condição de uso em MANAUS, Enviado 1 unidade (CORE) para reparo na oficina no RJ em 17/7, orçamento aprovado em 21/7 com DPE de 5 dias para entrega na V1 JPA, ATZ Marcio 21/7</t>
+  </si>
+  <si>
+    <t>material enviado com STK FAB - AWB 12748581702 - DPE 25/07/2026 - atz rc 22/07/2026- Enviado para o Operador dia 21/07/26 - AWB 127-4857 9742- REZ -22/07/26</t>
+  </si>
+  <si>
+    <t>Enviado para o Operador dia 21/07/26 - AWB 127-4858 1702 - REZ -22/07/26</t>
   </si>
   <si>
     <t>PEDIDO NO EPM E-C98-26059 - CLA-21-07</t>
+  </si>
+  <si>
+    <t>FOI TRANSFERIDO DA BAMN PARA BABR VIA GMM202667292001554 AWB 127-4830 1050 ENVIADO DIA 20-07-26 - CLA-21-07</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -413,8 +413,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -430,7 +438,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -438,12 +446,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -739,89 +765,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA22"/>
+  <dimension ref="A1:AA21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -836,37 +862,40 @@
         <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F2" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G2">
         <v>2730</v>
       </c>
       <c r="H2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="I2" t="s">
-        <v>99</v>
-      </c>
-      <c r="J2" s="1">
+        <v>95</v>
+      </c>
+      <c r="J2" s="2">
         <v>46076</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46080</v>
       </c>
       <c r="L2">
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>102</v>
-      </c>
-      <c r="N2" s="1">
+        <v>98</v>
+      </c>
+      <c r="N2" s="2">
         <v>46091</v>
+      </c>
+      <c r="O2" s="2">
+        <v>46287</v>
       </c>
       <c r="Q2">
         <v>135</v>
@@ -875,13 +904,13 @@
         <v>146</v>
       </c>
       <c r="S2" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="U2" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="V2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="W2" t="s">
         <v>129</v>
@@ -901,39 +930,39 @@
         <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G3">
         <v>2721</v>
       </c>
       <c r="H3" t="s">
+        <v>93</v>
+      </c>
+      <c r="I3" t="s">
         <v>96</v>
       </c>
-      <c r="I3" t="s">
-        <v>100</v>
-      </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>46185</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46185</v>
       </c>
       <c r="L3">
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>102</v>
-      </c>
-      <c r="N3" s="1">
+        <v>98</v>
+      </c>
+      <c r="N3" s="2">
         <v>46216</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46216</v>
       </c>
       <c r="Q3">
@@ -943,16 +972,16 @@
         <v>41</v>
       </c>
       <c r="S3" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="T3" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="U3" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="V3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="W3" t="s">
         <v>129</v>
@@ -972,39 +1001,39 @@
         <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F4" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G4">
         <v>2721</v>
       </c>
       <c r="H4" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="I4" t="s">
-        <v>101</v>
-      </c>
-      <c r="J4" s="1">
+        <v>97</v>
+      </c>
+      <c r="J4" s="2">
         <v>46209</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46210</v>
       </c>
       <c r="L4">
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>102</v>
-      </c>
-      <c r="N4" s="1">
+        <v>98</v>
+      </c>
+      <c r="N4" s="2">
         <v>46217</v>
       </c>
-      <c r="O4" s="1">
+      <c r="O4" s="2">
         <v>46216</v>
       </c>
       <c r="Q4">
@@ -1014,13 +1043,16 @@
         <v>16</v>
       </c>
       <c r="S4" t="s">
+        <v>99</v>
+      </c>
+      <c r="T4" t="s">
+        <v>99</v>
+      </c>
+      <c r="U4" t="s">
         <v>103</v>
       </c>
-      <c r="T4" t="s">
-        <v>103</v>
-      </c>
       <c r="V4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="W4" t="s">
         <v>129</v>
@@ -1040,39 +1072,39 @@
         <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F5" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="G5">
         <v>2719</v>
       </c>
       <c r="H5" t="s">
+        <v>93</v>
+      </c>
+      <c r="I5" t="s">
         <v>96</v>
       </c>
-      <c r="I5" t="s">
-        <v>100</v>
-      </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>46210</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46210</v>
       </c>
       <c r="L5">
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>102</v>
-      </c>
-      <c r="N5" s="1">
+        <v>98</v>
+      </c>
+      <c r="N5" s="2">
         <v>46241</v>
       </c>
-      <c r="O5" s="1">
+      <c r="O5" s="2">
         <v>46238</v>
       </c>
       <c r="Q5">
@@ -1082,10 +1114,10 @@
         <v>16</v>
       </c>
       <c r="S5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="V5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="W5" t="s">
         <v>129</v>
@@ -1105,39 +1137,39 @@
         <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F6" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G6">
         <v>2723</v>
       </c>
       <c r="H6" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="I6" t="s">
-        <v>101</v>
-      </c>
-      <c r="J6" s="1">
+        <v>97</v>
+      </c>
+      <c r="J6" s="2">
         <v>46210</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46211</v>
       </c>
       <c r="L6">
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>102</v>
-      </c>
-      <c r="N6" s="1">
+        <v>98</v>
+      </c>
+      <c r="N6" s="2">
         <v>46218</v>
       </c>
-      <c r="O6" s="1">
+      <c r="O6" s="2">
         <v>46213</v>
       </c>
       <c r="Q6">
@@ -1147,16 +1179,16 @@
         <v>15</v>
       </c>
       <c r="S6" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="T6" t="s">
+        <v>100</v>
+      </c>
+      <c r="U6" t="s">
         <v>104</v>
       </c>
-      <c r="U6" t="s">
-        <v>107</v>
-      </c>
       <c r="V6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="W6" t="s">
         <v>129</v>
@@ -1176,39 +1208,39 @@
         <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F7" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G7">
         <v>2733</v>
       </c>
       <c r="H7" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="I7" t="s">
-        <v>99</v>
-      </c>
-      <c r="J7" s="1">
+        <v>95</v>
+      </c>
+      <c r="J7" s="2">
         <v>46211</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46211</v>
       </c>
       <c r="L7">
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>102</v>
-      </c>
-      <c r="N7" s="1">
+        <v>98</v>
+      </c>
+      <c r="N7" s="2">
         <v>46222</v>
       </c>
-      <c r="O7" s="1">
+      <c r="O7" s="2">
         <v>46237</v>
       </c>
       <c r="Q7">
@@ -1218,13 +1250,16 @@
         <v>15</v>
       </c>
       <c r="S7" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="T7" t="s">
-        <v>104</v>
+        <v>100</v>
+      </c>
+      <c r="U7" t="s">
+        <v>105</v>
       </c>
       <c r="V7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="W7" t="s">
         <v>129</v>
@@ -1244,39 +1279,39 @@
         <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F8" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G8">
         <v>2726</v>
       </c>
       <c r="H8" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="I8" t="s">
-        <v>101</v>
-      </c>
-      <c r="J8" s="1">
+        <v>97</v>
+      </c>
+      <c r="J8" s="2">
         <v>46212</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46212</v>
       </c>
       <c r="L8">
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>102</v>
-      </c>
-      <c r="N8" s="1">
+        <v>98</v>
+      </c>
+      <c r="N8" s="2">
         <v>46219</v>
       </c>
-      <c r="O8" s="1">
+      <c r="O8" s="2">
         <v>46216</v>
       </c>
       <c r="Q8">
@@ -1286,13 +1321,13 @@
         <v>14</v>
       </c>
       <c r="S8" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="U8" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="V8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="W8" t="s">
         <v>129</v>
@@ -1312,39 +1347,39 @@
         <v>39</v>
       </c>
       <c r="D9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E9" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F9" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G9">
         <v>2723</v>
       </c>
       <c r="H9" t="s">
+        <v>94</v>
+      </c>
+      <c r="I9" t="s">
         <v>97</v>
       </c>
-      <c r="I9" t="s">
-        <v>101</v>
-      </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46211</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46212</v>
       </c>
       <c r="L9">
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>102</v>
-      </c>
-      <c r="N9" s="1">
+        <v>98</v>
+      </c>
+      <c r="N9" s="2">
         <v>46219</v>
       </c>
-      <c r="O9" s="1">
+      <c r="O9" s="2">
         <v>46237</v>
       </c>
       <c r="Q9">
@@ -1354,16 +1389,16 @@
         <v>14</v>
       </c>
       <c r="S9" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="T9" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="U9" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="V9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="W9" t="s">
         <v>129</v>
@@ -1383,36 +1418,36 @@
         <v>40</v>
       </c>
       <c r="D10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E10" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F10" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G10">
         <v>2702</v>
       </c>
       <c r="H10" t="s">
+        <v>93</v>
+      </c>
+      <c r="I10" t="s">
         <v>96</v>
       </c>
-      <c r="I10" t="s">
-        <v>100</v>
-      </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46212</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>46212</v>
       </c>
       <c r="L10">
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>102</v>
-      </c>
-      <c r="N10" s="1">
+        <v>98</v>
+      </c>
+      <c r="N10" s="2">
         <v>46243</v>
       </c>
       <c r="Q10">
@@ -1422,10 +1457,10 @@
         <v>14</v>
       </c>
       <c r="S10" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="V10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="W10" t="s">
         <v>129</v>
@@ -1445,39 +1480,39 @@
         <v>41</v>
       </c>
       <c r="D11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F11" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G11">
         <v>2736</v>
       </c>
       <c r="H11" t="s">
+        <v>93</v>
+      </c>
+      <c r="I11" t="s">
         <v>96</v>
       </c>
-      <c r="I11" t="s">
-        <v>100</v>
-      </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46216</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>46217</v>
       </c>
       <c r="L11">
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>102</v>
-      </c>
-      <c r="N11" s="1">
+        <v>98</v>
+      </c>
+      <c r="N11" s="2">
         <v>46248</v>
       </c>
-      <c r="O11" s="1">
+      <c r="O11" s="2">
         <v>46248</v>
       </c>
       <c r="Q11">
@@ -1487,10 +1522,10 @@
         <v>9</v>
       </c>
       <c r="S11" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="V11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="W11" t="s">
         <v>129</v>
@@ -1510,52 +1545,55 @@
         <v>42</v>
       </c>
       <c r="D12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E12" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F12" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="G12">
-        <v>2729</v>
+        <v>2722</v>
       </c>
       <c r="H12" t="s">
+        <v>93</v>
+      </c>
+      <c r="I12" t="s">
         <v>96</v>
       </c>
-      <c r="I12" t="s">
-        <v>99</v>
-      </c>
-      <c r="J12" s="1">
-        <v>46216</v>
-      </c>
-      <c r="K12" s="1">
-        <v>46217</v>
+      <c r="J12" s="2">
+        <v>46219</v>
+      </c>
+      <c r="K12" s="2">
+        <v>46218</v>
       </c>
       <c r="L12">
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>102</v>
-      </c>
-      <c r="N12" s="1">
-        <v>46228</v>
+        <v>98</v>
+      </c>
+      <c r="N12" s="2">
+        <v>46249</v>
       </c>
       <c r="Q12">
-        <v>-2</v>
+        <v>-23</v>
       </c>
       <c r="R12">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S12" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="T12" t="s">
-        <v>104</v>
+        <v>100</v>
+      </c>
+      <c r="U12" t="s">
+        <v>108</v>
       </c>
       <c r="V12" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="W12" t="s">
         <v>129</v>
@@ -1575,55 +1613,52 @@
         <v>43</v>
       </c>
       <c r="D13" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E13" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F13" t="s">
+        <v>91</v>
+      </c>
+      <c r="G13">
+        <v>2729</v>
+      </c>
+      <c r="H13" t="s">
+        <v>93</v>
+      </c>
+      <c r="I13" t="s">
         <v>95</v>
       </c>
-      <c r="G13">
-        <v>2722</v>
-      </c>
-      <c r="H13" t="s">
-        <v>96</v>
-      </c>
-      <c r="I13" t="s">
+      <c r="J13" s="2">
+        <v>46219</v>
+      </c>
+      <c r="K13" s="2">
+        <v>46219</v>
+      </c>
+      <c r="L13">
+        <v>1</v>
+      </c>
+      <c r="M13" t="s">
+        <v>98</v>
+      </c>
+      <c r="N13" s="2">
+        <v>46230</v>
+      </c>
+      <c r="Q13">
+        <v>-4</v>
+      </c>
+      <c r="R13">
+        <v>7</v>
+      </c>
+      <c r="S13" t="s">
+        <v>99</v>
+      </c>
+      <c r="T13" t="s">
         <v>100</v>
       </c>
-      <c r="J13" s="1">
-        <v>46219</v>
-      </c>
-      <c r="K13" s="1">
-        <v>46218</v>
-      </c>
-      <c r="L13">
-        <v>1</v>
-      </c>
-      <c r="M13" t="s">
-        <v>102</v>
-      </c>
-      <c r="N13" s="1">
-        <v>46249</v>
-      </c>
-      <c r="Q13">
-        <v>-23</v>
-      </c>
-      <c r="R13">
-        <v>8</v>
-      </c>
-      <c r="S13" t="s">
-        <v>103</v>
-      </c>
-      <c r="T13" t="s">
-        <v>104</v>
-      </c>
-      <c r="U13" t="s">
-        <v>110</v>
-      </c>
       <c r="V13" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="W13" t="s">
         <v>129</v>
@@ -1643,52 +1678,49 @@
         <v>44</v>
       </c>
       <c r="D14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E14" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F14" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="G14">
-        <v>2729</v>
+        <v>2703</v>
       </c>
       <c r="H14" t="s">
+        <v>93</v>
+      </c>
+      <c r="I14" t="s">
         <v>96</v>
       </c>
-      <c r="I14" t="s">
-        <v>99</v>
-      </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46219</v>
       </c>
-      <c r="K14" s="1">
-        <v>46219</v>
+      <c r="K14" s="2">
+        <v>46220</v>
       </c>
       <c r="L14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M14" t="s">
-        <v>102</v>
-      </c>
-      <c r="N14" s="1">
-        <v>46230</v>
+        <v>98</v>
+      </c>
+      <c r="N14" s="2">
+        <v>46251</v>
       </c>
       <c r="Q14">
-        <v>-4</v>
+        <v>-25</v>
       </c>
       <c r="R14">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S14" t="s">
-        <v>103</v>
-      </c>
-      <c r="T14" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="V14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="W14" t="s">
         <v>129</v>
@@ -1708,49 +1740,52 @@
         <v>45</v>
       </c>
       <c r="D15" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E15" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F15" t="s">
+        <v>92</v>
+      </c>
+      <c r="G15">
+        <v>2729</v>
+      </c>
+      <c r="H15" t="s">
         <v>93</v>
       </c>
-      <c r="G15">
-        <v>2703</v>
-      </c>
-      <c r="H15" t="s">
-        <v>96</v>
-      </c>
       <c r="I15" t="s">
+        <v>95</v>
+      </c>
+      <c r="J15" s="2">
+        <v>46219</v>
+      </c>
+      <c r="K15" s="2">
+        <v>46221</v>
+      </c>
+      <c r="L15">
+        <v>1</v>
+      </c>
+      <c r="M15" t="s">
+        <v>98</v>
+      </c>
+      <c r="N15" s="2">
+        <v>46232</v>
+      </c>
+      <c r="Q15">
+        <v>-6</v>
+      </c>
+      <c r="R15">
+        <v>5</v>
+      </c>
+      <c r="S15" t="s">
+        <v>99</v>
+      </c>
+      <c r="T15" t="s">
         <v>100</v>
       </c>
-      <c r="J15" s="1">
-        <v>46219</v>
-      </c>
-      <c r="K15" s="1">
-        <v>46220</v>
-      </c>
-      <c r="L15">
-        <v>2</v>
-      </c>
-      <c r="M15" t="s">
-        <v>102</v>
-      </c>
-      <c r="N15" s="1">
-        <v>46251</v>
-      </c>
-      <c r="Q15">
-        <v>-25</v>
-      </c>
-      <c r="R15">
-        <v>6</v>
-      </c>
-      <c r="S15" t="s">
-        <v>104</v>
-      </c>
       <c r="V15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="W15" t="s">
         <v>129</v>
@@ -1761,46 +1796,49 @@
     </row>
     <row r="16" spans="1:27">
       <c r="A16">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B16" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C16" t="s">
         <v>46</v>
       </c>
       <c r="D16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E16" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F16" t="s">
+        <v>92</v>
+      </c>
+      <c r="G16">
+        <v>2730</v>
+      </c>
+      <c r="H16" t="s">
+        <v>94</v>
+      </c>
+      <c r="I16" t="s">
         <v>95</v>
       </c>
-      <c r="G16">
-        <v>2729</v>
-      </c>
-      <c r="H16" t="s">
-        <v>96</v>
-      </c>
-      <c r="I16" t="s">
-        <v>99</v>
-      </c>
-      <c r="J16" s="1">
-        <v>46219</v>
-      </c>
-      <c r="K16" s="1">
+      <c r="J16" s="2">
+        <v>46220</v>
+      </c>
+      <c r="K16" s="2">
         <v>46221</v>
       </c>
       <c r="L16">
         <v>1</v>
       </c>
       <c r="M16" t="s">
-        <v>102</v>
-      </c>
-      <c r="N16" s="1">
+        <v>98</v>
+      </c>
+      <c r="N16" s="2">
         <v>46232</v>
+      </c>
+      <c r="O16" s="2">
+        <v>46228</v>
       </c>
       <c r="Q16">
         <v>-6</v>
@@ -1809,13 +1847,16 @@
         <v>5</v>
       </c>
       <c r="S16" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="T16" t="s">
-        <v>104</v>
+        <v>100</v>
+      </c>
+      <c r="U16" t="s">
+        <v>109</v>
       </c>
       <c r="V16" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="W16" t="s">
         <v>129</v>
@@ -1835,52 +1876,52 @@
         <v>47</v>
       </c>
       <c r="D17" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E17" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F17" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G17">
-        <v>2730</v>
+        <v>2741</v>
       </c>
       <c r="H17" t="s">
+        <v>93</v>
+      </c>
+      <c r="I17" t="s">
         <v>97</v>
       </c>
-      <c r="I17" t="s">
-        <v>101</v>
-      </c>
-      <c r="J17" s="1">
-        <v>46220</v>
-      </c>
-      <c r="K17" s="1">
-        <v>46221</v>
+      <c r="J17" s="2">
+        <v>46224</v>
+      </c>
+      <c r="K17" s="2">
+        <v>46222</v>
       </c>
       <c r="L17">
         <v>1</v>
       </c>
       <c r="M17" t="s">
-        <v>102</v>
-      </c>
-      <c r="N17" s="1">
-        <v>46228</v>
+        <v>98</v>
+      </c>
+      <c r="N17" s="2">
+        <v>46229</v>
       </c>
       <c r="Q17">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="R17">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S17" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="T17" t="s">
-        <v>104</v>
-      </c>
-      <c r="U17" t="s">
-        <v>111</v>
+        <v>100</v>
+      </c>
+      <c r="V17" t="s">
+        <v>126</v>
       </c>
       <c r="W17" t="s">
         <v>129</v>
@@ -1891,58 +1932,58 @@
     </row>
     <row r="18" spans="1:27">
       <c r="A18">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B18" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C18" t="s">
         <v>48</v>
       </c>
       <c r="D18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E18" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F18" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="G18">
-        <v>2741</v>
+        <v>2720</v>
       </c>
       <c r="H18" t="s">
+        <v>93</v>
+      </c>
+      <c r="I18" t="s">
         <v>96</v>
       </c>
-      <c r="I18" t="s">
-        <v>101</v>
-      </c>
-      <c r="J18" s="1">
-        <v>46224</v>
-      </c>
-      <c r="K18" s="1">
-        <v>46222</v>
+      <c r="J18" s="2">
+        <v>46220</v>
+      </c>
+      <c r="K18" s="2">
+        <v>46223</v>
       </c>
       <c r="L18">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="M18" t="s">
-        <v>102</v>
-      </c>
-      <c r="N18" s="1">
-        <v>46229</v>
+        <v>98</v>
+      </c>
+      <c r="N18" s="2">
+        <v>46254</v>
       </c>
       <c r="Q18">
-        <v>-3</v>
+        <v>-28</v>
       </c>
       <c r="R18">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S18" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="T18" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="V18" t="s">
         <v>127</v>
@@ -1965,49 +2006,52 @@
         <v>49</v>
       </c>
       <c r="D19" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E19" t="s">
+        <v>88</v>
+      </c>
+      <c r="F19" t="s">
         <v>90</v>
-      </c>
-      <c r="F19" t="s">
-        <v>93</v>
       </c>
       <c r="G19">
         <v>2720</v>
       </c>
       <c r="H19" t="s">
+        <v>93</v>
+      </c>
+      <c r="I19" t="s">
         <v>96</v>
       </c>
-      <c r="I19" t="s">
-        <v>100</v>
-      </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>46220</v>
       </c>
-      <c r="K19" s="1">
-        <v>46223</v>
+      <c r="K19" s="2">
+        <v>46224</v>
       </c>
       <c r="L19">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="M19" t="s">
-        <v>102</v>
-      </c>
-      <c r="N19" s="1">
-        <v>46254</v>
+        <v>98</v>
+      </c>
+      <c r="N19" s="2">
+        <v>46255</v>
       </c>
       <c r="Q19">
-        <v>-28</v>
+        <v>-29</v>
       </c>
       <c r="R19">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S19" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="T19" t="s">
-        <v>103</v>
+        <v>99</v>
+      </c>
+      <c r="U19" t="s">
+        <v>110</v>
       </c>
       <c r="V19" t="s">
         <v>128</v>
@@ -2030,49 +2074,55 @@
         <v>50</v>
       </c>
       <c r="D20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E20" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="F20" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G20">
         <v>2720</v>
       </c>
       <c r="H20" t="s">
+        <v>93</v>
+      </c>
+      <c r="I20" t="s">
         <v>96</v>
       </c>
-      <c r="I20" t="s">
-        <v>100</v>
-      </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>46220</v>
       </c>
-      <c r="K20" s="1">
-        <v>46224</v>
+      <c r="K20" s="2">
+        <v>46225</v>
       </c>
       <c r="L20">
         <v>6</v>
       </c>
       <c r="M20" t="s">
-        <v>102</v>
-      </c>
-      <c r="N20" s="1">
-        <v>46255</v>
+        <v>98</v>
+      </c>
+      <c r="N20" s="2">
+        <v>46256</v>
       </c>
       <c r="Q20">
-        <v>-29</v>
+        <v>-30</v>
       </c>
       <c r="R20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S20" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="T20" t="s">
-        <v>103</v>
+        <v>99</v>
+      </c>
+      <c r="U20" t="s">
+        <v>110</v>
+      </c>
+      <c r="V20" t="s">
+        <v>128</v>
       </c>
       <c r="W20" t="s">
         <v>129</v>
@@ -2092,116 +2142,54 @@
         <v>51</v>
       </c>
       <c r="D21" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E21" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F21" t="s">
+        <v>92</v>
+      </c>
+      <c r="G21">
+        <v>2721</v>
+      </c>
+      <c r="H21" t="s">
         <v>93</v>
       </c>
-      <c r="G21">
-        <v>2720</v>
-      </c>
-      <c r="H21" t="s">
-        <v>96</v>
-      </c>
       <c r="I21" t="s">
-        <v>100</v>
-      </c>
-      <c r="J21" s="1">
-        <v>46220</v>
-      </c>
-      <c r="K21" s="1">
+        <v>97</v>
+      </c>
+      <c r="J21" s="2">
         <v>46225</v>
       </c>
+      <c r="K21" s="2">
+        <v>46226</v>
+      </c>
       <c r="L21">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M21" t="s">
-        <v>102</v>
-      </c>
-      <c r="N21" s="1">
-        <v>46256</v>
+        <v>98</v>
+      </c>
+      <c r="N21" s="2">
+        <v>46233</v>
       </c>
       <c r="Q21">
-        <v>-30</v>
+        <v>-7</v>
       </c>
       <c r="R21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S21" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="T21" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="W21" t="s">
         <v>129</v>
       </c>
       <c r="AA21" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:27">
-      <c r="A22">
-        <v>329</v>
-      </c>
-      <c r="B22" t="s">
-        <v>28</v>
-      </c>
-      <c r="C22" t="s">
-        <v>52</v>
-      </c>
-      <c r="D22" t="s">
-        <v>73</v>
-      </c>
-      <c r="E22" t="s">
-        <v>92</v>
-      </c>
-      <c r="F22" t="s">
-        <v>95</v>
-      </c>
-      <c r="G22">
-        <v>2721</v>
-      </c>
-      <c r="H22" t="s">
-        <v>98</v>
-      </c>
-      <c r="I22" t="s">
-        <v>101</v>
-      </c>
-      <c r="J22" s="1">
-        <v>46225</v>
-      </c>
-      <c r="K22" s="1">
-        <v>46226</v>
-      </c>
-      <c r="L22">
-        <v>1</v>
-      </c>
-      <c r="M22" t="s">
-        <v>102</v>
-      </c>
-      <c r="N22" s="1">
-        <v>46233</v>
-      </c>
-      <c r="Q22">
-        <v>-7</v>
-      </c>
-      <c r="R22">
-        <v>0</v>
-      </c>
-      <c r="S22" t="s">
-        <v>103</v>
-      </c>
-      <c r="T22" t="s">
-        <v>103</v>
-      </c>
-      <c r="W22" t="s">
-        <v>129</v>
-      </c>
-      <c r="AA22" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (23/07/2026 16:17)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="125">
   <si>
     <t>om_emg</t>
   </si>
@@ -127,9 +127,6 @@
     <t>419260000556</t>
   </si>
   <si>
-    <t>396260016563</t>
-  </si>
-  <si>
     <t>396260016566</t>
   </si>
   <si>
@@ -187,9 +184,6 @@
     <t>066-3046-07</t>
   </si>
   <si>
-    <t>3244809-4</t>
-  </si>
-  <si>
     <t>060-0015-00</t>
   </si>
   <si>
@@ -247,9 +241,6 @@
     <t>CONTROL,INDICATOR</t>
   </si>
   <si>
-    <t>FUEL CONTROL,MAIN,TU</t>
-  </si>
-  <si>
     <t>CONTROL,DIRECTIONAL,</t>
   </si>
   <si>
@@ -331,9 +322,6 @@
     <t>AWB 12745918331 volume retirado na loja GOLLOG - BEL por bispo em 10/07/2026 - Godoy 13/07/2026. Recibo não se encontra na Pasta do DRIVE. Godoy 17/07/2026.</t>
   </si>
   <si>
-    <t>AWB 12748346281 -  volume retirado na loja GOLLOG - BEL por bispo em 23/07. Godoy 23/07/26.</t>
-  </si>
-  <si>
     <t>Cedeu o item para o C-98 2721. Ramon 09/07/26. AWB 12746175415 - 2 volumes retirados na loja GOLLOG - BEL por bispo em 13/07/26. Godoy 15/07/26. Vee One, não temos o recibo assinado. Godoy 16/07/26.</t>
   </si>
   <si>
@@ -362,9 +350,6 @@
   </si>
   <si>
     <t>MATERIAL EM TRANSITO - AWB 12745918331 dpe 11/07/2026 - atz rc 08/07/2026</t>
-  </si>
-  <si>
-    <t>Aguardando APROVAÇÃO PO 793/JPA/2026 em referencia ao orçamento 0274/26 - Prazo oficina 15 dias após aprovação. ATZ Marcio 9/7/26 14:50 ( MATERIAL EM SEPAÇÃO EM JPA - V1 ) 20/07 15:40. - AWB 12748346281 DPE 24/07/2026 - ATZ RC 22/07/2026</t>
   </si>
   <si>
     <t>Atendido em 09/07/26 AWB 12746175415 - CLA (09/07/26)</t>
@@ -413,16 +398,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -438,7 +415,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -446,30 +423,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -765,89 +724,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA21"/>
+  <dimension ref="A1:AA20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -862,39 +821,39 @@
         <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G2">
         <v>2730</v>
       </c>
       <c r="H2" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I2" t="s">
-        <v>95</v>
-      </c>
-      <c r="J2" s="2">
+        <v>92</v>
+      </c>
+      <c r="J2" s="1">
         <v>46076</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46080</v>
       </c>
       <c r="L2">
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>98</v>
-      </c>
-      <c r="N2" s="2">
+        <v>95</v>
+      </c>
+      <c r="N2" s="1">
         <v>46091</v>
       </c>
-      <c r="O2" s="2">
+      <c r="O2" s="1">
         <v>46287</v>
       </c>
       <c r="Q2">
@@ -904,16 +863,16 @@
         <v>146</v>
       </c>
       <c r="S2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="U2" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="V2" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="W2" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -930,39 +889,39 @@
         <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G3">
         <v>2721</v>
       </c>
       <c r="H3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I3" t="s">
         <v>93</v>
       </c>
-      <c r="I3" t="s">
-        <v>96</v>
-      </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>46185</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46185</v>
       </c>
       <c r="L3">
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>98</v>
-      </c>
-      <c r="N3" s="2">
+        <v>95</v>
+      </c>
+      <c r="N3" s="1">
         <v>46216</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46216</v>
       </c>
       <c r="Q3">
@@ -972,19 +931,19 @@
         <v>41</v>
       </c>
       <c r="S3" t="s">
+        <v>96</v>
+      </c>
+      <c r="T3" t="s">
+        <v>96</v>
+      </c>
+      <c r="U3" t="s">
         <v>99</v>
       </c>
-      <c r="T3" t="s">
-        <v>99</v>
-      </c>
-      <c r="U3" t="s">
-        <v>102</v>
-      </c>
       <c r="V3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="W3" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -1001,39 +960,39 @@
         <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E4" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F4" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G4">
         <v>2721</v>
       </c>
       <c r="H4" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I4" t="s">
-        <v>97</v>
-      </c>
-      <c r="J4" s="2">
+        <v>94</v>
+      </c>
+      <c r="J4" s="1">
         <v>46209</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46210</v>
       </c>
       <c r="L4">
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>98</v>
-      </c>
-      <c r="N4" s="2">
+        <v>95</v>
+      </c>
+      <c r="N4" s="1">
         <v>46217</v>
       </c>
-      <c r="O4" s="2">
+      <c r="O4" s="1">
         <v>46216</v>
       </c>
       <c r="Q4">
@@ -1043,19 +1002,19 @@
         <v>16</v>
       </c>
       <c r="S4" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="T4" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="U4" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="V4" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="W4" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -1072,39 +1031,39 @@
         <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F5" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="G5">
         <v>2719</v>
       </c>
       <c r="H5" t="s">
+        <v>90</v>
+      </c>
+      <c r="I5" t="s">
         <v>93</v>
       </c>
-      <c r="I5" t="s">
-        <v>96</v>
-      </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>46210</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46210</v>
       </c>
       <c r="L5">
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>98</v>
-      </c>
-      <c r="N5" s="2">
+        <v>95</v>
+      </c>
+      <c r="N5" s="1">
         <v>46241</v>
       </c>
-      <c r="O5" s="2">
+      <c r="O5" s="1">
         <v>46238</v>
       </c>
       <c r="Q5">
@@ -1114,13 +1073,13 @@
         <v>16</v>
       </c>
       <c r="S5" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="V5" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="W5" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1137,39 +1096,39 @@
         <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E6" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F6" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="G6">
         <v>2723</v>
       </c>
       <c r="H6" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I6" t="s">
-        <v>97</v>
-      </c>
-      <c r="J6" s="2">
+        <v>94</v>
+      </c>
+      <c r="J6" s="1">
         <v>46210</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46211</v>
       </c>
       <c r="L6">
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>98</v>
-      </c>
-      <c r="N6" s="2">
+        <v>95</v>
+      </c>
+      <c r="N6" s="1">
         <v>46218</v>
       </c>
-      <c r="O6" s="2">
+      <c r="O6" s="1">
         <v>46213</v>
       </c>
       <c r="Q6">
@@ -1179,19 +1138,19 @@
         <v>15</v>
       </c>
       <c r="S6" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="T6" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="U6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="V6" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="W6" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1208,61 +1167,58 @@
         <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F7" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="G7">
-        <v>2733</v>
+        <v>2726</v>
       </c>
       <c r="H7" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I7" t="s">
+        <v>94</v>
+      </c>
+      <c r="J7" s="1">
+        <v>46212</v>
+      </c>
+      <c r="K7" s="1">
+        <v>46212</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7" t="s">
         <v>95</v>
       </c>
-      <c r="J7" s="2">
-        <v>46211</v>
-      </c>
-      <c r="K7" s="2">
-        <v>46211</v>
-      </c>
-      <c r="L7">
-        <v>1</v>
-      </c>
-      <c r="M7" t="s">
-        <v>98</v>
-      </c>
-      <c r="N7" s="2">
-        <v>46222</v>
-      </c>
-      <c r="O7" s="2">
-        <v>46237</v>
+      <c r="N7" s="1">
+        <v>46219</v>
+      </c>
+      <c r="O7" s="1">
+        <v>46216</v>
       </c>
       <c r="Q7">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="R7">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="S7" t="s">
-        <v>99</v>
-      </c>
-      <c r="T7" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="U7" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="V7" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="W7" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1270,49 +1226,49 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>396</v>
+        <v>419</v>
       </c>
       <c r="B8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C8" t="s">
         <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E8" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F8" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="G8">
-        <v>2726</v>
+        <v>2723</v>
       </c>
       <c r="H8" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="I8" t="s">
-        <v>97</v>
-      </c>
-      <c r="J8" s="2">
+        <v>94</v>
+      </c>
+      <c r="J8" s="1">
+        <v>46211</v>
+      </c>
+      <c r="K8" s="1">
         <v>46212</v>
       </c>
-      <c r="K8" s="2">
-        <v>46212</v>
-      </c>
       <c r="L8">
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>98</v>
-      </c>
-      <c r="N8" s="2">
+        <v>95</v>
+      </c>
+      <c r="N8" s="1">
         <v>46219</v>
       </c>
-      <c r="O8" s="2">
-        <v>46216</v>
+      <c r="O8" s="1">
+        <v>46237</v>
       </c>
       <c r="Q8">
         <v>7</v>
@@ -1321,16 +1277,19 @@
         <v>14</v>
       </c>
       <c r="S8" t="s">
-        <v>100</v>
+        <v>96</v>
+      </c>
+      <c r="T8" t="s">
+        <v>96</v>
       </c>
       <c r="U8" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="V8" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="W8" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1338,70 +1297,61 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9">
-        <v>419</v>
+        <v>685</v>
       </c>
       <c r="B9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s">
         <v>39</v>
       </c>
       <c r="D9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E9" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F9" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G9">
-        <v>2723</v>
+        <v>2702</v>
       </c>
       <c r="H9" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="I9" t="s">
-        <v>97</v>
-      </c>
-      <c r="J9" s="2">
-        <v>46211</v>
-      </c>
-      <c r="K9" s="2">
+        <v>93</v>
+      </c>
+      <c r="J9" s="1">
         <v>46212</v>
       </c>
+      <c r="K9" s="1">
+        <v>46212</v>
+      </c>
       <c r="L9">
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>98</v>
-      </c>
-      <c r="N9" s="2">
-        <v>46219</v>
-      </c>
-      <c r="O9" s="2">
-        <v>46237</v>
+        <v>95</v>
+      </c>
+      <c r="N9" s="1">
+        <v>46243</v>
       </c>
       <c r="Q9">
-        <v>7</v>
+        <v>-17</v>
       </c>
       <c r="R9">
         <v>14</v>
       </c>
       <c r="S9" t="s">
-        <v>99</v>
-      </c>
-      <c r="T9" t="s">
-        <v>99</v>
-      </c>
-      <c r="U9" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="V9" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="W9" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1409,61 +1359,64 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C10" t="s">
         <v>40</v>
       </c>
       <c r="D10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E10" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="F10" t="s">
+        <v>87</v>
+      </c>
+      <c r="G10">
+        <v>2736</v>
+      </c>
+      <c r="H10" t="s">
         <v>90</v>
       </c>
-      <c r="G10">
-        <v>2702</v>
-      </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>93</v>
       </c>
-      <c r="I10" t="s">
-        <v>96</v>
-      </c>
-      <c r="J10" s="2">
-        <v>46212</v>
-      </c>
-      <c r="K10" s="2">
-        <v>46212</v>
+      <c r="J10" s="1">
+        <v>46216</v>
+      </c>
+      <c r="K10" s="1">
+        <v>46217</v>
       </c>
       <c r="L10">
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>98</v>
-      </c>
-      <c r="N10" s="2">
-        <v>46243</v>
+        <v>95</v>
+      </c>
+      <c r="N10" s="1">
+        <v>46248</v>
+      </c>
+      <c r="O10" s="1">
+        <v>46248</v>
       </c>
       <c r="Q10">
-        <v>-17</v>
+        <v>-22</v>
       </c>
       <c r="R10">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="S10" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="V10" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="W10" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1471,64 +1424,67 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C11" t="s">
         <v>41</v>
       </c>
       <c r="D11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E11" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F11" t="s">
+        <v>89</v>
+      </c>
+      <c r="G11">
+        <v>2722</v>
+      </c>
+      <c r="H11" t="s">
         <v>90</v>
       </c>
-      <c r="G11">
-        <v>2736</v>
-      </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>93</v>
       </c>
-      <c r="I11" t="s">
-        <v>96</v>
-      </c>
-      <c r="J11" s="2">
-        <v>46216</v>
-      </c>
-      <c r="K11" s="2">
-        <v>46217</v>
+      <c r="J11" s="1">
+        <v>46219</v>
+      </c>
+      <c r="K11" s="1">
+        <v>46218</v>
       </c>
       <c r="L11">
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>98</v>
-      </c>
-      <c r="N11" s="2">
-        <v>46248</v>
-      </c>
-      <c r="O11" s="2">
-        <v>46248</v>
+        <v>95</v>
+      </c>
+      <c r="N11" s="1">
+        <v>46249</v>
       </c>
       <c r="Q11">
-        <v>-22</v>
+        <v>-23</v>
       </c>
       <c r="R11">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S11" t="s">
-        <v>99</v>
+        <v>96</v>
+      </c>
+      <c r="T11" t="s">
+        <v>97</v>
+      </c>
+      <c r="U11" t="s">
+        <v>104</v>
       </c>
       <c r="V11" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="W11" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1545,58 +1501,55 @@
         <v>42</v>
       </c>
       <c r="D12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E12" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F12" t="s">
+        <v>88</v>
+      </c>
+      <c r="G12">
+        <v>2729</v>
+      </c>
+      <c r="H12" t="s">
+        <v>90</v>
+      </c>
+      <c r="I12" t="s">
         <v>92</v>
       </c>
-      <c r="G12">
-        <v>2722</v>
-      </c>
-      <c r="H12" t="s">
-        <v>93</v>
-      </c>
-      <c r="I12" t="s">
-        <v>96</v>
-      </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>46219</v>
       </c>
-      <c r="K12" s="2">
-        <v>46218</v>
+      <c r="K12" s="1">
+        <v>46219</v>
       </c>
       <c r="L12">
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>98</v>
-      </c>
-      <c r="N12" s="2">
-        <v>46249</v>
+        <v>95</v>
+      </c>
+      <c r="N12" s="1">
+        <v>46230</v>
       </c>
       <c r="Q12">
-        <v>-23</v>
+        <v>-4</v>
       </c>
       <c r="R12">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S12" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="T12" t="s">
-        <v>100</v>
-      </c>
-      <c r="U12" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="V12" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="W12" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1613,55 +1566,52 @@
         <v>43</v>
       </c>
       <c r="D13" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E13" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F13" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="G13">
-        <v>2729</v>
+        <v>2703</v>
       </c>
       <c r="H13" t="s">
+        <v>90</v>
+      </c>
+      <c r="I13" t="s">
         <v>93</v>
       </c>
-      <c r="I13" t="s">
+      <c r="J13" s="1">
+        <v>46219</v>
+      </c>
+      <c r="K13" s="1">
+        <v>46220</v>
+      </c>
+      <c r="L13">
+        <v>2</v>
+      </c>
+      <c r="M13" t="s">
         <v>95</v>
       </c>
-      <c r="J13" s="2">
-        <v>46219</v>
-      </c>
-      <c r="K13" s="2">
-        <v>46219</v>
-      </c>
-      <c r="L13">
-        <v>1</v>
-      </c>
-      <c r="M13" t="s">
-        <v>98</v>
-      </c>
-      <c r="N13" s="2">
-        <v>46230</v>
+      <c r="N13" s="1">
+        <v>46251</v>
       </c>
       <c r="Q13">
-        <v>-4</v>
+        <v>-25</v>
       </c>
       <c r="R13">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S13" t="s">
-        <v>99</v>
-      </c>
-      <c r="T13" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="V13" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="W13" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1678,52 +1628,55 @@
         <v>44</v>
       </c>
       <c r="D14" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E14" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F14" t="s">
+        <v>89</v>
+      </c>
+      <c r="G14">
+        <v>2729</v>
+      </c>
+      <c r="H14" t="s">
         <v>90</v>
       </c>
-      <c r="G14">
-        <v>2703</v>
-      </c>
-      <c r="H14" t="s">
-        <v>93</v>
-      </c>
       <c r="I14" t="s">
-        <v>96</v>
-      </c>
-      <c r="J14" s="2">
+        <v>92</v>
+      </c>
+      <c r="J14" s="1">
         <v>46219</v>
       </c>
-      <c r="K14" s="2">
-        <v>46220</v>
+      <c r="K14" s="1">
+        <v>46221</v>
       </c>
       <c r="L14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M14" t="s">
-        <v>98</v>
-      </c>
-      <c r="N14" s="2">
-        <v>46251</v>
+        <v>95</v>
+      </c>
+      <c r="N14" s="1">
+        <v>46232</v>
       </c>
       <c r="Q14">
-        <v>-25</v>
+        <v>-6</v>
       </c>
       <c r="R14">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S14" t="s">
-        <v>100</v>
+        <v>96</v>
+      </c>
+      <c r="T14" t="s">
+        <v>97</v>
       </c>
       <c r="V14" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="W14" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
@@ -1731,46 +1684,49 @@
     </row>
     <row r="15" spans="1:27">
       <c r="A15">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B15" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C15" t="s">
         <v>45</v>
       </c>
       <c r="D15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E15" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F15" t="s">
+        <v>89</v>
+      </c>
+      <c r="G15">
+        <v>2730</v>
+      </c>
+      <c r="H15" t="s">
+        <v>91</v>
+      </c>
+      <c r="I15" t="s">
         <v>92</v>
       </c>
-      <c r="G15">
-        <v>2729</v>
-      </c>
-      <c r="H15" t="s">
-        <v>93</v>
-      </c>
-      <c r="I15" t="s">
+      <c r="J15" s="1">
+        <v>46220</v>
+      </c>
+      <c r="K15" s="1">
+        <v>46221</v>
+      </c>
+      <c r="L15">
+        <v>1</v>
+      </c>
+      <c r="M15" t="s">
         <v>95</v>
       </c>
-      <c r="J15" s="2">
-        <v>46219</v>
-      </c>
-      <c r="K15" s="2">
-        <v>46221</v>
-      </c>
-      <c r="L15">
-        <v>1</v>
-      </c>
-      <c r="M15" t="s">
-        <v>98</v>
-      </c>
-      <c r="N15" s="2">
+      <c r="N15" s="1">
         <v>46232</v>
+      </c>
+      <c r="O15" s="1">
+        <v>46228</v>
       </c>
       <c r="Q15">
         <v>-6</v>
@@ -1779,16 +1735,19 @@
         <v>5</v>
       </c>
       <c r="S15" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="T15" t="s">
-        <v>100</v>
+        <v>97</v>
+      </c>
+      <c r="U15" t="s">
+        <v>105</v>
       </c>
       <c r="V15" t="s">
+        <v>120</v>
+      </c>
+      <c r="W15" t="s">
         <v>124</v>
-      </c>
-      <c r="W15" t="s">
-        <v>129</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
@@ -1805,61 +1764,55 @@
         <v>46</v>
       </c>
       <c r="D16" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E16" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F16" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="G16">
-        <v>2730</v>
+        <v>2741</v>
       </c>
       <c r="H16" t="s">
+        <v>90</v>
+      </c>
+      <c r="I16" t="s">
         <v>94</v>
       </c>
-      <c r="I16" t="s">
+      <c r="J16" s="1">
+        <v>46224</v>
+      </c>
+      <c r="K16" s="1">
+        <v>46222</v>
+      </c>
+      <c r="L16">
+        <v>1</v>
+      </c>
+      <c r="M16" t="s">
         <v>95</v>
       </c>
-      <c r="J16" s="2">
-        <v>46220</v>
-      </c>
-      <c r="K16" s="2">
-        <v>46221</v>
-      </c>
-      <c r="L16">
-        <v>1</v>
-      </c>
-      <c r="M16" t="s">
-        <v>98</v>
-      </c>
-      <c r="N16" s="2">
-        <v>46232</v>
-      </c>
-      <c r="O16" s="2">
-        <v>46228</v>
+      <c r="N16" s="1">
+        <v>46229</v>
       </c>
       <c r="Q16">
-        <v>-6</v>
+        <v>-3</v>
       </c>
       <c r="R16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S16" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="T16" t="s">
-        <v>100</v>
-      </c>
-      <c r="U16" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="V16" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="W16" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AA16" t="b">
         <v>1</v>
@@ -1867,64 +1820,64 @@
     </row>
     <row r="17" spans="1:27">
       <c r="A17">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B17" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C17" t="s">
         <v>47</v>
       </c>
       <c r="D17" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E17" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F17" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G17">
-        <v>2741</v>
+        <v>2720</v>
       </c>
       <c r="H17" t="s">
+        <v>90</v>
+      </c>
+      <c r="I17" t="s">
         <v>93</v>
       </c>
-      <c r="I17" t="s">
-        <v>97</v>
-      </c>
-      <c r="J17" s="2">
-        <v>46224</v>
-      </c>
-      <c r="K17" s="2">
-        <v>46222</v>
+      <c r="J17" s="1">
+        <v>46220</v>
+      </c>
+      <c r="K17" s="1">
+        <v>46223</v>
       </c>
       <c r="L17">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="M17" t="s">
-        <v>98</v>
-      </c>
-      <c r="N17" s="2">
-        <v>46229</v>
+        <v>95</v>
+      </c>
+      <c r="N17" s="1">
+        <v>46254</v>
       </c>
       <c r="Q17">
-        <v>-3</v>
+        <v>-28</v>
       </c>
       <c r="R17">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S17" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="T17" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="V17" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="W17" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AA17" t="b">
         <v>1</v>
@@ -1941,55 +1894,58 @@
         <v>48</v>
       </c>
       <c r="D18" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E18" t="s">
+        <v>85</v>
+      </c>
+      <c r="F18" t="s">
         <v>87</v>
-      </c>
-      <c r="F18" t="s">
-        <v>90</v>
       </c>
       <c r="G18">
         <v>2720</v>
       </c>
       <c r="H18" t="s">
+        <v>90</v>
+      </c>
+      <c r="I18" t="s">
         <v>93</v>
       </c>
-      <c r="I18" t="s">
-        <v>96</v>
-      </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46220</v>
       </c>
-      <c r="K18" s="2">
-        <v>46223</v>
+      <c r="K18" s="1">
+        <v>46224</v>
       </c>
       <c r="L18">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="M18" t="s">
-        <v>98</v>
-      </c>
-      <c r="N18" s="2">
-        <v>46254</v>
+        <v>95</v>
+      </c>
+      <c r="N18" s="1">
+        <v>46255</v>
       </c>
       <c r="Q18">
-        <v>-28</v>
+        <v>-29</v>
       </c>
       <c r="R18">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S18" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="T18" t="s">
-        <v>99</v>
+        <v>96</v>
+      </c>
+      <c r="U18" t="s">
+        <v>106</v>
       </c>
       <c r="V18" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="W18" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AA18" t="b">
         <v>1</v>
@@ -2006,58 +1962,58 @@
         <v>49</v>
       </c>
       <c r="D19" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E19" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="F19" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G19">
         <v>2720</v>
       </c>
       <c r="H19" t="s">
+        <v>90</v>
+      </c>
+      <c r="I19" t="s">
         <v>93</v>
       </c>
-      <c r="I19" t="s">
-        <v>96</v>
-      </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>46220</v>
       </c>
-      <c r="K19" s="2">
-        <v>46224</v>
+      <c r="K19" s="1">
+        <v>46225</v>
       </c>
       <c r="L19">
         <v>6</v>
       </c>
       <c r="M19" t="s">
-        <v>98</v>
-      </c>
-      <c r="N19" s="2">
-        <v>46255</v>
+        <v>95</v>
+      </c>
+      <c r="N19" s="1">
+        <v>46256</v>
       </c>
       <c r="Q19">
-        <v>-29</v>
+        <v>-30</v>
       </c>
       <c r="R19">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S19" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="T19" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="U19" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="V19" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="W19" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AA19" t="b">
         <v>1</v>
@@ -2074,122 +2030,54 @@
         <v>50</v>
       </c>
       <c r="D20" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E20" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F20" t="s">
+        <v>89</v>
+      </c>
+      <c r="G20">
+        <v>2721</v>
+      </c>
+      <c r="H20" t="s">
         <v>90</v>
       </c>
-      <c r="G20">
-        <v>2720</v>
-      </c>
-      <c r="H20" t="s">
-        <v>93</v>
-      </c>
       <c r="I20" t="s">
-        <v>96</v>
-      </c>
-      <c r="J20" s="2">
-        <v>46220</v>
-      </c>
-      <c r="K20" s="2">
+        <v>94</v>
+      </c>
+      <c r="J20" s="1">
         <v>46225</v>
       </c>
+      <c r="K20" s="1">
+        <v>46226</v>
+      </c>
       <c r="L20">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M20" t="s">
-        <v>98</v>
-      </c>
-      <c r="N20" s="2">
-        <v>46256</v>
+        <v>95</v>
+      </c>
+      <c r="N20" s="1">
+        <v>46233</v>
       </c>
       <c r="Q20">
-        <v>-30</v>
+        <v>-7</v>
       </c>
       <c r="R20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S20" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="T20" t="s">
-        <v>99</v>
-      </c>
-      <c r="U20" t="s">
-        <v>110</v>
-      </c>
-      <c r="V20" t="s">
-        <v>128</v>
+        <v>96</v>
       </c>
       <c r="W20" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AA20" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:27">
-      <c r="A21">
-        <v>329</v>
-      </c>
-      <c r="B21" t="s">
-        <v>28</v>
-      </c>
-      <c r="C21" t="s">
-        <v>51</v>
-      </c>
-      <c r="D21" t="s">
-        <v>71</v>
-      </c>
-      <c r="E21" t="s">
-        <v>89</v>
-      </c>
-      <c r="F21" t="s">
-        <v>92</v>
-      </c>
-      <c r="G21">
-        <v>2721</v>
-      </c>
-      <c r="H21" t="s">
-        <v>93</v>
-      </c>
-      <c r="I21" t="s">
-        <v>97</v>
-      </c>
-      <c r="J21" s="2">
-        <v>46225</v>
-      </c>
-      <c r="K21" s="2">
-        <v>46226</v>
-      </c>
-      <c r="L21">
-        <v>1</v>
-      </c>
-      <c r="M21" t="s">
-        <v>98</v>
-      </c>
-      <c r="N21" s="2">
-        <v>46233</v>
-      </c>
-      <c r="Q21">
-        <v>-7</v>
-      </c>
-      <c r="R21">
-        <v>0</v>
-      </c>
-      <c r="S21" t="s">
-        <v>99</v>
-      </c>
-      <c r="T21" t="s">
-        <v>99</v>
-      </c>
-      <c r="W21" t="s">
-        <v>129</v>
-      </c>
-      <c r="AA21" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (23/07/2026 20:41)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="126">
   <si>
     <t>om_emg</t>
   </si>
@@ -329,6 +329,9 @@
   </si>
   <si>
     <t>Alterado o tipo da emerg. de IPLR para ANCE. Godoy 22/07/26</t>
+  </si>
+  <si>
+    <t>Será atendido com o estoque FAB pedido 17963489. Godoy 23/07/2026</t>
   </si>
   <si>
     <t>Cedeu o item para o C-98 2737. Godoy 21/07/26.</t>
@@ -869,10 +872,10 @@
         <v>98</v>
       </c>
       <c r="V2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="W2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -940,10 +943,10 @@
         <v>99</v>
       </c>
       <c r="V3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="W3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -1011,10 +1014,10 @@
         <v>100</v>
       </c>
       <c r="V4" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="W4" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -1076,10 +1079,10 @@
         <v>96</v>
       </c>
       <c r="V5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="W5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1147,10 +1150,10 @@
         <v>101</v>
       </c>
       <c r="V6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="W6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1215,10 +1218,10 @@
         <v>102</v>
       </c>
       <c r="V7" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="W7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1286,10 +1289,10 @@
         <v>103</v>
       </c>
       <c r="V8" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="W8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1348,10 +1351,10 @@
         <v>96</v>
       </c>
       <c r="V9" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="W9" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1413,10 +1416,10 @@
         <v>96</v>
       </c>
       <c r="V10" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="W10" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1481,10 +1484,10 @@
         <v>104</v>
       </c>
       <c r="V11" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="W11" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1546,10 +1549,10 @@
         <v>97</v>
       </c>
       <c r="V12" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="W12" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1607,11 +1610,14 @@
       <c r="S13" t="s">
         <v>97</v>
       </c>
+      <c r="U13" t="s">
+        <v>105</v>
+      </c>
       <c r="V13" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="W13" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1673,10 +1679,10 @@
         <v>97</v>
       </c>
       <c r="V14" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="W14" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
@@ -1741,13 +1747,13 @@
         <v>97</v>
       </c>
       <c r="U15" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="V15" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="W15" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
@@ -1809,10 +1815,10 @@
         <v>97</v>
       </c>
       <c r="V16" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="W16" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AA16" t="b">
         <v>1</v>
@@ -1874,10 +1880,10 @@
         <v>96</v>
       </c>
       <c r="V17" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="W17" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AA17" t="b">
         <v>1</v>
@@ -1939,13 +1945,13 @@
         <v>96</v>
       </c>
       <c r="U18" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="V18" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="W18" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AA18" t="b">
         <v>1</v>
@@ -2007,13 +2013,13 @@
         <v>96</v>
       </c>
       <c r="U19" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="V19" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="W19" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AA19" t="b">
         <v>1</v>
@@ -2075,7 +2081,7 @@
         <v>96</v>
       </c>
       <c r="W20" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AA20" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (24/07/2026 17:52)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="100">
   <si>
     <t>om_emg</t>
   </si>
@@ -109,27 +109,15 @@
     <t>CLA</t>
   </si>
   <si>
-    <t>BABE</t>
-  </si>
-  <si>
     <t>313260017747</t>
   </si>
   <si>
-    <t>329260019153</t>
-  </si>
-  <si>
     <t>329260019181</t>
   </si>
   <si>
     <t>685260012303</t>
   </si>
   <si>
-    <t>419260000556</t>
-  </si>
-  <si>
-    <t>396260016566</t>
-  </si>
-  <si>
     <t>419260000557</t>
   </si>
   <si>
@@ -160,33 +148,15 @@
     <t>329260019225</t>
   </si>
   <si>
-    <t>329260019226</t>
-  </si>
-  <si>
-    <t>329260019227</t>
-  </si>
-  <si>
-    <t>329260019241</t>
-  </si>
-  <si>
     <t>1214134-1</t>
   </si>
   <si>
-    <t>TWINA0502</t>
-  </si>
-  <si>
     <t>C145-00-46</t>
   </si>
   <si>
     <t>065-0065-01</t>
   </si>
   <si>
-    <t>066-3046-07</t>
-  </si>
-  <si>
-    <t>060-0015-00</t>
-  </si>
-  <si>
     <t>3244897-4</t>
   </si>
   <si>
@@ -217,33 +187,15 @@
     <t>MS21442-121</t>
   </si>
   <si>
-    <t>2625014-10</t>
-  </si>
-  <si>
-    <t>2625014-9</t>
-  </si>
-  <si>
-    <t>9910592-2</t>
-  </si>
-  <si>
     <t>BELLCRANK ASSY</t>
   </si>
   <si>
-    <t>PROBE TEMPERATURE</t>
-  </si>
-  <si>
     <t>TRANSMISSION ASSY</t>
   </si>
   <si>
     <t>SELECTOR ALT</t>
   </si>
   <si>
-    <t>CONTROL,INDICATOR</t>
-  </si>
-  <si>
-    <t>CONTROL,DIRECTIONAL,</t>
-  </si>
-  <si>
     <t>FUEL CONTROL UNIT</t>
   </si>
   <si>
@@ -271,12 +223,6 @@
     <t>BEARING,ROLLER,NEEDL</t>
   </si>
   <si>
-    <t>SPACER</t>
-  </si>
-  <si>
-    <t>ALTERNADOR</t>
-  </si>
-  <si>
     <t>C</t>
   </si>
   <si>
@@ -295,12 +241,12 @@
     <t>IPLR</t>
   </si>
   <si>
+    <t>AIFP</t>
+  </si>
+  <si>
     <t>ANCE</t>
   </si>
   <si>
-    <t>AIFP</t>
-  </si>
-  <si>
     <t>EA</t>
   </si>
   <si>
@@ -313,18 +259,9 @@
     <t>Foram cedidos para o C-98 2733. / De acordo com o manual da aeronave, o QPA é 02 EA por cadeira. Sendo o total para a aeronave 04 EA.A demanda aberta foi de  4EA, o SO Bispo que intermediou . Wallace 29.05</t>
   </si>
   <si>
-    <t>Volume retirado na loja GOLLOG - BSB por tanise Assis em 03/07/2026 - Godoy 08/07/2026. Recibo não se encontra na Pasta do DRIVE. Godoy 08/07/2026.</t>
-  </si>
-  <si>
     <t>Vee One tem alguma atualização do DPE ?. Godoy 23/07/26</t>
   </si>
   <si>
-    <t>AWB 12745918331 volume retirado na loja GOLLOG - BEL por bispo em 10/07/2026 - Godoy 13/07/2026. Recibo não se encontra na Pasta do DRIVE. Godoy 17/07/2026.</t>
-  </si>
-  <si>
-    <t>Cedeu o item para o C-98 2721. Ramon 09/07/26. AWB 12746175415 - 2 volumes retirados na loja GOLLOG - BEL por bispo em 13/07/26. Godoy 15/07/26. Vee One, não temos o recibo assinado. Godoy 16/07/26.</t>
-  </si>
-  <si>
     <t>AWB 12747899051 volume retirado na loja GOLLOG - BEL por marlos em 20/07. Godoy 22/07/2026.</t>
   </si>
   <si>
@@ -337,46 +274,34 @@
     <t>Cedeu o item para o C-98 2737. Godoy 21/07/26.</t>
   </si>
   <si>
-    <t>AWB 12748301050 - volume retirado na loja GOLLOG - BSB por MARIO JORGE BARRIOLi em 21/07. Godoy 23/07/26</t>
-  </si>
-  <si>
     <t>Foi solicitado via email no dia 02-03-2 o atendimento do item com estoque FAB. Claudio -02-03-26 - Em resposta, a coordenadoria disse que o estque seria insuficiente. Foi verificado que na T.O da ANV o QPA para esse item são 2 EA, solicitei confirmação. - Cláudio -02-03-2026. Solicitado o cancelamento da emergência em função da quantidade cedida ao 2733 ter sido de 01ea. Considerando o QPA 02 ea. Encontra-se em tratativa junto a fiscalização e o gestor do contrato conforme mensagem de e-mail de 05/03. - SOLICITAÇÃO E-C98-26047.Colocado pedido AOG Textron WB0003068789 - previsão de entrega 60 dias em média. Os demais fornecedores informaram não ter em estoque ou não possuírem a certificação necessária da peça.</t>
   </si>
   <si>
-    <t>Colocado pedido na Textron IJ17507011. Previsão de entrega em Miami 17/06. Carga recepcionada no GIG 24/06. Canal verde dia 26/06. DPE V1 29/06. Verificar entrega do item. ATZ 30/06 - MATERIAL EM RECEBIMENTO V1 30-06-2026 - MATERIAL EM PROCESSO DE ENVIO RECIBO 524/FAB/26 ATZ RC 30-06-2026 - MATERIAL EM TRANSITO - AWB 12744330731 DPE 03/07/2026 - MATERIAL RECEBIDO POR tanise Assis RG 14807641751 DIA 03/07/2026</t>
-  </si>
-  <si>
     <t>Colocado pedido AOG Textron IJ17557538 - previsão de entrega em Miami 08/07. Previsão de chegada GIG 09/07 - MATERIAL EM TRANSITO - RECIBO 551/FAB/26 - ENVIADO PN COMPLETO PARA SANAR A EMERGENCIA DO 2709, ENVIADO MODAL TERRESTRE, DPE 13/07/2026</t>
   </si>
   <si>
-    <t>confirmado entrega 01 ea hj(21/07/26) pela William - REZ</t>
-  </si>
-  <si>
-    <t>MATERIAL EM TRANSITO - AWB 12745918331 dpe 11/07/2026 - atz rc 08/07/2026</t>
-  </si>
-  <si>
-    <t>Atendido em 09/07/26 AWB 12746175415 - CLA (09/07/26)</t>
+    <t>confirmado entrega 01 ea hj(21/07/26) pela William - REZ - item aguardando minuta e nota para transporte CLA-23-07</t>
   </si>
   <si>
     <t>Aguardando o retorno dos subcomponentes removidos da unidade para ser enviado a oficiana para aplicação na unidade Prazo apos aprovação 10 dias ATZ Marcio 9/7/26 14 53 - Enviado uma FCU em 17/7 fornecida pela FAB , ATZ Macio, Aguardando a atualização com o recibo e AWB ATZ Marcio 20/7 - FCU ENVIADA FOI RECUSADA PELA INSPETORIA DE RECEBIMENTO DA BABE - 20/07/2026 RC - ITEM ATENDIDO COM ESTOQUE FAB AWB 127-4789 9051</t>
   </si>
   <si>
-    <t>Colocado pedido junto ao fornecedor AEROBASE, aguardando pagamento proforma. ATZ 21/07</t>
-  </si>
-  <si>
-    <t>Colocado pedido Textron IJ17575583 - entregue em Miami 15/07. Carga rercepcionada GIG 19/07 - Aguardando liberação do SEFAZ. ATZ 21/07</t>
+    <t>Colocado pedido junto ao fornecedor LEGACY PARTS, validando prazo de entrega em Miami. ATZ 23/07</t>
+  </si>
+  <si>
+    <t>Colocado pedido Textron IJ17575583 - entregue em Miami 15/07. Carga rercepcionada GIG 19/07 - Aguardando liberação do SEFAZ. ATZ 21/07 - material em processo de expedição RC 23/07/2026</t>
   </si>
   <si>
     <t>Item em bancada porem em pessimo estado, foi solicitado recolhimento de mais unidades para envio a oficina para tentativa de reparo ATZ Marcio 17/7/26. Solicitado abertura de O.S. para 3EA do item no dia 16-07-26 via Email para a Coordenadoria - CLA-21-07-26</t>
   </si>
   <si>
-    <t>Nao temos oficina no Brasil para reparo desse item, temos que iniciar processo de aquisiçáo do material para atendimento a essa necessidade ATZ Marcio 17/7/26 - Efetuada compra em AOG , aguardando o AWB de envio para Natal, peça saindo do Espirito Santo ATZ Marcio 20/7 15:54</t>
-  </si>
-  <si>
-    <t>Validando atendimento via estoque FAB. ATZ 20/07</t>
-  </si>
-  <si>
-    <t>Consta 1 each em condição de uso em MANAUS, Enviado 1 unidade (CORE) para reparo na oficina no RJ em 17/7, orçamento aprovado em 21/7 com DPE de 5 dias para entrega na V1 JPA, ATZ Marcio 21/7</t>
+    <t>Nao temos oficina no Brasil para reparo desse item, temos que iniciar processo de aquisiçáo do material para atendimento a essa necessidade ATZ Marcio 17/7/26 - Efetuada compra em AOG , aguardando o AWB de envio para Natal, peça saindo do Espirito Santo ATZ Marcio 20/7 15:54 - AWB 12748559512 DPE 24/07/2026</t>
+  </si>
+  <si>
+    <t>Será atendido via estoque TSAU. ATZ 23/07. Foi solicitado o atendimento com estoque FAB -CLA -dia 23-07</t>
+  </si>
+  <si>
+    <t>Consta 1 each em condição de uso em MANAUS, Enviado 1 unidade (CORE) para reparo na oficina no RJ em 17/7, orçamento aprovado em 21/7 com DPE de 5 dias (27/7) para entrega na V1 JPA, ATZ Marcio 21/7</t>
   </si>
   <si>
     <t>material enviado com STK FAB - AWB 12748581702 - DPE 25/07/2026 - atz rc 22/07/2026- Enviado para o Operador dia 21/07/26 - AWB 127-4857 9742- REZ -22/07/26</t>
@@ -385,10 +310,7 @@
     <t>Enviado para o Operador dia 21/07/26 - AWB 127-4858 1702 - REZ -22/07/26</t>
   </si>
   <si>
-    <t>PEDIDO NO EPM E-C98-26059 - CLA-21-07</t>
-  </si>
-  <si>
-    <t>FOI TRANSFERIDO DA BAMN PARA BABR VIA GMM202667292001554 AWB 127-4830 1050 ENVIADO DIA 20-07-26 - CLA-21-07</t>
+    <t>Em processo de cotação junto aos fornecedores. ATZ 23/07</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -727,7 +649,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA20"/>
+  <dimension ref="A1:AA14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -821,25 +743,25 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="E2" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="F2" t="s">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="G2">
         <v>2730</v>
       </c>
       <c r="H2" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="I2" t="s">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="J2" s="1">
         <v>46076</v>
@@ -851,7 +773,7 @@
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="N2" s="1">
         <v>46091</v>
@@ -860,22 +782,22 @@
         <v>46287</v>
       </c>
       <c r="Q2">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="R2">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="S2" t="s">
-        <v>96</v>
+        <v>78</v>
       </c>
       <c r="U2" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="V2" t="s">
-        <v>108</v>
+        <v>86</v>
       </c>
       <c r="W2" t="s">
-        <v>125</v>
+        <v>99</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -889,40 +811,40 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="E3" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="F3" t="s">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="G3">
         <v>2721</v>
       </c>
       <c r="H3" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="I3" t="s">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="J3" s="1">
-        <v>46185</v>
+        <v>46209</v>
       </c>
       <c r="K3" s="1">
-        <v>46185</v>
+        <v>46210</v>
       </c>
       <c r="L3">
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="N3" s="1">
-        <v>46216</v>
+        <v>46217</v>
       </c>
       <c r="O3" s="1">
         <v>46216</v>
@@ -931,22 +853,22 @@
         <v>10</v>
       </c>
       <c r="R3">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="S3" t="s">
-        <v>96</v>
+        <v>78</v>
       </c>
       <c r="T3" t="s">
-        <v>96</v>
+        <v>78</v>
       </c>
       <c r="U3" t="s">
+        <v>81</v>
+      </c>
+      <c r="V3" t="s">
+        <v>87</v>
+      </c>
+      <c r="W3" t="s">
         <v>99</v>
-      </c>
-      <c r="V3" t="s">
-        <v>109</v>
-      </c>
-      <c r="W3" t="s">
-        <v>125</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -954,34 +876,34 @@
     </row>
     <row r="4" spans="1:27">
       <c r="A4">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="E4" t="s">
+        <v>59</v>
+      </c>
+      <c r="F4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G4">
+        <v>2719</v>
+      </c>
+      <c r="H4" t="s">
         <v>72</v>
       </c>
-      <c r="F4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G4">
-        <v>2721</v>
-      </c>
-      <c r="H4" t="s">
-        <v>90</v>
-      </c>
       <c r="I4" t="s">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="J4" s="1">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="K4" s="1">
         <v>46210</v>
@@ -990,34 +912,28 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="N4" s="1">
-        <v>46217</v>
+        <v>46241</v>
       </c>
       <c r="O4" s="1">
-        <v>46216</v>
+        <v>46238</v>
       </c>
       <c r="Q4">
-        <v>9</v>
+        <v>-14</v>
       </c>
       <c r="R4">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="S4" t="s">
-        <v>96</v>
-      </c>
-      <c r="T4" t="s">
-        <v>96</v>
-      </c>
-      <c r="U4" t="s">
-        <v>100</v>
+        <v>78</v>
       </c>
       <c r="V4" t="s">
-        <v>110</v>
+        <v>88</v>
       </c>
       <c r="W4" t="s">
-        <v>125</v>
+        <v>99</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -1025,64 +941,70 @@
     </row>
     <row r="5" spans="1:27">
       <c r="A5">
-        <v>685</v>
+        <v>419</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="E5" t="s">
+        <v>60</v>
+      </c>
+      <c r="F5" t="s">
+        <v>71</v>
+      </c>
+      <c r="G5">
+        <v>2723</v>
+      </c>
+      <c r="H5" t="s">
         <v>73</v>
       </c>
-      <c r="F5" t="s">
-        <v>88</v>
-      </c>
-      <c r="G5">
-        <v>2719</v>
-      </c>
-      <c r="H5" t="s">
-        <v>90</v>
-      </c>
       <c r="I5" t="s">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="J5" s="1">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="K5" s="1">
-        <v>46210</v>
+        <v>46212</v>
       </c>
       <c r="L5">
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="N5" s="1">
-        <v>46241</v>
+        <v>46219</v>
       </c>
       <c r="O5" s="1">
-        <v>46238</v>
+        <v>46237</v>
       </c>
       <c r="Q5">
-        <v>-15</v>
+        <v>8</v>
       </c>
       <c r="R5">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="S5" t="s">
-        <v>96</v>
+        <v>78</v>
+      </c>
+      <c r="T5" t="s">
+        <v>78</v>
+      </c>
+      <c r="U5" t="s">
+        <v>82</v>
       </c>
       <c r="V5" t="s">
-        <v>111</v>
+        <v>89</v>
       </c>
       <c r="W5" t="s">
-        <v>125</v>
+        <v>99</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1090,70 +1012,61 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6">
-        <v>419</v>
+        <v>685</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="E6" t="s">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="F6" t="s">
-        <v>89</v>
+        <v>69</v>
       </c>
       <c r="G6">
-        <v>2723</v>
+        <v>2702</v>
       </c>
       <c r="H6" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="I6" t="s">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="J6" s="1">
-        <v>46210</v>
+        <v>46212</v>
       </c>
       <c r="K6" s="1">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="L6">
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="N6" s="1">
-        <v>46218</v>
-      </c>
-      <c r="O6" s="1">
-        <v>46213</v>
+        <v>46243</v>
       </c>
       <c r="Q6">
-        <v>8</v>
+        <v>-16</v>
       </c>
       <c r="R6">
         <v>15</v>
       </c>
       <c r="S6" t="s">
-        <v>96</v>
-      </c>
-      <c r="T6" t="s">
-        <v>97</v>
-      </c>
-      <c r="U6" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="V6" t="s">
-        <v>112</v>
+        <v>90</v>
       </c>
       <c r="W6" t="s">
-        <v>125</v>
+        <v>99</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1161,67 +1074,64 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>396</v>
+        <v>313</v>
       </c>
       <c r="B7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="E7" t="s">
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="F7" t="s">
-        <v>89</v>
+        <v>69</v>
       </c>
       <c r="G7">
-        <v>2726</v>
+        <v>2736</v>
       </c>
       <c r="H7" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="I7" t="s">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="J7" s="1">
-        <v>46212</v>
+        <v>46216</v>
       </c>
       <c r="K7" s="1">
-        <v>46212</v>
+        <v>46217</v>
       </c>
       <c r="L7">
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="N7" s="1">
-        <v>46219</v>
+        <v>46248</v>
       </c>
       <c r="O7" s="1">
-        <v>46216</v>
+        <v>46248</v>
       </c>
       <c r="Q7">
-        <v>7</v>
+        <v>-21</v>
       </c>
       <c r="R7">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="S7" t="s">
-        <v>97</v>
-      </c>
-      <c r="U7" t="s">
-        <v>102</v>
+        <v>78</v>
       </c>
       <c r="V7" t="s">
-        <v>113</v>
+        <v>91</v>
       </c>
       <c r="W7" t="s">
-        <v>125</v>
+        <v>99</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1229,70 +1139,67 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>419</v>
+        <v>685</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D8" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="E8" t="s">
+        <v>62</v>
+      </c>
+      <c r="F8" t="s">
+        <v>71</v>
+      </c>
+      <c r="G8">
+        <v>2722</v>
+      </c>
+      <c r="H8" t="s">
+        <v>72</v>
+      </c>
+      <c r="I8" t="s">
         <v>76</v>
       </c>
-      <c r="F8" t="s">
-        <v>89</v>
-      </c>
-      <c r="G8">
-        <v>2723</v>
-      </c>
-      <c r="H8" t="s">
-        <v>91</v>
-      </c>
-      <c r="I8" t="s">
-        <v>94</v>
-      </c>
       <c r="J8" s="1">
-        <v>46211</v>
+        <v>46219</v>
       </c>
       <c r="K8" s="1">
-        <v>46212</v>
+        <v>46218</v>
       </c>
       <c r="L8">
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="N8" s="1">
-        <v>46219</v>
-      </c>
-      <c r="O8" s="1">
-        <v>46237</v>
+        <v>46249</v>
       </c>
       <c r="Q8">
-        <v>7</v>
+        <v>-22</v>
       </c>
       <c r="R8">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="S8" t="s">
-        <v>96</v>
+        <v>78</v>
       </c>
       <c r="T8" t="s">
-        <v>96</v>
+        <v>79</v>
       </c>
       <c r="U8" t="s">
-        <v>103</v>
+        <v>83</v>
       </c>
       <c r="V8" t="s">
-        <v>114</v>
+        <v>92</v>
       </c>
       <c r="W8" t="s">
-        <v>125</v>
+        <v>99</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1306,55 +1213,61 @@
         <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="E9" t="s">
+        <v>63</v>
+      </c>
+      <c r="F9" t="s">
+        <v>70</v>
+      </c>
+      <c r="G9">
+        <v>2729</v>
+      </c>
+      <c r="H9" t="s">
+        <v>72</v>
+      </c>
+      <c r="I9" t="s">
+        <v>74</v>
+      </c>
+      <c r="J9" s="1">
+        <v>46219</v>
+      </c>
+      <c r="K9" s="1">
+        <v>46219</v>
+      </c>
+      <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9" t="s">
         <v>77</v>
       </c>
-      <c r="F9" t="s">
-        <v>87</v>
-      </c>
-      <c r="G9">
-        <v>2702</v>
-      </c>
-      <c r="H9" t="s">
-        <v>90</v>
-      </c>
-      <c r="I9" t="s">
+      <c r="N9" s="1">
+        <v>46230</v>
+      </c>
+      <c r="O9" s="1">
+        <v>46227</v>
+      </c>
+      <c r="Q9">
+        <v>-3</v>
+      </c>
+      <c r="R9">
+        <v>8</v>
+      </c>
+      <c r="S9" t="s">
+        <v>78</v>
+      </c>
+      <c r="T9" t="s">
+        <v>79</v>
+      </c>
+      <c r="V9" t="s">
         <v>93</v>
       </c>
-      <c r="J9" s="1">
-        <v>46212</v>
-      </c>
-      <c r="K9" s="1">
-        <v>46212</v>
-      </c>
-      <c r="L9">
-        <v>1</v>
-      </c>
-      <c r="M9" t="s">
-        <v>95</v>
-      </c>
-      <c r="N9" s="1">
-        <v>46243</v>
-      </c>
-      <c r="Q9">
-        <v>-17</v>
-      </c>
-      <c r="R9">
-        <v>14</v>
-      </c>
-      <c r="S9" t="s">
-        <v>96</v>
-      </c>
-      <c r="V9" t="s">
-        <v>115</v>
-      </c>
       <c r="W9" t="s">
-        <v>125</v>
+        <v>99</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1362,64 +1275,64 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D10" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="E10" t="s">
+        <v>64</v>
+      </c>
+      <c r="F10" t="s">
+        <v>69</v>
+      </c>
+      <c r="G10">
+        <v>2703</v>
+      </c>
+      <c r="H10" t="s">
+        <v>73</v>
+      </c>
+      <c r="I10" t="s">
+        <v>76</v>
+      </c>
+      <c r="J10" s="1">
+        <v>46219</v>
+      </c>
+      <c r="K10" s="1">
+        <v>46220</v>
+      </c>
+      <c r="L10">
+        <v>2</v>
+      </c>
+      <c r="M10" t="s">
         <v>77</v>
       </c>
-      <c r="F10" t="s">
-        <v>87</v>
-      </c>
-      <c r="G10">
-        <v>2736</v>
-      </c>
-      <c r="H10" t="s">
-        <v>90</v>
-      </c>
-      <c r="I10" t="s">
-        <v>93</v>
-      </c>
-      <c r="J10" s="1">
-        <v>46216</v>
-      </c>
-      <c r="K10" s="1">
-        <v>46217</v>
-      </c>
-      <c r="L10">
-        <v>1</v>
-      </c>
-      <c r="M10" t="s">
-        <v>95</v>
-      </c>
       <c r="N10" s="1">
-        <v>46248</v>
-      </c>
-      <c r="O10" s="1">
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="Q10">
-        <v>-22</v>
+        <v>-24</v>
       </c>
       <c r="R10">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="S10" t="s">
-        <v>96</v>
+        <v>79</v>
+      </c>
+      <c r="U10" t="s">
+        <v>84</v>
       </c>
       <c r="V10" t="s">
-        <v>116</v>
+        <v>94</v>
       </c>
       <c r="W10" t="s">
-        <v>125</v>
+        <v>99</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1433,61 +1346,58 @@
         <v>29</v>
       </c>
       <c r="C11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D11" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="E11" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="F11" t="s">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="G11">
-        <v>2722</v>
+        <v>2729</v>
       </c>
       <c r="H11" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="I11" t="s">
-        <v>93</v>
+        <v>74</v>
       </c>
       <c r="J11" s="1">
         <v>46219</v>
       </c>
       <c r="K11" s="1">
-        <v>46218</v>
+        <v>46221</v>
       </c>
       <c r="L11">
         <v>1</v>
       </c>
       <c r="M11" t="s">
+        <v>77</v>
+      </c>
+      <c r="N11" s="1">
+        <v>46232</v>
+      </c>
+      <c r="Q11">
+        <v>-5</v>
+      </c>
+      <c r="R11">
+        <v>6</v>
+      </c>
+      <c r="S11" t="s">
+        <v>78</v>
+      </c>
+      <c r="T11" t="s">
+        <v>79</v>
+      </c>
+      <c r="V11" t="s">
         <v>95</v>
       </c>
-      <c r="N11" s="1">
-        <v>46249</v>
-      </c>
-      <c r="Q11">
-        <v>-23</v>
-      </c>
-      <c r="R11">
-        <v>8</v>
-      </c>
-      <c r="S11" t="s">
-        <v>96</v>
-      </c>
-      <c r="T11" t="s">
-        <v>97</v>
-      </c>
-      <c r="U11" t="s">
-        <v>104</v>
-      </c>
-      <c r="V11" t="s">
-        <v>117</v>
-      </c>
       <c r="W11" t="s">
-        <v>125</v>
+        <v>99</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1495,64 +1405,70 @@
     </row>
     <row r="12" spans="1:27">
       <c r="A12">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D12" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="E12" t="s">
+        <v>66</v>
+      </c>
+      <c r="F12" t="s">
+        <v>71</v>
+      </c>
+      <c r="G12">
+        <v>2730</v>
+      </c>
+      <c r="H12" t="s">
+        <v>73</v>
+      </c>
+      <c r="I12" t="s">
+        <v>74</v>
+      </c>
+      <c r="J12" s="1">
+        <v>46220</v>
+      </c>
+      <c r="K12" s="1">
+        <v>46221</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12" t="s">
+        <v>77</v>
+      </c>
+      <c r="N12" s="1">
+        <v>46232</v>
+      </c>
+      <c r="O12" s="1">
+        <v>46228</v>
+      </c>
+      <c r="Q12">
+        <v>-5</v>
+      </c>
+      <c r="R12">
+        <v>6</v>
+      </c>
+      <c r="S12" t="s">
+        <v>78</v>
+      </c>
+      <c r="T12" t="s">
         <v>79</v>
       </c>
-      <c r="F12" t="s">
-        <v>88</v>
-      </c>
-      <c r="G12">
-        <v>2729</v>
-      </c>
-      <c r="H12" t="s">
-        <v>90</v>
-      </c>
-      <c r="I12" t="s">
-        <v>92</v>
-      </c>
-      <c r="J12" s="1">
-        <v>46219</v>
-      </c>
-      <c r="K12" s="1">
-        <v>46219</v>
-      </c>
-      <c r="L12">
-        <v>1</v>
-      </c>
-      <c r="M12" t="s">
-        <v>95</v>
-      </c>
-      <c r="N12" s="1">
-        <v>46230</v>
-      </c>
-      <c r="Q12">
-        <v>-4</v>
-      </c>
-      <c r="R12">
-        <v>7</v>
-      </c>
-      <c r="S12" t="s">
+      <c r="U12" t="s">
+        <v>85</v>
+      </c>
+      <c r="V12" t="s">
         <v>96</v>
       </c>
-      <c r="T12" t="s">
-        <v>97</v>
-      </c>
-      <c r="V12" t="s">
-        <v>118</v>
-      </c>
       <c r="W12" t="s">
-        <v>125</v>
+        <v>99</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1560,64 +1476,64 @@
     </row>
     <row r="13" spans="1:27">
       <c r="A13">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C13" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D13" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="E13" t="s">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="F13" t="s">
-        <v>87</v>
+        <v>71</v>
       </c>
       <c r="G13">
-        <v>2703</v>
+        <v>2741</v>
       </c>
       <c r="H13" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="I13" t="s">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="J13" s="1">
-        <v>46219</v>
+        <v>46224</v>
       </c>
       <c r="K13" s="1">
-        <v>46220</v>
+        <v>46222</v>
       </c>
       <c r="L13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="N13" s="1">
-        <v>46251</v>
+        <v>46229</v>
       </c>
       <c r="Q13">
-        <v>-25</v>
+        <v>-2</v>
       </c>
       <c r="R13">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S13" t="s">
+        <v>78</v>
+      </c>
+      <c r="T13" t="s">
+        <v>79</v>
+      </c>
+      <c r="V13" t="s">
         <v>97</v>
       </c>
-      <c r="U13" t="s">
-        <v>105</v>
-      </c>
-      <c r="V13" t="s">
-        <v>119</v>
-      </c>
       <c r="W13" t="s">
-        <v>125</v>
+        <v>99</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1625,465 +1541,66 @@
     </row>
     <row r="14" spans="1:27">
       <c r="A14">
-        <v>685</v>
+        <v>329</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D14" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="E14" t="s">
-        <v>81</v>
+        <v>68</v>
       </c>
       <c r="F14" t="s">
-        <v>89</v>
+        <v>69</v>
       </c>
       <c r="G14">
-        <v>2729</v>
+        <v>2720</v>
       </c>
       <c r="H14" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="I14" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="J14" s="1">
-        <v>46219</v>
+        <v>46220</v>
       </c>
       <c r="K14" s="1">
-        <v>46221</v>
+        <v>46223</v>
       </c>
       <c r="L14">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="M14" t="s">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="N14" s="1">
-        <v>46232</v>
+        <v>46254</v>
       </c>
       <c r="Q14">
-        <v>-6</v>
+        <v>-27</v>
       </c>
       <c r="R14">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S14" t="s">
-        <v>96</v>
+        <v>78</v>
       </c>
       <c r="T14" t="s">
-        <v>97</v>
+        <v>78</v>
       </c>
       <c r="V14" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="W14" t="s">
-        <v>125</v>
+        <v>99</v>
       </c>
       <c r="AA14" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:27">
-      <c r="A15">
-        <v>313</v>
-      </c>
-      <c r="B15" t="s">
-        <v>27</v>
-      </c>
-      <c r="C15" t="s">
-        <v>45</v>
-      </c>
-      <c r="D15" t="s">
-        <v>64</v>
-      </c>
-      <c r="E15" t="s">
-        <v>82</v>
-      </c>
-      <c r="F15" t="s">
-        <v>89</v>
-      </c>
-      <c r="G15">
-        <v>2730</v>
-      </c>
-      <c r="H15" t="s">
-        <v>91</v>
-      </c>
-      <c r="I15" t="s">
-        <v>92</v>
-      </c>
-      <c r="J15" s="1">
-        <v>46220</v>
-      </c>
-      <c r="K15" s="1">
-        <v>46221</v>
-      </c>
-      <c r="L15">
-        <v>1</v>
-      </c>
-      <c r="M15" t="s">
-        <v>95</v>
-      </c>
-      <c r="N15" s="1">
-        <v>46232</v>
-      </c>
-      <c r="O15" s="1">
-        <v>46228</v>
-      </c>
-      <c r="Q15">
-        <v>-6</v>
-      </c>
-      <c r="R15">
-        <v>5</v>
-      </c>
-      <c r="S15" t="s">
-        <v>96</v>
-      </c>
-      <c r="T15" t="s">
-        <v>97</v>
-      </c>
-      <c r="U15" t="s">
-        <v>106</v>
-      </c>
-      <c r="V15" t="s">
-        <v>121</v>
-      </c>
-      <c r="W15" t="s">
-        <v>125</v>
-      </c>
-      <c r="AA15" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:27">
-      <c r="A16">
-        <v>313</v>
-      </c>
-      <c r="B16" t="s">
-        <v>27</v>
-      </c>
-      <c r="C16" t="s">
-        <v>46</v>
-      </c>
-      <c r="D16" t="s">
-        <v>65</v>
-      </c>
-      <c r="E16" t="s">
-        <v>83</v>
-      </c>
-      <c r="F16" t="s">
-        <v>89</v>
-      </c>
-      <c r="G16">
-        <v>2741</v>
-      </c>
-      <c r="H16" t="s">
-        <v>90</v>
-      </c>
-      <c r="I16" t="s">
-        <v>94</v>
-      </c>
-      <c r="J16" s="1">
-        <v>46224</v>
-      </c>
-      <c r="K16" s="1">
-        <v>46222</v>
-      </c>
-      <c r="L16">
-        <v>1</v>
-      </c>
-      <c r="M16" t="s">
-        <v>95</v>
-      </c>
-      <c r="N16" s="1">
-        <v>46229</v>
-      </c>
-      <c r="Q16">
-        <v>-3</v>
-      </c>
-      <c r="R16">
-        <v>4</v>
-      </c>
-      <c r="S16" t="s">
-        <v>96</v>
-      </c>
-      <c r="T16" t="s">
-        <v>97</v>
-      </c>
-      <c r="V16" t="s">
-        <v>122</v>
-      </c>
-      <c r="W16" t="s">
-        <v>125</v>
-      </c>
-      <c r="AA16" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:27">
-      <c r="A17">
-        <v>329</v>
-      </c>
-      <c r="B17" t="s">
-        <v>28</v>
-      </c>
-      <c r="C17" t="s">
-        <v>47</v>
-      </c>
-      <c r="D17" t="s">
-        <v>66</v>
-      </c>
-      <c r="E17" t="s">
-        <v>84</v>
-      </c>
-      <c r="F17" t="s">
-        <v>87</v>
-      </c>
-      <c r="G17">
-        <v>2720</v>
-      </c>
-      <c r="H17" t="s">
-        <v>90</v>
-      </c>
-      <c r="I17" t="s">
-        <v>93</v>
-      </c>
-      <c r="J17" s="1">
-        <v>46220</v>
-      </c>
-      <c r="K17" s="1">
-        <v>46223</v>
-      </c>
-      <c r="L17">
-        <v>10</v>
-      </c>
-      <c r="M17" t="s">
-        <v>95</v>
-      </c>
-      <c r="N17" s="1">
-        <v>46254</v>
-      </c>
-      <c r="Q17">
-        <v>-28</v>
-      </c>
-      <c r="R17">
-        <v>3</v>
-      </c>
-      <c r="S17" t="s">
-        <v>96</v>
-      </c>
-      <c r="T17" t="s">
-        <v>96</v>
-      </c>
-      <c r="V17" t="s">
-        <v>123</v>
-      </c>
-      <c r="W17" t="s">
-        <v>125</v>
-      </c>
-      <c r="AA17" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:27">
-      <c r="A18">
-        <v>329</v>
-      </c>
-      <c r="B18" t="s">
-        <v>28</v>
-      </c>
-      <c r="C18" t="s">
-        <v>48</v>
-      </c>
-      <c r="D18" t="s">
-        <v>67</v>
-      </c>
-      <c r="E18" t="s">
-        <v>85</v>
-      </c>
-      <c r="F18" t="s">
-        <v>87</v>
-      </c>
-      <c r="G18">
-        <v>2720</v>
-      </c>
-      <c r="H18" t="s">
-        <v>90</v>
-      </c>
-      <c r="I18" t="s">
-        <v>93</v>
-      </c>
-      <c r="J18" s="1">
-        <v>46220</v>
-      </c>
-      <c r="K18" s="1">
-        <v>46224</v>
-      </c>
-      <c r="L18">
-        <v>6</v>
-      </c>
-      <c r="M18" t="s">
-        <v>95</v>
-      </c>
-      <c r="N18" s="1">
-        <v>46255</v>
-      </c>
-      <c r="Q18">
-        <v>-29</v>
-      </c>
-      <c r="R18">
-        <v>2</v>
-      </c>
-      <c r="S18" t="s">
-        <v>96</v>
-      </c>
-      <c r="T18" t="s">
-        <v>96</v>
-      </c>
-      <c r="U18" t="s">
-        <v>107</v>
-      </c>
-      <c r="V18" t="s">
-        <v>124</v>
-      </c>
-      <c r="W18" t="s">
-        <v>125</v>
-      </c>
-      <c r="AA18" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:27">
-      <c r="A19">
-        <v>329</v>
-      </c>
-      <c r="B19" t="s">
-        <v>28</v>
-      </c>
-      <c r="C19" t="s">
-        <v>49</v>
-      </c>
-      <c r="D19" t="s">
-        <v>68</v>
-      </c>
-      <c r="E19" t="s">
-        <v>85</v>
-      </c>
-      <c r="F19" t="s">
-        <v>87</v>
-      </c>
-      <c r="G19">
-        <v>2720</v>
-      </c>
-      <c r="H19" t="s">
-        <v>90</v>
-      </c>
-      <c r="I19" t="s">
-        <v>93</v>
-      </c>
-      <c r="J19" s="1">
-        <v>46220</v>
-      </c>
-      <c r="K19" s="1">
-        <v>46225</v>
-      </c>
-      <c r="L19">
-        <v>6</v>
-      </c>
-      <c r="M19" t="s">
-        <v>95</v>
-      </c>
-      <c r="N19" s="1">
-        <v>46256</v>
-      </c>
-      <c r="Q19">
-        <v>-30</v>
-      </c>
-      <c r="R19">
-        <v>1</v>
-      </c>
-      <c r="S19" t="s">
-        <v>97</v>
-      </c>
-      <c r="T19" t="s">
-        <v>96</v>
-      </c>
-      <c r="U19" t="s">
-        <v>107</v>
-      </c>
-      <c r="V19" t="s">
-        <v>124</v>
-      </c>
-      <c r="W19" t="s">
-        <v>125</v>
-      </c>
-      <c r="AA19" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:27">
-      <c r="A20">
-        <v>329</v>
-      </c>
-      <c r="B20" t="s">
-        <v>28</v>
-      </c>
-      <c r="C20" t="s">
-        <v>50</v>
-      </c>
-      <c r="D20" t="s">
-        <v>69</v>
-      </c>
-      <c r="E20" t="s">
-        <v>86</v>
-      </c>
-      <c r="F20" t="s">
-        <v>89</v>
-      </c>
-      <c r="G20">
-        <v>2721</v>
-      </c>
-      <c r="H20" t="s">
-        <v>90</v>
-      </c>
-      <c r="I20" t="s">
-        <v>94</v>
-      </c>
-      <c r="J20" s="1">
-        <v>46225</v>
-      </c>
-      <c r="K20" s="1">
-        <v>46226</v>
-      </c>
-      <c r="L20">
-        <v>1</v>
-      </c>
-      <c r="M20" t="s">
-        <v>95</v>
-      </c>
-      <c r="N20" s="1">
-        <v>46233</v>
-      </c>
-      <c r="Q20">
-        <v>-7</v>
-      </c>
-      <c r="R20">
-        <v>0</v>
-      </c>
-      <c r="S20" t="s">
-        <v>96</v>
-      </c>
-      <c r="T20" t="s">
-        <v>96</v>
-      </c>
-      <c r="W20" t="s">
-        <v>125</v>
-      </c>
-      <c r="AA20" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (25/07/2026 03:07)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -782,10 +782,10 @@
         <v>46287</v>
       </c>
       <c r="Q2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="R2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="S2" t="s">
         <v>78</v>
@@ -850,10 +850,10 @@
         <v>46216</v>
       </c>
       <c r="Q3">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R3">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="S3" t="s">
         <v>78</v>
@@ -921,10 +921,10 @@
         <v>46238</v>
       </c>
       <c r="Q4">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="R4">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="S4" t="s">
         <v>78</v>
@@ -986,10 +986,10 @@
         <v>46237</v>
       </c>
       <c r="Q5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R5">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S5" t="s">
         <v>78</v>
@@ -1054,10 +1054,10 @@
         <v>46243</v>
       </c>
       <c r="Q6">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="R6">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S6" t="s">
         <v>78</v>
@@ -1119,10 +1119,10 @@
         <v>46248</v>
       </c>
       <c r="Q7">
-        <v>-21</v>
+        <v>-20</v>
       </c>
       <c r="R7">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S7" t="s">
         <v>78</v>
@@ -1181,10 +1181,10 @@
         <v>46249</v>
       </c>
       <c r="Q8">
-        <v>-22</v>
+        <v>-21</v>
       </c>
       <c r="R8">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="S8" t="s">
         <v>78</v>
@@ -1252,10 +1252,10 @@
         <v>46227</v>
       </c>
       <c r="Q9">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S9" t="s">
         <v>78</v>
@@ -1317,10 +1317,10 @@
         <v>46251</v>
       </c>
       <c r="Q10">
-        <v>-24</v>
+        <v>-23</v>
       </c>
       <c r="R10">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S10" t="s">
         <v>79</v>
@@ -1382,10 +1382,10 @@
         <v>46232</v>
       </c>
       <c r="Q11">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R11">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S11" t="s">
         <v>78</v>
@@ -1450,10 +1450,10 @@
         <v>46228</v>
       </c>
       <c r="Q12">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R12">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S12" t="s">
         <v>78</v>
@@ -1518,10 +1518,10 @@
         <v>46229</v>
       </c>
       <c r="Q13">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S13" t="s">
         <v>78</v>
@@ -1583,10 +1583,10 @@
         <v>46254</v>
       </c>
       <c r="Q14">
-        <v>-27</v>
+        <v>-26</v>
       </c>
       <c r="R14">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S14" t="s">
         <v>78</v>

</xml_diff>

<commit_message>
Atualização manual: emergencias (27/07/2026) — recalcula Cômputo Mensal até hoje
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -295,7 +295,7 @@
     <t>Item em bancada porem em pessimo estado, foi solicitado recolhimento de mais unidades para envio a oficina para tentativa de reparo ATZ Marcio 17/7/26. Solicitado abertura de O.S. para 3EA do item no dia 16-07-26 via Email para a Coordenadoria - CLA-21-07-26</t>
   </si>
   <si>
-    <t>Nao temos oficina no Brasil para reparo desse item, temos que iniciar processo de aquisiçáo do material para atendimento a essa necessidade ATZ Marcio 17/7/26 - Efetuada compra em AOG , aguardando o AWB de envio para Natal, peça saindo do Espirito Santo ATZ Marcio 20/7 15:54 - AWB 12748559512 DPE 24/07/2026</t>
+    <t>Nao temos oficina no Brasil para reparo desse item, temos que iniciar processo de aquisiçáo do material para atendimento a essa necessidade ATZ Marcio 17/7/26 - Efetuada compra em AOG , aguardando o AWB de envio para Natal, peça saindo do Espirito Santo ATZ Marcio 20/7 15:54 - AWB 12748559512 DPE 24/07/2026 - material entregue dia 24/07/2026 - recibo assinado no drive</t>
   </si>
   <si>
     <t>Será atendido via estoque TSAU. ATZ 23/07. Foi solicitado o atendimento com estoque FAB -CLA -dia 23-07</t>
@@ -323,8 +323,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -340,7 +348,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -348,12 +356,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -653,85 +679,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -763,10 +789,10 @@
       <c r="I2" t="s">
         <v>74</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>46076</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46080</v>
       </c>
       <c r="L2">
@@ -775,17 +801,17 @@
       <c r="M2" t="s">
         <v>77</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <v>46091</v>
       </c>
-      <c r="O2" s="1">
+      <c r="O2" s="2">
         <v>46287</v>
       </c>
       <c r="Q2">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="R2">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="S2" t="s">
         <v>78</v>
@@ -831,10 +857,10 @@
       <c r="I3" t="s">
         <v>75</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>46209</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46210</v>
       </c>
       <c r="L3">
@@ -843,17 +869,17 @@
       <c r="M3" t="s">
         <v>77</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <v>46217</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46216</v>
       </c>
       <c r="Q3">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="R3">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="S3" t="s">
         <v>78</v>
@@ -902,10 +928,10 @@
       <c r="I4" t="s">
         <v>76</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>46210</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46210</v>
       </c>
       <c r="L4">
@@ -914,17 +940,17 @@
       <c r="M4" t="s">
         <v>77</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="2">
         <v>46241</v>
       </c>
-      <c r="O4" s="1">
+      <c r="O4" s="2">
         <v>46238</v>
       </c>
       <c r="Q4">
-        <v>-13</v>
+        <v>-11</v>
       </c>
       <c r="R4">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="S4" t="s">
         <v>78</v>
@@ -967,10 +993,10 @@
       <c r="I5" t="s">
         <v>75</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>46211</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46212</v>
       </c>
       <c r="L5">
@@ -979,17 +1005,17 @@
       <c r="M5" t="s">
         <v>77</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <v>46219</v>
       </c>
-      <c r="O5" s="1">
+      <c r="O5" s="2">
         <v>46237</v>
       </c>
       <c r="Q5">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="R5">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="S5" t="s">
         <v>78</v>
@@ -1038,10 +1064,10 @@
       <c r="I6" t="s">
         <v>76</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>46212</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46212</v>
       </c>
       <c r="L6">
@@ -1050,14 +1076,14 @@
       <c r="M6" t="s">
         <v>77</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <v>46243</v>
       </c>
       <c r="Q6">
-        <v>-15</v>
+        <v>-13</v>
       </c>
       <c r="R6">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="S6" t="s">
         <v>78</v>
@@ -1100,10 +1126,10 @@
       <c r="I7" t="s">
         <v>76</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46216</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46217</v>
       </c>
       <c r="L7">
@@ -1112,17 +1138,17 @@
       <c r="M7" t="s">
         <v>77</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="2">
         <v>46248</v>
       </c>
-      <c r="O7" s="1">
+      <c r="O7" s="2">
         <v>46248</v>
       </c>
       <c r="Q7">
-        <v>-20</v>
+        <v>-18</v>
       </c>
       <c r="R7">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="S7" t="s">
         <v>78</v>
@@ -1165,10 +1191,10 @@
       <c r="I8" t="s">
         <v>76</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46219</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46218</v>
       </c>
       <c r="L8">
@@ -1177,14 +1203,14 @@
       <c r="M8" t="s">
         <v>77</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="2">
         <v>46249</v>
       </c>
       <c r="Q8">
-        <v>-21</v>
+        <v>-19</v>
       </c>
       <c r="R8">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="S8" t="s">
         <v>78</v>
@@ -1233,10 +1259,10 @@
       <c r="I9" t="s">
         <v>74</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46219</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46219</v>
       </c>
       <c r="L9">
@@ -1245,17 +1271,17 @@
       <c r="M9" t="s">
         <v>77</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>46230</v>
       </c>
-      <c r="O9" s="1">
+      <c r="O9" s="2">
         <v>46227</v>
       </c>
       <c r="Q9">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="R9">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="S9" t="s">
         <v>78</v>
@@ -1301,10 +1327,10 @@
       <c r="I10" t="s">
         <v>76</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46219</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>46220</v>
       </c>
       <c r="L10">
@@ -1313,14 +1339,14 @@
       <c r="M10" t="s">
         <v>77</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
         <v>46251</v>
       </c>
       <c r="Q10">
-        <v>-23</v>
+        <v>-21</v>
       </c>
       <c r="R10">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="S10" t="s">
         <v>79</v>
@@ -1366,10 +1392,10 @@
       <c r="I11" t="s">
         <v>74</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46219</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>46221</v>
       </c>
       <c r="L11">
@@ -1378,14 +1404,14 @@
       <c r="M11" t="s">
         <v>77</v>
       </c>
-      <c r="N11" s="1">
+      <c r="N11" s="2">
         <v>46232</v>
       </c>
       <c r="Q11">
-        <v>-4</v>
+        <v>-2</v>
       </c>
       <c r="R11">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="S11" t="s">
         <v>78</v>
@@ -1431,10 +1457,10 @@
       <c r="I12" t="s">
         <v>74</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>46220</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>46221</v>
       </c>
       <c r="L12">
@@ -1443,17 +1469,17 @@
       <c r="M12" t="s">
         <v>77</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="2">
         <v>46232</v>
       </c>
-      <c r="O12" s="1">
+      <c r="O12" s="2">
         <v>46228</v>
       </c>
       <c r="Q12">
-        <v>-4</v>
+        <v>-2</v>
       </c>
       <c r="R12">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="S12" t="s">
         <v>78</v>
@@ -1502,10 +1528,10 @@
       <c r="I13" t="s">
         <v>75</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46224</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>46222</v>
       </c>
       <c r="L13">
@@ -1514,14 +1540,14 @@
       <c r="M13" t="s">
         <v>77</v>
       </c>
-      <c r="N13" s="1">
+      <c r="N13" s="2">
         <v>46229</v>
       </c>
       <c r="Q13">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="R13">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S13" t="s">
         <v>78</v>
@@ -1567,10 +1593,10 @@
       <c r="I14" t="s">
         <v>76</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46220</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>46223</v>
       </c>
       <c r="L14">
@@ -1579,14 +1605,14 @@
       <c r="M14" t="s">
         <v>77</v>
       </c>
-      <c r="N14" s="1">
+      <c r="N14" s="2">
         <v>46254</v>
       </c>
       <c r="Q14">
-        <v>-26</v>
+        <v>-24</v>
       </c>
       <c r="R14">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="S14" t="s">
         <v>78</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (27/07/2026 14:22)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="102">
   <si>
     <t>om_emg</t>
   </si>
@@ -268,10 +268,16 @@
     <t>Alterado o tipo da emerg. de IPLR para ANCE. Godoy 22/07/26</t>
   </si>
   <si>
+    <t>AWB 127-4855 9512 retirado por Teodoro em 24/07/2026</t>
+  </si>
+  <si>
     <t>Será atendido com o estoque FAB pedido 17963489. Godoy 23/07/2026</t>
   </si>
   <si>
     <t>Cedeu o item para o C-98 2737. Godoy 21/07/26.</t>
+  </si>
+  <si>
+    <t>AWB 127-4858 1702 - REZ -22/07/26</t>
   </si>
   <si>
     <t>Foi solicitado via email no dia 02-03-2 o atendimento do item com estoque FAB. Claudio -02-03-26 - Em resposta, a coordenadoria disse que o estque seria insuficiente. Foi verificado que na T.O da ANV o QPA para esse item são 2 EA, solicitei confirmação. - Cláudio -02-03-2026. Solicitado o cancelamento da emergência em função da quantidade cedida ao 2733 ter sido de 01ea. Considerando o QPA 02 ea. Encontra-se em tratativa junto a fiscalização e o gestor do contrato conforme mensagem de e-mail de 05/03. - SOLICITAÇÃO E-C98-26047.Colocado pedido AOG Textron WB0003068789 - previsão de entrega 60 dias em média. Os demais fornecedores informaram não ter em estoque ou não possuírem a certificação necessária da peça.</t>
@@ -323,16 +329,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -348,7 +346,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -356,30 +354,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -679,85 +659,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -789,10 +769,10 @@
       <c r="I2" t="s">
         <v>74</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>46076</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46080</v>
       </c>
       <c r="L2">
@@ -801,10 +781,10 @@
       <c r="M2" t="s">
         <v>77</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="1">
         <v>46091</v>
       </c>
-      <c r="O2" s="2">
+      <c r="O2" s="1">
         <v>46287</v>
       </c>
       <c r="Q2">
@@ -820,10 +800,10 @@
         <v>80</v>
       </c>
       <c r="V2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="W2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -857,10 +837,10 @@
       <c r="I3" t="s">
         <v>75</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>46209</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46210</v>
       </c>
       <c r="L3">
@@ -869,10 +849,10 @@
       <c r="M3" t="s">
         <v>77</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="1">
         <v>46217</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46216</v>
       </c>
       <c r="Q3">
@@ -891,10 +871,10 @@
         <v>81</v>
       </c>
       <c r="V3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="W3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -928,10 +908,10 @@
       <c r="I4" t="s">
         <v>76</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>46210</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46210</v>
       </c>
       <c r="L4">
@@ -940,10 +920,10 @@
       <c r="M4" t="s">
         <v>77</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="1">
         <v>46241</v>
       </c>
-      <c r="O4" s="2">
+      <c r="O4" s="1">
         <v>46238</v>
       </c>
       <c r="Q4">
@@ -956,10 +936,10 @@
         <v>78</v>
       </c>
       <c r="V4" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="W4" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -993,10 +973,10 @@
       <c r="I5" t="s">
         <v>75</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>46211</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46212</v>
       </c>
       <c r="L5">
@@ -1005,10 +985,10 @@
       <c r="M5" t="s">
         <v>77</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="1">
         <v>46219</v>
       </c>
-      <c r="O5" s="2">
+      <c r="O5" s="1">
         <v>46237</v>
       </c>
       <c r="Q5">
@@ -1027,10 +1007,10 @@
         <v>82</v>
       </c>
       <c r="V5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="W5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1064,10 +1044,10 @@
       <c r="I6" t="s">
         <v>76</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>46212</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46212</v>
       </c>
       <c r="L6">
@@ -1076,7 +1056,7 @@
       <c r="M6" t="s">
         <v>77</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="1">
         <v>46243</v>
       </c>
       <c r="Q6">
@@ -1089,10 +1069,10 @@
         <v>78</v>
       </c>
       <c r="V6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="W6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1126,10 +1106,10 @@
       <c r="I7" t="s">
         <v>76</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46216</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>46217</v>
       </c>
       <c r="L7">
@@ -1138,10 +1118,10 @@
       <c r="M7" t="s">
         <v>77</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="1">
         <v>46248</v>
       </c>
-      <c r="O7" s="2">
+      <c r="O7" s="1">
         <v>46248</v>
       </c>
       <c r="Q7">
@@ -1154,10 +1134,10 @@
         <v>78</v>
       </c>
       <c r="V7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="W7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1191,10 +1171,10 @@
       <c r="I8" t="s">
         <v>76</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46219</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>46218</v>
       </c>
       <c r="L8">
@@ -1203,7 +1183,7 @@
       <c r="M8" t="s">
         <v>77</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="1">
         <v>46249</v>
       </c>
       <c r="Q8">
@@ -1222,10 +1202,10 @@
         <v>83</v>
       </c>
       <c r="V8" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="W8" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1259,10 +1239,10 @@
       <c r="I9" t="s">
         <v>74</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46219</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>46219</v>
       </c>
       <c r="L9">
@@ -1271,10 +1251,10 @@
       <c r="M9" t="s">
         <v>77</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="1">
         <v>46230</v>
       </c>
-      <c r="O9" s="2">
+      <c r="O9" s="1">
         <v>46227</v>
       </c>
       <c r="Q9">
@@ -1289,11 +1269,14 @@
       <c r="T9" t="s">
         <v>79</v>
       </c>
+      <c r="U9" t="s">
+        <v>84</v>
+      </c>
       <c r="V9" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="W9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1327,10 +1310,10 @@
       <c r="I10" t="s">
         <v>76</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>46219</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>46220</v>
       </c>
       <c r="L10">
@@ -1339,7 +1322,7 @@
       <c r="M10" t="s">
         <v>77</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="1">
         <v>46251</v>
       </c>
       <c r="Q10">
@@ -1352,13 +1335,13 @@
         <v>79</v>
       </c>
       <c r="U10" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="V10" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="W10" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1392,10 +1375,10 @@
       <c r="I11" t="s">
         <v>74</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46219</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>46221</v>
       </c>
       <c r="L11">
@@ -1404,7 +1387,7 @@
       <c r="M11" t="s">
         <v>77</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11" s="1">
         <v>46232</v>
       </c>
       <c r="Q11">
@@ -1420,10 +1403,10 @@
         <v>79</v>
       </c>
       <c r="V11" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="W11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1457,10 +1440,10 @@
       <c r="I12" t="s">
         <v>74</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>46220</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>46221</v>
       </c>
       <c r="L12">
@@ -1469,10 +1452,10 @@
       <c r="M12" t="s">
         <v>77</v>
       </c>
-      <c r="N12" s="2">
+      <c r="N12" s="1">
         <v>46232</v>
       </c>
-      <c r="O12" s="2">
+      <c r="O12" s="1">
         <v>46228</v>
       </c>
       <c r="Q12">
@@ -1488,13 +1471,13 @@
         <v>79</v>
       </c>
       <c r="U12" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="V12" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="W12" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1528,10 +1511,10 @@
       <c r="I13" t="s">
         <v>75</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46224</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>46222</v>
       </c>
       <c r="L13">
@@ -1540,7 +1523,7 @@
       <c r="M13" t="s">
         <v>77</v>
       </c>
-      <c r="N13" s="2">
+      <c r="N13" s="1">
         <v>46229</v>
       </c>
       <c r="Q13">
@@ -1555,11 +1538,14 @@
       <c r="T13" t="s">
         <v>79</v>
       </c>
+      <c r="U13" t="s">
+        <v>87</v>
+      </c>
       <c r="V13" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="W13" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1593,10 +1579,10 @@
       <c r="I14" t="s">
         <v>76</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46220</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>46223</v>
       </c>
       <c r="L14">
@@ -1605,7 +1591,7 @@
       <c r="M14" t="s">
         <v>77</v>
       </c>
-      <c r="N14" s="2">
+      <c r="N14" s="1">
         <v>46254</v>
       </c>
       <c r="Q14">
@@ -1621,10 +1607,10 @@
         <v>78</v>
       </c>
       <c r="V14" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="W14" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (27/07/2026 19:41)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="82">
   <si>
     <t>om_emg</t>
   </si>
@@ -106,21 +106,12 @@
     <t>BANT</t>
   </si>
   <si>
-    <t>CLA</t>
-  </si>
-  <si>
     <t>313260017747</t>
   </si>
   <si>
     <t>329260019181</t>
   </si>
   <si>
-    <t>685260012303</t>
-  </si>
-  <si>
-    <t>419260000557</t>
-  </si>
-  <si>
     <t>685260012350</t>
   </si>
   <si>
@@ -130,15 +121,9 @@
     <t>685260012387</t>
   </si>
   <si>
-    <t>685260012394</t>
-  </si>
-  <si>
     <t>685260012395</t>
   </si>
   <si>
-    <t>685260012396</t>
-  </si>
-  <si>
     <t>313260018675</t>
   </si>
   <si>
@@ -154,12 +139,6 @@
     <t>C145-00-46</t>
   </si>
   <si>
-    <t>065-0065-01</t>
-  </si>
-  <si>
-    <t>3244897-4</t>
-  </si>
-  <si>
     <t>030-1094-58</t>
   </si>
   <si>
@@ -169,15 +148,9 @@
     <t>066-3084-32</t>
   </si>
   <si>
-    <t>3011755</t>
-  </si>
-  <si>
     <t>2611024-1</t>
   </si>
   <si>
-    <t>540-1407-4</t>
-  </si>
-  <si>
     <t>011-00870-00</t>
   </si>
   <si>
@@ -193,27 +166,15 @@
     <t>TRANSMISSION ASSY</t>
   </si>
   <si>
-    <t>SELECTOR ALT</t>
-  </si>
-  <si>
-    <t>FUEL CONTROL UNIT</t>
-  </si>
-  <si>
     <t>CONNECTOR</t>
   </si>
   <si>
     <t>IND RDR 2000 IN-182A</t>
   </si>
   <si>
-    <t>INSULATION BLANKET,T</t>
-  </si>
-  <si>
     <t>WINDOW</t>
   </si>
   <si>
-    <t>VALVE,BLEED,TURBINEE</t>
-  </si>
-  <si>
     <t>MAGNETOMETER GMU 44</t>
   </si>
   <si>
@@ -226,9 +187,6 @@
     <t>C</t>
   </si>
   <si>
-    <t>T</t>
-  </si>
-  <si>
     <t>R</t>
   </si>
   <si>
@@ -262,15 +220,9 @@
     <t>Vee One tem alguma atualização do DPE ?. Godoy 23/07/26</t>
   </si>
   <si>
-    <t>AWB 12747899051 volume retirado na loja GOLLOG - BEL por marlos em 20/07. Godoy 22/07/2026.</t>
-  </si>
-  <si>
     <t>Alterado o tipo da emerg. de IPLR para ANCE. Godoy 22/07/26</t>
   </si>
   <si>
-    <t>AWB 127-4855 9512 retirado por Teodoro em 24/07/2026</t>
-  </si>
-  <si>
     <t>Será atendido com o estoque FAB pedido 17963489. Godoy 23/07/2026</t>
   </si>
   <si>
@@ -286,12 +238,6 @@
     <t>Colocado pedido AOG Textron IJ17557538 - previsão de entrega em Miami 08/07. Previsão de chegada GIG 09/07 - MATERIAL EM TRANSITO - RECIBO 551/FAB/26 - ENVIADO PN COMPLETO PARA SANAR A EMERGENCIA DO 2709, ENVIADO MODAL TERRESTRE, DPE 13/07/2026</t>
   </si>
   <si>
-    <t>confirmado entrega 01 ea hj(21/07/26) pela William - REZ - item aguardando minuta e nota para transporte CLA-23-07</t>
-  </si>
-  <si>
-    <t>Aguardando o retorno dos subcomponentes removidos da unidade para ser enviado a oficiana para aplicação na unidade Prazo apos aprovação 10 dias ATZ Marcio 9/7/26 14 53 - Enviado uma FCU em 17/7 fornecida pela FAB , ATZ Macio, Aguardando a atualização com o recibo e AWB ATZ Marcio 20/7 - FCU ENVIADA FOI RECUSADA PELA INSPETORIA DE RECEBIMENTO DA BABE - 20/07/2026 RC - ITEM ATENDIDO COM ESTOQUE FAB AWB 127-4789 9051</t>
-  </si>
-  <si>
     <t>Colocado pedido junto ao fornecedor LEGACY PARTS, validando prazo de entrega em Miami. ATZ 23/07</t>
   </si>
   <si>
@@ -301,13 +247,7 @@
     <t>Item em bancada porem em pessimo estado, foi solicitado recolhimento de mais unidades para envio a oficina para tentativa de reparo ATZ Marcio 17/7/26. Solicitado abertura de O.S. para 3EA do item no dia 16-07-26 via Email para a Coordenadoria - CLA-21-07-26</t>
   </si>
   <si>
-    <t>Nao temos oficina no Brasil para reparo desse item, temos que iniciar processo de aquisiçáo do material para atendimento a essa necessidade ATZ Marcio 17/7/26 - Efetuada compra em AOG , aguardando o AWB de envio para Natal, peça saindo do Espirito Santo ATZ Marcio 20/7 15:54 - AWB 12748559512 DPE 24/07/2026 - material entregue dia 24/07/2026 - recibo assinado no drive</t>
-  </si>
-  <si>
     <t>Será atendido via estoque TSAU. ATZ 23/07. Foi solicitado o atendimento com estoque FAB -CLA -dia 23-07</t>
-  </si>
-  <si>
-    <t>Consta 1 each em condição de uso em MANAUS, Enviado 1 unidade (CORE) para reparo na oficina no RJ em 17/7, orçamento aprovado em 21/7 com DPE de 5 dias (27/7) para entrega na V1 JPA, ATZ Marcio 21/7</t>
   </si>
   <si>
     <t>material enviado com STK FAB - AWB 12748581702 - DPE 25/07/2026 - atz rc 22/07/2026- Enviado para o Operador dia 21/07/26 - AWB 127-4857 9742- REZ -22/07/26</t>
@@ -655,7 +595,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA14"/>
+  <dimension ref="A1:AA10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -749,25 +689,25 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D2" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="E2" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="F2" t="s">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="G2">
         <v>2730</v>
       </c>
       <c r="H2" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="I2" t="s">
-        <v>74</v>
+        <v>60</v>
       </c>
       <c r="J2" s="1">
         <v>46076</v>
@@ -779,7 +719,7 @@
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="N2" s="1">
         <v>46091</v>
@@ -794,16 +734,16 @@
         <v>150</v>
       </c>
       <c r="S2" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="U2" t="s">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="V2" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="W2" t="s">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -817,25 +757,25 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D3" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="E3" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="F3" t="s">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="G3">
         <v>2721</v>
       </c>
       <c r="H3" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="I3" t="s">
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="J3" s="1">
         <v>46209</v>
@@ -847,7 +787,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="N3" s="1">
         <v>46217</v>
@@ -862,19 +802,19 @@
         <v>20</v>
       </c>
       <c r="S3" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="T3" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="U3" t="s">
+        <v>67</v>
+      </c>
+      <c r="V3" t="s">
+        <v>73</v>
+      </c>
+      <c r="W3" t="s">
         <v>81</v>
-      </c>
-      <c r="V3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W3" t="s">
-        <v>101</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -888,58 +828,55 @@
         <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D4" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E4" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="F4" t="s">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="G4">
-        <v>2719</v>
+        <v>2702</v>
       </c>
       <c r="H4" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="I4" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="J4" s="1">
-        <v>46210</v>
+        <v>46212</v>
       </c>
       <c r="K4" s="1">
-        <v>46210</v>
+        <v>46212</v>
       </c>
       <c r="L4">
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="N4" s="1">
-        <v>46241</v>
-      </c>
-      <c r="O4" s="1">
-        <v>46238</v>
+        <v>46243</v>
       </c>
       <c r="Q4">
-        <v>-11</v>
+        <v>-13</v>
       </c>
       <c r="R4">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="S4" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="V4" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="W4" t="s">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -947,70 +884,64 @@
     </row>
     <row r="5" spans="1:27">
       <c r="A5">
-        <v>419</v>
+        <v>313</v>
       </c>
       <c r="B5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D5" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="E5" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F5" t="s">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="G5">
-        <v>2723</v>
+        <v>2736</v>
       </c>
       <c r="H5" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="I5" t="s">
+        <v>62</v>
+      </c>
+      <c r="J5" s="1">
+        <v>46216</v>
+      </c>
+      <c r="K5" s="1">
+        <v>46217</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5" t="s">
+        <v>63</v>
+      </c>
+      <c r="N5" s="1">
+        <v>46248</v>
+      </c>
+      <c r="O5" s="1">
+        <v>46248</v>
+      </c>
+      <c r="Q5">
+        <v>-18</v>
+      </c>
+      <c r="R5">
+        <v>13</v>
+      </c>
+      <c r="S5" t="s">
+        <v>64</v>
+      </c>
+      <c r="V5" t="s">
         <v>75</v>
       </c>
-      <c r="J5" s="1">
-        <v>46211</v>
-      </c>
-      <c r="K5" s="1">
-        <v>46212</v>
-      </c>
-      <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5" t="s">
-        <v>77</v>
-      </c>
-      <c r="N5" s="1">
-        <v>46219</v>
-      </c>
-      <c r="O5" s="1">
-        <v>46237</v>
-      </c>
-      <c r="Q5">
-        <v>11</v>
-      </c>
-      <c r="R5">
-        <v>18</v>
-      </c>
-      <c r="S5" t="s">
-        <v>78</v>
-      </c>
-      <c r="T5" t="s">
-        <v>78</v>
-      </c>
-      <c r="U5" t="s">
-        <v>82</v>
-      </c>
-      <c r="V5" t="s">
-        <v>91</v>
-      </c>
       <c r="W5" t="s">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1024,55 +955,61 @@
         <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="E6" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="F6" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="G6">
-        <v>2702</v>
+        <v>2722</v>
       </c>
       <c r="H6" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="I6" t="s">
+        <v>62</v>
+      </c>
+      <c r="J6" s="1">
+        <v>46219</v>
+      </c>
+      <c r="K6" s="1">
+        <v>46218</v>
+      </c>
+      <c r="L6">
+        <v>1</v>
+      </c>
+      <c r="M6" t="s">
+        <v>63</v>
+      </c>
+      <c r="N6" s="1">
+        <v>46249</v>
+      </c>
+      <c r="Q6">
+        <v>-19</v>
+      </c>
+      <c r="R6">
+        <v>12</v>
+      </c>
+      <c r="S6" t="s">
+        <v>64</v>
+      </c>
+      <c r="T6" t="s">
+        <v>65</v>
+      </c>
+      <c r="U6" t="s">
+        <v>68</v>
+      </c>
+      <c r="V6" t="s">
         <v>76</v>
       </c>
-      <c r="J6" s="1">
-        <v>46212</v>
-      </c>
-      <c r="K6" s="1">
-        <v>46212</v>
-      </c>
-      <c r="L6">
-        <v>1</v>
-      </c>
-      <c r="M6" t="s">
-        <v>77</v>
-      </c>
-      <c r="N6" s="1">
-        <v>46243</v>
-      </c>
-      <c r="Q6">
-        <v>-13</v>
-      </c>
-      <c r="R6">
-        <v>18</v>
-      </c>
-      <c r="S6" t="s">
-        <v>78</v>
-      </c>
-      <c r="V6" t="s">
-        <v>92</v>
-      </c>
       <c r="W6" t="s">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1080,64 +1017,64 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D7" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E7" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="F7" t="s">
+        <v>56</v>
+      </c>
+      <c r="G7">
+        <v>2703</v>
+      </c>
+      <c r="H7" t="s">
+        <v>59</v>
+      </c>
+      <c r="I7" t="s">
+        <v>62</v>
+      </c>
+      <c r="J7" s="1">
+        <v>46219</v>
+      </c>
+      <c r="K7" s="1">
+        <v>46220</v>
+      </c>
+      <c r="L7">
+        <v>2</v>
+      </c>
+      <c r="M7" t="s">
+        <v>63</v>
+      </c>
+      <c r="N7" s="1">
+        <v>46251</v>
+      </c>
+      <c r="Q7">
+        <v>-21</v>
+      </c>
+      <c r="R7">
+        <v>10</v>
+      </c>
+      <c r="S7" t="s">
+        <v>65</v>
+      </c>
+      <c r="U7" t="s">
         <v>69</v>
       </c>
-      <c r="G7">
-        <v>2736</v>
-      </c>
-      <c r="H7" t="s">
-        <v>72</v>
-      </c>
-      <c r="I7" t="s">
-        <v>76</v>
-      </c>
-      <c r="J7" s="1">
-        <v>46216</v>
-      </c>
-      <c r="K7" s="1">
-        <v>46217</v>
-      </c>
-      <c r="L7">
-        <v>1</v>
-      </c>
-      <c r="M7" t="s">
+      <c r="V7" t="s">
         <v>77</v>
       </c>
-      <c r="N7" s="1">
-        <v>46248</v>
-      </c>
-      <c r="O7" s="1">
-        <v>46248</v>
-      </c>
-      <c r="Q7">
-        <v>-18</v>
-      </c>
-      <c r="R7">
-        <v>13</v>
-      </c>
-      <c r="S7" t="s">
-        <v>78</v>
-      </c>
-      <c r="V7" t="s">
-        <v>93</v>
-      </c>
       <c r="W7" t="s">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1145,67 +1082,70 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B8" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D8" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="E8" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="F8" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="G8">
-        <v>2722</v>
+        <v>2730</v>
       </c>
       <c r="H8" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="I8" t="s">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="J8" s="1">
-        <v>46219</v>
+        <v>46220</v>
       </c>
       <c r="K8" s="1">
-        <v>46218</v>
+        <v>46221</v>
       </c>
       <c r="L8">
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="N8" s="1">
-        <v>46249</v>
+        <v>46232</v>
+      </c>
+      <c r="O8" s="1">
+        <v>46228</v>
       </c>
       <c r="Q8">
-        <v>-19</v>
+        <v>-2</v>
       </c>
       <c r="R8">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="S8" t="s">
+        <v>64</v>
+      </c>
+      <c r="T8" t="s">
+        <v>65</v>
+      </c>
+      <c r="U8" t="s">
+        <v>70</v>
+      </c>
+      <c r="V8" t="s">
         <v>78</v>
       </c>
-      <c r="T8" t="s">
-        <v>79</v>
-      </c>
-      <c r="U8" t="s">
-        <v>83</v>
-      </c>
-      <c r="V8" t="s">
-        <v>94</v>
-      </c>
       <c r="W8" t="s">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1213,70 +1153,67 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D9" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="E9" t="s">
+        <v>54</v>
+      </c>
+      <c r="F9" t="s">
+        <v>57</v>
+      </c>
+      <c r="G9">
+        <v>2741</v>
+      </c>
+      <c r="H9" t="s">
+        <v>58</v>
+      </c>
+      <c r="I9" t="s">
+        <v>61</v>
+      </c>
+      <c r="J9" s="1">
+        <v>46224</v>
+      </c>
+      <c r="K9" s="1">
+        <v>46222</v>
+      </c>
+      <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9" t="s">
         <v>63</v>
       </c>
-      <c r="F9" t="s">
-        <v>70</v>
-      </c>
-      <c r="G9">
-        <v>2729</v>
-      </c>
-      <c r="H9" t="s">
-        <v>72</v>
-      </c>
-      <c r="I9" t="s">
-        <v>74</v>
-      </c>
-      <c r="J9" s="1">
-        <v>46219</v>
-      </c>
-      <c r="K9" s="1">
-        <v>46219</v>
-      </c>
-      <c r="L9">
-        <v>1</v>
-      </c>
-      <c r="M9" t="s">
-        <v>77</v>
-      </c>
       <c r="N9" s="1">
-        <v>46230</v>
-      </c>
-      <c r="O9" s="1">
-        <v>46227</v>
+        <v>46229</v>
       </c>
       <c r="Q9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R9">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="S9" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="T9" t="s">
+        <v>65</v>
+      </c>
+      <c r="U9" t="s">
+        <v>71</v>
+      </c>
+      <c r="V9" t="s">
         <v>79</v>
       </c>
-      <c r="U9" t="s">
-        <v>84</v>
-      </c>
-      <c r="V9" t="s">
-        <v>95</v>
-      </c>
       <c r="W9" t="s">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1284,335 +1221,66 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>685</v>
+        <v>329</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D10" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="E10" t="s">
+        <v>55</v>
+      </c>
+      <c r="F10" t="s">
+        <v>56</v>
+      </c>
+      <c r="G10">
+        <v>2720</v>
+      </c>
+      <c r="H10" t="s">
+        <v>58</v>
+      </c>
+      <c r="I10" t="s">
+        <v>62</v>
+      </c>
+      <c r="J10" s="1">
+        <v>46220</v>
+      </c>
+      <c r="K10" s="1">
+        <v>46223</v>
+      </c>
+      <c r="L10">
+        <v>10</v>
+      </c>
+      <c r="M10" t="s">
+        <v>63</v>
+      </c>
+      <c r="N10" s="1">
+        <v>46254</v>
+      </c>
+      <c r="Q10">
+        <v>-24</v>
+      </c>
+      <c r="R10">
+        <v>7</v>
+      </c>
+      <c r="S10" t="s">
         <v>64</v>
       </c>
-      <c r="F10" t="s">
-        <v>69</v>
-      </c>
-      <c r="G10">
-        <v>2703</v>
-      </c>
-      <c r="H10" t="s">
-        <v>73</v>
-      </c>
-      <c r="I10" t="s">
-        <v>76</v>
-      </c>
-      <c r="J10" s="1">
-        <v>46219</v>
-      </c>
-      <c r="K10" s="1">
-        <v>46220</v>
-      </c>
-      <c r="L10">
-        <v>2</v>
-      </c>
-      <c r="M10" t="s">
-        <v>77</v>
-      </c>
-      <c r="N10" s="1">
-        <v>46251</v>
-      </c>
-      <c r="Q10">
-        <v>-21</v>
-      </c>
-      <c r="R10">
-        <v>10</v>
-      </c>
-      <c r="S10" t="s">
-        <v>79</v>
-      </c>
-      <c r="U10" t="s">
-        <v>85</v>
+      <c r="T10" t="s">
+        <v>64</v>
       </c>
       <c r="V10" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="W10" t="s">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="AA10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:27">
-      <c r="A11">
-        <v>685</v>
-      </c>
-      <c r="B11" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" t="s">
-        <v>40</v>
-      </c>
-      <c r="D11" t="s">
-        <v>53</v>
-      </c>
-      <c r="E11" t="s">
-        <v>65</v>
-      </c>
-      <c r="F11" t="s">
-        <v>71</v>
-      </c>
-      <c r="G11">
-        <v>2729</v>
-      </c>
-      <c r="H11" t="s">
-        <v>72</v>
-      </c>
-      <c r="I11" t="s">
-        <v>74</v>
-      </c>
-      <c r="J11" s="1">
-        <v>46219</v>
-      </c>
-      <c r="K11" s="1">
-        <v>46221</v>
-      </c>
-      <c r="L11">
-        <v>1</v>
-      </c>
-      <c r="M11" t="s">
-        <v>77</v>
-      </c>
-      <c r="N11" s="1">
-        <v>46232</v>
-      </c>
-      <c r="Q11">
-        <v>-2</v>
-      </c>
-      <c r="R11">
-        <v>9</v>
-      </c>
-      <c r="S11" t="s">
-        <v>78</v>
-      </c>
-      <c r="T11" t="s">
-        <v>79</v>
-      </c>
-      <c r="V11" t="s">
-        <v>97</v>
-      </c>
-      <c r="W11" t="s">
-        <v>101</v>
-      </c>
-      <c r="AA11" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:27">
-      <c r="A12">
-        <v>313</v>
-      </c>
-      <c r="B12" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" t="s">
-        <v>41</v>
-      </c>
-      <c r="D12" t="s">
-        <v>54</v>
-      </c>
-      <c r="E12" t="s">
-        <v>66</v>
-      </c>
-      <c r="F12" t="s">
-        <v>71</v>
-      </c>
-      <c r="G12">
-        <v>2730</v>
-      </c>
-      <c r="H12" t="s">
-        <v>73</v>
-      </c>
-      <c r="I12" t="s">
-        <v>74</v>
-      </c>
-      <c r="J12" s="1">
-        <v>46220</v>
-      </c>
-      <c r="K12" s="1">
-        <v>46221</v>
-      </c>
-      <c r="L12">
-        <v>1</v>
-      </c>
-      <c r="M12" t="s">
-        <v>77</v>
-      </c>
-      <c r="N12" s="1">
-        <v>46232</v>
-      </c>
-      <c r="O12" s="1">
-        <v>46228</v>
-      </c>
-      <c r="Q12">
-        <v>-2</v>
-      </c>
-      <c r="R12">
-        <v>9</v>
-      </c>
-      <c r="S12" t="s">
-        <v>78</v>
-      </c>
-      <c r="T12" t="s">
-        <v>79</v>
-      </c>
-      <c r="U12" t="s">
-        <v>86</v>
-      </c>
-      <c r="V12" t="s">
-        <v>98</v>
-      </c>
-      <c r="W12" t="s">
-        <v>101</v>
-      </c>
-      <c r="AA12" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:27">
-      <c r="A13">
-        <v>313</v>
-      </c>
-      <c r="B13" t="s">
-        <v>27</v>
-      </c>
-      <c r="C13" t="s">
-        <v>42</v>
-      </c>
-      <c r="D13" t="s">
-        <v>55</v>
-      </c>
-      <c r="E13" t="s">
-        <v>67</v>
-      </c>
-      <c r="F13" t="s">
-        <v>71</v>
-      </c>
-      <c r="G13">
-        <v>2741</v>
-      </c>
-      <c r="H13" t="s">
-        <v>72</v>
-      </c>
-      <c r="I13" t="s">
-        <v>75</v>
-      </c>
-      <c r="J13" s="1">
-        <v>46224</v>
-      </c>
-      <c r="K13" s="1">
-        <v>46222</v>
-      </c>
-      <c r="L13">
-        <v>1</v>
-      </c>
-      <c r="M13" t="s">
-        <v>77</v>
-      </c>
-      <c r="N13" s="1">
-        <v>46229</v>
-      </c>
-      <c r="Q13">
-        <v>1</v>
-      </c>
-      <c r="R13">
-        <v>8</v>
-      </c>
-      <c r="S13" t="s">
-        <v>78</v>
-      </c>
-      <c r="T13" t="s">
-        <v>79</v>
-      </c>
-      <c r="U13" t="s">
-        <v>87</v>
-      </c>
-      <c r="V13" t="s">
-        <v>99</v>
-      </c>
-      <c r="W13" t="s">
-        <v>101</v>
-      </c>
-      <c r="AA13" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:27">
-      <c r="A14">
-        <v>329</v>
-      </c>
-      <c r="B14" t="s">
-        <v>28</v>
-      </c>
-      <c r="C14" t="s">
-        <v>43</v>
-      </c>
-      <c r="D14" t="s">
-        <v>56</v>
-      </c>
-      <c r="E14" t="s">
-        <v>68</v>
-      </c>
-      <c r="F14" t="s">
-        <v>69</v>
-      </c>
-      <c r="G14">
-        <v>2720</v>
-      </c>
-      <c r="H14" t="s">
-        <v>72</v>
-      </c>
-      <c r="I14" t="s">
-        <v>76</v>
-      </c>
-      <c r="J14" s="1">
-        <v>46220</v>
-      </c>
-      <c r="K14" s="1">
-        <v>46223</v>
-      </c>
-      <c r="L14">
-        <v>10</v>
-      </c>
-      <c r="M14" t="s">
-        <v>77</v>
-      </c>
-      <c r="N14" s="1">
-        <v>46254</v>
-      </c>
-      <c r="Q14">
-        <v>-24</v>
-      </c>
-      <c r="R14">
-        <v>7</v>
-      </c>
-      <c r="S14" t="s">
-        <v>78</v>
-      </c>
-      <c r="T14" t="s">
-        <v>78</v>
-      </c>
-      <c r="V14" t="s">
-        <v>100</v>
-      </c>
-      <c r="W14" t="s">
-        <v>101</v>
-      </c>
-      <c r="AA14" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (28/07/2026 05:07)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -728,10 +728,10 @@
         <v>46287</v>
       </c>
       <c r="Q2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="R2">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="S2" t="s">
         <v>64</v>
@@ -796,10 +796,10 @@
         <v>46216</v>
       </c>
       <c r="Q3">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R3">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="S3" t="s">
         <v>64</v>
@@ -864,10 +864,10 @@
         <v>46243</v>
       </c>
       <c r="Q4">
-        <v>-13</v>
+        <v>-12</v>
       </c>
       <c r="R4">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="S4" t="s">
         <v>64</v>
@@ -929,10 +929,10 @@
         <v>46248</v>
       </c>
       <c r="Q5">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="R5">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S5" t="s">
         <v>64</v>
@@ -991,10 +991,10 @@
         <v>46249</v>
       </c>
       <c r="Q6">
-        <v>-19</v>
+        <v>-18</v>
       </c>
       <c r="R6">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S6" t="s">
         <v>64</v>
@@ -1059,10 +1059,10 @@
         <v>46251</v>
       </c>
       <c r="Q7">
-        <v>-21</v>
+        <v>-20</v>
       </c>
       <c r="R7">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S7" t="s">
         <v>65</v>
@@ -1127,10 +1127,10 @@
         <v>46228</v>
       </c>
       <c r="Q8">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R8">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="S8" t="s">
         <v>64</v>
@@ -1195,10 +1195,10 @@
         <v>46229</v>
       </c>
       <c r="Q9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S9" t="s">
         <v>64</v>
@@ -1263,10 +1263,10 @@
         <v>46254</v>
       </c>
       <c r="Q10">
-        <v>-24</v>
+        <v>-23</v>
       </c>
       <c r="R10">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S10" t="s">
         <v>64</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (28/07/2026 13:55)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="70">
   <si>
     <t>om_emg</t>
   </si>
@@ -100,18 +100,15 @@
     <t>BAMN</t>
   </si>
   <si>
+    <t>BANT</t>
+  </si>
+  <si>
     <t>BABR</t>
   </si>
   <si>
-    <t>BANT</t>
-  </si>
-  <si>
     <t>313260017747</t>
   </si>
   <si>
-    <t>329260019181</t>
-  </si>
-  <si>
     <t>685260012350</t>
   </si>
   <si>
@@ -121,24 +118,18 @@
     <t>685260012387</t>
   </si>
   <si>
-    <t>685260012395</t>
-  </si>
-  <si>
     <t>313260018675</t>
   </si>
   <si>
-    <t>313260018676</t>
-  </si>
-  <si>
     <t>329260019225</t>
   </si>
   <si>
+    <t>329260019252</t>
+  </si>
+  <si>
     <t>1214134-1</t>
   </si>
   <si>
-    <t>C145-00-46</t>
-  </si>
-  <si>
     <t>030-1094-58</t>
   </si>
   <si>
@@ -148,42 +139,33 @@
     <t>066-3084-32</t>
   </si>
   <si>
-    <t>2611024-1</t>
-  </si>
-  <si>
     <t>011-00870-00</t>
   </si>
   <si>
-    <t>ASG12000-2</t>
-  </si>
-  <si>
     <t>MS21442-121</t>
   </si>
   <si>
+    <t>9910592-2</t>
+  </si>
+  <si>
     <t>BELLCRANK ASSY</t>
   </si>
   <si>
-    <t>TRANSMISSION ASSY</t>
-  </si>
-  <si>
     <t>CONNECTOR</t>
   </si>
   <si>
     <t>IND RDR 2000 IN-182A</t>
   </si>
   <si>
-    <t>WINDOW</t>
-  </si>
-  <si>
     <t>MAGNETOMETER GMU 44</t>
   </si>
   <si>
-    <t>ALTERNATOR</t>
-  </si>
-  <si>
     <t>BEARING,ROLLER,NEEDL</t>
   </si>
   <si>
+    <t>ALTERNADOR</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -196,12 +178,12 @@
     <t>Expedido total</t>
   </si>
   <si>
+    <t>Aguardando solução</t>
+  </si>
+  <si>
     <t>IPLR</t>
   </si>
   <si>
-    <t>AIFP</t>
-  </si>
-  <si>
     <t>ANCE</t>
   </si>
   <si>
@@ -217,27 +199,15 @@
     <t>Foram cedidos para o C-98 2733. / De acordo com o manual da aeronave, o QPA é 02 EA por cadeira. Sendo o total para a aeronave 04 EA.A demanda aberta foi de  4EA, o SO Bispo que intermediou . Wallace 29.05</t>
   </si>
   <si>
-    <t>Vee One tem alguma atualização do DPE ?. Godoy 23/07/26</t>
-  </si>
-  <si>
     <t>Alterado o tipo da emerg. de IPLR para ANCE. Godoy 22/07/26</t>
   </si>
   <si>
-    <t>Será atendido com o estoque FAB pedido 17963489. Godoy 23/07/2026</t>
-  </si>
-  <si>
-    <t>Cedeu o item para o C-98 2737. Godoy 21/07/26.</t>
-  </si>
-  <si>
-    <t>AWB 127-4858 1702 - REZ -22/07/26</t>
+    <t>Cedeu o item para o C-98 2737. Godoy 21/07/26.  AWB 127-4857 9742volume retirado na loja GOLLOG - QMA por Kleyton em 27/07. Godoy 28/07/26.</t>
   </si>
   <si>
     <t>Foi solicitado via email no dia 02-03-2 o atendimento do item com estoque FAB. Claudio -02-03-26 - Em resposta, a coordenadoria disse que o estque seria insuficiente. Foi verificado que na T.O da ANV o QPA para esse item são 2 EA, solicitei confirmação. - Cláudio -02-03-2026. Solicitado o cancelamento da emergência em função da quantidade cedida ao 2733 ter sido de 01ea. Considerando o QPA 02 ea. Encontra-se em tratativa junto a fiscalização e o gestor do contrato conforme mensagem de e-mail de 05/03. - SOLICITAÇÃO E-C98-26047.Colocado pedido AOG Textron WB0003068789 - previsão de entrega 60 dias em média. Os demais fornecedores informaram não ter em estoque ou não possuírem a certificação necessária da peça.</t>
   </si>
   <si>
-    <t>Colocado pedido AOG Textron IJ17557538 - previsão de entrega em Miami 08/07. Previsão de chegada GIG 09/07 - MATERIAL EM TRANSITO - RECIBO 551/FAB/26 - ENVIADO PN COMPLETO PARA SANAR A EMERGENCIA DO 2709, ENVIADO MODAL TERRESTRE, DPE 13/07/2026</t>
-  </si>
-  <si>
     <t>Colocado pedido junto ao fornecedor LEGACY PARTS, validando prazo de entrega em Miami. ATZ 23/07</t>
   </si>
   <si>
@@ -247,13 +217,7 @@
     <t>Item em bancada porem em pessimo estado, foi solicitado recolhimento de mais unidades para envio a oficina para tentativa de reparo ATZ Marcio 17/7/26. Solicitado abertura de O.S. para 3EA do item no dia 16-07-26 via Email para a Coordenadoria - CLA-21-07-26</t>
   </si>
   <si>
-    <t>Será atendido via estoque TSAU. ATZ 23/07. Foi solicitado o atendimento com estoque FAB -CLA -dia 23-07</t>
-  </si>
-  <si>
     <t>material enviado com STK FAB - AWB 12748581702 - DPE 25/07/2026 - atz rc 22/07/2026- Enviado para o Operador dia 21/07/26 - AWB 127-4857 9742- REZ -22/07/26</t>
-  </si>
-  <si>
-    <t>Enviado para o Operador dia 21/07/26 - AWB 127-4858 1702 - REZ -22/07/26</t>
   </si>
   <si>
     <t>Em processo de cotação junto aos fornecedores. ATZ 23/07</t>
@@ -595,7 +559,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA10"/>
+  <dimension ref="A1:AA8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -692,22 +656,22 @@
         <v>30</v>
       </c>
       <c r="D2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="F2" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="G2">
         <v>2730</v>
       </c>
       <c r="H2" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="I2" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="J2" s="1">
         <v>46076</v>
@@ -719,7 +683,7 @@
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="N2" s="1">
         <v>46091</v>
@@ -734,16 +698,16 @@
         <v>151</v>
       </c>
       <c r="S2" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="U2" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="V2" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="W2" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -751,7 +715,7 @@
     </row>
     <row r="3" spans="1:27">
       <c r="A3">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B3" t="s">
         <v>28</v>
@@ -760,61 +724,52 @@
         <v>31</v>
       </c>
       <c r="D3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E3" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="F3" t="s">
+        <v>50</v>
+      </c>
+      <c r="G3">
+        <v>2702</v>
+      </c>
+      <c r="H3" t="s">
+        <v>52</v>
+      </c>
+      <c r="I3" t="s">
         <v>56</v>
       </c>
-      <c r="G3">
-        <v>2721</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="J3" s="1">
+        <v>46212</v>
+      </c>
+      <c r="K3" s="1">
+        <v>46212</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3" t="s">
+        <v>57</v>
+      </c>
+      <c r="N3" s="1">
+        <v>46243</v>
+      </c>
+      <c r="Q3">
+        <v>-12</v>
+      </c>
+      <c r="R3">
+        <v>19</v>
+      </c>
+      <c r="S3" t="s">
         <v>58</v>
       </c>
-      <c r="I3" t="s">
-        <v>61</v>
-      </c>
-      <c r="J3" s="1">
-        <v>46209</v>
-      </c>
-      <c r="K3" s="1">
-        <v>46210</v>
-      </c>
-      <c r="L3">
-        <v>1</v>
-      </c>
-      <c r="M3" t="s">
-        <v>63</v>
-      </c>
-      <c r="N3" s="1">
-        <v>46217</v>
-      </c>
-      <c r="O3" s="1">
-        <v>46216</v>
-      </c>
-      <c r="Q3">
-        <v>14</v>
-      </c>
-      <c r="R3">
-        <v>21</v>
-      </c>
-      <c r="S3" t="s">
+      <c r="V3" t="s">
         <v>64</v>
       </c>
-      <c r="T3" t="s">
-        <v>64</v>
-      </c>
-      <c r="U3" t="s">
-        <v>67</v>
-      </c>
-      <c r="V3" t="s">
-        <v>73</v>
-      </c>
       <c r="W3" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -822,61 +777,64 @@
     </row>
     <row r="4" spans="1:27">
       <c r="A4">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C4" t="s">
         <v>32</v>
       </c>
       <c r="D4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F4" t="s">
         <v>50</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4">
+        <v>2736</v>
+      </c>
+      <c r="H4" t="s">
+        <v>52</v>
+      </c>
+      <c r="I4" t="s">
         <v>56</v>
       </c>
-      <c r="G4">
-        <v>2702</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="J4" s="1">
+        <v>46216</v>
+      </c>
+      <c r="K4" s="1">
+        <v>46217</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4" t="s">
+        <v>57</v>
+      </c>
+      <c r="N4" s="1">
+        <v>46248</v>
+      </c>
+      <c r="O4" s="1">
+        <v>46248</v>
+      </c>
+      <c r="Q4">
+        <v>-17</v>
+      </c>
+      <c r="R4">
+        <v>14</v>
+      </c>
+      <c r="S4" t="s">
         <v>58</v>
       </c>
-      <c r="I4" t="s">
-        <v>62</v>
-      </c>
-      <c r="J4" s="1">
-        <v>46212</v>
-      </c>
-      <c r="K4" s="1">
-        <v>46212</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4" t="s">
-        <v>63</v>
-      </c>
-      <c r="N4" s="1">
-        <v>46243</v>
-      </c>
-      <c r="Q4">
-        <v>-12</v>
-      </c>
-      <c r="R4">
-        <v>19</v>
-      </c>
-      <c r="S4" t="s">
-        <v>64</v>
-      </c>
       <c r="V4" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="W4" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -884,64 +842,67 @@
     </row>
     <row r="5" spans="1:27">
       <c r="A5">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
         <v>33</v>
       </c>
       <c r="D5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E5" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="F5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G5">
+        <v>2722</v>
+      </c>
+      <c r="H5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I5" t="s">
         <v>56</v>
       </c>
-      <c r="G5">
-        <v>2736</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="J5" s="1">
+        <v>46219</v>
+      </c>
+      <c r="K5" s="1">
+        <v>46218</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5" t="s">
+        <v>57</v>
+      </c>
+      <c r="N5" s="1">
+        <v>46249</v>
+      </c>
+      <c r="Q5">
+        <v>-18</v>
+      </c>
+      <c r="R5">
+        <v>13</v>
+      </c>
+      <c r="S5" t="s">
         <v>58</v>
       </c>
-      <c r="I5" t="s">
-        <v>62</v>
-      </c>
-      <c r="J5" s="1">
-        <v>46216</v>
-      </c>
-      <c r="K5" s="1">
-        <v>46217</v>
-      </c>
-      <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5" t="s">
-        <v>63</v>
-      </c>
-      <c r="N5" s="1">
-        <v>46248</v>
-      </c>
-      <c r="O5" s="1">
-        <v>46248</v>
-      </c>
-      <c r="Q5">
-        <v>-17</v>
-      </c>
-      <c r="R5">
-        <v>14</v>
-      </c>
-      <c r="S5" t="s">
-        <v>64</v>
+      <c r="T5" t="s">
+        <v>59</v>
+      </c>
+      <c r="U5" t="s">
+        <v>61</v>
       </c>
       <c r="V5" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="W5" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -949,67 +910,70 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C6" t="s">
         <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E6" t="s">
+        <v>47</v>
+      </c>
+      <c r="F6" t="s">
         <v>51</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6">
+        <v>2730</v>
+      </c>
+      <c r="H6" t="s">
+        <v>53</v>
+      </c>
+      <c r="I6" t="s">
+        <v>55</v>
+      </c>
+      <c r="J6" s="1">
+        <v>46220</v>
+      </c>
+      <c r="K6" s="1">
+        <v>46221</v>
+      </c>
+      <c r="L6">
+        <v>1</v>
+      </c>
+      <c r="M6" t="s">
         <v>57</v>
       </c>
-      <c r="G6">
-        <v>2722</v>
-      </c>
-      <c r="H6" t="s">
+      <c r="N6" s="1">
+        <v>46232</v>
+      </c>
+      <c r="O6" s="1">
+        <v>46228</v>
+      </c>
+      <c r="Q6">
+        <v>-1</v>
+      </c>
+      <c r="R6">
+        <v>10</v>
+      </c>
+      <c r="S6" t="s">
         <v>58</v>
       </c>
-      <c r="I6" t="s">
+      <c r="T6" t="s">
+        <v>59</v>
+      </c>
+      <c r="U6" t="s">
         <v>62</v>
       </c>
-      <c r="J6" s="1">
-        <v>46219</v>
-      </c>
-      <c r="K6" s="1">
-        <v>46218</v>
-      </c>
-      <c r="L6">
-        <v>1</v>
-      </c>
-      <c r="M6" t="s">
-        <v>63</v>
-      </c>
-      <c r="N6" s="1">
-        <v>46249</v>
-      </c>
-      <c r="Q6">
-        <v>-18</v>
-      </c>
-      <c r="R6">
-        <v>13</v>
-      </c>
-      <c r="S6" t="s">
-        <v>64</v>
-      </c>
-      <c r="T6" t="s">
-        <v>65</v>
-      </c>
-      <c r="U6" t="s">
-        <v>68</v>
-      </c>
       <c r="V6" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="W6" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1017,7 +981,7 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>685</v>
+        <v>329</v>
       </c>
       <c r="B7" t="s">
         <v>29</v>
@@ -1026,55 +990,55 @@
         <v>35</v>
       </c>
       <c r="D7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E7" t="s">
+        <v>48</v>
+      </c>
+      <c r="F7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G7">
+        <v>2720</v>
+      </c>
+      <c r="H7" t="s">
         <v>52</v>
       </c>
-      <c r="F7" t="s">
+      <c r="I7" t="s">
         <v>56</v>
       </c>
-      <c r="G7">
-        <v>2703</v>
-      </c>
-      <c r="H7" t="s">
-        <v>59</v>
-      </c>
-      <c r="I7" t="s">
-        <v>62</v>
-      </c>
       <c r="J7" s="1">
-        <v>46219</v>
+        <v>46220</v>
       </c>
       <c r="K7" s="1">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="L7">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="M7" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="N7" s="1">
-        <v>46251</v>
+        <v>46254</v>
       </c>
       <c r="Q7">
-        <v>-20</v>
+        <v>-23</v>
       </c>
       <c r="R7">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="S7" t="s">
-        <v>65</v>
-      </c>
-      <c r="U7" t="s">
+        <v>58</v>
+      </c>
+      <c r="T7" t="s">
+        <v>58</v>
+      </c>
+      <c r="V7" t="s">
+        <v>68</v>
+      </c>
+      <c r="W7" t="s">
         <v>69</v>
-      </c>
-      <c r="V7" t="s">
-        <v>77</v>
-      </c>
-      <c r="W7" t="s">
-        <v>81</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1082,205 +1046,60 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C8" t="s">
         <v>36</v>
       </c>
       <c r="D8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E8" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F8" t="s">
+        <v>51</v>
+      </c>
+      <c r="G8">
+        <v>2721</v>
+      </c>
+      <c r="H8" t="s">
+        <v>54</v>
+      </c>
+      <c r="I8" t="s">
+        <v>55</v>
+      </c>
+      <c r="J8" s="1">
+        <v>46230</v>
+      </c>
+      <c r="K8" s="1">
+        <v>46231</v>
+      </c>
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8" t="s">
         <v>57</v>
       </c>
-      <c r="G8">
-        <v>2730</v>
-      </c>
-      <c r="H8" t="s">
-        <v>59</v>
-      </c>
-      <c r="I8" t="s">
-        <v>60</v>
-      </c>
-      <c r="J8" s="1">
-        <v>46220</v>
-      </c>
-      <c r="K8" s="1">
-        <v>46221</v>
-      </c>
-      <c r="L8">
-        <v>1</v>
-      </c>
-      <c r="M8" t="s">
-        <v>63</v>
-      </c>
       <c r="N8" s="1">
-        <v>46232</v>
-      </c>
-      <c r="O8" s="1">
-        <v>46228</v>
+        <v>46242</v>
       </c>
       <c r="Q8">
-        <v>-1</v>
+        <v>-11</v>
       </c>
       <c r="R8">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="S8" t="s">
-        <v>64</v>
-      </c>
-      <c r="T8" t="s">
-        <v>65</v>
-      </c>
-      <c r="U8" t="s">
-        <v>70</v>
-      </c>
-      <c r="V8" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="W8" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="AA8" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:27">
-      <c r="A9">
-        <v>313</v>
-      </c>
-      <c r="B9" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D9" t="s">
-        <v>46</v>
-      </c>
-      <c r="E9" t="s">
-        <v>54</v>
-      </c>
-      <c r="F9" t="s">
-        <v>57</v>
-      </c>
-      <c r="G9">
-        <v>2741</v>
-      </c>
-      <c r="H9" t="s">
-        <v>58</v>
-      </c>
-      <c r="I9" t="s">
-        <v>61</v>
-      </c>
-      <c r="J9" s="1">
-        <v>46224</v>
-      </c>
-      <c r="K9" s="1">
-        <v>46222</v>
-      </c>
-      <c r="L9">
-        <v>1</v>
-      </c>
-      <c r="M9" t="s">
-        <v>63</v>
-      </c>
-      <c r="N9" s="1">
-        <v>46229</v>
-      </c>
-      <c r="Q9">
-        <v>2</v>
-      </c>
-      <c r="R9">
-        <v>9</v>
-      </c>
-      <c r="S9" t="s">
-        <v>64</v>
-      </c>
-      <c r="T9" t="s">
-        <v>65</v>
-      </c>
-      <c r="U9" t="s">
-        <v>71</v>
-      </c>
-      <c r="V9" t="s">
-        <v>79</v>
-      </c>
-      <c r="W9" t="s">
-        <v>81</v>
-      </c>
-      <c r="AA9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:27">
-      <c r="A10">
-        <v>329</v>
-      </c>
-      <c r="B10" t="s">
-        <v>28</v>
-      </c>
-      <c r="C10" t="s">
-        <v>38</v>
-      </c>
-      <c r="D10" t="s">
-        <v>47</v>
-      </c>
-      <c r="E10" t="s">
-        <v>55</v>
-      </c>
-      <c r="F10" t="s">
-        <v>56</v>
-      </c>
-      <c r="G10">
-        <v>2720</v>
-      </c>
-      <c r="H10" t="s">
-        <v>58</v>
-      </c>
-      <c r="I10" t="s">
-        <v>62</v>
-      </c>
-      <c r="J10" s="1">
-        <v>46220</v>
-      </c>
-      <c r="K10" s="1">
-        <v>46223</v>
-      </c>
-      <c r="L10">
-        <v>10</v>
-      </c>
-      <c r="M10" t="s">
-        <v>63</v>
-      </c>
-      <c r="N10" s="1">
-        <v>46254</v>
-      </c>
-      <c r="Q10">
-        <v>-23</v>
-      </c>
-      <c r="R10">
-        <v>8</v>
-      </c>
-      <c r="S10" t="s">
-        <v>64</v>
-      </c>
-      <c r="T10" t="s">
-        <v>64</v>
-      </c>
-      <c r="V10" t="s">
-        <v>80</v>
-      </c>
-      <c r="W10" t="s">
-        <v>81</v>
-      </c>
-      <c r="AA10" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (28/07/2026 17:50)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="64">
   <si>
     <t>om_emg</t>
   </si>
@@ -118,9 +118,6 @@
     <t>685260012387</t>
   </si>
   <si>
-    <t>313260018675</t>
-  </si>
-  <si>
     <t>329260019225</t>
   </si>
   <si>
@@ -139,9 +136,6 @@
     <t>066-3084-32</t>
   </si>
   <si>
-    <t>011-00870-00</t>
-  </si>
-  <si>
     <t>MS21442-121</t>
   </si>
   <si>
@@ -157,9 +151,6 @@
     <t>IND RDR 2000 IN-182A</t>
   </si>
   <si>
-    <t>MAGNETOMETER GMU 44</t>
-  </si>
-  <si>
     <t>BEARING,ROLLER,NEEDL</t>
   </si>
   <si>
@@ -175,9 +166,6 @@
     <t>Providência tomada</t>
   </si>
   <si>
-    <t>Expedido total</t>
-  </si>
-  <si>
     <t>Aguardando solução</t>
   </si>
   <si>
@@ -202,9 +190,6 @@
     <t>Alterado o tipo da emerg. de IPLR para ANCE. Godoy 22/07/26</t>
   </si>
   <si>
-    <t>Cedeu o item para o C-98 2737. Godoy 21/07/26.  AWB 127-4857 9742volume retirado na loja GOLLOG - QMA por Kleyton em 27/07. Godoy 28/07/26.</t>
-  </si>
-  <si>
     <t>Foi solicitado via email no dia 02-03-2 o atendimento do item com estoque FAB. Claudio -02-03-26 - Em resposta, a coordenadoria disse que o estque seria insuficiente. Foi verificado que na T.O da ANV o QPA para esse item são 2 EA, solicitei confirmação. - Cláudio -02-03-2026. Solicitado o cancelamento da emergência em função da quantidade cedida ao 2733 ter sido de 01ea. Considerando o QPA 02 ea. Encontra-se em tratativa junto a fiscalização e o gestor do contrato conforme mensagem de e-mail de 05/03. - SOLICITAÇÃO E-C98-26047.Colocado pedido AOG Textron WB0003068789 - previsão de entrega 60 dias em média. Os demais fornecedores informaram não ter em estoque ou não possuírem a certificação necessária da peça.</t>
   </si>
   <si>
@@ -215,9 +200,6 @@
   </si>
   <si>
     <t>Item em bancada porem em pessimo estado, foi solicitado recolhimento de mais unidades para envio a oficina para tentativa de reparo ATZ Marcio 17/7/26. Solicitado abertura de O.S. para 3EA do item no dia 16-07-26 via Email para a Coordenadoria - CLA-21-07-26</t>
-  </si>
-  <si>
-    <t>material enviado com STK FAB - AWB 12748581702 - DPE 25/07/2026 - atz rc 22/07/2026- Enviado para o Operador dia 21/07/26 - AWB 127-4857 9742- REZ -22/07/26</t>
   </si>
   <si>
     <t>Em processo de cotação junto aos fornecedores. ATZ 23/07</t>
@@ -559,7 +541,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA8"/>
+  <dimension ref="A1:AA7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -656,22 +638,22 @@
         <v>30</v>
       </c>
       <c r="D2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="G2">
         <v>2730</v>
       </c>
       <c r="H2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I2" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="J2" s="1">
         <v>46076</v>
@@ -683,7 +665,7 @@
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="N2" s="1">
         <v>46091</v>
@@ -698,16 +680,19 @@
         <v>151</v>
       </c>
       <c r="S2" t="s">
+        <v>54</v>
+      </c>
+      <c r="T2" t="s">
+        <v>55</v>
+      </c>
+      <c r="U2" t="s">
+        <v>56</v>
+      </c>
+      <c r="V2" t="s">
         <v>58</v>
       </c>
-      <c r="U2" t="s">
-        <v>60</v>
-      </c>
-      <c r="V2" t="s">
+      <c r="W2" t="s">
         <v>63</v>
-      </c>
-      <c r="W2" t="s">
-        <v>69</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -724,22 +709,22 @@
         <v>31</v>
       </c>
       <c r="D3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="G3">
         <v>2702</v>
       </c>
       <c r="H3" t="s">
+        <v>49</v>
+      </c>
+      <c r="I3" t="s">
         <v>52</v>
-      </c>
-      <c r="I3" t="s">
-        <v>56</v>
       </c>
       <c r="J3" s="1">
         <v>46212</v>
@@ -751,7 +736,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="N3" s="1">
         <v>46243</v>
@@ -763,13 +748,13 @@
         <v>19</v>
       </c>
       <c r="S3" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="V3" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="W3" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -786,22 +771,22 @@
         <v>32</v>
       </c>
       <c r="D4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="G4">
         <v>2736</v>
       </c>
       <c r="H4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I4" t="s">
         <v>52</v>
-      </c>
-      <c r="I4" t="s">
-        <v>56</v>
       </c>
       <c r="J4" s="1">
         <v>46216</v>
@@ -813,7 +798,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="N4" s="1">
         <v>46248</v>
@@ -828,13 +813,13 @@
         <v>14</v>
       </c>
       <c r="S4" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="V4" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="W4" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -851,22 +836,22 @@
         <v>33</v>
       </c>
       <c r="D5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="G5">
         <v>2722</v>
       </c>
       <c r="H5" t="s">
+        <v>49</v>
+      </c>
+      <c r="I5" t="s">
         <v>52</v>
-      </c>
-      <c r="I5" t="s">
-        <v>56</v>
       </c>
       <c r="J5" s="1">
         <v>46219</v>
@@ -878,7 +863,7 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="N5" s="1">
         <v>46249</v>
@@ -890,19 +875,19 @@
         <v>13</v>
       </c>
       <c r="S5" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="T5" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="U5" t="s">
+        <v>57</v>
+      </c>
+      <c r="V5" t="s">
         <v>61</v>
       </c>
-      <c r="V5" t="s">
-        <v>66</v>
-      </c>
       <c r="W5" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -910,70 +895,64 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C6" t="s">
         <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F6" t="s">
         <v>47</v>
       </c>
-      <c r="F6" t="s">
-        <v>51</v>
-      </c>
       <c r="G6">
-        <v>2730</v>
+        <v>2720</v>
       </c>
       <c r="H6" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="I6" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="J6" s="1">
         <v>46220</v>
       </c>
       <c r="K6" s="1">
-        <v>46221</v>
+        <v>46223</v>
       </c>
       <c r="L6">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="M6" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="N6" s="1">
-        <v>46232</v>
-      </c>
-      <c r="O6" s="1">
-        <v>46228</v>
+        <v>46254</v>
       </c>
       <c r="Q6">
-        <v>-1</v>
+        <v>-23</v>
       </c>
       <c r="R6">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="S6" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="T6" t="s">
-        <v>59</v>
-      </c>
-      <c r="U6" t="s">
+        <v>54</v>
+      </c>
+      <c r="V6" t="s">
         <v>62</v>
       </c>
-      <c r="V6" t="s">
-        <v>67</v>
-      </c>
       <c r="W6" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -990,116 +969,54 @@
         <v>35</v>
       </c>
       <c r="D7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E7" t="s">
+        <v>46</v>
+      </c>
+      <c r="F7" t="s">
         <v>48</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7">
+        <v>2721</v>
+      </c>
+      <c r="H7" t="s">
         <v>50</v>
       </c>
-      <c r="G7">
-        <v>2720</v>
-      </c>
-      <c r="H7" t="s">
-        <v>52</v>
-      </c>
       <c r="I7" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="J7" s="1">
-        <v>46220</v>
+        <v>46230</v>
       </c>
       <c r="K7" s="1">
-        <v>46223</v>
+        <v>46231</v>
       </c>
       <c r="L7">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="N7" s="1">
-        <v>46254</v>
+        <v>46242</v>
       </c>
       <c r="Q7">
-        <v>-23</v>
+        <v>-11</v>
       </c>
       <c r="R7">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S7" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="T7" t="s">
-        <v>58</v>
-      </c>
-      <c r="V7" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="W7" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="AA7" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:27">
-      <c r="A8">
-        <v>329</v>
-      </c>
-      <c r="B8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" t="s">
-        <v>43</v>
-      </c>
-      <c r="E8" t="s">
-        <v>49</v>
-      </c>
-      <c r="F8" t="s">
-        <v>51</v>
-      </c>
-      <c r="G8">
-        <v>2721</v>
-      </c>
-      <c r="H8" t="s">
-        <v>54</v>
-      </c>
-      <c r="I8" t="s">
-        <v>55</v>
-      </c>
-      <c r="J8" s="1">
-        <v>46230</v>
-      </c>
-      <c r="K8" s="1">
-        <v>46231</v>
-      </c>
-      <c r="L8">
-        <v>1</v>
-      </c>
-      <c r="M8" t="s">
-        <v>57</v>
-      </c>
-      <c r="N8" s="1">
-        <v>46242</v>
-      </c>
-      <c r="Q8">
-        <v>-11</v>
-      </c>
-      <c r="R8">
-        <v>0</v>
-      </c>
-      <c r="S8" t="s">
-        <v>58</v>
-      </c>
-      <c r="W8" t="s">
-        <v>69</v>
-      </c>
-      <c r="AA8" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (29/07/2026 13:12)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="68">
   <si>
     <t>om_emg</t>
   </si>
@@ -106,6 +106,9 @@
     <t>BABR</t>
   </si>
   <si>
+    <t>PAMA-LS</t>
+  </si>
+  <si>
     <t>313260017747</t>
   </si>
   <si>
@@ -124,6 +127,9 @@
     <t>329260019252</t>
   </si>
   <si>
+    <t>304260076647</t>
+  </si>
+  <si>
     <t>1214134-1</t>
   </si>
   <si>
@@ -142,6 +148,9 @@
     <t>9910592-2</t>
   </si>
   <si>
+    <t>2617015-23</t>
+  </si>
+  <si>
     <t>BELLCRANK ASSY</t>
   </si>
   <si>
@@ -157,6 +166,9 @@
     <t>ALTERNADOR</t>
   </si>
   <si>
+    <t>HINGE DOOR LH</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -166,9 +178,6 @@
     <t>Providência tomada</t>
   </si>
   <si>
-    <t>Aguardando solução</t>
-  </si>
-  <si>
     <t>IPLR</t>
   </si>
   <si>
@@ -190,10 +199,13 @@
     <t>Alterado o tipo da emerg. de IPLR para ANCE. Godoy 22/07/26</t>
   </si>
   <si>
+    <t>Cedeu o item para o 2704. Ramon 29/07/26</t>
+  </si>
+  <si>
     <t>Foi solicitado via email no dia 02-03-2 o atendimento do item com estoque FAB. Claudio -02-03-26 - Em resposta, a coordenadoria disse que o estque seria insuficiente. Foi verificado que na T.O da ANV o QPA para esse item são 2 EA, solicitei confirmação. - Cláudio -02-03-2026. Solicitado o cancelamento da emergência em função da quantidade cedida ao 2733 ter sido de 01ea. Considerando o QPA 02 ea. Encontra-se em tratativa junto a fiscalização e o gestor do contrato conforme mensagem de e-mail de 05/03. - SOLICITAÇÃO E-C98-26047.Colocado pedido AOG Textron WB0003068789 - previsão de entrega 60 dias em média. Os demais fornecedores informaram não ter em estoque ou não possuírem a certificação necessária da peça.</t>
   </si>
   <si>
-    <t>Colocado pedido junto ao fornecedor LEGACY PARTS, validando prazo de entrega em Miami. ATZ 23/07</t>
+    <t>Colocado pedido junto ao fornecedor LEGACY PARTS, validando prazo de entrega em Miami. ATZ 28/07</t>
   </si>
   <si>
     <t>Colocado pedido Textron IJ17575583 - entregue em Miami 15/07. Carga rercepcionada GIG 19/07 - Aguardando liberação do SEFAZ. ATZ 21/07 - material em processo de expedição RC 23/07/2026</t>
@@ -202,7 +214,7 @@
     <t>Item em bancada porem em pessimo estado, foi solicitado recolhimento de mais unidades para envio a oficina para tentativa de reparo ATZ Marcio 17/7/26. Solicitado abertura de O.S. para 3EA do item no dia 16-07-26 via Email para a Coordenadoria - CLA-21-07-26</t>
   </si>
   <si>
-    <t>Em processo de cotação junto aos fornecedores. ATZ 23/07</t>
+    <t>Pedido I816822 entregue em Miami 27/07. Consolidando próximo embarque GIG. ATZ 28/07</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -541,7 +553,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA7"/>
+  <dimension ref="A1:AA8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -635,25 +647,25 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="F2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="G2">
         <v>2730</v>
       </c>
       <c r="H2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="I2" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="J2" s="1">
         <v>46076</v>
@@ -665,7 +677,7 @@
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="N2" s="1">
         <v>46091</v>
@@ -674,25 +686,25 @@
         <v>46287</v>
       </c>
       <c r="Q2">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="R2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="S2" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="T2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="U2" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="V2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="W2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -706,25 +718,25 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E3" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="F3" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="G3">
         <v>2702</v>
       </c>
       <c r="H3" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="I3" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="J3" s="1">
         <v>46212</v>
@@ -736,25 +748,28 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="N3" s="1">
         <v>46243</v>
       </c>
       <c r="Q3">
-        <v>-12</v>
+        <v>-11</v>
       </c>
       <c r="R3">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="S3" t="s">
-        <v>54</v>
+        <v>57</v>
+      </c>
+      <c r="T3" t="s">
+        <v>58</v>
       </c>
       <c r="V3" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="W3" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -768,25 +783,25 @@
         <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E4" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="F4" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="G4">
         <v>2736</v>
       </c>
       <c r="H4" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="I4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="J4" s="1">
         <v>46216</v>
@@ -798,7 +813,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="N4" s="1">
         <v>46248</v>
@@ -807,19 +822,22 @@
         <v>46248</v>
       </c>
       <c r="Q4">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="R4">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S4" t="s">
-        <v>54</v>
+        <v>57</v>
+      </c>
+      <c r="T4" t="s">
+        <v>58</v>
       </c>
       <c r="V4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="W4" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -833,25 +851,25 @@
         <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E5" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F5" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="G5">
         <v>2722</v>
       </c>
       <c r="H5" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="I5" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="J5" s="1">
         <v>46219</v>
@@ -863,31 +881,31 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="N5" s="1">
         <v>46249</v>
       </c>
       <c r="Q5">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="R5">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S5" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="T5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="U5" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="V5" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="W5" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -901,25 +919,25 @@
         <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E6" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F6" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="G6">
         <v>2720</v>
       </c>
       <c r="H6" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="I6" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="J6" s="1">
         <v>46220</v>
@@ -931,28 +949,28 @@
         <v>10</v>
       </c>
       <c r="M6" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="N6" s="1">
         <v>46254</v>
       </c>
       <c r="Q6">
-        <v>-23</v>
+        <v>-22</v>
       </c>
       <c r="R6">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S6" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="T6" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="V6" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="W6" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -966,25 +984,25 @@
         <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E7" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F7" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="G7">
         <v>2721</v>
       </c>
       <c r="H7" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="I7" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="J7" s="1">
         <v>46230</v>
@@ -996,27 +1014,92 @@
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="N7" s="1">
         <v>46242</v>
       </c>
       <c r="Q7">
+        <v>-10</v>
+      </c>
+      <c r="R7">
+        <v>1</v>
+      </c>
+      <c r="S7" t="s">
+        <v>57</v>
+      </c>
+      <c r="T7" t="s">
+        <v>57</v>
+      </c>
+      <c r="W7" t="s">
+        <v>67</v>
+      </c>
+      <c r="AA7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27">
+      <c r="A8">
+        <v>304</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" t="s">
+        <v>44</v>
+      </c>
+      <c r="E8" t="s">
+        <v>50</v>
+      </c>
+      <c r="F8" t="s">
+        <v>51</v>
+      </c>
+      <c r="G8">
+        <v>2728</v>
+      </c>
+      <c r="H8" t="s">
+        <v>53</v>
+      </c>
+      <c r="I8" t="s">
+        <v>54</v>
+      </c>
+      <c r="J8" s="1">
+        <v>46231</v>
+      </c>
+      <c r="K8" s="1">
+        <v>46232</v>
+      </c>
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8" t="s">
+        <v>56</v>
+      </c>
+      <c r="N8" s="1">
+        <v>46243</v>
+      </c>
+      <c r="Q8">
         <v>-11</v>
       </c>
-      <c r="R7">
+      <c r="R8">
         <v>0</v>
       </c>
-      <c r="S7" t="s">
-        <v>54</v>
-      </c>
-      <c r="T7" t="s">
-        <v>54</v>
-      </c>
-      <c r="W7" t="s">
-        <v>63</v>
-      </c>
-      <c r="AA7" t="b">
+      <c r="S8" t="s">
+        <v>57</v>
+      </c>
+      <c r="T8" t="s">
+        <v>58</v>
+      </c>
+      <c r="U8" t="s">
+        <v>61</v>
+      </c>
+      <c r="W8" t="s">
+        <v>67</v>
+      </c>
+      <c r="AA8" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (29/07/2026 17:33)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -943,7 +943,7 @@
         <v>46220</v>
       </c>
       <c r="K6" s="1">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="L6">
         <v>10</v>
@@ -952,13 +952,13 @@
         <v>56</v>
       </c>
       <c r="N6" s="1">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="Q6">
-        <v>-22</v>
+        <v>-23</v>
       </c>
       <c r="R6">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S6" t="s">
         <v>57</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (30/07/2026 13:19)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="70">
   <si>
     <t>om_emg</t>
   </si>
@@ -124,12 +124,12 @@
     <t>329260019225</t>
   </si>
   <si>
-    <t>329260019252</t>
-  </si>
-  <si>
     <t>304260076647</t>
   </si>
   <si>
+    <t>313260018682</t>
+  </si>
+  <si>
     <t>1214134-1</t>
   </si>
   <si>
@@ -145,12 +145,12 @@
     <t>MS21442-121</t>
   </si>
   <si>
-    <t>9910592-2</t>
-  </si>
-  <si>
     <t>2617015-23</t>
   </si>
   <si>
+    <t>011-00916-10</t>
+  </si>
+  <si>
     <t>BELLCRANK ASSY</t>
   </si>
   <si>
@@ -163,12 +163,12 @@
     <t>BEARING,ROLLER,NEEDL</t>
   </si>
   <si>
-    <t>ALTERNADOR</t>
-  </si>
-  <si>
     <t>HINGE DOOR LH</t>
   </si>
   <si>
+    <t>DISPLAY UNIT,FLIGHT</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -178,6 +178,9 @@
     <t>Providência tomada</t>
   </si>
   <si>
+    <t>Aguardando solução</t>
+  </si>
+  <si>
     <t>IPLR</t>
   </si>
   <si>
@@ -215,6 +218,9 @@
   </si>
   <si>
     <t>Pedido I816822 entregue em Miami 27/07. Consolidando próximo embarque GIG. ATZ 28/07</t>
+  </si>
+  <si>
+    <t>Será atendido via estoque V1. ATZ 29/07</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -665,7 +671,7 @@
         <v>53</v>
       </c>
       <c r="I2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J2" s="1">
         <v>46076</v>
@@ -677,7 +683,7 @@
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N2" s="1">
         <v>46091</v>
@@ -686,25 +692,25 @@
         <v>46287</v>
       </c>
       <c r="Q2">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="R2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="S2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="T2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="U2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="V2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="W2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -736,7 +742,7 @@
         <v>53</v>
       </c>
       <c r="I3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J3" s="1">
         <v>46212</v>
@@ -748,28 +754,28 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N3" s="1">
         <v>46243</v>
       </c>
       <c r="Q3">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R3">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="S3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="T3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="V3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="W3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -801,7 +807,7 @@
         <v>53</v>
       </c>
       <c r="I4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J4" s="1">
         <v>46216</v>
@@ -813,7 +819,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N4" s="1">
         <v>46248</v>
@@ -822,22 +828,22 @@
         <v>46248</v>
       </c>
       <c r="Q4">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="R4">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="T4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="V4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="W4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -869,7 +875,7 @@
         <v>53</v>
       </c>
       <c r="I5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J5" s="1">
         <v>46219</v>
@@ -881,31 +887,31 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N5" s="1">
         <v>46249</v>
       </c>
       <c r="Q5">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="R5">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="T5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="U5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="V5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="W5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -937,7 +943,7 @@
         <v>53</v>
       </c>
       <c r="I6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J6" s="1">
         <v>46220</v>
@@ -949,28 +955,28 @@
         <v>10</v>
       </c>
       <c r="M6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N6" s="1">
         <v>46255</v>
       </c>
       <c r="Q6">
-        <v>-23</v>
+        <v>-22</v>
       </c>
       <c r="R6">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="T6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="V6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="W6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -978,10 +984,10 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>329</v>
+        <v>304</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C7" t="s">
         <v>36</v>
@@ -993,31 +999,31 @@
         <v>49</v>
       </c>
       <c r="F7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G7">
-        <v>2721</v>
+        <v>2728</v>
       </c>
       <c r="H7" t="s">
         <v>53</v>
       </c>
       <c r="I7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J7" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="K7" s="1">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="L7">
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N7" s="1">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="Q7">
         <v>-10</v>
@@ -1026,13 +1032,19 @@
         <v>1</v>
       </c>
       <c r="S7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="T7" t="s">
-        <v>57</v>
+        <v>59</v>
+      </c>
+      <c r="U7" t="s">
+        <v>62</v>
+      </c>
+      <c r="V7" t="s">
+        <v>68</v>
       </c>
       <c r="W7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1040,10 +1052,10 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>304</v>
+        <v>313</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C8" t="s">
         <v>37</v>
@@ -1055,49 +1067,43 @@
         <v>50</v>
       </c>
       <c r="F8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G8">
-        <v>2728</v>
+        <v>2741</v>
       </c>
       <c r="H8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J8" s="1">
         <v>46231</v>
       </c>
       <c r="K8" s="1">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="L8">
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N8" s="1">
-        <v>46243</v>
+        <v>46264</v>
       </c>
       <c r="Q8">
-        <v>-11</v>
+        <v>-31</v>
       </c>
       <c r="R8">
         <v>0</v>
       </c>
       <c r="S8" t="s">
-        <v>57</v>
-      </c>
-      <c r="T8" t="s">
         <v>58</v>
       </c>
-      <c r="U8" t="s">
-        <v>61</v>
-      </c>
       <c r="W8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (30/07/2026 17:47)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="69">
   <si>
     <t>om_emg</t>
   </si>
@@ -106,9 +106,6 @@
     <t>BABR</t>
   </si>
   <si>
-    <t>PAMA-LS</t>
-  </si>
-  <si>
     <t>313260017747</t>
   </si>
   <si>
@@ -124,12 +121,15 @@
     <t>329260019225</t>
   </si>
   <si>
-    <t>304260076647</t>
-  </si>
-  <si>
     <t>313260018682</t>
   </si>
   <si>
+    <t>313260018657</t>
+  </si>
+  <si>
+    <t>313260018658</t>
+  </si>
+  <si>
     <t>1214134-1</t>
   </si>
   <si>
@@ -145,12 +145,12 @@
     <t>MS21442-121</t>
   </si>
   <si>
-    <t>2617015-23</t>
-  </si>
-  <si>
     <t>011-00916-10</t>
   </si>
   <si>
+    <t>324843-W020</t>
+  </si>
+  <si>
     <t>BELLCRANK ASSY</t>
   </si>
   <si>
@@ -163,18 +163,21 @@
     <t>BEARING,ROLLER,NEEDL</t>
   </si>
   <si>
-    <t>HINGE DOOR LH</t>
-  </si>
-  <si>
     <t>DISPLAY UNIT,FLIGHT</t>
   </si>
   <si>
+    <t>HEADSET-MICROPHONE</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
     <t>R</t>
   </si>
   <si>
+    <t>T</t>
+  </si>
+  <si>
     <t>Providência tomada</t>
   </si>
   <si>
@@ -202,9 +205,6 @@
     <t>Alterado o tipo da emerg. de IPLR para ANCE. Godoy 22/07/26</t>
   </si>
   <si>
-    <t>Cedeu o item para o 2704. Ramon 29/07/26</t>
-  </si>
-  <si>
     <t>Foi solicitado via email no dia 02-03-2 o atendimento do item com estoque FAB. Claudio -02-03-26 - Em resposta, a coordenadoria disse que o estque seria insuficiente. Foi verificado que na T.O da ANV o QPA para esse item são 2 EA, solicitei confirmação. - Cláudio -02-03-2026. Solicitado o cancelamento da emergência em função da quantidade cedida ao 2733 ter sido de 01ea. Considerando o QPA 02 ea. Encontra-se em tratativa junto a fiscalização e o gestor do contrato conforme mensagem de e-mail de 05/03. - SOLICITAÇÃO E-C98-26047.Colocado pedido AOG Textron WB0003068789 - previsão de entrega 60 dias em média. Os demais fornecedores informaram não ter em estoque ou não possuírem a certificação necessária da peça.</t>
   </si>
   <si>
@@ -218,9 +218,6 @@
   </si>
   <si>
     <t>Pedido I816822 entregue em Miami 27/07. Consolidando próximo embarque GIG. ATZ 28/07</t>
-  </si>
-  <si>
-    <t>Será atendido via estoque V1. ATZ 29/07</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -559,7 +556,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA8"/>
+  <dimension ref="A1:AA9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -653,7 +650,7 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D2" t="s">
         <v>38</v>
@@ -668,10 +665,10 @@
         <v>2730</v>
       </c>
       <c r="H2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J2" s="1">
         <v>46076</v>
@@ -683,7 +680,7 @@
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N2" s="1">
         <v>46091</v>
@@ -698,19 +695,19 @@
         <v>153</v>
       </c>
       <c r="S2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="T2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="U2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="V2" t="s">
         <v>63</v>
       </c>
       <c r="W2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -724,7 +721,7 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D3" t="s">
         <v>39</v>
@@ -739,10 +736,10 @@
         <v>2702</v>
       </c>
       <c r="H3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J3" s="1">
         <v>46212</v>
@@ -754,7 +751,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N3" s="1">
         <v>46243</v>
@@ -766,16 +763,16 @@
         <v>21</v>
       </c>
       <c r="S3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="T3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="V3" t="s">
         <v>64</v>
       </c>
       <c r="W3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -789,7 +786,7 @@
         <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D4" t="s">
         <v>40</v>
@@ -804,10 +801,10 @@
         <v>2736</v>
       </c>
       <c r="H4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J4" s="1">
         <v>46216</v>
@@ -819,7 +816,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N4" s="1">
         <v>46248</v>
@@ -834,16 +831,16 @@
         <v>16</v>
       </c>
       <c r="S4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="T4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="V4" t="s">
         <v>65</v>
       </c>
       <c r="W4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -857,7 +854,7 @@
         <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D5" t="s">
         <v>41</v>
@@ -872,10 +869,10 @@
         <v>2722</v>
       </c>
       <c r="H5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J5" s="1">
         <v>46219</v>
@@ -887,7 +884,7 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N5" s="1">
         <v>46249</v>
@@ -899,19 +896,19 @@
         <v>15</v>
       </c>
       <c r="S5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="T5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="U5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="V5" t="s">
         <v>66</v>
       </c>
       <c r="W5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -925,7 +922,7 @@
         <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s">
         <v>42</v>
@@ -940,10 +937,10 @@
         <v>2720</v>
       </c>
       <c r="H6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J6" s="1">
         <v>46220</v>
@@ -955,7 +952,7 @@
         <v>10</v>
       </c>
       <c r="M6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N6" s="1">
         <v>46255</v>
@@ -967,16 +964,16 @@
         <v>9</v>
       </c>
       <c r="S6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="T6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="V6" t="s">
         <v>67</v>
       </c>
       <c r="W6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -984,13 +981,13 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>304</v>
+        <v>313</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D7" t="s">
         <v>43</v>
@@ -999,52 +996,43 @@
         <v>49</v>
       </c>
       <c r="F7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G7">
-        <v>2728</v>
+        <v>2741</v>
       </c>
       <c r="H7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I7" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="J7" s="1">
         <v>46231</v>
       </c>
       <c r="K7" s="1">
-        <v>46232</v>
+        <v>46234</v>
       </c>
       <c r="L7">
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N7" s="1">
-        <v>46243</v>
+        <v>46265</v>
       </c>
       <c r="Q7">
-        <v>-10</v>
+        <v>-32</v>
       </c>
       <c r="R7">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S7" t="s">
-        <v>58</v>
-      </c>
-      <c r="T7" t="s">
         <v>59</v>
       </c>
-      <c r="U7" t="s">
-        <v>62</v>
-      </c>
-      <c r="V7" t="s">
+      <c r="W7" t="s">
         <v>68</v>
-      </c>
-      <c r="W7" t="s">
-        <v>69</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1058,7 +1046,7 @@
         <v>27</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D8" t="s">
         <v>44</v>
@@ -1067,45 +1055,104 @@
         <v>50</v>
       </c>
       <c r="F8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G8">
-        <v>2741</v>
+        <v>2736</v>
       </c>
       <c r="H8" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J8" s="1">
-        <v>46231</v>
+        <v>46205</v>
       </c>
       <c r="K8" s="1">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="L8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M8" t="s">
+        <v>58</v>
+      </c>
+      <c r="N8" s="1">
+        <v>46265</v>
+      </c>
+      <c r="Q8">
+        <v>-32</v>
+      </c>
+      <c r="R8">
+        <v>-1</v>
+      </c>
+      <c r="S8" t="s">
+        <v>59</v>
+      </c>
+      <c r="W8" t="s">
+        <v>68</v>
+      </c>
+      <c r="AA8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27">
+      <c r="A9">
+        <v>313</v>
+      </c>
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" t="s">
+        <v>44</v>
+      </c>
+      <c r="E9" t="s">
+        <v>50</v>
+      </c>
+      <c r="F9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G9">
+        <v>2737</v>
+      </c>
+      <c r="H9" t="s">
+        <v>55</v>
+      </c>
+      <c r="I9" t="s">
         <v>57</v>
       </c>
-      <c r="N8" s="1">
-        <v>46264</v>
-      </c>
-      <c r="Q8">
-        <v>-31</v>
-      </c>
-      <c r="R8">
-        <v>0</v>
-      </c>
-      <c r="S8" t="s">
+      <c r="J9" s="1">
+        <v>46205</v>
+      </c>
+      <c r="K9" s="1">
+        <v>46234</v>
+      </c>
+      <c r="L9">
+        <v>3</v>
+      </c>
+      <c r="M9" t="s">
         <v>58</v>
       </c>
-      <c r="W8" t="s">
-        <v>69</v>
-      </c>
-      <c r="AA8" t="b">
+      <c r="N9" s="1">
+        <v>46265</v>
+      </c>
+      <c r="Q9">
+        <v>-32</v>
+      </c>
+      <c r="R9">
+        <v>-1</v>
+      </c>
+      <c r="S9" t="s">
+        <v>59</v>
+      </c>
+      <c r="W9" t="s">
+        <v>68</v>
+      </c>
+      <c r="AA9" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (31/07/2026 05:11)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -689,10 +689,10 @@
         <v>46287</v>
       </c>
       <c r="Q2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="R2">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="S2" t="s">
         <v>59</v>
@@ -757,10 +757,10 @@
         <v>46243</v>
       </c>
       <c r="Q3">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="R3">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S3" t="s">
         <v>59</v>
@@ -825,10 +825,10 @@
         <v>46248</v>
       </c>
       <c r="Q4">
-        <v>-15</v>
+        <v>-14</v>
       </c>
       <c r="R4">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="S4" t="s">
         <v>59</v>
@@ -890,10 +890,10 @@
         <v>46249</v>
       </c>
       <c r="Q5">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="R5">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S5" t="s">
         <v>59</v>
@@ -958,10 +958,10 @@
         <v>46255</v>
       </c>
       <c r="Q6">
-        <v>-22</v>
+        <v>-21</v>
       </c>
       <c r="R6">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="S6" t="s">
         <v>59</v>
@@ -1023,10 +1023,10 @@
         <v>46265</v>
       </c>
       <c r="Q7">
-        <v>-32</v>
+        <v>-31</v>
       </c>
       <c r="R7">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="S7" t="s">
         <v>59</v>
@@ -1082,10 +1082,10 @@
         <v>46265</v>
       </c>
       <c r="Q8">
-        <v>-32</v>
+        <v>-31</v>
       </c>
       <c r="R8">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="S8" t="s">
         <v>59</v>
@@ -1141,10 +1141,10 @@
         <v>46265</v>
       </c>
       <c r="Q9">
-        <v>-32</v>
+        <v>-31</v>
       </c>
       <c r="R9">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="S9" t="s">
         <v>59</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (31/07/2026 14:01)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="69">
   <si>
     <t>om_emg</t>
   </si>
@@ -1031,6 +1031,9 @@
       <c r="S7" t="s">
         <v>59</v>
       </c>
+      <c r="T7" t="s">
+        <v>60</v>
+      </c>
       <c r="W7" t="s">
         <v>68</v>
       </c>
@@ -1090,6 +1093,9 @@
       <c r="S8" t="s">
         <v>59</v>
       </c>
+      <c r="T8" t="s">
+        <v>60</v>
+      </c>
       <c r="W8" t="s">
         <v>68</v>
       </c>
@@ -1148,6 +1154,9 @@
       </c>
       <c r="S9" t="s">
         <v>59</v>
+      </c>
+      <c r="T9" t="s">
+        <v>60</v>
       </c>
       <c r="W9" t="s">
         <v>68</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (03/08/2026 14:30)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="72">
   <si>
     <t>om_emg</t>
   </si>
@@ -205,19 +205,28 @@
     <t>Alterado o tipo da emerg. de IPLR para ANCE. Godoy 22/07/26</t>
   </si>
   <si>
+    <t>Atendido 01 EA através da TSP 18122931. Outros 02 EA serão enviados pela empresa. Ramon 03/08/26.</t>
+  </si>
+  <si>
     <t>Foi solicitado via email no dia 02-03-2 o atendimento do item com estoque FAB. Claudio -02-03-26 - Em resposta, a coordenadoria disse que o estque seria insuficiente. Foi verificado que na T.O da ANV o QPA para esse item são 2 EA, solicitei confirmação. - Cláudio -02-03-2026. Solicitado o cancelamento da emergência em função da quantidade cedida ao 2733 ter sido de 01ea. Considerando o QPA 02 ea. Encontra-se em tratativa junto a fiscalização e o gestor do contrato conforme mensagem de e-mail de 05/03. - SOLICITAÇÃO E-C98-26047.Colocado pedido AOG Textron WB0003068789 - previsão de entrega 60 dias em média. Os demais fornecedores informaram não ter em estoque ou não possuírem a certificação necessária da peça.</t>
   </si>
   <si>
-    <t>Colocado pedido junto ao fornecedor LEGACY PARTS, validando prazo de entrega em Miami. ATZ 28/07</t>
-  </si>
-  <si>
-    <t>Colocado pedido Textron IJ17575583 - entregue em Miami 15/07. Carga rercepcionada GIG 19/07 - Aguardando liberação do SEFAZ. ATZ 21/07 - material em processo de expedição RC 23/07/2026</t>
+    <t>Colocado pedido junto ao fornecedor LEGACY PARTS, previsão de entrega em Miami 05/08</t>
+  </si>
+  <si>
+    <t>Colocado pedido Textron IJ17575583 - entregue em Miami 15/07. Carga rercepcionada GIG 19/07 - Aguardando liberação do SEFAZ. ATZ 21/07 - material em processo de expedição RC 23/07/2026 - MATERIAL ENVIADO PELO RECIBO 639/FAB/26 AWB A SER GERADA NA GOLLOG</t>
   </si>
   <si>
     <t>Item em bancada porem em pessimo estado, foi solicitado recolhimento de mais unidades para envio a oficina para tentativa de reparo ATZ Marcio 17/7/26. Solicitado abertura de O.S. para 3EA do item no dia 16-07-26 via Email para a Coordenadoria - CLA-21-07-26</t>
   </si>
   <si>
-    <t>Pedido I816822 entregue em Miami 27/07. Consolidando próximo embarque GIG. ATZ 28/07</t>
+    <t>Pedido I816822 entregue em Miami 27/07. Previsão de chegada GIG 30/07 (voo 4208). Previsão de canal 31/07</t>
+  </si>
+  <si>
+    <t>Enviado para o Operador(02 EA), atendimento parcial, em 31/07/2026 - REZ - o outro 1 EA será atendido pelo estoque FAB. conforme solicitado por Email- CLA-03-08</t>
+  </si>
+  <si>
+    <t>Temos 4 EA em manutenção na William, será pedido prioridade. CLA-03-08</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -689,10 +698,10 @@
         <v>46287</v>
       </c>
       <c r="Q2">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="R2">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="S2" t="s">
         <v>59</v>
@@ -704,10 +713,10 @@
         <v>61</v>
       </c>
       <c r="V2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="W2" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -757,10 +766,10 @@
         <v>46243</v>
       </c>
       <c r="Q3">
-        <v>-9</v>
+        <v>-6</v>
       </c>
       <c r="R3">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="S3" t="s">
         <v>59</v>
@@ -769,10 +778,10 @@
         <v>60</v>
       </c>
       <c r="V3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="W3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -825,10 +834,10 @@
         <v>46248</v>
       </c>
       <c r="Q4">
-        <v>-14</v>
+        <v>-11</v>
       </c>
       <c r="R4">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="S4" t="s">
         <v>59</v>
@@ -837,10 +846,10 @@
         <v>60</v>
       </c>
       <c r="V4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="W4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -890,10 +899,10 @@
         <v>46249</v>
       </c>
       <c r="Q5">
-        <v>-15</v>
+        <v>-12</v>
       </c>
       <c r="R5">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="S5" t="s">
         <v>59</v>
@@ -905,10 +914,10 @@
         <v>62</v>
       </c>
       <c r="V5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="W5" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -958,10 +967,10 @@
         <v>46255</v>
       </c>
       <c r="Q6">
-        <v>-21</v>
+        <v>-18</v>
       </c>
       <c r="R6">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="S6" t="s">
         <v>59</v>
@@ -970,10 +979,10 @@
         <v>59</v>
       </c>
       <c r="V6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="W6" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1023,10 +1032,10 @@
         <v>46265</v>
       </c>
       <c r="Q7">
-        <v>-31</v>
+        <v>-28</v>
       </c>
       <c r="R7">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S7" t="s">
         <v>59</v>
@@ -1035,7 +1044,7 @@
         <v>60</v>
       </c>
       <c r="W7" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1085,10 +1094,10 @@
         <v>46265</v>
       </c>
       <c r="Q8">
-        <v>-31</v>
+        <v>-28</v>
       </c>
       <c r="R8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S8" t="s">
         <v>59</v>
@@ -1096,8 +1105,14 @@
       <c r="T8" t="s">
         <v>60</v>
       </c>
+      <c r="U8" t="s">
+        <v>63</v>
+      </c>
+      <c r="V8" t="s">
+        <v>69</v>
+      </c>
       <c r="W8" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1147,10 +1162,10 @@
         <v>46265</v>
       </c>
       <c r="Q9">
-        <v>-31</v>
+        <v>-28</v>
       </c>
       <c r="R9">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S9" t="s">
         <v>59</v>
@@ -1158,8 +1173,11 @@
       <c r="T9" t="s">
         <v>60</v>
       </c>
+      <c r="V9" t="s">
+        <v>70</v>
+      </c>
       <c r="W9" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (04/08/2026 05:11)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -698,10 +698,10 @@
         <v>46287</v>
       </c>
       <c r="Q2">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="R2">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S2" t="s">
         <v>59</v>
@@ -766,10 +766,10 @@
         <v>46243</v>
       </c>
       <c r="Q3">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R3">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="S3" t="s">
         <v>59</v>
@@ -834,10 +834,10 @@
         <v>46248</v>
       </c>
       <c r="Q4">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R4">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="S4" t="s">
         <v>59</v>
@@ -899,10 +899,10 @@
         <v>46249</v>
       </c>
       <c r="Q5">
-        <v>-12</v>
+        <v>-11</v>
       </c>
       <c r="R5">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="S5" t="s">
         <v>59</v>
@@ -967,10 +967,10 @@
         <v>46255</v>
       </c>
       <c r="Q6">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="R6">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S6" t="s">
         <v>59</v>
@@ -1032,10 +1032,10 @@
         <v>46265</v>
       </c>
       <c r="Q7">
-        <v>-28</v>
+        <v>-27</v>
       </c>
       <c r="R7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S7" t="s">
         <v>59</v>
@@ -1094,10 +1094,10 @@
         <v>46265</v>
       </c>
       <c r="Q8">
-        <v>-28</v>
+        <v>-27</v>
       </c>
       <c r="R8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S8" t="s">
         <v>59</v>
@@ -1162,10 +1162,10 @@
         <v>46265</v>
       </c>
       <c r="Q9">
-        <v>-28</v>
+        <v>-27</v>
       </c>
       <c r="R9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S9" t="s">
         <v>59</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (04/08/2026 14:16)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="79">
   <si>
     <t>om_emg</t>
   </si>
@@ -130,6 +130,12 @@
     <t>313260018658</t>
   </si>
   <si>
+    <t>329260019260</t>
+  </si>
+  <si>
+    <t>329260019261</t>
+  </si>
+  <si>
     <t>1214134-1</t>
   </si>
   <si>
@@ -151,6 +157,12 @@
     <t>324843-W020</t>
   </si>
   <si>
+    <t>068-02800</t>
+  </si>
+  <si>
+    <t>C668050-1108</t>
+  </si>
+  <si>
     <t>BELLCRANK ASSY</t>
   </si>
   <si>
@@ -169,6 +181,12 @@
     <t>HEADSET-MICROPHONE</t>
   </si>
   <si>
+    <t>INSULATOR</t>
+  </si>
+  <si>
+    <t>TRANSMITTER FUEL</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -188,6 +206,9 @@
   </si>
   <si>
     <t>ANCE</t>
+  </si>
+  <si>
+    <t>AIFP</t>
   </si>
   <si>
     <t>EA</t>
@@ -565,7 +586,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA9"/>
+  <dimension ref="A1:AA11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -662,22 +683,22 @@
         <v>30</v>
       </c>
       <c r="D2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F2" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="G2">
         <v>2730</v>
       </c>
       <c r="H2" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="I2" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="J2" s="1">
         <v>46076</v>
@@ -689,7 +710,7 @@
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="N2" s="1">
         <v>46091</v>
@@ -704,19 +725,19 @@
         <v>158</v>
       </c>
       <c r="S2" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="T2" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="U2" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="V2" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="W2" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -733,22 +754,22 @@
         <v>31</v>
       </c>
       <c r="D3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E3" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F3" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="G3">
         <v>2702</v>
       </c>
       <c r="H3" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="I3" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="J3" s="1">
         <v>46212</v>
@@ -760,7 +781,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="N3" s="1">
         <v>46243</v>
@@ -772,16 +793,16 @@
         <v>26</v>
       </c>
       <c r="S3" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="T3" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="V3" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="W3" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -798,22 +819,22 @@
         <v>32</v>
       </c>
       <c r="D4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E4" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F4" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="G4">
         <v>2736</v>
       </c>
       <c r="H4" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="I4" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="J4" s="1">
         <v>46216</v>
@@ -825,7 +846,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="N4" s="1">
         <v>46248</v>
@@ -840,16 +861,16 @@
         <v>21</v>
       </c>
       <c r="S4" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="T4" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="V4" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="W4" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -866,22 +887,22 @@
         <v>33</v>
       </c>
       <c r="D5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E5" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F5" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="G5">
         <v>2722</v>
       </c>
       <c r="H5" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="I5" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="J5" s="1">
         <v>46219</v>
@@ -893,7 +914,7 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="N5" s="1">
         <v>46249</v>
@@ -905,19 +926,19 @@
         <v>20</v>
       </c>
       <c r="S5" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="T5" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="U5" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="V5" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="W5" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -934,22 +955,22 @@
         <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E6" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F6" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="G6">
         <v>2720</v>
       </c>
       <c r="H6" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="I6" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="J6" s="1">
         <v>46220</v>
@@ -961,7 +982,7 @@
         <v>10</v>
       </c>
       <c r="M6" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="N6" s="1">
         <v>46255</v>
@@ -973,16 +994,16 @@
         <v>14</v>
       </c>
       <c r="S6" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="T6" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="V6" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="W6" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -999,22 +1020,22 @@
         <v>35</v>
       </c>
       <c r="D7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E7" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F7" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="G7">
         <v>2741</v>
       </c>
       <c r="H7" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="I7" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="J7" s="1">
         <v>46231</v>
@@ -1026,7 +1047,7 @@
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="N7" s="1">
         <v>46265</v>
@@ -1038,13 +1059,13 @@
         <v>4</v>
       </c>
       <c r="S7" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="T7" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="W7" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1061,22 +1082,22 @@
         <v>36</v>
       </c>
       <c r="D8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E8" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="F8" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="G8">
         <v>2736</v>
       </c>
       <c r="H8" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="I8" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="J8" s="1">
         <v>46205</v>
@@ -1088,7 +1109,7 @@
         <v>3</v>
       </c>
       <c r="M8" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="N8" s="1">
         <v>46265</v>
@@ -1100,19 +1121,19 @@
         <v>4</v>
       </c>
       <c r="S8" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="T8" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="U8" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="V8" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="W8" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1129,22 +1150,22 @@
         <v>37</v>
       </c>
       <c r="D9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E9" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="F9" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="G9">
         <v>2737</v>
       </c>
       <c r="H9" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="I9" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="J9" s="1">
         <v>46205</v>
@@ -1156,7 +1177,7 @@
         <v>3</v>
       </c>
       <c r="M9" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="N9" s="1">
         <v>46265</v>
@@ -1168,18 +1189,142 @@
         <v>4</v>
       </c>
       <c r="S9" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="T9" t="s">
+        <v>67</v>
+      </c>
+      <c r="V9" t="s">
+        <v>77</v>
+      </c>
+      <c r="W9" t="s">
+        <v>78</v>
+      </c>
+      <c r="AA9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27">
+      <c r="A10">
+        <v>329</v>
+      </c>
+      <c r="B10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" t="s">
+        <v>55</v>
+      </c>
+      <c r="F10" t="s">
+        <v>57</v>
+      </c>
+      <c r="G10">
+        <v>2709</v>
+      </c>
+      <c r="H10" t="s">
         <v>60</v>
       </c>
-      <c r="V9" t="s">
-        <v>70</v>
-      </c>
-      <c r="W9" t="s">
-        <v>71</v>
-      </c>
-      <c r="AA9" t="b">
+      <c r="I10" t="s">
+        <v>62</v>
+      </c>
+      <c r="J10" s="1">
+        <v>46237</v>
+      </c>
+      <c r="K10" s="1">
+        <v>46238</v>
+      </c>
+      <c r="L10">
+        <v>2</v>
+      </c>
+      <c r="M10" t="s">
+        <v>65</v>
+      </c>
+      <c r="N10" s="1">
+        <v>46249</v>
+      </c>
+      <c r="Q10">
+        <v>-11</v>
+      </c>
+      <c r="R10">
+        <v>0</v>
+      </c>
+      <c r="S10" t="s">
+        <v>67</v>
+      </c>
+      <c r="T10" t="s">
+        <v>66</v>
+      </c>
+      <c r="W10" t="s">
+        <v>78</v>
+      </c>
+      <c r="AA10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27">
+      <c r="A11">
+        <v>329</v>
+      </c>
+      <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" t="s">
+        <v>48</v>
+      </c>
+      <c r="E11" t="s">
+        <v>56</v>
+      </c>
+      <c r="F11" t="s">
+        <v>57</v>
+      </c>
+      <c r="G11">
+        <v>2720</v>
+      </c>
+      <c r="H11" t="s">
+        <v>60</v>
+      </c>
+      <c r="I11" t="s">
+        <v>64</v>
+      </c>
+      <c r="J11" s="1">
+        <v>46238</v>
+      </c>
+      <c r="K11" s="1">
+        <v>46238</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11" t="s">
+        <v>65</v>
+      </c>
+      <c r="N11" s="1">
+        <v>46245</v>
+      </c>
+      <c r="Q11">
+        <v>-7</v>
+      </c>
+      <c r="R11">
+        <v>0</v>
+      </c>
+      <c r="S11" t="s">
+        <v>66</v>
+      </c>
+      <c r="T11" t="s">
+        <v>66</v>
+      </c>
+      <c r="W11" t="s">
+        <v>78</v>
+      </c>
+      <c r="AA11" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (05/08/2026 05:09)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -719,10 +719,10 @@
         <v>46287</v>
       </c>
       <c r="Q2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="R2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S2" t="s">
         <v>66</v>
@@ -787,10 +787,10 @@
         <v>46243</v>
       </c>
       <c r="Q3">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R3">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S3" t="s">
         <v>66</v>
@@ -855,10 +855,10 @@
         <v>46248</v>
       </c>
       <c r="Q4">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="R4">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S4" t="s">
         <v>66</v>
@@ -920,10 +920,10 @@
         <v>46249</v>
       </c>
       <c r="Q5">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R5">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="S5" t="s">
         <v>66</v>
@@ -988,10 +988,10 @@
         <v>46255</v>
       </c>
       <c r="Q6">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="R6">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S6" t="s">
         <v>66</v>
@@ -1053,10 +1053,10 @@
         <v>46265</v>
       </c>
       <c r="Q7">
-        <v>-27</v>
+        <v>-26</v>
       </c>
       <c r="R7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S7" t="s">
         <v>66</v>
@@ -1115,10 +1115,10 @@
         <v>46265</v>
       </c>
       <c r="Q8">
-        <v>-27</v>
+        <v>-26</v>
       </c>
       <c r="R8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S8" t="s">
         <v>66</v>
@@ -1183,10 +1183,10 @@
         <v>46265</v>
       </c>
       <c r="Q9">
-        <v>-27</v>
+        <v>-26</v>
       </c>
       <c r="R9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S9" t="s">
         <v>66</v>
@@ -1248,10 +1248,10 @@
         <v>46249</v>
       </c>
       <c r="Q10">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S10" t="s">
         <v>67</v>
@@ -1310,10 +1310,10 @@
         <v>46245</v>
       </c>
       <c r="Q11">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S11" t="s">
         <v>66</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (05/08/2026 10:00)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="72">
   <si>
     <t>om_emg</t>
   </si>
@@ -130,12 +130,6 @@
     <t>313260018658</t>
   </si>
   <si>
-    <t>329260019260</t>
-  </si>
-  <si>
-    <t>329260019261</t>
-  </si>
-  <si>
     <t>1214134-1</t>
   </si>
   <si>
@@ -157,12 +151,6 @@
     <t>324843-W020</t>
   </si>
   <si>
-    <t>068-02800</t>
-  </si>
-  <si>
-    <t>C668050-1108</t>
-  </si>
-  <si>
     <t>BELLCRANK ASSY</t>
   </si>
   <si>
@@ -181,12 +169,6 @@
     <t>HEADSET-MICROPHONE</t>
   </si>
   <si>
-    <t>INSULATOR</t>
-  </si>
-  <si>
-    <t>TRANSMITTER FUEL</t>
-  </si>
-  <si>
     <t>C</t>
   </si>
   <si>
@@ -208,9 +190,6 @@
     <t>ANCE</t>
   </si>
   <si>
-    <t>AIFP</t>
-  </si>
-  <si>
     <t>EA</t>
   </si>
   <si>
@@ -235,19 +214,19 @@
     <t>Colocado pedido junto ao fornecedor LEGACY PARTS, previsão de entrega em Miami 05/08</t>
   </si>
   <si>
-    <t>Colocado pedido Textron IJ17575583 - entregue em Miami 15/07. Carga rercepcionada GIG 19/07 - Aguardando liberação do SEFAZ. ATZ 21/07 - material em processo de expedição RC 23/07/2026 - MATERIAL ENVIADO PELO RECIBO 639/FAB/26 AWB A SER GERADA NA GOLLOG</t>
+    <t>Colocado pedido Textron IJ17575583 - entregue em Miami 15/07. Carga rercepcionada GIG 19/07 - Aguardando liberação do SEFAZ. ATZ 21/07 - material em processo de expedição RC 23/07/2026 - MATERIAL ENVIADO PELO RECIBO 639/FAB/26 AWB A SER GERADA</t>
   </si>
   <si>
     <t>Item em bancada porem em pessimo estado, foi solicitado recolhimento de mais unidades para envio a oficina para tentativa de reparo ATZ Marcio 17/7/26. Solicitado abertura de O.S. para 3EA do item no dia 16-07-26 via Email para a Coordenadoria - CLA-21-07-26</t>
   </si>
   <si>
-    <t>Pedido I816822 entregue em Miami 27/07. Previsão de chegada GIG 30/07 (voo 4208). Previsão de canal 31/07</t>
-  </si>
-  <si>
-    <t>Enviado para o Operador(02 EA), atendimento parcial, em 31/07/2026 - REZ - o outro 1 EA será atendido pelo estoque FAB. conforme solicitado por Email- CLA-03-08</t>
-  </si>
-  <si>
-    <t>Temos 4 EA em manutenção na William, será pedido prioridade. CLA-03-08</t>
+    <t>Pedido I816822 entregue em Miami 27/07. Previsão de chegada GIG 30/07 (voo 4208). Previsão de canal 31/07 - MATERIAL RECEBIDO NA VEE ONE, EM PROCESSO DE EXPEDIÇÃO 04/08/2026 - ATZ RC</t>
+  </si>
+  <si>
+    <t>item sendo preparado para transporte - CLA-03-08- AWB 127-5082 1282- CLA-04-08</t>
+  </si>
+  <si>
+    <t>Enviado para o Operador(02 EA), atendimento parcial, em 31/07/2026 -AWB 127-5041 6833- REZ - o outro 1 EA será atendido pelo estoque FAB. conforme solicitado por Email- CLA-03-08 - AWB 127-5082 1282 -1 EA ENVIADO ESTOQUE FAB</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -586,7 +565,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA11"/>
+  <dimension ref="A1:AA9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -683,22 +662,22 @@
         <v>30</v>
       </c>
       <c r="D2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="F2" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="G2">
         <v>2730</v>
       </c>
       <c r="H2" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="I2" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="J2" s="1">
         <v>46076</v>
@@ -710,7 +689,7 @@
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="N2" s="1">
         <v>46091</v>
@@ -725,19 +704,19 @@
         <v>159</v>
       </c>
       <c r="S2" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="T2" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="U2" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="V2" t="s">
+        <v>64</v>
+      </c>
+      <c r="W2" t="s">
         <v>71</v>
-      </c>
-      <c r="W2" t="s">
-        <v>78</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -754,22 +733,22 @@
         <v>31</v>
       </c>
       <c r="D3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E3" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="F3" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="G3">
         <v>2702</v>
       </c>
       <c r="H3" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="I3" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="J3" s="1">
         <v>46212</v>
@@ -781,7 +760,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="N3" s="1">
         <v>46243</v>
@@ -793,16 +772,16 @@
         <v>27</v>
       </c>
       <c r="S3" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="T3" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="V3" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="W3" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -819,22 +798,22 @@
         <v>32</v>
       </c>
       <c r="D4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E4" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="F4" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="G4">
         <v>2736</v>
       </c>
       <c r="H4" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="I4" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="J4" s="1">
         <v>46216</v>
@@ -846,7 +825,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="N4" s="1">
         <v>46248</v>
@@ -861,16 +840,16 @@
         <v>22</v>
       </c>
       <c r="S4" t="s">
+        <v>59</v>
+      </c>
+      <c r="T4" t="s">
+        <v>60</v>
+      </c>
+      <c r="V4" t="s">
         <v>66</v>
       </c>
-      <c r="T4" t="s">
-        <v>67</v>
-      </c>
-      <c r="V4" t="s">
-        <v>73</v>
-      </c>
       <c r="W4" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -887,22 +866,22 @@
         <v>33</v>
       </c>
       <c r="D5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E5" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F5" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="G5">
         <v>2722</v>
       </c>
       <c r="H5" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="I5" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="J5" s="1">
         <v>46219</v>
@@ -914,7 +893,7 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="N5" s="1">
         <v>46249</v>
@@ -926,19 +905,19 @@
         <v>21</v>
       </c>
       <c r="S5" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="T5" t="s">
+        <v>60</v>
+      </c>
+      <c r="U5" t="s">
+        <v>62</v>
+      </c>
+      <c r="V5" t="s">
         <v>67</v>
       </c>
-      <c r="U5" t="s">
-        <v>69</v>
-      </c>
-      <c r="V5" t="s">
-        <v>74</v>
-      </c>
       <c r="W5" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -955,22 +934,22 @@
         <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E6" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F6" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="G6">
         <v>2720</v>
       </c>
       <c r="H6" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="I6" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="J6" s="1">
         <v>46220</v>
@@ -982,11 +961,14 @@
         <v>10</v>
       </c>
       <c r="M6" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="N6" s="1">
         <v>46255</v>
       </c>
+      <c r="O6" s="1">
+        <v>46240</v>
+      </c>
       <c r="Q6">
         <v>-16</v>
       </c>
@@ -994,16 +976,16 @@
         <v>15</v>
       </c>
       <c r="S6" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="T6" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="V6" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="W6" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1020,22 +1002,22 @@
         <v>35</v>
       </c>
       <c r="D7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E7" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F7" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="G7">
         <v>2741</v>
       </c>
       <c r="H7" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="I7" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="J7" s="1">
         <v>46231</v>
@@ -1047,11 +1029,14 @@
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="N7" s="1">
         <v>46265</v>
       </c>
+      <c r="O7" s="1">
+        <v>46239</v>
+      </c>
       <c r="Q7">
         <v>-26</v>
       </c>
@@ -1059,13 +1044,16 @@
         <v>5</v>
       </c>
       <c r="S7" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="T7" t="s">
-        <v>67</v>
+        <v>60</v>
+      </c>
+      <c r="V7" t="s">
+        <v>69</v>
       </c>
       <c r="W7" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1082,22 +1070,22 @@
         <v>36</v>
       </c>
       <c r="D8" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E8" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F8" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="G8">
         <v>2736</v>
       </c>
       <c r="H8" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="I8" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="J8" s="1">
         <v>46205</v>
@@ -1109,11 +1097,14 @@
         <v>3</v>
       </c>
       <c r="M8" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="N8" s="1">
         <v>46265</v>
       </c>
+      <c r="O8" s="1">
+        <v>46239</v>
+      </c>
       <c r="Q8">
         <v>-26</v>
       </c>
@@ -1121,19 +1112,19 @@
         <v>5</v>
       </c>
       <c r="S8" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="T8" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="U8" t="s">
+        <v>63</v>
+      </c>
+      <c r="V8" t="s">
         <v>70</v>
       </c>
-      <c r="V8" t="s">
-        <v>76</v>
-      </c>
       <c r="W8" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1150,22 +1141,22 @@
         <v>37</v>
       </c>
       <c r="D9" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E9" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F9" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="G9">
         <v>2737</v>
       </c>
       <c r="H9" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="I9" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="J9" s="1">
         <v>46205</v>
@@ -1177,7 +1168,7 @@
         <v>3</v>
       </c>
       <c r="M9" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="N9" s="1">
         <v>46265</v>
@@ -1189,142 +1180,15 @@
         <v>5</v>
       </c>
       <c r="S9" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="T9" t="s">
-        <v>67</v>
-      </c>
-      <c r="V9" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="W9" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="AA9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:27">
-      <c r="A10">
-        <v>329</v>
-      </c>
-      <c r="B10" t="s">
-        <v>29</v>
-      </c>
-      <c r="C10" t="s">
-        <v>38</v>
-      </c>
-      <c r="D10" t="s">
-        <v>47</v>
-      </c>
-      <c r="E10" t="s">
-        <v>55</v>
-      </c>
-      <c r="F10" t="s">
-        <v>57</v>
-      </c>
-      <c r="G10">
-        <v>2709</v>
-      </c>
-      <c r="H10" t="s">
-        <v>60</v>
-      </c>
-      <c r="I10" t="s">
-        <v>62</v>
-      </c>
-      <c r="J10" s="1">
-        <v>46237</v>
-      </c>
-      <c r="K10" s="1">
-        <v>46238</v>
-      </c>
-      <c r="L10">
-        <v>2</v>
-      </c>
-      <c r="M10" t="s">
-        <v>65</v>
-      </c>
-      <c r="N10" s="1">
-        <v>46249</v>
-      </c>
-      <c r="Q10">
-        <v>-10</v>
-      </c>
-      <c r="R10">
-        <v>1</v>
-      </c>
-      <c r="S10" t="s">
-        <v>67</v>
-      </c>
-      <c r="T10" t="s">
-        <v>66</v>
-      </c>
-      <c r="W10" t="s">
-        <v>78</v>
-      </c>
-      <c r="AA10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:27">
-      <c r="A11">
-        <v>329</v>
-      </c>
-      <c r="B11" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" t="s">
-        <v>39</v>
-      </c>
-      <c r="D11" t="s">
-        <v>48</v>
-      </c>
-      <c r="E11" t="s">
-        <v>56</v>
-      </c>
-      <c r="F11" t="s">
-        <v>57</v>
-      </c>
-      <c r="G11">
-        <v>2720</v>
-      </c>
-      <c r="H11" t="s">
-        <v>60</v>
-      </c>
-      <c r="I11" t="s">
-        <v>64</v>
-      </c>
-      <c r="J11" s="1">
-        <v>46238</v>
-      </c>
-      <c r="K11" s="1">
-        <v>46238</v>
-      </c>
-      <c r="L11">
-        <v>1</v>
-      </c>
-      <c r="M11" t="s">
-        <v>65</v>
-      </c>
-      <c r="N11" s="1">
-        <v>46245</v>
-      </c>
-      <c r="Q11">
-        <v>-6</v>
-      </c>
-      <c r="R11">
-        <v>1</v>
-      </c>
-      <c r="S11" t="s">
-        <v>66</v>
-      </c>
-      <c r="T11" t="s">
-        <v>66</v>
-      </c>
-      <c r="W11" t="s">
-        <v>78</v>
-      </c>
-      <c r="AA11" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (05/08/2026 12:22)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="76">
   <si>
     <t>om_emg</t>
   </si>
@@ -106,6 +106,9 @@
     <t>BABR</t>
   </si>
   <si>
+    <t>BABE</t>
+  </si>
+  <si>
     <t>313260017747</t>
   </si>
   <si>
@@ -130,6 +133,9 @@
     <t>313260018658</t>
   </si>
   <si>
+    <t>396260016580</t>
+  </si>
+  <si>
     <t>1214134-1</t>
   </si>
   <si>
@@ -151,6 +157,9 @@
     <t>324843-W020</t>
   </si>
   <si>
+    <t>2601188-204</t>
+  </si>
+  <si>
     <t>BELLCRANK ASSY</t>
   </si>
   <si>
@@ -167,6 +176,9 @@
   </si>
   <si>
     <t>HEADSET-MICROPHONE</t>
+  </si>
+  <si>
+    <t>COMPRESSOR DRIVE ASS</t>
   </si>
   <si>
     <t>C</t>
@@ -565,7 +577,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA9"/>
+  <dimension ref="A1:AA10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -659,25 +671,25 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F2" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G2">
         <v>2730</v>
       </c>
       <c r="H2" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="I2" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="J2" s="1">
         <v>46076</v>
@@ -689,7 +701,7 @@
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="N2" s="1">
         <v>46091</v>
@@ -704,19 +716,19 @@
         <v>159</v>
       </c>
       <c r="S2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="T2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="U2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="V2" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="W2" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -730,25 +742,25 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F3" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G3">
         <v>2702</v>
       </c>
       <c r="H3" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="I3" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J3" s="1">
         <v>46212</v>
@@ -760,7 +772,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="N3" s="1">
         <v>46243</v>
@@ -772,16 +784,16 @@
         <v>27</v>
       </c>
       <c r="S3" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="T3" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="V3" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="W3" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -795,25 +807,25 @@
         <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E4" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F4" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G4">
         <v>2736</v>
       </c>
       <c r="H4" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="I4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J4" s="1">
         <v>46216</v>
@@ -825,7 +837,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="N4" s="1">
         <v>46248</v>
@@ -840,16 +852,16 @@
         <v>22</v>
       </c>
       <c r="S4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="T4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="V4" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="W4" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -863,25 +875,25 @@
         <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E5" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="F5" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="G5">
         <v>2722</v>
       </c>
       <c r="H5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="I5" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J5" s="1">
         <v>46219</v>
@@ -893,7 +905,7 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="N5" s="1">
         <v>46249</v>
@@ -905,19 +917,19 @@
         <v>21</v>
       </c>
       <c r="S5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="T5" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="U5" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="V5" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="W5" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -931,25 +943,25 @@
         <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E6" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F6" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G6">
         <v>2720</v>
       </c>
       <c r="H6" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="I6" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J6" s="1">
         <v>46220</v>
@@ -961,7 +973,7 @@
         <v>10</v>
       </c>
       <c r="M6" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="N6" s="1">
         <v>46255</v>
@@ -976,16 +988,16 @@
         <v>15</v>
       </c>
       <c r="S6" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="T6" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="V6" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="W6" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -999,25 +1011,25 @@
         <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E7" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="F7" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="G7">
         <v>2741</v>
       </c>
       <c r="H7" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="I7" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J7" s="1">
         <v>46231</v>
@@ -1029,7 +1041,7 @@
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="N7" s="1">
         <v>46265</v>
@@ -1044,16 +1056,16 @@
         <v>5</v>
       </c>
       <c r="S7" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="T7" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="V7" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="W7" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1067,25 +1079,25 @@
         <v>27</v>
       </c>
       <c r="C8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E8" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="F8" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G8">
         <v>2736</v>
       </c>
       <c r="H8" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="I8" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J8" s="1">
         <v>46205</v>
@@ -1097,7 +1109,7 @@
         <v>3</v>
       </c>
       <c r="M8" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="N8" s="1">
         <v>46265</v>
@@ -1112,19 +1124,19 @@
         <v>5</v>
       </c>
       <c r="S8" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="T8" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="U8" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="V8" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="W8" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1138,25 +1150,25 @@
         <v>27</v>
       </c>
       <c r="C9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E9" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="F9" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G9">
         <v>2737</v>
       </c>
       <c r="H9" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="I9" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J9" s="1">
         <v>46205</v>
@@ -1168,7 +1180,7 @@
         <v>3</v>
       </c>
       <c r="M9" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="N9" s="1">
         <v>46265</v>
@@ -1180,15 +1192,74 @@
         <v>5</v>
       </c>
       <c r="S9" t="s">
+        <v>63</v>
+      </c>
+      <c r="T9" t="s">
+        <v>64</v>
+      </c>
+      <c r="W9" t="s">
+        <v>75</v>
+      </c>
+      <c r="AA9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27">
+      <c r="A10">
+        <v>396</v>
+      </c>
+      <c r="B10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" t="s">
+        <v>54</v>
+      </c>
+      <c r="F10" t="s">
+        <v>55</v>
+      </c>
+      <c r="G10">
+        <v>2733</v>
+      </c>
+      <c r="H10" t="s">
         <v>59</v>
       </c>
-      <c r="T9" t="s">
-        <v>60</v>
-      </c>
-      <c r="W9" t="s">
-        <v>71</v>
-      </c>
-      <c r="AA9" t="b">
+      <c r="I10" t="s">
+        <v>61</v>
+      </c>
+      <c r="J10" s="1">
+        <v>46238</v>
+      </c>
+      <c r="K10" s="1">
+        <v>46235</v>
+      </c>
+      <c r="L10">
+        <v>1</v>
+      </c>
+      <c r="M10" t="s">
+        <v>62</v>
+      </c>
+      <c r="N10" s="1">
+        <v>46266</v>
+      </c>
+      <c r="Q10">
+        <v>-27</v>
+      </c>
+      <c r="R10">
+        <v>4</v>
+      </c>
+      <c r="S10" t="s">
+        <v>63</v>
+      </c>
+      <c r="W10" t="s">
+        <v>75</v>
+      </c>
+      <c r="AA10" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (05/08/2026 15:41)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -220,10 +220,10 @@
     <t>Atendido 01 EA através da TSP 18122931. Outros 02 EA serão enviados pela empresa. Ramon 03/08/26.</t>
   </si>
   <si>
-    <t>Foi solicitado via email no dia 02-03-2 o atendimento do item com estoque FAB. Claudio -02-03-26 - Em resposta, a coordenadoria disse que o estque seria insuficiente. Foi verificado que na T.O da ANV o QPA para esse item são 2 EA, solicitei confirmação. - Cláudio -02-03-2026. Solicitado o cancelamento da emergência em função da quantidade cedida ao 2733 ter sido de 01ea. Considerando o QPA 02 ea. Encontra-se em tratativa junto a fiscalização e o gestor do contrato conforme mensagem de e-mail de 05/03. - SOLICITAÇÃO E-C98-26047.Colocado pedido AOG Textron WB0003068789 - previsão de entrega 60 dias em média. Os demais fornecedores informaram não ter em estoque ou não possuírem a certificação necessária da peça.</t>
-  </si>
-  <si>
-    <t>Colocado pedido junto ao fornecedor LEGACY PARTS, previsão de entrega em Miami 05/08</t>
+    <t>Foi solicitado via email no dia 02-03-2 o atendimento do item com estoque FAB. Claudio -02-03-26 - Em resposta, a coordenadoria disse que o estque seria insuficiente. Foi verificado que na T.O da ANV o QPA para esse item são 2 EA, solicitei confirmação. - Cláudio -02-03-2026. Solicitado o cancelamento da emergência em função da quantidade cedida ao 2733 ter sido de 01ea. Considerando o QPA 02 ea. Encontra-se em tratativa junto a fiscalização e o gestor do contrato conforme mensagem de e-mail de 05/03. - SOLICITAÇÃO E-C98-26047.Colocado pedido AOG Textron J17626242 - previsão de entrega em Miami 05/08</t>
+  </si>
+  <si>
+    <t>Colocado pedido junto ao fornecedor LEGACY PARTS, previsão de entrega em Miami 06/08</t>
   </si>
   <si>
     <t>Colocado pedido Textron IJ17575583 - entregue em Miami 15/07. Carga rercepcionada GIG 19/07 - Aguardando liberação do SEFAZ. ATZ 21/07 - material em processo de expedição RC 23/07/2026 - MATERIAL ENVIADO PELO RECIBO 639/FAB/26 AWB A SER GERADA</t>

</xml_diff>

<commit_message>
Atualização automática: emergencias (06/08/2026 10:01)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -710,10 +710,10 @@
         <v>46287</v>
       </c>
       <c r="Q2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="R2">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="S2" t="s">
         <v>63</v>
@@ -778,10 +778,10 @@
         <v>46243</v>
       </c>
       <c r="Q3">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R3">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="S3" t="s">
         <v>63</v>
@@ -846,10 +846,10 @@
         <v>46248</v>
       </c>
       <c r="Q4">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="R4">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="S4" t="s">
         <v>63</v>
@@ -911,10 +911,10 @@
         <v>46249</v>
       </c>
       <c r="Q5">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="R5">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S5" t="s">
         <v>63</v>
@@ -982,10 +982,10 @@
         <v>46240</v>
       </c>
       <c r="Q6">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="R6">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S6" t="s">
         <v>63</v>
@@ -1050,10 +1050,10 @@
         <v>46239</v>
       </c>
       <c r="Q7">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="R7">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S7" t="s">
         <v>63</v>
@@ -1118,10 +1118,10 @@
         <v>46239</v>
       </c>
       <c r="Q8">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="R8">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S8" t="s">
         <v>63</v>
@@ -1186,10 +1186,10 @@
         <v>46265</v>
       </c>
       <c r="Q9">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="R9">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S9" t="s">
         <v>63</v>
@@ -1248,10 +1248,10 @@
         <v>46266</v>
       </c>
       <c r="Q10">
-        <v>-27</v>
+        <v>-26</v>
       </c>
       <c r="R10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S10" t="s">
         <v>63</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (06/08/2026 21:44)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -1236,7 +1236,7 @@
         <v>46238</v>
       </c>
       <c r="K10" s="1">
-        <v>46235</v>
+        <v>46238</v>
       </c>
       <c r="L10">
         <v>1</v>
@@ -1245,13 +1245,13 @@
         <v>62</v>
       </c>
       <c r="N10" s="1">
-        <v>46266</v>
+        <v>46269</v>
       </c>
       <c r="Q10">
-        <v>-26</v>
+        <v>-29</v>
       </c>
       <c r="R10">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="S10" t="s">
         <v>63</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (07/08/2026 08:51)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -710,10 +710,10 @@
         <v>46287</v>
       </c>
       <c r="Q2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="R2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="S2" t="s">
         <v>63</v>
@@ -778,10 +778,10 @@
         <v>46243</v>
       </c>
       <c r="Q3">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R3">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S3" t="s">
         <v>63</v>
@@ -846,10 +846,10 @@
         <v>46248</v>
       </c>
       <c r="Q4">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="R4">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="S4" t="s">
         <v>63</v>
@@ -911,10 +911,10 @@
         <v>46249</v>
       </c>
       <c r="Q5">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="R5">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="S5" t="s">
         <v>63</v>
@@ -982,10 +982,10 @@
         <v>46240</v>
       </c>
       <c r="Q6">
-        <v>-15</v>
+        <v>-14</v>
       </c>
       <c r="R6">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="S6" t="s">
         <v>63</v>
@@ -1050,10 +1050,10 @@
         <v>46239</v>
       </c>
       <c r="Q7">
-        <v>-25</v>
+        <v>-24</v>
       </c>
       <c r="R7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S7" t="s">
         <v>63</v>
@@ -1118,10 +1118,10 @@
         <v>46239</v>
       </c>
       <c r="Q8">
-        <v>-25</v>
+        <v>-24</v>
       </c>
       <c r="R8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S8" t="s">
         <v>63</v>
@@ -1186,10 +1186,10 @@
         <v>46265</v>
       </c>
       <c r="Q9">
-        <v>-25</v>
+        <v>-24</v>
       </c>
       <c r="R9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S9" t="s">
         <v>63</v>
@@ -1248,10 +1248,10 @@
         <v>46269</v>
       </c>
       <c r="Q10">
-        <v>-29</v>
+        <v>-28</v>
       </c>
       <c r="R10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S10" t="s">
         <v>63</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (07/08/2026 13:02)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="81">
   <si>
     <t>om_emg</t>
   </si>
@@ -136,6 +136,9 @@
     <t>396260016580</t>
   </si>
   <si>
+    <t>329260019264</t>
+  </si>
+  <si>
     <t>1214134-1</t>
   </si>
   <si>
@@ -160,6 +163,9 @@
     <t>2601188-204</t>
   </si>
   <si>
+    <t>C662041-0102</t>
+  </si>
+  <si>
     <t>BELLCRANK ASSY</t>
   </si>
   <si>
@@ -181,6 +187,9 @@
     <t>COMPRESSOR DRIVE ASS</t>
   </si>
   <si>
+    <t>INDICATOR FUEL</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -193,6 +202,9 @@
     <t>Providência tomada</t>
   </si>
   <si>
+    <t>Atendido parcialmente</t>
+  </si>
+  <si>
     <t>Aguardando solução</t>
   </si>
   <si>
@@ -200,6 +212,9 @@
   </si>
   <si>
     <t>ANCE</t>
+  </si>
+  <si>
+    <t>AIFP</t>
   </si>
   <si>
     <t>EA</t>
@@ -577,7 +592,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA10"/>
+  <dimension ref="A1:AA11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -674,22 +689,22 @@
         <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G2">
         <v>2730</v>
       </c>
       <c r="H2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="J2" s="1">
         <v>46076</v>
@@ -701,7 +716,7 @@
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="N2" s="1">
         <v>46091</v>
@@ -716,19 +731,19 @@
         <v>161</v>
       </c>
       <c r="S2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="T2" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="U2" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="V2" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="W2" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -745,22 +760,22 @@
         <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G3">
         <v>2702</v>
       </c>
       <c r="H3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="J3" s="1">
         <v>46212</v>
@@ -772,7 +787,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="N3" s="1">
         <v>46243</v>
@@ -784,16 +799,16 @@
         <v>29</v>
       </c>
       <c r="S3" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="T3" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="V3" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="W3" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -810,22 +825,22 @@
         <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G4">
         <v>2736</v>
       </c>
       <c r="H4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I4" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="J4" s="1">
         <v>46216</v>
@@ -837,7 +852,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="N4" s="1">
         <v>46248</v>
@@ -852,16 +867,16 @@
         <v>24</v>
       </c>
       <c r="S4" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="T4" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="V4" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="W4" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -878,22 +893,22 @@
         <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F5" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G5">
         <v>2722</v>
       </c>
       <c r="H5" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I5" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="J5" s="1">
         <v>46219</v>
@@ -905,7 +920,7 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="N5" s="1">
         <v>46249</v>
@@ -917,19 +932,19 @@
         <v>23</v>
       </c>
       <c r="S5" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="T5" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="U5" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="V5" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="W5" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -946,22 +961,22 @@
         <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F6" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G6">
         <v>2720</v>
       </c>
       <c r="H6" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I6" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="J6" s="1">
         <v>46220</v>
@@ -973,7 +988,7 @@
         <v>10</v>
       </c>
       <c r="M6" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="N6" s="1">
         <v>46255</v>
@@ -988,16 +1003,16 @@
         <v>17</v>
       </c>
       <c r="S6" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="T6" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="V6" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="W6" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1014,22 +1029,22 @@
         <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E7" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F7" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G7">
         <v>2741</v>
       </c>
       <c r="H7" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I7" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="J7" s="1">
         <v>46231</v>
@@ -1041,7 +1056,7 @@
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="N7" s="1">
         <v>46265</v>
@@ -1056,16 +1071,16 @@
         <v>7</v>
       </c>
       <c r="S7" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="T7" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="V7" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="W7" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1082,22 +1097,22 @@
         <v>37</v>
       </c>
       <c r="D8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F8" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G8">
         <v>2736</v>
       </c>
       <c r="H8" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="I8" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="J8" s="1">
         <v>46205</v>
@@ -1109,7 +1124,7 @@
         <v>3</v>
       </c>
       <c r="M8" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="N8" s="1">
         <v>46265</v>
@@ -1124,19 +1139,19 @@
         <v>7</v>
       </c>
       <c r="S8" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="T8" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="U8" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="V8" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="W8" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1153,22 +1168,22 @@
         <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E9" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F9" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G9">
         <v>2737</v>
       </c>
       <c r="H9" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="I9" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="J9" s="1">
         <v>46205</v>
@@ -1180,7 +1195,7 @@
         <v>3</v>
       </c>
       <c r="M9" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="N9" s="1">
         <v>46265</v>
@@ -1192,13 +1207,13 @@
         <v>7</v>
       </c>
       <c r="S9" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="T9" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="W9" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1215,22 +1230,22 @@
         <v>39</v>
       </c>
       <c r="D10" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E10" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F10" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G10">
         <v>2733</v>
       </c>
       <c r="H10" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I10" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="J10" s="1">
         <v>46238</v>
@@ -1242,7 +1257,7 @@
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="N10" s="1">
         <v>46269</v>
@@ -1254,12 +1269,71 @@
         <v>3</v>
       </c>
       <c r="S10" t="s">
+        <v>68</v>
+      </c>
+      <c r="W10" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27">
+      <c r="A11">
+        <v>329</v>
+      </c>
+      <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" t="s">
+        <v>49</v>
+      </c>
+      <c r="E11" t="s">
+        <v>57</v>
+      </c>
+      <c r="F11" t="s">
+        <v>59</v>
+      </c>
+      <c r="G11">
+        <v>2721</v>
+      </c>
+      <c r="H11" t="s">
         <v>63</v>
       </c>
-      <c r="W10" t="s">
-        <v>75</v>
-      </c>
-      <c r="AA10" t="b">
+      <c r="I11" t="s">
+        <v>66</v>
+      </c>
+      <c r="J11" s="1">
+        <v>46241</v>
+      </c>
+      <c r="K11" s="1">
+        <v>46239</v>
+      </c>
+      <c r="L11">
+        <v>2</v>
+      </c>
+      <c r="M11" t="s">
+        <v>67</v>
+      </c>
+      <c r="N11" s="1">
+        <v>46246</v>
+      </c>
+      <c r="Q11">
+        <v>-5</v>
+      </c>
+      <c r="R11">
+        <v>2</v>
+      </c>
+      <c r="S11" t="s">
+        <v>68</v>
+      </c>
+      <c r="W11" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA11" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (10/08/2026 08:55)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -725,10 +725,10 @@
         <v>46287</v>
       </c>
       <c r="Q2">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="R2">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="S2" t="s">
         <v>68</v>
@@ -793,10 +793,10 @@
         <v>46243</v>
       </c>
       <c r="Q3">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="R3">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="S3" t="s">
         <v>68</v>
@@ -861,10 +861,10 @@
         <v>46248</v>
       </c>
       <c r="Q4">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="R4">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="S4" t="s">
         <v>68</v>
@@ -926,10 +926,10 @@
         <v>46249</v>
       </c>
       <c r="Q5">
-        <v>-8</v>
+        <v>-5</v>
       </c>
       <c r="R5">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="S5" t="s">
         <v>68</v>
@@ -997,10 +997,10 @@
         <v>46240</v>
       </c>
       <c r="Q6">
-        <v>-14</v>
+        <v>-11</v>
       </c>
       <c r="R6">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="S6" t="s">
         <v>68</v>
@@ -1065,10 +1065,10 @@
         <v>46239</v>
       </c>
       <c r="Q7">
-        <v>-24</v>
+        <v>-21</v>
       </c>
       <c r="R7">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S7" t="s">
         <v>68</v>
@@ -1133,10 +1133,10 @@
         <v>46239</v>
       </c>
       <c r="Q8">
-        <v>-24</v>
+        <v>-21</v>
       </c>
       <c r="R8">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S8" t="s">
         <v>68</v>
@@ -1201,10 +1201,10 @@
         <v>46265</v>
       </c>
       <c r="Q9">
-        <v>-24</v>
+        <v>-21</v>
       </c>
       <c r="R9">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S9" t="s">
         <v>68</v>
@@ -1263,10 +1263,10 @@
         <v>46269</v>
       </c>
       <c r="Q10">
-        <v>-28</v>
+        <v>-25</v>
       </c>
       <c r="R10">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="S10" t="s">
         <v>68</v>
@@ -1322,10 +1322,10 @@
         <v>46246</v>
       </c>
       <c r="Q11">
-        <v>-5</v>
+        <v>-2</v>
       </c>
       <c r="R11">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S11" t="s">
         <v>68</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (10/08/2026 11:23)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="77">
   <si>
     <t>om_emg</t>
   </si>
@@ -124,9 +124,6 @@
     <t>329260019225</t>
   </si>
   <si>
-    <t>313260018682</t>
-  </si>
-  <si>
     <t>313260018657</t>
   </si>
   <si>
@@ -154,9 +151,6 @@
     <t>MS21442-121</t>
   </si>
   <si>
-    <t>011-00916-10</t>
-  </si>
-  <si>
     <t>324843-W020</t>
   </si>
   <si>
@@ -178,9 +172,6 @@
     <t>BEARING,ROLLER,NEEDL</t>
   </si>
   <si>
-    <t>DISPLAY UNIT,FLIGHT</t>
-  </si>
-  <si>
     <t>HEADSET-MICROPHONE</t>
   </si>
   <si>
@@ -235,22 +226,19 @@
     <t>Atendido 01 EA através da TSP 18122931. Outros 02 EA serão enviados pela empresa. Ramon 03/08/26.</t>
   </si>
   <si>
-    <t>Foi solicitado via email no dia 02-03-2 o atendimento do item com estoque FAB. Claudio -02-03-26 - Em resposta, a coordenadoria disse que o estque seria insuficiente. Foi verificado que na T.O da ANV o QPA para esse item são 2 EA, solicitei confirmação. - Cláudio -02-03-2026. Solicitado o cancelamento da emergência em função da quantidade cedida ao 2733 ter sido de 01ea. Considerando o QPA 02 ea. Encontra-se em tratativa junto a fiscalização e o gestor do contrato conforme mensagem de e-mail de 05/03. - SOLICITAÇÃO E-C98-26047.Colocado pedido AOG Textron J17626242 - previsão de entrega em Miami 05/08</t>
+    <t>Foi solicitado via email no dia 02-03-2 o atendimento do item com estoque FAB. Claudio -02-03-26 - Em resposta, a coordenadoria disse que o estque seria insuficiente. Foi verificado que na T.O da ANV o QPA para esse item são 2 EA, solicitei confirmação. - Cláudio -02-03-2026. Solicitado o cancelamento da emergência em função da quantidade cedida ao 2733 ter sido de 01ea. Considerando o QPA 02 ea. Encontra-se em tratativa junto a fiscalização e o gestor do contrato conforme mensagem de e-mail de 05/03. - SOLICITAÇÃO E-C98-26047.Colocado pedido AOG Textron J17626242 - previsão de entrega em Miami 05/08 AWB4238 em desembaraço no GIGRJ em 06/8/2026, previsao de CANAL hoje às 18 horas ATZ Marcio 6/8/2026</t>
   </si>
   <si>
     <t>Colocado pedido junto ao fornecedor LEGACY PARTS, previsão de entrega em Miami 06/08</t>
   </si>
   <si>
-    <t>Colocado pedido Textron IJ17575583 - entregue em Miami 15/07. Carga rercepcionada GIG 19/07 - Aguardando liberação do SEFAZ. ATZ 21/07 - material em processo de expedição RC 23/07/2026 - MATERIAL ENVIADO PELO RECIBO 639/FAB/26 AWB A SER GERADA</t>
+    <t>Colocado pedido Textron IJ17575583 - entregue em Miami 15/07. Carga rercepcionada GIG 19/07 - Aguardando liberação do SEFAZ. ATZ 21/07 - material em processo de expedição RC 23/07/2026 - MATERIAL ENVIADO PELO RECIBO 639/FAB/26</t>
   </si>
   <si>
     <t>Item em bancada porem em pessimo estado, foi solicitado recolhimento de mais unidades para envio a oficina para tentativa de reparo ATZ Marcio 17/7/26. Solicitado abertura de O.S. para 3EA do item no dia 16-07-26 via Email para a Coordenadoria - CLA-21-07-26</t>
   </si>
   <si>
-    <t>Pedido I816822 entregue em Miami 27/07. Previsão de chegada GIG 30/07 (voo 4208). Previsão de canal 31/07 - MATERIAL RECEBIDO NA VEE ONE, EM PROCESSO DE EXPEDIÇÃO 04/08/2026 - ATZ RC</t>
-  </si>
-  <si>
-    <t>item sendo preparado para transporte - CLA-03-08- AWB 127-5082 1282- CLA-04-08</t>
+    <t>Pedido I816822 entregue em Miami 27/07. Previsão de chegada GIG 30/07 (voo 4208). Previsão de canal 31/07 - MATERIAL RECEBIDO NA VEE ONE, EM PROCESSO DE EXPEDIÇÃO 04/08/2026 - ATZ RC - MATERIAL ENVIADO VIA RECIBO 650/FAB/26 - AWB 12750991113 DPE 06/08/2026, ESTÁ DISPONÍVEL PARA RETIRADA DESDE 04/08/2026</t>
   </si>
   <si>
     <t>Enviado para o Operador(02 EA), atendimento parcial, em 31/07/2026 -AWB 127-5041 6833- REZ - o outro 1 EA será atendido pelo estoque FAB. conforme solicitado por Email- CLA-03-08 - AWB 127-5082 1282 -1 EA ENVIADO ESTOQUE FAB</t>
@@ -592,7 +580,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA11"/>
+  <dimension ref="A1:AA10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -689,22 +677,22 @@
         <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G2">
         <v>2730</v>
       </c>
       <c r="H2" t="s">
+        <v>58</v>
+      </c>
+      <c r="I2" t="s">
         <v>61</v>
-      </c>
-      <c r="I2" t="s">
-        <v>64</v>
       </c>
       <c r="J2" s="1">
         <v>46076</v>
@@ -716,7 +704,7 @@
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="N2" s="1">
         <v>46091</v>
@@ -731,19 +719,19 @@
         <v>164</v>
       </c>
       <c r="S2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="T2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="U2" t="s">
+        <v>67</v>
+      </c>
+      <c r="V2" t="s">
         <v>70</v>
       </c>
-      <c r="V2" t="s">
-        <v>73</v>
-      </c>
       <c r="W2" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -760,22 +748,22 @@
         <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F3" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G3">
         <v>2702</v>
       </c>
       <c r="H3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="I3" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="J3" s="1">
         <v>46212</v>
@@ -787,7 +775,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="N3" s="1">
         <v>46243</v>
@@ -799,16 +787,16 @@
         <v>32</v>
       </c>
       <c r="S3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="T3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="V3" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="W3" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -825,22 +813,22 @@
         <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G4">
         <v>2736</v>
       </c>
       <c r="H4" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="I4" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="J4" s="1">
         <v>46216</v>
@@ -852,7 +840,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="N4" s="1">
         <v>46248</v>
@@ -867,16 +855,16 @@
         <v>27</v>
       </c>
       <c r="S4" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="T4" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="V4" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="W4" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -893,22 +881,22 @@
         <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F5" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G5">
         <v>2722</v>
       </c>
       <c r="H5" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="I5" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="J5" s="1">
         <v>46219</v>
@@ -920,7 +908,7 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="N5" s="1">
         <v>46249</v>
@@ -932,19 +920,19 @@
         <v>26</v>
       </c>
       <c r="S5" t="s">
+        <v>65</v>
+      </c>
+      <c r="T5" t="s">
+        <v>66</v>
+      </c>
+      <c r="U5" t="s">
         <v>68</v>
       </c>
-      <c r="T5" t="s">
-        <v>69</v>
-      </c>
-      <c r="U5" t="s">
-        <v>71</v>
-      </c>
       <c r="V5" t="s">
+        <v>73</v>
+      </c>
+      <c r="W5" t="s">
         <v>76</v>
-      </c>
-      <c r="W5" t="s">
-        <v>80</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -961,22 +949,22 @@
         <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F6" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G6">
         <v>2720</v>
       </c>
       <c r="H6" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="I6" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="J6" s="1">
         <v>46220</v>
@@ -988,7 +976,7 @@
         <v>10</v>
       </c>
       <c r="M6" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="N6" s="1">
         <v>46255</v>
@@ -1003,16 +991,16 @@
         <v>20</v>
       </c>
       <c r="S6" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="T6" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="V6" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="W6" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1029,34 +1017,34 @@
         <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E7" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F7" t="s">
+        <v>57</v>
+      </c>
+      <c r="G7">
+        <v>2736</v>
+      </c>
+      <c r="H7" t="s">
         <v>59</v>
       </c>
-      <c r="G7">
-        <v>2741</v>
-      </c>
-      <c r="H7" t="s">
-        <v>61</v>
-      </c>
       <c r="I7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="J7" s="1">
-        <v>46231</v>
+        <v>46205</v>
       </c>
       <c r="K7" s="1">
         <v>46234</v>
       </c>
       <c r="L7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="N7" s="1">
         <v>46265</v>
@@ -1071,16 +1059,19 @@
         <v>10</v>
       </c>
       <c r="S7" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="T7" t="s">
+        <v>66</v>
+      </c>
+      <c r="U7" t="s">
         <v>69</v>
       </c>
       <c r="V7" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="W7" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1097,22 +1088,22 @@
         <v>37</v>
       </c>
       <c r="D8" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E8" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F8" t="s">
+        <v>57</v>
+      </c>
+      <c r="G8">
+        <v>2737</v>
+      </c>
+      <c r="H8" t="s">
         <v>60</v>
       </c>
-      <c r="G8">
-        <v>2736</v>
-      </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>62</v>
-      </c>
-      <c r="I8" t="s">
-        <v>65</v>
       </c>
       <c r="J8" s="1">
         <v>46205</v>
@@ -1124,14 +1115,11 @@
         <v>3</v>
       </c>
       <c r="M8" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="N8" s="1">
         <v>46265</v>
       </c>
-      <c r="O8" s="1">
-        <v>46239</v>
-      </c>
       <c r="Q8">
         <v>-21</v>
       </c>
@@ -1139,19 +1127,13 @@
         <v>10</v>
       </c>
       <c r="S8" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="T8" t="s">
-        <v>69</v>
-      </c>
-      <c r="U8" t="s">
-        <v>72</v>
-      </c>
-      <c r="V8" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="W8" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1159,61 +1141,58 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9">
-        <v>313</v>
+        <v>396</v>
       </c>
       <c r="B9" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C9" t="s">
         <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E9" t="s">
+        <v>53</v>
+      </c>
+      <c r="F9" t="s">
         <v>55</v>
       </c>
-      <c r="F9" t="s">
-        <v>60</v>
-      </c>
       <c r="G9">
-        <v>2737</v>
+        <v>2733</v>
       </c>
       <c r="H9" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="I9" t="s">
+        <v>62</v>
+      </c>
+      <c r="J9" s="1">
+        <v>46238</v>
+      </c>
+      <c r="K9" s="1">
+        <v>46238</v>
+      </c>
+      <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9" t="s">
+        <v>64</v>
+      </c>
+      <c r="N9" s="1">
+        <v>46269</v>
+      </c>
+      <c r="Q9">
+        <v>-25</v>
+      </c>
+      <c r="R9">
+        <v>6</v>
+      </c>
+      <c r="S9" t="s">
         <v>65</v>
       </c>
-      <c r="J9" s="1">
-        <v>46205</v>
-      </c>
-      <c r="K9" s="1">
-        <v>46234</v>
-      </c>
-      <c r="L9">
-        <v>3</v>
-      </c>
-      <c r="M9" t="s">
-        <v>67</v>
-      </c>
-      <c r="N9" s="1">
-        <v>46265</v>
-      </c>
-      <c r="Q9">
-        <v>-21</v>
-      </c>
-      <c r="R9">
-        <v>10</v>
-      </c>
-      <c r="S9" t="s">
-        <v>68</v>
-      </c>
-      <c r="T9" t="s">
-        <v>69</v>
-      </c>
       <c r="W9" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1221,119 +1200,60 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>396</v>
+        <v>329</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C10" t="s">
         <v>39</v>
       </c>
       <c r="D10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E10" t="s">
+        <v>54</v>
+      </c>
+      <c r="F10" t="s">
         <v>56</v>
       </c>
-      <c r="F10" t="s">
-        <v>58</v>
-      </c>
       <c r="G10">
-        <v>2733</v>
+        <v>2721</v>
       </c>
       <c r="H10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I10" t="s">
+        <v>63</v>
+      </c>
+      <c r="J10" s="1">
+        <v>46241</v>
+      </c>
+      <c r="K10" s="1">
+        <v>46239</v>
+      </c>
+      <c r="L10">
+        <v>2</v>
+      </c>
+      <c r="M10" t="s">
+        <v>64</v>
+      </c>
+      <c r="N10" s="1">
+        <v>46246</v>
+      </c>
+      <c r="Q10">
+        <v>-2</v>
+      </c>
+      <c r="R10">
+        <v>5</v>
+      </c>
+      <c r="S10" t="s">
         <v>65</v>
       </c>
-      <c r="J10" s="1">
-        <v>46238</v>
-      </c>
-      <c r="K10" s="1">
-        <v>46238</v>
-      </c>
-      <c r="L10">
-        <v>1</v>
-      </c>
-      <c r="M10" t="s">
-        <v>67</v>
-      </c>
-      <c r="N10" s="1">
-        <v>46269</v>
-      </c>
-      <c r="Q10">
-        <v>-25</v>
-      </c>
-      <c r="R10">
-        <v>6</v>
-      </c>
-      <c r="S10" t="s">
-        <v>68</v>
-      </c>
       <c r="W10" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AA10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:27">
-      <c r="A11">
-        <v>329</v>
-      </c>
-      <c r="B11" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" t="s">
-        <v>40</v>
-      </c>
-      <c r="D11" t="s">
-        <v>49</v>
-      </c>
-      <c r="E11" t="s">
-        <v>57</v>
-      </c>
-      <c r="F11" t="s">
-        <v>59</v>
-      </c>
-      <c r="G11">
-        <v>2721</v>
-      </c>
-      <c r="H11" t="s">
-        <v>63</v>
-      </c>
-      <c r="I11" t="s">
-        <v>66</v>
-      </c>
-      <c r="J11" s="1">
-        <v>46241</v>
-      </c>
-      <c r="K11" s="1">
-        <v>46239</v>
-      </c>
-      <c r="L11">
-        <v>2</v>
-      </c>
-      <c r="M11" t="s">
-        <v>67</v>
-      </c>
-      <c r="N11" s="1">
-        <v>46246</v>
-      </c>
-      <c r="Q11">
-        <v>-2</v>
-      </c>
-      <c r="R11">
-        <v>5</v>
-      </c>
-      <c r="S11" t="s">
-        <v>68</v>
-      </c>
-      <c r="W11" t="s">
-        <v>80</v>
-      </c>
-      <c r="AA11" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (10/08/2026 13:05)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="80">
   <si>
     <t>om_emg</t>
   </si>
@@ -136,6 +136,9 @@
     <t>329260019264</t>
   </si>
   <si>
+    <t>685260012560</t>
+  </si>
+  <si>
     <t>1214134-1</t>
   </si>
   <si>
@@ -160,6 +163,9 @@
     <t>C662041-0102</t>
   </si>
   <si>
+    <t>2641010-3</t>
+  </si>
+  <si>
     <t>BELLCRANK ASSY</t>
   </si>
   <si>
@@ -179,6 +185,9 @@
   </si>
   <si>
     <t>INDICATOR FUEL</t>
+  </si>
+  <si>
+    <t>AXLE FITTING</t>
   </si>
   <si>
     <t>C</t>
@@ -580,7 +589,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA10"/>
+  <dimension ref="A1:AA11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -677,22 +686,22 @@
         <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G2">
         <v>2730</v>
       </c>
       <c r="H2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J2" s="1">
         <v>46076</v>
@@ -704,7 +713,7 @@
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="N2" s="1">
         <v>46091</v>
@@ -719,19 +728,19 @@
         <v>164</v>
       </c>
       <c r="S2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="T2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="U2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="V2" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="W2" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -748,22 +757,22 @@
         <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G3">
         <v>2702</v>
       </c>
       <c r="H3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="J3" s="1">
         <v>46212</v>
@@ -775,7 +784,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="N3" s="1">
         <v>46243</v>
@@ -787,16 +796,16 @@
         <v>32</v>
       </c>
       <c r="S3" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="T3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="V3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="W3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -813,22 +822,22 @@
         <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G4">
         <v>2736</v>
       </c>
       <c r="H4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I4" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="J4" s="1">
         <v>46216</v>
@@ -840,7 +849,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="N4" s="1">
         <v>46248</v>
@@ -855,16 +864,16 @@
         <v>27</v>
       </c>
       <c r="S4" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="T4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="V4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="W4" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -881,22 +890,22 @@
         <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F5" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G5">
         <v>2722</v>
       </c>
       <c r="H5" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I5" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="J5" s="1">
         <v>46219</v>
@@ -908,7 +917,7 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="N5" s="1">
         <v>46249</v>
@@ -920,19 +929,19 @@
         <v>26</v>
       </c>
       <c r="S5" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="T5" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="U5" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="V5" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="W5" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -949,22 +958,22 @@
         <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F6" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G6">
         <v>2720</v>
       </c>
       <c r="H6" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="J6" s="1">
         <v>46220</v>
@@ -976,7 +985,7 @@
         <v>10</v>
       </c>
       <c r="M6" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="N6" s="1">
         <v>46255</v>
@@ -991,16 +1000,16 @@
         <v>20</v>
       </c>
       <c r="S6" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="T6" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="V6" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="W6" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1017,22 +1026,22 @@
         <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E7" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F7" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G7">
         <v>2736</v>
       </c>
       <c r="H7" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="I7" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="J7" s="1">
         <v>46205</v>
@@ -1044,7 +1053,7 @@
         <v>3</v>
       </c>
       <c r="M7" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="N7" s="1">
         <v>46265</v>
@@ -1059,19 +1068,19 @@
         <v>10</v>
       </c>
       <c r="S7" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="T7" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="U7" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="V7" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="W7" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1088,22 +1097,22 @@
         <v>37</v>
       </c>
       <c r="D8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F8" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G8">
         <v>2737</v>
       </c>
       <c r="H8" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="I8" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="J8" s="1">
         <v>46205</v>
@@ -1115,7 +1124,7 @@
         <v>3</v>
       </c>
       <c r="M8" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="N8" s="1">
         <v>46265</v>
@@ -1127,13 +1136,13 @@
         <v>10</v>
       </c>
       <c r="S8" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="T8" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="W8" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1150,22 +1159,22 @@
         <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E9" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G9">
         <v>2733</v>
       </c>
       <c r="H9" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I9" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="J9" s="1">
         <v>46238</v>
@@ -1177,7 +1186,7 @@
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="N9" s="1">
         <v>46269</v>
@@ -1189,10 +1198,13 @@
         <v>6</v>
       </c>
       <c r="S9" t="s">
-        <v>65</v>
+        <v>68</v>
+      </c>
+      <c r="T9" t="s">
+        <v>69</v>
       </c>
       <c r="W9" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1209,22 +1221,22 @@
         <v>39</v>
       </c>
       <c r="D10" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E10" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F10" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G10">
         <v>2721</v>
       </c>
       <c r="H10" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="I10" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="J10" s="1">
         <v>46241</v>
@@ -1236,7 +1248,7 @@
         <v>2</v>
       </c>
       <c r="M10" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="N10" s="1">
         <v>46246</v>
@@ -1248,12 +1260,74 @@
         <v>5</v>
       </c>
       <c r="S10" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="W10" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="AA10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27">
+      <c r="A11">
+        <v>685</v>
+      </c>
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" t="s">
+        <v>49</v>
+      </c>
+      <c r="E11" t="s">
+        <v>57</v>
+      </c>
+      <c r="F11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G11">
+        <v>2729</v>
+      </c>
+      <c r="H11" t="s">
+        <v>63</v>
+      </c>
+      <c r="I11" t="s">
+        <v>64</v>
+      </c>
+      <c r="J11" s="1">
+        <v>46244</v>
+      </c>
+      <c r="K11" s="1">
+        <v>46244</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11" t="s">
+        <v>67</v>
+      </c>
+      <c r="N11" s="1">
+        <v>46255</v>
+      </c>
+      <c r="Q11">
+        <v>-11</v>
+      </c>
+      <c r="R11">
+        <v>0</v>
+      </c>
+      <c r="S11" t="s">
+        <v>69</v>
+      </c>
+      <c r="T11" t="s">
+        <v>69</v>
+      </c>
+      <c r="W11" t="s">
+        <v>79</v>
+      </c>
+      <c r="AA11" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (11/08/2026 08:51)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -722,10 +722,10 @@
         <v>46287</v>
       </c>
       <c r="Q2">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="R2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="S2" t="s">
         <v>68</v>
@@ -790,10 +790,10 @@
         <v>46243</v>
       </c>
       <c r="Q3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R3">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S3" t="s">
         <v>68</v>
@@ -858,10 +858,10 @@
         <v>46248</v>
       </c>
       <c r="Q4">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R4">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="S4" t="s">
         <v>68</v>
@@ -923,10 +923,10 @@
         <v>46249</v>
       </c>
       <c r="Q5">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R5">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S5" t="s">
         <v>68</v>
@@ -994,10 +994,10 @@
         <v>46240</v>
       </c>
       <c r="Q6">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R6">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="S6" t="s">
         <v>68</v>
@@ -1062,10 +1062,10 @@
         <v>46239</v>
       </c>
       <c r="Q7">
-        <v>-21</v>
+        <v>-20</v>
       </c>
       <c r="R7">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S7" t="s">
         <v>68</v>
@@ -1130,10 +1130,10 @@
         <v>46265</v>
       </c>
       <c r="Q8">
-        <v>-21</v>
+        <v>-20</v>
       </c>
       <c r="R8">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S8" t="s">
         <v>68</v>
@@ -1192,10 +1192,10 @@
         <v>46269</v>
       </c>
       <c r="Q9">
-        <v>-25</v>
+        <v>-24</v>
       </c>
       <c r="R9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S9" t="s">
         <v>68</v>
@@ -1254,10 +1254,10 @@
         <v>46246</v>
       </c>
       <c r="Q10">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S10" t="s">
         <v>68</v>
@@ -1313,10 +1313,10 @@
         <v>46255</v>
       </c>
       <c r="Q11">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S11" t="s">
         <v>69</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (11/08/2026 11:23)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="78">
   <si>
     <t>om_emg</t>
   </si>
@@ -136,9 +136,6 @@
     <t>329260019264</t>
   </si>
   <si>
-    <t>685260012560</t>
-  </si>
-  <si>
     <t>1214134-1</t>
   </si>
   <si>
@@ -163,9 +160,6 @@
     <t>C662041-0102</t>
   </si>
   <si>
-    <t>2641010-3</t>
-  </si>
-  <si>
     <t>BELLCRANK ASSY</t>
   </si>
   <si>
@@ -187,9 +181,6 @@
     <t>INDICATOR FUEL</t>
   </si>
   <si>
-    <t>AXLE FITTING</t>
-  </si>
-  <si>
     <t>C</t>
   </si>
   <si>
@@ -235,13 +226,13 @@
     <t>Atendido 01 EA através da TSP 18122931. Outros 02 EA serão enviados pela empresa. Ramon 03/08/26.</t>
   </si>
   <si>
-    <t>Foi solicitado via email no dia 02-03-2 o atendimento do item com estoque FAB. Claudio -02-03-26 - Em resposta, a coordenadoria disse que o estque seria insuficiente. Foi verificado que na T.O da ANV o QPA para esse item são 2 EA, solicitei confirmação. - Cláudio -02-03-2026. Solicitado o cancelamento da emergência em função da quantidade cedida ao 2733 ter sido de 01ea. Considerando o QPA 02 ea. Encontra-se em tratativa junto a fiscalização e o gestor do contrato conforme mensagem de e-mail de 05/03. - SOLICITAÇÃO E-C98-26047.Colocado pedido AOG Textron J17626242 - previsão de entrega em Miami 05/08 AWB4238 em desembaraço no GIGRJ em 06/8/2026, previsao de CANAL hoje às 18 horas ATZ Marcio 6/8/2026</t>
-  </si>
-  <si>
-    <t>Colocado pedido junto ao fornecedor LEGACY PARTS, previsão de entrega em Miami 06/08</t>
-  </si>
-  <si>
-    <t>Colocado pedido Textron IJ17575583 - entregue em Miami 15/07. Carga rercepcionada GIG 19/07 - Aguardando liberação do SEFAZ. ATZ 21/07 - material em processo de expedição RC 23/07/2026 - MATERIAL ENVIADO PELO RECIBO 639/FAB/26</t>
+    <t>Foi solicitado via email no dia 02-03-2 o atendimento do item com estoque FAB. Claudio -02-03-26 - Em resposta, a coordenadoria disse que o estque seria insuficiente. Foi verificado que na T.O da ANV o QPA para esse item são 2 EA, solicitei confirmação. - Cláudio -02-03-2026. Solicitado o cancelamento da emergência em função da quantidade cedida ao 2733 ter sido de 01ea. Considerando o QPA 02 ea. Encontra-se em tratativa junto a fiscalização e o gestor do contrato conforme mensagem de e-mail de 05/03. - SOLICITAÇÃO E-C98-26047.Colocado pedido AOG Textron J17626242 - previsão de entrega em Miami 05/08 AWB4238 em desembaraço no GIGRJ em 06/8/2026, previsao de CANAL hoje às 18 horas ATZ Marcio 6/8/2026 - MATERIAL EM RECEBIMENTO VEE ONE 07/08/2026 16:31, SERÁ ENVIADO NA SEGUNDA FEIRA</t>
+  </si>
+  <si>
+    <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - previsão de entrega em Miami 12/08</t>
+  </si>
+  <si>
+    <t>Colocado pedido Textron IJ17575583 - entregue em Miami 15/07. Carga rercepcionada GIG 19/07 - Aguardando liberação do SEFAZ. ATZ 21/07 - material em processo de expedição RC 23/07/2026 - MATERIAL ENVIADO PELO RECIBO 639/FAB/26 - AWB 12750389603 DPE 13/08/2026</t>
   </si>
   <si>
     <t>Item em bancada porem em pessimo estado, foi solicitado recolhimento de mais unidades para envio a oficina para tentativa de reparo ATZ Marcio 17/7/26. Solicitado abertura de O.S. para 3EA do item no dia 16-07-26 via Email para a Coordenadoria - CLA-21-07-26</t>
@@ -250,7 +241,10 @@
     <t>Pedido I816822 entregue em Miami 27/07. Previsão de chegada GIG 30/07 (voo 4208). Previsão de canal 31/07 - MATERIAL RECEBIDO NA VEE ONE, EM PROCESSO DE EXPEDIÇÃO 04/08/2026 - ATZ RC - MATERIAL ENVIADO VIA RECIBO 650/FAB/26 - AWB 12750991113 DPE 06/08/2026, ESTÁ DISPONÍVEL PARA RETIRADA DESDE 04/08/2026</t>
   </si>
   <si>
-    <t>Enviado para o Operador(02 EA), atendimento parcial, em 31/07/2026 -AWB 127-5041 6833- REZ - o outro 1 EA será atendido pelo estoque FAB. conforme solicitado por Email- CLA-03-08 - AWB 127-5082 1282 -1 EA ENVIADO ESTOQUE FAB</t>
+    <t>Enviado para o Operador(02 EA), atendimento parcial, em 31/07/2026 -AWB 127-5041 6833- REZ - o outro 1 EA será atendido pelo estoque FAB. conforme solicitado por Email- CLA-03-08 - AWB 127-5082 1282 -1 EA ENVIADO ESTOQUE FAB - Material entregue dia 06/08/2026</t>
+  </si>
+  <si>
+    <t>Temos 4 EA em manutenção na William, será pedido prioridade. CLA-03-08</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -589,7 +583,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA11"/>
+  <dimension ref="A1:AA10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -686,22 +680,22 @@
         <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G2">
         <v>2730</v>
       </c>
       <c r="H2" t="s">
+        <v>58</v>
+      </c>
+      <c r="I2" t="s">
         <v>61</v>
-      </c>
-      <c r="I2" t="s">
-        <v>64</v>
       </c>
       <c r="J2" s="1">
         <v>46076</v>
@@ -713,7 +707,7 @@
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="N2" s="1">
         <v>46091</v>
@@ -728,19 +722,19 @@
         <v>165</v>
       </c>
       <c r="S2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="T2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="U2" t="s">
+        <v>67</v>
+      </c>
+      <c r="V2" t="s">
         <v>70</v>
       </c>
-      <c r="V2" t="s">
-        <v>73</v>
-      </c>
       <c r="W2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -757,22 +751,22 @@
         <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F3" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G3">
         <v>2702</v>
       </c>
       <c r="H3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="I3" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="J3" s="1">
         <v>46212</v>
@@ -784,7 +778,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="N3" s="1">
         <v>46243</v>
@@ -796,16 +790,16 @@
         <v>33</v>
       </c>
       <c r="S3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="T3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="V3" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="W3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -822,22 +816,22 @@
         <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G4">
         <v>2736</v>
       </c>
       <c r="H4" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="I4" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="J4" s="1">
         <v>46216</v>
@@ -849,7 +843,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="N4" s="1">
         <v>46248</v>
@@ -864,16 +858,16 @@
         <v>28</v>
       </c>
       <c r="S4" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="T4" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="V4" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="W4" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -890,22 +884,22 @@
         <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F5" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G5">
         <v>2722</v>
       </c>
       <c r="H5" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="I5" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="J5" s="1">
         <v>46219</v>
@@ -917,7 +911,7 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="N5" s="1">
         <v>46249</v>
@@ -929,19 +923,19 @@
         <v>27</v>
       </c>
       <c r="S5" t="s">
+        <v>65</v>
+      </c>
+      <c r="T5" t="s">
+        <v>66</v>
+      </c>
+      <c r="U5" t="s">
         <v>68</v>
       </c>
-      <c r="T5" t="s">
-        <v>69</v>
-      </c>
-      <c r="U5" t="s">
-        <v>71</v>
-      </c>
       <c r="V5" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="W5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -958,22 +952,22 @@
         <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F6" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G6">
         <v>2720</v>
       </c>
       <c r="H6" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="I6" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="J6" s="1">
         <v>46220</v>
@@ -985,7 +979,7 @@
         <v>10</v>
       </c>
       <c r="M6" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="N6" s="1">
         <v>46255</v>
@@ -1000,16 +994,16 @@
         <v>21</v>
       </c>
       <c r="S6" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="T6" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="V6" t="s">
+        <v>74</v>
+      </c>
+      <c r="W6" t="s">
         <v>77</v>
-      </c>
-      <c r="W6" t="s">
-        <v>79</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1026,22 +1020,22 @@
         <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E7" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F7" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="G7">
         <v>2736</v>
       </c>
       <c r="H7" t="s">
+        <v>59</v>
+      </c>
+      <c r="I7" t="s">
         <v>62</v>
-      </c>
-      <c r="I7" t="s">
-        <v>65</v>
       </c>
       <c r="J7" s="1">
         <v>46205</v>
@@ -1053,7 +1047,7 @@
         <v>3</v>
       </c>
       <c r="M7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="N7" s="1">
         <v>46265</v>
@@ -1068,19 +1062,19 @@
         <v>11</v>
       </c>
       <c r="S7" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="T7" t="s">
+        <v>66</v>
+      </c>
+      <c r="U7" t="s">
         <v>69</v>
       </c>
-      <c r="U7" t="s">
-        <v>72</v>
-      </c>
       <c r="V7" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="W7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1097,22 +1091,22 @@
         <v>37</v>
       </c>
       <c r="D8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F8" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="G8">
         <v>2737</v>
       </c>
       <c r="H8" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="I8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="J8" s="1">
         <v>46205</v>
@@ -1124,7 +1118,7 @@
         <v>3</v>
       </c>
       <c r="M8" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="N8" s="1">
         <v>46265</v>
@@ -1136,13 +1130,16 @@
         <v>11</v>
       </c>
       <c r="S8" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="T8" t="s">
-        <v>69</v>
+        <v>66</v>
+      </c>
+      <c r="V8" t="s">
+        <v>76</v>
       </c>
       <c r="W8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1159,22 +1156,22 @@
         <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E9" t="s">
+        <v>53</v>
+      </c>
+      <c r="F9" t="s">
         <v>55</v>
-      </c>
-      <c r="F9" t="s">
-        <v>58</v>
       </c>
       <c r="G9">
         <v>2733</v>
       </c>
       <c r="H9" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="I9" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="J9" s="1">
         <v>46238</v>
@@ -1186,7 +1183,7 @@
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="N9" s="1">
         <v>46269</v>
@@ -1198,13 +1195,13 @@
         <v>7</v>
       </c>
       <c r="S9" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="T9" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="W9" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1221,22 +1218,22 @@
         <v>39</v>
       </c>
       <c r="D10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E10" t="s">
+        <v>54</v>
+      </c>
+      <c r="F10" t="s">
         <v>56</v>
-      </c>
-      <c r="F10" t="s">
-        <v>59</v>
       </c>
       <c r="G10">
         <v>2721</v>
       </c>
       <c r="H10" t="s">
+        <v>60</v>
+      </c>
+      <c r="I10" t="s">
         <v>63</v>
-      </c>
-      <c r="I10" t="s">
-        <v>66</v>
       </c>
       <c r="J10" s="1">
         <v>46241</v>
@@ -1248,7 +1245,7 @@
         <v>2</v>
       </c>
       <c r="M10" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="N10" s="1">
         <v>46246</v>
@@ -1260,74 +1257,12 @@
         <v>6</v>
       </c>
       <c r="S10" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="W10" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="AA10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:27">
-      <c r="A11">
-        <v>685</v>
-      </c>
-      <c r="B11" t="s">
-        <v>28</v>
-      </c>
-      <c r="C11" t="s">
-        <v>40</v>
-      </c>
-      <c r="D11" t="s">
-        <v>49</v>
-      </c>
-      <c r="E11" t="s">
-        <v>57</v>
-      </c>
-      <c r="F11" t="s">
-        <v>60</v>
-      </c>
-      <c r="G11">
-        <v>2729</v>
-      </c>
-      <c r="H11" t="s">
-        <v>63</v>
-      </c>
-      <c r="I11" t="s">
-        <v>64</v>
-      </c>
-      <c r="J11" s="1">
-        <v>46244</v>
-      </c>
-      <c r="K11" s="1">
-        <v>46244</v>
-      </c>
-      <c r="L11">
-        <v>1</v>
-      </c>
-      <c r="M11" t="s">
-        <v>67</v>
-      </c>
-      <c r="N11" s="1">
-        <v>46255</v>
-      </c>
-      <c r="Q11">
-        <v>-10</v>
-      </c>
-      <c r="R11">
-        <v>1</v>
-      </c>
-      <c r="S11" t="s">
-        <v>69</v>
-      </c>
-      <c r="T11" t="s">
-        <v>69</v>
-      </c>
-      <c r="W11" t="s">
-        <v>79</v>
-      </c>
-      <c r="AA11" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (11/08/2026 15:01)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="82">
   <si>
     <t>om_emg</t>
   </si>
@@ -109,6 +109,9 @@
     <t>BABE</t>
   </si>
   <si>
+    <t>BACO</t>
+  </si>
+  <si>
     <t>313260017747</t>
   </si>
   <si>
@@ -136,6 +139,9 @@
     <t>329260019264</t>
   </si>
   <si>
+    <t>386260013489</t>
+  </si>
+  <si>
     <t>1214134-1</t>
   </si>
   <si>
@@ -160,6 +166,9 @@
     <t>C662041-0102</t>
   </si>
   <si>
+    <t>9910333-1</t>
+  </si>
+  <si>
     <t>BELLCRANK ASSY</t>
   </si>
   <si>
@@ -179,6 +188,9 @@
   </si>
   <si>
     <t>INDICATOR FUEL</t>
+  </si>
+  <si>
+    <t>ENGINE MOUNT</t>
   </si>
   <si>
     <t>C</t>
@@ -583,7 +595,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA10"/>
+  <dimension ref="A1:AA11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -677,25 +689,25 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F2" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G2">
         <v>2730</v>
       </c>
       <c r="H2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="J2" s="1">
         <v>46076</v>
@@ -707,7 +719,7 @@
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="N2" s="1">
         <v>46091</v>
@@ -722,19 +734,19 @@
         <v>165</v>
       </c>
       <c r="S2" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="T2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="U2" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="V2" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="W2" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -748,25 +760,25 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E3" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="F3" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G3">
         <v>2702</v>
       </c>
       <c r="H3" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I3" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="J3" s="1">
         <v>46212</v>
@@ -778,7 +790,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="N3" s="1">
         <v>46243</v>
@@ -790,16 +802,16 @@
         <v>33</v>
       </c>
       <c r="S3" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="T3" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="V3" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="W3" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -813,25 +825,25 @@
         <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E4" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="F4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G4">
         <v>2736</v>
       </c>
       <c r="H4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I4" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="J4" s="1">
         <v>46216</v>
@@ -843,7 +855,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="N4" s="1">
         <v>46248</v>
@@ -858,16 +870,16 @@
         <v>28</v>
       </c>
       <c r="S4" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="T4" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="V4" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="W4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -881,25 +893,25 @@
         <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E5" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="F5" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G5">
         <v>2722</v>
       </c>
       <c r="H5" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I5" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="J5" s="1">
         <v>46219</v>
@@ -911,7 +923,7 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="N5" s="1">
         <v>46249</v>
@@ -923,19 +935,19 @@
         <v>27</v>
       </c>
       <c r="S5" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="T5" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="U5" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="V5" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="W5" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -949,25 +961,25 @@
         <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E6" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="F6" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G6">
         <v>2720</v>
       </c>
       <c r="H6" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I6" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="J6" s="1">
         <v>46220</v>
@@ -979,7 +991,7 @@
         <v>10</v>
       </c>
       <c r="M6" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="N6" s="1">
         <v>46255</v>
@@ -994,16 +1006,16 @@
         <v>21</v>
       </c>
       <c r="S6" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="T6" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="V6" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="W6" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1017,25 +1029,25 @@
         <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E7" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F7" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="G7">
         <v>2736</v>
       </c>
       <c r="H7" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="I7" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="J7" s="1">
         <v>46205</v>
@@ -1047,7 +1059,7 @@
         <v>3</v>
       </c>
       <c r="M7" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="N7" s="1">
         <v>46265</v>
@@ -1062,19 +1074,19 @@
         <v>11</v>
       </c>
       <c r="S7" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="T7" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="U7" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="V7" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="W7" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1088,25 +1100,25 @@
         <v>27</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E8" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F8" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="G8">
         <v>2737</v>
       </c>
       <c r="H8" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="I8" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="J8" s="1">
         <v>46205</v>
@@ -1118,7 +1130,7 @@
         <v>3</v>
       </c>
       <c r="M8" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="N8" s="1">
         <v>46265</v>
@@ -1130,16 +1142,16 @@
         <v>11</v>
       </c>
       <c r="S8" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="T8" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="V8" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="W8" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1153,25 +1165,25 @@
         <v>30</v>
       </c>
       <c r="C9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E9" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F9" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G9">
         <v>2733</v>
       </c>
       <c r="H9" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I9" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="J9" s="1">
         <v>46238</v>
@@ -1183,7 +1195,7 @@
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="N9" s="1">
         <v>46269</v>
@@ -1195,13 +1207,13 @@
         <v>7</v>
       </c>
       <c r="S9" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="T9" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="W9" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1215,54 +1227,113 @@
         <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E10" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F10" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G10">
         <v>2721</v>
       </c>
       <c r="H10" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="I10" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="J10" s="1">
         <v>46241</v>
       </c>
       <c r="K10" s="1">
-        <v>46239</v>
+        <v>46241</v>
       </c>
       <c r="L10">
         <v>2</v>
       </c>
       <c r="M10" t="s">
+        <v>68</v>
+      </c>
+      <c r="N10" s="1">
+        <v>46248</v>
+      </c>
+      <c r="Q10">
+        <v>-3</v>
+      </c>
+      <c r="R10">
+        <v>4</v>
+      </c>
+      <c r="S10" t="s">
+        <v>69</v>
+      </c>
+      <c r="W10" t="s">
+        <v>81</v>
+      </c>
+      <c r="AA10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27">
+      <c r="A11">
+        <v>386</v>
+      </c>
+      <c r="B11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" t="s">
+        <v>50</v>
+      </c>
+      <c r="E11" t="s">
+        <v>58</v>
+      </c>
+      <c r="F11" t="s">
+        <v>59</v>
+      </c>
+      <c r="G11">
+        <v>2743</v>
+      </c>
+      <c r="H11" t="s">
         <v>64</v>
       </c>
-      <c r="N10" s="1">
+      <c r="I11" t="s">
+        <v>66</v>
+      </c>
+      <c r="J11" s="1">
+        <v>46244</v>
+      </c>
+      <c r="K11" s="1">
         <v>46246</v>
       </c>
-      <c r="Q10">
+      <c r="L11">
+        <v>6</v>
+      </c>
+      <c r="M11" t="s">
+        <v>68</v>
+      </c>
+      <c r="N11" s="1">
+        <v>46277</v>
+      </c>
+      <c r="Q11">
+        <v>-32</v>
+      </c>
+      <c r="R11">
         <v>-1</v>
       </c>
-      <c r="R10">
-        <v>6</v>
-      </c>
-      <c r="S10" t="s">
-        <v>65</v>
-      </c>
-      <c r="W10" t="s">
-        <v>77</v>
-      </c>
-      <c r="AA10" t="b">
+      <c r="T11" t="s">
+        <v>69</v>
+      </c>
+      <c r="W11" t="s">
+        <v>81</v>
+      </c>
+      <c r="AA11" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza Emergências (Contrato 005) e recalcula Cômputo Mensal (Fechamento Mensal)
10 emergências em aberto, 588 no histórico completo. Sem inconsistências.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="82">
   <si>
     <t>om_emg</t>
   </si>
@@ -109,6 +109,9 @@
     <t>BABE</t>
   </si>
   <si>
+    <t>BACO</t>
+  </si>
+  <si>
     <t>313260017747</t>
   </si>
   <si>
@@ -136,6 +139,9 @@
     <t>329260019264</t>
   </si>
   <si>
+    <t>386260013489</t>
+  </si>
+  <si>
     <t>1214134-1</t>
   </si>
   <si>
@@ -160,6 +166,9 @@
     <t>C662041-0102</t>
   </si>
   <si>
+    <t>9910333-1</t>
+  </si>
+  <si>
     <t>BELLCRANK ASSY</t>
   </si>
   <si>
@@ -179,6 +188,9 @@
   </si>
   <si>
     <t>INDICATOR FUEL</t>
+  </si>
+  <si>
+    <t>ENGINE MOUNT</t>
   </si>
   <si>
     <t>C</t>
@@ -257,8 +269,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -274,7 +294,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -282,12 +302,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -583,89 +621,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA10"/>
+  <dimension ref="A1:AA11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -677,42 +715,42 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F2" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G2">
         <v>2730</v>
       </c>
       <c r="H2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I2" t="s">
-        <v>61</v>
-      </c>
-      <c r="J2" s="1">
+        <v>65</v>
+      </c>
+      <c r="J2" s="2">
         <v>46076</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46080</v>
       </c>
       <c r="L2">
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>64</v>
-      </c>
-      <c r="N2" s="1">
+        <v>68</v>
+      </c>
+      <c r="N2" s="2">
         <v>46091</v>
       </c>
-      <c r="O2" s="1">
+      <c r="O2" s="2">
         <v>46287</v>
       </c>
       <c r="Q2">
@@ -722,19 +760,19 @@
         <v>165</v>
       </c>
       <c r="S2" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="T2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="U2" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="V2" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="W2" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -748,39 +786,39 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E3" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="F3" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G3">
         <v>2702</v>
       </c>
       <c r="H3" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I3" t="s">
-        <v>62</v>
-      </c>
-      <c r="J3" s="1">
+        <v>66</v>
+      </c>
+      <c r="J3" s="2">
         <v>46212</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46212</v>
       </c>
       <c r="L3">
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>64</v>
-      </c>
-      <c r="N3" s="1">
+        <v>68</v>
+      </c>
+      <c r="N3" s="2">
         <v>46243</v>
       </c>
       <c r="Q3">
@@ -790,16 +828,16 @@
         <v>33</v>
       </c>
       <c r="S3" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="T3" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="V3" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="W3" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -813,42 +851,42 @@
         <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E4" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="F4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G4">
         <v>2736</v>
       </c>
       <c r="H4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I4" t="s">
-        <v>62</v>
-      </c>
-      <c r="J4" s="1">
+        <v>66</v>
+      </c>
+      <c r="J4" s="2">
         <v>46216</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46217</v>
       </c>
       <c r="L4">
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>64</v>
-      </c>
-      <c r="N4" s="1">
+        <v>68</v>
+      </c>
+      <c r="N4" s="2">
         <v>46248</v>
       </c>
-      <c r="O4" s="1">
+      <c r="O4" s="2">
         <v>46248</v>
       </c>
       <c r="Q4">
@@ -858,16 +896,16 @@
         <v>28</v>
       </c>
       <c r="S4" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="T4" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="V4" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="W4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -881,39 +919,39 @@
         <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E5" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="F5" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G5">
         <v>2722</v>
       </c>
       <c r="H5" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I5" t="s">
-        <v>62</v>
-      </c>
-      <c r="J5" s="1">
+        <v>66</v>
+      </c>
+      <c r="J5" s="2">
         <v>46219</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46218</v>
       </c>
       <c r="L5">
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>64</v>
-      </c>
-      <c r="N5" s="1">
+        <v>68</v>
+      </c>
+      <c r="N5" s="2">
         <v>46249</v>
       </c>
       <c r="Q5">
@@ -923,19 +961,19 @@
         <v>27</v>
       </c>
       <c r="S5" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="T5" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="U5" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="V5" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="W5" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -949,42 +987,42 @@
         <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E6" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="F6" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G6">
         <v>2720</v>
       </c>
       <c r="H6" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I6" t="s">
-        <v>62</v>
-      </c>
-      <c r="J6" s="1">
+        <v>66</v>
+      </c>
+      <c r="J6" s="2">
         <v>46220</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46224</v>
       </c>
       <c r="L6">
         <v>10</v>
       </c>
       <c r="M6" t="s">
-        <v>64</v>
-      </c>
-      <c r="N6" s="1">
+        <v>68</v>
+      </c>
+      <c r="N6" s="2">
         <v>46255</v>
       </c>
-      <c r="O6" s="1">
+      <c r="O6" s="2">
         <v>46240</v>
       </c>
       <c r="Q6">
@@ -994,16 +1032,16 @@
         <v>21</v>
       </c>
       <c r="S6" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="T6" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="V6" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="W6" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1017,42 +1055,42 @@
         <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E7" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F7" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="G7">
         <v>2736</v>
       </c>
       <c r="H7" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="I7" t="s">
-        <v>62</v>
-      </c>
-      <c r="J7" s="1">
+        <v>66</v>
+      </c>
+      <c r="J7" s="2">
         <v>46205</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46234</v>
       </c>
       <c r="L7">
         <v>3</v>
       </c>
       <c r="M7" t="s">
-        <v>64</v>
-      </c>
-      <c r="N7" s="1">
+        <v>68</v>
+      </c>
+      <c r="N7" s="2">
         <v>46265</v>
       </c>
-      <c r="O7" s="1">
+      <c r="O7" s="2">
         <v>46239</v>
       </c>
       <c r="Q7">
@@ -1062,19 +1100,19 @@
         <v>11</v>
       </c>
       <c r="S7" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="T7" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="U7" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="V7" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="W7" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1088,39 +1126,39 @@
         <v>27</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E8" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F8" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="G8">
         <v>2737</v>
       </c>
       <c r="H8" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="I8" t="s">
-        <v>62</v>
-      </c>
-      <c r="J8" s="1">
+        <v>66</v>
+      </c>
+      <c r="J8" s="2">
         <v>46205</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46234</v>
       </c>
       <c r="L8">
         <v>3</v>
       </c>
       <c r="M8" t="s">
-        <v>64</v>
-      </c>
-      <c r="N8" s="1">
+        <v>68</v>
+      </c>
+      <c r="N8" s="2">
         <v>46265</v>
       </c>
       <c r="Q8">
@@ -1130,16 +1168,16 @@
         <v>11</v>
       </c>
       <c r="S8" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="T8" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="V8" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="W8" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1153,39 +1191,39 @@
         <v>30</v>
       </c>
       <c r="C9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E9" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F9" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G9">
         <v>2733</v>
       </c>
       <c r="H9" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I9" t="s">
-        <v>62</v>
-      </c>
-      <c r="J9" s="1">
+        <v>66</v>
+      </c>
+      <c r="J9" s="2">
         <v>46238</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46238</v>
       </c>
       <c r="L9">
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>64</v>
-      </c>
-      <c r="N9" s="1">
+        <v>68</v>
+      </c>
+      <c r="N9" s="2">
         <v>46269</v>
       </c>
       <c r="Q9">
@@ -1195,13 +1233,13 @@
         <v>7</v>
       </c>
       <c r="S9" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="T9" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="W9" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1215,54 +1253,113 @@
         <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E10" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F10" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G10">
         <v>2721</v>
       </c>
       <c r="H10" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="I10" t="s">
-        <v>63</v>
-      </c>
-      <c r="J10" s="1">
+        <v>67</v>
+      </c>
+      <c r="J10" s="2">
         <v>46241</v>
       </c>
-      <c r="K10" s="1">
-        <v>46239</v>
+      <c r="K10" s="2">
+        <v>46241</v>
       </c>
       <c r="L10">
         <v>2</v>
       </c>
       <c r="M10" t="s">
+        <v>68</v>
+      </c>
+      <c r="N10" s="2">
+        <v>46248</v>
+      </c>
+      <c r="Q10">
+        <v>-3</v>
+      </c>
+      <c r="R10">
+        <v>4</v>
+      </c>
+      <c r="S10" t="s">
+        <v>69</v>
+      </c>
+      <c r="W10" t="s">
+        <v>81</v>
+      </c>
+      <c r="AA10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27">
+      <c r="A11">
+        <v>386</v>
+      </c>
+      <c r="B11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" t="s">
+        <v>50</v>
+      </c>
+      <c r="E11" t="s">
+        <v>58</v>
+      </c>
+      <c r="F11" t="s">
+        <v>59</v>
+      </c>
+      <c r="G11">
+        <v>2743</v>
+      </c>
+      <c r="H11" t="s">
         <v>64</v>
       </c>
-      <c r="N10" s="1">
+      <c r="I11" t="s">
+        <v>66</v>
+      </c>
+      <c r="J11" s="2">
+        <v>46244</v>
+      </c>
+      <c r="K11" s="2">
         <v>46246</v>
       </c>
-      <c r="Q10">
+      <c r="L11">
+        <v>6</v>
+      </c>
+      <c r="M11" t="s">
+        <v>68</v>
+      </c>
+      <c r="N11" s="2">
+        <v>46277</v>
+      </c>
+      <c r="Q11">
+        <v>-32</v>
+      </c>
+      <c r="R11">
         <v>-1</v>
       </c>
-      <c r="R10">
-        <v>6</v>
-      </c>
-      <c r="S10" t="s">
-        <v>65</v>
-      </c>
-      <c r="W10" t="s">
-        <v>77</v>
-      </c>
-      <c r="AA10" t="b">
+      <c r="T11" t="s">
+        <v>69</v>
+      </c>
+      <c r="W11" t="s">
+        <v>81</v>
+      </c>
+      <c r="AA11" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (12/08/2026 08:54)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="84">
   <si>
     <t>om_emg</t>
   </si>
@@ -235,28 +235,34 @@
     <t>Alterado o tipo da emerg. de IPLR para ANCE. Godoy 22/07/26</t>
   </si>
   <si>
-    <t>Atendido 01 EA através da TSP 18122931. Outros 02 EA serão enviados pela empresa. Ramon 03/08/26.</t>
-  </si>
-  <si>
-    <t>Foi solicitado via email no dia 02-03-2 o atendimento do item com estoque FAB. Claudio -02-03-26 - Em resposta, a coordenadoria disse que o estque seria insuficiente. Foi verificado que na T.O da ANV o QPA para esse item são 2 EA, solicitei confirmação. - Cláudio -02-03-2026. Solicitado o cancelamento da emergência em função da quantidade cedida ao 2733 ter sido de 01ea. Considerando o QPA 02 ea. Encontra-se em tratativa junto a fiscalização e o gestor do contrato conforme mensagem de e-mail de 05/03. - SOLICITAÇÃO E-C98-26047.Colocado pedido AOG Textron J17626242 - previsão de entrega em Miami 05/08 AWB4238 em desembaraço no GIGRJ em 06/8/2026, previsao de CANAL hoje às 18 horas ATZ Marcio 6/8/2026 - MATERIAL EM RECEBIMENTO VEE ONE 07/08/2026 16:31, SERÁ ENVIADO NA SEGUNDA FEIRA</t>
-  </si>
-  <si>
-    <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - previsão de entrega em Miami 12/08</t>
+    <t>AWB 12750991113 volume retirado na loja GOLLOG - BSB por MICHELLIBCRISTINI DE BARROS em 10/08. Godoy 12/08/26.</t>
+  </si>
+  <si>
+    <t>Atendido 01 EA através da TSP 18122931. Outros 02 EA serão enviados pela empresa. Ramon 03/08/26. AWB 12750821282 volume retirado na loja GOLLOG - MAO por kleyton EM 06/08. Godoy 12/08/26.</t>
+  </si>
+  <si>
+    <t>Estoque com 12 EA do Pn LM600-9 (Alternado), Godoy 12/08/26.</t>
+  </si>
+  <si>
+    <t>Foi solicitado via email no dia 02-03-2 o atendimento do item com estoque FAB. Claudio -02-03-26 - Em resposta, a coordenadoria disse que o estque seria insuficiente. Foi verificado que na T.O da ANV o QPA para esse item são 2 EA, solicitei confirmação. - Cláudio -02-03-2026. Solicitado o cancelamento da emergência em função da quantidade cedida ao 2733 ter sido de 01ea. Considerando o QPA 02 ea. Encontra-se em tratativa junto a fiscalização e o gestor do contrato conforme mensagem de e-mail de 05/03. - SOLICITAÇÃO E-C98-26047.Colocado pedido AOG Textron J17626242 - previsão de entrega em Miami 05/08 AWB4238 em desembaraço no GIGRJ em 06/8/2026, previsao de CANAL hoje às 18 horas ATZ Marcio 6/8/2026 - MATERIAL EM RECEBIMENTO VEE ONE 07/08/2026 16:31, SERÁ ENVIADO NA SEGUNDA FEIRA - AWB 12752106375 dpe 14/08/2026</t>
+  </si>
+  <si>
+    <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - previsão de entrega em Miami 11/08</t>
   </si>
   <si>
     <t>Colocado pedido Textron IJ17575583 - entregue em Miami 15/07. Carga rercepcionada GIG 19/07 - Aguardando liberação do SEFAZ. ATZ 21/07 - material em processo de expedição RC 23/07/2026 - MATERIAL ENVIADO PELO RECIBO 639/FAB/26 - AWB 12750389603 DPE 13/08/2026</t>
   </si>
   <si>
-    <t>Item em bancada porem em pessimo estado, foi solicitado recolhimento de mais unidades para envio a oficina para tentativa de reparo ATZ Marcio 17/7/26. Solicitado abertura de O.S. para 3EA do item no dia 16-07-26 via Email para a Coordenadoria - CLA-21-07-26</t>
-  </si>
-  <si>
-    <t>Pedido I816822 entregue em Miami 27/07. Previsão de chegada GIG 30/07 (voo 4208). Previsão de canal 31/07 - MATERIAL RECEBIDO NA VEE ONE, EM PROCESSO DE EXPEDIÇÃO 04/08/2026 - ATZ RC - MATERIAL ENVIADO VIA RECIBO 650/FAB/26 - AWB 12750991113 DPE 06/08/2026, ESTÁ DISPONÍVEL PARA RETIRADA DESDE 04/08/2026</t>
+    <t>Item em bancada porem em pessimo estado, foi solicitado recolhimento de mais unidades para envio a oficina para tentativa de reparo ATZ Marcio 17/7/26. Solicitado abertura de O.S. para 3EA do item no dia 16-07-26 via Email para a Coordenadoria - CLA-21-07-26- SERÁ ENTREGUE PELA WILLIAM DPE DIA 12-08-26 - CLA-11-08</t>
+  </si>
+  <si>
+    <t>Pedido I816822 entregue em Miami 27/07. Previsão de chegada GIG 30/07 (voo 4208). Previsão de canal 31/07 - MATERIAL RECEBIDO NA VEE ONE, EM PROCESSO DE EXPEDIÇÃO 04/08/2026 - ATZ RC - MATERIAL ENVIADO VIA RECIBO 650/FAB/26 - AWB 12750991113 DPE 06/08/2026, ESTÁ DISPONÍVEL PARA RETIRADA DESDE 04/08/2026 - retirado na Gollog dia 10/08/2026</t>
   </si>
   <si>
     <t>Enviado para o Operador(02 EA), atendimento parcial, em 31/07/2026 -AWB 127-5041 6833- REZ - o outro 1 EA será atendido pelo estoque FAB. conforme solicitado por Email- CLA-03-08 - AWB 127-5082 1282 -1 EA ENVIADO ESTOQUE FAB - Material entregue dia 06/08/2026</t>
   </si>
   <si>
-    <t>Temos 4 EA em manutenção na William, será pedido prioridade. CLA-03-08</t>
+    <t>Foi solicitado abertura de O.S. no dia 7 -08-26 de 6 EA. As OSs foram abertas e aguardando recolhimento para reparo. CLA-10-08 - ITEM FOI RECOLHIDO PELA WILLIAM- CLA-11-08</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -725,13 +731,13 @@
         <v>46091</v>
       </c>
       <c r="O2" s="1">
-        <v>46287</v>
+        <v>46248</v>
       </c>
       <c r="Q2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R2">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="S2" t="s">
         <v>69</v>
@@ -743,10 +749,10 @@
         <v>71</v>
       </c>
       <c r="V2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="W2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -795,11 +801,14 @@
       <c r="N3" s="1">
         <v>46243</v>
       </c>
+      <c r="O3" s="1">
+        <v>46251</v>
+      </c>
       <c r="Q3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R3">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="S3" t="s">
         <v>69</v>
@@ -808,10 +817,10 @@
         <v>70</v>
       </c>
       <c r="V3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="W3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -864,10 +873,10 @@
         <v>46248</v>
       </c>
       <c r="Q4">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R4">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S4" t="s">
         <v>69</v>
@@ -876,10 +885,10 @@
         <v>70</v>
       </c>
       <c r="V4" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="W4" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -928,11 +937,14 @@
       <c r="N5" s="1">
         <v>46249</v>
       </c>
+      <c r="O5" s="1">
+        <v>46249</v>
+      </c>
       <c r="Q5">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="S5" t="s">
         <v>69</v>
@@ -944,10 +956,10 @@
         <v>72</v>
       </c>
       <c r="V5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="W5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -997,13 +1009,13 @@
         <v>46255</v>
       </c>
       <c r="O6" s="1">
-        <v>46240</v>
+        <v>46244</v>
       </c>
       <c r="Q6">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="R6">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S6" t="s">
         <v>69</v>
@@ -1011,11 +1023,14 @@
       <c r="T6" t="s">
         <v>69</v>
       </c>
+      <c r="U6" t="s">
+        <v>73</v>
+      </c>
       <c r="V6" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="W6" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1065,13 +1080,13 @@
         <v>46265</v>
       </c>
       <c r="O7" s="1">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="Q7">
-        <v>-20</v>
+        <v>-19</v>
       </c>
       <c r="R7">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="S7" t="s">
         <v>69</v>
@@ -1080,13 +1095,13 @@
         <v>70</v>
       </c>
       <c r="U7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="V7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="W7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1136,10 +1151,10 @@
         <v>46265</v>
       </c>
       <c r="Q8">
-        <v>-20</v>
+        <v>-19</v>
       </c>
       <c r="R8">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="S8" t="s">
         <v>69</v>
@@ -1147,11 +1162,8 @@
       <c r="T8" t="s">
         <v>70</v>
       </c>
-      <c r="V8" t="s">
-        <v>80</v>
-      </c>
       <c r="W8" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1201,10 +1213,10 @@
         <v>46269</v>
       </c>
       <c r="Q9">
-        <v>-24</v>
+        <v>-23</v>
       </c>
       <c r="R9">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S9" t="s">
         <v>69</v>
@@ -1213,7 +1225,7 @@
         <v>70</v>
       </c>
       <c r="W9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1263,16 +1275,19 @@
         <v>46248</v>
       </c>
       <c r="Q10">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S10" t="s">
         <v>69</v>
       </c>
+      <c r="V10" t="s">
+        <v>82</v>
+      </c>
       <c r="W10" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1322,16 +1337,22 @@
         <v>46277</v>
       </c>
       <c r="Q11">
-        <v>-32</v>
+        <v>-31</v>
       </c>
       <c r="R11">
-        <v>-1</v>
+        <v>0</v>
+      </c>
+      <c r="S11" t="s">
+        <v>70</v>
       </c>
       <c r="T11" t="s">
         <v>69</v>
       </c>
+      <c r="U11" t="s">
+        <v>75</v>
+      </c>
       <c r="W11" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (12/08/2026 11:23)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="104">
   <si>
     <t>om_emg</t>
   </si>
@@ -112,6 +112,12 @@
     <t>BACO</t>
   </si>
   <si>
+    <t>BACG</t>
+  </si>
+  <si>
+    <t>DACTA II</t>
+  </si>
+  <si>
     <t>313260017747</t>
   </si>
   <si>
@@ -139,9 +145,24 @@
     <t>329260019264</t>
   </si>
   <si>
+    <t>685260012560</t>
+  </si>
+  <si>
     <t>386260013489</t>
   </si>
   <si>
+    <t>685260012588</t>
+  </si>
+  <si>
+    <t>690260002522</t>
+  </si>
+  <si>
+    <t>384260009395</t>
+  </si>
+  <si>
+    <t>384260009396</t>
+  </si>
+  <si>
     <t>1214134-1</t>
   </si>
   <si>
@@ -166,9 +187,24 @@
     <t>C662041-0102</t>
   </si>
   <si>
+    <t>2641010-3</t>
+  </si>
+  <si>
     <t>9910333-1</t>
   </si>
   <si>
+    <t>51539-012N</t>
+  </si>
+  <si>
+    <t>3244897-4</t>
+  </si>
+  <si>
+    <t>2618510-10</t>
+  </si>
+  <si>
+    <t>S2616-285K4</t>
+  </si>
+  <si>
     <t>BELLCRANK ASSY</t>
   </si>
   <si>
@@ -190,9 +226,24 @@
     <t>INDICATOR FUEL</t>
   </si>
   <si>
+    <t>AXLE FITTING</t>
+  </si>
+  <si>
     <t>ENGINE MOUNT</t>
   </si>
   <si>
+    <t>CONTROL UNIT ASSY-GE</t>
+  </si>
+  <si>
+    <t>FUEL CONTROL UNIT</t>
+  </si>
+  <si>
+    <t>ALTERNATOR CONTROL U</t>
+  </si>
+  <si>
+    <t>ALTERNAD BELT</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -211,6 +262,9 @@
     <t>Aguardando solução</t>
   </si>
   <si>
+    <t>Expedido total</t>
+  </si>
+  <si>
     <t>IPLR</t>
   </si>
   <si>
@@ -241,7 +295,13 @@
     <t>Atendido 01 EA através da TSP 18122931. Outros 02 EA serão enviados pela empresa. Ramon 03/08/26. AWB 12750821282 volume retirado na loja GOLLOG - MAO por kleyton EM 06/08. Godoy 12/08/26.</t>
   </si>
   <si>
-    <t>Estoque com 12 EA do Pn LM600-9 (Alternado), Godoy 12/08/26.</t>
+    <t>item atendido com o estoque local pedido 18171852 em 10/08. Godoy 11/08. Está sendo definido se o PN está correto. Ramon 11/08/26.</t>
+  </si>
+  <si>
+    <t>Estoque com 12 EA do Pn LM600-9 (Alternado). Godoy 12/08/26.</t>
+  </si>
+  <si>
+    <t>Estoque no alternado 285K4. Caso use do estoque, verificar validade que consta no item. Ramon 12/08/26.</t>
   </si>
   <si>
     <t>Foi solicitado via email no dia 02-03-2 o atendimento do item com estoque FAB. Claudio -02-03-26 - Em resposta, a coordenadoria disse que o estque seria insuficiente. Foi verificado que na T.O da ANV o QPA para esse item são 2 EA, solicitei confirmação. - Cláudio -02-03-2026. Solicitado o cancelamento da emergência em função da quantidade cedida ao 2733 ter sido de 01ea. Considerando o QPA 02 ea. Encontra-se em tratativa junto a fiscalização e o gestor do contrato conforme mensagem de e-mail de 05/03. - SOLICITAÇÃO E-C98-26047.Colocado pedido AOG Textron J17626242 - previsão de entrega em Miami 05/08 AWB4238 em desembaraço no GIGRJ em 06/8/2026, previsao de CANAL hoje às 18 horas ATZ Marcio 6/8/2026 - MATERIAL EM RECEBIMENTO VEE ONE 07/08/2026 16:31, SERÁ ENVIADO NA SEGUNDA FEIRA - AWB 12752106375 dpe 14/08/2026</t>
@@ -601,7 +661,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA11"/>
+  <dimension ref="A1:AA16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -695,25 +755,25 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="E2" t="s">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="F2" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="G2">
         <v>2730</v>
       </c>
       <c r="H2" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="I2" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="J2" s="1">
         <v>46076</v>
@@ -725,7 +785,7 @@
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="N2" s="1">
         <v>46091</v>
@@ -740,19 +800,19 @@
         <v>166</v>
       </c>
       <c r="S2" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="T2" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="U2" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="V2" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="W2" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -766,25 +826,25 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="E3" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="F3" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="G3">
         <v>2702</v>
       </c>
       <c r="H3" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="I3" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="J3" s="1">
         <v>46212</v>
@@ -796,7 +856,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="N3" s="1">
         <v>46243</v>
@@ -811,16 +871,16 @@
         <v>34</v>
       </c>
       <c r="S3" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="T3" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="V3" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="W3" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -834,25 +894,25 @@
         <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E4" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="F4" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="G4">
         <v>2736</v>
       </c>
       <c r="H4" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="I4" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="J4" s="1">
         <v>46216</v>
@@ -864,7 +924,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="N4" s="1">
         <v>46248</v>
@@ -879,16 +939,16 @@
         <v>29</v>
       </c>
       <c r="S4" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="T4" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="V4" t="s">
-        <v>78</v>
+        <v>98</v>
       </c>
       <c r="W4" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -902,25 +962,25 @@
         <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="E5" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="F5" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="G5">
         <v>2722</v>
       </c>
       <c r="H5" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="I5" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="J5" s="1">
         <v>46219</v>
@@ -932,7 +992,7 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="N5" s="1">
         <v>46249</v>
@@ -947,19 +1007,19 @@
         <v>28</v>
       </c>
       <c r="S5" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="T5" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="U5" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="V5" t="s">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="W5" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -973,25 +1033,25 @@
         <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D6" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="E6" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="F6" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="G6">
         <v>2720</v>
       </c>
       <c r="H6" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="I6" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="J6" s="1">
         <v>46220</v>
@@ -1003,7 +1063,7 @@
         <v>10</v>
       </c>
       <c r="M6" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="N6" s="1">
         <v>46255</v>
@@ -1018,19 +1078,19 @@
         <v>22</v>
       </c>
       <c r="S6" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="T6" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="U6" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="V6" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="W6" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1044,25 +1104,25 @@
         <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D7" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="E7" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="F7" t="s">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="G7">
         <v>2736</v>
       </c>
       <c r="H7" t="s">
-        <v>63</v>
+        <v>80</v>
       </c>
       <c r="I7" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="J7" s="1">
         <v>46205</v>
@@ -1074,7 +1134,7 @@
         <v>3</v>
       </c>
       <c r="M7" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="N7" s="1">
         <v>46265</v>
@@ -1089,19 +1149,19 @@
         <v>12</v>
       </c>
       <c r="S7" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="T7" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="U7" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="V7" t="s">
-        <v>81</v>
+        <v>101</v>
       </c>
       <c r="W7" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1115,25 +1175,25 @@
         <v>27</v>
       </c>
       <c r="C8" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D8" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="E8" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="F8" t="s">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="G8">
         <v>2737</v>
       </c>
       <c r="H8" t="s">
-        <v>64</v>
+        <v>81</v>
       </c>
       <c r="I8" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="J8" s="1">
         <v>46205</v>
@@ -1145,7 +1205,7 @@
         <v>3</v>
       </c>
       <c r="M8" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="N8" s="1">
         <v>46265</v>
@@ -1157,13 +1217,13 @@
         <v>12</v>
       </c>
       <c r="S8" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="T8" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="W8" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1177,25 +1237,25 @@
         <v>30</v>
       </c>
       <c r="C9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D9" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="E9" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="F9" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="G9">
         <v>2733</v>
       </c>
       <c r="H9" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="I9" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="J9" s="1">
         <v>46238</v>
@@ -1207,7 +1267,7 @@
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="N9" s="1">
         <v>46269</v>
@@ -1219,13 +1279,13 @@
         <v>8</v>
       </c>
       <c r="S9" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="T9" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="W9" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1239,25 +1299,25 @@
         <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="E10" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="F10" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="G10">
         <v>2721</v>
       </c>
       <c r="H10" t="s">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="I10" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="J10" s="1">
         <v>46241</v>
@@ -1269,7 +1329,7 @@
         <v>2</v>
       </c>
       <c r="M10" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="N10" s="1">
         <v>46248</v>
@@ -1281,13 +1341,13 @@
         <v>5</v>
       </c>
       <c r="S10" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="V10" t="s">
-        <v>82</v>
+        <v>102</v>
       </c>
       <c r="W10" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1295,66 +1355,382 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>386</v>
+        <v>685</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D11" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="E11" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="F11" t="s">
-        <v>59</v>
+        <v>78</v>
       </c>
       <c r="G11">
-        <v>2743</v>
+        <v>2729</v>
       </c>
       <c r="H11" t="s">
-        <v>64</v>
+        <v>82</v>
       </c>
       <c r="I11" t="s">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="J11" s="1">
         <v>46244</v>
       </c>
       <c r="K11" s="1">
+        <v>46244</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11" t="s">
+        <v>86</v>
+      </c>
+      <c r="N11" s="1">
+        <v>46255</v>
+      </c>
+      <c r="Q11">
+        <v>-9</v>
+      </c>
+      <c r="R11">
+        <v>2</v>
+      </c>
+      <c r="S11" t="s">
+        <v>88</v>
+      </c>
+      <c r="T11" t="s">
+        <v>88</v>
+      </c>
+      <c r="U11" t="s">
+        <v>93</v>
+      </c>
+      <c r="W11" t="s">
+        <v>103</v>
+      </c>
+      <c r="AA11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27">
+      <c r="A12">
+        <v>386</v>
+      </c>
+      <c r="B12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" t="s">
+        <v>58</v>
+      </c>
+      <c r="E12" t="s">
+        <v>71</v>
+      </c>
+      <c r="F12" t="s">
+        <v>76</v>
+      </c>
+      <c r="G12">
+        <v>2743</v>
+      </c>
+      <c r="H12" t="s">
+        <v>81</v>
+      </c>
+      <c r="I12" t="s">
+        <v>84</v>
+      </c>
+      <c r="J12" s="1">
+        <v>46244</v>
+      </c>
+      <c r="K12" s="1">
         <v>46246</v>
       </c>
-      <c r="L11">
+      <c r="L12">
         <v>6</v>
       </c>
-      <c r="M11" t="s">
-        <v>68</v>
-      </c>
-      <c r="N11" s="1">
+      <c r="M12" t="s">
+        <v>86</v>
+      </c>
+      <c r="N12" s="1">
         <v>46277</v>
       </c>
-      <c r="Q11">
+      <c r="Q12">
         <v>-31</v>
       </c>
-      <c r="R11">
+      <c r="R12">
         <v>0</v>
       </c>
-      <c r="S11" t="s">
-        <v>70</v>
-      </c>
-      <c r="T11" t="s">
-        <v>69</v>
-      </c>
-      <c r="U11" t="s">
+      <c r="S12" t="s">
+        <v>88</v>
+      </c>
+      <c r="T12" t="s">
+        <v>87</v>
+      </c>
+      <c r="U12" t="s">
+        <v>94</v>
+      </c>
+      <c r="W12" t="s">
+        <v>103</v>
+      </c>
+      <c r="AA12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27">
+      <c r="A13">
+        <v>685</v>
+      </c>
+      <c r="B13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" t="s">
+        <v>45</v>
+      </c>
+      <c r="D13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E13" t="s">
+        <v>72</v>
+      </c>
+      <c r="F13" t="s">
+        <v>77</v>
+      </c>
+      <c r="G13">
+        <v>2729</v>
+      </c>
+      <c r="H13" t="s">
+        <v>81</v>
+      </c>
+      <c r="I13" t="s">
+        <v>83</v>
+      </c>
+      <c r="J13" s="1">
+        <v>46245</v>
+      </c>
+      <c r="K13" s="1">
+        <v>46246</v>
+      </c>
+      <c r="L13">
+        <v>1</v>
+      </c>
+      <c r="M13" t="s">
+        <v>86</v>
+      </c>
+      <c r="N13" s="1">
+        <v>46257</v>
+      </c>
+      <c r="Q13">
+        <v>-11</v>
+      </c>
+      <c r="R13">
+        <v>0</v>
+      </c>
+      <c r="S13" t="s">
+        <v>87</v>
+      </c>
+      <c r="T13" t="s">
+        <v>88</v>
+      </c>
+      <c r="W13" t="s">
+        <v>103</v>
+      </c>
+      <c r="AA13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:27">
+      <c r="A14">
+        <v>690</v>
+      </c>
+      <c r="B14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" t="s">
+        <v>60</v>
+      </c>
+      <c r="E14" t="s">
+        <v>73</v>
+      </c>
+      <c r="F14" t="s">
+        <v>77</v>
+      </c>
+      <c r="G14">
+        <v>2727</v>
+      </c>
+      <c r="H14" t="s">
+        <v>81</v>
+      </c>
+      <c r="I14" t="s">
+        <v>83</v>
+      </c>
+      <c r="J14" s="1">
+        <v>46245</v>
+      </c>
+      <c r="K14" s="1">
+        <v>46246</v>
+      </c>
+      <c r="L14">
+        <v>1</v>
+      </c>
+      <c r="M14" t="s">
+        <v>86</v>
+      </c>
+      <c r="N14" s="1">
+        <v>46257</v>
+      </c>
+      <c r="Q14">
+        <v>-11</v>
+      </c>
+      <c r="R14">
+        <v>0</v>
+      </c>
+      <c r="S14" t="s">
+        <v>87</v>
+      </c>
+      <c r="T14" t="s">
+        <v>87</v>
+      </c>
+      <c r="W14" t="s">
+        <v>103</v>
+      </c>
+      <c r="AA14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27">
+      <c r="A15">
+        <v>384</v>
+      </c>
+      <c r="B15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" t="s">
+        <v>47</v>
+      </c>
+      <c r="D15" t="s">
+        <v>61</v>
+      </c>
+      <c r="E15" t="s">
+        <v>74</v>
+      </c>
+      <c r="F15" t="s">
+        <v>78</v>
+      </c>
+      <c r="G15">
+        <v>2742</v>
+      </c>
+      <c r="H15" t="s">
+        <v>81</v>
+      </c>
+      <c r="I15" t="s">
+        <v>84</v>
+      </c>
+      <c r="J15" s="1">
+        <v>46245</v>
+      </c>
+      <c r="K15" s="1">
+        <v>46246</v>
+      </c>
+      <c r="L15">
+        <v>1</v>
+      </c>
+      <c r="M15" t="s">
+        <v>86</v>
+      </c>
+      <c r="N15" s="1">
+        <v>46277</v>
+      </c>
+      <c r="Q15">
+        <v>-31</v>
+      </c>
+      <c r="R15">
+        <v>0</v>
+      </c>
+      <c r="S15" t="s">
+        <v>87</v>
+      </c>
+      <c r="T15" t="s">
+        <v>87</v>
+      </c>
+      <c r="W15" t="s">
+        <v>103</v>
+      </c>
+      <c r="AA15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27">
+      <c r="A16">
+        <v>384</v>
+      </c>
+      <c r="B16" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" t="s">
+        <v>48</v>
+      </c>
+      <c r="D16" t="s">
+        <v>62</v>
+      </c>
+      <c r="E16" t="s">
         <v>75</v>
       </c>
-      <c r="W11" t="s">
-        <v>83</v>
-      </c>
-      <c r="AA11" t="b">
+      <c r="F16" t="s">
+        <v>76</v>
+      </c>
+      <c r="G16">
+        <v>2742</v>
+      </c>
+      <c r="H16" t="s">
+        <v>81</v>
+      </c>
+      <c r="I16" t="s">
+        <v>84</v>
+      </c>
+      <c r="J16" s="1">
+        <v>46245</v>
+      </c>
+      <c r="K16" s="1">
+        <v>46246</v>
+      </c>
+      <c r="L16">
+        <v>1</v>
+      </c>
+      <c r="M16" t="s">
+        <v>86</v>
+      </c>
+      <c r="N16" s="1">
+        <v>46277</v>
+      </c>
+      <c r="Q16">
+        <v>-31</v>
+      </c>
+      <c r="R16">
+        <v>0</v>
+      </c>
+      <c r="S16" t="s">
+        <v>88</v>
+      </c>
+      <c r="T16" t="s">
+        <v>87</v>
+      </c>
+      <c r="U16" t="s">
+        <v>95</v>
+      </c>
+      <c r="W16" t="s">
+        <v>103</v>
+      </c>
+      <c r="AA16" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (13/08/2026 08:55)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="104">
   <si>
     <t>om_emg</t>
   </si>
@@ -97,15 +97,15 @@
     <t>em_aberto</t>
   </si>
   <si>
+    <t>BANT</t>
+  </si>
+  <si>
+    <t>BABR</t>
+  </si>
+  <si>
     <t>BAMN</t>
   </si>
   <si>
-    <t>BANT</t>
-  </si>
-  <si>
-    <t>BABR</t>
-  </si>
-  <si>
     <t>BABE</t>
   </si>
   <si>
@@ -118,15 +118,9 @@
     <t>DACTA II</t>
   </si>
   <si>
-    <t>313260017747</t>
-  </si>
-  <si>
     <t>685260012350</t>
   </si>
   <si>
-    <t>313260018674</t>
-  </si>
-  <si>
     <t>685260012387</t>
   </si>
   <si>
@@ -163,15 +157,9 @@
     <t>384260009396</t>
   </si>
   <si>
-    <t>1214134-1</t>
-  </si>
-  <si>
     <t>030-1094-58</t>
   </si>
   <si>
-    <t>205842-1</t>
-  </si>
-  <si>
     <t>066-3084-32</t>
   </si>
   <si>
@@ -205,9 +193,6 @@
     <t>S2616-285K4</t>
   </si>
   <si>
-    <t>BELLCRANK ASSY</t>
-  </si>
-  <si>
     <t>CONNECTOR</t>
   </si>
   <si>
@@ -265,15 +250,15 @@
     <t>Expedido total</t>
   </si>
   <si>
+    <t>ANCE</t>
+  </si>
+  <si>
+    <t>AIFP</t>
+  </si>
+  <si>
     <t>IPLR</t>
   </si>
   <si>
-    <t>ANCE</t>
-  </si>
-  <si>
-    <t>AIFP</t>
-  </si>
-  <si>
     <t>EA</t>
   </si>
   <si>
@@ -283,9 +268,6 @@
     <t>Sim</t>
   </si>
   <si>
-    <t>Foram cedidos para o C-98 2733. / De acordo com o manual da aeronave, o QPA é 02 EA por cadeira. Sendo o total para a aeronave 04 EA.A demanda aberta foi de  4EA, o SO Bispo que intermediou . Wallace 29.05</t>
-  </si>
-  <si>
     <t>Alterado o tipo da emerg. de IPLR para ANCE. Godoy 22/07/26</t>
   </si>
   <si>
@@ -301,16 +283,13 @@
     <t>Estoque com 12 EA do Pn LM600-9 (Alternado). Godoy 12/08/26.</t>
   </si>
   <si>
+    <t>AWB 127-5256 7745 com previsão de entrega em 14/08. Ramon 13/08/26</t>
+  </si>
+  <si>
     <t>Estoque no alternado 285K4. Caso use do estoque, verificar validade que consta no item. Ramon 12/08/26.</t>
   </si>
   <si>
-    <t>Foi solicitado via email no dia 02-03-2 o atendimento do item com estoque FAB. Claudio -02-03-26 - Em resposta, a coordenadoria disse que o estque seria insuficiente. Foi verificado que na T.O da ANV o QPA para esse item são 2 EA, solicitei confirmação. - Cláudio -02-03-2026. Solicitado o cancelamento da emergência em função da quantidade cedida ao 2733 ter sido de 01ea. Considerando o QPA 02 ea. Encontra-se em tratativa junto a fiscalização e o gestor do contrato conforme mensagem de e-mail de 05/03. - SOLICITAÇÃO E-C98-26047.Colocado pedido AOG Textron J17626242 - previsão de entrega em Miami 05/08 AWB4238 em desembaraço no GIGRJ em 06/8/2026, previsao de CANAL hoje às 18 horas ATZ Marcio 6/8/2026 - MATERIAL EM RECEBIMENTO VEE ONE 07/08/2026 16:31, SERÁ ENVIADO NA SEGUNDA FEIRA - AWB 12752106375 dpe 14/08/2026</t>
-  </si>
-  <si>
-    <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - previsão de entrega em Miami 11/08</t>
-  </si>
-  <si>
-    <t>Colocado pedido Textron IJ17575583 - entregue em Miami 15/07. Carga rercepcionada GIG 19/07 - Aguardando liberação do SEFAZ. ATZ 21/07 - material em processo de expedição RC 23/07/2026 - MATERIAL ENVIADO PELO RECIBO 639/FAB/26 - AWB 12750389603 DPE 13/08/2026</t>
+    <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Consolidando embarque próximo voo para o GIG</t>
   </si>
   <si>
     <t>Item em bancada porem em pessimo estado, foi solicitado recolhimento de mais unidades para envio a oficina para tentativa de reparo ATZ Marcio 17/7/26. Solicitado abertura de O.S. para 3EA do item no dia 16-07-26 via Email para a Coordenadoria - CLA-21-07-26- SERÁ ENTREGUE PELA WILLIAM DPE DIA 12-08-26 - CLA-11-08</t>
@@ -322,7 +301,28 @@
     <t>Enviado para o Operador(02 EA), atendimento parcial, em 31/07/2026 -AWB 127-5041 6833- REZ - o outro 1 EA será atendido pelo estoque FAB. conforme solicitado por Email- CLA-03-08 - AWB 127-5082 1282 -1 EA ENVIADO ESTOQUE FAB - Material entregue dia 06/08/2026</t>
   </si>
   <si>
+    <t>Temos 4 EA em manutenção na William, será pedido prioridade. CLA-03-08</t>
+  </si>
+  <si>
+    <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
+  </si>
+  <si>
     <t>Foi solicitado abertura de O.S. no dia 7 -08-26 de 6 EA. As OSs foram abertas e aguardando recolhimento para reparo. CLA-10-08 - ITEM FOI RECOLHIDO PELA WILLIAM- CLA-11-08</t>
+  </si>
+  <si>
+    <t>Foi solicitado atendimento com estoque FAB - CLA- 10-08, ITEM PRONTO PARA EMBARQUE, AGUARDANDO NOTA FISCAL - CLA-11-08</t>
+  </si>
+  <si>
+    <t>TEM ESTOQUE NA VEEONE</t>
+  </si>
+  <si>
+    <t>Em estoque na V1 JPA 12/8/26 Marcio 13:23</t>
+  </si>
+  <si>
+    <t>Previsao de entrega da oficina do RJ na V1 JPA 13/8/2026 durante o dia, horario comercial, ATZ Marcio 12/8 13:22hs</t>
+  </si>
+  <si>
+    <t>1 Unidade na oficina em BH William, solicitado prioridade na entrega DPE 14/8, aguardando orçamento final ATZ Marcio 12/8 13:24hs</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -661,7 +661,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA16"/>
+  <dimension ref="A1:AA14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -749,7 +749,7 @@
     </row>
     <row r="2" spans="1:27">
       <c r="A2">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B2" t="s">
         <v>27</v>
@@ -758,58 +758,55 @@
         <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F2" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="G2">
-        <v>2730</v>
+        <v>2702</v>
       </c>
       <c r="H2" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="I2" t="s">
+        <v>78</v>
+      </c>
+      <c r="J2" s="1">
+        <v>46212</v>
+      </c>
+      <c r="K2" s="1">
+        <v>46212</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2" t="s">
+        <v>81</v>
+      </c>
+      <c r="N2" s="1">
+        <v>46243</v>
+      </c>
+      <c r="O2" s="1">
+        <v>46251</v>
+      </c>
+      <c r="Q2">
+        <v>4</v>
+      </c>
+      <c r="R2">
+        <v>35</v>
+      </c>
+      <c r="S2" t="s">
+        <v>82</v>
+      </c>
+      <c r="T2" t="s">
         <v>83</v>
       </c>
-      <c r="J2" s="1">
-        <v>46076</v>
-      </c>
-      <c r="K2" s="1">
-        <v>46080</v>
-      </c>
-      <c r="L2">
-        <v>4</v>
-      </c>
-      <c r="M2" t="s">
-        <v>86</v>
-      </c>
-      <c r="N2" s="1">
-        <v>46091</v>
-      </c>
-      <c r="O2" s="1">
-        <v>46248</v>
-      </c>
-      <c r="Q2">
-        <v>155</v>
-      </c>
-      <c r="R2">
-        <v>166</v>
-      </c>
-      <c r="S2" t="s">
-        <v>87</v>
-      </c>
-      <c r="T2" t="s">
-        <v>88</v>
-      </c>
-      <c r="U2" t="s">
-        <v>89</v>
-      </c>
       <c r="V2" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="W2" t="s">
         <v>103</v>
@@ -823,61 +820,64 @@
         <v>685</v>
       </c>
       <c r="B3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C3" t="s">
         <v>35</v>
       </c>
       <c r="D3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F3" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="G3">
-        <v>2702</v>
+        <v>2722</v>
       </c>
       <c r="H3" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="I3" t="s">
+        <v>78</v>
+      </c>
+      <c r="J3" s="1">
+        <v>46219</v>
+      </c>
+      <c r="K3" s="1">
+        <v>46218</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3" t="s">
+        <v>81</v>
+      </c>
+      <c r="N3" s="1">
+        <v>46249</v>
+      </c>
+      <c r="O3" s="1">
+        <v>46249</v>
+      </c>
+      <c r="Q3">
+        <v>-2</v>
+      </c>
+      <c r="R3">
+        <v>29</v>
+      </c>
+      <c r="S3" t="s">
+        <v>82</v>
+      </c>
+      <c r="T3" t="s">
+        <v>83</v>
+      </c>
+      <c r="U3" t="s">
         <v>84</v>
       </c>
-      <c r="J3" s="1">
-        <v>46212</v>
-      </c>
-      <c r="K3" s="1">
-        <v>46212</v>
-      </c>
-      <c r="L3">
-        <v>1</v>
-      </c>
-      <c r="M3" t="s">
-        <v>86</v>
-      </c>
-      <c r="N3" s="1">
-        <v>46243</v>
-      </c>
-      <c r="O3" s="1">
-        <v>46251</v>
-      </c>
-      <c r="Q3">
-        <v>3</v>
-      </c>
-      <c r="R3">
-        <v>34</v>
-      </c>
-      <c r="S3" t="s">
-        <v>87</v>
-      </c>
-      <c r="T3" t="s">
-        <v>88</v>
-      </c>
       <c r="V3" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="W3" t="s">
         <v>103</v>
@@ -888,64 +888,67 @@
     </row>
     <row r="4" spans="1:27">
       <c r="A4">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s">
         <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F4" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="G4">
-        <v>2736</v>
+        <v>2720</v>
       </c>
       <c r="H4" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="I4" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="J4" s="1">
-        <v>46216</v>
+        <v>46220</v>
       </c>
       <c r="K4" s="1">
-        <v>46217</v>
+        <v>46224</v>
       </c>
       <c r="L4">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="M4" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="N4" s="1">
-        <v>46248</v>
+        <v>46255</v>
       </c>
       <c r="O4" s="1">
-        <v>46248</v>
+        <v>46244</v>
       </c>
       <c r="Q4">
-        <v>-2</v>
+        <v>-8</v>
       </c>
       <c r="R4">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="S4" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="T4" t="s">
-        <v>88</v>
+        <v>82</v>
+      </c>
+      <c r="U4" t="s">
+        <v>85</v>
       </c>
       <c r="V4" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="W4" t="s">
         <v>103</v>
@@ -956,67 +959,67 @@
     </row>
     <row r="5" spans="1:27">
       <c r="A5">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C5" t="s">
         <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E5" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F5" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="G5">
-        <v>2722</v>
+        <v>2736</v>
       </c>
       <c r="H5" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="I5" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="J5" s="1">
-        <v>46219</v>
+        <v>46205</v>
       </c>
       <c r="K5" s="1">
-        <v>46218</v>
+        <v>46234</v>
       </c>
       <c r="L5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M5" t="s">
+        <v>81</v>
+      </c>
+      <c r="N5" s="1">
+        <v>46265</v>
+      </c>
+      <c r="O5" s="1">
+        <v>46240</v>
+      </c>
+      <c r="Q5">
+        <v>-18</v>
+      </c>
+      <c r="R5">
+        <v>13</v>
+      </c>
+      <c r="S5" t="s">
+        <v>82</v>
+      </c>
+      <c r="T5" t="s">
+        <v>83</v>
+      </c>
+      <c r="U5" t="s">
         <v>86</v>
       </c>
-      <c r="N5" s="1">
-        <v>46249</v>
-      </c>
-      <c r="O5" s="1">
-        <v>46249</v>
-      </c>
-      <c r="Q5">
-        <v>-3</v>
-      </c>
-      <c r="R5">
-        <v>28</v>
-      </c>
-      <c r="S5" t="s">
-        <v>87</v>
-      </c>
-      <c r="T5" t="s">
-        <v>88</v>
-      </c>
-      <c r="U5" t="s">
-        <v>90</v>
-      </c>
       <c r="V5" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="W5" t="s">
         <v>103</v>
@@ -1027,7 +1030,7 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6">
-        <v>329</v>
+        <v>313</v>
       </c>
       <c r="B6" t="s">
         <v>29</v>
@@ -1036,58 +1039,55 @@
         <v>38</v>
       </c>
       <c r="D6" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E6" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F6" t="s">
+        <v>73</v>
+      </c>
+      <c r="G6">
+        <v>2737</v>
+      </c>
+      <c r="H6" t="s">
         <v>76</v>
       </c>
-      <c r="G6">
-        <v>2720</v>
-      </c>
-      <c r="H6" t="s">
-        <v>79</v>
-      </c>
       <c r="I6" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="J6" s="1">
-        <v>46220</v>
+        <v>46205</v>
       </c>
       <c r="K6" s="1">
-        <v>46224</v>
+        <v>46234</v>
       </c>
       <c r="L6">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="M6" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="N6" s="1">
-        <v>46255</v>
+        <v>46265</v>
       </c>
       <c r="O6" s="1">
-        <v>46244</v>
+        <v>46265</v>
       </c>
       <c r="Q6">
-        <v>-9</v>
+        <v>-18</v>
       </c>
       <c r="R6">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="S6" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="T6" t="s">
-        <v>87</v>
-      </c>
-      <c r="U6" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="V6" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="W6" t="s">
         <v>103</v>
@@ -1098,67 +1098,64 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>313</v>
+        <v>396</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C7" t="s">
         <v>39</v>
       </c>
       <c r="D7" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E7" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="F7" t="s">
+        <v>71</v>
+      </c>
+      <c r="G7">
+        <v>2733</v>
+      </c>
+      <c r="H7" t="s">
+        <v>74</v>
+      </c>
+      <c r="I7" t="s">
         <v>78</v>
       </c>
-      <c r="G7">
-        <v>2736</v>
-      </c>
-      <c r="H7" t="s">
-        <v>80</v>
-      </c>
-      <c r="I7" t="s">
-        <v>84</v>
-      </c>
       <c r="J7" s="1">
-        <v>46205</v>
+        <v>46238</v>
       </c>
       <c r="K7" s="1">
-        <v>46234</v>
+        <v>46238</v>
       </c>
       <c r="L7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="N7" s="1">
-        <v>46265</v>
+        <v>46269</v>
       </c>
       <c r="O7" s="1">
-        <v>46240</v>
+        <v>46269</v>
       </c>
       <c r="Q7">
-        <v>-19</v>
+        <v>-22</v>
       </c>
       <c r="R7">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="S7" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="T7" t="s">
-        <v>88</v>
-      </c>
-      <c r="U7" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="V7" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="W7" t="s">
         <v>103</v>
@@ -1169,58 +1166,58 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
         <v>40</v>
       </c>
       <c r="D8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E8" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="F8" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="G8">
-        <v>2737</v>
+        <v>2721</v>
       </c>
       <c r="H8" t="s">
+        <v>74</v>
+      </c>
+      <c r="I8" t="s">
+        <v>79</v>
+      </c>
+      <c r="J8" s="1">
+        <v>46241</v>
+      </c>
+      <c r="K8" s="1">
+        <v>46241</v>
+      </c>
+      <c r="L8">
+        <v>2</v>
+      </c>
+      <c r="M8" t="s">
         <v>81</v>
       </c>
-      <c r="I8" t="s">
-        <v>84</v>
-      </c>
-      <c r="J8" s="1">
-        <v>46205</v>
-      </c>
-      <c r="K8" s="1">
-        <v>46234</v>
-      </c>
-      <c r="L8">
-        <v>3</v>
-      </c>
-      <c r="M8" t="s">
-        <v>86</v>
-      </c>
       <c r="N8" s="1">
-        <v>46265</v>
+        <v>46248</v>
       </c>
       <c r="Q8">
-        <v>-19</v>
+        <v>-1</v>
       </c>
       <c r="R8">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="S8" t="s">
-        <v>87</v>
-      </c>
-      <c r="T8" t="s">
-        <v>88</v>
+        <v>82</v>
+      </c>
+      <c r="V8" t="s">
+        <v>97</v>
       </c>
       <c r="W8" t="s">
         <v>103</v>
@@ -1231,58 +1228,67 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9">
-        <v>396</v>
+        <v>685</v>
       </c>
       <c r="B9" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C9" t="s">
         <v>41</v>
       </c>
       <c r="D9" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E9" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F9" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="G9">
-        <v>2733</v>
+        <v>2729</v>
       </c>
       <c r="H9" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="I9" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="J9" s="1">
-        <v>46238</v>
+        <v>46244</v>
       </c>
       <c r="K9" s="1">
-        <v>46238</v>
+        <v>46244</v>
       </c>
       <c r="L9">
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="N9" s="1">
-        <v>46269</v>
+        <v>46255</v>
+      </c>
+      <c r="O9" s="1">
+        <v>46255</v>
       </c>
       <c r="Q9">
-        <v>-23</v>
+        <v>-8</v>
       </c>
       <c r="R9">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="S9" t="s">
+        <v>83</v>
+      </c>
+      <c r="T9" t="s">
+        <v>83</v>
+      </c>
+      <c r="U9" t="s">
         <v>87</v>
       </c>
-      <c r="T9" t="s">
-        <v>88</v>
+      <c r="V9" t="s">
+        <v>98</v>
       </c>
       <c r="W9" t="s">
         <v>103</v>
@@ -1293,58 +1299,64 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>329</v>
+        <v>386</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C10" t="s">
         <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E10" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="F10" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="G10">
-        <v>2721</v>
+        <v>2743</v>
       </c>
       <c r="H10" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="I10" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="J10" s="1">
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="K10" s="1">
-        <v>46241</v>
+        <v>46246</v>
       </c>
       <c r="L10">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="M10" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="N10" s="1">
-        <v>46248</v>
+        <v>46277</v>
       </c>
       <c r="Q10">
-        <v>-2</v>
+        <v>-30</v>
       </c>
       <c r="R10">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="S10" t="s">
-        <v>87</v>
+        <v>83</v>
+      </c>
+      <c r="T10" t="s">
+        <v>82</v>
+      </c>
+      <c r="U10" t="s">
+        <v>88</v>
       </c>
       <c r="V10" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="W10" t="s">
         <v>103</v>
@@ -1358,58 +1370,61 @@
         <v>685</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C11" t="s">
         <v>43</v>
       </c>
       <c r="D11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E11" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="F11" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="G11">
         <v>2729</v>
       </c>
       <c r="H11" t="s">
+        <v>76</v>
+      </c>
+      <c r="I11" t="s">
+        <v>80</v>
+      </c>
+      <c r="J11" s="1">
+        <v>46245</v>
+      </c>
+      <c r="K11" s="1">
+        <v>46246</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11" t="s">
+        <v>81</v>
+      </c>
+      <c r="N11" s="1">
+        <v>46257</v>
+      </c>
+      <c r="Q11">
+        <v>-10</v>
+      </c>
+      <c r="R11">
+        <v>1</v>
+      </c>
+      <c r="S11" t="s">
         <v>82</v>
       </c>
-      <c r="I11" t="s">
+      <c r="T11" t="s">
         <v>83</v>
       </c>
-      <c r="J11" s="1">
-        <v>46244</v>
-      </c>
-      <c r="K11" s="1">
-        <v>46244</v>
-      </c>
-      <c r="L11">
-        <v>1</v>
-      </c>
-      <c r="M11" t="s">
-        <v>86</v>
-      </c>
-      <c r="N11" s="1">
-        <v>46255</v>
-      </c>
-      <c r="Q11">
-        <v>-9</v>
-      </c>
-      <c r="R11">
-        <v>2</v>
-      </c>
-      <c r="S11" t="s">
-        <v>88</v>
-      </c>
-      <c r="T11" t="s">
-        <v>88</v>
-      </c>
       <c r="U11" t="s">
-        <v>93</v>
+        <v>89</v>
+      </c>
+      <c r="V11" t="s">
+        <v>100</v>
       </c>
       <c r="W11" t="s">
         <v>103</v>
@@ -1420,61 +1435,61 @@
     </row>
     <row r="12" spans="1:27">
       <c r="A12">
-        <v>386</v>
+        <v>690</v>
       </c>
       <c r="B12" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C12" t="s">
         <v>44</v>
       </c>
       <c r="D12" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E12" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F12" t="s">
+        <v>72</v>
+      </c>
+      <c r="G12">
+        <v>2727</v>
+      </c>
+      <c r="H12" t="s">
         <v>76</v>
       </c>
-      <c r="G12">
-        <v>2743</v>
-      </c>
-      <c r="H12" t="s">
-        <v>81</v>
-      </c>
       <c r="I12" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="J12" s="1">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="K12" s="1">
         <v>46246</v>
       </c>
       <c r="L12">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="N12" s="1">
-        <v>46277</v>
+        <v>46257</v>
       </c>
       <c r="Q12">
-        <v>-31</v>
+        <v>-10</v>
       </c>
       <c r="R12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S12" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="T12" t="s">
-        <v>87</v>
-      </c>
-      <c r="U12" t="s">
-        <v>94</v>
+        <v>82</v>
+      </c>
+      <c r="V12" t="s">
+        <v>101</v>
       </c>
       <c r="W12" t="s">
         <v>103</v>
@@ -1485,31 +1500,31 @@
     </row>
     <row r="13" spans="1:27">
       <c r="A13">
-        <v>685</v>
+        <v>384</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="C13" t="s">
         <v>45</v>
       </c>
       <c r="D13" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E13" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="F13" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="G13">
-        <v>2729</v>
+        <v>2742</v>
       </c>
       <c r="H13" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="I13" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="J13" s="1">
         <v>46245</v>
@@ -1521,22 +1536,25 @@
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="N13" s="1">
-        <v>46257</v>
+        <v>46277</v>
       </c>
       <c r="Q13">
-        <v>-11</v>
+        <v>-30</v>
       </c>
       <c r="R13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S13" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="T13" t="s">
-        <v>88</v>
+        <v>82</v>
+      </c>
+      <c r="V13" t="s">
+        <v>102</v>
       </c>
       <c r="W13" t="s">
         <v>103</v>
@@ -1547,31 +1565,31 @@
     </row>
     <row r="14" spans="1:27">
       <c r="A14">
-        <v>690</v>
+        <v>384</v>
       </c>
       <c r="B14" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C14" t="s">
         <v>46</v>
       </c>
       <c r="D14" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E14" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="F14" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="G14">
-        <v>2727</v>
+        <v>2742</v>
       </c>
       <c r="H14" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="I14" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="J14" s="1">
         <v>46245</v>
@@ -1583,154 +1601,33 @@
         <v>1</v>
       </c>
       <c r="M14" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="N14" s="1">
-        <v>46257</v>
+        <v>46277</v>
       </c>
       <c r="Q14">
-        <v>-11</v>
+        <v>-30</v>
       </c>
       <c r="R14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S14" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="T14" t="s">
-        <v>87</v>
+        <v>82</v>
+      </c>
+      <c r="U14" t="s">
+        <v>90</v>
+      </c>
+      <c r="V14" t="s">
+        <v>99</v>
       </c>
       <c r="W14" t="s">
         <v>103</v>
       </c>
       <c r="AA14" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:27">
-      <c r="A15">
-        <v>384</v>
-      </c>
-      <c r="B15" t="s">
-        <v>33</v>
-      </c>
-      <c r="C15" t="s">
-        <v>47</v>
-      </c>
-      <c r="D15" t="s">
-        <v>61</v>
-      </c>
-      <c r="E15" t="s">
-        <v>74</v>
-      </c>
-      <c r="F15" t="s">
-        <v>78</v>
-      </c>
-      <c r="G15">
-        <v>2742</v>
-      </c>
-      <c r="H15" t="s">
-        <v>81</v>
-      </c>
-      <c r="I15" t="s">
-        <v>84</v>
-      </c>
-      <c r="J15" s="1">
-        <v>46245</v>
-      </c>
-      <c r="K15" s="1">
-        <v>46246</v>
-      </c>
-      <c r="L15">
-        <v>1</v>
-      </c>
-      <c r="M15" t="s">
-        <v>86</v>
-      </c>
-      <c r="N15" s="1">
-        <v>46277</v>
-      </c>
-      <c r="Q15">
-        <v>-31</v>
-      </c>
-      <c r="R15">
-        <v>0</v>
-      </c>
-      <c r="S15" t="s">
-        <v>87</v>
-      </c>
-      <c r="T15" t="s">
-        <v>87</v>
-      </c>
-      <c r="W15" t="s">
-        <v>103</v>
-      </c>
-      <c r="AA15" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:27">
-      <c r="A16">
-        <v>384</v>
-      </c>
-      <c r="B16" t="s">
-        <v>33</v>
-      </c>
-      <c r="C16" t="s">
-        <v>48</v>
-      </c>
-      <c r="D16" t="s">
-        <v>62</v>
-      </c>
-      <c r="E16" t="s">
-        <v>75</v>
-      </c>
-      <c r="F16" t="s">
-        <v>76</v>
-      </c>
-      <c r="G16">
-        <v>2742</v>
-      </c>
-      <c r="H16" t="s">
-        <v>81</v>
-      </c>
-      <c r="I16" t="s">
-        <v>84</v>
-      </c>
-      <c r="J16" s="1">
-        <v>46245</v>
-      </c>
-      <c r="K16" s="1">
-        <v>46246</v>
-      </c>
-      <c r="L16">
-        <v>1</v>
-      </c>
-      <c r="M16" t="s">
-        <v>86</v>
-      </c>
-      <c r="N16" s="1">
-        <v>46277</v>
-      </c>
-      <c r="Q16">
-        <v>-31</v>
-      </c>
-      <c r="R16">
-        <v>0</v>
-      </c>
-      <c r="S16" t="s">
-        <v>88</v>
-      </c>
-      <c r="T16" t="s">
-        <v>87</v>
-      </c>
-      <c r="U16" t="s">
-        <v>95</v>
-      </c>
-      <c r="W16" t="s">
-        <v>103</v>
-      </c>
-      <c r="AA16" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (13/08/2026 11:25)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="103">
   <si>
     <t>om_emg</t>
   </si>
@@ -100,15 +100,15 @@
     <t>BANT</t>
   </si>
   <si>
+    <t>BAMN</t>
+  </si>
+  <si>
+    <t>BABE</t>
+  </si>
+  <si>
     <t>BABR</t>
   </si>
   <si>
-    <t>BAMN</t>
-  </si>
-  <si>
-    <t>BABE</t>
-  </si>
-  <si>
     <t>BACO</t>
   </si>
   <si>
@@ -124,9 +124,6 @@
     <t>685260012387</t>
   </si>
   <si>
-    <t>329260019225</t>
-  </si>
-  <si>
     <t>313260018657</t>
   </si>
   <si>
@@ -157,15 +154,15 @@
     <t>384260009396</t>
   </si>
   <si>
+    <t>384260009397</t>
+  </si>
+  <si>
     <t>030-1094-58</t>
   </si>
   <si>
     <t>066-3084-32</t>
   </si>
   <si>
-    <t>MS21442-121</t>
-  </si>
-  <si>
     <t>324843-W020</t>
   </si>
   <si>
@@ -193,15 +190,15 @@
     <t>S2616-285K4</t>
   </si>
   <si>
+    <t>C611505-0201</t>
+  </si>
+  <si>
     <t>CONNECTOR</t>
   </si>
   <si>
     <t>IND RDR 2000 IN-182A</t>
   </si>
   <si>
-    <t>BEARING,ROLLER,NEEDL</t>
-  </si>
-  <si>
     <t>HEADSET-MICROPHONE</t>
   </si>
   <si>
@@ -229,6 +226,9 @@
     <t>ALTERNAD BELT</t>
   </si>
   <si>
+    <t>ALTERNATOR</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -244,12 +244,12 @@
     <t>Atendido parcialmente</t>
   </si>
   <si>
+    <t>Expedido total</t>
+  </si>
+  <si>
     <t>Aguardando solução</t>
   </si>
   <si>
-    <t>Expedido total</t>
-  </si>
-  <si>
     <t>ANCE</t>
   </si>
   <si>
@@ -271,31 +271,28 @@
     <t>Alterado o tipo da emerg. de IPLR para ANCE. Godoy 22/07/26</t>
   </si>
   <si>
-    <t>AWB 12750991113 volume retirado na loja GOLLOG - BSB por MICHELLIBCRISTINI DE BARROS em 10/08. Godoy 12/08/26.</t>
-  </si>
-  <si>
     <t>Atendido 01 EA através da TSP 18122931. Outros 02 EA serão enviados pela empresa. Ramon 03/08/26. AWB 12750821282 volume retirado na loja GOLLOG - MAO por kleyton EM 06/08. Godoy 12/08/26.</t>
   </si>
   <si>
     <t>item atendido com o estoque local pedido 18171852 em 10/08. Godoy 11/08. Está sendo definido se o PN está correto. Ramon 11/08/26.</t>
   </si>
   <si>
-    <t>Estoque com 12 EA do Pn LM600-9 (Alternado). Godoy 12/08/26.</t>
+    <t>Estoque com 12 EA do Pn LM600-9 (Alternado). Godoy 12/08/26. Atendido com estoque local em 13/08. Ramon 13/08/26</t>
   </si>
   <si>
     <t>AWB 127-5256 7745 com previsão de entrega em 14/08. Ramon 13/08/26</t>
   </si>
   <si>
-    <t>Estoque no alternado 285K4. Caso use do estoque, verificar validade que consta no item. Ramon 12/08/26.</t>
+    <t>Item em pane, anv autorizada a voar por 3 dias pela MMEL a contar de 12/08. Ramon 13/08/26</t>
+  </si>
+  <si>
+    <t>Estoque no alternado 285K4. Caso use do estoque, verificar validade que consta no item. Ramon 12/08/26. Item em pane, anv autorizada a voar por 3 dias pela MMEL a contar de 12/08. Ramon 13/08/26</t>
   </si>
   <si>
     <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Consolidando embarque próximo voo para o GIG</t>
   </si>
   <si>
     <t>Item em bancada porem em pessimo estado, foi solicitado recolhimento de mais unidades para envio a oficina para tentativa de reparo ATZ Marcio 17/7/26. Solicitado abertura de O.S. para 3EA do item no dia 16-07-26 via Email para a Coordenadoria - CLA-21-07-26- SERÁ ENTREGUE PELA WILLIAM DPE DIA 12-08-26 - CLA-11-08</t>
-  </si>
-  <si>
-    <t>Pedido I816822 entregue em Miami 27/07. Previsão de chegada GIG 30/07 (voo 4208). Previsão de canal 31/07 - MATERIAL RECEBIDO NA VEE ONE, EM PROCESSO DE EXPEDIÇÃO 04/08/2026 - ATZ RC - MATERIAL ENVIADO VIA RECIBO 650/FAB/26 - AWB 12750991113 DPE 06/08/2026, ESTÁ DISPONÍVEL PARA RETIRADA DESDE 04/08/2026 - retirado na Gollog dia 10/08/2026</t>
   </si>
   <si>
     <t>Enviado para o Operador(02 EA), atendimento parcial, em 31/07/2026 -AWB 127-5041 6833- REZ - o outro 1 EA será atendido pelo estoque FAB. conforme solicitado por Email- CLA-03-08 - AWB 127-5082 1282 -1 EA ENVIADO ESTOQUE FAB - Material entregue dia 06/08/2026</t>
@@ -809,7 +806,7 @@
         <v>91</v>
       </c>
       <c r="W2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -880,7 +877,7 @@
         <v>92</v>
       </c>
       <c r="W3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -888,7 +885,7 @@
     </row>
     <row r="4" spans="1:27">
       <c r="A4">
-        <v>329</v>
+        <v>313</v>
       </c>
       <c r="B4" t="s">
         <v>28</v>
@@ -903,46 +900,46 @@
         <v>61</v>
       </c>
       <c r="F4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G4">
-        <v>2720</v>
+        <v>2736</v>
       </c>
       <c r="H4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I4" t="s">
         <v>78</v>
       </c>
       <c r="J4" s="1">
-        <v>46220</v>
+        <v>46205</v>
       </c>
       <c r="K4" s="1">
-        <v>46224</v>
+        <v>46234</v>
       </c>
       <c r="L4">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="M4" t="s">
         <v>81</v>
       </c>
       <c r="N4" s="1">
-        <v>46255</v>
+        <v>46265</v>
       </c>
       <c r="O4" s="1">
-        <v>46244</v>
+        <v>46240</v>
       </c>
       <c r="Q4">
-        <v>-8</v>
+        <v>-18</v>
       </c>
       <c r="R4">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="S4" t="s">
         <v>82</v>
       </c>
       <c r="T4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="U4" t="s">
         <v>85</v>
@@ -951,7 +948,7 @@
         <v>93</v>
       </c>
       <c r="W4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -962,25 +959,25 @@
         <v>313</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
         <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F5" t="s">
         <v>73</v>
       </c>
       <c r="G5">
-        <v>2736</v>
+        <v>2737</v>
       </c>
       <c r="H5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I5" t="s">
         <v>78</v>
@@ -1001,7 +998,7 @@
         <v>46265</v>
       </c>
       <c r="O5" s="1">
-        <v>46240</v>
+        <v>46265</v>
       </c>
       <c r="Q5">
         <v>-18</v>
@@ -1015,14 +1012,11 @@
       <c r="T5" t="s">
         <v>83</v>
       </c>
-      <c r="U5" t="s">
-        <v>86</v>
-      </c>
       <c r="V5" t="s">
         <v>94</v>
       </c>
       <c r="W5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1030,7 +1024,7 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6">
-        <v>313</v>
+        <v>396</v>
       </c>
       <c r="B6" t="s">
         <v>29</v>
@@ -1045,40 +1039,40 @@
         <v>62</v>
       </c>
       <c r="F6" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G6">
-        <v>2737</v>
+        <v>2733</v>
       </c>
       <c r="H6" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="I6" t="s">
         <v>78</v>
       </c>
       <c r="J6" s="1">
-        <v>46205</v>
+        <v>46238</v>
       </c>
       <c r="K6" s="1">
-        <v>46234</v>
+        <v>46238</v>
       </c>
       <c r="L6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M6" t="s">
         <v>81</v>
       </c>
       <c r="N6" s="1">
-        <v>46265</v>
+        <v>46269</v>
       </c>
       <c r="O6" s="1">
-        <v>46265</v>
+        <v>46269</v>
       </c>
       <c r="Q6">
-        <v>-18</v>
+        <v>-22</v>
       </c>
       <c r="R6">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="S6" t="s">
         <v>82</v>
@@ -1090,7 +1084,7 @@
         <v>95</v>
       </c>
       <c r="W6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1098,7 +1092,7 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>396</v>
+        <v>329</v>
       </c>
       <c r="B7" t="s">
         <v>30</v>
@@ -1113,52 +1107,46 @@
         <v>63</v>
       </c>
       <c r="F7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G7">
-        <v>2733</v>
+        <v>2721</v>
       </c>
       <c r="H7" t="s">
         <v>74</v>
       </c>
       <c r="I7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J7" s="1">
-        <v>46238</v>
+        <v>46241</v>
       </c>
       <c r="K7" s="1">
-        <v>46238</v>
+        <v>46241</v>
       </c>
       <c r="L7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M7" t="s">
         <v>81</v>
       </c>
       <c r="N7" s="1">
-        <v>46269</v>
-      </c>
-      <c r="O7" s="1">
-        <v>46269</v>
+        <v>46248</v>
       </c>
       <c r="Q7">
-        <v>-22</v>
+        <v>-1</v>
       </c>
       <c r="R7">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="S7" t="s">
         <v>82</v>
       </c>
-      <c r="T7" t="s">
-        <v>83</v>
-      </c>
       <c r="V7" t="s">
         <v>96</v>
       </c>
       <c r="W7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1166,10 +1154,10 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C8" t="s">
         <v>40</v>
@@ -1181,46 +1169,55 @@
         <v>64</v>
       </c>
       <c r="F8" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G8">
-        <v>2721</v>
+        <v>2729</v>
       </c>
       <c r="H8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I8" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J8" s="1">
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="K8" s="1">
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="L8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M8" t="s">
         <v>81</v>
       </c>
       <c r="N8" s="1">
-        <v>46248</v>
+        <v>46255</v>
+      </c>
+      <c r="O8" s="1">
+        <v>46255</v>
       </c>
       <c r="Q8">
-        <v>-1</v>
+        <v>-8</v>
       </c>
       <c r="R8">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="S8" t="s">
-        <v>82</v>
+        <v>83</v>
+      </c>
+      <c r="T8" t="s">
+        <v>83</v>
+      </c>
+      <c r="U8" t="s">
+        <v>86</v>
       </c>
       <c r="V8" t="s">
         <v>97</v>
       </c>
       <c r="W8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1228,10 +1225,10 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9">
-        <v>685</v>
+        <v>386</v>
       </c>
       <c r="B9" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C9" t="s">
         <v>41</v>
@@ -1243,46 +1240,46 @@
         <v>65</v>
       </c>
       <c r="F9" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G9">
-        <v>2729</v>
+        <v>2743</v>
       </c>
       <c r="H9" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="I9" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="J9" s="1">
         <v>46244</v>
       </c>
       <c r="K9" s="1">
-        <v>46244</v>
+        <v>46246</v>
       </c>
       <c r="L9">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="M9" t="s">
         <v>81</v>
       </c>
       <c r="N9" s="1">
-        <v>46255</v>
+        <v>46277</v>
       </c>
       <c r="O9" s="1">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="Q9">
-        <v>-8</v>
+        <v>-30</v>
       </c>
       <c r="R9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S9" t="s">
         <v>83</v>
       </c>
       <c r="T9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="U9" t="s">
         <v>87</v>
@@ -1291,7 +1288,7 @@
         <v>98</v>
       </c>
       <c r="W9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1299,10 +1296,10 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>386</v>
+        <v>685</v>
       </c>
       <c r="B10" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C10" t="s">
         <v>42</v>
@@ -1314,43 +1311,46 @@
         <v>66</v>
       </c>
       <c r="F10" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G10">
-        <v>2743</v>
+        <v>2729</v>
       </c>
       <c r="H10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I10" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="J10" s="1">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="K10" s="1">
         <v>46246</v>
       </c>
       <c r="L10">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M10" t="s">
         <v>81</v>
       </c>
       <c r="N10" s="1">
-        <v>46277</v>
+        <v>46257</v>
+      </c>
+      <c r="O10" s="1">
+        <v>46248</v>
       </c>
       <c r="Q10">
-        <v>-30</v>
+        <v>-10</v>
       </c>
       <c r="R10">
         <v>1</v>
       </c>
       <c r="S10" t="s">
+        <v>82</v>
+      </c>
+      <c r="T10" t="s">
         <v>83</v>
-      </c>
-      <c r="T10" t="s">
-        <v>82</v>
       </c>
       <c r="U10" t="s">
         <v>88</v>
@@ -1359,7 +1359,7 @@
         <v>99</v>
       </c>
       <c r="W10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1367,10 +1367,10 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>685</v>
+        <v>690</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C11" t="s">
         <v>43</v>
@@ -1385,10 +1385,10 @@
         <v>72</v>
       </c>
       <c r="G11">
-        <v>2729</v>
+        <v>2727</v>
       </c>
       <c r="H11" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I11" t="s">
         <v>80</v>
@@ -1408,6 +1408,9 @@
       <c r="N11" s="1">
         <v>46257</v>
       </c>
+      <c r="O11" s="1">
+        <v>46257</v>
+      </c>
       <c r="Q11">
         <v>-10</v>
       </c>
@@ -1418,16 +1421,13 @@
         <v>82</v>
       </c>
       <c r="T11" t="s">
-        <v>83</v>
-      </c>
-      <c r="U11" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="V11" t="s">
         <v>100</v>
       </c>
       <c r="W11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1435,10 +1435,10 @@
     </row>
     <row r="12" spans="1:27">
       <c r="A12">
-        <v>690</v>
+        <v>384</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C12" t="s">
         <v>44</v>
@@ -1450,16 +1450,16 @@
         <v>68</v>
       </c>
       <c r="F12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G12">
-        <v>2727</v>
+        <v>2742</v>
       </c>
       <c r="H12" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="I12" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="J12" s="1">
         <v>46245</v>
@@ -1474,10 +1474,13 @@
         <v>81</v>
       </c>
       <c r="N12" s="1">
-        <v>46257</v>
+        <v>46277</v>
+      </c>
+      <c r="O12" s="1">
+        <v>46254</v>
       </c>
       <c r="Q12">
-        <v>-10</v>
+        <v>-30</v>
       </c>
       <c r="R12">
         <v>1</v>
@@ -1488,11 +1491,14 @@
       <c r="T12" t="s">
         <v>82</v>
       </c>
+      <c r="U12" t="s">
+        <v>89</v>
+      </c>
       <c r="V12" t="s">
         <v>101</v>
       </c>
       <c r="W12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1515,13 +1521,13 @@
         <v>69</v>
       </c>
       <c r="F13" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G13">
         <v>2742</v>
       </c>
       <c r="H13" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="I13" t="s">
         <v>78</v>
@@ -1541,6 +1547,9 @@
       <c r="N13" s="1">
         <v>46277</v>
       </c>
+      <c r="O13" s="1">
+        <v>46254</v>
+      </c>
       <c r="Q13">
         <v>-30</v>
       </c>
@@ -1548,16 +1557,19 @@
         <v>1</v>
       </c>
       <c r="S13" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="T13" t="s">
         <v>82</v>
       </c>
+      <c r="U13" t="s">
+        <v>90</v>
+      </c>
       <c r="V13" t="s">
+        <v>98</v>
+      </c>
+      <c r="W13" t="s">
         <v>102</v>
-      </c>
-      <c r="W13" t="s">
-        <v>103</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1580,22 +1592,22 @@
         <v>70</v>
       </c>
       <c r="F14" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G14">
         <v>2742</v>
       </c>
       <c r="H14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I14" t="s">
         <v>78</v>
       </c>
       <c r="J14" s="1">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="K14" s="1">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="L14">
         <v>1</v>
@@ -1604,28 +1616,25 @@
         <v>81</v>
       </c>
       <c r="N14" s="1">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="Q14">
-        <v>-30</v>
+        <v>-31</v>
       </c>
       <c r="R14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="T14" t="s">
         <v>82</v>
       </c>
       <c r="U14" t="s">
-        <v>90</v>
-      </c>
-      <c r="V14" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="W14" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (13/08/2026 16:58)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="104">
   <si>
     <t>om_emg</t>
   </si>
@@ -292,34 +292,37 @@
     <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Consolidando embarque próximo voo para o GIG</t>
   </si>
   <si>
-    <t>Item em bancada porem em pessimo estado, foi solicitado recolhimento de mais unidades para envio a oficina para tentativa de reparo ATZ Marcio 17/7/26. Solicitado abertura de O.S. para 3EA do item no dia 16-07-26 via Email para a Coordenadoria - CLA-21-07-26- SERÁ ENTREGUE PELA WILLIAM DPE DIA 12-08-26 - CLA-11-08</t>
+    <t>Item em bancada porem em pessimo estado, foi solicitado recolhimento de mais unidades para envio a oficina para tentativa de reparo ATZ Marcio 17/7/26. Solicitado abertura de O.S. para 3EA do item no dia 16-07-26 via Email para a Coordenadoria - CLA-21-07-26- SERÁ ENTREGUE PELA WILLIAM DPE DIA 14-08-26 - CLA-13-08</t>
   </si>
   <si>
     <t>Enviado para o Operador(02 EA), atendimento parcial, em 31/07/2026 -AWB 127-5041 6833- REZ - o outro 1 EA será atendido pelo estoque FAB. conforme solicitado por Email- CLA-03-08 - AWB 127-5082 1282 -1 EA ENVIADO ESTOQUE FAB - Material entregue dia 06/08/2026</t>
   </si>
   <si>
-    <t>Temos 4 EA em manutenção na William, será pedido prioridade. CLA-03-08</t>
+    <t>Temos 4 EA em manutenção na William, será pedido prioridade. CLA-03-08 - DPE DIA 14-08 - CLA 13-08</t>
   </si>
   <si>
     <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
   </si>
   <si>
-    <t>Foi solicitado abertura de O.S. no dia 7 -08-26 de 6 EA. As OSs foram abertas e aguardando recolhimento para reparo. CLA-10-08 - ITEM FOI RECOLHIDO PELA WILLIAM- CLA-11-08</t>
-  </si>
-  <si>
-    <t>Foi solicitado atendimento com estoque FAB - CLA- 10-08, ITEM PRONTO PARA EMBARQUE, AGUARDANDO NOTA FISCAL - CLA-11-08</t>
-  </si>
-  <si>
-    <t>TEM ESTOQUE NA VEEONE</t>
-  </si>
-  <si>
-    <t>Em estoque na V1 JPA 12/8/26 Marcio 13:23</t>
+    <t>Foi solicitado abertura de O.S. no dia 7 -08-26 de 6 EA. As OSs foram abertas e aguardando recolhimento para reparo. CLA-10-08 - ITEM FOI RECOLHIDO PELA WILLIAM- CLA-11-08 - DPE 14-08</t>
+  </si>
+  <si>
+    <t>Foi solicitado atendimento com estoque FAB - CLA- 10-08, ITEM PRONTO PARA EMBARQUE, AGUARDANDO NOTA FISCAL - CLA-11-08- ITEM AGUARDANDO DEFINIÇÃO DA COORDENADORIA QUANTO A EFETIVIDADE PARA APLICAÇÃO NA REFERIDA ANV.- CLA-13-08</t>
+  </si>
+  <si>
+    <t>Temos somente 03 ea em STK, favor utilizar o estoque FAB para posterior devolução. ATZ RC 13/08 - FOI SOLICITADO O ATENDIMENTO COM ESTOQUE FAB -CLA-13-08</t>
+  </si>
+  <si>
+    <t>Estoque veeone da base pamals- AWB 12752567745 - DPE 14/08/2026 - recibo 680/FAB/26</t>
   </si>
   <si>
     <t>Previsao de entrega da oficina do RJ na V1 JPA 13/8/2026 durante o dia, horario comercial, ATZ Marcio 12/8 13:22hs</t>
   </si>
   <si>
-    <t>1 Unidade na oficina em BH William, solicitado prioridade na entrega DPE 14/8, aguardando orçamento final ATZ Marcio 12/8 13:24hs</t>
+    <t>1 Unidade na oficina em BH William, solicitado prioridade na entrega DPE 14/8, aguardando orçamento final ATZ Marcio 12/8 13:24hs- DPE 14-08</t>
+  </si>
+  <si>
+    <t>Temos no STK V1, material em separação, recibo 682/FAB/26 - atz rc 13/08</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -806,7 +809,7 @@
         <v>91</v>
       </c>
       <c r="W2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -877,7 +880,7 @@
         <v>92</v>
       </c>
       <c r="W3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -948,7 +951,7 @@
         <v>93</v>
       </c>
       <c r="W4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -1016,7 +1019,7 @@
         <v>94</v>
       </c>
       <c r="W5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1084,7 +1087,7 @@
         <v>95</v>
       </c>
       <c r="W6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1146,7 +1149,7 @@
         <v>96</v>
       </c>
       <c r="W7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1217,7 +1220,7 @@
         <v>97</v>
       </c>
       <c r="W8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1288,7 +1291,7 @@
         <v>98</v>
       </c>
       <c r="W9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1359,7 +1362,7 @@
         <v>99</v>
       </c>
       <c r="W10" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1427,7 +1430,7 @@
         <v>100</v>
       </c>
       <c r="W11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1498,7 +1501,7 @@
         <v>101</v>
       </c>
       <c r="W12" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1566,10 +1569,10 @@
         <v>90</v>
       </c>
       <c r="V13" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="W13" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1634,7 +1637,7 @@
         <v>89</v>
       </c>
       <c r="W14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (14/08/2026 08:52)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -794,10 +794,10 @@
         <v>46251</v>
       </c>
       <c r="Q2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R2">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="S2" t="s">
         <v>82</v>
@@ -862,10 +862,10 @@
         <v>46249</v>
       </c>
       <c r="Q3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R3">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="S3" t="s">
         <v>82</v>
@@ -933,10 +933,10 @@
         <v>46240</v>
       </c>
       <c r="Q4">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="R4">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S4" t="s">
         <v>82</v>
@@ -1004,10 +1004,10 @@
         <v>46265</v>
       </c>
       <c r="Q5">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="R5">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S5" t="s">
         <v>82</v>
@@ -1072,10 +1072,10 @@
         <v>46269</v>
       </c>
       <c r="Q6">
-        <v>-22</v>
+        <v>-21</v>
       </c>
       <c r="R6">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="S6" t="s">
         <v>82</v>
@@ -1137,10 +1137,10 @@
         <v>46248</v>
       </c>
       <c r="Q7">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S7" t="s">
         <v>82</v>
@@ -1202,10 +1202,10 @@
         <v>46255</v>
       </c>
       <c r="Q8">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="R8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S8" t="s">
         <v>83</v>
@@ -1273,10 +1273,10 @@
         <v>46254</v>
       </c>
       <c r="Q9">
-        <v>-30</v>
+        <v>-29</v>
       </c>
       <c r="R9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S9" t="s">
         <v>83</v>
@@ -1344,10 +1344,10 @@
         <v>46248</v>
       </c>
       <c r="Q10">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="R10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S10" t="s">
         <v>82</v>
@@ -1415,10 +1415,10 @@
         <v>46257</v>
       </c>
       <c r="Q11">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="R11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S11" t="s">
         <v>82</v>
@@ -1483,10 +1483,10 @@
         <v>46254</v>
       </c>
       <c r="Q12">
-        <v>-30</v>
+        <v>-29</v>
       </c>
       <c r="R12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S12" t="s">
         <v>82</v>
@@ -1554,10 +1554,10 @@
         <v>46254</v>
       </c>
       <c r="Q13">
-        <v>-30</v>
+        <v>-29</v>
       </c>
       <c r="R13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S13" t="s">
         <v>83</v>
@@ -1622,10 +1622,10 @@
         <v>46278</v>
       </c>
       <c r="Q14">
-        <v>-31</v>
+        <v>-30</v>
       </c>
       <c r="R14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S14" t="s">
         <v>82</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (14/08/2026 12:59)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="111">
   <si>
     <t>om_emg</t>
   </si>
@@ -142,9 +142,6 @@
     <t>386260013489</t>
   </si>
   <si>
-    <t>685260012588</t>
-  </si>
-  <si>
     <t>690260002522</t>
   </si>
   <si>
@@ -157,6 +154,18 @@
     <t>384260009397</t>
   </si>
   <si>
+    <t>329260019269</t>
+  </si>
+  <si>
+    <t>329260019270</t>
+  </si>
+  <si>
+    <t>685260012609</t>
+  </si>
+  <si>
+    <t>685260012610</t>
+  </si>
+  <si>
     <t>030-1094-58</t>
   </si>
   <si>
@@ -178,9 +187,6 @@
     <t>9910333-1</t>
   </si>
   <si>
-    <t>51539-012N</t>
-  </si>
-  <si>
     <t>3244897-4</t>
   </si>
   <si>
@@ -193,6 +199,18 @@
     <t>C611505-0201</t>
   </si>
   <si>
+    <t>069-01033-0101</t>
+  </si>
+  <si>
+    <t>C662504-0101</t>
+  </si>
+  <si>
+    <t>162-10700</t>
+  </si>
+  <si>
+    <t>2650113-5</t>
+  </si>
+  <si>
     <t>CONNECTOR</t>
   </si>
   <si>
@@ -214,9 +232,6 @@
     <t>ENGINE MOUNT</t>
   </si>
   <si>
-    <t>CONTROL UNIT ASSY-GE</t>
-  </si>
-  <si>
     <t>FUEL CONTROL UNIT</t>
   </si>
   <si>
@@ -229,6 +244,18 @@
     <t>ALTERNATOR</t>
   </si>
   <si>
+    <t>RECEIVER-TRANSMITTER</t>
+  </si>
+  <si>
+    <t>GAGE VOLT AMME</t>
+  </si>
+  <si>
+    <t>OUTER WHEEL HALF ASS</t>
+  </si>
+  <si>
+    <t>BRACKET</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -280,9 +307,6 @@
     <t>Estoque com 12 EA do Pn LM600-9 (Alternado). Godoy 12/08/26. Atendido com estoque local em 13/08. Ramon 13/08/26</t>
   </si>
   <si>
-    <t>AWB 127-5256 7745 com previsão de entrega em 14/08. Ramon 13/08/26. Recibo 680/FAB/26 (NF 2082) assinados em 13/08. Ramon 14/08/26</t>
-  </si>
-  <si>
     <t>Item em pane, anv autorizada a voar por 3 dias pela MMEL a contar de 12/08. Ramon 13/08/26</t>
   </si>
   <si>
@@ -311,9 +335,6 @@
   </si>
   <si>
     <t>Temos somente 03 ea em STK, favor utilizar o estoque FAB para posterior devolução. ATZ RC 13/08 - FOI SOLICITADO O ATENDIMENTO COM ESTOQUE FAB -CLA-13-08</t>
-  </si>
-  <si>
-    <t>Estoque veeone da base pamals- AWB 12752567745 - DPE 14/08/2026 - recibo 680/FAB/26</t>
   </si>
   <si>
     <t>Previsao de entrega da oficina do RJ na V1 JPA 13/8/2026 durante o dia, horario comercial, ATZ Marcio 12/8 13:22hs</t>
@@ -661,7 +682,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA14"/>
+  <dimension ref="A1:AA17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -758,22 +779,22 @@
         <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="E2" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="F2" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="G2">
         <v>2702</v>
       </c>
       <c r="H2" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="I2" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="J2" s="1">
         <v>46212</v>
@@ -785,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="N2" s="1">
         <v>46243</v>
@@ -800,16 +821,16 @@
         <v>36</v>
       </c>
       <c r="S2" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="T2" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="V2" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="W2" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -826,22 +847,22 @@
         <v>35</v>
       </c>
       <c r="D3" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="E3" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="F3" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="G3">
         <v>2722</v>
       </c>
       <c r="H3" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="I3" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="J3" s="1">
         <v>46219</v>
@@ -853,7 +874,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="N3" s="1">
         <v>46249</v>
@@ -868,19 +889,19 @@
         <v>30</v>
       </c>
       <c r="S3" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="T3" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="U3" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="V3" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="W3" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -897,22 +918,22 @@
         <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E4" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="F4" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="G4">
         <v>2736</v>
       </c>
       <c r="H4" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="I4" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="J4" s="1">
         <v>46205</v>
@@ -924,7 +945,7 @@
         <v>3</v>
       </c>
       <c r="M4" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="N4" s="1">
         <v>46265</v>
@@ -939,19 +960,19 @@
         <v>14</v>
       </c>
       <c r="S4" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="T4" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="U4" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="V4" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="W4" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -968,22 +989,22 @@
         <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E5" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="F5" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="G5">
         <v>2737</v>
       </c>
       <c r="H5" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="I5" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="J5" s="1">
         <v>46205</v>
@@ -995,7 +1016,7 @@
         <v>3</v>
       </c>
       <c r="M5" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="N5" s="1">
         <v>46265</v>
@@ -1010,16 +1031,16 @@
         <v>14</v>
       </c>
       <c r="S5" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="T5" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="V5" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="W5" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1036,22 +1057,22 @@
         <v>38</v>
       </c>
       <c r="D6" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="E6" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="F6" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="G6">
         <v>2733</v>
       </c>
       <c r="H6" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="I6" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="J6" s="1">
         <v>46238</v>
@@ -1063,7 +1084,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="N6" s="1">
         <v>46269</v>
@@ -1078,16 +1099,16 @@
         <v>10</v>
       </c>
       <c r="S6" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="T6" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="V6" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="W6" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1104,22 +1125,22 @@
         <v>39</v>
       </c>
       <c r="D7" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="E7" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="F7" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="G7">
         <v>2721</v>
       </c>
       <c r="H7" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="I7" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="J7" s="1">
         <v>46241</v>
@@ -1131,7 +1152,7 @@
         <v>2</v>
       </c>
       <c r="M7" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="N7" s="1">
         <v>46248</v>
@@ -1143,13 +1164,13 @@
         <v>7</v>
       </c>
       <c r="S7" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="V7" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="W7" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1166,22 +1187,22 @@
         <v>40</v>
       </c>
       <c r="D8" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E8" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="F8" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="G8">
         <v>2729</v>
       </c>
       <c r="H8" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="I8" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="J8" s="1">
         <v>46244</v>
@@ -1193,7 +1214,7 @@
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="N8" s="1">
         <v>46255</v>
@@ -1208,19 +1229,19 @@
         <v>4</v>
       </c>
       <c r="S8" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="T8" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="U8" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="V8" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="W8" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1237,22 +1258,22 @@
         <v>41</v>
       </c>
       <c r="D9" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="E9" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="F9" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="G9">
         <v>2743</v>
       </c>
       <c r="H9" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="I9" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="J9" s="1">
         <v>46244</v>
@@ -1264,7 +1285,7 @@
         <v>6</v>
       </c>
       <c r="M9" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="N9" s="1">
         <v>46277</v>
@@ -1279,19 +1300,19 @@
         <v>2</v>
       </c>
       <c r="S9" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="T9" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="U9" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="V9" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="W9" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1299,31 +1320,31 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>685</v>
+        <v>690</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C10" t="s">
         <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="E10" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F10" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="G10">
-        <v>2729</v>
+        <v>2727</v>
       </c>
       <c r="H10" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="I10" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="J10" s="1">
         <v>46245</v>
@@ -1335,13 +1356,13 @@
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="N10" s="1">
         <v>46257</v>
       </c>
       <c r="O10" s="1">
-        <v>46248</v>
+        <v>46257</v>
       </c>
       <c r="Q10">
         <v>-9</v>
@@ -1350,19 +1371,16 @@
         <v>2</v>
       </c>
       <c r="S10" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="T10" t="s">
-        <v>83</v>
-      </c>
-      <c r="U10" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="V10" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="W10" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1370,31 +1388,31 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>690</v>
+        <v>384</v>
       </c>
       <c r="B11" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C11" t="s">
         <v>43</v>
       </c>
       <c r="D11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="E11" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="F11" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="G11">
-        <v>2727</v>
+        <v>2742</v>
       </c>
       <c r="H11" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="I11" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="J11" s="1">
         <v>46245</v>
@@ -1406,31 +1424,34 @@
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="N11" s="1">
-        <v>46257</v>
+        <v>46277</v>
       </c>
       <c r="O11" s="1">
-        <v>46257</v>
+        <v>46254</v>
       </c>
       <c r="Q11">
-        <v>-9</v>
+        <v>-29</v>
       </c>
       <c r="R11">
         <v>2</v>
       </c>
       <c r="S11" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="T11" t="s">
-        <v>82</v>
+        <v>91</v>
+      </c>
+      <c r="U11" t="s">
+        <v>97</v>
       </c>
       <c r="V11" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="W11" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1447,22 +1468,22 @@
         <v>44</v>
       </c>
       <c r="D12" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="E12" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="F12" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="G12">
         <v>2742</v>
       </c>
       <c r="H12" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="I12" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="J12" s="1">
         <v>46245</v>
@@ -1474,7 +1495,7 @@
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="N12" s="1">
         <v>46277</v>
@@ -1489,19 +1510,19 @@
         <v>2</v>
       </c>
       <c r="S12" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="T12" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="U12" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="V12" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="W12" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1518,61 +1539,55 @@
         <v>45</v>
       </c>
       <c r="D13" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E13" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="F13" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="G13">
         <v>2742</v>
       </c>
       <c r="H13" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="I13" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="J13" s="1">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="K13" s="1">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="L13">
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="N13" s="1">
-        <v>46277</v>
-      </c>
-      <c r="O13" s="1">
-        <v>46254</v>
+        <v>46278</v>
       </c>
       <c r="Q13">
-        <v>-29</v>
+        <v>-30</v>
       </c>
       <c r="R13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S13" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="T13" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="U13" t="s">
-        <v>90</v>
-      </c>
-      <c r="V13" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="W13" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1580,66 +1595,249 @@
     </row>
     <row r="14" spans="1:27">
       <c r="A14">
-        <v>384</v>
+        <v>329</v>
       </c>
       <c r="B14" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C14" t="s">
         <v>46</v>
       </c>
       <c r="D14" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="E14" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="F14" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="G14">
-        <v>2742</v>
+        <v>2721</v>
       </c>
       <c r="H14" t="s">
+        <v>86</v>
+      </c>
+      <c r="I14" t="s">
+        <v>87</v>
+      </c>
+      <c r="J14" s="1">
+        <v>46248</v>
+      </c>
+      <c r="K14" s="1">
+        <v>46248</v>
+      </c>
+      <c r="L14">
+        <v>1</v>
+      </c>
+      <c r="M14" t="s">
+        <v>90</v>
+      </c>
+      <c r="N14" s="1">
+        <v>46279</v>
+      </c>
+      <c r="Q14">
+        <v>-31</v>
+      </c>
+      <c r="R14">
+        <v>0</v>
+      </c>
+      <c r="S14" t="s">
+        <v>92</v>
+      </c>
+      <c r="T14" t="s">
+        <v>91</v>
+      </c>
+      <c r="W14" t="s">
+        <v>110</v>
+      </c>
+      <c r="AA14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27">
+      <c r="A15">
+        <v>329</v>
+      </c>
+      <c r="B15" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" t="s">
+        <v>47</v>
+      </c>
+      <c r="D15" t="s">
+        <v>62</v>
+      </c>
+      <c r="E15" t="s">
         <v>77</v>
       </c>
-      <c r="I14" t="s">
+      <c r="F15" t="s">
+        <v>82</v>
+      </c>
+      <c r="G15">
+        <v>2720</v>
+      </c>
+      <c r="H15" t="s">
+        <v>86</v>
+      </c>
+      <c r="I15" t="s">
+        <v>89</v>
+      </c>
+      <c r="J15" s="1">
+        <v>46248</v>
+      </c>
+      <c r="K15" s="1">
+        <v>46248</v>
+      </c>
+      <c r="L15">
+        <v>1</v>
+      </c>
+      <c r="M15" t="s">
+        <v>90</v>
+      </c>
+      <c r="N15" s="1">
+        <v>46259</v>
+      </c>
+      <c r="Q15">
+        <v>-11</v>
+      </c>
+      <c r="R15">
+        <v>0</v>
+      </c>
+      <c r="S15" t="s">
+        <v>92</v>
+      </c>
+      <c r="T15" t="s">
+        <v>91</v>
+      </c>
+      <c r="W15" t="s">
+        <v>110</v>
+      </c>
+      <c r="AA15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27">
+      <c r="A16">
+        <v>685</v>
+      </c>
+      <c r="B16" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" t="s">
+        <v>48</v>
+      </c>
+      <c r="D16" t="s">
+        <v>63</v>
+      </c>
+      <c r="E16" t="s">
         <v>78</v>
       </c>
-      <c r="J14" s="1">
-        <v>46246</v>
-      </c>
-      <c r="K14" s="1">
-        <v>46247</v>
-      </c>
-      <c r="L14">
-        <v>1</v>
-      </c>
-      <c r="M14" t="s">
-        <v>81</v>
-      </c>
-      <c r="N14" s="1">
-        <v>46278</v>
-      </c>
-      <c r="Q14">
-        <v>-30</v>
-      </c>
-      <c r="R14">
-        <v>1</v>
-      </c>
-      <c r="S14" t="s">
+      <c r="F16" t="s">
         <v>82</v>
       </c>
-      <c r="T14" t="s">
-        <v>82</v>
-      </c>
-      <c r="U14" t="s">
+      <c r="G16">
+        <v>2729</v>
+      </c>
+      <c r="H16" t="s">
+        <v>86</v>
+      </c>
+      <c r="I16" t="s">
         <v>89</v>
       </c>
-      <c r="W14" t="s">
-        <v>103</v>
-      </c>
-      <c r="AA14" t="b">
+      <c r="J16" s="1">
+        <v>46248</v>
+      </c>
+      <c r="K16" s="1">
+        <v>46248</v>
+      </c>
+      <c r="L16">
+        <v>1</v>
+      </c>
+      <c r="M16" t="s">
+        <v>90</v>
+      </c>
+      <c r="N16" s="1">
+        <v>46259</v>
+      </c>
+      <c r="Q16">
+        <v>-11</v>
+      </c>
+      <c r="R16">
+        <v>0</v>
+      </c>
+      <c r="S16" t="s">
+        <v>91</v>
+      </c>
+      <c r="T16" t="s">
+        <v>92</v>
+      </c>
+      <c r="W16" t="s">
+        <v>110</v>
+      </c>
+      <c r="AA16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:27">
+      <c r="A17">
+        <v>685</v>
+      </c>
+      <c r="B17" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" t="s">
+        <v>49</v>
+      </c>
+      <c r="D17" t="s">
+        <v>64</v>
+      </c>
+      <c r="E17" t="s">
+        <v>79</v>
+      </c>
+      <c r="F17" t="s">
+        <v>80</v>
+      </c>
+      <c r="G17">
+        <v>2729</v>
+      </c>
+      <c r="H17" t="s">
+        <v>86</v>
+      </c>
+      <c r="I17" t="s">
+        <v>89</v>
+      </c>
+      <c r="J17" s="1">
+        <v>46248</v>
+      </c>
+      <c r="K17" s="1">
+        <v>46248</v>
+      </c>
+      <c r="L17">
+        <v>2</v>
+      </c>
+      <c r="M17" t="s">
+        <v>90</v>
+      </c>
+      <c r="N17" s="1">
+        <v>46259</v>
+      </c>
+      <c r="Q17">
+        <v>-11</v>
+      </c>
+      <c r="R17">
+        <v>0</v>
+      </c>
+      <c r="S17" t="s">
+        <v>91</v>
+      </c>
+      <c r="T17" t="s">
+        <v>92</v>
+      </c>
+      <c r="W17" t="s">
+        <v>110</v>
+      </c>
+      <c r="AA17" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (17/08/2026 08:34)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -815,10 +815,10 @@
         <v>46251</v>
       </c>
       <c r="Q2">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="R2">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="S2" t="s">
         <v>91</v>
@@ -883,10 +883,10 @@
         <v>46249</v>
       </c>
       <c r="Q3">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="R3">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="S3" t="s">
         <v>91</v>
@@ -954,10 +954,10 @@
         <v>46240</v>
       </c>
       <c r="Q4">
-        <v>-17</v>
+        <v>-14</v>
       </c>
       <c r="R4">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="S4" t="s">
         <v>91</v>
@@ -1025,10 +1025,10 @@
         <v>46265</v>
       </c>
       <c r="Q5">
-        <v>-17</v>
+        <v>-14</v>
       </c>
       <c r="R5">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="S5" t="s">
         <v>91</v>
@@ -1093,10 +1093,10 @@
         <v>46269</v>
       </c>
       <c r="Q6">
-        <v>-21</v>
+        <v>-18</v>
       </c>
       <c r="R6">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="S6" t="s">
         <v>91</v>
@@ -1158,10 +1158,10 @@
         <v>46248</v>
       </c>
       <c r="Q7">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R7">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S7" t="s">
         <v>91</v>
@@ -1223,10 +1223,10 @@
         <v>46255</v>
       </c>
       <c r="Q8">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="R8">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="S8" t="s">
         <v>92</v>
@@ -1294,10 +1294,10 @@
         <v>46254</v>
       </c>
       <c r="Q9">
-        <v>-29</v>
+        <v>-26</v>
       </c>
       <c r="R9">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S9" t="s">
         <v>92</v>
@@ -1365,10 +1365,10 @@
         <v>46257</v>
       </c>
       <c r="Q10">
-        <v>-9</v>
+        <v>-6</v>
       </c>
       <c r="R10">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S10" t="s">
         <v>91</v>
@@ -1433,10 +1433,10 @@
         <v>46254</v>
       </c>
       <c r="Q11">
-        <v>-29</v>
+        <v>-26</v>
       </c>
       <c r="R11">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S11" t="s">
         <v>91</v>
@@ -1504,10 +1504,10 @@
         <v>46254</v>
       </c>
       <c r="Q12">
-        <v>-29</v>
+        <v>-26</v>
       </c>
       <c r="R12">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S12" t="s">
         <v>92</v>
@@ -1572,10 +1572,10 @@
         <v>46278</v>
       </c>
       <c r="Q13">
-        <v>-30</v>
+        <v>-27</v>
       </c>
       <c r="R13">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S13" t="s">
         <v>91</v>
@@ -1637,10 +1637,10 @@
         <v>46279</v>
       </c>
       <c r="Q14">
-        <v>-31</v>
+        <v>-28</v>
       </c>
       <c r="R14">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S14" t="s">
         <v>92</v>
@@ -1699,10 +1699,10 @@
         <v>46259</v>
       </c>
       <c r="Q15">
-        <v>-11</v>
+        <v>-8</v>
       </c>
       <c r="R15">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S15" t="s">
         <v>92</v>
@@ -1761,10 +1761,10 @@
         <v>46259</v>
       </c>
       <c r="Q16">
-        <v>-11</v>
+        <v>-8</v>
       </c>
       <c r="R16">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S16" t="s">
         <v>91</v>
@@ -1823,10 +1823,10 @@
         <v>46259</v>
       </c>
       <c r="Q17">
-        <v>-11</v>
+        <v>-8</v>
       </c>
       <c r="R17">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S17" t="s">
         <v>91</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (17/08/2026 10:45)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="112">
   <si>
     <t>om_emg</t>
   </si>
@@ -344,6 +344,9 @@
   </si>
   <si>
     <t>Temos no STK V1, material em separação, recibo 682/FAB/26 - atz rc 13/08</t>
+  </si>
+  <si>
+    <t>será enviado o pn 9910592-2 do estoque da VeeOne base PAMALS. -CLA -14-08</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -830,7 +833,7 @@
         <v>99</v>
       </c>
       <c r="W2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -901,7 +904,7 @@
         <v>100</v>
       </c>
       <c r="W3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -972,7 +975,7 @@
         <v>101</v>
       </c>
       <c r="W4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -1040,7 +1043,7 @@
         <v>102</v>
       </c>
       <c r="W5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1108,7 +1111,7 @@
         <v>103</v>
       </c>
       <c r="W6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1170,7 +1173,7 @@
         <v>104</v>
       </c>
       <c r="W7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1241,7 +1244,7 @@
         <v>105</v>
       </c>
       <c r="W8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1312,7 +1315,7 @@
         <v>106</v>
       </c>
       <c r="W9" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1380,7 +1383,7 @@
         <v>107</v>
       </c>
       <c r="W10" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1451,7 +1454,7 @@
         <v>108</v>
       </c>
       <c r="W11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1522,7 +1525,7 @@
         <v>109</v>
       </c>
       <c r="W12" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1586,8 +1589,11 @@
       <c r="U13" t="s">
         <v>97</v>
       </c>
+      <c r="V13" t="s">
+        <v>110</v>
+      </c>
       <c r="W13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1649,7 +1655,7 @@
         <v>91</v>
       </c>
       <c r="W14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
@@ -1711,7 +1717,7 @@
         <v>91</v>
       </c>
       <c r="W15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
@@ -1773,7 +1779,7 @@
         <v>92</v>
       </c>
       <c r="W16" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AA16" t="b">
         <v>1</v>
@@ -1835,7 +1841,7 @@
         <v>92</v>
       </c>
       <c r="W17" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AA17" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (17/08/2026 12:33)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="110">
   <si>
     <t>om_emg</t>
   </si>
@@ -163,9 +163,6 @@
     <t>685260012609</t>
   </si>
   <si>
-    <t>685260012610</t>
-  </si>
-  <si>
     <t>030-1094-58</t>
   </si>
   <si>
@@ -208,9 +205,6 @@
     <t>162-10700</t>
   </si>
   <si>
-    <t>2650113-5</t>
-  </si>
-  <si>
     <t>CONNECTOR</t>
   </si>
   <si>
@@ -253,9 +247,6 @@
     <t>OUTER WHEEL HALF ASS</t>
   </si>
   <si>
-    <t>BRACKET</t>
-  </si>
-  <si>
     <t>C</t>
   </si>
   <si>
@@ -311,6 +302,9 @@
   </si>
   <si>
     <t>Estoque no alternado 285K4. Caso use do estoque, verificar validade que consta no item. Ramon 12/08/26. Item em pane, anv autorizada a voar por 3 dias pela MMEL a contar de 12/08. Ramon 13/08/26</t>
+  </si>
+  <si>
+    <t>item será atendido com o estoque local pedido 18216324. Godoy 17/08.</t>
   </si>
   <si>
     <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Consolidando embarque próximo voo para o GIG</t>
@@ -685,7 +679,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA17"/>
+  <dimension ref="A1:AA16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -782,22 +776,22 @@
         <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="G2">
         <v>2702</v>
       </c>
       <c r="H2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="I2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="J2" s="1">
         <v>46212</v>
@@ -809,7 +803,7 @@
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="N2" s="1">
         <v>46243</v>
@@ -824,16 +818,16 @@
         <v>39</v>
       </c>
       <c r="S2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="T2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="V2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="W2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -850,22 +844,22 @@
         <v>35</v>
       </c>
       <c r="D3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F3" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="G3">
         <v>2722</v>
       </c>
       <c r="H3" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="I3" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="J3" s="1">
         <v>46219</v>
@@ -877,7 +871,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="N3" s="1">
         <v>46249</v>
@@ -892,19 +886,19 @@
         <v>33</v>
       </c>
       <c r="S3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="T3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="U3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="V3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="W3" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -921,22 +915,22 @@
         <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F4" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="G4">
         <v>2736</v>
       </c>
       <c r="H4" t="s">
+        <v>81</v>
+      </c>
+      <c r="I4" t="s">
         <v>84</v>
-      </c>
-      <c r="I4" t="s">
-        <v>87</v>
       </c>
       <c r="J4" s="1">
         <v>46205</v>
@@ -948,7 +942,7 @@
         <v>3</v>
       </c>
       <c r="M4" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="N4" s="1">
         <v>46265</v>
@@ -963,19 +957,19 @@
         <v>17</v>
       </c>
       <c r="S4" t="s">
+        <v>88</v>
+      </c>
+      <c r="T4" t="s">
+        <v>89</v>
+      </c>
+      <c r="U4" t="s">
         <v>91</v>
       </c>
-      <c r="T4" t="s">
-        <v>92</v>
-      </c>
-      <c r="U4" t="s">
-        <v>94</v>
-      </c>
       <c r="V4" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="W4" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -992,22 +986,22 @@
         <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F5" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="G5">
         <v>2737</v>
       </c>
       <c r="H5" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="I5" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="J5" s="1">
         <v>46205</v>
@@ -1019,7 +1013,7 @@
         <v>3</v>
       </c>
       <c r="M5" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="N5" s="1">
         <v>46265</v>
@@ -1034,16 +1028,16 @@
         <v>17</v>
       </c>
       <c r="S5" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="T5" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="V5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="W5" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1060,22 +1054,22 @@
         <v>38</v>
       </c>
       <c r="D6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F6" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="G6">
         <v>2733</v>
       </c>
       <c r="H6" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="I6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="J6" s="1">
         <v>46238</v>
@@ -1087,7 +1081,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="N6" s="1">
         <v>46269</v>
@@ -1102,16 +1096,16 @@
         <v>13</v>
       </c>
       <c r="S6" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="T6" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="V6" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="W6" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1128,22 +1122,22 @@
         <v>39</v>
       </c>
       <c r="D7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F7" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="G7">
         <v>2721</v>
       </c>
       <c r="H7" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="I7" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="J7" s="1">
         <v>46241</v>
@@ -1155,7 +1149,7 @@
         <v>2</v>
       </c>
       <c r="M7" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="N7" s="1">
         <v>46248</v>
@@ -1167,13 +1161,13 @@
         <v>10</v>
       </c>
       <c r="S7" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="V7" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="W7" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1190,22 +1184,22 @@
         <v>40</v>
       </c>
       <c r="D8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E8" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F8" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="G8">
         <v>2729</v>
       </c>
       <c r="H8" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="I8" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="J8" s="1">
         <v>46244</v>
@@ -1217,7 +1211,7 @@
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="N8" s="1">
         <v>46255</v>
@@ -1232,19 +1226,19 @@
         <v>7</v>
       </c>
       <c r="S8" t="s">
+        <v>89</v>
+      </c>
+      <c r="T8" t="s">
+        <v>89</v>
+      </c>
+      <c r="U8" t="s">
         <v>92</v>
       </c>
-      <c r="T8" t="s">
-        <v>92</v>
-      </c>
-      <c r="U8" t="s">
-        <v>95</v>
-      </c>
       <c r="V8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="W8" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1261,22 +1255,22 @@
         <v>41</v>
       </c>
       <c r="D9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F9" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="G9">
         <v>2743</v>
       </c>
       <c r="H9" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="I9" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="J9" s="1">
         <v>46244</v>
@@ -1288,7 +1282,7 @@
         <v>6</v>
       </c>
       <c r="M9" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="N9" s="1">
         <v>46277</v>
@@ -1303,19 +1297,19 @@
         <v>5</v>
       </c>
       <c r="S9" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="T9" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="U9" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="V9" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="W9" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1332,22 +1326,22 @@
         <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E10" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F10" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="G10">
         <v>2727</v>
       </c>
       <c r="H10" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="I10" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="J10" s="1">
         <v>46245</v>
@@ -1359,7 +1353,7 @@
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="N10" s="1">
         <v>46257</v>
@@ -1374,16 +1368,16 @@
         <v>5</v>
       </c>
       <c r="S10" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="T10" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="V10" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="W10" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1400,22 +1394,22 @@
         <v>43</v>
       </c>
       <c r="D11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E11" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F11" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="G11">
         <v>2742</v>
       </c>
       <c r="H11" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="I11" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="J11" s="1">
         <v>46245</v>
@@ -1427,7 +1421,7 @@
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="N11" s="1">
         <v>46277</v>
@@ -1442,19 +1436,19 @@
         <v>5</v>
       </c>
       <c r="S11" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="T11" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="U11" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="V11" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="W11" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1471,22 +1465,22 @@
         <v>44</v>
       </c>
       <c r="D12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E12" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F12" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="G12">
         <v>2742</v>
       </c>
       <c r="H12" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="I12" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="J12" s="1">
         <v>46245</v>
@@ -1498,7 +1492,7 @@
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="N12" s="1">
         <v>46277</v>
@@ -1513,19 +1507,19 @@
         <v>5</v>
       </c>
       <c r="S12" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="T12" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="U12" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="V12" t="s">
+        <v>107</v>
+      </c>
+      <c r="W12" t="s">
         <v>109</v>
-      </c>
-      <c r="W12" t="s">
-        <v>111</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1542,22 +1536,22 @@
         <v>45</v>
       </c>
       <c r="D13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E13" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F13" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="G13">
         <v>2742</v>
       </c>
       <c r="H13" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="I13" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="J13" s="1">
         <v>46246</v>
@@ -1569,7 +1563,7 @@
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="N13" s="1">
         <v>46278</v>
@@ -1581,19 +1575,19 @@
         <v>4</v>
       </c>
       <c r="S13" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="T13" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="U13" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="V13" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="W13" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1610,22 +1604,22 @@
         <v>46</v>
       </c>
       <c r="D14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E14" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F14" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="G14">
         <v>2721</v>
       </c>
       <c r="H14" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="I14" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="J14" s="1">
         <v>46248</v>
@@ -1637,7 +1631,7 @@
         <v>1</v>
       </c>
       <c r="M14" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="N14" s="1">
         <v>46279</v>
@@ -1649,13 +1643,13 @@
         <v>3</v>
       </c>
       <c r="S14" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="T14" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="W14" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
@@ -1672,22 +1666,22 @@
         <v>47</v>
       </c>
       <c r="D15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E15" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F15" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="G15">
         <v>2720</v>
       </c>
       <c r="H15" t="s">
+        <v>80</v>
+      </c>
+      <c r="I15" t="s">
         <v>86</v>
-      </c>
-      <c r="I15" t="s">
-        <v>89</v>
       </c>
       <c r="J15" s="1">
         <v>46248</v>
@@ -1699,7 +1693,7 @@
         <v>1</v>
       </c>
       <c r="M15" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="N15" s="1">
         <v>46259</v>
@@ -1711,13 +1705,16 @@
         <v>3</v>
       </c>
       <c r="S15" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="T15" t="s">
-        <v>91</v>
+        <v>88</v>
+      </c>
+      <c r="U15" t="s">
+        <v>96</v>
       </c>
       <c r="W15" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
@@ -1734,22 +1731,22 @@
         <v>48</v>
       </c>
       <c r="D16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E16" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F16" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="G16">
         <v>2729</v>
       </c>
       <c r="H16" t="s">
+        <v>83</v>
+      </c>
+      <c r="I16" t="s">
         <v>86</v>
-      </c>
-      <c r="I16" t="s">
-        <v>89</v>
       </c>
       <c r="J16" s="1">
         <v>46248</v>
@@ -1761,7 +1758,7 @@
         <v>1</v>
       </c>
       <c r="M16" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="N16" s="1">
         <v>46259</v>
@@ -1773,77 +1770,15 @@
         <v>3</v>
       </c>
       <c r="S16" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="T16" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="W16" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="AA16" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:27">
-      <c r="A17">
-        <v>685</v>
-      </c>
-      <c r="B17" t="s">
-        <v>27</v>
-      </c>
-      <c r="C17" t="s">
-        <v>49</v>
-      </c>
-      <c r="D17" t="s">
-        <v>64</v>
-      </c>
-      <c r="E17" t="s">
-        <v>79</v>
-      </c>
-      <c r="F17" t="s">
-        <v>80</v>
-      </c>
-      <c r="G17">
-        <v>2729</v>
-      </c>
-      <c r="H17" t="s">
-        <v>86</v>
-      </c>
-      <c r="I17" t="s">
-        <v>89</v>
-      </c>
-      <c r="J17" s="1">
-        <v>46248</v>
-      </c>
-      <c r="K17" s="1">
-        <v>46248</v>
-      </c>
-      <c r="L17">
-        <v>2</v>
-      </c>
-      <c r="M17" t="s">
-        <v>90</v>
-      </c>
-      <c r="N17" s="1">
-        <v>46259</v>
-      </c>
-      <c r="Q17">
-        <v>-8</v>
-      </c>
-      <c r="R17">
-        <v>3</v>
-      </c>
-      <c r="S17" t="s">
-        <v>91</v>
-      </c>
-      <c r="T17" t="s">
-        <v>92</v>
-      </c>
-      <c r="W17" t="s">
-        <v>111</v>
-      </c>
-      <c r="AA17" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (17/08/2026 14:35)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="111">
   <si>
     <t>om_emg</t>
   </si>
@@ -305,6 +305,9 @@
   </si>
   <si>
     <t>item será atendido com o estoque local pedido 18216324. Godoy 17/08.</t>
+  </si>
+  <si>
+    <t>Estoque alterado de "Nao" para "SIM"  daremos prioridade para movimentar o item.  Godoy 17/08/226</t>
   </si>
   <si>
     <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Consolidando embarque próximo voo para o GIG</t>
@@ -824,10 +827,10 @@
         <v>89</v>
       </c>
       <c r="V2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="W2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -895,10 +898,10 @@
         <v>90</v>
       </c>
       <c r="V3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="W3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -966,10 +969,10 @@
         <v>91</v>
       </c>
       <c r="V4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="W4" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -1034,10 +1037,10 @@
         <v>89</v>
       </c>
       <c r="V5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="W5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1102,10 +1105,10 @@
         <v>89</v>
       </c>
       <c r="V6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="W6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1164,10 +1167,10 @@
         <v>88</v>
       </c>
       <c r="V7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="W7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1235,10 +1238,10 @@
         <v>92</v>
       </c>
       <c r="V8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="W8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1306,10 +1309,10 @@
         <v>93</v>
       </c>
       <c r="V9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="W9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1374,10 +1377,10 @@
         <v>88</v>
       </c>
       <c r="V10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="W10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1445,10 +1448,10 @@
         <v>94</v>
       </c>
       <c r="V11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="W11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1516,10 +1519,10 @@
         <v>95</v>
       </c>
       <c r="V12" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="W12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1584,10 +1587,10 @@
         <v>94</v>
       </c>
       <c r="V13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="W13" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1649,7 +1652,7 @@
         <v>88</v>
       </c>
       <c r="W14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
@@ -1714,7 +1717,7 @@
         <v>96</v>
       </c>
       <c r="W15" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
@@ -1770,13 +1773,16 @@
         <v>3</v>
       </c>
       <c r="S16" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="T16" t="s">
         <v>89</v>
       </c>
+      <c r="U16" t="s">
+        <v>97</v>
+      </c>
       <c r="W16" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AA16" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (18/08/2026 08:33)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -815,10 +815,10 @@
         <v>46251</v>
       </c>
       <c r="Q2">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R2">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="S2" t="s">
         <v>88</v>
@@ -883,10 +883,10 @@
         <v>46249</v>
       </c>
       <c r="Q3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R3">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="S3" t="s">
         <v>88</v>
@@ -954,10 +954,10 @@
         <v>46240</v>
       </c>
       <c r="Q4">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="R4">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="S4" t="s">
         <v>88</v>
@@ -1025,10 +1025,10 @@
         <v>46265</v>
       </c>
       <c r="Q5">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="R5">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="S5" t="s">
         <v>88</v>
@@ -1093,10 +1093,10 @@
         <v>46269</v>
       </c>
       <c r="Q6">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="R6">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S6" t="s">
         <v>88</v>
@@ -1158,10 +1158,10 @@
         <v>46248</v>
       </c>
       <c r="Q7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R7">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S7" t="s">
         <v>88</v>
@@ -1223,10 +1223,10 @@
         <v>46255</v>
       </c>
       <c r="Q8">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S8" t="s">
         <v>89</v>
@@ -1294,10 +1294,10 @@
         <v>46254</v>
       </c>
       <c r="Q9">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="R9">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S9" t="s">
         <v>89</v>
@@ -1365,10 +1365,10 @@
         <v>46257</v>
       </c>
       <c r="Q10">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S10" t="s">
         <v>88</v>
@@ -1433,10 +1433,10 @@
         <v>46254</v>
       </c>
       <c r="Q11">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="R11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S11" t="s">
         <v>88</v>
@@ -1504,10 +1504,10 @@
         <v>46254</v>
       </c>
       <c r="Q12">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="R12">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S12" t="s">
         <v>89</v>
@@ -1572,10 +1572,10 @@
         <v>46278</v>
       </c>
       <c r="Q13">
-        <v>-27</v>
+        <v>-26</v>
       </c>
       <c r="R13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S13" t="s">
         <v>88</v>
@@ -1640,10 +1640,10 @@
         <v>46279</v>
       </c>
       <c r="Q14">
-        <v>-28</v>
+        <v>-27</v>
       </c>
       <c r="R14">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S14" t="s">
         <v>89</v>
@@ -1702,10 +1702,10 @@
         <v>46259</v>
       </c>
       <c r="Q15">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="R15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S15" t="s">
         <v>89</v>
@@ -1767,10 +1767,10 @@
         <v>46259</v>
       </c>
       <c r="Q16">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="R16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S16" t="s">
         <v>89</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (18/08/2026 10:49)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="101">
   <si>
     <t>om_emg</t>
   </si>
@@ -106,36 +106,27 @@
     <t>BABE</t>
   </si>
   <si>
+    <t>BACO</t>
+  </si>
+  <si>
+    <t>BACG</t>
+  </si>
+  <si>
+    <t>DACTA II</t>
+  </si>
+  <si>
     <t>BABR</t>
   </si>
   <si>
-    <t>BACO</t>
-  </si>
-  <si>
-    <t>BACG</t>
-  </si>
-  <si>
-    <t>DACTA II</t>
-  </si>
-  <si>
     <t>685260012350</t>
   </si>
   <si>
-    <t>685260012387</t>
-  </si>
-  <si>
-    <t>313260018657</t>
-  </si>
-  <si>
     <t>313260018658</t>
   </si>
   <si>
     <t>396260016580</t>
   </si>
   <si>
-    <t>329260019264</t>
-  </si>
-  <si>
     <t>685260012560</t>
   </si>
   <si>
@@ -166,18 +157,12 @@
     <t>030-1094-58</t>
   </si>
   <si>
-    <t>066-3084-32</t>
-  </si>
-  <si>
     <t>324843-W020</t>
   </si>
   <si>
     <t>2601188-204</t>
   </si>
   <si>
-    <t>C662041-0102</t>
-  </si>
-  <si>
     <t>2641010-3</t>
   </si>
   <si>
@@ -208,18 +193,12 @@
     <t>CONNECTOR</t>
   </si>
   <si>
-    <t>IND RDR 2000 IN-182A</t>
-  </si>
-  <si>
     <t>HEADSET-MICROPHONE</t>
   </si>
   <si>
     <t>COMPRESSOR DRIVE ASS</t>
   </si>
   <si>
-    <t>INDICATOR FUEL</t>
-  </si>
-  <si>
     <t>AXLE FITTING</t>
   </si>
   <si>
@@ -250,18 +229,15 @@
     <t>C</t>
   </si>
   <si>
+    <t>T</t>
+  </si>
+  <si>
     <t>R</t>
   </si>
   <si>
-    <t>T</t>
-  </si>
-  <si>
     <t>Providência tomada</t>
   </si>
   <si>
-    <t>Atendido parcialmente</t>
-  </si>
-  <si>
     <t>Expedido total</t>
   </si>
   <si>
@@ -271,9 +247,6 @@
     <t>ANCE</t>
   </si>
   <si>
-    <t>AIFP</t>
-  </si>
-  <si>
     <t>IPLR</t>
   </si>
   <si>
@@ -286,19 +259,16 @@
     <t>Sim</t>
   </si>
   <si>
-    <t>Alterado o tipo da emerg. de IPLR para ANCE. Godoy 22/07/26</t>
-  </si>
-  <si>
-    <t>Atendido 01 EA através da TSP 18122931. Outros 02 EA serão enviados pela empresa. Ramon 03/08/26. AWB 12750821282 volume retirado na loja GOLLOG - MAO por kleyton EM 06/08. Godoy 12/08/26.</t>
-  </si>
-  <si>
     <t>item atendido com o estoque local pedido 18171852 em 10/08. Godoy 11/08. Está sendo definido se o PN está correto. Ramon 11/08/26.</t>
   </si>
   <si>
     <t>Estoque com 12 EA do Pn LM600-9 (Alternado). Godoy 12/08/26. Atendido com estoque local em 13/08. Ramon 13/08/26</t>
   </si>
   <si>
-    <t>Item em pane, anv autorizada a voar por 3 dias pela MMEL a contar de 12/08. Ramon 13/08/26</t>
+    <t>RECIBO não se encontra na pasta do drive. Godoy 18/08/26.</t>
+  </si>
+  <si>
+    <t>Item em pane, anv autorizada a voar por 3 dias pela MMEL a contar de 12/08. Ramon 13/08/26. AWB 12752990604 - volume retirado na loja GOLLOG - CWB por RAFAEL MAIA DE LIMA em 15/08. Godoy 18/08/26.</t>
   </si>
   <si>
     <t>Estoque no alternado 285K4. Caso use do estoque, verificar validade que consta no item. Ramon 12/08/26. Item em pane, anv autorizada a voar por 3 dias pela MMEL a contar de 12/08. Ramon 13/08/26</t>
@@ -310,40 +280,40 @@
     <t>Estoque alterado de "Nao" para "SIM"  daremos prioridade para movimentar o item.  Godoy 17/08/226</t>
   </si>
   <si>
-    <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Consolidando embarque próximo voo para o GIG</t>
-  </si>
-  <si>
-    <t>Item em bancada porem em pessimo estado, foi solicitado recolhimento de mais unidades para envio a oficina para tentativa de reparo ATZ Marcio 17/7/26. Solicitado abertura de O.S. para 3EA do item no dia 16-07-26 via Email para a Coordenadoria - CLA-21-07-26- SERÁ ENTREGUE PELA WILLIAM DPE DIA 14-08-26 - CLA-13-08</t>
-  </si>
-  <si>
-    <t>Enviado para o Operador(02 EA), atendimento parcial, em 31/07/2026 -AWB 127-5041 6833- REZ - o outro 1 EA será atendido pelo estoque FAB. conforme solicitado por Email- CLA-03-08 - AWB 127-5082 1282 -1 EA ENVIADO ESTOQUE FAB - Material entregue dia 06/08/2026</t>
-  </si>
-  <si>
-    <t>Temos 4 EA em manutenção na William, será pedido prioridade. CLA-03-08 - DPE DIA 14-08 - CLA 13-08</t>
+    <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Chegada GIG dia 15-08 (voo 4273). Canal verde dia 17/08. Aguardando SEFAZ.</t>
+  </si>
+  <si>
+    <t>Temos 4 EA em manutenção na William, será pedido prioridade. CLA-03-08 - DPE DIA 14-08 - CLA 13-08 - AWB 127-5299 2505 DPE 18/08/2026</t>
   </si>
   <si>
     <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
   </si>
   <si>
-    <t>Foi solicitado abertura de O.S. no dia 7 -08-26 de 6 EA. As OSs foram abertas e aguardando recolhimento para reparo. CLA-10-08 - ITEM FOI RECOLHIDO PELA WILLIAM- CLA-11-08 - DPE 14-08</t>
-  </si>
-  <si>
     <t>Foi solicitado atendimento com estoque FAB - CLA- 10-08, ITEM PRONTO PARA EMBARQUE, AGUARDANDO NOTA FISCAL - CLA-11-08- ITEM AGUARDANDO DEFINIÇÃO DA COORDENADORIA QUANTO A EFETIVIDADE PARA APLICAÇÃO NA REFERIDA ANV.- CLA-13-08</t>
   </si>
   <si>
-    <t>Temos somente 03 ea em STK, favor utilizar o estoque FAB para posterior devolução. ATZ RC 13/08 - FOI SOLICITADO O ATENDIMENTO COM ESTOQUE FAB -CLA-13-08</t>
-  </si>
-  <si>
-    <t>Previsao de entrega da oficina do RJ na V1 JPA 13/8/2026 durante o dia, horario comercial, ATZ Marcio 12/8 13:22hs</t>
-  </si>
-  <si>
-    <t>1 Unidade na oficina em BH William, solicitado prioridade na entrega DPE 14/8, aguardando orçamento final ATZ Marcio 12/8 13:24hs- DPE 14-08</t>
-  </si>
-  <si>
-    <t>Temos no STK V1, material em separação, recibo 682/FAB/26 - atz rc 13/08</t>
-  </si>
-  <si>
-    <t>será enviado o pn 9910592-2 do estoque da VeeOne base PAMALS. -CLA -14-08</t>
+    <t>Temos somente 03 ea em STK, favor utilizar o estoque FAB para posterior devolução. ATZ RC 13/08 - FOI SOLICITADO O ATENDIMENTO COM ESTOQUE FAB -CLA-13-08 - AWB 127-5299 0173 DPE 18/08/2026</t>
+  </si>
+  <si>
+    <t>Previsao de entrega da oficina do RJ na V1 JPA 13/8/2026 durante o dia, horario comercial, ATZ Marcio 12/8 13:22hs - Material entregue dia 17/08/2026 - Retirado pelo TEN Goncalves</t>
+  </si>
+  <si>
+    <t>1 Unidade na oficina em BH William, solicitado prioridade na entrega DPE 14/8, aguardando orçamento final ATZ Marcio 12/8 13:24hs- DPE 14-08 - AWB 127-5299 0604 DPE 15-08-26 CLA-17-08</t>
+  </si>
+  <si>
+    <t>Temos no STK V1, material em separação, recibo 682/FAB/26 - atz rc 13/08 - MATERIAL ENVIADO VIA AWB 12752709016 - DPE 18/08/2026</t>
+  </si>
+  <si>
+    <t>será enviado o pn 9910592-2 do estoque da VeeOne base PAMALS. -CLA -14-08- AWB 127-5299 0604 DPE 15-08-26 CLA-17-08</t>
+  </si>
+  <si>
+    <t>foi solicitoado o atendimento com o estoque FAB. CLA-17-08 - o item PN superado 069-1025-25 não serve na ANV 2721 - temos 4ea na wiliam para reparo, já foi solicitado o DPE.</t>
+  </si>
+  <si>
+    <t>foi solicitoado o atendimento com o estoque FAB. CLA-17-08</t>
+  </si>
+  <si>
+    <t>ITEM FOI ENTREGUE PARA A FAB VIA RECIBO 598/FAB/26 31-07-26 - AINDA NÃO FOI PARA O ESTOQUECLA-17-08</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -682,7 +652,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA16"/>
+  <dimension ref="A1:AA13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -779,22 +749,22 @@
         <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E2" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="F2" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="G2">
         <v>2702</v>
       </c>
       <c r="H2" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="I2" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="J2" s="1">
         <v>46212</v>
@@ -806,7 +776,7 @@
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="N2" s="1">
         <v>46243</v>
@@ -821,16 +791,16 @@
         <v>40</v>
       </c>
       <c r="S2" t="s">
+        <v>79</v>
+      </c>
+      <c r="T2" t="s">
+        <v>80</v>
+      </c>
+      <c r="V2" t="s">
         <v>88</v>
       </c>
-      <c r="T2" t="s">
-        <v>89</v>
-      </c>
-      <c r="V2" t="s">
-        <v>98</v>
-      </c>
       <c r="W2" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -838,70 +808,67 @@
     </row>
     <row r="3" spans="1:27">
       <c r="A3">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
         <v>35</v>
       </c>
       <c r="D3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E3" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="F3" t="s">
+        <v>71</v>
+      </c>
+      <c r="G3">
+        <v>2737</v>
+      </c>
+      <c r="H3" t="s">
+        <v>73</v>
+      </c>
+      <c r="I3" t="s">
+        <v>76</v>
+      </c>
+      <c r="J3" s="1">
+        <v>46205</v>
+      </c>
+      <c r="K3" s="1">
+        <v>46234</v>
+      </c>
+      <c r="L3">
+        <v>3</v>
+      </c>
+      <c r="M3" t="s">
         <v>78</v>
       </c>
-      <c r="G3">
-        <v>2722</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="N3" s="1">
+        <v>46265</v>
+      </c>
+      <c r="O3" s="1">
+        <v>46252</v>
+      </c>
+      <c r="Q3">
+        <v>-13</v>
+      </c>
+      <c r="R3">
+        <v>18</v>
+      </c>
+      <c r="S3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T3" t="s">
         <v>80</v>
       </c>
-      <c r="I3" t="s">
-        <v>84</v>
-      </c>
-      <c r="J3" s="1">
-        <v>46219</v>
-      </c>
-      <c r="K3" s="1">
-        <v>46218</v>
-      </c>
-      <c r="L3">
-        <v>1</v>
-      </c>
-      <c r="M3" t="s">
-        <v>87</v>
-      </c>
-      <c r="N3" s="1">
-        <v>46249</v>
-      </c>
-      <c r="O3" s="1">
-        <v>46249</v>
-      </c>
-      <c r="Q3">
-        <v>3</v>
-      </c>
-      <c r="R3">
-        <v>34</v>
-      </c>
-      <c r="S3" t="s">
-        <v>88</v>
-      </c>
-      <c r="T3" t="s">
+      <c r="V3" t="s">
         <v>89</v>
       </c>
-      <c r="U3" t="s">
-        <v>90</v>
-      </c>
-      <c r="V3" t="s">
-        <v>99</v>
-      </c>
       <c r="W3" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -909,70 +876,67 @@
     </row>
     <row r="4" spans="1:27">
       <c r="A4">
-        <v>313</v>
+        <v>396</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C4" t="s">
         <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E4" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G4">
+        <v>2733</v>
+      </c>
+      <c r="H4" t="s">
+        <v>73</v>
+      </c>
+      <c r="I4" t="s">
+        <v>76</v>
+      </c>
+      <c r="J4" s="1">
+        <v>46238</v>
+      </c>
+      <c r="K4" s="1">
+        <v>46238</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4" t="s">
+        <v>78</v>
+      </c>
+      <c r="N4" s="1">
+        <v>46269</v>
+      </c>
+      <c r="O4" s="1">
+        <v>46269</v>
+      </c>
+      <c r="Q4">
+        <v>-17</v>
+      </c>
+      <c r="R4">
+        <v>14</v>
+      </c>
+      <c r="S4" t="s">
         <v>79</v>
       </c>
-      <c r="G4">
-        <v>2736</v>
-      </c>
-      <c r="H4" t="s">
-        <v>81</v>
-      </c>
-      <c r="I4" t="s">
-        <v>84</v>
-      </c>
-      <c r="J4" s="1">
-        <v>46205</v>
-      </c>
-      <c r="K4" s="1">
-        <v>46234</v>
-      </c>
-      <c r="L4">
-        <v>3</v>
-      </c>
-      <c r="M4" t="s">
-        <v>87</v>
-      </c>
-      <c r="N4" s="1">
-        <v>46265</v>
-      </c>
-      <c r="O4" s="1">
-        <v>46240</v>
-      </c>
-      <c r="Q4">
-        <v>-13</v>
-      </c>
-      <c r="R4">
-        <v>18</v>
-      </c>
-      <c r="S4" t="s">
-        <v>88</v>
-      </c>
       <c r="T4" t="s">
-        <v>89</v>
-      </c>
-      <c r="U4" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="V4" t="s">
+        <v>90</v>
+      </c>
+      <c r="W4" t="s">
         <v>100</v>
-      </c>
-      <c r="W4" t="s">
-        <v>110</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -980,67 +944,70 @@
     </row>
     <row r="5" spans="1:27">
       <c r="A5">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C5" t="s">
         <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E5" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F5" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="G5">
-        <v>2737</v>
+        <v>2729</v>
       </c>
       <c r="H5" t="s">
+        <v>74</v>
+      </c>
+      <c r="I5" t="s">
+        <v>77</v>
+      </c>
+      <c r="J5" s="1">
+        <v>46244</v>
+      </c>
+      <c r="K5" s="1">
+        <v>46244</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5" t="s">
+        <v>78</v>
+      </c>
+      <c r="N5" s="1">
+        <v>46255</v>
+      </c>
+      <c r="O5" s="1">
+        <v>46255</v>
+      </c>
+      <c r="Q5">
+        <v>-3</v>
+      </c>
+      <c r="R5">
+        <v>8</v>
+      </c>
+      <c r="S5" t="s">
         <v>80</v>
       </c>
-      <c r="I5" t="s">
-        <v>84</v>
-      </c>
-      <c r="J5" s="1">
-        <v>46205</v>
-      </c>
-      <c r="K5" s="1">
-        <v>46234</v>
-      </c>
-      <c r="L5">
-        <v>3</v>
-      </c>
-      <c r="M5" t="s">
-        <v>87</v>
-      </c>
-      <c r="N5" s="1">
-        <v>46265</v>
-      </c>
-      <c r="O5" s="1">
-        <v>46265</v>
-      </c>
-      <c r="Q5">
-        <v>-13</v>
-      </c>
-      <c r="R5">
-        <v>18</v>
-      </c>
-      <c r="S5" t="s">
-        <v>88</v>
-      </c>
       <c r="T5" t="s">
-        <v>89</v>
+        <v>80</v>
+      </c>
+      <c r="U5" t="s">
+        <v>81</v>
       </c>
       <c r="V5" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="W5" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1048,67 +1015,70 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6">
-        <v>396</v>
+        <v>386</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C6" t="s">
         <v>38</v>
       </c>
       <c r="D6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E6" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F6" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="G6">
-        <v>2733</v>
+        <v>2743</v>
       </c>
       <c r="H6" t="s">
+        <v>74</v>
+      </c>
+      <c r="I6" t="s">
+        <v>76</v>
+      </c>
+      <c r="J6" s="1">
+        <v>46244</v>
+      </c>
+      <c r="K6" s="1">
+        <v>46246</v>
+      </c>
+      <c r="L6">
+        <v>6</v>
+      </c>
+      <c r="M6" t="s">
+        <v>78</v>
+      </c>
+      <c r="N6" s="1">
+        <v>46277</v>
+      </c>
+      <c r="O6" s="1">
+        <v>46254</v>
+      </c>
+      <c r="Q6">
+        <v>-25</v>
+      </c>
+      <c r="R6">
+        <v>6</v>
+      </c>
+      <c r="S6" t="s">
         <v>80</v>
       </c>
-      <c r="I6" t="s">
-        <v>84</v>
-      </c>
-      <c r="J6" s="1">
-        <v>46238</v>
-      </c>
-      <c r="K6" s="1">
-        <v>46238</v>
-      </c>
-      <c r="L6">
-        <v>1</v>
-      </c>
-      <c r="M6" t="s">
-        <v>87</v>
-      </c>
-      <c r="N6" s="1">
-        <v>46269</v>
-      </c>
-      <c r="O6" s="1">
-        <v>46269</v>
-      </c>
-      <c r="Q6">
-        <v>-17</v>
-      </c>
-      <c r="R6">
-        <v>14</v>
-      </c>
-      <c r="S6" t="s">
-        <v>88</v>
-      </c>
       <c r="T6" t="s">
-        <v>89</v>
+        <v>79</v>
+      </c>
+      <c r="U6" t="s">
+        <v>82</v>
       </c>
       <c r="V6" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="W6" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1116,61 +1086,70 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>329</v>
+        <v>690</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C7" t="s">
         <v>39</v>
       </c>
       <c r="D7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E7" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="F7" t="s">
+        <v>72</v>
+      </c>
+      <c r="G7">
+        <v>2727</v>
+      </c>
+      <c r="H7" t="s">
+        <v>73</v>
+      </c>
+      <c r="I7" t="s">
+        <v>77</v>
+      </c>
+      <c r="J7" s="1">
+        <v>46245</v>
+      </c>
+      <c r="K7" s="1">
+        <v>46246</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7" t="s">
         <v>78</v>
       </c>
-      <c r="G7">
-        <v>2721</v>
-      </c>
-      <c r="H7" t="s">
-        <v>80</v>
-      </c>
-      <c r="I7" t="s">
-        <v>85</v>
-      </c>
-      <c r="J7" s="1">
-        <v>46241</v>
-      </c>
-      <c r="K7" s="1">
-        <v>46241</v>
-      </c>
-      <c r="L7">
-        <v>2</v>
-      </c>
-      <c r="M7" t="s">
-        <v>87</v>
-      </c>
       <c r="N7" s="1">
-        <v>46248</v>
+        <v>46257</v>
+      </c>
+      <c r="O7" s="1">
+        <v>46251</v>
       </c>
       <c r="Q7">
-        <v>4</v>
+        <v>-5</v>
       </c>
       <c r="R7">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="S7" t="s">
-        <v>88</v>
+        <v>79</v>
+      </c>
+      <c r="T7" t="s">
+        <v>79</v>
+      </c>
+      <c r="U7" t="s">
+        <v>83</v>
       </c>
       <c r="V7" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="W7" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1178,70 +1157,70 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>685</v>
+        <v>384</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C8" t="s">
         <v>40</v>
       </c>
       <c r="D8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E8" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="F8" t="s">
+        <v>71</v>
+      </c>
+      <c r="G8">
+        <v>2742</v>
+      </c>
+      <c r="H8" t="s">
+        <v>73</v>
+      </c>
+      <c r="I8" t="s">
+        <v>76</v>
+      </c>
+      <c r="J8" s="1">
+        <v>46245</v>
+      </c>
+      <c r="K8" s="1">
+        <v>46246</v>
+      </c>
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8" t="s">
+        <v>78</v>
+      </c>
+      <c r="N8" s="1">
+        <v>46277</v>
+      </c>
+      <c r="O8" s="1">
+        <v>46254</v>
+      </c>
+      <c r="Q8">
+        <v>-25</v>
+      </c>
+      <c r="R8">
+        <v>6</v>
+      </c>
+      <c r="S8" t="s">
         <v>79</v>
       </c>
-      <c r="G8">
-        <v>2729</v>
-      </c>
-      <c r="H8" t="s">
-        <v>82</v>
-      </c>
-      <c r="I8" t="s">
-        <v>86</v>
-      </c>
-      <c r="J8" s="1">
-        <v>46244</v>
-      </c>
-      <c r="K8" s="1">
-        <v>46244</v>
-      </c>
-      <c r="L8">
-        <v>1</v>
-      </c>
-      <c r="M8" t="s">
-        <v>87</v>
-      </c>
-      <c r="N8" s="1">
-        <v>46255</v>
-      </c>
-      <c r="O8" s="1">
-        <v>46255</v>
-      </c>
-      <c r="Q8">
-        <v>-3</v>
-      </c>
-      <c r="R8">
-        <v>8</v>
-      </c>
-      <c r="S8" t="s">
-        <v>89</v>
-      </c>
       <c r="T8" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="U8" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="V8" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="W8" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1249,43 +1228,43 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C9" t="s">
         <v>41</v>
       </c>
       <c r="D9" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E9" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="F9" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="G9">
-        <v>2743</v>
+        <v>2742</v>
       </c>
       <c r="H9" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="I9" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="J9" s="1">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="K9" s="1">
         <v>46246</v>
       </c>
       <c r="L9">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="N9" s="1">
         <v>46277</v>
@@ -1300,19 +1279,19 @@
         <v>6</v>
       </c>
       <c r="S9" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="T9" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="U9" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="V9" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="W9" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1320,7 +1299,7 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>690</v>
+        <v>384</v>
       </c>
       <c r="B10" t="s">
         <v>32</v>
@@ -1329,58 +1308,61 @@
         <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E10" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="F10" t="s">
+        <v>72</v>
+      </c>
+      <c r="G10">
+        <v>2742</v>
+      </c>
+      <c r="H10" t="s">
+        <v>73</v>
+      </c>
+      <c r="I10" t="s">
+        <v>76</v>
+      </c>
+      <c r="J10" s="1">
+        <v>46246</v>
+      </c>
+      <c r="K10" s="1">
+        <v>46247</v>
+      </c>
+      <c r="L10">
+        <v>1</v>
+      </c>
+      <c r="M10" t="s">
         <v>78</v>
       </c>
-      <c r="G10">
-        <v>2727</v>
-      </c>
-      <c r="H10" t="s">
-        <v>80</v>
-      </c>
-      <c r="I10" t="s">
-        <v>86</v>
-      </c>
-      <c r="J10" s="1">
-        <v>46245</v>
-      </c>
-      <c r="K10" s="1">
-        <v>46246</v>
-      </c>
-      <c r="L10">
-        <v>1</v>
-      </c>
-      <c r="M10" t="s">
-        <v>87</v>
-      </c>
       <c r="N10" s="1">
-        <v>46257</v>
+        <v>46278</v>
       </c>
       <c r="O10" s="1">
-        <v>46257</v>
+        <v>46249</v>
       </c>
       <c r="Q10">
-        <v>-5</v>
+        <v>-26</v>
       </c>
       <c r="R10">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S10" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="T10" t="s">
-        <v>88</v>
+        <v>79</v>
+      </c>
+      <c r="U10" t="s">
+        <v>84</v>
       </c>
       <c r="V10" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="W10" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1388,7 +1370,7 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>384</v>
+        <v>329</v>
       </c>
       <c r="B11" t="s">
         <v>33</v>
@@ -1397,61 +1379,55 @@
         <v>43</v>
       </c>
       <c r="D11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E11" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="F11" t="s">
+        <v>72</v>
+      </c>
+      <c r="G11">
+        <v>2721</v>
+      </c>
+      <c r="H11" t="s">
+        <v>75</v>
+      </c>
+      <c r="I11" t="s">
+        <v>76</v>
+      </c>
+      <c r="J11" s="1">
+        <v>46248</v>
+      </c>
+      <c r="K11" s="1">
+        <v>46248</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11" t="s">
+        <v>78</v>
+      </c>
+      <c r="N11" s="1">
+        <v>46279</v>
+      </c>
+      <c r="Q11">
+        <v>-27</v>
+      </c>
+      <c r="R11">
+        <v>4</v>
+      </c>
+      <c r="S11" t="s">
+        <v>80</v>
+      </c>
+      <c r="T11" t="s">
         <v>79</v>
       </c>
-      <c r="G11">
-        <v>2742</v>
-      </c>
-      <c r="H11" t="s">
-        <v>80</v>
-      </c>
-      <c r="I11" t="s">
-        <v>84</v>
-      </c>
-      <c r="J11" s="1">
-        <v>46245</v>
-      </c>
-      <c r="K11" s="1">
-        <v>46246</v>
-      </c>
-      <c r="L11">
-        <v>1</v>
-      </c>
-      <c r="M11" t="s">
-        <v>87</v>
-      </c>
-      <c r="N11" s="1">
-        <v>46277</v>
-      </c>
-      <c r="O11" s="1">
-        <v>46254</v>
-      </c>
-      <c r="Q11">
-        <v>-25</v>
-      </c>
-      <c r="R11">
-        <v>6</v>
-      </c>
-      <c r="S11" t="s">
-        <v>88</v>
-      </c>
-      <c r="T11" t="s">
-        <v>88</v>
-      </c>
-      <c r="U11" t="s">
-        <v>94</v>
-      </c>
       <c r="V11" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="W11" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1459,7 +1435,7 @@
     </row>
     <row r="12" spans="1:27">
       <c r="A12">
-        <v>384</v>
+        <v>329</v>
       </c>
       <c r="B12" t="s">
         <v>33</v>
@@ -1468,61 +1444,58 @@
         <v>44</v>
       </c>
       <c r="D12" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E12" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="F12" t="s">
+        <v>71</v>
+      </c>
+      <c r="G12">
+        <v>2720</v>
+      </c>
+      <c r="H12" t="s">
+        <v>73</v>
+      </c>
+      <c r="I12" t="s">
         <v>77</v>
       </c>
-      <c r="G12">
-        <v>2742</v>
-      </c>
-      <c r="H12" t="s">
+      <c r="J12" s="1">
+        <v>46248</v>
+      </c>
+      <c r="K12" s="1">
+        <v>46248</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12" t="s">
+        <v>78</v>
+      </c>
+      <c r="N12" s="1">
+        <v>46259</v>
+      </c>
+      <c r="Q12">
+        <v>-7</v>
+      </c>
+      <c r="R12">
+        <v>4</v>
+      </c>
+      <c r="S12" t="s">
         <v>80</v>
       </c>
-      <c r="I12" t="s">
-        <v>84</v>
-      </c>
-      <c r="J12" s="1">
-        <v>46245</v>
-      </c>
-      <c r="K12" s="1">
-        <v>46246</v>
-      </c>
-      <c r="L12">
-        <v>1</v>
-      </c>
-      <c r="M12" t="s">
-        <v>87</v>
-      </c>
-      <c r="N12" s="1">
-        <v>46277</v>
-      </c>
-      <c r="O12" s="1">
-        <v>46254</v>
-      </c>
-      <c r="Q12">
-        <v>-25</v>
-      </c>
-      <c r="R12">
-        <v>6</v>
-      </c>
-      <c r="S12" t="s">
-        <v>89</v>
-      </c>
       <c r="T12" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="U12" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="V12" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="W12" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1530,261 +1503,69 @@
     </row>
     <row r="13" spans="1:27">
       <c r="A13">
-        <v>384</v>
+        <v>685</v>
       </c>
       <c r="B13" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C13" t="s">
         <v>45</v>
       </c>
       <c r="D13" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E13" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F13" t="s">
+        <v>71</v>
+      </c>
+      <c r="G13">
+        <v>2729</v>
+      </c>
+      <c r="H13" t="s">
+        <v>75</v>
+      </c>
+      <c r="I13" t="s">
+        <v>77</v>
+      </c>
+      <c r="J13" s="1">
+        <v>46248</v>
+      </c>
+      <c r="K13" s="1">
+        <v>46248</v>
+      </c>
+      <c r="L13">
+        <v>1</v>
+      </c>
+      <c r="M13" t="s">
         <v>78</v>
       </c>
-      <c r="G13">
-        <v>2742</v>
-      </c>
-      <c r="H13" t="s">
+      <c r="N13" s="1">
+        <v>46259</v>
+      </c>
+      <c r="Q13">
+        <v>-7</v>
+      </c>
+      <c r="R13">
+        <v>4</v>
+      </c>
+      <c r="S13" t="s">
         <v>80</v>
       </c>
-      <c r="I13" t="s">
-        <v>84</v>
-      </c>
-      <c r="J13" s="1">
-        <v>46246</v>
-      </c>
-      <c r="K13" s="1">
-        <v>46247</v>
-      </c>
-      <c r="L13">
-        <v>1</v>
-      </c>
-      <c r="M13" t="s">
+      <c r="T13" t="s">
+        <v>80</v>
+      </c>
+      <c r="U13" t="s">
         <v>87</v>
       </c>
-      <c r="N13" s="1">
-        <v>46278</v>
-      </c>
-      <c r="Q13">
-        <v>-26</v>
-      </c>
-      <c r="R13">
-        <v>5</v>
-      </c>
-      <c r="S13" t="s">
-        <v>88</v>
-      </c>
-      <c r="T13" t="s">
-        <v>88</v>
-      </c>
-      <c r="U13" t="s">
-        <v>94</v>
-      </c>
       <c r="V13" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="W13" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="AA13" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:27">
-      <c r="A14">
-        <v>329</v>
-      </c>
-      <c r="B14" t="s">
-        <v>30</v>
-      </c>
-      <c r="C14" t="s">
-        <v>46</v>
-      </c>
-      <c r="D14" t="s">
-        <v>60</v>
-      </c>
-      <c r="E14" t="s">
-        <v>74</v>
-      </c>
-      <c r="F14" t="s">
-        <v>78</v>
-      </c>
-      <c r="G14">
-        <v>2721</v>
-      </c>
-      <c r="H14" t="s">
-        <v>83</v>
-      </c>
-      <c r="I14" t="s">
-        <v>84</v>
-      </c>
-      <c r="J14" s="1">
-        <v>46248</v>
-      </c>
-      <c r="K14" s="1">
-        <v>46248</v>
-      </c>
-      <c r="L14">
-        <v>1</v>
-      </c>
-      <c r="M14" t="s">
-        <v>87</v>
-      </c>
-      <c r="N14" s="1">
-        <v>46279</v>
-      </c>
-      <c r="Q14">
-        <v>-27</v>
-      </c>
-      <c r="R14">
-        <v>4</v>
-      </c>
-      <c r="S14" t="s">
-        <v>89</v>
-      </c>
-      <c r="T14" t="s">
-        <v>88</v>
-      </c>
-      <c r="W14" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA14" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:27">
-      <c r="A15">
-        <v>329</v>
-      </c>
-      <c r="B15" t="s">
-        <v>30</v>
-      </c>
-      <c r="C15" t="s">
-        <v>47</v>
-      </c>
-      <c r="D15" t="s">
-        <v>61</v>
-      </c>
-      <c r="E15" t="s">
-        <v>75</v>
-      </c>
-      <c r="F15" t="s">
-        <v>79</v>
-      </c>
-      <c r="G15">
-        <v>2720</v>
-      </c>
-      <c r="H15" t="s">
-        <v>80</v>
-      </c>
-      <c r="I15" t="s">
-        <v>86</v>
-      </c>
-      <c r="J15" s="1">
-        <v>46248</v>
-      </c>
-      <c r="K15" s="1">
-        <v>46248</v>
-      </c>
-      <c r="L15">
-        <v>1</v>
-      </c>
-      <c r="M15" t="s">
-        <v>87</v>
-      </c>
-      <c r="N15" s="1">
-        <v>46259</v>
-      </c>
-      <c r="Q15">
-        <v>-7</v>
-      </c>
-      <c r="R15">
-        <v>4</v>
-      </c>
-      <c r="S15" t="s">
-        <v>89</v>
-      </c>
-      <c r="T15" t="s">
-        <v>88</v>
-      </c>
-      <c r="U15" t="s">
-        <v>96</v>
-      </c>
-      <c r="W15" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA15" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:27">
-      <c r="A16">
-        <v>685</v>
-      </c>
-      <c r="B16" t="s">
-        <v>27</v>
-      </c>
-      <c r="C16" t="s">
-        <v>48</v>
-      </c>
-      <c r="D16" t="s">
-        <v>62</v>
-      </c>
-      <c r="E16" t="s">
-        <v>76</v>
-      </c>
-      <c r="F16" t="s">
-        <v>79</v>
-      </c>
-      <c r="G16">
-        <v>2729</v>
-      </c>
-      <c r="H16" t="s">
-        <v>83</v>
-      </c>
-      <c r="I16" t="s">
-        <v>86</v>
-      </c>
-      <c r="J16" s="1">
-        <v>46248</v>
-      </c>
-      <c r="K16" s="1">
-        <v>46248</v>
-      </c>
-      <c r="L16">
-        <v>1</v>
-      </c>
-      <c r="M16" t="s">
-        <v>87</v>
-      </c>
-      <c r="N16" s="1">
-        <v>46259</v>
-      </c>
-      <c r="Q16">
-        <v>-7</v>
-      </c>
-      <c r="R16">
-        <v>4</v>
-      </c>
-      <c r="S16" t="s">
-        <v>89</v>
-      </c>
-      <c r="T16" t="s">
-        <v>89</v>
-      </c>
-      <c r="U16" t="s">
-        <v>97</v>
-      </c>
-      <c r="W16" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA16" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (18/08/2026 12:31)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="107">
   <si>
     <t>om_emg</t>
   </si>
@@ -154,6 +154,12 @@
     <t>685260012609</t>
   </si>
   <si>
+    <t>313260018702</t>
+  </si>
+  <si>
+    <t>685260012619</t>
+  </si>
+  <si>
     <t>030-1094-58</t>
   </si>
   <si>
@@ -190,6 +196,12 @@
     <t>162-10700</t>
   </si>
   <si>
+    <t>040-0043</t>
+  </si>
+  <si>
+    <t>071-01519-0101</t>
+  </si>
+  <si>
     <t>CONNECTOR</t>
   </si>
   <si>
@@ -224,6 +236,12 @@
   </si>
   <si>
     <t>OUTER WHEEL HALF ASS</t>
+  </si>
+  <si>
+    <t>STROB TUB</t>
+  </si>
+  <si>
+    <t>RECEIVER-EXCITER,RAD</t>
   </si>
   <si>
     <t>C</t>
@@ -326,8 +344,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -343,7 +369,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -351,12 +377,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -652,89 +696,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA13"/>
+  <dimension ref="A1:AA15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -749,39 +793,39 @@
         <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="F2" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="G2">
         <v>2702</v>
       </c>
       <c r="H2" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="I2" t="s">
-        <v>76</v>
-      </c>
-      <c r="J2" s="1">
+        <v>82</v>
+      </c>
+      <c r="J2" s="2">
         <v>46212</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46212</v>
       </c>
       <c r="L2">
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>78</v>
-      </c>
-      <c r="N2" s="1">
+        <v>84</v>
+      </c>
+      <c r="N2" s="2">
         <v>46243</v>
       </c>
-      <c r="O2" s="1">
+      <c r="O2" s="2">
         <v>46251</v>
       </c>
       <c r="Q2">
@@ -791,16 +835,16 @@
         <v>40</v>
       </c>
       <c r="S2" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="T2" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="V2" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="W2" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -817,39 +861,39 @@
         <v>35</v>
       </c>
       <c r="D3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E3" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F3" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="G3">
         <v>2737</v>
       </c>
       <c r="H3" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="I3" t="s">
-        <v>76</v>
-      </c>
-      <c r="J3" s="1">
+        <v>82</v>
+      </c>
+      <c r="J3" s="2">
         <v>46205</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46234</v>
       </c>
       <c r="L3">
         <v>3</v>
       </c>
       <c r="M3" t="s">
-        <v>78</v>
-      </c>
-      <c r="N3" s="1">
+        <v>84</v>
+      </c>
+      <c r="N3" s="2">
         <v>46265</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46252</v>
       </c>
       <c r="Q3">
@@ -859,16 +903,16 @@
         <v>18</v>
       </c>
       <c r="S3" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="T3" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="V3" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="W3" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -885,39 +929,39 @@
         <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="F4" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="G4">
         <v>2733</v>
       </c>
       <c r="H4" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="I4" t="s">
-        <v>76</v>
-      </c>
-      <c r="J4" s="1">
+        <v>82</v>
+      </c>
+      <c r="J4" s="2">
         <v>46238</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46238</v>
       </c>
       <c r="L4">
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>78</v>
-      </c>
-      <c r="N4" s="1">
+        <v>84</v>
+      </c>
+      <c r="N4" s="2">
         <v>46269</v>
       </c>
-      <c r="O4" s="1">
+      <c r="O4" s="2">
         <v>46269</v>
       </c>
       <c r="Q4">
@@ -927,16 +971,16 @@
         <v>14</v>
       </c>
       <c r="S4" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="T4" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="V4" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="W4" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -953,39 +997,39 @@
         <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E5" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="F5" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="G5">
         <v>2729</v>
       </c>
       <c r="H5" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="I5" t="s">
-        <v>77</v>
-      </c>
-      <c r="J5" s="1">
+        <v>83</v>
+      </c>
+      <c r="J5" s="2">
         <v>46244</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46244</v>
       </c>
       <c r="L5">
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>78</v>
-      </c>
-      <c r="N5" s="1">
+        <v>84</v>
+      </c>
+      <c r="N5" s="2">
         <v>46255</v>
       </c>
-      <c r="O5" s="1">
+      <c r="O5" s="2">
         <v>46255</v>
       </c>
       <c r="Q5">
@@ -995,19 +1039,19 @@
         <v>8</v>
       </c>
       <c r="S5" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="T5" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="U5" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="V5" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="W5" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1024,39 +1068,39 @@
         <v>38</v>
       </c>
       <c r="D6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E6" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="G6">
         <v>2743</v>
       </c>
       <c r="H6" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="I6" t="s">
-        <v>76</v>
-      </c>
-      <c r="J6" s="1">
+        <v>82</v>
+      </c>
+      <c r="J6" s="2">
         <v>46244</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46246</v>
       </c>
       <c r="L6">
         <v>6</v>
       </c>
       <c r="M6" t="s">
-        <v>78</v>
-      </c>
-      <c r="N6" s="1">
+        <v>84</v>
+      </c>
+      <c r="N6" s="2">
         <v>46277</v>
       </c>
-      <c r="O6" s="1">
+      <c r="O6" s="2">
         <v>46254</v>
       </c>
       <c r="Q6">
@@ -1066,19 +1110,19 @@
         <v>6</v>
       </c>
       <c r="S6" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="T6" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="U6" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="V6" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="W6" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1095,39 +1139,39 @@
         <v>39</v>
       </c>
       <c r="D7" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E7" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="F7" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="G7">
         <v>2727</v>
       </c>
       <c r="H7" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="I7" t="s">
-        <v>77</v>
-      </c>
-      <c r="J7" s="1">
+        <v>83</v>
+      </c>
+      <c r="J7" s="2">
         <v>46245</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46246</v>
       </c>
       <c r="L7">
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>78</v>
-      </c>
-      <c r="N7" s="1">
+        <v>84</v>
+      </c>
+      <c r="N7" s="2">
         <v>46257</v>
       </c>
-      <c r="O7" s="1">
+      <c r="O7" s="2">
         <v>46251</v>
       </c>
       <c r="Q7">
@@ -1137,19 +1181,19 @@
         <v>6</v>
       </c>
       <c r="S7" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="T7" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="U7" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="V7" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="W7" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1166,39 +1210,39 @@
         <v>40</v>
       </c>
       <c r="D8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E8" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="F8" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="G8">
         <v>2742</v>
       </c>
       <c r="H8" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="I8" t="s">
-        <v>76</v>
-      </c>
-      <c r="J8" s="1">
+        <v>82</v>
+      </c>
+      <c r="J8" s="2">
         <v>46245</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46246</v>
       </c>
       <c r="L8">
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>78</v>
-      </c>
-      <c r="N8" s="1">
+        <v>84</v>
+      </c>
+      <c r="N8" s="2">
         <v>46277</v>
       </c>
-      <c r="O8" s="1">
+      <c r="O8" s="2">
         <v>46254</v>
       </c>
       <c r="Q8">
@@ -1208,19 +1252,19 @@
         <v>6</v>
       </c>
       <c r="S8" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="T8" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="U8" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="V8" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="W8" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1237,39 +1281,39 @@
         <v>41</v>
       </c>
       <c r="D9" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E9" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="F9" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="G9">
         <v>2742</v>
       </c>
       <c r="H9" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="I9" t="s">
-        <v>76</v>
-      </c>
-      <c r="J9" s="1">
+        <v>82</v>
+      </c>
+      <c r="J9" s="2">
         <v>46245</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46246</v>
       </c>
       <c r="L9">
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>78</v>
-      </c>
-      <c r="N9" s="1">
+        <v>84</v>
+      </c>
+      <c r="N9" s="2">
         <v>46277</v>
       </c>
-      <c r="O9" s="1">
+      <c r="O9" s="2">
         <v>46254</v>
       </c>
       <c r="Q9">
@@ -1279,19 +1323,19 @@
         <v>6</v>
       </c>
       <c r="S9" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="T9" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="U9" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="V9" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="W9" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1308,39 +1352,39 @@
         <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E10" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="F10" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="G10">
         <v>2742</v>
       </c>
       <c r="H10" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="I10" t="s">
-        <v>76</v>
-      </c>
-      <c r="J10" s="1">
+        <v>82</v>
+      </c>
+      <c r="J10" s="2">
         <v>46246</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>46247</v>
       </c>
       <c r="L10">
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>78</v>
-      </c>
-      <c r="N10" s="1">
+        <v>84</v>
+      </c>
+      <c r="N10" s="2">
         <v>46278</v>
       </c>
-      <c r="O10" s="1">
+      <c r="O10" s="2">
         <v>46249</v>
       </c>
       <c r="Q10">
@@ -1350,19 +1394,19 @@
         <v>5</v>
       </c>
       <c r="S10" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="T10" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="U10" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="V10" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="W10" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1379,36 +1423,36 @@
         <v>43</v>
       </c>
       <c r="D11" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E11" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="F11" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="G11">
         <v>2721</v>
       </c>
       <c r="H11" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="I11" t="s">
-        <v>76</v>
-      </c>
-      <c r="J11" s="1">
+        <v>82</v>
+      </c>
+      <c r="J11" s="2">
         <v>46248</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>46248</v>
       </c>
       <c r="L11">
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>78</v>
-      </c>
-      <c r="N11" s="1">
+        <v>84</v>
+      </c>
+      <c r="N11" s="2">
         <v>46279</v>
       </c>
       <c r="Q11">
@@ -1418,16 +1462,16 @@
         <v>4</v>
       </c>
       <c r="S11" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="T11" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="V11" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="W11" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1444,36 +1488,36 @@
         <v>44</v>
       </c>
       <c r="D12" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E12" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="F12" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="G12">
         <v>2720</v>
       </c>
       <c r="H12" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="I12" t="s">
-        <v>77</v>
-      </c>
-      <c r="J12" s="1">
+        <v>83</v>
+      </c>
+      <c r="J12" s="2">
         <v>46248</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>46248</v>
       </c>
       <c r="L12">
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>78</v>
-      </c>
-      <c r="N12" s="1">
+        <v>84</v>
+      </c>
+      <c r="N12" s="2">
         <v>46259</v>
       </c>
       <c r="Q12">
@@ -1483,19 +1527,19 @@
         <v>4</v>
       </c>
       <c r="S12" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="T12" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="U12" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="V12" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="W12" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1512,36 +1556,36 @@
         <v>45</v>
       </c>
       <c r="D13" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E13" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F13" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="G13">
         <v>2729</v>
       </c>
       <c r="H13" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="I13" t="s">
-        <v>77</v>
-      </c>
-      <c r="J13" s="1">
+        <v>83</v>
+      </c>
+      <c r="J13" s="2">
         <v>46248</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>46248</v>
       </c>
       <c r="L13">
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>78</v>
-      </c>
-      <c r="N13" s="1">
+        <v>84</v>
+      </c>
+      <c r="N13" s="2">
         <v>46259</v>
       </c>
       <c r="Q13">
@@ -1551,21 +1595,145 @@
         <v>4</v>
       </c>
       <c r="S13" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="T13" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="U13" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="V13" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="W13" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="AA13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:27">
+      <c r="A14">
+        <v>313</v>
+      </c>
+      <c r="B14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" t="s">
+        <v>60</v>
+      </c>
+      <c r="E14" t="s">
+        <v>74</v>
+      </c>
+      <c r="F14" t="s">
+        <v>76</v>
+      </c>
+      <c r="G14">
+        <v>2741</v>
+      </c>
+      <c r="H14" t="s">
+        <v>81</v>
+      </c>
+      <c r="I14" t="s">
+        <v>82</v>
+      </c>
+      <c r="J14" s="2">
+        <v>46251</v>
+      </c>
+      <c r="K14" s="2">
+        <v>46249</v>
+      </c>
+      <c r="L14">
+        <v>2</v>
+      </c>
+      <c r="M14" t="s">
+        <v>84</v>
+      </c>
+      <c r="N14" s="2">
+        <v>46280</v>
+      </c>
+      <c r="Q14">
+        <v>-28</v>
+      </c>
+      <c r="R14">
+        <v>3</v>
+      </c>
+      <c r="S14" t="s">
+        <v>85</v>
+      </c>
+      <c r="T14" t="s">
+        <v>86</v>
+      </c>
+      <c r="W14" t="s">
+        <v>106</v>
+      </c>
+      <c r="AA14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27">
+      <c r="A15">
+        <v>685</v>
+      </c>
+      <c r="B15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" t="s">
+        <v>47</v>
+      </c>
+      <c r="D15" t="s">
+        <v>61</v>
+      </c>
+      <c r="E15" t="s">
+        <v>75</v>
+      </c>
+      <c r="F15" t="s">
+        <v>78</v>
+      </c>
+      <c r="G15">
+        <v>2729</v>
+      </c>
+      <c r="H15" t="s">
+        <v>81</v>
+      </c>
+      <c r="I15" t="s">
+        <v>82</v>
+      </c>
+      <c r="J15" s="2">
+        <v>46251</v>
+      </c>
+      <c r="K15" s="2">
+        <v>46251</v>
+      </c>
+      <c r="L15">
+        <v>1</v>
+      </c>
+      <c r="M15" t="s">
+        <v>84</v>
+      </c>
+      <c r="N15" s="2">
+        <v>46282</v>
+      </c>
+      <c r="Q15">
+        <v>-30</v>
+      </c>
+      <c r="R15">
+        <v>1</v>
+      </c>
+      <c r="S15" t="s">
+        <v>85</v>
+      </c>
+      <c r="T15" t="s">
+        <v>86</v>
+      </c>
+      <c r="W15" t="s">
+        <v>106</v>
+      </c>
+      <c r="AA15" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (18/08/2026 12:39)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -344,16 +344,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -369,7 +361,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -377,30 +369,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -700,85 +674,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -810,10 +784,10 @@
       <c r="I2" t="s">
         <v>82</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>46212</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46212</v>
       </c>
       <c r="L2">
@@ -822,10 +796,10 @@
       <c r="M2" t="s">
         <v>84</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="1">
         <v>46243</v>
       </c>
-      <c r="O2" s="2">
+      <c r="O2" s="1">
         <v>46251</v>
       </c>
       <c r="Q2">
@@ -878,10 +852,10 @@
       <c r="I3" t="s">
         <v>82</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>46205</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46234</v>
       </c>
       <c r="L3">
@@ -890,10 +864,10 @@
       <c r="M3" t="s">
         <v>84</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="1">
         <v>46265</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46252</v>
       </c>
       <c r="Q3">
@@ -946,10 +920,10 @@
       <c r="I4" t="s">
         <v>82</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>46238</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46238</v>
       </c>
       <c r="L4">
@@ -958,10 +932,10 @@
       <c r="M4" t="s">
         <v>84</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="1">
         <v>46269</v>
       </c>
-      <c r="O4" s="2">
+      <c r="O4" s="1">
         <v>46269</v>
       </c>
       <c r="Q4">
@@ -1014,10 +988,10 @@
       <c r="I5" t="s">
         <v>83</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>46244</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46244</v>
       </c>
       <c r="L5">
@@ -1026,10 +1000,10 @@
       <c r="M5" t="s">
         <v>84</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="1">
         <v>46255</v>
       </c>
-      <c r="O5" s="2">
+      <c r="O5" s="1">
         <v>46255</v>
       </c>
       <c r="Q5">
@@ -1085,10 +1059,10 @@
       <c r="I6" t="s">
         <v>82</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>46244</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46246</v>
       </c>
       <c r="L6">
@@ -1097,10 +1071,10 @@
       <c r="M6" t="s">
         <v>84</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="1">
         <v>46277</v>
       </c>
-      <c r="O6" s="2">
+      <c r="O6" s="1">
         <v>46254</v>
       </c>
       <c r="Q6">
@@ -1156,10 +1130,10 @@
       <c r="I7" t="s">
         <v>83</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46245</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>46246</v>
       </c>
       <c r="L7">
@@ -1168,10 +1142,10 @@
       <c r="M7" t="s">
         <v>84</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="1">
         <v>46257</v>
       </c>
-      <c r="O7" s="2">
+      <c r="O7" s="1">
         <v>46251</v>
       </c>
       <c r="Q7">
@@ -1227,10 +1201,10 @@
       <c r="I8" t="s">
         <v>82</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46245</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>46246</v>
       </c>
       <c r="L8">
@@ -1239,10 +1213,10 @@
       <c r="M8" t="s">
         <v>84</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="1">
         <v>46277</v>
       </c>
-      <c r="O8" s="2">
+      <c r="O8" s="1">
         <v>46254</v>
       </c>
       <c r="Q8">
@@ -1298,10 +1272,10 @@
       <c r="I9" t="s">
         <v>82</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46245</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>46246</v>
       </c>
       <c r="L9">
@@ -1310,10 +1284,10 @@
       <c r="M9" t="s">
         <v>84</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="1">
         <v>46277</v>
       </c>
-      <c r="O9" s="2">
+      <c r="O9" s="1">
         <v>46254</v>
       </c>
       <c r="Q9">
@@ -1369,10 +1343,10 @@
       <c r="I10" t="s">
         <v>82</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>46246</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>46247</v>
       </c>
       <c r="L10">
@@ -1381,10 +1355,10 @@
       <c r="M10" t="s">
         <v>84</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="1">
         <v>46278</v>
       </c>
-      <c r="O10" s="2">
+      <c r="O10" s="1">
         <v>46249</v>
       </c>
       <c r="Q10">
@@ -1440,10 +1414,10 @@
       <c r="I11" t="s">
         <v>82</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46248</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>46248</v>
       </c>
       <c r="L11">
@@ -1452,7 +1426,7 @@
       <c r="M11" t="s">
         <v>84</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11" s="1">
         <v>46279</v>
       </c>
       <c r="Q11">
@@ -1505,10 +1479,10 @@
       <c r="I12" t="s">
         <v>83</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>46248</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>46248</v>
       </c>
       <c r="L12">
@@ -1517,7 +1491,7 @@
       <c r="M12" t="s">
         <v>84</v>
       </c>
-      <c r="N12" s="2">
+      <c r="N12" s="1">
         <v>46259</v>
       </c>
       <c r="Q12">
@@ -1573,10 +1547,10 @@
       <c r="I13" t="s">
         <v>83</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46248</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>46248</v>
       </c>
       <c r="L13">
@@ -1585,7 +1559,7 @@
       <c r="M13" t="s">
         <v>84</v>
       </c>
-      <c r="N13" s="2">
+      <c r="N13" s="1">
         <v>46259</v>
       </c>
       <c r="Q13">
@@ -1641,10 +1615,10 @@
       <c r="I14" t="s">
         <v>82</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46251</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>46249</v>
       </c>
       <c r="L14">
@@ -1653,7 +1627,7 @@
       <c r="M14" t="s">
         <v>84</v>
       </c>
-      <c r="N14" s="2">
+      <c r="N14" s="1">
         <v>46280</v>
       </c>
       <c r="Q14">
@@ -1703,10 +1677,10 @@
       <c r="I15" t="s">
         <v>82</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46251</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46251</v>
       </c>
       <c r="L15">
@@ -1715,7 +1689,7 @@
       <c r="M15" t="s">
         <v>84</v>
       </c>
-      <c r="N15" s="2">
+      <c r="N15" s="1">
         <v>46282</v>
       </c>
       <c r="Q15">

</xml_diff>

<commit_message>
Atualização automática: emergencias (18/08/2026 14:35)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="94">
   <si>
     <t>om_emg</t>
   </si>
@@ -100,30 +100,27 @@
     <t>BANT</t>
   </si>
   <si>
+    <t>BABE</t>
+  </si>
+  <si>
+    <t>BACO</t>
+  </si>
+  <si>
+    <t>BACG</t>
+  </si>
+  <si>
+    <t>DACTA II</t>
+  </si>
+  <si>
+    <t>BABR</t>
+  </si>
+  <si>
     <t>BAMN</t>
   </si>
   <si>
-    <t>BABE</t>
-  </si>
-  <si>
-    <t>BACO</t>
-  </si>
-  <si>
-    <t>BACG</t>
-  </si>
-  <si>
-    <t>DACTA II</t>
-  </si>
-  <si>
-    <t>BABR</t>
-  </si>
-  <si>
     <t>685260012350</t>
   </si>
   <si>
-    <t>313260018658</t>
-  </si>
-  <si>
     <t>396260016580</t>
   </si>
   <si>
@@ -136,15 +133,9 @@
     <t>690260002522</t>
   </si>
   <si>
-    <t>384260009395</t>
-  </si>
-  <si>
     <t>384260009396</t>
   </si>
   <si>
-    <t>384260009397</t>
-  </si>
-  <si>
     <t>329260019269</t>
   </si>
   <si>
@@ -163,9 +154,6 @@
     <t>030-1094-58</t>
   </si>
   <si>
-    <t>324843-W020</t>
-  </si>
-  <si>
     <t>2601188-204</t>
   </si>
   <si>
@@ -178,15 +166,9 @@
     <t>3244897-4</t>
   </si>
   <si>
-    <t>2618510-10</t>
-  </si>
-  <si>
     <t>S2616-285K4</t>
   </si>
   <si>
-    <t>C611505-0201</t>
-  </si>
-  <si>
     <t>069-01033-0101</t>
   </si>
   <si>
@@ -205,9 +187,6 @@
     <t>CONNECTOR</t>
   </si>
   <si>
-    <t>HEADSET-MICROPHONE</t>
-  </si>
-  <si>
     <t>COMPRESSOR DRIVE ASS</t>
   </si>
   <si>
@@ -220,15 +199,9 @@
     <t>FUEL CONTROL UNIT</t>
   </si>
   <si>
-    <t>ALTERNATOR CONTROL U</t>
-  </si>
-  <si>
     <t>ALTERNAD BELT</t>
   </si>
   <si>
-    <t>ALTERNATOR</t>
-  </si>
-  <si>
     <t>RECEIVER-TRANSMITTER</t>
   </si>
   <si>
@@ -286,9 +259,6 @@
     <t>RECIBO não se encontra na pasta do drive. Godoy 18/08/26.</t>
   </si>
   <si>
-    <t>Item em pane, anv autorizada a voar por 3 dias pela MMEL a contar de 12/08. Ramon 13/08/26. AWB 12752990604 - volume retirado na loja GOLLOG - CWB por RAFAEL MAIA DE LIMA em 15/08. Godoy 18/08/26.</t>
-  </si>
-  <si>
     <t>Estoque no alternado 285K4. Caso use do estoque, verificar validade que consta no item. Ramon 12/08/26. Item em pane, anv autorizada a voar por 3 dias pela MMEL a contar de 12/08. Ramon 13/08/26</t>
   </si>
   <si>
@@ -301,9 +271,6 @@
     <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Chegada GIG dia 15-08 (voo 4273). Canal verde dia 17/08. Aguardando SEFAZ.</t>
   </si>
   <si>
-    <t>Temos 4 EA em manutenção na William, será pedido prioridade. CLA-03-08 - DPE DIA 14-08 - CLA 13-08 - AWB 127-5299 2505 DPE 18/08/2026</t>
-  </si>
-  <si>
     <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
   </si>
   <si>
@@ -316,13 +283,7 @@
     <t>Previsao de entrega da oficina do RJ na V1 JPA 13/8/2026 durante o dia, horario comercial, ATZ Marcio 12/8 13:22hs - Material entregue dia 17/08/2026 - Retirado pelo TEN Goncalves</t>
   </si>
   <si>
-    <t>1 Unidade na oficina em BH William, solicitado prioridade na entrega DPE 14/8, aguardando orçamento final ATZ Marcio 12/8 13:24hs- DPE 14-08 - AWB 127-5299 0604 DPE 15-08-26 CLA-17-08</t>
-  </si>
-  <si>
     <t>Temos no STK V1, material em separação, recibo 682/FAB/26 - atz rc 13/08 - MATERIAL ENVIADO VIA AWB 12752709016 - DPE 18/08/2026</t>
-  </si>
-  <si>
-    <t>será enviado o pn 9910592-2 do estoque da VeeOne base PAMALS. -CLA -14-08- AWB 127-5299 0604 DPE 15-08-26 CLA-17-08</t>
   </si>
   <si>
     <t>foi solicitoado o atendimento com o estoque FAB. CLA-17-08 - o item PN superado 069-1025-25 não serve na ANV 2721 - temos 4ea na wiliam para reparo, já foi solicitado o DPE.</t>
@@ -670,7 +631,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA15"/>
+  <dimension ref="A1:AA12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -767,22 +728,22 @@
         <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E2" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="F2" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="G2">
         <v>2702</v>
       </c>
       <c r="H2" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="I2" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="J2" s="1">
         <v>46212</v>
@@ -794,7 +755,7 @@
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="N2" s="1">
         <v>46243</v>
@@ -809,16 +770,16 @@
         <v>40</v>
       </c>
       <c r="S2" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="T2" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="V2" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="W2" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -826,7 +787,7 @@
     </row>
     <row r="3" spans="1:27">
       <c r="A3">
-        <v>313</v>
+        <v>396</v>
       </c>
       <c r="B3" t="s">
         <v>28</v>
@@ -835,58 +796,58 @@
         <v>35</v>
       </c>
       <c r="D3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E3" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="F3" t="s">
+        <v>67</v>
+      </c>
+      <c r="G3">
+        <v>2733</v>
+      </c>
+      <c r="H3" t="s">
+        <v>70</v>
+      </c>
+      <c r="I3" t="s">
+        <v>73</v>
+      </c>
+      <c r="J3" s="1">
+        <v>46238</v>
+      </c>
+      <c r="K3" s="1">
+        <v>46238</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3" t="s">
+        <v>75</v>
+      </c>
+      <c r="N3" s="1">
+        <v>46269</v>
+      </c>
+      <c r="O3" s="1">
+        <v>46269</v>
+      </c>
+      <c r="Q3">
+        <v>-17</v>
+      </c>
+      <c r="R3">
+        <v>14</v>
+      </c>
+      <c r="S3" t="s">
+        <v>76</v>
+      </c>
+      <c r="T3" t="s">
         <v>77</v>
       </c>
-      <c r="G3">
-        <v>2737</v>
-      </c>
-      <c r="H3" t="s">
-        <v>79</v>
-      </c>
-      <c r="I3" t="s">
-        <v>82</v>
-      </c>
-      <c r="J3" s="1">
-        <v>46205</v>
-      </c>
-      <c r="K3" s="1">
-        <v>46234</v>
-      </c>
-      <c r="L3">
-        <v>3</v>
-      </c>
-      <c r="M3" t="s">
-        <v>84</v>
-      </c>
-      <c r="N3" s="1">
-        <v>46265</v>
-      </c>
-      <c r="O3" s="1">
-        <v>46252</v>
-      </c>
-      <c r="Q3">
-        <v>-13</v>
-      </c>
-      <c r="R3">
-        <v>18</v>
-      </c>
-      <c r="S3" t="s">
+      <c r="V3" t="s">
         <v>85</v>
       </c>
-      <c r="T3" t="s">
-        <v>86</v>
-      </c>
-      <c r="V3" t="s">
-        <v>95</v>
-      </c>
       <c r="W3" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -894,67 +855,70 @@
     </row>
     <row r="4" spans="1:27">
       <c r="A4">
-        <v>396</v>
+        <v>685</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C4" t="s">
         <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E4" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="F4" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="G4">
-        <v>2733</v>
+        <v>2729</v>
       </c>
       <c r="H4" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="I4" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="J4" s="1">
-        <v>46238</v>
+        <v>46244</v>
       </c>
       <c r="K4" s="1">
-        <v>46238</v>
+        <v>46244</v>
       </c>
       <c r="L4">
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="N4" s="1">
-        <v>46269</v>
+        <v>46255</v>
       </c>
       <c r="O4" s="1">
-        <v>46269</v>
+        <v>46255</v>
       </c>
       <c r="Q4">
-        <v>-17</v>
+        <v>-3</v>
       </c>
       <c r="R4">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="S4" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="T4" t="s">
+        <v>77</v>
+      </c>
+      <c r="U4" t="s">
+        <v>78</v>
+      </c>
+      <c r="V4" t="s">
         <v>86</v>
       </c>
-      <c r="V4" t="s">
-        <v>96</v>
-      </c>
       <c r="W4" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -962,70 +926,70 @@
     </row>
     <row r="5" spans="1:27">
       <c r="A5">
-        <v>685</v>
+        <v>386</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C5" t="s">
         <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E5" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="F5" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="G5">
-        <v>2729</v>
+        <v>2743</v>
       </c>
       <c r="H5" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="I5" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="J5" s="1">
         <v>46244</v>
       </c>
       <c r="K5" s="1">
-        <v>46244</v>
+        <v>46246</v>
       </c>
       <c r="L5">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="M5" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="N5" s="1">
-        <v>46255</v>
+        <v>46277</v>
       </c>
       <c r="O5" s="1">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="Q5">
-        <v>-3</v>
+        <v>-25</v>
       </c>
       <c r="R5">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="S5" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="T5" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="U5" t="s">
+        <v>79</v>
+      </c>
+      <c r="V5" t="s">
         <v>87</v>
       </c>
-      <c r="V5" t="s">
-        <v>97</v>
-      </c>
       <c r="W5" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1033,7 +997,7 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6">
-        <v>386</v>
+        <v>690</v>
       </c>
       <c r="B6" t="s">
         <v>30</v>
@@ -1042,61 +1006,61 @@
         <v>38</v>
       </c>
       <c r="D6" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E6" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="F6" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="G6">
-        <v>2743</v>
+        <v>2727</v>
       </c>
       <c r="H6" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="I6" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="J6" s="1">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="K6" s="1">
         <v>46246</v>
       </c>
       <c r="L6">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="N6" s="1">
-        <v>46277</v>
+        <v>46257</v>
       </c>
       <c r="O6" s="1">
-        <v>46254</v>
+        <v>46251</v>
       </c>
       <c r="Q6">
-        <v>-25</v>
+        <v>-5</v>
       </c>
       <c r="R6">
         <v>6</v>
       </c>
       <c r="S6" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="T6" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="U6" t="s">
+        <v>80</v>
+      </c>
+      <c r="V6" t="s">
         <v>88</v>
       </c>
-      <c r="V6" t="s">
-        <v>98</v>
-      </c>
       <c r="W6" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1104,7 +1068,7 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>690</v>
+        <v>384</v>
       </c>
       <c r="B7" t="s">
         <v>31</v>
@@ -1113,22 +1077,22 @@
         <v>39</v>
       </c>
       <c r="D7" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E7" t="s">
+        <v>61</v>
+      </c>
+      <c r="F7" t="s">
         <v>67</v>
       </c>
-      <c r="F7" t="s">
-        <v>78</v>
-      </c>
       <c r="G7">
-        <v>2727</v>
+        <v>2742</v>
       </c>
       <c r="H7" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="I7" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="J7" s="1">
         <v>46245</v>
@@ -1140,34 +1104,34 @@
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="N7" s="1">
-        <v>46257</v>
+        <v>46277</v>
       </c>
       <c r="O7" s="1">
-        <v>46251</v>
+        <v>46254</v>
       </c>
       <c r="Q7">
-        <v>-5</v>
+        <v>-25</v>
       </c>
       <c r="R7">
         <v>6</v>
       </c>
       <c r="S7" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="T7" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="U7" t="s">
+        <v>81</v>
+      </c>
+      <c r="V7" t="s">
         <v>89</v>
       </c>
-      <c r="V7" t="s">
-        <v>99</v>
-      </c>
       <c r="W7" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1175,7 +1139,7 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>384</v>
+        <v>329</v>
       </c>
       <c r="B8" t="s">
         <v>32</v>
@@ -1184,61 +1148,55 @@
         <v>40</v>
       </c>
       <c r="D8" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E8" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="F8" t="s">
+        <v>69</v>
+      </c>
+      <c r="G8">
+        <v>2721</v>
+      </c>
+      <c r="H8" t="s">
+        <v>72</v>
+      </c>
+      <c r="I8" t="s">
+        <v>73</v>
+      </c>
+      <c r="J8" s="1">
+        <v>46248</v>
+      </c>
+      <c r="K8" s="1">
+        <v>46248</v>
+      </c>
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8" t="s">
+        <v>75</v>
+      </c>
+      <c r="N8" s="1">
+        <v>46279</v>
+      </c>
+      <c r="Q8">
+        <v>-27</v>
+      </c>
+      <c r="R8">
+        <v>4</v>
+      </c>
+      <c r="S8" t="s">
         <v>77</v>
       </c>
-      <c r="G8">
-        <v>2742</v>
-      </c>
-      <c r="H8" t="s">
-        <v>79</v>
-      </c>
-      <c r="I8" t="s">
-        <v>82</v>
-      </c>
-      <c r="J8" s="1">
-        <v>46245</v>
-      </c>
-      <c r="K8" s="1">
-        <v>46246</v>
-      </c>
-      <c r="L8">
-        <v>1</v>
-      </c>
-      <c r="M8" t="s">
-        <v>84</v>
-      </c>
-      <c r="N8" s="1">
-        <v>46277</v>
-      </c>
-      <c r="O8" s="1">
-        <v>46254</v>
-      </c>
-      <c r="Q8">
-        <v>-25</v>
-      </c>
-      <c r="R8">
-        <v>6</v>
-      </c>
-      <c r="S8" t="s">
-        <v>85</v>
-      </c>
       <c r="T8" t="s">
-        <v>85</v>
-      </c>
-      <c r="U8" t="s">
+        <v>76</v>
+      </c>
+      <c r="V8" t="s">
         <v>90</v>
       </c>
-      <c r="V8" t="s">
-        <v>100</v>
-      </c>
       <c r="W8" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1246,7 +1204,7 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9">
-        <v>384</v>
+        <v>329</v>
       </c>
       <c r="B9" t="s">
         <v>32</v>
@@ -1255,61 +1213,58 @@
         <v>41</v>
       </c>
       <c r="D9" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E9" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="F9" t="s">
+        <v>68</v>
+      </c>
+      <c r="G9">
+        <v>2720</v>
+      </c>
+      <c r="H9" t="s">
+        <v>71</v>
+      </c>
+      <c r="I9" t="s">
+        <v>74</v>
+      </c>
+      <c r="J9" s="1">
+        <v>46248</v>
+      </c>
+      <c r="K9" s="1">
+        <v>46248</v>
+      </c>
+      <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9" t="s">
+        <v>75</v>
+      </c>
+      <c r="N9" s="1">
+        <v>46259</v>
+      </c>
+      <c r="Q9">
+        <v>-7</v>
+      </c>
+      <c r="R9">
+        <v>4</v>
+      </c>
+      <c r="S9" t="s">
+        <v>77</v>
+      </c>
+      <c r="T9" t="s">
         <v>76</v>
       </c>
-      <c r="G9">
-        <v>2742</v>
-      </c>
-      <c r="H9" t="s">
-        <v>79</v>
-      </c>
-      <c r="I9" t="s">
+      <c r="U9" t="s">
         <v>82</v>
       </c>
-      <c r="J9" s="1">
-        <v>46245</v>
-      </c>
-      <c r="K9" s="1">
-        <v>46246</v>
-      </c>
-      <c r="L9">
-        <v>1</v>
-      </c>
-      <c r="M9" t="s">
-        <v>84</v>
-      </c>
-      <c r="N9" s="1">
-        <v>46277</v>
-      </c>
-      <c r="O9" s="1">
-        <v>46254</v>
-      </c>
-      <c r="Q9">
-        <v>-25</v>
-      </c>
-      <c r="R9">
-        <v>6</v>
-      </c>
-      <c r="S9" t="s">
-        <v>86</v>
-      </c>
-      <c r="T9" t="s">
-        <v>85</v>
-      </c>
-      <c r="U9" t="s">
+      <c r="V9" t="s">
         <v>91</v>
       </c>
-      <c r="V9" t="s">
-        <v>101</v>
-      </c>
       <c r="W9" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1317,70 +1272,67 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>384</v>
+        <v>685</v>
       </c>
       <c r="B10" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C10" t="s">
         <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E10" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="F10" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G10">
-        <v>2742</v>
+        <v>2729</v>
       </c>
       <c r="H10" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="I10" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="J10" s="1">
-        <v>46246</v>
+        <v>46248</v>
       </c>
       <c r="K10" s="1">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="L10">
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="N10" s="1">
-        <v>46278</v>
-      </c>
-      <c r="O10" s="1">
-        <v>46249</v>
+        <v>46259</v>
       </c>
       <c r="Q10">
-        <v>-26</v>
+        <v>-7</v>
       </c>
       <c r="R10">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S10" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="T10" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="U10" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="V10" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="W10" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1388,7 +1340,7 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>329</v>
+        <v>313</v>
       </c>
       <c r="B11" t="s">
         <v>33</v>
@@ -1397,55 +1349,52 @@
         <v>43</v>
       </c>
       <c r="D11" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E11" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="F11" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="G11">
-        <v>2721</v>
+        <v>2741</v>
       </c>
       <c r="H11" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="I11" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="J11" s="1">
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="K11" s="1">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="L11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M11" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="N11" s="1">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="Q11">
-        <v>-27</v>
+        <v>-28</v>
       </c>
       <c r="R11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S11" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="T11" t="s">
-        <v>85</v>
-      </c>
-      <c r="V11" t="s">
-        <v>103</v>
+        <v>77</v>
       </c>
       <c r="W11" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1453,261 +1402,63 @@
     </row>
     <row r="12" spans="1:27">
       <c r="A12">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B12" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C12" t="s">
         <v>44</v>
       </c>
       <c r="D12" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E12" t="s">
+        <v>66</v>
+      </c>
+      <c r="F12" t="s">
+        <v>69</v>
+      </c>
+      <c r="G12">
+        <v>2729</v>
+      </c>
+      <c r="H12" t="s">
         <v>72</v>
       </c>
-      <c r="F12" t="s">
+      <c r="I12" t="s">
+        <v>73</v>
+      </c>
+      <c r="J12" s="1">
+        <v>46251</v>
+      </c>
+      <c r="K12" s="1">
+        <v>46251</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12" t="s">
+        <v>75</v>
+      </c>
+      <c r="N12" s="1">
+        <v>46282</v>
+      </c>
+      <c r="Q12">
+        <v>-30</v>
+      </c>
+      <c r="R12">
+        <v>1</v>
+      </c>
+      <c r="S12" t="s">
+        <v>76</v>
+      </c>
+      <c r="T12" t="s">
         <v>77</v>
       </c>
-      <c r="G12">
-        <v>2720</v>
-      </c>
-      <c r="H12" t="s">
-        <v>80</v>
-      </c>
-      <c r="I12" t="s">
-        <v>83</v>
-      </c>
-      <c r="J12" s="1">
-        <v>46248</v>
-      </c>
-      <c r="K12" s="1">
-        <v>46248</v>
-      </c>
-      <c r="L12">
-        <v>1</v>
-      </c>
-      <c r="M12" t="s">
-        <v>84</v>
-      </c>
-      <c r="N12" s="1">
-        <v>46259</v>
-      </c>
-      <c r="Q12">
-        <v>-7</v>
-      </c>
-      <c r="R12">
-        <v>4</v>
-      </c>
-      <c r="S12" t="s">
-        <v>86</v>
-      </c>
-      <c r="T12" t="s">
-        <v>85</v>
-      </c>
-      <c r="U12" t="s">
-        <v>92</v>
-      </c>
-      <c r="V12" t="s">
-        <v>104</v>
-      </c>
       <c r="W12" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="AA12" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:27">
-      <c r="A13">
-        <v>685</v>
-      </c>
-      <c r="B13" t="s">
-        <v>27</v>
-      </c>
-      <c r="C13" t="s">
-        <v>45</v>
-      </c>
-      <c r="D13" t="s">
-        <v>59</v>
-      </c>
-      <c r="E13" t="s">
-        <v>73</v>
-      </c>
-      <c r="F13" t="s">
-        <v>77</v>
-      </c>
-      <c r="G13">
-        <v>2729</v>
-      </c>
-      <c r="H13" t="s">
-        <v>81</v>
-      </c>
-      <c r="I13" t="s">
-        <v>83</v>
-      </c>
-      <c r="J13" s="1">
-        <v>46248</v>
-      </c>
-      <c r="K13" s="1">
-        <v>46248</v>
-      </c>
-      <c r="L13">
-        <v>1</v>
-      </c>
-      <c r="M13" t="s">
-        <v>84</v>
-      </c>
-      <c r="N13" s="1">
-        <v>46259</v>
-      </c>
-      <c r="Q13">
-        <v>-7</v>
-      </c>
-      <c r="R13">
-        <v>4</v>
-      </c>
-      <c r="S13" t="s">
-        <v>86</v>
-      </c>
-      <c r="T13" t="s">
-        <v>86</v>
-      </c>
-      <c r="U13" t="s">
-        <v>93</v>
-      </c>
-      <c r="V13" t="s">
-        <v>105</v>
-      </c>
-      <c r="W13" t="s">
-        <v>106</v>
-      </c>
-      <c r="AA13" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:27">
-      <c r="A14">
-        <v>313</v>
-      </c>
-      <c r="B14" t="s">
-        <v>28</v>
-      </c>
-      <c r="C14" t="s">
-        <v>46</v>
-      </c>
-      <c r="D14" t="s">
-        <v>60</v>
-      </c>
-      <c r="E14" t="s">
-        <v>74</v>
-      </c>
-      <c r="F14" t="s">
-        <v>76</v>
-      </c>
-      <c r="G14">
-        <v>2741</v>
-      </c>
-      <c r="H14" t="s">
-        <v>81</v>
-      </c>
-      <c r="I14" t="s">
-        <v>82</v>
-      </c>
-      <c r="J14" s="1">
-        <v>46251</v>
-      </c>
-      <c r="K14" s="1">
-        <v>46249</v>
-      </c>
-      <c r="L14">
-        <v>2</v>
-      </c>
-      <c r="M14" t="s">
-        <v>84</v>
-      </c>
-      <c r="N14" s="1">
-        <v>46280</v>
-      </c>
-      <c r="Q14">
-        <v>-28</v>
-      </c>
-      <c r="R14">
-        <v>3</v>
-      </c>
-      <c r="S14" t="s">
-        <v>85</v>
-      </c>
-      <c r="T14" t="s">
-        <v>86</v>
-      </c>
-      <c r="W14" t="s">
-        <v>106</v>
-      </c>
-      <c r="AA14" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:27">
-      <c r="A15">
-        <v>685</v>
-      </c>
-      <c r="B15" t="s">
-        <v>27</v>
-      </c>
-      <c r="C15" t="s">
-        <v>47</v>
-      </c>
-      <c r="D15" t="s">
-        <v>61</v>
-      </c>
-      <c r="E15" t="s">
-        <v>75</v>
-      </c>
-      <c r="F15" t="s">
-        <v>78</v>
-      </c>
-      <c r="G15">
-        <v>2729</v>
-      </c>
-      <c r="H15" t="s">
-        <v>81</v>
-      </c>
-      <c r="I15" t="s">
-        <v>82</v>
-      </c>
-      <c r="J15" s="1">
-        <v>46251</v>
-      </c>
-      <c r="K15" s="1">
-        <v>46251</v>
-      </c>
-      <c r="L15">
-        <v>1</v>
-      </c>
-      <c r="M15" t="s">
-        <v>84</v>
-      </c>
-      <c r="N15" s="1">
-        <v>46282</v>
-      </c>
-      <c r="Q15">
-        <v>-30</v>
-      </c>
-      <c r="R15">
-        <v>1</v>
-      </c>
-      <c r="S15" t="s">
-        <v>85</v>
-      </c>
-      <c r="T15" t="s">
-        <v>86</v>
-      </c>
-      <c r="W15" t="s">
-        <v>106</v>
-      </c>
-      <c r="AA15" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (19/08/2026 08:33)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -764,10 +764,10 @@
         <v>46251</v>
       </c>
       <c r="Q2">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R2">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="S2" t="s">
         <v>76</v>
@@ -832,10 +832,10 @@
         <v>46269</v>
       </c>
       <c r="Q3">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="R3">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S3" t="s">
         <v>76</v>
@@ -900,10 +900,10 @@
         <v>46255</v>
       </c>
       <c r="Q4">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R4">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S4" t="s">
         <v>77</v>
@@ -971,10 +971,10 @@
         <v>46254</v>
       </c>
       <c r="Q5">
-        <v>-25</v>
+        <v>-24</v>
       </c>
       <c r="R5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S5" t="s">
         <v>77</v>
@@ -1042,10 +1042,10 @@
         <v>46251</v>
       </c>
       <c r="Q6">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R6">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S6" t="s">
         <v>76</v>
@@ -1113,10 +1113,10 @@
         <v>46254</v>
       </c>
       <c r="Q7">
-        <v>-25</v>
+        <v>-24</v>
       </c>
       <c r="R7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S7" t="s">
         <v>77</v>
@@ -1181,10 +1181,10 @@
         <v>46279</v>
       </c>
       <c r="Q8">
-        <v>-27</v>
+        <v>-26</v>
       </c>
       <c r="R8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S8" t="s">
         <v>77</v>
@@ -1246,10 +1246,10 @@
         <v>46259</v>
       </c>
       <c r="Q9">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S9" t="s">
         <v>77</v>
@@ -1314,10 +1314,10 @@
         <v>46259</v>
       </c>
       <c r="Q10">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S10" t="s">
         <v>77</v>
@@ -1382,10 +1382,10 @@
         <v>46280</v>
       </c>
       <c r="Q11">
-        <v>-28</v>
+        <v>-27</v>
       </c>
       <c r="R11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S11" t="s">
         <v>76</v>
@@ -1444,10 +1444,10 @@
         <v>46282</v>
       </c>
       <c r="Q12">
-        <v>-30</v>
+        <v>-29</v>
       </c>
       <c r="R12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S12" t="s">
         <v>76</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (19/08/2026 13:06)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -305,8 +305,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -322,7 +330,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -330,12 +338,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -635,85 +661,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -745,10 +771,10 @@
       <c r="I2" t="s">
         <v>73</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>46212</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46212</v>
       </c>
       <c r="L2">
@@ -757,10 +783,10 @@
       <c r="M2" t="s">
         <v>75</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <v>46243</v>
       </c>
-      <c r="O2" s="1">
+      <c r="O2" s="2">
         <v>46251</v>
       </c>
       <c r="Q2">
@@ -813,10 +839,10 @@
       <c r="I3" t="s">
         <v>73</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>46238</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46238</v>
       </c>
       <c r="L3">
@@ -825,10 +851,10 @@
       <c r="M3" t="s">
         <v>75</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <v>46269</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46269</v>
       </c>
       <c r="Q3">
@@ -881,10 +907,10 @@
       <c r="I4" t="s">
         <v>74</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>46244</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46244</v>
       </c>
       <c r="L4">
@@ -893,10 +919,10 @@
       <c r="M4" t="s">
         <v>75</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="2">
         <v>46255</v>
       </c>
-      <c r="O4" s="1">
+      <c r="O4" s="2">
         <v>46255</v>
       </c>
       <c r="Q4">
@@ -952,10 +978,10 @@
       <c r="I5" t="s">
         <v>73</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>46244</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46246</v>
       </c>
       <c r="L5">
@@ -964,10 +990,10 @@
       <c r="M5" t="s">
         <v>75</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <v>46277</v>
       </c>
-      <c r="O5" s="1">
+      <c r="O5" s="2">
         <v>46254</v>
       </c>
       <c r="Q5">
@@ -1023,10 +1049,10 @@
       <c r="I6" t="s">
         <v>74</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>46245</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46246</v>
       </c>
       <c r="L6">
@@ -1035,10 +1061,10 @@
       <c r="M6" t="s">
         <v>75</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <v>46257</v>
       </c>
-      <c r="O6" s="1">
+      <c r="O6" s="2">
         <v>46251</v>
       </c>
       <c r="Q6">
@@ -1094,10 +1120,10 @@
       <c r="I7" t="s">
         <v>73</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46245</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46246</v>
       </c>
       <c r="L7">
@@ -1106,10 +1132,10 @@
       <c r="M7" t="s">
         <v>75</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="2">
         <v>46277</v>
       </c>
-      <c r="O7" s="1">
+      <c r="O7" s="2">
         <v>46254</v>
       </c>
       <c r="Q7">
@@ -1165,10 +1191,10 @@
       <c r="I8" t="s">
         <v>73</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46248</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46248</v>
       </c>
       <c r="L8">
@@ -1177,7 +1203,7 @@
       <c r="M8" t="s">
         <v>75</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="2">
         <v>46279</v>
       </c>
       <c r="Q8">
@@ -1230,10 +1256,10 @@
       <c r="I9" t="s">
         <v>74</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46248</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46248</v>
       </c>
       <c r="L9">
@@ -1242,7 +1268,7 @@
       <c r="M9" t="s">
         <v>75</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>46259</v>
       </c>
       <c r="Q9">
@@ -1298,10 +1324,10 @@
       <c r="I10" t="s">
         <v>74</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46248</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>46248</v>
       </c>
       <c r="L10">
@@ -1310,7 +1336,7 @@
       <c r="M10" t="s">
         <v>75</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
         <v>46259</v>
       </c>
       <c r="Q10">
@@ -1366,10 +1392,10 @@
       <c r="I11" t="s">
         <v>73</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46251</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>46249</v>
       </c>
       <c r="L11">
@@ -1378,7 +1404,7 @@
       <c r="M11" t="s">
         <v>75</v>
       </c>
-      <c r="N11" s="1">
+      <c r="N11" s="2">
         <v>46280</v>
       </c>
       <c r="Q11">
@@ -1428,10 +1454,10 @@
       <c r="I12" t="s">
         <v>73</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>46251</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>46251</v>
       </c>
       <c r="L12">
@@ -1440,7 +1466,7 @@
       <c r="M12" t="s">
         <v>75</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="2">
         <v>46282</v>
       </c>
       <c r="Q12">

</xml_diff>

<commit_message>
Atualização automática: emergencias (19/08/2026 14:34)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="90">
   <si>
     <t>om_emg</t>
   </si>
@@ -106,9 +106,6 @@
     <t>BACO</t>
   </si>
   <si>
-    <t>BACG</t>
-  </si>
-  <si>
     <t>DACTA II</t>
   </si>
   <si>
@@ -130,9 +127,6 @@
     <t>386260013489</t>
   </si>
   <si>
-    <t>690260002522</t>
-  </si>
-  <si>
     <t>384260009396</t>
   </si>
   <si>
@@ -163,9 +157,6 @@
     <t>9910333-1</t>
   </si>
   <si>
-    <t>3244897-4</t>
-  </si>
-  <si>
     <t>S2616-285K4</t>
   </si>
   <si>
@@ -196,9 +187,6 @@
     <t>ENGINE MOUNT</t>
   </si>
   <si>
-    <t>FUEL CONTROL UNIT</t>
-  </si>
-  <si>
     <t>ALTERNAD BELT</t>
   </si>
   <si>
@@ -256,9 +244,6 @@
     <t>Estoque com 12 EA do Pn LM600-9 (Alternado). Godoy 12/08/26. Atendido com estoque local em 13/08. Ramon 13/08/26</t>
   </si>
   <si>
-    <t>RECIBO não se encontra na pasta do drive. Godoy 18/08/26.</t>
-  </si>
-  <si>
     <t>Estoque no alternado 285K4. Caso use do estoque, verificar validade que consta no item. Ramon 12/08/26. Item em pane, anv autorizada a voar por 3 dias pela MMEL a contar de 12/08. Ramon 13/08/26</t>
   </si>
   <si>
@@ -268,7 +253,7 @@
     <t>Estoque alterado de "Nao" para "SIM"  daremos prioridade para movimentar o item.  Godoy 17/08/226</t>
   </si>
   <si>
-    <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Chegada GIG dia 15-08 (voo 4273). Canal verde dia 17/08. Aguardando SEFAZ.</t>
+    <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Chegada GIG dia 15-08 (voo 4273). Entregue V1 JPA 17/08</t>
   </si>
   <si>
     <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
@@ -280,19 +265,22 @@
     <t>Temos somente 03 ea em STK, favor utilizar o estoque FAB para posterior devolução. ATZ RC 13/08 - FOI SOLICITADO O ATENDIMENTO COM ESTOQUE FAB -CLA-13-08 - AWB 127-5299 0173 DPE 18/08/2026</t>
   </si>
   <si>
-    <t>Previsao de entrega da oficina do RJ na V1 JPA 13/8/2026 durante o dia, horario comercial, ATZ Marcio 12/8 13:22hs - Material entregue dia 17/08/2026 - Retirado pelo TEN Goncalves</t>
-  </si>
-  <si>
     <t>Temos no STK V1, material em separação, recibo 682/FAB/26 - atz rc 13/08 - MATERIAL ENVIADO VIA AWB 12752709016 - DPE 18/08/2026</t>
   </si>
   <si>
     <t>foi solicitoado o atendimento com o estoque FAB. CLA-17-08 - o item PN superado 069-1025-25 não serve na ANV 2721 - temos 4ea na wiliam para reparo, já foi solicitado o DPE.</t>
   </si>
   <si>
-    <t>foi solicitoado o atendimento com o estoque FAB. CLA-17-08</t>
+    <t>Enviado para o Operador dia 17/08/26, AWB 127-5332-5834 - REZ</t>
   </si>
   <si>
     <t>ITEM FOI ENTREGUE PARA A FAB VIA RECIBO 598/FAB/26 31-07-26 - AINDA NÃO FOI PARA O ESTOQUECLA-17-08</t>
+  </si>
+  <si>
+    <t>pedido no EPM E-C98-26061 -CLA-18-08</t>
+  </si>
+  <si>
+    <t>DPE DA WILLIAM DIA 20-08-2026 -CLA-18-08</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -305,16 +293,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -330,7 +310,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -338,30 +318,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -657,89 +619,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA12"/>
+  <dimension ref="A1:AA11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -751,42 +713,42 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G2">
         <v>2702</v>
       </c>
       <c r="H2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="I2" t="s">
-        <v>73</v>
-      </c>
-      <c r="J2" s="2">
+        <v>69</v>
+      </c>
+      <c r="J2" s="1">
         <v>46212</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46212</v>
       </c>
       <c r="L2">
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>75</v>
-      </c>
-      <c r="N2" s="2">
+        <v>71</v>
+      </c>
+      <c r="N2" s="1">
         <v>46243</v>
       </c>
-      <c r="O2" s="2">
+      <c r="O2" s="1">
         <v>46251</v>
       </c>
       <c r="Q2">
@@ -796,16 +758,16 @@
         <v>41</v>
       </c>
       <c r="S2" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="T2" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="V2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="W2" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -819,42 +781,42 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E3" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="F3" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G3">
         <v>2733</v>
       </c>
       <c r="H3" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="I3" t="s">
-        <v>73</v>
-      </c>
-      <c r="J3" s="2">
+        <v>69</v>
+      </c>
+      <c r="J3" s="1">
         <v>46238</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46238</v>
       </c>
       <c r="L3">
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>75</v>
-      </c>
-      <c r="N3" s="2">
+        <v>71</v>
+      </c>
+      <c r="N3" s="1">
         <v>46269</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46269</v>
       </c>
       <c r="Q3">
@@ -864,16 +826,16 @@
         <v>15</v>
       </c>
       <c r="S3" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="T3" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="V3" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="W3" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -887,42 +849,42 @@
         <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="F4" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="G4">
         <v>2729</v>
       </c>
       <c r="H4" t="s">
+        <v>67</v>
+      </c>
+      <c r="I4" t="s">
+        <v>70</v>
+      </c>
+      <c r="J4" s="1">
+        <v>46244</v>
+      </c>
+      <c r="K4" s="1">
+        <v>46244</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4" t="s">
         <v>71</v>
       </c>
-      <c r="I4" t="s">
-        <v>74</v>
-      </c>
-      <c r="J4" s="2">
-        <v>46244</v>
-      </c>
-      <c r="K4" s="2">
-        <v>46244</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4" t="s">
-        <v>75</v>
-      </c>
-      <c r="N4" s="2">
+      <c r="N4" s="1">
         <v>46255</v>
       </c>
-      <c r="O4" s="2">
+      <c r="O4" s="1">
         <v>46255</v>
       </c>
       <c r="Q4">
@@ -932,19 +894,19 @@
         <v>9</v>
       </c>
       <c r="S4" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="T4" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="U4" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="V4" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="W4" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -958,42 +920,42 @@
         <v>29</v>
       </c>
       <c r="C5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E5" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F5" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G5">
         <v>2743</v>
       </c>
       <c r="H5" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="I5" t="s">
-        <v>73</v>
-      </c>
-      <c r="J5" s="2">
+        <v>69</v>
+      </c>
+      <c r="J5" s="1">
         <v>46244</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46246</v>
       </c>
       <c r="L5">
         <v>6</v>
       </c>
       <c r="M5" t="s">
-        <v>75</v>
-      </c>
-      <c r="N5" s="2">
+        <v>71</v>
+      </c>
+      <c r="N5" s="1">
         <v>46277</v>
       </c>
-      <c r="O5" s="2">
+      <c r="O5" s="1">
         <v>46254</v>
       </c>
       <c r="Q5">
@@ -1003,19 +965,19 @@
         <v>7</v>
       </c>
       <c r="S5" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="T5" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="U5" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="V5" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="W5" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1023,70 +985,70 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6">
-        <v>690</v>
+        <v>384</v>
       </c>
       <c r="B6" t="s">
         <v>30</v>
       </c>
       <c r="C6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E6" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="F6" t="s">
+        <v>63</v>
+      </c>
+      <c r="G6">
+        <v>2742</v>
+      </c>
+      <c r="H6" t="s">
+        <v>66</v>
+      </c>
+      <c r="I6" t="s">
         <v>69</v>
       </c>
-      <c r="G6">
-        <v>2727</v>
-      </c>
-      <c r="H6" t="s">
-        <v>70</v>
-      </c>
-      <c r="I6" t="s">
-        <v>74</v>
-      </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>46245</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46246</v>
       </c>
       <c r="L6">
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>75</v>
-      </c>
-      <c r="N6" s="2">
-        <v>46257</v>
-      </c>
-      <c r="O6" s="2">
-        <v>46251</v>
+        <v>71</v>
+      </c>
+      <c r="N6" s="1">
+        <v>46277</v>
+      </c>
+      <c r="O6" s="1">
+        <v>46254</v>
       </c>
       <c r="Q6">
-        <v>-4</v>
+        <v>-24</v>
       </c>
       <c r="R6">
         <v>7</v>
       </c>
       <c r="S6" t="s">
+        <v>73</v>
+      </c>
+      <c r="T6" t="s">
+        <v>72</v>
+      </c>
+      <c r="U6" t="s">
         <v>76</v>
       </c>
-      <c r="T6" t="s">
-        <v>76</v>
-      </c>
-      <c r="U6" t="s">
-        <v>80</v>
-      </c>
       <c r="V6" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="W6" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1094,70 +1056,64 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>384</v>
+        <v>329</v>
       </c>
       <c r="B7" t="s">
         <v>31</v>
       </c>
       <c r="C7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E7" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="F7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G7">
-        <v>2742</v>
+        <v>2721</v>
       </c>
       <c r="H7" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I7" t="s">
+        <v>69</v>
+      </c>
+      <c r="J7" s="1">
+        <v>46248</v>
+      </c>
+      <c r="K7" s="1">
+        <v>46248</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7" t="s">
+        <v>71</v>
+      </c>
+      <c r="N7" s="1">
+        <v>46279</v>
+      </c>
+      <c r="Q7">
+        <v>-26</v>
+      </c>
+      <c r="R7">
+        <v>5</v>
+      </c>
+      <c r="S7" t="s">
         <v>73</v>
       </c>
-      <c r="J7" s="2">
-        <v>46245</v>
-      </c>
-      <c r="K7" s="2">
-        <v>46246</v>
-      </c>
-      <c r="L7">
-        <v>1</v>
-      </c>
-      <c r="M7" t="s">
-        <v>75</v>
-      </c>
-      <c r="N7" s="2">
-        <v>46277</v>
-      </c>
-      <c r="O7" s="2">
-        <v>46254</v>
-      </c>
-      <c r="Q7">
-        <v>-24</v>
-      </c>
-      <c r="R7">
-        <v>7</v>
-      </c>
-      <c r="S7" t="s">
-        <v>77</v>
-      </c>
       <c r="T7" t="s">
-        <v>76</v>
-      </c>
-      <c r="U7" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="V7" t="s">
+        <v>84</v>
+      </c>
+      <c r="W7" t="s">
         <v>89</v>
-      </c>
-      <c r="W7" t="s">
-        <v>93</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1168,61 +1124,64 @@
         <v>329</v>
       </c>
       <c r="B8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E8" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="F8" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="G8">
-        <v>2721</v>
+        <v>2720</v>
       </c>
       <c r="H8" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="I8" t="s">
-        <v>73</v>
-      </c>
-      <c r="J8" s="2">
+        <v>70</v>
+      </c>
+      <c r="J8" s="1">
         <v>46248</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>46248</v>
       </c>
       <c r="L8">
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>75</v>
-      </c>
-      <c r="N8" s="2">
-        <v>46279</v>
+        <v>71</v>
+      </c>
+      <c r="N8" s="1">
+        <v>46259</v>
       </c>
       <c r="Q8">
-        <v>-26</v>
+        <v>-6</v>
       </c>
       <c r="R8">
         <v>5</v>
       </c>
       <c r="S8" t="s">
+        <v>73</v>
+      </c>
+      <c r="T8" t="s">
+        <v>72</v>
+      </c>
+      <c r="U8" t="s">
         <v>77</v>
       </c>
-      <c r="T8" t="s">
-        <v>76</v>
-      </c>
       <c r="V8" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="W8" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1230,45 +1189,45 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D9" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E9" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="F9" t="s">
+        <v>64</v>
+      </c>
+      <c r="G9">
+        <v>2729</v>
+      </c>
+      <c r="H9" t="s">
         <v>68</v>
       </c>
-      <c r="G9">
-        <v>2720</v>
-      </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
+        <v>70</v>
+      </c>
+      <c r="J9" s="1">
+        <v>46248</v>
+      </c>
+      <c r="K9" s="1">
+        <v>46248</v>
+      </c>
+      <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9" t="s">
         <v>71</v>
       </c>
-      <c r="I9" t="s">
-        <v>74</v>
-      </c>
-      <c r="J9" s="2">
-        <v>46248</v>
-      </c>
-      <c r="K9" s="2">
-        <v>46248</v>
-      </c>
-      <c r="L9">
-        <v>1</v>
-      </c>
-      <c r="M9" t="s">
-        <v>75</v>
-      </c>
-      <c r="N9" s="2">
+      <c r="N9" s="1">
         <v>46259</v>
       </c>
       <c r="Q9">
@@ -1278,19 +1237,19 @@
         <v>5</v>
       </c>
       <c r="S9" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="T9" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="U9" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="V9" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="W9" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1298,67 +1257,64 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D10" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E10" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F10" t="s">
+        <v>63</v>
+      </c>
+      <c r="G10">
+        <v>2741</v>
+      </c>
+      <c r="H10" t="s">
         <v>68</v>
       </c>
-      <c r="G10">
-        <v>2729</v>
-      </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
+        <v>69</v>
+      </c>
+      <c r="J10" s="1">
+        <v>46251</v>
+      </c>
+      <c r="K10" s="1">
+        <v>46249</v>
+      </c>
+      <c r="L10">
+        <v>2</v>
+      </c>
+      <c r="M10" t="s">
+        <v>71</v>
+      </c>
+      <c r="N10" s="1">
+        <v>46280</v>
+      </c>
+      <c r="Q10">
+        <v>-27</v>
+      </c>
+      <c r="R10">
+        <v>4</v>
+      </c>
+      <c r="S10" t="s">
         <v>72</v>
       </c>
-      <c r="I10" t="s">
-        <v>74</v>
-      </c>
-      <c r="J10" s="2">
-        <v>46248</v>
-      </c>
-      <c r="K10" s="2">
-        <v>46248</v>
-      </c>
-      <c r="L10">
-        <v>1</v>
-      </c>
-      <c r="M10" t="s">
-        <v>75</v>
-      </c>
-      <c r="N10" s="2">
-        <v>46259</v>
-      </c>
-      <c r="Q10">
-        <v>-6</v>
-      </c>
-      <c r="R10">
-        <v>5</v>
-      </c>
-      <c r="S10" t="s">
-        <v>77</v>
-      </c>
       <c r="T10" t="s">
-        <v>77</v>
-      </c>
-      <c r="U10" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="V10" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="W10" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1366,125 +1322,66 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B11" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E11" t="s">
+        <v>62</v>
+      </c>
+      <c r="F11" t="s">
         <v>65</v>
       </c>
-      <c r="F11" t="s">
-        <v>67</v>
-      </c>
       <c r="G11">
-        <v>2741</v>
+        <v>2729</v>
       </c>
       <c r="H11" t="s">
+        <v>68</v>
+      </c>
+      <c r="I11" t="s">
+        <v>69</v>
+      </c>
+      <c r="J11" s="1">
+        <v>46251</v>
+      </c>
+      <c r="K11" s="1">
+        <v>46251</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11" t="s">
+        <v>71</v>
+      </c>
+      <c r="N11" s="1">
+        <v>46282</v>
+      </c>
+      <c r="Q11">
+        <v>-29</v>
+      </c>
+      <c r="R11">
+        <v>2</v>
+      </c>
+      <c r="S11" t="s">
         <v>72</v>
       </c>
-      <c r="I11" t="s">
+      <c r="T11" t="s">
         <v>73</v>
       </c>
-      <c r="J11" s="2">
-        <v>46251</v>
-      </c>
-      <c r="K11" s="2">
-        <v>46249</v>
-      </c>
-      <c r="L11">
-        <v>2</v>
-      </c>
-      <c r="M11" t="s">
-        <v>75</v>
-      </c>
-      <c r="N11" s="2">
-        <v>46280</v>
-      </c>
-      <c r="Q11">
-        <v>-27</v>
-      </c>
-      <c r="R11">
-        <v>4</v>
-      </c>
-      <c r="S11" t="s">
-        <v>76</v>
-      </c>
-      <c r="T11" t="s">
-        <v>77</v>
+      <c r="V11" t="s">
+        <v>88</v>
       </c>
       <c r="W11" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="AA11" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:27">
-      <c r="A12">
-        <v>685</v>
-      </c>
-      <c r="B12" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" t="s">
-        <v>44</v>
-      </c>
-      <c r="D12" t="s">
-        <v>55</v>
-      </c>
-      <c r="E12" t="s">
-        <v>66</v>
-      </c>
-      <c r="F12" t="s">
-        <v>69</v>
-      </c>
-      <c r="G12">
-        <v>2729</v>
-      </c>
-      <c r="H12" t="s">
-        <v>72</v>
-      </c>
-      <c r="I12" t="s">
-        <v>73</v>
-      </c>
-      <c r="J12" s="2">
-        <v>46251</v>
-      </c>
-      <c r="K12" s="2">
-        <v>46251</v>
-      </c>
-      <c r="L12">
-        <v>1</v>
-      </c>
-      <c r="M12" t="s">
-        <v>75</v>
-      </c>
-      <c r="N12" s="2">
-        <v>46282</v>
-      </c>
-      <c r="Q12">
-        <v>-29</v>
-      </c>
-      <c r="R12">
-        <v>2</v>
-      </c>
-      <c r="S12" t="s">
-        <v>76</v>
-      </c>
-      <c r="T12" t="s">
-        <v>77</v>
-      </c>
-      <c r="W12" t="s">
-        <v>93</v>
-      </c>
-      <c r="AA12" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (19/08/2026 16:33)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="97">
   <si>
     <t>om_emg</t>
   </si>
@@ -145,6 +145,12 @@
     <t>685260012619</t>
   </si>
   <si>
+    <t>313260018708</t>
+  </si>
+  <si>
+    <t>396260016588</t>
+  </si>
+  <si>
     <t>030-1094-58</t>
   </si>
   <si>
@@ -175,6 +181,12 @@
     <t>071-01519-0101</t>
   </si>
   <si>
+    <t>2698010-7</t>
+  </si>
+  <si>
+    <t>0750220-1</t>
+  </si>
+  <si>
     <t>CONNECTOR</t>
   </si>
   <si>
@@ -205,6 +217,12 @@
     <t>RECEIVER-EXCITER,RAD</t>
   </si>
   <si>
+    <t>PASSENGER DOOR - LOW</t>
+  </si>
+  <si>
+    <t>BOLT,MACHINE</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -227,6 +245,9 @@
   </si>
   <si>
     <t>IPLR</t>
+  </si>
+  <si>
+    <t>AIFP</t>
   </si>
   <si>
     <t>EA</t>
@@ -619,7 +640,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA11"/>
+  <dimension ref="A1:AA13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -716,22 +737,22 @@
         <v>33</v>
       </c>
       <c r="D2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="F2" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="G2">
         <v>2702</v>
       </c>
       <c r="H2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I2" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="J2" s="1">
         <v>46212</v>
@@ -743,7 +764,7 @@
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="N2" s="1">
         <v>46243</v>
@@ -758,16 +779,16 @@
         <v>41</v>
       </c>
       <c r="S2" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="T2" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="V2" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="W2" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -784,22 +805,22 @@
         <v>34</v>
       </c>
       <c r="D3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E3" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="F3" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="G3">
         <v>2733</v>
       </c>
       <c r="H3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I3" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="J3" s="1">
         <v>46238</v>
@@ -811,7 +832,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="N3" s="1">
         <v>46269</v>
@@ -826,16 +847,16 @@
         <v>15</v>
       </c>
       <c r="S3" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="T3" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="V3" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="W3" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -852,22 +873,22 @@
         <v>35</v>
       </c>
       <c r="D4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="F4" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="G4">
         <v>2729</v>
       </c>
       <c r="H4" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="I4" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="J4" s="1">
         <v>46244</v>
@@ -879,7 +900,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="N4" s="1">
         <v>46255</v>
@@ -894,19 +915,19 @@
         <v>9</v>
       </c>
       <c r="S4" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="T4" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="U4" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="V4" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="W4" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -923,22 +944,22 @@
         <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E5" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="F5" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="G5">
         <v>2743</v>
       </c>
       <c r="H5" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="I5" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="J5" s="1">
         <v>46244</v>
@@ -950,7 +971,7 @@
         <v>6</v>
       </c>
       <c r="M5" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="N5" s="1">
         <v>46277</v>
@@ -965,19 +986,19 @@
         <v>7</v>
       </c>
       <c r="S5" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="T5" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="U5" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="V5" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="W5" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -994,22 +1015,22 @@
         <v>37</v>
       </c>
       <c r="D6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E6" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F6" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="G6">
         <v>2742</v>
       </c>
       <c r="H6" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I6" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="J6" s="1">
         <v>46245</v>
@@ -1021,7 +1042,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="N6" s="1">
         <v>46277</v>
@@ -1036,19 +1057,19 @@
         <v>7</v>
       </c>
       <c r="S6" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="T6" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="U6" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="V6" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="W6" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1065,22 +1086,22 @@
         <v>38</v>
       </c>
       <c r="D7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E7" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="F7" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="G7">
         <v>2721</v>
       </c>
       <c r="H7" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I7" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="J7" s="1">
         <v>46248</v>
@@ -1092,7 +1113,7 @@
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="N7" s="1">
         <v>46279</v>
@@ -1104,16 +1125,16 @@
         <v>5</v>
       </c>
       <c r="S7" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="T7" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="V7" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="W7" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1130,22 +1151,22 @@
         <v>39</v>
       </c>
       <c r="D8" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E8" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F8" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="G8">
         <v>2720</v>
       </c>
       <c r="H8" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="I8" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="J8" s="1">
         <v>46248</v>
@@ -1157,7 +1178,7 @@
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="N8" s="1">
         <v>46259</v>
@@ -1169,19 +1190,19 @@
         <v>5</v>
       </c>
       <c r="S8" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="T8" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="U8" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="V8" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="W8" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1198,22 +1219,22 @@
         <v>40</v>
       </c>
       <c r="D9" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E9" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="F9" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="G9">
         <v>2729</v>
       </c>
       <c r="H9" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I9" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="J9" s="1">
         <v>46248</v>
@@ -1225,7 +1246,7 @@
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="N9" s="1">
         <v>46259</v>
@@ -1237,19 +1258,19 @@
         <v>5</v>
       </c>
       <c r="S9" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="T9" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="U9" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="V9" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="W9" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1266,22 +1287,22 @@
         <v>41</v>
       </c>
       <c r="D10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E10" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="F10" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="G10">
         <v>2741</v>
       </c>
       <c r="H10" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I10" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="J10" s="1">
         <v>46251</v>
@@ -1293,7 +1314,7 @@
         <v>2</v>
       </c>
       <c r="M10" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="N10" s="1">
         <v>46280</v>
@@ -1305,16 +1326,16 @@
         <v>4</v>
       </c>
       <c r="S10" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="T10" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="V10" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="W10" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1331,22 +1352,22 @@
         <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E11" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F11" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="G11">
         <v>2729</v>
       </c>
       <c r="H11" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I11" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="J11" s="1">
         <v>46251</v>
@@ -1358,7 +1379,7 @@
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="N11" s="1">
         <v>46282</v>
@@ -1370,18 +1391,142 @@
         <v>2</v>
       </c>
       <c r="S11" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="T11" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="V11" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="W11" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="AA11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27">
+      <c r="A12">
+        <v>313</v>
+      </c>
+      <c r="B12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12" t="s">
+        <v>55</v>
+      </c>
+      <c r="E12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F12" t="s">
+        <v>70</v>
+      </c>
+      <c r="G12">
+        <v>2741</v>
+      </c>
+      <c r="H12" t="s">
+        <v>74</v>
+      </c>
+      <c r="I12" t="s">
+        <v>75</v>
+      </c>
+      <c r="J12" s="1">
+        <v>46253</v>
+      </c>
+      <c r="K12" s="1">
+        <v>46252</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12" t="s">
+        <v>78</v>
+      </c>
+      <c r="N12" s="1">
+        <v>46283</v>
+      </c>
+      <c r="Q12">
+        <v>-30</v>
+      </c>
+      <c r="R12">
+        <v>1</v>
+      </c>
+      <c r="S12" t="s">
+        <v>79</v>
+      </c>
+      <c r="T12" t="s">
+        <v>80</v>
+      </c>
+      <c r="W12" t="s">
+        <v>96</v>
+      </c>
+      <c r="AA12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27">
+      <c r="A13">
+        <v>396</v>
+      </c>
+      <c r="B13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" t="s">
+        <v>56</v>
+      </c>
+      <c r="E13" t="s">
+        <v>68</v>
+      </c>
+      <c r="F13" t="s">
+        <v>69</v>
+      </c>
+      <c r="G13">
+        <v>2731</v>
+      </c>
+      <c r="H13" t="s">
+        <v>74</v>
+      </c>
+      <c r="I13" t="s">
+        <v>77</v>
+      </c>
+      <c r="J13" s="1">
+        <v>46252</v>
+      </c>
+      <c r="K13" s="1">
+        <v>46253</v>
+      </c>
+      <c r="L13">
+        <v>1</v>
+      </c>
+      <c r="M13" t="s">
+        <v>78</v>
+      </c>
+      <c r="N13" s="1">
+        <v>46260</v>
+      </c>
+      <c r="Q13">
+        <v>-7</v>
+      </c>
+      <c r="R13">
+        <v>0</v>
+      </c>
+      <c r="S13" t="s">
+        <v>79</v>
+      </c>
+      <c r="T13" t="s">
+        <v>80</v>
+      </c>
+      <c r="W13" t="s">
+        <v>96</v>
+      </c>
+      <c r="AA13" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (20/08/2026 08:35)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -773,10 +773,10 @@
         <v>46251</v>
       </c>
       <c r="Q2">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R2">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="S2" t="s">
         <v>79</v>
@@ -841,10 +841,10 @@
         <v>46269</v>
       </c>
       <c r="Q3">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="R3">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S3" t="s">
         <v>79</v>
@@ -909,10 +909,10 @@
         <v>46255</v>
       </c>
       <c r="Q4">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R4">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="S4" t="s">
         <v>80</v>
@@ -980,10 +980,10 @@
         <v>46254</v>
       </c>
       <c r="Q5">
-        <v>-24</v>
+        <v>-23</v>
       </c>
       <c r="R5">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S5" t="s">
         <v>80</v>
@@ -1051,10 +1051,10 @@
         <v>46254</v>
       </c>
       <c r="Q6">
-        <v>-24</v>
+        <v>-23</v>
       </c>
       <c r="R6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S6" t="s">
         <v>80</v>
@@ -1119,10 +1119,10 @@
         <v>46279</v>
       </c>
       <c r="Q7">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="R7">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S7" t="s">
         <v>80</v>
@@ -1184,10 +1184,10 @@
         <v>46259</v>
       </c>
       <c r="Q8">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R8">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S8" t="s">
         <v>80</v>
@@ -1252,10 +1252,10 @@
         <v>46259</v>
       </c>
       <c r="Q9">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R9">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S9" t="s">
         <v>80</v>
@@ -1320,10 +1320,10 @@
         <v>46280</v>
       </c>
       <c r="Q10">
-        <v>-27</v>
+        <v>-26</v>
       </c>
       <c r="R10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S10" t="s">
         <v>79</v>
@@ -1385,10 +1385,10 @@
         <v>46282</v>
       </c>
       <c r="Q11">
-        <v>-29</v>
+        <v>-28</v>
       </c>
       <c r="R11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S11" t="s">
         <v>79</v>
@@ -1450,10 +1450,10 @@
         <v>46283</v>
       </c>
       <c r="Q12">
-        <v>-30</v>
+        <v>-29</v>
       </c>
       <c r="R12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S12" t="s">
         <v>79</v>
@@ -1512,10 +1512,10 @@
         <v>46260</v>
       </c>
       <c r="Q13">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S13" t="s">
         <v>79</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (20/08/2026 12:42)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -1231,7 +1231,7 @@
         <v>2729</v>
       </c>
       <c r="H9" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I9" t="s">
         <v>76</v>
@@ -1491,7 +1491,7 @@
         <v>2731</v>
       </c>
       <c r="H13" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I13" t="s">
         <v>77</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (20/08/2026 14:37)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="100">
   <si>
     <t>om_emg</t>
   </si>
@@ -151,6 +151,9 @@
     <t>396260016588</t>
   </si>
   <si>
+    <t>313260018713</t>
+  </si>
+  <si>
     <t>030-1094-58</t>
   </si>
   <si>
@@ -187,6 +190,9 @@
     <t>0750220-1</t>
   </si>
   <si>
+    <t>2115040-8</t>
+  </si>
+  <si>
     <t>CONNECTOR</t>
   </si>
   <si>
@@ -221,6 +227,9 @@
   </si>
   <si>
     <t>BOLT,MACHINE</t>
+  </si>
+  <si>
+    <t>CYLINDER GAS S</t>
   </si>
   <si>
     <t>C</t>
@@ -640,7 +649,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA13"/>
+  <dimension ref="A1:AA14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -737,22 +746,22 @@
         <v>33</v>
       </c>
       <c r="D2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G2">
         <v>2702</v>
       </c>
       <c r="H2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I2" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="J2" s="1">
         <v>46212</v>
@@ -764,7 +773,7 @@
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="N2" s="1">
         <v>46243</v>
@@ -779,16 +788,16 @@
         <v>42</v>
       </c>
       <c r="S2" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="T2" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="V2" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="W2" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -805,22 +814,22 @@
         <v>34</v>
       </c>
       <c r="D3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G3">
         <v>2733</v>
       </c>
       <c r="H3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I3" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="J3" s="1">
         <v>46238</v>
@@ -832,7 +841,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="N3" s="1">
         <v>46269</v>
@@ -847,16 +856,16 @@
         <v>16</v>
       </c>
       <c r="S3" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="T3" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="V3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="W3" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -873,22 +882,22 @@
         <v>35</v>
       </c>
       <c r="D4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F4" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G4">
         <v>2729</v>
       </c>
       <c r="H4" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I4" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="J4" s="1">
         <v>46244</v>
@@ -900,7 +909,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="N4" s="1">
         <v>46255</v>
@@ -915,19 +924,19 @@
         <v>10</v>
       </c>
       <c r="S4" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="T4" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="U4" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="V4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="W4" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -944,22 +953,22 @@
         <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F5" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G5">
         <v>2743</v>
       </c>
       <c r="H5" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="J5" s="1">
         <v>46244</v>
@@ -971,7 +980,7 @@
         <v>6</v>
       </c>
       <c r="M5" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="N5" s="1">
         <v>46277</v>
@@ -986,19 +995,19 @@
         <v>8</v>
       </c>
       <c r="S5" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="T5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="U5" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="V5" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="W5" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1015,22 +1024,22 @@
         <v>37</v>
       </c>
       <c r="D6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E6" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F6" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G6">
         <v>2742</v>
       </c>
       <c r="H6" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I6" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="J6" s="1">
         <v>46245</v>
@@ -1042,7 +1051,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="N6" s="1">
         <v>46277</v>
@@ -1057,19 +1066,19 @@
         <v>8</v>
       </c>
       <c r="S6" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="T6" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="U6" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="V6" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="W6" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1086,22 +1095,22 @@
         <v>38</v>
       </c>
       <c r="D7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F7" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="G7">
         <v>2721</v>
       </c>
       <c r="H7" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="I7" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="J7" s="1">
         <v>46248</v>
@@ -1113,7 +1122,7 @@
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="N7" s="1">
         <v>46279</v>
@@ -1125,16 +1134,16 @@
         <v>6</v>
       </c>
       <c r="S7" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="T7" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="V7" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="W7" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1151,22 +1160,22 @@
         <v>39</v>
       </c>
       <c r="D8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E8" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F8" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G8">
         <v>2720</v>
       </c>
       <c r="H8" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I8" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="J8" s="1">
         <v>46248</v>
@@ -1178,7 +1187,7 @@
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="N8" s="1">
         <v>46259</v>
@@ -1190,19 +1199,19 @@
         <v>6</v>
       </c>
       <c r="S8" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="T8" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="U8" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="V8" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="W8" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1219,22 +1228,22 @@
         <v>40</v>
       </c>
       <c r="D9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F9" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G9">
         <v>2729</v>
       </c>
       <c r="H9" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I9" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="J9" s="1">
         <v>46248</v>
@@ -1246,7 +1255,7 @@
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="N9" s="1">
         <v>46259</v>
@@ -1258,19 +1267,19 @@
         <v>6</v>
       </c>
       <c r="S9" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="T9" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="U9" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="V9" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="W9" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1287,22 +1296,22 @@
         <v>41</v>
       </c>
       <c r="D10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E10" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F10" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G10">
         <v>2741</v>
       </c>
       <c r="H10" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="I10" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="J10" s="1">
         <v>46251</v>
@@ -1314,7 +1323,7 @@
         <v>2</v>
       </c>
       <c r="M10" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="N10" s="1">
         <v>46280</v>
@@ -1326,16 +1335,16 @@
         <v>5</v>
       </c>
       <c r="S10" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="T10" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="V10" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="W10" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1352,22 +1361,22 @@
         <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E11" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F11" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="G11">
         <v>2729</v>
       </c>
       <c r="H11" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="I11" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="J11" s="1">
         <v>46251</v>
@@ -1379,7 +1388,7 @@
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="N11" s="1">
         <v>46282</v>
@@ -1391,16 +1400,16 @@
         <v>3</v>
       </c>
       <c r="S11" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="T11" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="V11" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="W11" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1417,22 +1426,22 @@
         <v>43</v>
       </c>
       <c r="D12" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E12" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F12" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G12">
         <v>2741</v>
       </c>
       <c r="H12" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="I12" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="J12" s="1">
         <v>46253</v>
@@ -1444,7 +1453,7 @@
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="N12" s="1">
         <v>46283</v>
@@ -1456,13 +1465,13 @@
         <v>2</v>
       </c>
       <c r="S12" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="T12" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="W12" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1479,22 +1488,22 @@
         <v>44</v>
       </c>
       <c r="D13" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E13" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F13" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G13">
         <v>2731</v>
       </c>
       <c r="H13" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I13" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="J13" s="1">
         <v>46252</v>
@@ -1506,7 +1515,7 @@
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="N13" s="1">
         <v>46260</v>
@@ -1518,15 +1527,77 @@
         <v>1</v>
       </c>
       <c r="S13" t="s">
+        <v>82</v>
+      </c>
+      <c r="T13" t="s">
+        <v>83</v>
+      </c>
+      <c r="W13" t="s">
+        <v>99</v>
+      </c>
+      <c r="AA13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:27">
+      <c r="A14">
+        <v>313</v>
+      </c>
+      <c r="B14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" t="s">
+        <v>45</v>
+      </c>
+      <c r="D14" t="s">
+        <v>58</v>
+      </c>
+      <c r="E14" t="s">
+        <v>71</v>
+      </c>
+      <c r="F14" t="s">
+        <v>72</v>
+      </c>
+      <c r="G14">
+        <v>2737</v>
+      </c>
+      <c r="H14" t="s">
+        <v>77</v>
+      </c>
+      <c r="I14" t="s">
         <v>79</v>
       </c>
-      <c r="T13" t="s">
-        <v>80</v>
-      </c>
-      <c r="W13" t="s">
-        <v>96</v>
-      </c>
-      <c r="AA13" t="b">
+      <c r="J14" s="1">
+        <v>46254</v>
+      </c>
+      <c r="K14" s="1">
+        <v>46255</v>
+      </c>
+      <c r="L14">
+        <v>2</v>
+      </c>
+      <c r="M14" t="s">
+        <v>81</v>
+      </c>
+      <c r="N14" s="1">
+        <v>46266</v>
+      </c>
+      <c r="Q14">
+        <v>-12</v>
+      </c>
+      <c r="R14">
+        <v>-1</v>
+      </c>
+      <c r="S14" t="s">
+        <v>82</v>
+      </c>
+      <c r="T14" t="s">
+        <v>83</v>
+      </c>
+      <c r="W14" t="s">
+        <v>99</v>
+      </c>
+      <c r="AA14" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (21/08/2026 08:33)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="102">
   <si>
     <t>om_emg</t>
   </si>
@@ -289,16 +289,16 @@
     <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
   </si>
   <si>
-    <t>Foi solicitado atendimento com estoque FAB - CLA- 10-08, ITEM PRONTO PARA EMBARQUE, AGUARDANDO NOTA FISCAL - CLA-11-08- ITEM AGUARDANDO DEFINIÇÃO DA COORDENADORIA QUANTO A EFETIVIDADE PARA APLICAÇÃO NA REFERIDA ANV.- CLA-13-08</t>
-  </si>
-  <si>
-    <t>Temos somente 03 ea em STK, favor utilizar o estoque FAB para posterior devolução. ATZ RC 13/08 - FOI SOLICITADO O ATENDIMENTO COM ESTOQUE FAB -CLA-13-08 - AWB 127-5299 0173 DPE 18/08/2026</t>
-  </si>
-  <si>
-    <t>Temos no STK V1, material em separação, recibo 682/FAB/26 - atz rc 13/08 - MATERIAL ENVIADO VIA AWB 12752709016 - DPE 18/08/2026</t>
-  </si>
-  <si>
-    <t>foi solicitoado o atendimento com o estoque FAB. CLA-17-08 - o item PN superado 069-1025-25 não serve na ANV 2721 - temos 4ea na wiliam para reparo, já foi solicitado o DPE.</t>
+    <t>Foi solicitado atendimento com estoque FAB - CLA- 10-08, ITEM PRONTO PARA EMBARQUE, AGUARDANDO NOTA FISCAL - CLA-11-08- ITEM AGUARDANDO DEFINIÇÃO DA COORDENADORIA QUANTO A EFETIVIDADE PARA APLICAÇÃO NA REFERIDA ANV.- CLA-13-08 - AT 685000002258</t>
+  </si>
+  <si>
+    <t>Temos somente 03 ea em STK, favor utilizar o estoque FAB para posterior devolução. ATZ RC 13/08 - FOI SOLICITADO O ATENDIMENTO COM ESTOQUE FAB -CLA-13-08 - AWB 127-5299 0173 DPE 18/08/2026 - ENTREGUE DIA 18/08/2026</t>
+  </si>
+  <si>
+    <t>Temos no STK V1, material em separação, recibo 682/FAB/26 - atz rc 13/08 - MATERIAL ENVIADO VIA AWB 12752709016 - DPE 18/08/2026 - ENTREGUE DIA 18/08/2026</t>
+  </si>
+  <si>
+    <t>foi solicitoado o atendimento com o estoque FAB. CLA-17-08 - o item PN superado 069-1025-25 não serve na ANV 2721 - temos 4ea na wiliam para reparo, já foi solicitado o DPE - OS 4 ITENS ESTÃO COM PROBLEMAS NO DISPAY. -FOI ENVIADO PARA O WIILIAM MAIS 3 UNS PARA REPARO - AINDA SEM DPE -CLA-20-08</t>
   </si>
   <si>
     <t>Enviado para o Operador dia 17/08/26, AWB 127-5332-5834 - REZ</t>
@@ -307,10 +307,16 @@
     <t>ITEM FOI ENTREGUE PARA A FAB VIA RECIBO 598/FAB/26 31-07-26 - AINDA NÃO FOI PARA O ESTOQUECLA-17-08</t>
   </si>
   <si>
-    <t>pedido no EPM E-C98-26061 -CLA-18-08</t>
-  </si>
-  <si>
-    <t>DPE DA WILLIAM DIA 20-08-2026 -CLA-18-08</t>
+    <t>pedido no EPM E-C98-26061 -CLA-18-08 - em cotação no mercado. Validar se os alternados PN A-7512-24 ou MS25309-7512 ou M6363/2-2 atendem</t>
+  </si>
+  <si>
+    <t>DPE DA WILLIAM DIA 20-08-2026 -CLA-18-08 -ENTREGUE NA BASE DO PAMALS 1 EA , SERÁ ENVIAO AO OPERADOR- CLA-20-08</t>
+  </si>
+  <si>
+    <t>Colocado pedido Textron WB0003128625 - direto para o Brasil</t>
+  </si>
+  <si>
+    <t>Colocado pedido no fornecedor - validando entrega em Miami</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -782,10 +788,10 @@
         <v>46251</v>
       </c>
       <c r="Q2">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="R2">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="S2" t="s">
         <v>82</v>
@@ -797,7 +803,7 @@
         <v>89</v>
       </c>
       <c r="W2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -850,10 +856,10 @@
         <v>46269</v>
       </c>
       <c r="Q3">
-        <v>-15</v>
+        <v>-14</v>
       </c>
       <c r="R3">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="S3" t="s">
         <v>82</v>
@@ -865,7 +871,7 @@
         <v>90</v>
       </c>
       <c r="W3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -918,10 +924,10 @@
         <v>46255</v>
       </c>
       <c r="Q4">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R4">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S4" t="s">
         <v>83</v>
@@ -936,7 +942,7 @@
         <v>91</v>
       </c>
       <c r="W4" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -986,13 +992,13 @@
         <v>46277</v>
       </c>
       <c r="O5" s="1">
-        <v>46254</v>
+        <v>46252</v>
       </c>
       <c r="Q5">
-        <v>-23</v>
+        <v>-22</v>
       </c>
       <c r="R5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S5" t="s">
         <v>83</v>
@@ -1007,7 +1013,7 @@
         <v>92</v>
       </c>
       <c r="W5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1057,13 +1063,13 @@
         <v>46277</v>
       </c>
       <c r="O6" s="1">
-        <v>46254</v>
+        <v>46252</v>
       </c>
       <c r="Q6">
-        <v>-23</v>
+        <v>-22</v>
       </c>
       <c r="R6">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S6" t="s">
         <v>83</v>
@@ -1078,7 +1084,7 @@
         <v>93</v>
       </c>
       <c r="W6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1128,10 +1134,10 @@
         <v>46279</v>
       </c>
       <c r="Q7">
-        <v>-25</v>
+        <v>-24</v>
       </c>
       <c r="R7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S7" t="s">
         <v>83</v>
@@ -1143,7 +1149,7 @@
         <v>94</v>
       </c>
       <c r="W7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1193,10 +1199,10 @@
         <v>46259</v>
       </c>
       <c r="Q8">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S8" t="s">
         <v>83</v>
@@ -1211,7 +1217,7 @@
         <v>95</v>
       </c>
       <c r="W8" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1261,10 +1267,10 @@
         <v>46259</v>
       </c>
       <c r="Q9">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S9" t="s">
         <v>83</v>
@@ -1279,7 +1285,7 @@
         <v>96</v>
       </c>
       <c r="W9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1329,10 +1335,10 @@
         <v>46280</v>
       </c>
       <c r="Q10">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="R10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S10" t="s">
         <v>82</v>
@@ -1344,7 +1350,7 @@
         <v>97</v>
       </c>
       <c r="W10" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1394,10 +1400,10 @@
         <v>46282</v>
       </c>
       <c r="Q11">
-        <v>-28</v>
+        <v>-27</v>
       </c>
       <c r="R11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S11" t="s">
         <v>82</v>
@@ -1409,7 +1415,7 @@
         <v>98</v>
       </c>
       <c r="W11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1459,10 +1465,10 @@
         <v>46283</v>
       </c>
       <c r="Q12">
-        <v>-29</v>
+        <v>-28</v>
       </c>
       <c r="R12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S12" t="s">
         <v>82</v>
@@ -1471,7 +1477,7 @@
         <v>83</v>
       </c>
       <c r="W12" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1521,10 +1527,10 @@
         <v>46260</v>
       </c>
       <c r="Q13">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S13" t="s">
         <v>82</v>
@@ -1532,8 +1538,11 @@
       <c r="T13" t="s">
         <v>83</v>
       </c>
+      <c r="V13" t="s">
+        <v>99</v>
+      </c>
       <c r="W13" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1583,10 +1592,10 @@
         <v>46266</v>
       </c>
       <c r="Q14">
-        <v>-12</v>
+        <v>-11</v>
       </c>
       <c r="R14">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="S14" t="s">
         <v>82</v>
@@ -1594,8 +1603,11 @@
       <c r="T14" t="s">
         <v>83</v>
       </c>
+      <c r="V14" t="s">
+        <v>100</v>
+      </c>
       <c r="W14" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (21/08/2026 09:06)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -271,13 +271,13 @@
     <t>item atendido com o estoque local pedido 18171852 em 10/08. Godoy 11/08. Está sendo definido se o PN está correto. Ramon 11/08/26.</t>
   </si>
   <si>
-    <t>Estoque com 12 EA do Pn LM600-9 (Alternado). Godoy 12/08/26. Atendido com estoque local em 13/08. Ramon 13/08/26</t>
+    <t>Estoque com 12 EA do Pn LM600-9 (Alternado). Godoy 12/08/26. Atendido com estoque local em 13/08. Ramon 13/08/26.  AWB 12752990173 - volume retirado na loja GOLLOG - POA por Djalma Pacheco em 18/08. Godoy 21/08/26.</t>
   </si>
   <si>
     <t>Estoque no alternado 285K4. Caso use do estoque, verificar validade que consta no item. Ramon 12/08/26. Item em pane, anv autorizada a voar por 3 dias pela MMEL a contar de 12/08. Ramon 13/08/26</t>
   </si>
   <si>
-    <t>item será atendido com o estoque local pedido 18216324. Godoy 17/08.</t>
+    <t>item será atendido com o estoque local pedido 18216324. Godoy 17/08. 20/08. AWB 12753325834 - volume retirado na loja GOLLOG - BSB por MATHEUS PINHO em 20/08. Godoy 21/08/26.</t>
   </si>
   <si>
     <t>Estoque alterado de "Nao" para "SIM"  daremos prioridade para movimentar o item.  Godoy 17/08/226</t>
@@ -329,8 +329,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -346,7 +354,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -354,12 +362,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -659,85 +685,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -769,10 +795,10 @@
       <c r="I2" t="s">
         <v>78</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>46212</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46212</v>
       </c>
       <c r="L2">
@@ -781,10 +807,10 @@
       <c r="M2" t="s">
         <v>81</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <v>46243</v>
       </c>
-      <c r="O2" s="1">
+      <c r="O2" s="2">
         <v>46251</v>
       </c>
       <c r="Q2">
@@ -837,10 +863,10 @@
       <c r="I3" t="s">
         <v>78</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>46238</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46238</v>
       </c>
       <c r="L3">
@@ -849,10 +875,10 @@
       <c r="M3" t="s">
         <v>81</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <v>46269</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46269</v>
       </c>
       <c r="Q3">
@@ -905,10 +931,10 @@
       <c r="I4" t="s">
         <v>79</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>46244</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46244</v>
       </c>
       <c r="L4">
@@ -917,10 +943,10 @@
       <c r="M4" t="s">
         <v>81</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="2">
         <v>46255</v>
       </c>
-      <c r="O4" s="1">
+      <c r="O4" s="2">
         <v>46255</v>
       </c>
       <c r="Q4">
@@ -976,10 +1002,10 @@
       <c r="I5" t="s">
         <v>78</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>46244</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46246</v>
       </c>
       <c r="L5">
@@ -988,10 +1014,10 @@
       <c r="M5" t="s">
         <v>81</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <v>46277</v>
       </c>
-      <c r="O5" s="1">
+      <c r="O5" s="2">
         <v>46252</v>
       </c>
       <c r="Q5">
@@ -1047,10 +1073,10 @@
       <c r="I6" t="s">
         <v>78</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>46245</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46246</v>
       </c>
       <c r="L6">
@@ -1059,10 +1085,10 @@
       <c r="M6" t="s">
         <v>81</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <v>46277</v>
       </c>
-      <c r="O6" s="1">
+      <c r="O6" s="2">
         <v>46252</v>
       </c>
       <c r="Q6">
@@ -1118,10 +1144,10 @@
       <c r="I7" t="s">
         <v>78</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46248</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46248</v>
       </c>
       <c r="L7">
@@ -1130,7 +1156,7 @@
       <c r="M7" t="s">
         <v>81</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="2">
         <v>46279</v>
       </c>
       <c r="Q7">
@@ -1183,10 +1209,10 @@
       <c r="I8" t="s">
         <v>79</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46248</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46248</v>
       </c>
       <c r="L8">
@@ -1195,7 +1221,7 @@
       <c r="M8" t="s">
         <v>81</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="2">
         <v>46259</v>
       </c>
       <c r="Q8">
@@ -1251,10 +1277,10 @@
       <c r="I9" t="s">
         <v>79</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46248</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46248</v>
       </c>
       <c r="L9">
@@ -1263,7 +1289,7 @@
       <c r="M9" t="s">
         <v>81</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>46259</v>
       </c>
       <c r="Q9">
@@ -1319,10 +1345,10 @@
       <c r="I10" t="s">
         <v>78</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46251</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>46249</v>
       </c>
       <c r="L10">
@@ -1331,7 +1357,7 @@
       <c r="M10" t="s">
         <v>81</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
         <v>46280</v>
       </c>
       <c r="Q10">
@@ -1384,10 +1410,10 @@
       <c r="I11" t="s">
         <v>78</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46251</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>46251</v>
       </c>
       <c r="L11">
@@ -1396,7 +1422,7 @@
       <c r="M11" t="s">
         <v>81</v>
       </c>
-      <c r="N11" s="1">
+      <c r="N11" s="2">
         <v>46282</v>
       </c>
       <c r="Q11">
@@ -1449,10 +1475,10 @@
       <c r="I12" t="s">
         <v>78</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>46253</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>46252</v>
       </c>
       <c r="L12">
@@ -1461,7 +1487,7 @@
       <c r="M12" t="s">
         <v>81</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="2">
         <v>46283</v>
       </c>
       <c r="Q12">
@@ -1511,10 +1537,10 @@
       <c r="I13" t="s">
         <v>80</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46252</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>46253</v>
       </c>
       <c r="L13">
@@ -1523,7 +1549,7 @@
       <c r="M13" t="s">
         <v>81</v>
       </c>
-      <c r="N13" s="1">
+      <c r="N13" s="2">
         <v>46260</v>
       </c>
       <c r="Q13">
@@ -1576,10 +1602,10 @@
       <c r="I14" t="s">
         <v>79</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46254</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>46255</v>
       </c>
       <c r="L14">
@@ -1588,7 +1614,7 @@
       <c r="M14" t="s">
         <v>81</v>
       </c>
-      <c r="N14" s="1">
+      <c r="N14" s="2">
         <v>46266</v>
       </c>
       <c r="Q14">

</xml_diff>

<commit_message>
Atualização automática: emergencias (21/08/2026 10:51)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -329,16 +329,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -354,7 +346,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -362,30 +354,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -685,85 +659,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -795,10 +769,10 @@
       <c r="I2" t="s">
         <v>78</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>46212</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46212</v>
       </c>
       <c r="L2">
@@ -807,10 +781,10 @@
       <c r="M2" t="s">
         <v>81</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="1">
         <v>46243</v>
       </c>
-      <c r="O2" s="2">
+      <c r="O2" s="1">
         <v>46251</v>
       </c>
       <c r="Q2">
@@ -863,10 +837,10 @@
       <c r="I3" t="s">
         <v>78</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>46238</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46238</v>
       </c>
       <c r="L3">
@@ -875,10 +849,10 @@
       <c r="M3" t="s">
         <v>81</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="1">
         <v>46269</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46269</v>
       </c>
       <c r="Q3">
@@ -931,10 +905,10 @@
       <c r="I4" t="s">
         <v>79</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>46244</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46244</v>
       </c>
       <c r="L4">
@@ -943,10 +917,10 @@
       <c r="M4" t="s">
         <v>81</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="1">
         <v>46255</v>
       </c>
-      <c r="O4" s="2">
+      <c r="O4" s="1">
         <v>46255</v>
       </c>
       <c r="Q4">
@@ -1002,10 +976,10 @@
       <c r="I5" t="s">
         <v>78</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>46244</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46246</v>
       </c>
       <c r="L5">
@@ -1014,10 +988,10 @@
       <c r="M5" t="s">
         <v>81</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="1">
         <v>46277</v>
       </c>
-      <c r="O5" s="2">
+      <c r="O5" s="1">
         <v>46252</v>
       </c>
       <c r="Q5">
@@ -1073,10 +1047,10 @@
       <c r="I6" t="s">
         <v>78</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>46245</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46246</v>
       </c>
       <c r="L6">
@@ -1085,10 +1059,10 @@
       <c r="M6" t="s">
         <v>81</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="1">
         <v>46277</v>
       </c>
-      <c r="O6" s="2">
+      <c r="O6" s="1">
         <v>46252</v>
       </c>
       <c r="Q6">
@@ -1144,10 +1118,10 @@
       <c r="I7" t="s">
         <v>78</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46248</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>46248</v>
       </c>
       <c r="L7">
@@ -1156,7 +1130,7 @@
       <c r="M7" t="s">
         <v>81</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="1">
         <v>46279</v>
       </c>
       <c r="Q7">
@@ -1209,10 +1183,10 @@
       <c r="I8" t="s">
         <v>79</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46248</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>46248</v>
       </c>
       <c r="L8">
@@ -1221,7 +1195,7 @@
       <c r="M8" t="s">
         <v>81</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="1">
         <v>46259</v>
       </c>
       <c r="Q8">
@@ -1277,10 +1251,10 @@
       <c r="I9" t="s">
         <v>79</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46248</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>46248</v>
       </c>
       <c r="L9">
@@ -1289,7 +1263,7 @@
       <c r="M9" t="s">
         <v>81</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="1">
         <v>46259</v>
       </c>
       <c r="Q9">
@@ -1345,10 +1319,10 @@
       <c r="I10" t="s">
         <v>78</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>46251</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>46249</v>
       </c>
       <c r="L10">
@@ -1357,7 +1331,7 @@
       <c r="M10" t="s">
         <v>81</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="1">
         <v>46280</v>
       </c>
       <c r="Q10">
@@ -1410,10 +1384,10 @@
       <c r="I11" t="s">
         <v>78</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46251</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>46251</v>
       </c>
       <c r="L11">
@@ -1422,7 +1396,7 @@
       <c r="M11" t="s">
         <v>81</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11" s="1">
         <v>46282</v>
       </c>
       <c r="Q11">
@@ -1475,10 +1449,10 @@
       <c r="I12" t="s">
         <v>78</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>46253</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>46252</v>
       </c>
       <c r="L12">
@@ -1487,7 +1461,7 @@
       <c r="M12" t="s">
         <v>81</v>
       </c>
-      <c r="N12" s="2">
+      <c r="N12" s="1">
         <v>46283</v>
       </c>
       <c r="Q12">
@@ -1537,10 +1511,10 @@
       <c r="I13" t="s">
         <v>80</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46252</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>46253</v>
       </c>
       <c r="L13">
@@ -1549,7 +1523,7 @@
       <c r="M13" t="s">
         <v>81</v>
       </c>
-      <c r="N13" s="2">
+      <c r="N13" s="1">
         <v>46260</v>
       </c>
       <c r="Q13">
@@ -1602,10 +1576,10 @@
       <c r="I14" t="s">
         <v>79</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46254</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>46255</v>
       </c>
       <c r="L14">
@@ -1614,7 +1588,7 @@
       <c r="M14" t="s">
         <v>81</v>
       </c>
-      <c r="N14" s="2">
+      <c r="N14" s="1">
         <v>46266</v>
       </c>
       <c r="Q14">

</xml_diff>

<commit_message>
Atualização automática: emergencias (21/08/2026 12:41)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="93">
   <si>
     <t>om_emg</t>
   </si>
@@ -103,9 +103,6 @@
     <t>BABE</t>
   </si>
   <si>
-    <t>BACO</t>
-  </si>
-  <si>
     <t>DACTA II</t>
   </si>
   <si>
@@ -124,18 +121,12 @@
     <t>685260012560</t>
   </si>
   <si>
-    <t>386260013489</t>
-  </si>
-  <si>
     <t>384260009396</t>
   </si>
   <si>
     <t>329260019269</t>
   </si>
   <si>
-    <t>329260019270</t>
-  </si>
-  <si>
     <t>685260012609</t>
   </si>
   <si>
@@ -154,6 +145,9 @@
     <t>313260018713</t>
   </si>
   <si>
+    <t>685260012655</t>
+  </si>
+  <si>
     <t>030-1094-58</t>
   </si>
   <si>
@@ -163,18 +157,12 @@
     <t>2641010-3</t>
   </si>
   <si>
-    <t>9910333-1</t>
-  </si>
-  <si>
     <t>S2616-285K4</t>
   </si>
   <si>
     <t>069-01033-0101</t>
   </si>
   <si>
-    <t>C662504-0101</t>
-  </si>
-  <si>
     <t>162-10700</t>
   </si>
   <si>
@@ -193,6 +181,9 @@
     <t>2115040-8</t>
   </si>
   <si>
+    <t>F2552-070</t>
+  </si>
+  <si>
     <t>CONNECTOR</t>
   </si>
   <si>
@@ -202,18 +193,12 @@
     <t>AXLE FITTING</t>
   </si>
   <si>
-    <t>ENGINE MOUNT</t>
-  </si>
-  <si>
     <t>ALTERNAD BELT</t>
   </si>
   <si>
     <t>RECEIVER-TRANSMITTER</t>
   </si>
   <si>
-    <t>GAGE VOLT AMME</t>
-  </si>
-  <si>
     <t>OUTER WHEEL HALF ASS</t>
   </si>
   <si>
@@ -232,6 +217,9 @@
     <t>CYLINDER GAS S</t>
   </si>
   <si>
+    <t>BARREL NUT</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -256,9 +244,6 @@
     <t>IPLR</t>
   </si>
   <si>
-    <t>AIFP</t>
-  </si>
-  <si>
     <t>EA</t>
   </si>
   <si>
@@ -271,15 +256,9 @@
     <t>item atendido com o estoque local pedido 18171852 em 10/08. Godoy 11/08. Está sendo definido se o PN está correto. Ramon 11/08/26.</t>
   </si>
   <si>
-    <t>Estoque com 12 EA do Pn LM600-9 (Alternado). Godoy 12/08/26. Atendido com estoque local em 13/08. Ramon 13/08/26.  AWB 12752990173 - volume retirado na loja GOLLOG - POA por Djalma Pacheco em 18/08. Godoy 21/08/26.</t>
-  </si>
-  <si>
     <t>Estoque no alternado 285K4. Caso use do estoque, verificar validade que consta no item. Ramon 12/08/26. Item em pane, anv autorizada a voar por 3 dias pela MMEL a contar de 12/08. Ramon 13/08/26</t>
   </si>
   <si>
-    <t>item será atendido com o estoque local pedido 18216324. Godoy 17/08. 20/08. AWB 12753325834 - volume retirado na loja GOLLOG - BSB por MATHEUS PINHO em 20/08. Godoy 21/08/26.</t>
-  </si>
-  <si>
     <t>Estoque alterado de "Nao" para "SIM"  daremos prioridade para movimentar o item.  Godoy 17/08/226</t>
   </si>
   <si>
@@ -292,16 +271,10 @@
     <t>Foi solicitado atendimento com estoque FAB - CLA- 10-08, ITEM PRONTO PARA EMBARQUE, AGUARDANDO NOTA FISCAL - CLA-11-08- ITEM AGUARDANDO DEFINIÇÃO DA COORDENADORIA QUANTO A EFETIVIDADE PARA APLICAÇÃO NA REFERIDA ANV.- CLA-13-08 - AT 685000002258</t>
   </si>
   <si>
-    <t>Temos somente 03 ea em STK, favor utilizar o estoque FAB para posterior devolução. ATZ RC 13/08 - FOI SOLICITADO O ATENDIMENTO COM ESTOQUE FAB -CLA-13-08 - AWB 127-5299 0173 DPE 18/08/2026 - ENTREGUE DIA 18/08/2026</t>
-  </si>
-  <si>
     <t>Temos no STK V1, material em separação, recibo 682/FAB/26 - atz rc 13/08 - MATERIAL ENVIADO VIA AWB 12752709016 - DPE 18/08/2026 - ENTREGUE DIA 18/08/2026</t>
   </si>
   <si>
     <t>foi solicitoado o atendimento com o estoque FAB. CLA-17-08 - o item PN superado 069-1025-25 não serve na ANV 2721 - temos 4ea na wiliam para reparo, já foi solicitado o DPE - OS 4 ITENS ESTÃO COM PROBLEMAS NO DISPAY. -FOI ENVIADO PARA O WIILIAM MAIS 3 UNS PARA REPARO - AINDA SEM DPE -CLA-20-08</t>
-  </si>
-  <si>
-    <t>Enviado para o Operador dia 17/08/26, AWB 127-5332-5834 - REZ</t>
   </si>
   <si>
     <t>ITEM FOI ENTREGUE PARA A FAB VIA RECIBO 598/FAB/26 31-07-26 - AINDA NÃO FOI PARA O ESTOQUECLA-17-08</t>
@@ -655,7 +628,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA14"/>
+  <dimension ref="A1:AA13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -749,25 +722,25 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F2" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G2">
         <v>2702</v>
       </c>
       <c r="H2" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="I2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="J2" s="1">
         <v>46212</v>
@@ -779,7 +752,7 @@
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="N2" s="1">
         <v>46243</v>
@@ -794,16 +767,16 @@
         <v>43</v>
       </c>
       <c r="S2" t="s">
+        <v>77</v>
+      </c>
+      <c r="T2" t="s">
+        <v>78</v>
+      </c>
+      <c r="V2" t="s">
         <v>82</v>
       </c>
-      <c r="T2" t="s">
-        <v>83</v>
-      </c>
-      <c r="V2" t="s">
-        <v>89</v>
-      </c>
       <c r="W2" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -817,25 +790,25 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="F3" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G3">
         <v>2733</v>
       </c>
       <c r="H3" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="I3" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="J3" s="1">
         <v>46238</v>
@@ -847,7 +820,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="N3" s="1">
         <v>46269</v>
@@ -862,16 +835,16 @@
         <v>17</v>
       </c>
       <c r="S3" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="T3" t="s">
+        <v>78</v>
+      </c>
+      <c r="V3" t="s">
         <v>83</v>
       </c>
-      <c r="V3" t="s">
-        <v>90</v>
-      </c>
       <c r="W3" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -885,25 +858,25 @@
         <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E4" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="F4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G4">
         <v>2729</v>
       </c>
       <c r="H4" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="I4" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="J4" s="1">
         <v>46244</v>
@@ -915,7 +888,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="N4" s="1">
         <v>46255</v>
@@ -930,19 +903,19 @@
         <v>11</v>
       </c>
       <c r="S4" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="T4" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="U4" t="s">
+        <v>79</v>
+      </c>
+      <c r="V4" t="s">
         <v>84</v>
       </c>
-      <c r="V4" t="s">
-        <v>91</v>
-      </c>
       <c r="W4" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -950,43 +923,43 @@
     </row>
     <row r="5" spans="1:27">
       <c r="A5">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B5" t="s">
         <v>29</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="F5" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G5">
-        <v>2743</v>
+        <v>2742</v>
       </c>
       <c r="H5" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="I5" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="J5" s="1">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="K5" s="1">
         <v>46246</v>
       </c>
       <c r="L5">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="N5" s="1">
         <v>46277</v>
@@ -1001,19 +974,19 @@
         <v>9</v>
       </c>
       <c r="S5" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="T5" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="U5" t="s">
+        <v>80</v>
+      </c>
+      <c r="V5" t="s">
         <v>85</v>
       </c>
-      <c r="V5" t="s">
+      <c r="W5" t="s">
         <v>92</v>
-      </c>
-      <c r="W5" t="s">
-        <v>101</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1021,70 +994,64 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6">
-        <v>384</v>
+        <v>329</v>
       </c>
       <c r="B6" t="s">
         <v>30</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E6" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="F6" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G6">
-        <v>2742</v>
+        <v>2721</v>
       </c>
       <c r="H6" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="I6" t="s">
+        <v>74</v>
+      </c>
+      <c r="J6" s="1">
+        <v>46248</v>
+      </c>
+      <c r="K6" s="1">
+        <v>46248</v>
+      </c>
+      <c r="L6">
+        <v>1</v>
+      </c>
+      <c r="M6" t="s">
+        <v>76</v>
+      </c>
+      <c r="N6" s="1">
+        <v>46279</v>
+      </c>
+      <c r="Q6">
+        <v>-24</v>
+      </c>
+      <c r="R6">
+        <v>7</v>
+      </c>
+      <c r="S6" t="s">
         <v>78</v>
       </c>
-      <c r="J6" s="1">
-        <v>46245</v>
-      </c>
-      <c r="K6" s="1">
-        <v>46246</v>
-      </c>
-      <c r="L6">
-        <v>1</v>
-      </c>
-      <c r="M6" t="s">
-        <v>81</v>
-      </c>
-      <c r="N6" s="1">
-        <v>46277</v>
-      </c>
-      <c r="O6" s="1">
-        <v>46252</v>
-      </c>
-      <c r="Q6">
-        <v>-22</v>
-      </c>
-      <c r="R6">
-        <v>9</v>
-      </c>
-      <c r="S6" t="s">
-        <v>83</v>
-      </c>
       <c r="T6" t="s">
-        <v>82</v>
-      </c>
-      <c r="U6" t="s">
+        <v>77</v>
+      </c>
+      <c r="V6" t="s">
         <v>86</v>
       </c>
-      <c r="V6" t="s">
-        <v>93</v>
-      </c>
       <c r="W6" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1092,31 +1059,31 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F7" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="G7">
-        <v>2721</v>
+        <v>2729</v>
       </c>
       <c r="H7" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="I7" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="J7" s="1">
         <v>46248</v>
@@ -1128,28 +1095,31 @@
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="N7" s="1">
-        <v>46279</v>
+        <v>46259</v>
       </c>
       <c r="Q7">
-        <v>-24</v>
+        <v>-4</v>
       </c>
       <c r="R7">
         <v>7</v>
       </c>
       <c r="S7" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="T7" t="s">
-        <v>82</v>
+        <v>78</v>
+      </c>
+      <c r="U7" t="s">
+        <v>81</v>
       </c>
       <c r="V7" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="W7" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1157,67 +1127,64 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>329</v>
+        <v>313</v>
       </c>
       <c r="B8" t="s">
         <v>31</v>
       </c>
       <c r="C8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F8" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="G8">
-        <v>2720</v>
+        <v>2741</v>
       </c>
       <c r="H8" t="s">
+        <v>71</v>
+      </c>
+      <c r="I8" t="s">
+        <v>74</v>
+      </c>
+      <c r="J8" s="1">
+        <v>46251</v>
+      </c>
+      <c r="K8" s="1">
+        <v>46249</v>
+      </c>
+      <c r="L8">
+        <v>2</v>
+      </c>
+      <c r="M8" t="s">
         <v>76</v>
       </c>
-      <c r="I8" t="s">
-        <v>79</v>
-      </c>
-      <c r="J8" s="1">
-        <v>46248</v>
-      </c>
-      <c r="K8" s="1">
-        <v>46248</v>
-      </c>
-      <c r="L8">
-        <v>1</v>
-      </c>
-      <c r="M8" t="s">
-        <v>81</v>
-      </c>
       <c r="N8" s="1">
-        <v>46259</v>
+        <v>46280</v>
       </c>
       <c r="Q8">
-        <v>-4</v>
+        <v>-25</v>
       </c>
       <c r="R8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S8" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="T8" t="s">
-        <v>82</v>
-      </c>
-      <c r="U8" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="V8" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="W8" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1231,61 +1198,58 @@
         <v>27</v>
       </c>
       <c r="C9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E9" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="F9" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="G9">
         <v>2729</v>
       </c>
       <c r="H9" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="I9" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="J9" s="1">
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="K9" s="1">
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="L9">
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="N9" s="1">
-        <v>46259</v>
+        <v>46282</v>
       </c>
       <c r="Q9">
-        <v>-4</v>
+        <v>-27</v>
       </c>
       <c r="R9">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="S9" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="T9" t="s">
-        <v>83</v>
-      </c>
-      <c r="U9" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="V9" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="W9" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1296,61 +1260,58 @@
         <v>313</v>
       </c>
       <c r="B10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D10" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E10" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="F10" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="G10">
         <v>2741</v>
       </c>
       <c r="H10" t="s">
+        <v>71</v>
+      </c>
+      <c r="I10" t="s">
+        <v>74</v>
+      </c>
+      <c r="J10" s="1">
+        <v>46253</v>
+      </c>
+      <c r="K10" s="1">
+        <v>46252</v>
+      </c>
+      <c r="L10">
+        <v>1</v>
+      </c>
+      <c r="M10" t="s">
+        <v>76</v>
+      </c>
+      <c r="N10" s="1">
+        <v>46283</v>
+      </c>
+      <c r="Q10">
+        <v>-28</v>
+      </c>
+      <c r="R10">
+        <v>3</v>
+      </c>
+      <c r="S10" t="s">
         <v>77</v>
       </c>
-      <c r="I10" t="s">
+      <c r="T10" t="s">
         <v>78</v>
       </c>
-      <c r="J10" s="1">
-        <v>46251</v>
-      </c>
-      <c r="K10" s="1">
-        <v>46249</v>
-      </c>
-      <c r="L10">
-        <v>2</v>
-      </c>
-      <c r="M10" t="s">
-        <v>81</v>
-      </c>
-      <c r="N10" s="1">
-        <v>46280</v>
-      </c>
-      <c r="Q10">
-        <v>-25</v>
-      </c>
-      <c r="R10">
-        <v>6</v>
-      </c>
-      <c r="S10" t="s">
-        <v>82</v>
-      </c>
-      <c r="T10" t="s">
-        <v>83</v>
-      </c>
-      <c r="V10" t="s">
-        <v>97</v>
-      </c>
       <c r="W10" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1358,64 +1319,64 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>685</v>
+        <v>396</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D11" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E11" t="s">
+        <v>65</v>
+      </c>
+      <c r="F11" t="s">
         <v>68</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11">
+        <v>2731</v>
+      </c>
+      <c r="H11" t="s">
+        <v>71</v>
+      </c>
+      <c r="I11" t="s">
         <v>74</v>
       </c>
-      <c r="G11">
-        <v>2729</v>
-      </c>
-      <c r="H11" t="s">
+      <c r="J11" s="1">
+        <v>46252</v>
+      </c>
+      <c r="K11" s="1">
+        <v>46253</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11" t="s">
+        <v>76</v>
+      </c>
+      <c r="N11" s="1">
+        <v>46284</v>
+      </c>
+      <c r="Q11">
+        <v>-29</v>
+      </c>
+      <c r="R11">
+        <v>2</v>
+      </c>
+      <c r="S11" t="s">
         <v>77</v>
       </c>
-      <c r="I11" t="s">
+      <c r="T11" t="s">
         <v>78</v>
       </c>
-      <c r="J11" s="1">
-        <v>46251</v>
-      </c>
-      <c r="K11" s="1">
-        <v>46251</v>
-      </c>
-      <c r="L11">
-        <v>1</v>
-      </c>
-      <c r="M11" t="s">
-        <v>81</v>
-      </c>
-      <c r="N11" s="1">
-        <v>46282</v>
-      </c>
-      <c r="Q11">
-        <v>-27</v>
-      </c>
-      <c r="R11">
-        <v>4</v>
-      </c>
-      <c r="S11" t="s">
-        <v>82</v>
-      </c>
-      <c r="T11" t="s">
-        <v>83</v>
-      </c>
       <c r="V11" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="W11" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1426,58 +1387,61 @@
         <v>313</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C12" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D12" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E12" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="F12" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="G12">
-        <v>2741</v>
+        <v>2737</v>
       </c>
       <c r="H12" t="s">
+        <v>71</v>
+      </c>
+      <c r="I12" t="s">
+        <v>75</v>
+      </c>
+      <c r="J12" s="1">
+        <v>46254</v>
+      </c>
+      <c r="K12" s="1">
+        <v>46255</v>
+      </c>
+      <c r="L12">
+        <v>2</v>
+      </c>
+      <c r="M12" t="s">
+        <v>76</v>
+      </c>
+      <c r="N12" s="1">
+        <v>46266</v>
+      </c>
+      <c r="Q12">
+        <v>-11</v>
+      </c>
+      <c r="R12">
+        <v>0</v>
+      </c>
+      <c r="S12" t="s">
         <v>77</v>
       </c>
-      <c r="I12" t="s">
+      <c r="T12" t="s">
         <v>78</v>
       </c>
-      <c r="J12" s="1">
-        <v>46253</v>
-      </c>
-      <c r="K12" s="1">
-        <v>46252</v>
-      </c>
-      <c r="L12">
-        <v>1</v>
-      </c>
-      <c r="M12" t="s">
-        <v>81</v>
-      </c>
-      <c r="N12" s="1">
-        <v>46283</v>
-      </c>
-      <c r="Q12">
-        <v>-28</v>
-      </c>
-      <c r="R12">
-        <v>3</v>
-      </c>
-      <c r="S12" t="s">
-        <v>82</v>
-      </c>
-      <c r="T12" t="s">
-        <v>83</v>
+      <c r="V12" t="s">
+        <v>91</v>
       </c>
       <c r="W12" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1485,131 +1449,63 @@
     </row>
     <row r="13" spans="1:27">
       <c r="A13">
-        <v>396</v>
+        <v>685</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C13" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E13" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="F13" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G13">
-        <v>2731</v>
+        <v>2729</v>
       </c>
       <c r="H13" t="s">
+        <v>73</v>
+      </c>
+      <c r="I13" t="s">
         <v>75</v>
       </c>
-      <c r="I13" t="s">
-        <v>80</v>
-      </c>
       <c r="J13" s="1">
-        <v>46252</v>
+        <v>46254</v>
       </c>
       <c r="K13" s="1">
         <v>46253</v>
       </c>
       <c r="L13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M13" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="N13" s="1">
-        <v>46260</v>
+        <v>46264</v>
       </c>
       <c r="Q13">
-        <v>-5</v>
+        <v>-9</v>
       </c>
       <c r="R13">
         <v>2</v>
       </c>
       <c r="S13" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="T13" t="s">
-        <v>83</v>
-      </c>
-      <c r="V13" t="s">
-        <v>99</v>
+        <v>78</v>
       </c>
       <c r="W13" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="AA13" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:27">
-      <c r="A14">
-        <v>313</v>
-      </c>
-      <c r="B14" t="s">
-        <v>32</v>
-      </c>
-      <c r="C14" t="s">
-        <v>45</v>
-      </c>
-      <c r="D14" t="s">
-        <v>58</v>
-      </c>
-      <c r="E14" t="s">
-        <v>71</v>
-      </c>
-      <c r="F14" t="s">
-        <v>72</v>
-      </c>
-      <c r="G14">
-        <v>2737</v>
-      </c>
-      <c r="H14" t="s">
-        <v>77</v>
-      </c>
-      <c r="I14" t="s">
-        <v>79</v>
-      </c>
-      <c r="J14" s="1">
-        <v>46254</v>
-      </c>
-      <c r="K14" s="1">
-        <v>46255</v>
-      </c>
-      <c r="L14">
-        <v>2</v>
-      </c>
-      <c r="M14" t="s">
-        <v>81</v>
-      </c>
-      <c r="N14" s="1">
-        <v>46266</v>
-      </c>
-      <c r="Q14">
-        <v>-11</v>
-      </c>
-      <c r="R14">
-        <v>0</v>
-      </c>
-      <c r="S14" t="s">
-        <v>82</v>
-      </c>
-      <c r="T14" t="s">
-        <v>83</v>
-      </c>
-      <c r="V14" t="s">
-        <v>100</v>
-      </c>
-      <c r="W14" t="s">
-        <v>101</v>
-      </c>
-      <c r="AA14" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (24/08/2026 08:36)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="94">
   <si>
     <t>om_emg</t>
   </si>
@@ -283,13 +283,16 @@
     <t>pedido no EPM E-C98-26061 -CLA-18-08 - em cotação no mercado. Validar se os alternados PN A-7512-24 ou MS25309-7512 ou M6363/2-2 atendem</t>
   </si>
   <si>
-    <t>DPE DA WILLIAM DIA 20-08-2026 -CLA-18-08 -ENTREGUE NA BASE DO PAMALS 1 EA , SERÁ ENVIAO AO OPERADOR- CLA-20-08</t>
-  </si>
-  <si>
-    <t>Colocado pedido Textron WB0003128625 - direto para o Brasil</t>
-  </si>
-  <si>
-    <t>Colocado pedido no fornecedor - validando entrega em Miami</t>
+    <t>DPE DA WILLIAM DIA 20-08-2026 -CLA-18-08 -ENTREGUE NA BASE DO PAMALS 1 EA , SERÁ ENVIAO AO OPERADOR- CLA-20-08 - AWB127-5408 8775- CLA-21-08</t>
+  </si>
+  <si>
+    <t>Colocado pedido Textron WB0003128625 - tracking 535477333011 - previsão de entrega 24/08</t>
+  </si>
+  <si>
+    <t>Colocado pedido no fornecedor S624333 - validando entrega em Miami - TEMOS 3 EA NO ESTOQUE DA BANT</t>
+  </si>
+  <si>
+    <t>Será atendido via estoque V1 JPA. Em processo de envio. ATZ 21/08</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -761,10 +764,10 @@
         <v>46251</v>
       </c>
       <c r="Q2">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="R2">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="S2" t="s">
         <v>77</v>
@@ -776,7 +779,7 @@
         <v>82</v>
       </c>
       <c r="W2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -829,10 +832,10 @@
         <v>46269</v>
       </c>
       <c r="Q3">
-        <v>-14</v>
+        <v>-11</v>
       </c>
       <c r="R3">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="S3" t="s">
         <v>77</v>
@@ -844,7 +847,7 @@
         <v>83</v>
       </c>
       <c r="W3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -897,10 +900,10 @@
         <v>46255</v>
       </c>
       <c r="Q4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R4">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="S4" t="s">
         <v>78</v>
@@ -915,7 +918,7 @@
         <v>84</v>
       </c>
       <c r="W4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -968,10 +971,10 @@
         <v>46252</v>
       </c>
       <c r="Q5">
-        <v>-22</v>
+        <v>-19</v>
       </c>
       <c r="R5">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="S5" t="s">
         <v>78</v>
@@ -986,7 +989,7 @@
         <v>85</v>
       </c>
       <c r="W5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1036,10 +1039,10 @@
         <v>46279</v>
       </c>
       <c r="Q6">
-        <v>-24</v>
+        <v>-21</v>
       </c>
       <c r="R6">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S6" t="s">
         <v>78</v>
@@ -1051,7 +1054,7 @@
         <v>86</v>
       </c>
       <c r="W6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1101,10 +1104,10 @@
         <v>46259</v>
       </c>
       <c r="Q7">
-        <v>-4</v>
+        <v>-1</v>
       </c>
       <c r="R7">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S7" t="s">
         <v>78</v>
@@ -1119,7 +1122,7 @@
         <v>87</v>
       </c>
       <c r="W7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1169,10 +1172,10 @@
         <v>46280</v>
       </c>
       <c r="Q8">
-        <v>-25</v>
+        <v>-22</v>
       </c>
       <c r="R8">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="S8" t="s">
         <v>77</v>
@@ -1184,7 +1187,7 @@
         <v>88</v>
       </c>
       <c r="W8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1233,11 +1236,14 @@
       <c r="N9" s="1">
         <v>46282</v>
       </c>
+      <c r="O9" s="1">
+        <v>46255</v>
+      </c>
       <c r="Q9">
-        <v>-27</v>
+        <v>-24</v>
       </c>
       <c r="R9">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="S9" t="s">
         <v>77</v>
@@ -1249,7 +1255,7 @@
         <v>89</v>
       </c>
       <c r="W9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1299,10 +1305,10 @@
         <v>46283</v>
       </c>
       <c r="Q10">
-        <v>-28</v>
+        <v>-25</v>
       </c>
       <c r="R10">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="S10" t="s">
         <v>77</v>
@@ -1311,7 +1317,7 @@
         <v>78</v>
       </c>
       <c r="W10" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1361,10 +1367,10 @@
         <v>46284</v>
       </c>
       <c r="Q11">
-        <v>-29</v>
+        <v>-26</v>
       </c>
       <c r="R11">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S11" t="s">
         <v>77</v>
@@ -1376,7 +1382,7 @@
         <v>90</v>
       </c>
       <c r="W11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1426,10 +1432,10 @@
         <v>46266</v>
       </c>
       <c r="Q12">
-        <v>-11</v>
+        <v>-8</v>
       </c>
       <c r="R12">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S12" t="s">
         <v>77</v>
@@ -1441,7 +1447,7 @@
         <v>91</v>
       </c>
       <c r="W12" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1491,10 +1497,10 @@
         <v>46264</v>
       </c>
       <c r="Q13">
-        <v>-9</v>
+        <v>-6</v>
       </c>
       <c r="R13">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S13" t="s">
         <v>77</v>
@@ -1502,8 +1508,11 @@
       <c r="T13" t="s">
         <v>78</v>
       </c>
+      <c r="V13" t="s">
+        <v>92</v>
+      </c>
       <c r="W13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (24/08/2026 10:56)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="93">
   <si>
     <t>om_emg</t>
   </si>
@@ -145,7 +145,7 @@
     <t>313260018713</t>
   </si>
   <si>
-    <t>685260012655</t>
+    <t>329260019279</t>
   </si>
   <si>
     <t>030-1094-58</t>
@@ -181,7 +181,7 @@
     <t>2115040-8</t>
   </si>
   <si>
-    <t>F2552-070</t>
+    <t>2N6576</t>
   </si>
   <si>
     <t>CONNECTOR</t>
@@ -217,7 +217,7 @@
     <t>CYLINDER GAS S</t>
   </si>
   <si>
-    <t>BARREL NUT</t>
+    <t>TRANSISTOR</t>
   </si>
   <si>
     <t>C</t>
@@ -235,9 +235,6 @@
     <t>Expedido total</t>
   </si>
   <si>
-    <t>Aguardando solução</t>
-  </si>
-  <si>
     <t>ANCE</t>
   </si>
   <si>
@@ -262,6 +259,9 @@
     <t>Estoque alterado de "Nao" para "SIM"  daremos prioridade para movimentar o item.  Godoy 17/08/226</t>
   </si>
   <si>
+    <t>Emergência transformada em ANCE em 24/08. Aguardaremos atendimento com item da Vee One. Ramon 24/08/26.</t>
+  </si>
+  <si>
     <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Chegada GIG dia 15-08 (voo 4273). Entregue V1 JPA 17/08</t>
   </si>
   <si>
@@ -290,9 +290,6 @@
   </si>
   <si>
     <t>Colocado pedido no fornecedor S624333 - validando entrega em Miami - TEMOS 3 EA NO ESTOQUE DA BANT</t>
-  </si>
-  <si>
-    <t>Será atendido via estoque V1 JPA. Em processo de envio. ATZ 21/08</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -743,7 +740,7 @@
         <v>71</v>
       </c>
       <c r="I2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J2" s="1">
         <v>46212</v>
@@ -755,7 +752,7 @@
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="N2" s="1">
         <v>46243</v>
@@ -770,16 +767,16 @@
         <v>46</v>
       </c>
       <c r="S2" t="s">
+        <v>76</v>
+      </c>
+      <c r="T2" t="s">
         <v>77</v>
-      </c>
-      <c r="T2" t="s">
-        <v>78</v>
       </c>
       <c r="V2" t="s">
         <v>82</v>
       </c>
       <c r="W2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -811,7 +808,7 @@
         <v>71</v>
       </c>
       <c r="I3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J3" s="1">
         <v>46238</v>
@@ -823,7 +820,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="N3" s="1">
         <v>46269</v>
@@ -838,16 +835,16 @@
         <v>20</v>
       </c>
       <c r="S3" t="s">
+        <v>76</v>
+      </c>
+      <c r="T3" t="s">
         <v>77</v>
-      </c>
-      <c r="T3" t="s">
-        <v>78</v>
       </c>
       <c r="V3" t="s">
         <v>83</v>
       </c>
       <c r="W3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -879,7 +876,7 @@
         <v>72</v>
       </c>
       <c r="I4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J4" s="1">
         <v>46244</v>
@@ -891,7 +888,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="N4" s="1">
         <v>46255</v>
@@ -906,19 +903,19 @@
         <v>14</v>
       </c>
       <c r="S4" t="s">
+        <v>77</v>
+      </c>
+      <c r="T4" t="s">
+        <v>77</v>
+      </c>
+      <c r="U4" t="s">
         <v>78</v>
-      </c>
-      <c r="T4" t="s">
-        <v>78</v>
-      </c>
-      <c r="U4" t="s">
-        <v>79</v>
       </c>
       <c r="V4" t="s">
         <v>84</v>
       </c>
       <c r="W4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -950,7 +947,7 @@
         <v>71</v>
       </c>
       <c r="I5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J5" s="1">
         <v>46245</v>
@@ -962,7 +959,7 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="N5" s="1">
         <v>46277</v>
@@ -977,19 +974,19 @@
         <v>12</v>
       </c>
       <c r="S5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="T5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="U5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="V5" t="s">
         <v>85</v>
       </c>
       <c r="W5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1021,7 +1018,7 @@
         <v>71</v>
       </c>
       <c r="I6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J6" s="1">
         <v>46248</v>
@@ -1033,7 +1030,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="N6" s="1">
         <v>46279</v>
@@ -1045,16 +1042,16 @@
         <v>10</v>
       </c>
       <c r="S6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="T6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="V6" t="s">
         <v>86</v>
       </c>
       <c r="W6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1086,7 +1083,7 @@
         <v>71</v>
       </c>
       <c r="I7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J7" s="1">
         <v>46248</v>
@@ -1098,7 +1095,7 @@
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="N7" s="1">
         <v>46259</v>
@@ -1110,19 +1107,19 @@
         <v>10</v>
       </c>
       <c r="S7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="T7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="U7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="V7" t="s">
         <v>87</v>
       </c>
       <c r="W7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1154,7 +1151,7 @@
         <v>71</v>
       </c>
       <c r="I8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J8" s="1">
         <v>46251</v>
@@ -1166,7 +1163,7 @@
         <v>2</v>
       </c>
       <c r="M8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="N8" s="1">
         <v>46280</v>
@@ -1178,16 +1175,16 @@
         <v>9</v>
       </c>
       <c r="S8" t="s">
+        <v>76</v>
+      </c>
+      <c r="T8" t="s">
         <v>77</v>
-      </c>
-      <c r="T8" t="s">
-        <v>78</v>
       </c>
       <c r="V8" t="s">
         <v>88</v>
       </c>
       <c r="W8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1219,7 +1216,7 @@
         <v>71</v>
       </c>
       <c r="I9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J9" s="1">
         <v>46251</v>
@@ -1231,7 +1228,7 @@
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="N9" s="1">
         <v>46282</v>
@@ -1246,16 +1243,16 @@
         <v>7</v>
       </c>
       <c r="S9" t="s">
+        <v>76</v>
+      </c>
+      <c r="T9" t="s">
         <v>77</v>
-      </c>
-      <c r="T9" t="s">
-        <v>78</v>
       </c>
       <c r="V9" t="s">
         <v>89</v>
       </c>
       <c r="W9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1287,7 +1284,7 @@
         <v>71</v>
       </c>
       <c r="I10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J10" s="1">
         <v>46253</v>
@@ -1299,7 +1296,7 @@
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="N10" s="1">
         <v>46283</v>
@@ -1311,13 +1308,13 @@
         <v>6</v>
       </c>
       <c r="S10" t="s">
+        <v>76</v>
+      </c>
+      <c r="T10" t="s">
         <v>77</v>
       </c>
-      <c r="T10" t="s">
-        <v>78</v>
-      </c>
       <c r="W10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1349,7 +1346,7 @@
         <v>71</v>
       </c>
       <c r="I11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J11" s="1">
         <v>46252</v>
@@ -1361,7 +1358,7 @@
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="N11" s="1">
         <v>46284</v>
@@ -1373,16 +1370,16 @@
         <v>5</v>
       </c>
       <c r="S11" t="s">
+        <v>76</v>
+      </c>
+      <c r="T11" t="s">
         <v>77</v>
-      </c>
-      <c r="T11" t="s">
-        <v>78</v>
       </c>
       <c r="V11" t="s">
         <v>90</v>
       </c>
       <c r="W11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1414,7 +1411,7 @@
         <v>71</v>
       </c>
       <c r="I12" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J12" s="1">
         <v>46254</v>
@@ -1426,28 +1423,31 @@
         <v>2</v>
       </c>
       <c r="M12" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="N12" s="1">
-        <v>46266</v>
+        <v>46286</v>
       </c>
       <c r="Q12">
-        <v>-8</v>
+        <v>-28</v>
       </c>
       <c r="R12">
         <v>3</v>
       </c>
       <c r="S12" t="s">
+        <v>76</v>
+      </c>
+      <c r="T12" t="s">
         <v>77</v>
       </c>
-      <c r="T12" t="s">
-        <v>78</v>
+      <c r="U12" t="s">
+        <v>81</v>
       </c>
       <c r="V12" t="s">
         <v>91</v>
       </c>
       <c r="W12" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1455,10 +1455,10 @@
     </row>
     <row r="13" spans="1:27">
       <c r="A13">
-        <v>685</v>
+        <v>329</v>
       </c>
       <c r="B13" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C13" t="s">
         <v>43</v>
@@ -1473,46 +1473,40 @@
         <v>68</v>
       </c>
       <c r="G13">
-        <v>2729</v>
+        <v>2721</v>
       </c>
       <c r="H13" t="s">
+        <v>71</v>
+      </c>
+      <c r="I13" t="s">
         <v>73</v>
       </c>
-      <c r="I13" t="s">
-        <v>75</v>
-      </c>
       <c r="J13" s="1">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="K13" s="1">
-        <v>46253</v>
+        <v>46258</v>
       </c>
       <c r="L13">
         <v>2</v>
       </c>
       <c r="M13" t="s">
+        <v>75</v>
+      </c>
+      <c r="N13" s="1">
+        <v>46289</v>
+      </c>
+      <c r="Q13">
+        <v>-31</v>
+      </c>
+      <c r="R13">
+        <v>0</v>
+      </c>
+      <c r="T13" t="s">
         <v>76</v>
       </c>
-      <c r="N13" s="1">
-        <v>46264</v>
-      </c>
-      <c r="Q13">
-        <v>-6</v>
-      </c>
-      <c r="R13">
-        <v>5</v>
-      </c>
-      <c r="S13" t="s">
-        <v>77</v>
-      </c>
-      <c r="T13" t="s">
-        <v>78</v>
-      </c>
-      <c r="V13" t="s">
+      <c r="W13" t="s">
         <v>92</v>
-      </c>
-      <c r="W13" t="s">
-        <v>93</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (24/08/2026 12:23)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -302,8 +302,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -319,7 +327,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -327,12 +335,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -632,85 +658,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -742,10 +768,10 @@
       <c r="I2" t="s">
         <v>73</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>46212</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46212</v>
       </c>
       <c r="L2">
@@ -754,10 +780,10 @@
       <c r="M2" t="s">
         <v>75</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <v>46243</v>
       </c>
-      <c r="O2" s="1">
+      <c r="O2" s="2">
         <v>46251</v>
       </c>
       <c r="Q2">
@@ -810,10 +836,10 @@
       <c r="I3" t="s">
         <v>73</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>46238</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46238</v>
       </c>
       <c r="L3">
@@ -822,10 +848,10 @@
       <c r="M3" t="s">
         <v>75</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <v>46269</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46269</v>
       </c>
       <c r="Q3">
@@ -878,10 +904,10 @@
       <c r="I4" t="s">
         <v>74</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>46244</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46244</v>
       </c>
       <c r="L4">
@@ -890,10 +916,10 @@
       <c r="M4" t="s">
         <v>75</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="2">
         <v>46255</v>
       </c>
-      <c r="O4" s="1">
+      <c r="O4" s="2">
         <v>46255</v>
       </c>
       <c r="Q4">
@@ -949,10 +975,10 @@
       <c r="I5" t="s">
         <v>73</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>46245</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46246</v>
       </c>
       <c r="L5">
@@ -961,10 +987,10 @@
       <c r="M5" t="s">
         <v>75</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <v>46277</v>
       </c>
-      <c r="O5" s="1">
+      <c r="O5" s="2">
         <v>46252</v>
       </c>
       <c r="Q5">
@@ -1020,10 +1046,10 @@
       <c r="I6" t="s">
         <v>73</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>46248</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46248</v>
       </c>
       <c r="L6">
@@ -1032,7 +1058,7 @@
       <c r="M6" t="s">
         <v>75</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <v>46279</v>
       </c>
       <c r="Q6">
@@ -1085,10 +1111,10 @@
       <c r="I7" t="s">
         <v>74</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46248</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46248</v>
       </c>
       <c r="L7">
@@ -1097,7 +1123,7 @@
       <c r="M7" t="s">
         <v>75</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="2">
         <v>46259</v>
       </c>
       <c r="Q7">
@@ -1153,10 +1179,10 @@
       <c r="I8" t="s">
         <v>73</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46251</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46249</v>
       </c>
       <c r="L8">
@@ -1165,7 +1191,7 @@
       <c r="M8" t="s">
         <v>75</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="2">
         <v>46280</v>
       </c>
       <c r="Q8">
@@ -1218,10 +1244,10 @@
       <c r="I9" t="s">
         <v>73</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46251</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46251</v>
       </c>
       <c r="L9">
@@ -1230,10 +1256,10 @@
       <c r="M9" t="s">
         <v>75</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>46282</v>
       </c>
-      <c r="O9" s="1">
+      <c r="O9" s="2">
         <v>46255</v>
       </c>
       <c r="Q9">
@@ -1286,10 +1312,10 @@
       <c r="I10" t="s">
         <v>73</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46253</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>46252</v>
       </c>
       <c r="L10">
@@ -1298,7 +1324,7 @@
       <c r="M10" t="s">
         <v>75</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
         <v>46283</v>
       </c>
       <c r="Q10">
@@ -1348,10 +1374,10 @@
       <c r="I11" t="s">
         <v>73</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46252</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>46253</v>
       </c>
       <c r="L11">
@@ -1360,7 +1386,7 @@
       <c r="M11" t="s">
         <v>75</v>
       </c>
-      <c r="N11" s="1">
+      <c r="N11" s="2">
         <v>46284</v>
       </c>
       <c r="Q11">
@@ -1413,10 +1439,10 @@
       <c r="I12" t="s">
         <v>73</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>46254</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>46255</v>
       </c>
       <c r="L12">
@@ -1425,7 +1451,7 @@
       <c r="M12" t="s">
         <v>75</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="2">
         <v>46286</v>
       </c>
       <c r="Q12">
@@ -1481,10 +1507,10 @@
       <c r="I13" t="s">
         <v>73</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46255</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>46258</v>
       </c>
       <c r="L13">
@@ -1493,7 +1519,7 @@
       <c r="M13" t="s">
         <v>75</v>
       </c>
-      <c r="N13" s="1">
+      <c r="N13" s="2">
         <v>46289</v>
       </c>
       <c r="Q13">

</xml_diff>

<commit_message>
Atualização automática: emergencias (24/08/2026 12:48)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -302,16 +302,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -327,7 +319,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -335,30 +327,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -658,85 +632,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -768,10 +742,10 @@
       <c r="I2" t="s">
         <v>73</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>46212</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46212</v>
       </c>
       <c r="L2">
@@ -780,10 +754,10 @@
       <c r="M2" t="s">
         <v>75</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="1">
         <v>46243</v>
       </c>
-      <c r="O2" s="2">
+      <c r="O2" s="1">
         <v>46251</v>
       </c>
       <c r="Q2">
@@ -836,10 +810,10 @@
       <c r="I3" t="s">
         <v>73</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>46238</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46238</v>
       </c>
       <c r="L3">
@@ -848,10 +822,10 @@
       <c r="M3" t="s">
         <v>75</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="1">
         <v>46269</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46269</v>
       </c>
       <c r="Q3">
@@ -904,10 +878,10 @@
       <c r="I4" t="s">
         <v>74</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>46244</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46244</v>
       </c>
       <c r="L4">
@@ -916,10 +890,10 @@
       <c r="M4" t="s">
         <v>75</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="1">
         <v>46255</v>
       </c>
-      <c r="O4" s="2">
+      <c r="O4" s="1">
         <v>46255</v>
       </c>
       <c r="Q4">
@@ -975,10 +949,10 @@
       <c r="I5" t="s">
         <v>73</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>46245</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46246</v>
       </c>
       <c r="L5">
@@ -987,10 +961,10 @@
       <c r="M5" t="s">
         <v>75</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="1">
         <v>46277</v>
       </c>
-      <c r="O5" s="2">
+      <c r="O5" s="1">
         <v>46252</v>
       </c>
       <c r="Q5">
@@ -1046,10 +1020,10 @@
       <c r="I6" t="s">
         <v>73</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>46248</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46248</v>
       </c>
       <c r="L6">
@@ -1058,7 +1032,7 @@
       <c r="M6" t="s">
         <v>75</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="1">
         <v>46279</v>
       </c>
       <c r="Q6">
@@ -1111,10 +1085,10 @@
       <c r="I7" t="s">
         <v>74</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46248</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>46248</v>
       </c>
       <c r="L7">
@@ -1123,7 +1097,7 @@
       <c r="M7" t="s">
         <v>75</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="1">
         <v>46259</v>
       </c>
       <c r="Q7">
@@ -1179,10 +1153,10 @@
       <c r="I8" t="s">
         <v>73</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46251</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>46249</v>
       </c>
       <c r="L8">
@@ -1191,7 +1165,7 @@
       <c r="M8" t="s">
         <v>75</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="1">
         <v>46280</v>
       </c>
       <c r="Q8">
@@ -1244,10 +1218,10 @@
       <c r="I9" t="s">
         <v>73</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46251</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>46251</v>
       </c>
       <c r="L9">
@@ -1256,10 +1230,10 @@
       <c r="M9" t="s">
         <v>75</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="1">
         <v>46282</v>
       </c>
-      <c r="O9" s="2">
+      <c r="O9" s="1">
         <v>46255</v>
       </c>
       <c r="Q9">
@@ -1312,10 +1286,10 @@
       <c r="I10" t="s">
         <v>73</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>46253</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>46252</v>
       </c>
       <c r="L10">
@@ -1324,7 +1298,7 @@
       <c r="M10" t="s">
         <v>75</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="1">
         <v>46283</v>
       </c>
       <c r="Q10">
@@ -1374,10 +1348,10 @@
       <c r="I11" t="s">
         <v>73</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46252</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>46253</v>
       </c>
       <c r="L11">
@@ -1386,7 +1360,7 @@
       <c r="M11" t="s">
         <v>75</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11" s="1">
         <v>46284</v>
       </c>
       <c r="Q11">
@@ -1439,10 +1413,10 @@
       <c r="I12" t="s">
         <v>73</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>46254</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>46255</v>
       </c>
       <c r="L12">
@@ -1451,7 +1425,7 @@
       <c r="M12" t="s">
         <v>75</v>
       </c>
-      <c r="N12" s="2">
+      <c r="N12" s="1">
         <v>46286</v>
       </c>
       <c r="Q12">
@@ -1507,10 +1481,10 @@
       <c r="I13" t="s">
         <v>73</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46255</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>46258</v>
       </c>
       <c r="L13">
@@ -1519,7 +1493,7 @@
       <c r="M13" t="s">
         <v>75</v>
       </c>
-      <c r="N13" s="2">
+      <c r="N13" s="1">
         <v>46289</v>
       </c>
       <c r="Q13">

</xml_diff>

<commit_message>
Atualização automática: emergencias (24/08/2026 14:38)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="87">
   <si>
     <t>om_emg</t>
   </si>
@@ -103,9 +103,6 @@
     <t>BABE</t>
   </si>
   <si>
-    <t>DACTA II</t>
-  </si>
-  <si>
     <t>BABR</t>
   </si>
   <si>
@@ -121,9 +118,6 @@
     <t>685260012560</t>
   </si>
   <si>
-    <t>384260009396</t>
-  </si>
-  <si>
     <t>329260019269</t>
   </si>
   <si>
@@ -157,9 +151,6 @@
     <t>2641010-3</t>
   </si>
   <si>
-    <t>S2616-285K4</t>
-  </si>
-  <si>
     <t>069-01033-0101</t>
   </si>
   <si>
@@ -193,9 +184,6 @@
     <t>AXLE FITTING</t>
   </si>
   <si>
-    <t>ALTERNAD BELT</t>
-  </si>
-  <si>
     <t>RECEIVER-TRANSMITTER</t>
   </si>
   <si>
@@ -253,9 +241,6 @@
     <t>item atendido com o estoque local pedido 18171852 em 10/08. Godoy 11/08. Está sendo definido se o PN está correto. Ramon 11/08/26.</t>
   </si>
   <si>
-    <t>Estoque no alternado 285K4. Caso use do estoque, verificar validade que consta no item. Ramon 12/08/26. Item em pane, anv autorizada a voar por 3 dias pela MMEL a contar de 12/08. Ramon 13/08/26</t>
-  </si>
-  <si>
     <t>Estoque alterado de "Nao" para "SIM"  daremos prioridade para movimentar o item.  Godoy 17/08/226</t>
   </si>
   <si>
@@ -269,9 +254,6 @@
   </si>
   <si>
     <t>Foi solicitado atendimento com estoque FAB - CLA- 10-08, ITEM PRONTO PARA EMBARQUE, AGUARDANDO NOTA FISCAL - CLA-11-08- ITEM AGUARDANDO DEFINIÇÃO DA COORDENADORIA QUANTO A EFETIVIDADE PARA APLICAÇÃO NA REFERIDA ANV.- CLA-13-08 - AT 685000002258</t>
-  </si>
-  <si>
-    <t>Temos no STK V1, material em separação, recibo 682/FAB/26 - atz rc 13/08 - MATERIAL ENVIADO VIA AWB 12752709016 - DPE 18/08/2026 - ENTREGUE DIA 18/08/2026</t>
   </si>
   <si>
     <t>foi solicitoado o atendimento com o estoque FAB. CLA-17-08 - o item PN superado 069-1025-25 não serve na ANV 2721 - temos 4ea na wiliam para reparo, já foi solicitado o DPE - OS 4 ITENS ESTÃO COM PROBLEMAS NO DISPAY. -FOI ENVIADO PARA O WIILIAM MAIS 3 UNS PARA REPARO - AINDA SEM DPE -CLA-20-08</t>
@@ -628,7 +610,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA13"/>
+  <dimension ref="A1:AA12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -722,25 +704,25 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F2" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="G2">
         <v>2702</v>
       </c>
       <c r="H2" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="I2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J2" s="1">
         <v>46212</v>
@@ -752,7 +734,7 @@
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="N2" s="1">
         <v>46243</v>
@@ -767,16 +749,16 @@
         <v>46</v>
       </c>
       <c r="S2" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="T2" t="s">
+        <v>73</v>
+      </c>
+      <c r="V2" t="s">
         <v>77</v>
       </c>
-      <c r="V2" t="s">
-        <v>82</v>
-      </c>
       <c r="W2" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -790,25 +772,25 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E3" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="F3" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="G3">
         <v>2733</v>
       </c>
       <c r="H3" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="I3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J3" s="1">
         <v>46238</v>
@@ -820,7 +802,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="N3" s="1">
         <v>46269</v>
@@ -835,16 +817,16 @@
         <v>20</v>
       </c>
       <c r="S3" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="T3" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="V3" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="W3" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -858,25 +840,25 @@
         <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="F4" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="G4">
         <v>2729</v>
       </c>
       <c r="H4" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="I4" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="J4" s="1">
         <v>46244</v>
@@ -888,7 +870,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="N4" s="1">
         <v>46255</v>
@@ -903,19 +885,19 @@
         <v>14</v>
       </c>
       <c r="S4" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="T4" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="U4" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="V4" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="W4" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -923,70 +905,64 @@
     </row>
     <row r="5" spans="1:27">
       <c r="A5">
-        <v>384</v>
+        <v>329</v>
       </c>
       <c r="B5" t="s">
         <v>29</v>
       </c>
       <c r="C5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E5" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G5">
-        <v>2742</v>
+        <v>2721</v>
       </c>
       <c r="H5" t="s">
+        <v>67</v>
+      </c>
+      <c r="I5" t="s">
+        <v>69</v>
+      </c>
+      <c r="J5" s="1">
+        <v>46248</v>
+      </c>
+      <c r="K5" s="1">
+        <v>46248</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5" t="s">
         <v>71</v>
       </c>
-      <c r="I5" t="s">
+      <c r="N5" s="1">
+        <v>46279</v>
+      </c>
+      <c r="Q5">
+        <v>-21</v>
+      </c>
+      <c r="R5">
+        <v>10</v>
+      </c>
+      <c r="S5" t="s">
         <v>73</v>
       </c>
-      <c r="J5" s="1">
-        <v>46245</v>
-      </c>
-      <c r="K5" s="1">
-        <v>46246</v>
-      </c>
-      <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5" t="s">
-        <v>75</v>
-      </c>
-      <c r="N5" s="1">
-        <v>46277</v>
-      </c>
-      <c r="O5" s="1">
-        <v>46252</v>
-      </c>
-      <c r="Q5">
-        <v>-19</v>
-      </c>
-      <c r="R5">
-        <v>12</v>
-      </c>
-      <c r="S5" t="s">
-        <v>77</v>
-      </c>
       <c r="T5" t="s">
-        <v>76</v>
-      </c>
-      <c r="U5" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="V5" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="W5" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -994,31 +970,31 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E6" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="F6" t="s">
+        <v>65</v>
+      </c>
+      <c r="G6">
+        <v>2729</v>
+      </c>
+      <c r="H6" t="s">
+        <v>67</v>
+      </c>
+      <c r="I6" t="s">
         <v>70</v>
-      </c>
-      <c r="G6">
-        <v>2721</v>
-      </c>
-      <c r="H6" t="s">
-        <v>71</v>
-      </c>
-      <c r="I6" t="s">
-        <v>73</v>
       </c>
       <c r="J6" s="1">
         <v>46248</v>
@@ -1030,28 +1006,31 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="N6" s="1">
-        <v>46279</v>
+        <v>46259</v>
       </c>
       <c r="Q6">
-        <v>-21</v>
+        <v>-1</v>
       </c>
       <c r="R6">
         <v>10</v>
       </c>
       <c r="S6" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="T6" t="s">
-        <v>76</v>
+        <v>73</v>
+      </c>
+      <c r="U6" t="s">
+        <v>75</v>
       </c>
       <c r="V6" t="s">
+        <v>81</v>
+      </c>
+      <c r="W6" t="s">
         <v>86</v>
-      </c>
-      <c r="W6" t="s">
-        <v>92</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1059,67 +1038,64 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E7" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="F7" t="s">
+        <v>64</v>
+      </c>
+      <c r="G7">
+        <v>2741</v>
+      </c>
+      <c r="H7" t="s">
+        <v>67</v>
+      </c>
+      <c r="I7" t="s">
         <v>69</v>
       </c>
-      <c r="G7">
-        <v>2729</v>
-      </c>
-      <c r="H7" t="s">
+      <c r="J7" s="1">
+        <v>46251</v>
+      </c>
+      <c r="K7" s="1">
+        <v>46249</v>
+      </c>
+      <c r="L7">
+        <v>2</v>
+      </c>
+      <c r="M7" t="s">
         <v>71</v>
       </c>
-      <c r="I7" t="s">
-        <v>74</v>
-      </c>
-      <c r="J7" s="1">
-        <v>46248</v>
-      </c>
-      <c r="K7" s="1">
-        <v>46248</v>
-      </c>
-      <c r="L7">
-        <v>1</v>
-      </c>
-      <c r="M7" t="s">
-        <v>75</v>
-      </c>
       <c r="N7" s="1">
-        <v>46259</v>
+        <v>46280</v>
       </c>
       <c r="Q7">
-        <v>-1</v>
+        <v>-22</v>
       </c>
       <c r="R7">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="S7" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="T7" t="s">
-        <v>77</v>
-      </c>
-      <c r="U7" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="V7" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="W7" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1127,64 +1103,67 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B8" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D8" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E8" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="F8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G8">
-        <v>2741</v>
+        <v>2729</v>
       </c>
       <c r="H8" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="I8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J8" s="1">
         <v>46251</v>
       </c>
       <c r="K8" s="1">
-        <v>46249</v>
+        <v>46251</v>
       </c>
       <c r="L8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="N8" s="1">
-        <v>46280</v>
+        <v>46282</v>
+      </c>
+      <c r="O8" s="1">
+        <v>46255</v>
       </c>
       <c r="Q8">
-        <v>-22</v>
+        <v>-24</v>
       </c>
       <c r="R8">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="S8" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="T8" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="V8" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="W8" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1192,67 +1171,61 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B9" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E9" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="F9" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="G9">
-        <v>2729</v>
+        <v>2741</v>
       </c>
       <c r="H9" t="s">
+        <v>67</v>
+      </c>
+      <c r="I9" t="s">
+        <v>69</v>
+      </c>
+      <c r="J9" s="1">
+        <v>46253</v>
+      </c>
+      <c r="K9" s="1">
+        <v>46252</v>
+      </c>
+      <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9" t="s">
         <v>71</v>
       </c>
-      <c r="I9" t="s">
+      <c r="N9" s="1">
+        <v>46283</v>
+      </c>
+      <c r="Q9">
+        <v>-25</v>
+      </c>
+      <c r="R9">
+        <v>6</v>
+      </c>
+      <c r="S9" t="s">
+        <v>72</v>
+      </c>
+      <c r="T9" t="s">
         <v>73</v>
       </c>
-      <c r="J9" s="1">
-        <v>46251</v>
-      </c>
-      <c r="K9" s="1">
-        <v>46251</v>
-      </c>
-      <c r="L9">
-        <v>1</v>
-      </c>
-      <c r="M9" t="s">
-        <v>75</v>
-      </c>
-      <c r="N9" s="1">
-        <v>46282</v>
-      </c>
-      <c r="O9" s="1">
-        <v>46255</v>
-      </c>
-      <c r="Q9">
-        <v>-24</v>
-      </c>
-      <c r="R9">
-        <v>7</v>
-      </c>
-      <c r="S9" t="s">
-        <v>76</v>
-      </c>
-      <c r="T9" t="s">
-        <v>77</v>
-      </c>
-      <c r="V9" t="s">
-        <v>89</v>
-      </c>
       <c r="W9" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1260,61 +1233,64 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>313</v>
+        <v>396</v>
       </c>
       <c r="B10" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D10" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E10" t="s">
+        <v>61</v>
+      </c>
+      <c r="F10" t="s">
         <v>64</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10">
+        <v>2731</v>
+      </c>
+      <c r="H10" t="s">
+        <v>67</v>
+      </c>
+      <c r="I10" t="s">
         <v>69</v>
       </c>
-      <c r="G10">
-        <v>2741</v>
-      </c>
-      <c r="H10" t="s">
+      <c r="J10" s="1">
+        <v>46252</v>
+      </c>
+      <c r="K10" s="1">
+        <v>46253</v>
+      </c>
+      <c r="L10">
+        <v>1</v>
+      </c>
+      <c r="M10" t="s">
         <v>71</v>
       </c>
-      <c r="I10" t="s">
+      <c r="N10" s="1">
+        <v>46284</v>
+      </c>
+      <c r="Q10">
+        <v>-26</v>
+      </c>
+      <c r="R10">
+        <v>5</v>
+      </c>
+      <c r="S10" t="s">
+        <v>72</v>
+      </c>
+      <c r="T10" t="s">
         <v>73</v>
       </c>
-      <c r="J10" s="1">
-        <v>46253</v>
-      </c>
-      <c r="K10" s="1">
-        <v>46252</v>
-      </c>
-      <c r="L10">
-        <v>1</v>
-      </c>
-      <c r="M10" t="s">
-        <v>75</v>
-      </c>
-      <c r="N10" s="1">
-        <v>46283</v>
-      </c>
-      <c r="Q10">
-        <v>-25</v>
-      </c>
-      <c r="R10">
-        <v>6</v>
-      </c>
-      <c r="S10" t="s">
-        <v>76</v>
-      </c>
-      <c r="T10" t="s">
-        <v>77</v>
+      <c r="V10" t="s">
+        <v>84</v>
       </c>
       <c r="W10" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1322,64 +1298,67 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>396</v>
+        <v>313</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D11" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E11" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F11" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="G11">
-        <v>2731</v>
+        <v>2737</v>
       </c>
       <c r="H11" t="s">
+        <v>67</v>
+      </c>
+      <c r="I11" t="s">
+        <v>69</v>
+      </c>
+      <c r="J11" s="1">
+        <v>46254</v>
+      </c>
+      <c r="K11" s="1">
+        <v>46255</v>
+      </c>
+      <c r="L11">
+        <v>2</v>
+      </c>
+      <c r="M11" t="s">
         <v>71</v>
       </c>
-      <c r="I11" t="s">
+      <c r="N11" s="1">
+        <v>46286</v>
+      </c>
+      <c r="Q11">
+        <v>-28</v>
+      </c>
+      <c r="R11">
+        <v>3</v>
+      </c>
+      <c r="S11" t="s">
+        <v>72</v>
+      </c>
+      <c r="T11" t="s">
         <v>73</v>
       </c>
-      <c r="J11" s="1">
-        <v>46252</v>
-      </c>
-      <c r="K11" s="1">
-        <v>46253</v>
-      </c>
-      <c r="L11">
-        <v>1</v>
-      </c>
-      <c r="M11" t="s">
-        <v>75</v>
-      </c>
-      <c r="N11" s="1">
-        <v>46284</v>
-      </c>
-      <c r="Q11">
-        <v>-26</v>
-      </c>
-      <c r="R11">
-        <v>5</v>
-      </c>
-      <c r="S11" t="s">
+      <c r="U11" t="s">
         <v>76</v>
       </c>
-      <c r="T11" t="s">
-        <v>77</v>
-      </c>
       <c r="V11" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="W11" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1387,128 +1366,60 @@
     </row>
     <row r="12" spans="1:27">
       <c r="A12">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B12" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D12" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E12" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="F12" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="G12">
-        <v>2737</v>
+        <v>2721</v>
       </c>
       <c r="H12" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="I12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J12" s="1">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="K12" s="1">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="L12">
         <v>2</v>
       </c>
       <c r="M12" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="N12" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="Q12">
-        <v>-28</v>
+        <v>-31</v>
       </c>
       <c r="R12">
-        <v>3</v>
-      </c>
-      <c r="S12" t="s">
-        <v>76</v>
+        <v>0</v>
       </c>
       <c r="T12" t="s">
-        <v>77</v>
-      </c>
-      <c r="U12" t="s">
-        <v>81</v>
-      </c>
-      <c r="V12" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="W12" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="AA12" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:27">
-      <c r="A13">
-        <v>329</v>
-      </c>
-      <c r="B13" t="s">
-        <v>30</v>
-      </c>
-      <c r="C13" t="s">
-        <v>43</v>
-      </c>
-      <c r="D13" t="s">
-        <v>55</v>
-      </c>
-      <c r="E13" t="s">
-        <v>67</v>
-      </c>
-      <c r="F13" t="s">
-        <v>68</v>
-      </c>
-      <c r="G13">
-        <v>2721</v>
-      </c>
-      <c r="H13" t="s">
-        <v>71</v>
-      </c>
-      <c r="I13" t="s">
-        <v>73</v>
-      </c>
-      <c r="J13" s="1">
-        <v>46255</v>
-      </c>
-      <c r="K13" s="1">
-        <v>46258</v>
-      </c>
-      <c r="L13">
-        <v>2</v>
-      </c>
-      <c r="M13" t="s">
-        <v>75</v>
-      </c>
-      <c r="N13" s="1">
-        <v>46289</v>
-      </c>
-      <c r="Q13">
-        <v>-31</v>
-      </c>
-      <c r="R13">
-        <v>0</v>
-      </c>
-      <c r="T13" t="s">
-        <v>76</v>
-      </c>
-      <c r="W13" t="s">
-        <v>92</v>
-      </c>
-      <c r="AA13" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (24/08/2026 18:37)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -284,16 +284,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -309,7 +301,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -317,30 +309,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -640,85 +614,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -750,10 +724,10 @@
       <c r="I2" t="s">
         <v>69</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>46212</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46212</v>
       </c>
       <c r="L2">
@@ -762,10 +736,10 @@
       <c r="M2" t="s">
         <v>71</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="1">
         <v>46243</v>
       </c>
-      <c r="O2" s="2">
+      <c r="O2" s="1">
         <v>46251</v>
       </c>
       <c r="Q2">
@@ -818,10 +792,10 @@
       <c r="I3" t="s">
         <v>69</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>46238</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46238</v>
       </c>
       <c r="L3">
@@ -830,10 +804,10 @@
       <c r="M3" t="s">
         <v>71</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="1">
         <v>46269</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46269</v>
       </c>
       <c r="Q3">
@@ -886,10 +860,10 @@
       <c r="I4" t="s">
         <v>70</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>46244</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46244</v>
       </c>
       <c r="L4">
@@ -898,10 +872,10 @@
       <c r="M4" t="s">
         <v>71</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="1">
         <v>46255</v>
       </c>
-      <c r="O4" s="2">
+      <c r="O4" s="1">
         <v>46255</v>
       </c>
       <c r="Q4">
@@ -957,10 +931,10 @@
       <c r="I5" t="s">
         <v>69</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>46248</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46248</v>
       </c>
       <c r="L5">
@@ -969,7 +943,7 @@
       <c r="M5" t="s">
         <v>71</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="1">
         <v>46279</v>
       </c>
       <c r="Q5">
@@ -1022,10 +996,10 @@
       <c r="I6" t="s">
         <v>70</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>46248</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46248</v>
       </c>
       <c r="L6">
@@ -1034,7 +1008,7 @@
       <c r="M6" t="s">
         <v>71</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="1">
         <v>46259</v>
       </c>
       <c r="Q6">
@@ -1090,10 +1064,10 @@
       <c r="I7" t="s">
         <v>69</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46251</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>46249</v>
       </c>
       <c r="L7">
@@ -1102,7 +1076,7 @@
       <c r="M7" t="s">
         <v>71</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="1">
         <v>46280</v>
       </c>
       <c r="Q7">
@@ -1155,10 +1129,10 @@
       <c r="I8" t="s">
         <v>69</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46251</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>46251</v>
       </c>
       <c r="L8">
@@ -1167,10 +1141,10 @@
       <c r="M8" t="s">
         <v>71</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="1">
         <v>46282</v>
       </c>
-      <c r="O8" s="2">
+      <c r="O8" s="1">
         <v>46255</v>
       </c>
       <c r="Q8">
@@ -1223,10 +1197,10 @@
       <c r="I9" t="s">
         <v>69</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46253</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>46252</v>
       </c>
       <c r="L9">
@@ -1235,7 +1209,7 @@
       <c r="M9" t="s">
         <v>71</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="1">
         <v>46283</v>
       </c>
       <c r="Q9">
@@ -1285,10 +1259,10 @@
       <c r="I10" t="s">
         <v>69</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>46252</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>46253</v>
       </c>
       <c r="L10">
@@ -1297,7 +1271,7 @@
       <c r="M10" t="s">
         <v>71</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="1">
         <v>46284</v>
       </c>
       <c r="Q10">
@@ -1350,10 +1324,10 @@
       <c r="I11" t="s">
         <v>69</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46254</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>46255</v>
       </c>
       <c r="L11">
@@ -1362,7 +1336,7 @@
       <c r="M11" t="s">
         <v>71</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11" s="1">
         <v>46286</v>
       </c>
       <c r="Q11">
@@ -1418,10 +1392,10 @@
       <c r="I12" t="s">
         <v>69</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>46255</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>46258</v>
       </c>
       <c r="L12">
@@ -1430,7 +1404,7 @@
       <c r="M12" t="s">
         <v>71</v>
       </c>
-      <c r="N12" s="2">
+      <c r="N12" s="1">
         <v>46289</v>
       </c>
       <c r="Q12">

</xml_diff>

<commit_message>
Atualização automática: emergencias (25/08/2026 08:30)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -284,8 +284,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -301,7 +309,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -309,12 +317,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -614,85 +640,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -724,10 +750,10 @@
       <c r="I2" t="s">
         <v>69</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>46212</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46212</v>
       </c>
       <c r="L2">
@@ -736,17 +762,17 @@
       <c r="M2" t="s">
         <v>71</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <v>46243</v>
       </c>
-      <c r="O2" s="1">
+      <c r="O2" s="2">
         <v>46251</v>
       </c>
       <c r="Q2">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="R2">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="S2" t="s">
         <v>72</v>
@@ -792,10 +818,10 @@
       <c r="I3" t="s">
         <v>69</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>46238</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46238</v>
       </c>
       <c r="L3">
@@ -804,17 +830,17 @@
       <c r="M3" t="s">
         <v>71</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <v>46269</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46269</v>
       </c>
       <c r="Q3">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R3">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="S3" t="s">
         <v>72</v>
@@ -860,10 +886,10 @@
       <c r="I4" t="s">
         <v>70</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>46244</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46244</v>
       </c>
       <c r="L4">
@@ -872,17 +898,17 @@
       <c r="M4" t="s">
         <v>71</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="2">
         <v>46255</v>
       </c>
-      <c r="O4" s="1">
+      <c r="O4" s="2">
         <v>46255</v>
       </c>
       <c r="Q4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R4">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S4" t="s">
         <v>73</v>
@@ -931,10 +957,10 @@
       <c r="I5" t="s">
         <v>69</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>46248</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46248</v>
       </c>
       <c r="L5">
@@ -943,14 +969,14 @@
       <c r="M5" t="s">
         <v>71</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <v>46279</v>
       </c>
       <c r="Q5">
-        <v>-21</v>
+        <v>-20</v>
       </c>
       <c r="R5">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S5" t="s">
         <v>73</v>
@@ -996,10 +1022,10 @@
       <c r="I6" t="s">
         <v>70</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>46248</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46248</v>
       </c>
       <c r="L6">
@@ -1008,14 +1034,14 @@
       <c r="M6" t="s">
         <v>71</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <v>46259</v>
       </c>
       <c r="Q6">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R6">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S6" t="s">
         <v>73</v>
@@ -1064,10 +1090,10 @@
       <c r="I7" t="s">
         <v>69</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46251</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46249</v>
       </c>
       <c r="L7">
@@ -1076,14 +1102,14 @@
       <c r="M7" t="s">
         <v>71</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="2">
         <v>46280</v>
       </c>
       <c r="Q7">
-        <v>-22</v>
+        <v>-21</v>
       </c>
       <c r="R7">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="S7" t="s">
         <v>72</v>
@@ -1129,10 +1155,10 @@
       <c r="I8" t="s">
         <v>69</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46251</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46251</v>
       </c>
       <c r="L8">
@@ -1141,17 +1167,17 @@
       <c r="M8" t="s">
         <v>71</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="2">
         <v>46282</v>
       </c>
-      <c r="O8" s="1">
+      <c r="O8" s="2">
         <v>46255</v>
       </c>
       <c r="Q8">
-        <v>-24</v>
+        <v>-23</v>
       </c>
       <c r="R8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S8" t="s">
         <v>72</v>
@@ -1197,10 +1223,10 @@
       <c r="I9" t="s">
         <v>69</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46253</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46252</v>
       </c>
       <c r="L9">
@@ -1209,14 +1235,14 @@
       <c r="M9" t="s">
         <v>71</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>46283</v>
       </c>
       <c r="Q9">
-        <v>-25</v>
+        <v>-24</v>
       </c>
       <c r="R9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S9" t="s">
         <v>72</v>
@@ -1259,10 +1285,10 @@
       <c r="I10" t="s">
         <v>69</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46252</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>46253</v>
       </c>
       <c r="L10">
@@ -1271,14 +1297,14 @@
       <c r="M10" t="s">
         <v>71</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
         <v>46284</v>
       </c>
       <c r="Q10">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="R10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S10" t="s">
         <v>72</v>
@@ -1324,10 +1350,10 @@
       <c r="I11" t="s">
         <v>69</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46254</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>46255</v>
       </c>
       <c r="L11">
@@ -1336,14 +1362,14 @@
       <c r="M11" t="s">
         <v>71</v>
       </c>
-      <c r="N11" s="1">
+      <c r="N11" s="2">
         <v>46286</v>
       </c>
       <c r="Q11">
-        <v>-28</v>
+        <v>-27</v>
       </c>
       <c r="R11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S11" t="s">
         <v>72</v>
@@ -1392,10 +1418,10 @@
       <c r="I12" t="s">
         <v>69</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>46255</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>46258</v>
       </c>
       <c r="L12">
@@ -1404,14 +1430,14 @@
       <c r="M12" t="s">
         <v>71</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="2">
         <v>46289</v>
       </c>
       <c r="Q12">
-        <v>-31</v>
+        <v>-30</v>
       </c>
       <c r="R12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T12" t="s">
         <v>72</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (25/08/2026 08:36)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -284,16 +284,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -309,7 +301,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -317,30 +309,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -640,85 +614,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -750,10 +724,10 @@
       <c r="I2" t="s">
         <v>69</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>46212</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46212</v>
       </c>
       <c r="L2">
@@ -762,10 +736,10 @@
       <c r="M2" t="s">
         <v>71</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="1">
         <v>46243</v>
       </c>
-      <c r="O2" s="2">
+      <c r="O2" s="1">
         <v>46251</v>
       </c>
       <c r="Q2">
@@ -818,10 +792,10 @@
       <c r="I3" t="s">
         <v>69</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>46238</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46238</v>
       </c>
       <c r="L3">
@@ -830,10 +804,10 @@
       <c r="M3" t="s">
         <v>71</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="1">
         <v>46269</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46269</v>
       </c>
       <c r="Q3">
@@ -886,10 +860,10 @@
       <c r="I4" t="s">
         <v>70</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>46244</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46244</v>
       </c>
       <c r="L4">
@@ -898,10 +872,10 @@
       <c r="M4" t="s">
         <v>71</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="1">
         <v>46255</v>
       </c>
-      <c r="O4" s="2">
+      <c r="O4" s="1">
         <v>46255</v>
       </c>
       <c r="Q4">
@@ -957,10 +931,10 @@
       <c r="I5" t="s">
         <v>69</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>46248</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46248</v>
       </c>
       <c r="L5">
@@ -969,7 +943,7 @@
       <c r="M5" t="s">
         <v>71</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="1">
         <v>46279</v>
       </c>
       <c r="Q5">
@@ -1022,10 +996,10 @@
       <c r="I6" t="s">
         <v>70</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>46248</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46248</v>
       </c>
       <c r="L6">
@@ -1034,7 +1008,7 @@
       <c r="M6" t="s">
         <v>71</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="1">
         <v>46259</v>
       </c>
       <c r="Q6">
@@ -1090,10 +1064,10 @@
       <c r="I7" t="s">
         <v>69</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46251</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>46249</v>
       </c>
       <c r="L7">
@@ -1102,7 +1076,7 @@
       <c r="M7" t="s">
         <v>71</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="1">
         <v>46280</v>
       </c>
       <c r="Q7">
@@ -1155,10 +1129,10 @@
       <c r="I8" t="s">
         <v>69</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46251</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>46251</v>
       </c>
       <c r="L8">
@@ -1167,10 +1141,10 @@
       <c r="M8" t="s">
         <v>71</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="1">
         <v>46282</v>
       </c>
-      <c r="O8" s="2">
+      <c r="O8" s="1">
         <v>46255</v>
       </c>
       <c r="Q8">
@@ -1223,10 +1197,10 @@
       <c r="I9" t="s">
         <v>69</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46253</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>46252</v>
       </c>
       <c r="L9">
@@ -1235,7 +1209,7 @@
       <c r="M9" t="s">
         <v>71</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="1">
         <v>46283</v>
       </c>
       <c r="Q9">
@@ -1285,10 +1259,10 @@
       <c r="I10" t="s">
         <v>69</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>46252</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>46253</v>
       </c>
       <c r="L10">
@@ -1297,7 +1271,7 @@
       <c r="M10" t="s">
         <v>71</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="1">
         <v>46284</v>
       </c>
       <c r="Q10">
@@ -1350,10 +1324,10 @@
       <c r="I11" t="s">
         <v>69</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46254</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>46255</v>
       </c>
       <c r="L11">
@@ -1362,7 +1336,7 @@
       <c r="M11" t="s">
         <v>71</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11" s="1">
         <v>46286</v>
       </c>
       <c r="Q11">
@@ -1418,10 +1392,10 @@
       <c r="I12" t="s">
         <v>69</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>46255</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>46258</v>
       </c>
       <c r="L12">
@@ -1430,7 +1404,7 @@
       <c r="M12" t="s">
         <v>71</v>
       </c>
-      <c r="N12" s="2">
+      <c r="N12" s="1">
         <v>46289</v>
       </c>
       <c r="Q12">

</xml_diff>

<commit_message>
Atualização automática: emergencias (25/08/2026 10:56)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="89">
   <si>
     <t>om_emg</t>
   </si>
@@ -244,10 +244,13 @@
     <t>Estoque alterado de "Nao" para "SIM"  daremos prioridade para movimentar o item.  Godoy 17/08/226</t>
   </si>
   <si>
+    <t>AWB 12754088775 - volume retirado na loja GOLLOG - NAT por Teodoro silva em 22/08. Godoy 25/08/26.</t>
+  </si>
+  <si>
     <t>Emergência transformada em ANCE em 24/08. Aguardaremos atendimento com item da Vee One. Ramon 24/08/26.</t>
   </si>
   <si>
-    <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Chegada GIG dia 15-08 (voo 4273). Entregue V1 JPA 17/08</t>
+    <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Chegada GIG dia 15-08 (voo 4273). Entregue V1 JPA 17/08 - MATERIAL EM TRANSITO - RECIBO 722/FAB/26 DPE 24/08/2026</t>
   </si>
   <si>
     <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
@@ -256,22 +259,25 @@
     <t>Foi solicitado atendimento com estoque FAB - CLA- 10-08, ITEM PRONTO PARA EMBARQUE, AGUARDANDO NOTA FISCAL - CLA-11-08- ITEM AGUARDANDO DEFINIÇÃO DA COORDENADORIA QUANTO A EFETIVIDADE PARA APLICAÇÃO NA REFERIDA ANV.- CLA-13-08 - AT 685000002258</t>
   </si>
   <si>
-    <t>foi solicitoado o atendimento com o estoque FAB. CLA-17-08 - o item PN superado 069-1025-25 não serve na ANV 2721 - temos 4ea na wiliam para reparo, já foi solicitado o DPE - OS 4 ITENS ESTÃO COM PROBLEMAS NO DISPAY. -FOI ENVIADO PARA O WIILIAM MAIS 3 UNS PARA REPARO - AINDA SEM DPE -CLA-20-08</t>
-  </si>
-  <si>
-    <t>ITEM FOI ENTREGUE PARA A FAB VIA RECIBO 598/FAB/26 31-07-26 - AINDA NÃO FOI PARA O ESTOQUECLA-17-08</t>
-  </si>
-  <si>
-    <t>pedido no EPM E-C98-26061 -CLA-18-08 - em cotação no mercado. Validar se os alternados PN A-7512-24 ou MS25309-7512 ou M6363/2-2 atendem</t>
-  </si>
-  <si>
-    <t>DPE DA WILLIAM DIA 20-08-2026 -CLA-18-08 -ENTREGUE NA BASE DO PAMALS 1 EA , SERÁ ENVIAO AO OPERADOR- CLA-20-08 - AWB127-5408 8775- CLA-21-08</t>
-  </si>
-  <si>
-    <t>Colocado pedido Textron WB0003128625 - tracking 535477333011 - previsão de entrega 24/08</t>
+    <t>Enviado para o Operador em 24/08/26 - AWB 127-5459 2764 - REZ 24/08/26</t>
+  </si>
+  <si>
+    <t>ITEM FOI ENTREGUE PARA A FAB VIA RECIBO 598/FAB/26 31-07-26 - AINDA NÃO FOI PARA O ESTOQUECLA-17-08 - material enviado via awb 12754592764, DPE 25/08/2026</t>
+  </si>
+  <si>
+    <t>Colocado pedido no fornecedor WAGA INTERNATIONAL - aguardando proforma invoice para pagamento. ATZ 21/08</t>
+  </si>
+  <si>
+    <t>DPE DA WILLIAM DIA 20-08-2026 -CLA-18-08 -ENTREGUE NA BASE DO PAMALS 1 EA , SERÁ ENVIAO AO OPERADOR- CLA-20-08 - AWB 12754088775 - CLA-21-08</t>
+  </si>
+  <si>
+    <t>Colocado pedido Textron WB0003128625 - tracking 535477333011 - previsão de entrega 24/08 V1 JPA</t>
   </si>
   <si>
     <t>Colocado pedido no fornecedor S624333 - validando entrega em Miami - TEMOS 3 EA NO ESTOQUE DA BANT</t>
+  </si>
+  <si>
+    <t>Material enviado via recibo 720/FAB/26 DPE 24/08/2026</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -755,10 +761,10 @@
         <v>73</v>
       </c>
       <c r="V2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="W2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -823,10 +829,10 @@
         <v>73</v>
       </c>
       <c r="V3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="W3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -894,10 +900,10 @@
         <v>74</v>
       </c>
       <c r="V4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="W4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -959,10 +965,10 @@
         <v>72</v>
       </c>
       <c r="V5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="W5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1011,6 +1017,9 @@
       <c r="N6" s="1">
         <v>46259</v>
       </c>
+      <c r="O6" s="1">
+        <v>46259</v>
+      </c>
       <c r="Q6">
         <v>0</v>
       </c>
@@ -1027,10 +1036,10 @@
         <v>75</v>
       </c>
       <c r="V6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="W6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1092,10 +1101,10 @@
         <v>73</v>
       </c>
       <c r="V7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="W7" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1159,11 +1168,14 @@
       <c r="T8" t="s">
         <v>73</v>
       </c>
+      <c r="U8" t="s">
+        <v>76</v>
+      </c>
       <c r="V8" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="W8" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1225,7 +1237,7 @@
         <v>73</v>
       </c>
       <c r="W9" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1287,10 +1299,10 @@
         <v>73</v>
       </c>
       <c r="V10" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="W10" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1352,13 +1364,13 @@
         <v>73</v>
       </c>
       <c r="U11" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="V11" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="W11" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1407,17 +1419,26 @@
       <c r="N12" s="1">
         <v>46289</v>
       </c>
+      <c r="O12" s="1">
+        <v>46258</v>
+      </c>
       <c r="Q12">
         <v>-30</v>
       </c>
       <c r="R12">
         <v>1</v>
       </c>
+      <c r="S12" t="s">
+        <v>73</v>
+      </c>
       <c r="T12" t="s">
         <v>72</v>
       </c>
+      <c r="V12" t="s">
+        <v>87</v>
+      </c>
       <c r="W12" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (26/08/2026 08:37)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -250,34 +250,34 @@
     <t>Emergência transformada em ANCE em 24/08. Aguardaremos atendimento com item da Vee One. Ramon 24/08/26.</t>
   </si>
   <si>
-    <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Chegada GIG dia 15-08 (voo 4273). Entregue V1 JPA 17/08 - MATERIAL EM TRANSITO - RECIBO 722/FAB/26 DPE 24/08/2026</t>
+    <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Chegada GIG dia 15-08 (voo 4273). Entregue V1 JPA 17/08 - MATERIAL EM TRANSITO - RECIBO 722/FAB/26</t>
   </si>
   <si>
     <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
   </si>
   <si>
-    <t>Foi solicitado atendimento com estoque FAB - CLA- 10-08, ITEM PRONTO PARA EMBARQUE, AGUARDANDO NOTA FISCAL - CLA-11-08- ITEM AGUARDANDO DEFINIÇÃO DA COORDENADORIA QUANTO A EFETIVIDADE PARA APLICAÇÃO NA REFERIDA ANV.- CLA-13-08 - AT 685000002258</t>
+    <t>Foi solicitado atendimento com estoque FAB - CLA- 10-08, ITEM PRONTO PARA EMBARQUE, AGUARDANDO NOTA FISCAL - CLA-11-08- ITEM AGUARDANDO DEFINIÇÃO DA COORDENADORIA QUANTO A EFETIVIDADE PARA APLICAÇÃO NA REFERIDA ANV.- CLA-13-08 - AT 685000002258. Conforme relatado pela Coordenadoria, foi enviado, via CAN, um item novo, PN 2641010-3. Dessa forma, o item que atualmente se encontra em poder da VeeOne deverá ser estornado ao estoque.CLA-25-08</t>
   </si>
   <si>
     <t>Enviado para o Operador em 24/08/26 - AWB 127-5459 2764 - REZ 24/08/26</t>
   </si>
   <si>
-    <t>ITEM FOI ENTREGUE PARA A FAB VIA RECIBO 598/FAB/26 31-07-26 - AINDA NÃO FOI PARA O ESTOQUECLA-17-08 - material enviado via awb 12754592764, DPE 25/08/2026</t>
-  </si>
-  <si>
-    <t>Colocado pedido no fornecedor WAGA INTERNATIONAL - aguardando proforma invoice para pagamento. ATZ 21/08</t>
-  </si>
-  <si>
-    <t>DPE DA WILLIAM DIA 20-08-2026 -CLA-18-08 -ENTREGUE NA BASE DO PAMALS 1 EA , SERÁ ENVIAO AO OPERADOR- CLA-20-08 - AWB 12754088775 - CLA-21-08</t>
-  </si>
-  <si>
-    <t>Colocado pedido Textron WB0003128625 - tracking 535477333011 - previsão de entrega 24/08 V1 JPA</t>
-  </si>
-  <si>
-    <t>Colocado pedido no fornecedor S624333 - validando entrega em Miami - TEMOS 3 EA NO ESTOQUE DA BANT</t>
-  </si>
-  <si>
-    <t>Material enviado via recibo 720/FAB/26 DPE 24/08/2026</t>
+    <t>ITEM FOI ENTREGUE PARA A FAB PAMALS VIA RECIBO 598/FAB/26 31-07-26 - AINDA NÃO FOI PARA O ESTOQUE CLA-17-08 - Aguardando autorização para movimentação a BANT 25/08/2026</t>
+  </si>
+  <si>
+    <t>Colocado pedido no fornecedor WAGA INTERNATIONAL - validando previsão de entrega em Miami. ATZ 25/08</t>
+  </si>
+  <si>
+    <t>DPE DA WILLIAM DIA 20-08-2026 -CLA-18-08 -ENTREGUE NA BASE DO PAMALS 1 EA , SERÁ ENVIAO AO OPERADOR- CLA-20-08 - AWB 12754088775 - CLA-21-08 - recebido dia 22/08/2026</t>
+  </si>
+  <si>
+    <t>Colocado pedido Textron WB0003128625 - tracking 535477333011 - previsão de entrega 25/08 V1 JPA - MATERIAL ENVIADO VIA RECIBO 726/FAB/26, AWB A SER GERADA PELA GOLLOG RC 25/08/2026</t>
+  </si>
+  <si>
+    <t>Colocado pedido no fornecedor I823285 - entregue em Miami 21/08 - TEMOS 3 EA NO ESTOQUE DA BANT. Material seguiu via awb 12754249845. Recebido por Kleyton em 24/08. Atl Ges.</t>
+  </si>
+  <si>
+    <t>Material enviado via recibo 720/FAB/26 DPE 24/08/2026 - Retirado dia 24/08/2026 por Paula Pereira id 569968</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -749,10 +749,10 @@
         <v>46251</v>
       </c>
       <c r="Q2">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="R2">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="S2" t="s">
         <v>72</v>
@@ -817,10 +817,10 @@
         <v>46269</v>
       </c>
       <c r="Q3">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="R3">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S3" t="s">
         <v>72</v>
@@ -885,10 +885,10 @@
         <v>46255</v>
       </c>
       <c r="Q4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R4">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S4" t="s">
         <v>73</v>
@@ -953,10 +953,10 @@
         <v>46279</v>
       </c>
       <c r="Q5">
-        <v>-20</v>
+        <v>-19</v>
       </c>
       <c r="R5">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="S5" t="s">
         <v>73</v>
@@ -1021,10 +1021,10 @@
         <v>46259</v>
       </c>
       <c r="Q6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R6">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="S6" t="s">
         <v>73</v>
@@ -1089,10 +1089,10 @@
         <v>46280</v>
       </c>
       <c r="Q7">
-        <v>-21</v>
+        <v>-20</v>
       </c>
       <c r="R7">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S7" t="s">
         <v>72</v>
@@ -1157,10 +1157,10 @@
         <v>46255</v>
       </c>
       <c r="Q8">
-        <v>-23</v>
+        <v>-22</v>
       </c>
       <c r="R8">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S8" t="s">
         <v>72</v>
@@ -1225,10 +1225,10 @@
         <v>46283</v>
       </c>
       <c r="Q9">
-        <v>-24</v>
+        <v>-23</v>
       </c>
       <c r="R9">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S9" t="s">
         <v>72</v>
@@ -1286,11 +1286,14 @@
       <c r="N10" s="1">
         <v>46284</v>
       </c>
+      <c r="O10" s="1">
+        <v>46262</v>
+      </c>
       <c r="Q10">
-        <v>-25</v>
+        <v>-24</v>
       </c>
       <c r="R10">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S10" t="s">
         <v>72</v>
@@ -1351,11 +1354,14 @@
       <c r="N11" s="1">
         <v>46286</v>
       </c>
+      <c r="O11" s="1">
+        <v>46258</v>
+      </c>
       <c r="Q11">
-        <v>-27</v>
+        <v>-26</v>
       </c>
       <c r="R11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S11" t="s">
         <v>72</v>
@@ -1423,10 +1429,10 @@
         <v>46258</v>
       </c>
       <c r="Q12">
-        <v>-30</v>
+        <v>-29</v>
       </c>
       <c r="R12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S12" t="s">
         <v>73</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (26/08/2026 10:59)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="87">
   <si>
     <t>om_emg</t>
   </si>
@@ -103,12 +103,12 @@
     <t>BABE</t>
   </si>
   <si>
+    <t>BAMN</t>
+  </si>
+  <si>
     <t>BABR</t>
   </si>
   <si>
-    <t>BAMN</t>
-  </si>
-  <si>
     <t>685260012350</t>
   </si>
   <si>
@@ -118,9 +118,6 @@
     <t>685260012560</t>
   </si>
   <si>
-    <t>329260019269</t>
-  </si>
-  <si>
     <t>685260012609</t>
   </si>
   <si>
@@ -136,12 +133,15 @@
     <t>396260016588</t>
   </si>
   <si>
-    <t>313260018713</t>
-  </si>
-  <si>
     <t>329260019279</t>
   </si>
   <si>
+    <t>329260019286</t>
+  </si>
+  <si>
+    <t>396260016593</t>
+  </si>
+  <si>
     <t>030-1094-58</t>
   </si>
   <si>
@@ -151,9 +151,6 @@
     <t>2641010-3</t>
   </si>
   <si>
-    <t>069-01033-0101</t>
-  </si>
-  <si>
     <t>162-10700</t>
   </si>
   <si>
@@ -169,12 +166,15 @@
     <t>0750220-1</t>
   </si>
   <si>
-    <t>2115040-8</t>
-  </si>
-  <si>
     <t>2N6576</t>
   </si>
   <si>
+    <t>C662504-0101</t>
+  </si>
+  <si>
+    <t>4626</t>
+  </si>
+  <si>
     <t>CONNECTOR</t>
   </si>
   <si>
@@ -184,9 +184,6 @@
     <t>AXLE FITTING</t>
   </si>
   <si>
-    <t>RECEIVER-TRANSMITTER</t>
-  </si>
-  <si>
     <t>OUTER WHEEL HALF ASS</t>
   </si>
   <si>
@@ -202,12 +199,15 @@
     <t>BOLT,MACHINE</t>
   </si>
   <si>
-    <t>CYLINDER GAS S</t>
-  </si>
-  <si>
     <t>TRANSISTOR</t>
   </si>
   <si>
+    <t>GAGE VOLT AMME</t>
+  </si>
+  <si>
+    <t>LAMP,INCANDESCENT</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -223,6 +223,9 @@
     <t>Expedido total</t>
   </si>
   <si>
+    <t>Aguardando solução</t>
+  </si>
+  <si>
     <t>ANCE</t>
   </si>
   <si>
@@ -247,9 +250,6 @@
     <t>AWB 12754088775 - volume retirado na loja GOLLOG - NAT por Teodoro silva em 22/08. Godoy 25/08/26.</t>
   </si>
   <si>
-    <t>Emergência transformada em ANCE em 24/08. Aguardaremos atendimento com item da Vee One. Ramon 24/08/26.</t>
-  </si>
-  <si>
     <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Chegada GIG dia 15-08 (voo 4273). Entregue V1 JPA 17/08 - MATERIAL EM TRANSITO - RECIBO 722/FAB/26</t>
   </si>
   <si>
@@ -259,9 +259,6 @@
     <t>Foi solicitado atendimento com estoque FAB - CLA- 10-08, ITEM PRONTO PARA EMBARQUE, AGUARDANDO NOTA FISCAL - CLA-11-08- ITEM AGUARDANDO DEFINIÇÃO DA COORDENADORIA QUANTO A EFETIVIDADE PARA APLICAÇÃO NA REFERIDA ANV.- CLA-13-08 - AT 685000002258. Conforme relatado pela Coordenadoria, foi enviado, via CAN, um item novo, PN 2641010-3. Dessa forma, o item que atualmente se encontra em poder da VeeOne deverá ser estornado ao estoque.CLA-25-08</t>
   </si>
   <si>
-    <t>Enviado para o Operador em 24/08/26 - AWB 127-5459 2764 - REZ 24/08/26</t>
-  </si>
-  <si>
     <t>ITEM FOI ENTREGUE PARA A FAB PAMALS VIA RECIBO 598/FAB/26 31-07-26 - AINDA NÃO FOI PARA O ESTOQUE CLA-17-08 - Aguardando autorização para movimentação a BANT 25/08/2026</t>
   </si>
   <si>
@@ -272,9 +269,6 @@
   </si>
   <si>
     <t>Colocado pedido Textron WB0003128625 - tracking 535477333011 - previsão de entrega 25/08 V1 JPA - MATERIAL ENVIADO VIA RECIBO 726/FAB/26, AWB A SER GERADA PELA GOLLOG RC 25/08/2026</t>
-  </si>
-  <si>
-    <t>Colocado pedido no fornecedor I823285 - entregue em Miami 21/08 - TEMOS 3 EA NO ESTOQUE DA BANT. Material seguiu via awb 12754249845. Recebido por Kleyton em 24/08. Atl Ges.</t>
   </si>
   <si>
     <t>Material enviado via recibo 720/FAB/26 DPE 24/08/2026 - Retirado dia 24/08/2026 por Paula Pereira id 569968</t>
@@ -728,7 +722,7 @@
         <v>67</v>
       </c>
       <c r="I2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J2" s="1">
         <v>46212</v>
@@ -740,7 +734,7 @@
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N2" s="1">
         <v>46243</v>
@@ -755,16 +749,16 @@
         <v>48</v>
       </c>
       <c r="S2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="T2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="V2" t="s">
         <v>78</v>
       </c>
       <c r="W2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -796,7 +790,7 @@
         <v>67</v>
       </c>
       <c r="I3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J3" s="1">
         <v>46238</v>
@@ -808,7 +802,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N3" s="1">
         <v>46269</v>
@@ -823,16 +817,16 @@
         <v>22</v>
       </c>
       <c r="S3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="T3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="V3" t="s">
         <v>79</v>
       </c>
       <c r="W3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -864,7 +858,7 @@
         <v>68</v>
       </c>
       <c r="I4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J4" s="1">
         <v>46244</v>
@@ -876,7 +870,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N4" s="1">
         <v>46255</v>
@@ -891,19 +885,19 @@
         <v>16</v>
       </c>
       <c r="S4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="T4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="U4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="V4" t="s">
         <v>80</v>
       </c>
       <c r="W4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -911,10 +905,10 @@
     </row>
     <row r="5" spans="1:27">
       <c r="A5">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C5" t="s">
         <v>34</v>
@@ -926,16 +920,16 @@
         <v>56</v>
       </c>
       <c r="F5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G5">
-        <v>2721</v>
+        <v>2729</v>
       </c>
       <c r="H5" t="s">
         <v>67</v>
       </c>
       <c r="I5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="J5" s="1">
         <v>46248</v>
@@ -947,28 +941,34 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N5" s="1">
-        <v>46279</v>
+        <v>46259</v>
+      </c>
+      <c r="O5" s="1">
+        <v>46259</v>
       </c>
       <c r="Q5">
-        <v>-19</v>
+        <v>1</v>
       </c>
       <c r="R5">
         <v>12</v>
       </c>
       <c r="S5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="T5" t="s">
-        <v>72</v>
+        <v>74</v>
+      </c>
+      <c r="U5" t="s">
+        <v>76</v>
       </c>
       <c r="V5" t="s">
         <v>81</v>
       </c>
       <c r="W5" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -976,10 +976,10 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C6" t="s">
         <v>35</v>
@@ -991,10 +991,10 @@
         <v>57</v>
       </c>
       <c r="F6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G6">
-        <v>2729</v>
+        <v>2741</v>
       </c>
       <c r="H6" t="s">
         <v>67</v>
@@ -1003,43 +1003,37 @@
         <v>70</v>
       </c>
       <c r="J6" s="1">
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="K6" s="1">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="L6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N6" s="1">
-        <v>46259</v>
-      </c>
-      <c r="O6" s="1">
-        <v>46259</v>
+        <v>46280</v>
       </c>
       <c r="Q6">
-        <v>1</v>
+        <v>-20</v>
       </c>
       <c r="R6">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="S6" t="s">
         <v>73</v>
       </c>
       <c r="T6" t="s">
-        <v>73</v>
-      </c>
-      <c r="U6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="V6" t="s">
         <v>82</v>
       </c>
       <c r="W6" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1047,10 +1041,10 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C7" t="s">
         <v>36</v>
@@ -1062,49 +1056,55 @@
         <v>58</v>
       </c>
       <c r="F7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G7">
-        <v>2741</v>
+        <v>2729</v>
       </c>
       <c r="H7" t="s">
         <v>67</v>
       </c>
       <c r="I7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J7" s="1">
         <v>46251</v>
       </c>
       <c r="K7" s="1">
-        <v>46249</v>
+        <v>46251</v>
       </c>
       <c r="L7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N7" s="1">
-        <v>46280</v>
+        <v>46282</v>
+      </c>
+      <c r="O7" s="1">
+        <v>46255</v>
       </c>
       <c r="Q7">
-        <v>-20</v>
+        <v>-22</v>
       </c>
       <c r="R7">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="S7" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="T7" t="s">
-        <v>73</v>
+        <v>74</v>
+      </c>
+      <c r="U7" t="s">
+        <v>77</v>
       </c>
       <c r="V7" t="s">
         <v>83</v>
       </c>
       <c r="W7" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1112,10 +1112,10 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C8" t="s">
         <v>37</v>
@@ -1127,55 +1127,46 @@
         <v>59</v>
       </c>
       <c r="F8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G8">
-        <v>2729</v>
+        <v>2741</v>
       </c>
       <c r="H8" t="s">
         <v>67</v>
       </c>
       <c r="I8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J8" s="1">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="K8" s="1">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="L8">
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N8" s="1">
-        <v>46282</v>
-      </c>
-      <c r="O8" s="1">
-        <v>46255</v>
+        <v>46283</v>
       </c>
       <c r="Q8">
-        <v>-22</v>
+        <v>-23</v>
       </c>
       <c r="R8">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S8" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="T8" t="s">
-        <v>73</v>
-      </c>
-      <c r="U8" t="s">
-        <v>76</v>
-      </c>
-      <c r="V8" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="W8" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1183,10 +1174,10 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9">
-        <v>313</v>
+        <v>396</v>
       </c>
       <c r="B9" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C9" t="s">
         <v>38</v>
@@ -1198,46 +1189,52 @@
         <v>60</v>
       </c>
       <c r="F9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G9">
-        <v>2741</v>
+        <v>2731</v>
       </c>
       <c r="H9" t="s">
         <v>67</v>
       </c>
       <c r="I9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J9" s="1">
+        <v>46252</v>
+      </c>
+      <c r="K9" s="1">
         <v>46253</v>
       </c>
-      <c r="K9" s="1">
-        <v>46252</v>
-      </c>
       <c r="L9">
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N9" s="1">
-        <v>46283</v>
+        <v>46284</v>
+      </c>
+      <c r="O9" s="1">
+        <v>46262</v>
       </c>
       <c r="Q9">
-        <v>-23</v>
+        <v>-24</v>
       </c>
       <c r="R9">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="T9" t="s">
-        <v>73</v>
+        <v>74</v>
+      </c>
+      <c r="V9" t="s">
+        <v>84</v>
       </c>
       <c r="W9" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1245,10 +1242,10 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>396</v>
+        <v>329</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C10" t="s">
         <v>39</v>
@@ -1263,40 +1260,40 @@
         <v>64</v>
       </c>
       <c r="G10">
-        <v>2731</v>
+        <v>2721</v>
       </c>
       <c r="H10" t="s">
         <v>67</v>
       </c>
       <c r="I10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J10" s="1">
-        <v>46252</v>
+        <v>46255</v>
       </c>
       <c r="K10" s="1">
-        <v>46253</v>
+        <v>46258</v>
       </c>
       <c r="L10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M10" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N10" s="1">
-        <v>46284</v>
+        <v>46289</v>
       </c>
       <c r="O10" s="1">
-        <v>46262</v>
+        <v>46258</v>
       </c>
       <c r="Q10">
-        <v>-24</v>
+        <v>-29</v>
       </c>
       <c r="R10">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="S10" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="T10" t="s">
         <v>73</v>
@@ -1305,7 +1302,7 @@
         <v>85</v>
       </c>
       <c r="W10" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1313,7 +1310,7 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B11" t="s">
         <v>30</v>
@@ -1328,55 +1325,46 @@
         <v>62</v>
       </c>
       <c r="F11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G11">
-        <v>2737</v>
+        <v>2709</v>
       </c>
       <c r="H11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I11" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J11" s="1">
-        <v>46254</v>
+        <v>46259</v>
       </c>
       <c r="K11" s="1">
-        <v>46255</v>
+        <v>46261</v>
       </c>
       <c r="L11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N11" s="1">
-        <v>46286</v>
-      </c>
-      <c r="O11" s="1">
-        <v>46258</v>
+        <v>46292</v>
       </c>
       <c r="Q11">
-        <v>-26</v>
+        <v>-32</v>
       </c>
       <c r="R11">
-        <v>5</v>
+        <v>-1</v>
       </c>
       <c r="S11" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="T11" t="s">
         <v>73</v>
       </c>
-      <c r="U11" t="s">
-        <v>77</v>
-      </c>
-      <c r="V11" t="s">
+      <c r="W11" t="s">
         <v>86</v>
-      </c>
-      <c r="W11" t="s">
-        <v>88</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1384,10 +1372,10 @@
     </row>
     <row r="12" spans="1:27">
       <c r="A12">
-        <v>329</v>
+        <v>396</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C12" t="s">
         <v>41</v>
@@ -1402,49 +1390,43 @@
         <v>64</v>
       </c>
       <c r="G12">
-        <v>2721</v>
+        <v>2731</v>
       </c>
       <c r="H12" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J12" s="1">
-        <v>46255</v>
+        <v>46259</v>
       </c>
       <c r="K12" s="1">
-        <v>46258</v>
+        <v>46262</v>
       </c>
       <c r="L12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N12" s="1">
-        <v>46289</v>
-      </c>
-      <c r="O12" s="1">
-        <v>46258</v>
+        <v>46293</v>
       </c>
       <c r="Q12">
-        <v>-29</v>
+        <v>-33</v>
       </c>
       <c r="R12">
-        <v>2</v>
+        <v>-2</v>
       </c>
       <c r="S12" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="T12" t="s">
-        <v>72</v>
-      </c>
-      <c r="V12" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="W12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (26/08/2026 13:24)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -1340,7 +1340,7 @@
         <v>46259</v>
       </c>
       <c r="K11" s="1">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="L11">
         <v>1</v>
@@ -1349,13 +1349,13 @@
         <v>72</v>
       </c>
       <c r="N11" s="1">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="Q11">
-        <v>-32</v>
+        <v>-31</v>
       </c>
       <c r="R11">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="S11" t="s">
         <v>74</v>
@@ -1402,7 +1402,7 @@
         <v>46259</v>
       </c>
       <c r="K12" s="1">
-        <v>46262</v>
+        <v>46260</v>
       </c>
       <c r="L12">
         <v>1</v>
@@ -1411,13 +1411,13 @@
         <v>72</v>
       </c>
       <c r="N12" s="1">
-        <v>46293</v>
+        <v>46291</v>
       </c>
       <c r="Q12">
-        <v>-33</v>
+        <v>-31</v>
       </c>
       <c r="R12">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="S12" t="s">
         <v>74</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (26/08/2026 16:12)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="89">
   <si>
     <t>om_emg</t>
   </si>
@@ -248,6 +248,12 @@
   </si>
   <si>
     <t>AWB 12754088775 - volume retirado na loja GOLLOG - NAT por Teodoro silva em 22/08. Godoy 25/08/26.</t>
+  </si>
+  <si>
+    <t>item será atendido com o estoque local pedido 18294676. Godoy 26/08.</t>
+  </si>
+  <si>
+    <t>item será atendido com o estoque local pedido 18295192. Godoy 26/08.</t>
   </si>
   <si>
     <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Chegada GIG dia 15-08 (voo 4273). Entregue V1 JPA 17/08 - MATERIAL EM TRANSITO - RECIBO 722/FAB/26</t>
@@ -755,10 +761,10 @@
         <v>74</v>
       </c>
       <c r="V2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="W2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -823,10 +829,10 @@
         <v>74</v>
       </c>
       <c r="V3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="W3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -894,10 +900,10 @@
         <v>75</v>
       </c>
       <c r="V4" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="W4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -965,10 +971,10 @@
         <v>76</v>
       </c>
       <c r="V5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="W5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1030,10 +1036,10 @@
         <v>74</v>
       </c>
       <c r="V6" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="W6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1101,10 +1107,10 @@
         <v>77</v>
       </c>
       <c r="V7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="W7" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1166,7 +1172,7 @@
         <v>74</v>
       </c>
       <c r="W8" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1231,10 +1237,10 @@
         <v>74</v>
       </c>
       <c r="V9" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="W9" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1299,10 +1305,10 @@
         <v>73</v>
       </c>
       <c r="V10" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="W10" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1363,8 +1369,11 @@
       <c r="T11" t="s">
         <v>73</v>
       </c>
+      <c r="U11" t="s">
+        <v>78</v>
+      </c>
       <c r="W11" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1425,8 +1434,11 @@
       <c r="T12" t="s">
         <v>74</v>
       </c>
+      <c r="U12" t="s">
+        <v>79</v>
+      </c>
       <c r="W12" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (27/08/2026 17:59)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="90">
   <si>
     <t>om_emg</t>
   </si>
@@ -115,9 +115,6 @@
     <t>396260016580</t>
   </si>
   <si>
-    <t>685260012560</t>
-  </si>
-  <si>
     <t>685260012609</t>
   </si>
   <si>
@@ -133,6 +130,9 @@
     <t>396260016588</t>
   </si>
   <si>
+    <t>313260018713</t>
+  </si>
+  <si>
     <t>329260019279</t>
   </si>
   <si>
@@ -148,9 +148,6 @@
     <t>2601188-204</t>
   </si>
   <si>
-    <t>2641010-3</t>
-  </si>
-  <si>
     <t>162-10700</t>
   </si>
   <si>
@@ -166,6 +163,9 @@
     <t>0750220-1</t>
   </si>
   <si>
+    <t>2115040-8</t>
+  </si>
+  <si>
     <t>2N6576</t>
   </si>
   <si>
@@ -181,9 +181,6 @@
     <t>COMPRESSOR DRIVE ASS</t>
   </si>
   <si>
-    <t>AXLE FITTING</t>
-  </si>
-  <si>
     <t>OUTER WHEEL HALF ASS</t>
   </si>
   <si>
@@ -199,6 +196,9 @@
     <t>BOLT,MACHINE</t>
   </si>
   <si>
+    <t>CYLINDER GAS S</t>
+  </si>
+  <si>
     <t>TRANSISTOR</t>
   </si>
   <si>
@@ -223,15 +223,15 @@
     <t>Expedido total</t>
   </si>
   <si>
-    <t>Aguardando solução</t>
-  </si>
-  <si>
     <t>ANCE</t>
   </si>
   <si>
     <t>IPLR</t>
   </si>
   <si>
+    <t>AIFP</t>
+  </si>
+  <si>
     <t>EA</t>
   </si>
   <si>
@@ -241,16 +241,19 @@
     <t>Sim</t>
   </si>
   <si>
-    <t>item atendido com o estoque local pedido 18171852 em 10/08. Godoy 11/08. Está sendo definido se o PN está correto. Ramon 11/08/26.</t>
-  </si>
-  <si>
-    <t>Estoque alterado de "Nao" para "SIM"  daremos prioridade para movimentar o item.  Godoy 17/08/226</t>
+    <t>Estoque alterado de "Nao" para "SIM"  daremos prioridade para movimentar o item. Godoy 17/08/226</t>
   </si>
   <si>
     <t>AWB 12754088775 - volume retirado na loja GOLLOG - NAT por Teodoro silva em 22/08. Godoy 25/08/26.</t>
   </si>
   <si>
-    <t>item será atendido com o estoque local pedido 18294676. Godoy 26/08.</t>
+    <t>Emergência transformada em ANCE em 24/08. Aguardaremos atendimento com item da Vee One. Ramon 24/08/26.</t>
+  </si>
+  <si>
+    <t>Possui AWB ou recibo assinado? Ramon 28/08/26.</t>
+  </si>
+  <si>
+    <t>item será atendido com o estoque local pedido 18294676. Godoy 26/08. Emg é na verdade AIFP, corrigido na planilha de 28/08. Ramon 28/08/26.</t>
   </si>
   <si>
     <t>item será atendido com o estoque local pedido 18295192. Godoy 26/08.</t>
@@ -262,9 +265,6 @@
     <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
   </si>
   <si>
-    <t>Foi solicitado atendimento com estoque FAB - CLA- 10-08, ITEM PRONTO PARA EMBARQUE, AGUARDANDO NOTA FISCAL - CLA-11-08- ITEM AGUARDANDO DEFINIÇÃO DA COORDENADORIA QUANTO A EFETIVIDADE PARA APLICAÇÃO NA REFERIDA ANV.- CLA-13-08 - AT 685000002258. Conforme relatado pela Coordenadoria, foi enviado, via CAN, um item novo, PN 2641010-3. Dessa forma, o item que atualmente se encontra em poder da VeeOne deverá ser estornado ao estoque.CLA-25-08</t>
-  </si>
-  <si>
     <t>ITEM FOI ENTREGUE PARA A FAB PAMALS VIA RECIBO 598/FAB/26 31-07-26 - AINDA NÃO FOI PARA O ESTOQUE CLA-17-08 - Aguardando autorização para movimentação a BANT 25/08/2026</t>
   </si>
   <si>
@@ -275,6 +275,9 @@
   </si>
   <si>
     <t>Colocado pedido Textron WB0003128625 - tracking 535477333011 - previsão de entrega 25/08 V1 JPA - MATERIAL ENVIADO VIA RECIBO 726/FAB/26, AWB A SER GERADA PELA GOLLOG RC 25/08/2026</t>
+  </si>
+  <si>
+    <t>Colocado pedido no fornecedor I823285 - entregue em Miami 21/08 - TEMOS 3 EA NO ESTOQUE DA BANT. Material seguiu via awb 12754249845. Recebido por Kleyton em 24/08. Atl Ges.</t>
   </si>
   <si>
     <t>Material enviado via recibo 720/FAB/26 DPE 24/08/2026 - Retirado dia 24/08/2026 por Paula Pereira id 569968</t>
@@ -728,7 +731,7 @@
         <v>67</v>
       </c>
       <c r="I2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J2" s="1">
         <v>46212</v>
@@ -749,10 +752,10 @@
         <v>46251</v>
       </c>
       <c r="Q2">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="R2">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="S2" t="s">
         <v>73</v>
@@ -761,10 +764,10 @@
         <v>74</v>
       </c>
       <c r="V2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="W2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -796,7 +799,7 @@
         <v>67</v>
       </c>
       <c r="I3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J3" s="1">
         <v>46238</v>
@@ -817,10 +820,10 @@
         <v>46269</v>
       </c>
       <c r="Q3">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="R3">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="S3" t="s">
         <v>73</v>
@@ -829,10 +832,10 @@
         <v>74</v>
       </c>
       <c r="V3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="W3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -861,16 +864,16 @@
         <v>2729</v>
       </c>
       <c r="H4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J4" s="1">
-        <v>46244</v>
+        <v>46248</v>
       </c>
       <c r="K4" s="1">
-        <v>46244</v>
+        <v>46248</v>
       </c>
       <c r="L4">
         <v>1</v>
@@ -879,16 +882,16 @@
         <v>72</v>
       </c>
       <c r="N4" s="1">
-        <v>46255</v>
+        <v>46259</v>
       </c>
       <c r="O4" s="1">
-        <v>46255</v>
+        <v>46259</v>
       </c>
       <c r="Q4">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="R4">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="S4" t="s">
         <v>74</v>
@@ -900,10 +903,10 @@
         <v>75</v>
       </c>
       <c r="V4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="W4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -911,10 +914,10 @@
     </row>
     <row r="5" spans="1:27">
       <c r="A5">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C5" t="s">
         <v>34</v>
@@ -926,55 +929,49 @@
         <v>56</v>
       </c>
       <c r="F5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G5">
-        <v>2729</v>
+        <v>2741</v>
       </c>
       <c r="H5" t="s">
         <v>67</v>
       </c>
       <c r="I5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J5" s="1">
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="K5" s="1">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="L5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M5" t="s">
         <v>72</v>
       </c>
       <c r="N5" s="1">
-        <v>46259</v>
-      </c>
-      <c r="O5" s="1">
-        <v>46259</v>
+        <v>46280</v>
       </c>
       <c r="Q5">
-        <v>1</v>
+        <v>-19</v>
       </c>
       <c r="R5">
         <v>12</v>
       </c>
       <c r="S5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="T5" t="s">
         <v>74</v>
       </c>
-      <c r="U5" t="s">
-        <v>76</v>
-      </c>
       <c r="V5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="W5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -982,10 +979,10 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C6" t="s">
         <v>35</v>
@@ -997,37 +994,40 @@
         <v>57</v>
       </c>
       <c r="F6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G6">
-        <v>2741</v>
+        <v>2729</v>
       </c>
       <c r="H6" t="s">
         <v>67</v>
       </c>
       <c r="I6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J6" s="1">
         <v>46251</v>
       </c>
       <c r="K6" s="1">
-        <v>46249</v>
+        <v>46251</v>
       </c>
       <c r="L6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M6" t="s">
         <v>72</v>
       </c>
       <c r="N6" s="1">
-        <v>46280</v>
+        <v>46282</v>
+      </c>
+      <c r="O6" s="1">
+        <v>46255</v>
       </c>
       <c r="Q6">
-        <v>-20</v>
+        <v>-21</v>
       </c>
       <c r="R6">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="S6" t="s">
         <v>73</v>
@@ -1035,11 +1035,14 @@
       <c r="T6" t="s">
         <v>74</v>
       </c>
+      <c r="U6" t="s">
+        <v>76</v>
+      </c>
       <c r="V6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="W6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1047,10 +1050,10 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
         <v>36</v>
@@ -1062,22 +1065,22 @@
         <v>58</v>
       </c>
       <c r="F7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G7">
-        <v>2729</v>
+        <v>2741</v>
       </c>
       <c r="H7" t="s">
         <v>67</v>
       </c>
       <c r="I7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J7" s="1">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="K7" s="1">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="L7">
         <v>1</v>
@@ -1086,10 +1089,7 @@
         <v>72</v>
       </c>
       <c r="N7" s="1">
-        <v>46282</v>
-      </c>
-      <c r="O7" s="1">
-        <v>46255</v>
+        <v>46283</v>
       </c>
       <c r="Q7">
         <v>-22</v>
@@ -1103,14 +1103,8 @@
       <c r="T7" t="s">
         <v>74</v>
       </c>
-      <c r="U7" t="s">
-        <v>77</v>
-      </c>
-      <c r="V7" t="s">
-        <v>85</v>
-      </c>
       <c r="W7" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1118,10 +1112,10 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>313</v>
+        <v>396</v>
       </c>
       <c r="B8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
         <v>37</v>
@@ -1133,22 +1127,22 @@
         <v>59</v>
       </c>
       <c r="F8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G8">
-        <v>2741</v>
+        <v>2731</v>
       </c>
       <c r="H8" t="s">
         <v>67</v>
       </c>
       <c r="I8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J8" s="1">
+        <v>46252</v>
+      </c>
+      <c r="K8" s="1">
         <v>46253</v>
-      </c>
-      <c r="K8" s="1">
-        <v>46252</v>
       </c>
       <c r="L8">
         <v>1</v>
@@ -1157,7 +1151,10 @@
         <v>72</v>
       </c>
       <c r="N8" s="1">
-        <v>46283</v>
+        <v>46284</v>
+      </c>
+      <c r="O8" s="1">
+        <v>46262</v>
       </c>
       <c r="Q8">
         <v>-23</v>
@@ -1171,8 +1168,11 @@
       <c r="T8" t="s">
         <v>74</v>
       </c>
+      <c r="V8" t="s">
+        <v>86</v>
+      </c>
       <c r="W8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1180,10 +1180,10 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9">
-        <v>396</v>
+        <v>313</v>
       </c>
       <c r="B9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s">
         <v>38</v>
@@ -1198,37 +1198,37 @@
         <v>64</v>
       </c>
       <c r="G9">
-        <v>2731</v>
+        <v>2737</v>
       </c>
       <c r="H9" t="s">
         <v>67</v>
       </c>
       <c r="I9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J9" s="1">
-        <v>46252</v>
+        <v>46254</v>
       </c>
       <c r="K9" s="1">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="L9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M9" t="s">
         <v>72</v>
       </c>
       <c r="N9" s="1">
-        <v>46284</v>
+        <v>46286</v>
       </c>
       <c r="O9" s="1">
-        <v>46262</v>
+        <v>46258</v>
       </c>
       <c r="Q9">
-        <v>-24</v>
+        <v>-25</v>
       </c>
       <c r="R9">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S9" t="s">
         <v>73</v>
@@ -1236,11 +1236,14 @@
       <c r="T9" t="s">
         <v>74</v>
       </c>
+      <c r="U9" t="s">
+        <v>77</v>
+      </c>
       <c r="V9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="W9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1272,7 +1275,7 @@
         <v>67</v>
       </c>
       <c r="I10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J10" s="1">
         <v>46255</v>
@@ -1293,10 +1296,10 @@
         <v>46258</v>
       </c>
       <c r="Q10">
-        <v>-29</v>
+        <v>-28</v>
       </c>
       <c r="R10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S10" t="s">
         <v>74</v>
@@ -1304,11 +1307,14 @@
       <c r="T10" t="s">
         <v>73</v>
       </c>
+      <c r="U10" t="s">
+        <v>78</v>
+      </c>
       <c r="V10" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="W10" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1337,10 +1343,10 @@
         <v>2709</v>
       </c>
       <c r="H11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J11" s="1">
         <v>46259</v>
@@ -1355,13 +1361,13 @@
         <v>72</v>
       </c>
       <c r="N11" s="1">
-        <v>46291</v>
+        <v>46267</v>
       </c>
       <c r="Q11">
-        <v>-31</v>
+        <v>-6</v>
       </c>
       <c r="R11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S11" t="s">
         <v>74</v>
@@ -1370,10 +1376,10 @@
         <v>73</v>
       </c>
       <c r="U11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="W11" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1402,10 +1408,10 @@
         <v>2731</v>
       </c>
       <c r="H12" t="s">
+        <v>68</v>
+      </c>
+      <c r="I12" t="s">
         <v>69</v>
-      </c>
-      <c r="I12" t="s">
-        <v>70</v>
       </c>
       <c r="J12" s="1">
         <v>46259</v>
@@ -1423,10 +1429,10 @@
         <v>46291</v>
       </c>
       <c r="Q12">
-        <v>-31</v>
+        <v>-30</v>
       </c>
       <c r="R12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S12" t="s">
         <v>74</v>
@@ -1435,10 +1441,10 @@
         <v>74</v>
       </c>
       <c r="U12" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="W12" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (28/08/2026 02:13)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -752,10 +752,10 @@
         <v>46251</v>
       </c>
       <c r="Q2">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="R2">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="S2" t="s">
         <v>73</v>
@@ -820,10 +820,10 @@
         <v>46269</v>
       </c>
       <c r="Q3">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="R3">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="S3" t="s">
         <v>73</v>
@@ -888,10 +888,10 @@
         <v>46259</v>
       </c>
       <c r="Q4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R4">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S4" t="s">
         <v>74</v>
@@ -956,10 +956,10 @@
         <v>46280</v>
       </c>
       <c r="Q5">
-        <v>-19</v>
+        <v>-18</v>
       </c>
       <c r="R5">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S5" t="s">
         <v>73</v>
@@ -1024,10 +1024,10 @@
         <v>46255</v>
       </c>
       <c r="Q6">
-        <v>-21</v>
+        <v>-20</v>
       </c>
       <c r="R6">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S6" t="s">
         <v>73</v>
@@ -1092,10 +1092,10 @@
         <v>46283</v>
       </c>
       <c r="Q7">
-        <v>-22</v>
+        <v>-21</v>
       </c>
       <c r="R7">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="S7" t="s">
         <v>73</v>
@@ -1157,10 +1157,10 @@
         <v>46262</v>
       </c>
       <c r="Q8">
-        <v>-23</v>
+        <v>-22</v>
       </c>
       <c r="R8">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S8" t="s">
         <v>73</v>
@@ -1225,10 +1225,10 @@
         <v>46258</v>
       </c>
       <c r="Q9">
-        <v>-25</v>
+        <v>-24</v>
       </c>
       <c r="R9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S9" t="s">
         <v>73</v>
@@ -1296,10 +1296,10 @@
         <v>46258</v>
       </c>
       <c r="Q10">
-        <v>-28</v>
+        <v>-27</v>
       </c>
       <c r="R10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S10" t="s">
         <v>74</v>
@@ -1364,10 +1364,10 @@
         <v>46267</v>
       </c>
       <c r="Q11">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S11" t="s">
         <v>74</v>
@@ -1429,10 +1429,10 @@
         <v>46291</v>
       </c>
       <c r="Q12">
-        <v>-30</v>
+        <v>-29</v>
       </c>
       <c r="R12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S12" t="s">
         <v>74</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (28/08/2026 18:21)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="90">
   <si>
     <t>om_emg</t>
   </si>
@@ -121,9 +121,6 @@
     <t>313260018702</t>
   </si>
   <si>
-    <t>685260012619</t>
-  </si>
-  <si>
     <t>313260018708</t>
   </si>
   <si>
@@ -142,6 +139,12 @@
     <t>396260016593</t>
   </si>
   <si>
+    <t>329260019288</t>
+  </si>
+  <si>
+    <t>396260016603</t>
+  </si>
+  <si>
     <t>030-1094-58</t>
   </si>
   <si>
@@ -154,9 +157,6 @@
     <t>040-0043</t>
   </si>
   <si>
-    <t>071-01519-0101</t>
-  </si>
-  <si>
     <t>2698010-7</t>
   </si>
   <si>
@@ -175,6 +175,9 @@
     <t>4626</t>
   </si>
   <si>
+    <t>OD1232-24MB</t>
+  </si>
+  <si>
     <t>CONNECTOR</t>
   </si>
   <si>
@@ -187,9 +190,6 @@
     <t>STROB TUB</t>
   </si>
   <si>
-    <t>RECEIVER-EXCITER,RAD</t>
-  </si>
-  <si>
     <t>PASSENGER DOOR - LOW</t>
   </si>
   <si>
@@ -208,21 +208,24 @@
     <t>LAMP,INCANDESCENT</t>
   </si>
   <si>
+    <t>DC FAN</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
     <t>T</t>
   </si>
   <si>
-    <t>R</t>
-  </si>
-  <si>
     <t>Providência tomada</t>
   </si>
   <si>
     <t>Expedido total</t>
   </si>
   <si>
+    <t>Aguardando solução</t>
+  </si>
+  <si>
     <t>ANCE</t>
   </si>
   <si>
@@ -244,9 +247,6 @@
     <t>Estoque alterado de "Nao" para "SIM"  daremos prioridade para movimentar o item. Godoy 17/08/226</t>
   </si>
   <si>
-    <t>AWB 12754088775 - volume retirado na loja GOLLOG - NAT por Teodoro silva em 22/08. Godoy 25/08/26.</t>
-  </si>
-  <si>
     <t>Emergência transformada em ANCE em 24/08. Aguardaremos atendimento com item da Vee One. Ramon 24/08/26.</t>
   </si>
   <si>
@@ -271,9 +271,6 @@
     <t>Colocado pedido no fornecedor WAGA INTERNATIONAL - validando previsão de entrega em Miami. ATZ 25/08</t>
   </si>
   <si>
-    <t>DPE DA WILLIAM DIA 20-08-2026 -CLA-18-08 -ENTREGUE NA BASE DO PAMALS 1 EA , SERÁ ENVIAO AO OPERADOR- CLA-20-08 - AWB 12754088775 - CLA-21-08 - recebido dia 22/08/2026</t>
-  </si>
-  <si>
     <t>Colocado pedido Textron WB0003128625 - tracking 535477333011 - previsão de entrega 25/08 V1 JPA - MATERIAL ENVIADO VIA RECIBO 726/FAB/26, AWB A SER GERADA PELA GOLLOG RC 25/08/2026</t>
   </si>
   <si>
@@ -281,6 +278,9 @@
   </si>
   <si>
     <t>Material enviado via recibo 720/FAB/26 DPE 24/08/2026 - Retirado dia 24/08/2026 por Paula Pereira id 569968</t>
+  </si>
+  <si>
+    <t>Será atendido via estoque Vee One</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -619,7 +619,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA12"/>
+  <dimension ref="A1:AA13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -716,13 +716,13 @@
         <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G2">
         <v>2702</v>
@@ -731,7 +731,7 @@
         <v>67</v>
       </c>
       <c r="I2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J2" s="1">
         <v>46212</v>
@@ -743,7 +743,7 @@
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N2" s="1">
         <v>46243</v>
@@ -758,10 +758,10 @@
         <v>50</v>
       </c>
       <c r="S2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="T2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="V2" t="s">
         <v>81</v>
@@ -784,13 +784,13 @@
         <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G3">
         <v>2733</v>
@@ -799,7 +799,7 @@
         <v>67</v>
       </c>
       <c r="I3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J3" s="1">
         <v>46238</v>
@@ -811,7 +811,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N3" s="1">
         <v>46269</v>
@@ -826,10 +826,10 @@
         <v>24</v>
       </c>
       <c r="S3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="T3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="V3" t="s">
         <v>82</v>
@@ -852,22 +852,22 @@
         <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G4">
         <v>2729</v>
       </c>
       <c r="H4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J4" s="1">
         <v>46248</v>
@@ -879,7 +879,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N4" s="1">
         <v>46259</v>
@@ -894,13 +894,13 @@
         <v>14</v>
       </c>
       <c r="S4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="T4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="U4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="V4" t="s">
         <v>83</v>
@@ -923,13 +923,13 @@
         <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G5">
         <v>2741</v>
@@ -938,7 +938,7 @@
         <v>67</v>
       </c>
       <c r="I5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J5" s="1">
         <v>46251</v>
@@ -950,7 +950,7 @@
         <v>2</v>
       </c>
       <c r="M5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N5" s="1">
         <v>46280</v>
@@ -962,10 +962,10 @@
         <v>13</v>
       </c>
       <c r="S5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="T5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="V5" t="s">
         <v>84</v>
@@ -979,67 +979,58 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C6" t="s">
         <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F6" t="s">
         <v>66</v>
       </c>
       <c r="G6">
-        <v>2729</v>
+        <v>2741</v>
       </c>
       <c r="H6" t="s">
         <v>67</v>
       </c>
       <c r="I6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J6" s="1">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="K6" s="1">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="L6">
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N6" s="1">
-        <v>46282</v>
-      </c>
-      <c r="O6" s="1">
-        <v>46255</v>
+        <v>46283</v>
       </c>
       <c r="Q6">
-        <v>-20</v>
+        <v>-21</v>
       </c>
       <c r="R6">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="S6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="T6" t="s">
-        <v>74</v>
-      </c>
-      <c r="U6" t="s">
-        <v>76</v>
-      </c>
-      <c r="V6" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="W6" t="s">
         <v>89</v>
@@ -1050,58 +1041,64 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>313</v>
+        <v>396</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C7" t="s">
         <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F7" t="s">
         <v>65</v>
       </c>
       <c r="G7">
-        <v>2741</v>
+        <v>2731</v>
       </c>
       <c r="H7" t="s">
         <v>67</v>
       </c>
       <c r="I7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J7" s="1">
+        <v>46252</v>
+      </c>
+      <c r="K7" s="1">
         <v>46253</v>
       </c>
-      <c r="K7" s="1">
-        <v>46252</v>
-      </c>
       <c r="L7">
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N7" s="1">
-        <v>46283</v>
+        <v>46284</v>
+      </c>
+      <c r="O7" s="1">
+        <v>46262</v>
       </c>
       <c r="Q7">
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="R7">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="S7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="T7" t="s">
-        <v>74</v>
+        <v>75</v>
+      </c>
+      <c r="V7" t="s">
+        <v>85</v>
       </c>
       <c r="W7" t="s">
         <v>89</v>
@@ -1112,61 +1109,64 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>396</v>
+        <v>313</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C8" t="s">
         <v>37</v>
       </c>
       <c r="D8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G8">
-        <v>2731</v>
+        <v>2737</v>
       </c>
       <c r="H8" t="s">
         <v>67</v>
       </c>
       <c r="I8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J8" s="1">
-        <v>46252</v>
+        <v>46254</v>
       </c>
       <c r="K8" s="1">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="L8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M8" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N8" s="1">
-        <v>46284</v>
+        <v>46286</v>
       </c>
       <c r="O8" s="1">
-        <v>46262</v>
+        <v>46258</v>
       </c>
       <c r="Q8">
-        <v>-22</v>
+        <v>-24</v>
       </c>
       <c r="R8">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="S8" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="T8" t="s">
-        <v>74</v>
+        <v>75</v>
+      </c>
+      <c r="U8" t="s">
+        <v>77</v>
       </c>
       <c r="V8" t="s">
         <v>86</v>
@@ -1180,64 +1180,64 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C9" t="s">
         <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G9">
-        <v>2737</v>
+        <v>2721</v>
       </c>
       <c r="H9" t="s">
         <v>67</v>
       </c>
       <c r="I9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J9" s="1">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="K9" s="1">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="L9">
         <v>2</v>
       </c>
       <c r="M9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N9" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="O9" s="1">
         <v>46258</v>
       </c>
       <c r="Q9">
-        <v>-24</v>
+        <v>-27</v>
       </c>
       <c r="R9">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="S9" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="T9" t="s">
         <v>74</v>
       </c>
       <c r="U9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="V9" t="s">
         <v>87</v>
@@ -1260,58 +1260,52 @@
         <v>39</v>
       </c>
       <c r="D10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E10" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G10">
-        <v>2721</v>
+        <v>2709</v>
       </c>
       <c r="H10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I10" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="J10" s="1">
-        <v>46255</v>
+        <v>46259</v>
       </c>
       <c r="K10" s="1">
-        <v>46258</v>
+        <v>46260</v>
       </c>
       <c r="L10">
+        <v>1</v>
+      </c>
+      <c r="M10" t="s">
+        <v>73</v>
+      </c>
+      <c r="N10" s="1">
+        <v>46267</v>
+      </c>
+      <c r="Q10">
+        <v>-5</v>
+      </c>
+      <c r="R10">
         <v>2</v>
       </c>
-      <c r="M10" t="s">
-        <v>72</v>
-      </c>
-      <c r="N10" s="1">
-        <v>46289</v>
-      </c>
-      <c r="O10" s="1">
-        <v>46258</v>
-      </c>
-      <c r="Q10">
-        <v>-27</v>
-      </c>
-      <c r="R10">
-        <v>4</v>
-      </c>
       <c r="S10" t="s">
+        <v>75</v>
+      </c>
+      <c r="T10" t="s">
         <v>74</v>
       </c>
-      <c r="T10" t="s">
-        <v>73</v>
-      </c>
       <c r="U10" t="s">
-        <v>78</v>
-      </c>
-      <c r="V10" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="W10" t="s">
         <v>89</v>
@@ -1322,31 +1316,31 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>329</v>
+        <v>396</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C11" t="s">
         <v>40</v>
       </c>
       <c r="D11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E11" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F11" t="s">
         <v>65</v>
       </c>
       <c r="G11">
-        <v>2709</v>
+        <v>2731</v>
       </c>
       <c r="H11" t="s">
         <v>68</v>
       </c>
       <c r="I11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J11" s="1">
         <v>46259</v>
@@ -1358,25 +1352,28 @@
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N11" s="1">
-        <v>46267</v>
+        <v>46291</v>
       </c>
       <c r="Q11">
-        <v>-5</v>
+        <v>-29</v>
       </c>
       <c r="R11">
         <v>2</v>
       </c>
       <c r="S11" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="T11" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="U11" t="s">
-        <v>79</v>
+        <v>80</v>
+      </c>
+      <c r="V11" t="s">
+        <v>88</v>
       </c>
       <c r="W11" t="s">
         <v>89</v>
@@ -1387,52 +1384,52 @@
     </row>
     <row r="12" spans="1:27">
       <c r="A12">
-        <v>396</v>
+        <v>329</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C12" t="s">
         <v>41</v>
       </c>
       <c r="D12" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F12" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G12">
-        <v>2731</v>
+        <v>2721</v>
       </c>
       <c r="H12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I12" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="J12" s="1">
-        <v>46259</v>
+        <v>46262</v>
       </c>
       <c r="K12" s="1">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="L12">
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N12" s="1">
-        <v>46291</v>
+        <v>46269</v>
       </c>
       <c r="Q12">
-        <v>-29</v>
+        <v>-7</v>
       </c>
       <c r="R12">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S12" t="s">
         <v>74</v>
@@ -1440,13 +1437,72 @@
       <c r="T12" t="s">
         <v>74</v>
       </c>
-      <c r="U12" t="s">
-        <v>80</v>
-      </c>
       <c r="W12" t="s">
         <v>89</v>
       </c>
       <c r="AA12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27">
+      <c r="A13">
+        <v>396</v>
+      </c>
+      <c r="B13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" t="s">
+        <v>42</v>
+      </c>
+      <c r="D13" t="s">
+        <v>53</v>
+      </c>
+      <c r="E13" t="s">
+        <v>64</v>
+      </c>
+      <c r="F13" t="s">
+        <v>65</v>
+      </c>
+      <c r="G13">
+        <v>2733</v>
+      </c>
+      <c r="H13" t="s">
+        <v>69</v>
+      </c>
+      <c r="I13" t="s">
+        <v>70</v>
+      </c>
+      <c r="J13" s="1">
+        <v>46262</v>
+      </c>
+      <c r="K13" s="1">
+        <v>46262</v>
+      </c>
+      <c r="L13">
+        <v>1</v>
+      </c>
+      <c r="M13" t="s">
+        <v>73</v>
+      </c>
+      <c r="N13" s="1">
+        <v>46293</v>
+      </c>
+      <c r="Q13">
+        <v>-31</v>
+      </c>
+      <c r="R13">
+        <v>0</v>
+      </c>
+      <c r="S13" t="s">
+        <v>74</v>
+      </c>
+      <c r="T13" t="s">
+        <v>75</v>
+      </c>
+      <c r="W13" t="s">
+        <v>89</v>
+      </c>
+      <c r="AA13" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (29/08/2026 01:07)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -752,10 +752,10 @@
         <v>46251</v>
       </c>
       <c r="Q2">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="R2">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="S2" t="s">
         <v>74</v>
@@ -820,10 +820,10 @@
         <v>46269</v>
       </c>
       <c r="Q3">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R3">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="S3" t="s">
         <v>74</v>
@@ -888,10 +888,10 @@
         <v>46259</v>
       </c>
       <c r="Q4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R4">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S4" t="s">
         <v>75</v>
@@ -956,10 +956,10 @@
         <v>46280</v>
       </c>
       <c r="Q5">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="R5">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S5" t="s">
         <v>74</v>
@@ -1021,10 +1021,10 @@
         <v>46283</v>
       </c>
       <c r="Q6">
-        <v>-21</v>
+        <v>-20</v>
       </c>
       <c r="R6">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S6" t="s">
         <v>74</v>
@@ -1086,10 +1086,10 @@
         <v>46262</v>
       </c>
       <c r="Q7">
-        <v>-22</v>
+        <v>-21</v>
       </c>
       <c r="R7">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="S7" t="s">
         <v>74</v>
@@ -1154,10 +1154,10 @@
         <v>46258</v>
       </c>
       <c r="Q8">
-        <v>-24</v>
+        <v>-23</v>
       </c>
       <c r="R8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S8" t="s">
         <v>74</v>
@@ -1225,10 +1225,10 @@
         <v>46258</v>
       </c>
       <c r="Q9">
-        <v>-27</v>
+        <v>-26</v>
       </c>
       <c r="R9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S9" t="s">
         <v>75</v>
@@ -1293,10 +1293,10 @@
         <v>46267</v>
       </c>
       <c r="Q10">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S10" t="s">
         <v>75</v>
@@ -1358,10 +1358,10 @@
         <v>46291</v>
       </c>
       <c r="Q11">
-        <v>-29</v>
+        <v>-28</v>
       </c>
       <c r="R11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S11" t="s">
         <v>75</v>
@@ -1426,10 +1426,10 @@
         <v>46269</v>
       </c>
       <c r="Q12">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S12" t="s">
         <v>74</v>
@@ -1488,10 +1488,10 @@
         <v>46293</v>
       </c>
       <c r="Q13">
-        <v>-31</v>
+        <v>-30</v>
       </c>
       <c r="R13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S13" t="s">
         <v>74</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (31/08/2026 14:59)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="92">
   <si>
     <t>om_emg</t>
   </si>
@@ -244,10 +244,10 @@
     <t>Sim</t>
   </si>
   <si>
-    <t>Estoque alterado de "Nao" para "SIM"  daremos prioridade para movimentar o item. Godoy 17/08/226</t>
-  </si>
-  <si>
-    <t>Emergência transformada em ANCE em 24/08. Aguardaremos atendimento com item da Vee One. Ramon 24/08/26.</t>
+    <t>Estoque alterado de "Nao" para "SIM"  daremos prioridade para movimentar o item. Godoy 17/08/26. AWB 12755178874 -  volume retirado na loja GOLLOG - NAT por Teodoro silva em 29/08. Godoy 31/08/26.</t>
+  </si>
+  <si>
+    <t>Emergência transformada em ANCE em 24/08. Aguardaremos atendimento com item da Vee One. Ramon 24/08/26. AWB 12754249845 - volume retirado na loja GOLLOG - QMA por Kleyton em 24/08. Godoy 31/08/26.</t>
   </si>
   <si>
     <t>Possui AWB ou recibo assinado? Ramon 28/08/26.</t>
@@ -259,19 +259,19 @@
     <t>item será atendido com o estoque local pedido 18295192. Godoy 26/08.</t>
   </si>
   <si>
-    <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Chegada GIG dia 15-08 (voo 4273). Entregue V1 JPA 17/08 - MATERIAL EM TRANSITO - RECIBO 722/FAB/26</t>
+    <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Chegada GIG dia 15-08 (voo 4273). Entregue V1 JPA 17/08 - MATERIAL EM TRANSITO - RECIBO 722/FAB/26 awb 12754830370 DPE 28/08/2026</t>
   </si>
   <si>
     <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
   </si>
   <si>
-    <t>ITEM FOI ENTREGUE PARA A FAB PAMALS VIA RECIBO 598/FAB/26 31-07-26 - AINDA NÃO FOI PARA O ESTOQUE CLA-17-08 - Aguardando autorização para movimentação a BANT 25/08/2026</t>
-  </si>
-  <si>
-    <t>Colocado pedido no fornecedor WAGA INTERNATIONAL - validando previsão de entrega em Miami. ATZ 25/08</t>
-  </si>
-  <si>
-    <t>Colocado pedido Textron WB0003128625 - tracking 535477333011 - previsão de entrega 25/08 V1 JPA - MATERIAL ENVIADO VIA RECIBO 726/FAB/26, AWB A SER GERADA PELA GOLLOG RC 25/08/2026</t>
+    <t>ITEM FOI ENTREGUE PARA A FAB PAMALS VIA RECIBO 598/FAB/26 31-07-26 - AINDA NÃO FOI PARA O ESTOQUE CLA-17-08 -Enviado para o Operador em 27/08/26 - AWB 12755178874 - REZ DPE 29/08/2026</t>
+  </si>
+  <si>
+    <t>Colocado pedido no fornecedor WAGA INTERNATIONAL INV26-00008 - tracking 876324334524 - previsão de entrega em Miami 31/08</t>
+  </si>
+  <si>
+    <t>Colocado pedido Textron WB0003128625 - tracking 535477333011 - previsão de entrega 25/08 V1 JPA - MATERIAL ENVIADO VIA RECIBO 726/FAB/26, AWB A SER GERADA PELA GOLLOG RC 25/08/2026 - AWB 12754866615 DPE 28/08/2026</t>
   </si>
   <si>
     <t>Colocado pedido no fornecedor I823285 - entregue em Miami 21/08 - TEMOS 3 EA NO ESTOQUE DA BANT. Material seguiu via awb 12754249845. Recebido por Kleyton em 24/08. Atl Ges.</t>
@@ -280,7 +280,13 @@
     <t>Material enviado via recibo 720/FAB/26 DPE 24/08/2026 - Retirado dia 24/08/2026 por Paula Pereira id 569968</t>
   </si>
   <si>
-    <t>Será atendido via estoque Vee One</t>
+    <t>Enviado para o Operador em 27/08/26- AWB 127-5516 5121 - REZ - MATERIAL DISPONIVEL PRA RETIRADA DIA 28/08/2026</t>
+  </si>
+  <si>
+    <t>Enviado para o Operador em 27/08/26- AWB 12755165585 - REZ DPE 01/09/2026</t>
+  </si>
+  <si>
+    <t>em cotação no mercado. ATZ 28/08</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -749,13 +755,13 @@
         <v>46243</v>
       </c>
       <c r="O2" s="1">
-        <v>46251</v>
+        <v>46262</v>
       </c>
       <c r="Q2">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="R2">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="S2" t="s">
         <v>74</v>
@@ -767,7 +773,7 @@
         <v>81</v>
       </c>
       <c r="W2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -820,10 +826,10 @@
         <v>46269</v>
       </c>
       <c r="Q3">
-        <v>-6</v>
+        <v>-4</v>
       </c>
       <c r="R3">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="S3" t="s">
         <v>74</v>
@@ -835,7 +841,7 @@
         <v>82</v>
       </c>
       <c r="W3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -885,13 +891,13 @@
         <v>46259</v>
       </c>
       <c r="O4" s="1">
-        <v>46259</v>
+        <v>46263</v>
       </c>
       <c r="Q4">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R4">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="S4" t="s">
         <v>75</v>
@@ -906,7 +912,7 @@
         <v>83</v>
       </c>
       <c r="W4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -955,11 +961,14 @@
       <c r="N5" s="1">
         <v>46280</v>
       </c>
+      <c r="O5" s="1">
+        <v>46280</v>
+      </c>
       <c r="Q5">
-        <v>-17</v>
+        <v>-15</v>
       </c>
       <c r="R5">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="S5" t="s">
         <v>74</v>
@@ -971,7 +980,7 @@
         <v>84</v>
       </c>
       <c r="W5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1021,10 +1030,10 @@
         <v>46283</v>
       </c>
       <c r="Q6">
-        <v>-20</v>
+        <v>-18</v>
       </c>
       <c r="R6">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="S6" t="s">
         <v>74</v>
@@ -1033,7 +1042,7 @@
         <v>75</v>
       </c>
       <c r="W6" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1086,10 +1095,10 @@
         <v>46262</v>
       </c>
       <c r="Q7">
-        <v>-21</v>
+        <v>-19</v>
       </c>
       <c r="R7">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="S7" t="s">
         <v>74</v>
@@ -1101,7 +1110,7 @@
         <v>85</v>
       </c>
       <c r="W7" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1154,10 +1163,10 @@
         <v>46258</v>
       </c>
       <c r="Q8">
-        <v>-23</v>
+        <v>-21</v>
       </c>
       <c r="R8">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="S8" t="s">
         <v>74</v>
@@ -1172,7 +1181,7 @@
         <v>86</v>
       </c>
       <c r="W8" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1225,10 +1234,10 @@
         <v>46258</v>
       </c>
       <c r="Q9">
-        <v>-26</v>
+        <v>-24</v>
       </c>
       <c r="R9">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="S9" t="s">
         <v>75</v>
@@ -1243,7 +1252,7 @@
         <v>87</v>
       </c>
       <c r="W9" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1292,11 +1301,14 @@
       <c r="N10" s="1">
         <v>46267</v>
       </c>
+      <c r="O10" s="1">
+        <v>46262</v>
+      </c>
       <c r="Q10">
-        <v>-4</v>
+        <v>-2</v>
       </c>
       <c r="R10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S10" t="s">
         <v>75</v>
@@ -1307,8 +1319,11 @@
       <c r="U10" t="s">
         <v>79</v>
       </c>
+      <c r="V10" t="s">
+        <v>88</v>
+      </c>
       <c r="W10" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1357,11 +1372,14 @@
       <c r="N11" s="1">
         <v>46291</v>
       </c>
+      <c r="O11" s="1">
+        <v>46266</v>
+      </c>
       <c r="Q11">
-        <v>-28</v>
+        <v>-26</v>
       </c>
       <c r="R11">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S11" t="s">
         <v>75</v>
@@ -1373,10 +1391,10 @@
         <v>80</v>
       </c>
       <c r="V11" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="W11" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1405,7 +1423,7 @@
         <v>2721</v>
       </c>
       <c r="H12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I12" t="s">
         <v>72</v>
@@ -1426,10 +1444,10 @@
         <v>46269</v>
       </c>
       <c r="Q12">
-        <v>-6</v>
+        <v>-4</v>
       </c>
       <c r="R12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S12" t="s">
         <v>74</v>
@@ -1438,7 +1456,7 @@
         <v>74</v>
       </c>
       <c r="W12" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1488,10 +1506,10 @@
         <v>46293</v>
       </c>
       <c r="Q13">
-        <v>-30</v>
+        <v>-28</v>
       </c>
       <c r="R13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S13" t="s">
         <v>74</v>
@@ -1499,8 +1517,11 @@
       <c r="T13" t="s">
         <v>75</v>
       </c>
+      <c r="V13" t="s">
+        <v>90</v>
+      </c>
       <c r="W13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (31/08/2026 20:11)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="87">
   <si>
     <t>om_emg</t>
   </si>
@@ -130,9 +130,6 @@
     <t>313260018713</t>
   </si>
   <si>
-    <t>329260019279</t>
-  </si>
-  <si>
     <t>329260019286</t>
   </si>
   <si>
@@ -166,9 +163,6 @@
     <t>2115040-8</t>
   </si>
   <si>
-    <t>2N6576</t>
-  </si>
-  <si>
     <t>C662504-0101</t>
   </si>
   <si>
@@ -199,9 +193,6 @@
     <t>CYLINDER GAS S</t>
   </si>
   <si>
-    <t>TRANSISTOR</t>
-  </si>
-  <si>
     <t>GAGE VOLT AMME</t>
   </si>
   <si>
@@ -250,9 +241,6 @@
     <t>Emergência transformada em ANCE em 24/08. Aguardaremos atendimento com item da Vee One. Ramon 24/08/26. AWB 12754249845 - volume retirado na loja GOLLOG - QMA por Kleyton em 24/08. Godoy 31/08/26.</t>
   </si>
   <si>
-    <t>Possui AWB ou recibo assinado? Ramon 28/08/26.</t>
-  </si>
-  <si>
     <t>item será atendido com o estoque local pedido 18294676. Godoy 26/08. Emg é na verdade AIFP, corrigido na planilha de 28/08. Ramon 28/08/26.</t>
   </si>
   <si>
@@ -275,9 +263,6 @@
   </si>
   <si>
     <t>Colocado pedido no fornecedor I823285 - entregue em Miami 21/08 - TEMOS 3 EA NO ESTOQUE DA BANT. Material seguiu via awb 12754249845. Recebido por Kleyton em 24/08. Atl Ges.</t>
-  </si>
-  <si>
-    <t>Material enviado via recibo 720/FAB/26 DPE 24/08/2026 - Retirado dia 24/08/2026 por Paula Pereira id 569968</t>
   </si>
   <si>
     <t>Enviado para o Operador em 27/08/26- AWB 127-5516 5121 - REZ - MATERIAL DISPONIVEL PRA RETIRADA DIA 28/08/2026</t>
@@ -625,7 +610,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA13"/>
+  <dimension ref="A1:AA12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -722,22 +707,22 @@
         <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F2" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="G2">
         <v>2702</v>
       </c>
       <c r="H2" t="s">
+        <v>64</v>
+      </c>
+      <c r="I2" t="s">
         <v>67</v>
-      </c>
-      <c r="I2" t="s">
-        <v>70</v>
       </c>
       <c r="J2" s="1">
         <v>46212</v>
@@ -749,7 +734,7 @@
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="N2" s="1">
         <v>46243</v>
@@ -764,16 +749,16 @@
         <v>53</v>
       </c>
       <c r="S2" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="T2" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="V2" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="W2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -790,22 +775,22 @@
         <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F3" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="G3">
         <v>2733</v>
       </c>
       <c r="H3" t="s">
+        <v>64</v>
+      </c>
+      <c r="I3" t="s">
         <v>67</v>
-      </c>
-      <c r="I3" t="s">
-        <v>70</v>
       </c>
       <c r="J3" s="1">
         <v>46238</v>
@@ -817,7 +802,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="N3" s="1">
         <v>46269</v>
@@ -832,16 +817,16 @@
         <v>27</v>
       </c>
       <c r="S3" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="T3" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="V3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="W3" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -858,22 +843,22 @@
         <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="G4">
         <v>2729</v>
       </c>
       <c r="H4" t="s">
+        <v>65</v>
+      </c>
+      <c r="I4" t="s">
         <v>68</v>
-      </c>
-      <c r="I4" t="s">
-        <v>71</v>
       </c>
       <c r="J4" s="1">
         <v>46248</v>
@@ -885,7 +870,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="N4" s="1">
         <v>46259</v>
@@ -900,19 +885,19 @@
         <v>17</v>
       </c>
       <c r="S4" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="T4" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="U4" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="V4" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="W4" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -929,22 +914,22 @@
         <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F5" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="G5">
         <v>2741</v>
       </c>
       <c r="H5" t="s">
+        <v>64</v>
+      </c>
+      <c r="I5" t="s">
         <v>67</v>
-      </c>
-      <c r="I5" t="s">
-        <v>70</v>
       </c>
       <c r="J5" s="1">
         <v>46251</v>
@@ -956,7 +941,7 @@
         <v>2</v>
       </c>
       <c r="M5" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="N5" s="1">
         <v>46280</v>
@@ -971,16 +956,16 @@
         <v>16</v>
       </c>
       <c r="S5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="T5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="V5" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="W5" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -997,22 +982,22 @@
         <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E6" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F6" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="G6">
         <v>2741</v>
       </c>
       <c r="H6" t="s">
+        <v>64</v>
+      </c>
+      <c r="I6" t="s">
         <v>67</v>
-      </c>
-      <c r="I6" t="s">
-        <v>70</v>
       </c>
       <c r="J6" s="1">
         <v>46253</v>
@@ -1024,7 +1009,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="N6" s="1">
         <v>46283</v>
@@ -1036,13 +1021,13 @@
         <v>13</v>
       </c>
       <c r="S6" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="T6" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="W6" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1059,22 +1044,22 @@
         <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="G7">
         <v>2731</v>
       </c>
       <c r="H7" t="s">
+        <v>64</v>
+      </c>
+      <c r="I7" t="s">
         <v>67</v>
-      </c>
-      <c r="I7" t="s">
-        <v>70</v>
       </c>
       <c r="J7" s="1">
         <v>46252</v>
@@ -1086,7 +1071,7 @@
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="N7" s="1">
         <v>46284</v>
@@ -1101,16 +1086,16 @@
         <v>12</v>
       </c>
       <c r="S7" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="T7" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="V7" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="W7" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1127,22 +1112,22 @@
         <v>37</v>
       </c>
       <c r="D8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E8" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="G8">
         <v>2737</v>
       </c>
       <c r="H8" t="s">
+        <v>64</v>
+      </c>
+      <c r="I8" t="s">
         <v>67</v>
-      </c>
-      <c r="I8" t="s">
-        <v>70</v>
       </c>
       <c r="J8" s="1">
         <v>46254</v>
@@ -1154,7 +1139,7 @@
         <v>2</v>
       </c>
       <c r="M8" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="N8" s="1">
         <v>46286</v>
@@ -1169,19 +1154,19 @@
         <v>10</v>
       </c>
       <c r="S8" t="s">
+        <v>71</v>
+      </c>
+      <c r="T8" t="s">
+        <v>72</v>
+      </c>
+      <c r="U8" t="s">
         <v>74</v>
       </c>
-      <c r="T8" t="s">
-        <v>75</v>
-      </c>
-      <c r="U8" t="s">
-        <v>77</v>
-      </c>
       <c r="V8" t="s">
+        <v>82</v>
+      </c>
+      <c r="W8" t="s">
         <v>86</v>
-      </c>
-      <c r="W8" t="s">
-        <v>91</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1198,61 +1183,61 @@
         <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E9" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F9" t="s">
+        <v>63</v>
+      </c>
+      <c r="G9">
+        <v>2709</v>
+      </c>
+      <c r="H9" t="s">
         <v>65</v>
       </c>
-      <c r="G9">
-        <v>2721</v>
-      </c>
-      <c r="H9" t="s">
-        <v>67</v>
-      </c>
       <c r="I9" t="s">
+        <v>69</v>
+      </c>
+      <c r="J9" s="1">
+        <v>46259</v>
+      </c>
+      <c r="K9" s="1">
+        <v>46260</v>
+      </c>
+      <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9" t="s">
         <v>70</v>
       </c>
-      <c r="J9" s="1">
-        <v>46255</v>
-      </c>
-      <c r="K9" s="1">
-        <v>46258</v>
-      </c>
-      <c r="L9">
-        <v>2</v>
-      </c>
-      <c r="M9" t="s">
-        <v>73</v>
-      </c>
       <c r="N9" s="1">
-        <v>46289</v>
+        <v>46267</v>
       </c>
       <c r="O9" s="1">
-        <v>46258</v>
+        <v>46262</v>
       </c>
       <c r="Q9">
-        <v>-24</v>
+        <v>-2</v>
       </c>
       <c r="R9">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="S9" t="s">
+        <v>72</v>
+      </c>
+      <c r="T9" t="s">
+        <v>71</v>
+      </c>
+      <c r="U9" t="s">
         <v>75</v>
       </c>
-      <c r="T9" t="s">
-        <v>74</v>
-      </c>
-      <c r="U9" t="s">
-        <v>78</v>
-      </c>
       <c r="V9" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="W9" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1260,31 +1245,31 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>329</v>
+        <v>396</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C10" t="s">
         <v>39</v>
       </c>
       <c r="D10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E10" t="s">
+        <v>60</v>
+      </c>
+      <c r="F10" t="s">
         <v>62</v>
       </c>
-      <c r="F10" t="s">
-        <v>66</v>
-      </c>
       <c r="G10">
-        <v>2709</v>
+        <v>2731</v>
       </c>
       <c r="H10" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="I10" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="J10" s="1">
         <v>46259</v>
@@ -1296,34 +1281,34 @@
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="N10" s="1">
-        <v>46267</v>
+        <v>46291</v>
       </c>
       <c r="O10" s="1">
-        <v>46262</v>
+        <v>46266</v>
       </c>
       <c r="Q10">
-        <v>-2</v>
+        <v>-26</v>
       </c>
       <c r="R10">
         <v>5</v>
       </c>
       <c r="S10" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="T10" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="U10" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="V10" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="W10" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1331,70 +1316,61 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>396</v>
+        <v>329</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C11" t="s">
         <v>40</v>
       </c>
       <c r="D11" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E11" t="s">
+        <v>59</v>
+      </c>
+      <c r="F11" t="s">
         <v>63</v>
       </c>
-      <c r="F11" t="s">
-        <v>65</v>
-      </c>
       <c r="G11">
-        <v>2731</v>
+        <v>2721</v>
       </c>
       <c r="H11" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="I11" t="s">
+        <v>69</v>
+      </c>
+      <c r="J11" s="1">
+        <v>46262</v>
+      </c>
+      <c r="K11" s="1">
+        <v>46262</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11" t="s">
         <v>70</v>
       </c>
-      <c r="J11" s="1">
-        <v>46259</v>
-      </c>
-      <c r="K11" s="1">
-        <v>46260</v>
-      </c>
-      <c r="L11">
-        <v>1</v>
-      </c>
-      <c r="M11" t="s">
-        <v>73</v>
-      </c>
       <c r="N11" s="1">
-        <v>46291</v>
-      </c>
-      <c r="O11" s="1">
-        <v>46266</v>
+        <v>46269</v>
       </c>
       <c r="Q11">
-        <v>-26</v>
+        <v>-4</v>
       </c>
       <c r="R11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="S11" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="T11" t="s">
-        <v>75</v>
-      </c>
-      <c r="U11" t="s">
-        <v>80</v>
-      </c>
-      <c r="V11" t="s">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="W11" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1402,10 +1378,10 @@
     </row>
     <row r="12" spans="1:27">
       <c r="A12">
-        <v>329</v>
+        <v>396</v>
       </c>
       <c r="B12" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C12" t="s">
         <v>41</v>
@@ -1414,19 +1390,19 @@
         <v>51</v>
       </c>
       <c r="E12" t="s">
+        <v>61</v>
+      </c>
+      <c r="F12" t="s">
         <v>62</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12">
+        <v>2733</v>
+      </c>
+      <c r="H12" t="s">
         <v>66</v>
       </c>
-      <c r="G12">
-        <v>2721</v>
-      </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
         <v>67</v>
-      </c>
-      <c r="I12" t="s">
-        <v>72</v>
       </c>
       <c r="J12" s="1">
         <v>46262</v>
@@ -1438,92 +1414,30 @@
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="N12" s="1">
-        <v>46269</v>
+        <v>46293</v>
       </c>
       <c r="Q12">
-        <v>-4</v>
+        <v>-28</v>
       </c>
       <c r="R12">
         <v>3</v>
       </c>
       <c r="S12" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="T12" t="s">
-        <v>74</v>
+        <v>72</v>
+      </c>
+      <c r="V12" t="s">
+        <v>85</v>
       </c>
       <c r="W12" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="AA12" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:27">
-      <c r="A13">
-        <v>396</v>
-      </c>
-      <c r="B13" t="s">
-        <v>28</v>
-      </c>
-      <c r="C13" t="s">
-        <v>42</v>
-      </c>
-      <c r="D13" t="s">
-        <v>53</v>
-      </c>
-      <c r="E13" t="s">
-        <v>64</v>
-      </c>
-      <c r="F13" t="s">
-        <v>65</v>
-      </c>
-      <c r="G13">
-        <v>2733</v>
-      </c>
-      <c r="H13" t="s">
-        <v>69</v>
-      </c>
-      <c r="I13" t="s">
-        <v>70</v>
-      </c>
-      <c r="J13" s="1">
-        <v>46262</v>
-      </c>
-      <c r="K13" s="1">
-        <v>46262</v>
-      </c>
-      <c r="L13">
-        <v>1</v>
-      </c>
-      <c r="M13" t="s">
-        <v>73</v>
-      </c>
-      <c r="N13" s="1">
-        <v>46293</v>
-      </c>
-      <c r="Q13">
-        <v>-28</v>
-      </c>
-      <c r="R13">
-        <v>3</v>
-      </c>
-      <c r="S13" t="s">
-        <v>74</v>
-      </c>
-      <c r="T13" t="s">
-        <v>75</v>
-      </c>
-      <c r="V13" t="s">
-        <v>90</v>
-      </c>
-      <c r="W13" t="s">
-        <v>91</v>
-      </c>
-      <c r="AA13" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (01/09/2026 11:15)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="90">
   <si>
     <t>om_emg</t>
   </si>
@@ -109,15 +109,15 @@
     <t>BABR</t>
   </si>
   <si>
+    <t>BACG</t>
+  </si>
+  <si>
     <t>685260012350</t>
   </si>
   <si>
     <t>396260016580</t>
   </si>
   <si>
-    <t>685260012609</t>
-  </si>
-  <si>
     <t>313260018702</t>
   </si>
   <si>
@@ -133,24 +133,27 @@
     <t>329260019286</t>
   </si>
   <si>
-    <t>396260016593</t>
-  </si>
-  <si>
     <t>329260019288</t>
   </si>
   <si>
     <t>396260016603</t>
   </si>
   <si>
+    <t>396260016605</t>
+  </si>
+  <si>
+    <t>396260016606</t>
+  </si>
+  <si>
+    <t>690260002556</t>
+  </si>
+  <si>
     <t>030-1094-58</t>
   </si>
   <si>
     <t>2601188-204</t>
   </si>
   <si>
-    <t>162-10700</t>
-  </si>
-  <si>
     <t>040-0043</t>
   </si>
   <si>
@@ -166,21 +169,24 @@
     <t>C662504-0101</t>
   </si>
   <si>
-    <t>4626</t>
-  </si>
-  <si>
     <t>OD1232-24MB</t>
   </si>
   <si>
+    <t>2641011-5</t>
+  </si>
+  <si>
+    <t>030-18200</t>
+  </si>
+  <si>
+    <t>C592001-0206</t>
+  </si>
+  <si>
     <t>CONNECTOR</t>
   </si>
   <si>
     <t>COMPRESSOR DRIVE ASS</t>
   </si>
   <si>
-    <t>OUTER WHEEL HALF ASS</t>
-  </si>
-  <si>
     <t>STROB TUB</t>
   </si>
   <si>
@@ -196,12 +202,18 @@
     <t>GAGE VOLT AMME</t>
   </si>
   <si>
-    <t>LAMP,INCANDESCENT</t>
-  </si>
-  <si>
     <t>DC FAN</t>
   </si>
   <si>
+    <t>AXLE-MAIN GEAR</t>
+  </si>
+  <si>
+    <t>MAIN WHEEL BRAKE</t>
+  </si>
+  <si>
+    <t>WICK-STAT DISC</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -220,9 +232,6 @@
     <t>ANCE</t>
   </si>
   <si>
-    <t>IPLR</t>
-  </si>
-  <si>
     <t>AIFP</t>
   </si>
   <si>
@@ -235,7 +244,10 @@
     <t>Sim</t>
   </si>
   <si>
-    <t>Estoque alterado de "Nao" para "SIM"  daremos prioridade para movimentar o item. Godoy 17/08/26. AWB 12755178874 -  volume retirado na loja GOLLOG - NAT por Teodoro silva em 29/08. Godoy 31/08/26.</t>
+    <t>AWB 12754830370 -  volume retirado na loja GOLLOG - NAT por Teodoro silva em 29/08. Godoy 01/09/26.</t>
+  </si>
+  <si>
+    <t>AWB 12754866615 -  volume retirado na loja GOLLOG - BEL por Marcos bispo em 31/08. Godoy 01/09/26.</t>
   </si>
   <si>
     <t>Emergência transformada em ANCE em 24/08. Aguardaremos atendimento com item da Vee One. Ramon 24/08/26. AWB 12754249845 - volume retirado na loja GOLLOG - QMA por Kleyton em 24/08. Godoy 31/08/26.</t>
@@ -244,31 +256,28 @@
     <t>item será atendido com o estoque local pedido 18294676. Godoy 26/08. Emg é na verdade AIFP, corrigido na planilha de 28/08. Ramon 28/08/26.</t>
   </si>
   <si>
-    <t>item será atendido com o estoque local pedido 18295192. Godoy 26/08.</t>
-  </si>
-  <si>
-    <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Chegada GIG dia 15-08 (voo 4273). Entregue V1 JPA 17/08 - MATERIAL EM TRANSITO - RECIBO 722/FAB/26 awb 12754830370 DPE 28/08/2026</t>
+    <t>Cedeu o item para o 2739. Ramon 01/09/26</t>
+  </si>
+  <si>
+    <t>Cedeu o item para o 2733. Ramon 01/09/26</t>
+  </si>
+  <si>
+    <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Chegada GIG dia 15-08 (voo 4273). Entregue V1 JPA 17/08 - MATERIAL EM TRANSITO - RECIBO 722/FAB/26 awb 12754830370 DPE 28/08/2026 - entregue 29/08/2026</t>
   </si>
   <si>
     <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
   </si>
   <si>
-    <t>ITEM FOI ENTREGUE PARA A FAB PAMALS VIA RECIBO 598/FAB/26 31-07-26 - AINDA NÃO FOI PARA O ESTOQUE CLA-17-08 -Enviado para o Operador em 27/08/26 - AWB 12755178874 - REZ DPE 29/08/2026</t>
-  </si>
-  <si>
     <t>Colocado pedido no fornecedor WAGA INTERNATIONAL INV26-00008 - tracking 876324334524 - previsão de entrega em Miami 31/08</t>
   </si>
   <si>
-    <t>Colocado pedido Textron WB0003128625 - tracking 535477333011 - previsão de entrega 25/08 V1 JPA - MATERIAL ENVIADO VIA RECIBO 726/FAB/26, AWB A SER GERADA PELA GOLLOG RC 25/08/2026 - AWB 12754866615 DPE 28/08/2026</t>
+    <t>Colocado pedido Textron WB0003128625 - tracking 535477333011 - previsão de entrega 25/08 V1 JPA - MATERIAL ENVIADO VIA RECIBO 726/FAB/26, AWB A SER GERADA PELA GOLLOG RC 25/08/2026 - AWB 12754866615 DPE 28/08/2026 - recebido dia 31/08/2026</t>
   </si>
   <si>
     <t>Colocado pedido no fornecedor I823285 - entregue em Miami 21/08 - TEMOS 3 EA NO ESTOQUE DA BANT. Material seguiu via awb 12754249845. Recebido por Kleyton em 24/08. Atl Ges.</t>
   </si>
   <si>
     <t>Enviado para o Operador em 27/08/26- AWB 127-5516 5121 - REZ - MATERIAL DISPONIVEL PRA RETIRADA DIA 28/08/2026</t>
-  </si>
-  <si>
-    <t>Enviado para o Operador em 27/08/26- AWB 12755165585 - REZ DPE 01/09/2026</t>
   </si>
   <si>
     <t>em cotação no mercado. ATZ 28/08</t>
@@ -284,8 +293,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -301,7 +318,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -309,12 +326,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -610,89 +645,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA12"/>
+  <dimension ref="A1:AA13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -704,61 +739,64 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="G2">
         <v>2702</v>
       </c>
       <c r="H2" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="I2" t="s">
-        <v>67</v>
-      </c>
-      <c r="J2" s="1">
+        <v>71</v>
+      </c>
+      <c r="J2" s="2">
         <v>46212</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46212</v>
       </c>
       <c r="L2">
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>70</v>
-      </c>
-      <c r="N2" s="1">
+        <v>73</v>
+      </c>
+      <c r="N2" s="2">
         <v>46243</v>
       </c>
-      <c r="O2" s="1">
-        <v>46262</v>
+      <c r="O2" s="2">
+        <v>46263</v>
       </c>
       <c r="Q2">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="R2">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="S2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="T2" t="s">
-        <v>72</v>
+        <v>75</v>
+      </c>
+      <c r="U2" t="s">
+        <v>76</v>
       </c>
       <c r="V2" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="W2" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -772,61 +810,61 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F3" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="G3">
         <v>2733</v>
       </c>
       <c r="H3" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="I3" t="s">
-        <v>67</v>
-      </c>
-      <c r="J3" s="1">
+        <v>71</v>
+      </c>
+      <c r="J3" s="2">
         <v>46238</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46238</v>
       </c>
       <c r="L3">
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>70</v>
-      </c>
-      <c r="N3" s="1">
+        <v>73</v>
+      </c>
+      <c r="N3" s="2">
         <v>46269</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46269</v>
       </c>
       <c r="Q3">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R3">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="S3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="T3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="V3" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="W3" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -834,70 +872,67 @@
     </row>
     <row r="4" spans="1:27">
       <c r="A4">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E4" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F4" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G4">
-        <v>2729</v>
+        <v>2741</v>
       </c>
       <c r="H4" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="I4" t="s">
-        <v>68</v>
-      </c>
-      <c r="J4" s="1">
-        <v>46248</v>
-      </c>
-      <c r="K4" s="1">
-        <v>46248</v>
+        <v>71</v>
+      </c>
+      <c r="J4" s="2">
+        <v>46251</v>
+      </c>
+      <c r="K4" s="2">
+        <v>46249</v>
       </c>
       <c r="L4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M4" t="s">
-        <v>70</v>
-      </c>
-      <c r="N4" s="1">
-        <v>46259</v>
-      </c>
-      <c r="O4" s="1">
-        <v>46263</v>
+        <v>73</v>
+      </c>
+      <c r="N4" s="2">
+        <v>46280</v>
+      </c>
+      <c r="O4" s="2">
+        <v>46280</v>
       </c>
       <c r="Q4">
-        <v>6</v>
+        <v>-14</v>
       </c>
       <c r="R4">
         <v>17</v>
       </c>
       <c r="S4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="T4" t="s">
-        <v>72</v>
-      </c>
-      <c r="U4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="V4" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="W4" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -911,61 +946,55 @@
         <v>29</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="F5" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="G5">
         <v>2741</v>
       </c>
       <c r="H5" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="I5" t="s">
-        <v>67</v>
-      </c>
-      <c r="J5" s="1">
-        <v>46251</v>
-      </c>
-      <c r="K5" s="1">
-        <v>46249</v>
+        <v>71</v>
+      </c>
+      <c r="J5" s="2">
+        <v>46253</v>
+      </c>
+      <c r="K5" s="2">
+        <v>46252</v>
       </c>
       <c r="L5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>70</v>
-      </c>
-      <c r="N5" s="1">
-        <v>46280</v>
-      </c>
-      <c r="O5" s="1">
-        <v>46280</v>
+        <v>73</v>
+      </c>
+      <c r="N5" s="2">
+        <v>46283</v>
       </c>
       <c r="Q5">
-        <v>-15</v>
+        <v>-17</v>
       </c>
       <c r="R5">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="S5" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="T5" t="s">
-        <v>72</v>
-      </c>
-      <c r="V5" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="W5" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -973,46 +1002,49 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6">
-        <v>313</v>
+        <v>396</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E6" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="F6" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G6">
-        <v>2741</v>
+        <v>2731</v>
       </c>
       <c r="H6" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="I6" t="s">
-        <v>67</v>
-      </c>
-      <c r="J6" s="1">
+        <v>71</v>
+      </c>
+      <c r="J6" s="2">
+        <v>46252</v>
+      </c>
+      <c r="K6" s="2">
         <v>46253</v>
       </c>
-      <c r="K6" s="1">
-        <v>46252</v>
-      </c>
       <c r="L6">
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>70</v>
-      </c>
-      <c r="N6" s="1">
-        <v>46283</v>
+        <v>73</v>
+      </c>
+      <c r="N6" s="2">
+        <v>46284</v>
+      </c>
+      <c r="O6" s="2">
+        <v>46265</v>
       </c>
       <c r="Q6">
         <v>-18</v>
@@ -1021,13 +1053,19 @@
         <v>13</v>
       </c>
       <c r="S6" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="T6" t="s">
-        <v>72</v>
+        <v>75</v>
+      </c>
+      <c r="U6" t="s">
+        <v>77</v>
+      </c>
+      <c r="V6" t="s">
+        <v>85</v>
       </c>
       <c r="W6" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1035,67 +1073,70 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>396</v>
+        <v>313</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E7" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F7" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="G7">
-        <v>2731</v>
+        <v>2737</v>
       </c>
       <c r="H7" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="I7" t="s">
-        <v>67</v>
-      </c>
-      <c r="J7" s="1">
-        <v>46252</v>
-      </c>
-      <c r="K7" s="1">
-        <v>46253</v>
+        <v>71</v>
+      </c>
+      <c r="J7" s="2">
+        <v>46254</v>
+      </c>
+      <c r="K7" s="2">
+        <v>46255</v>
       </c>
       <c r="L7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M7" t="s">
-        <v>70</v>
-      </c>
-      <c r="N7" s="1">
-        <v>46284</v>
-      </c>
-      <c r="O7" s="1">
-        <v>46262</v>
+        <v>73</v>
+      </c>
+      <c r="N7" s="2">
+        <v>46286</v>
+      </c>
+      <c r="O7" s="2">
+        <v>46258</v>
       </c>
       <c r="Q7">
-        <v>-19</v>
+        <v>-20</v>
       </c>
       <c r="R7">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="S7" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="T7" t="s">
-        <v>72</v>
+        <v>75</v>
+      </c>
+      <c r="U7" t="s">
+        <v>78</v>
       </c>
       <c r="V7" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="W7" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1103,70 +1144,70 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E8" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="F8" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="G8">
-        <v>2737</v>
+        <v>2709</v>
       </c>
       <c r="H8" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="I8" t="s">
-        <v>67</v>
-      </c>
-      <c r="J8" s="1">
-        <v>46254</v>
-      </c>
-      <c r="K8" s="1">
-        <v>46255</v>
+        <v>72</v>
+      </c>
+      <c r="J8" s="2">
+        <v>46259</v>
+      </c>
+      <c r="K8" s="2">
+        <v>46260</v>
       </c>
       <c r="L8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>70</v>
-      </c>
-      <c r="N8" s="1">
-        <v>46286</v>
-      </c>
-      <c r="O8" s="1">
-        <v>46258</v>
+        <v>73</v>
+      </c>
+      <c r="N8" s="2">
+        <v>46267</v>
+      </c>
+      <c r="O8" s="2">
+        <v>46262</v>
       </c>
       <c r="Q8">
-        <v>-21</v>
+        <v>-1</v>
       </c>
       <c r="R8">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="S8" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="T8" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="U8" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="V8" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="W8" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1180,64 +1221,55 @@
         <v>30</v>
       </c>
       <c r="C9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F9" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="G9">
-        <v>2709</v>
+        <v>2721</v>
       </c>
       <c r="H9" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="I9" t="s">
-        <v>69</v>
-      </c>
-      <c r="J9" s="1">
-        <v>46259</v>
-      </c>
-      <c r="K9" s="1">
-        <v>46260</v>
+        <v>72</v>
+      </c>
+      <c r="J9" s="2">
+        <v>46262</v>
+      </c>
+      <c r="K9" s="2">
+        <v>46262</v>
       </c>
       <c r="L9">
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>70</v>
-      </c>
-      <c r="N9" s="1">
-        <v>46267</v>
-      </c>
-      <c r="O9" s="1">
-        <v>46262</v>
+        <v>73</v>
+      </c>
+      <c r="N9" s="2">
+        <v>46269</v>
       </c>
       <c r="Q9">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="R9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S9" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="T9" t="s">
-        <v>71</v>
-      </c>
-      <c r="U9" t="s">
-        <v>75</v>
-      </c>
-      <c r="V9" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="W9" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1251,64 +1283,58 @@
         <v>28</v>
       </c>
       <c r="C10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F10" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="G10">
-        <v>2731</v>
+        <v>2733</v>
       </c>
       <c r="H10" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="I10" t="s">
-        <v>67</v>
-      </c>
-      <c r="J10" s="1">
-        <v>46259</v>
-      </c>
-      <c r="K10" s="1">
-        <v>46260</v>
+        <v>71</v>
+      </c>
+      <c r="J10" s="2">
+        <v>46262</v>
+      </c>
+      <c r="K10" s="2">
+        <v>46262</v>
       </c>
       <c r="L10">
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>70</v>
-      </c>
-      <c r="N10" s="1">
-        <v>46291</v>
-      </c>
-      <c r="O10" s="1">
-        <v>46266</v>
+        <v>73</v>
+      </c>
+      <c r="N10" s="2">
+        <v>46293</v>
       </c>
       <c r="Q10">
-        <v>-26</v>
+        <v>-27</v>
       </c>
       <c r="R10">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S10" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="T10" t="s">
-        <v>72</v>
-      </c>
-      <c r="U10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="V10" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="W10" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1316,61 +1342,64 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>329</v>
+        <v>396</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D11" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E11" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F11" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="G11">
-        <v>2721</v>
+        <v>2731</v>
       </c>
       <c r="H11" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="I11" t="s">
-        <v>69</v>
-      </c>
-      <c r="J11" s="1">
-        <v>46262</v>
-      </c>
-      <c r="K11" s="1">
-        <v>46262</v>
+        <v>72</v>
+      </c>
+      <c r="J11" s="2">
+        <v>46265</v>
+      </c>
+      <c r="K11" s="2">
+        <v>46266</v>
       </c>
       <c r="L11">
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>70</v>
-      </c>
-      <c r="N11" s="1">
-        <v>46269</v>
+        <v>73</v>
+      </c>
+      <c r="N11" s="2">
+        <v>46273</v>
       </c>
       <c r="Q11">
-        <v>-4</v>
+        <v>-7</v>
       </c>
       <c r="R11">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S11" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="T11" t="s">
-        <v>71</v>
+        <v>75</v>
+      </c>
+      <c r="U11" t="s">
+        <v>80</v>
       </c>
       <c r="W11" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1384,60 +1413,122 @@
         <v>28</v>
       </c>
       <c r="C12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D12" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E12" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="F12" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="G12">
-        <v>2733</v>
+        <v>2731</v>
       </c>
       <c r="H12" t="s">
+        <v>70</v>
+      </c>
+      <c r="I12" t="s">
+        <v>72</v>
+      </c>
+      <c r="J12" s="2">
+        <v>46265</v>
+      </c>
+      <c r="K12" s="2">
+        <v>46266</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12" t="s">
+        <v>73</v>
+      </c>
+      <c r="N12" s="2">
+        <v>46273</v>
+      </c>
+      <c r="Q12">
+        <v>-7</v>
+      </c>
+      <c r="R12">
+        <v>0</v>
+      </c>
+      <c r="S12" t="s">
+        <v>75</v>
+      </c>
+      <c r="T12" t="s">
+        <v>75</v>
+      </c>
+      <c r="U12" t="s">
+        <v>81</v>
+      </c>
+      <c r="W12" t="s">
+        <v>89</v>
+      </c>
+      <c r="AA12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27">
+      <c r="A13">
+        <v>690</v>
+      </c>
+      <c r="B13" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" t="s">
+        <v>54</v>
+      </c>
+      <c r="E13" t="s">
+        <v>65</v>
+      </c>
+      <c r="F13" t="s">
         <v>66</v>
       </c>
-      <c r="I12" t="s">
-        <v>67</v>
-      </c>
-      <c r="J12" s="1">
-        <v>46262</v>
-      </c>
-      <c r="K12" s="1">
-        <v>46262</v>
-      </c>
-      <c r="L12">
-        <v>1</v>
-      </c>
-      <c r="M12" t="s">
+      <c r="G13">
+        <v>2727</v>
+      </c>
+      <c r="H13" t="s">
         <v>70</v>
       </c>
-      <c r="N12" s="1">
-        <v>46293</v>
-      </c>
-      <c r="Q12">
-        <v>-28</v>
-      </c>
-      <c r="R12">
-        <v>3</v>
-      </c>
-      <c r="S12" t="s">
+      <c r="I13" t="s">
         <v>71</v>
       </c>
-      <c r="T12" t="s">
-        <v>72</v>
-      </c>
-      <c r="V12" t="s">
-        <v>85</v>
-      </c>
-      <c r="W12" t="s">
-        <v>86</v>
-      </c>
-      <c r="AA12" t="b">
+      <c r="J13" s="2">
+        <v>46265</v>
+      </c>
+      <c r="K13" s="2">
+        <v>46266</v>
+      </c>
+      <c r="L13">
+        <v>5</v>
+      </c>
+      <c r="M13" t="s">
+        <v>73</v>
+      </c>
+      <c r="N13" s="2">
+        <v>46297</v>
+      </c>
+      <c r="Q13">
+        <v>-31</v>
+      </c>
+      <c r="R13">
+        <v>0</v>
+      </c>
+      <c r="S13" t="s">
+        <v>75</v>
+      </c>
+      <c r="T13" t="s">
+        <v>74</v>
+      </c>
+      <c r="W13" t="s">
+        <v>89</v>
+      </c>
+      <c r="AA13" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (01/09/2026 12:27)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -293,16 +293,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -318,7 +310,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -326,30 +318,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -649,85 +623,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -759,10 +733,10 @@
       <c r="I2" t="s">
         <v>71</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>46212</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46212</v>
       </c>
       <c r="L2">
@@ -771,10 +745,10 @@
       <c r="M2" t="s">
         <v>73</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="1">
         <v>46243</v>
       </c>
-      <c r="O2" s="2">
+      <c r="O2" s="1">
         <v>46263</v>
       </c>
       <c r="Q2">
@@ -830,10 +804,10 @@
       <c r="I3" t="s">
         <v>71</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>46238</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46238</v>
       </c>
       <c r="L3">
@@ -842,10 +816,10 @@
       <c r="M3" t="s">
         <v>73</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="1">
         <v>46269</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46269</v>
       </c>
       <c r="Q3">
@@ -898,10 +872,10 @@
       <c r="I4" t="s">
         <v>71</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>46251</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46249</v>
       </c>
       <c r="L4">
@@ -910,10 +884,10 @@
       <c r="M4" t="s">
         <v>73</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="1">
         <v>46280</v>
       </c>
-      <c r="O4" s="2">
+      <c r="O4" s="1">
         <v>46280</v>
       </c>
       <c r="Q4">
@@ -966,10 +940,10 @@
       <c r="I5" t="s">
         <v>71</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>46253</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46252</v>
       </c>
       <c r="L5">
@@ -978,7 +952,7 @@
       <c r="M5" t="s">
         <v>73</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="1">
         <v>46283</v>
       </c>
       <c r="Q5">
@@ -1028,10 +1002,10 @@
       <c r="I6" t="s">
         <v>71</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>46252</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46253</v>
       </c>
       <c r="L6">
@@ -1040,10 +1014,10 @@
       <c r="M6" t="s">
         <v>73</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="1">
         <v>46284</v>
       </c>
-      <c r="O6" s="2">
+      <c r="O6" s="1">
         <v>46265</v>
       </c>
       <c r="Q6">
@@ -1099,10 +1073,10 @@
       <c r="I7" t="s">
         <v>71</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46254</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>46255</v>
       </c>
       <c r="L7">
@@ -1111,10 +1085,10 @@
       <c r="M7" t="s">
         <v>73</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="1">
         <v>46286</v>
       </c>
-      <c r="O7" s="2">
+      <c r="O7" s="1">
         <v>46258</v>
       </c>
       <c r="Q7">
@@ -1170,10 +1144,10 @@
       <c r="I8" t="s">
         <v>72</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46259</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>46260</v>
       </c>
       <c r="L8">
@@ -1182,10 +1156,10 @@
       <c r="M8" t="s">
         <v>73</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="1">
         <v>46267</v>
       </c>
-      <c r="O8" s="2">
+      <c r="O8" s="1">
         <v>46262</v>
       </c>
       <c r="Q8">
@@ -1241,10 +1215,10 @@
       <c r="I9" t="s">
         <v>72</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46262</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>46262</v>
       </c>
       <c r="L9">
@@ -1253,7 +1227,7 @@
       <c r="M9" t="s">
         <v>73</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="1">
         <v>46269</v>
       </c>
       <c r="Q9">
@@ -1303,10 +1277,10 @@
       <c r="I10" t="s">
         <v>71</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>46262</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>46262</v>
       </c>
       <c r="L10">
@@ -1315,7 +1289,7 @@
       <c r="M10" t="s">
         <v>73</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="1">
         <v>46293</v>
       </c>
       <c r="Q10">
@@ -1368,10 +1342,10 @@
       <c r="I11" t="s">
         <v>72</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46265</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>46266</v>
       </c>
       <c r="L11">
@@ -1380,7 +1354,7 @@
       <c r="M11" t="s">
         <v>73</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11" s="1">
         <v>46273</v>
       </c>
       <c r="Q11">
@@ -1433,10 +1407,10 @@
       <c r="I12" t="s">
         <v>72</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>46265</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>46266</v>
       </c>
       <c r="L12">
@@ -1445,7 +1419,7 @@
       <c r="M12" t="s">
         <v>73</v>
       </c>
-      <c r="N12" s="2">
+      <c r="N12" s="1">
         <v>46273</v>
       </c>
       <c r="Q12">
@@ -1498,10 +1472,10 @@
       <c r="I13" t="s">
         <v>71</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46265</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>46266</v>
       </c>
       <c r="L13">
@@ -1510,7 +1484,7 @@
       <c r="M13" t="s">
         <v>73</v>
       </c>
-      <c r="N13" s="2">
+      <c r="N13" s="1">
         <v>46297</v>
       </c>
       <c r="Q13">

</xml_diff>

<commit_message>
Atualização automática: emergencias (02/09/2026 09:38)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="94">
   <si>
     <t>om_emg</t>
   </si>
@@ -250,7 +250,7 @@
     <t>AWB 12754866615 -  volume retirado na loja GOLLOG - BEL por Marcos bispo em 31/08. Godoy 01/09/26.</t>
   </si>
   <si>
-    <t>Emergência transformada em ANCE em 24/08. Aguardaremos atendimento com item da Vee One. Ramon 24/08/26. AWB 12754249845 - volume retirado na loja GOLLOG - QMA por Kleyton em 24/08. Godoy 31/08/26.</t>
+    <t>Emergência transformada em ANCE em 24/08. Aguardaremos atendimento com item da Vee One. Ramon 24/08/26.</t>
   </si>
   <si>
     <t>item será atendido com o estoque local pedido 18294676. Godoy 26/08. Emg é na verdade AIFP, corrigido na planilha de 28/08. Ramon 28/08/26.</t>
@@ -259,7 +259,7 @@
     <t>Cedeu o item para o 2739. Ramon 01/09/26</t>
   </si>
   <si>
-    <t>Cedeu o item para o 2733. Ramon 01/09/26</t>
+    <t>Cedeu o item para o 2733. Ramon 01/09/26. AWB 112755521406 - volume retirado na loja GOLLOG - BEL por Marlon bispo em 01/09. Godoy 02/09/26. Recibo 734/FAB/26 assinado em 01/09. Ramon 02/09/26.</t>
   </si>
   <si>
     <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Chegada GIG dia 15-08 (voo 4273). Entregue V1 JPA 17/08 - MATERIAL EM TRANSITO - RECIBO 722/FAB/26 awb 12754830370 DPE 28/08/2026 - entregue 29/08/2026</t>
@@ -280,7 +280,19 @@
     <t>Enviado para o Operador em 27/08/26- AWB 127-5516 5121 - REZ - MATERIAL DISPONIVEL PRA RETIRADA DIA 28/08/2026</t>
   </si>
   <si>
-    <t>em cotação no mercado. ATZ 28/08</t>
+    <t>EM REPARO NA WILLIAM, DPE (confirmado) dia 02/09/2026 - REZ</t>
+  </si>
+  <si>
+    <t>Colocado pedido WB0003139756 - previsão de entrega em Miami 02/09</t>
+  </si>
+  <si>
+    <t>material será atendido pelo item reparado no estoque V1 01/09/2026</t>
+  </si>
+  <si>
+    <t>Material enviado dia 31/08/2026 VIA AWB 12755521406 DPE 01/09/2026</t>
+  </si>
+  <si>
+    <t>Não temos em estoque, podemos movimentar o estoque da FAB para atendimento? RC 01/09/2026</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -293,8 +305,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -310,7 +330,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -318,12 +338,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -623,85 +661,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -733,10 +771,10 @@
       <c r="I2" t="s">
         <v>71</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>46212</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46212</v>
       </c>
       <c r="L2">
@@ -745,17 +783,17 @@
       <c r="M2" t="s">
         <v>73</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <v>46243</v>
       </c>
-      <c r="O2" s="1">
+      <c r="O2" s="2">
         <v>46263</v>
       </c>
       <c r="Q2">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="R2">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="S2" t="s">
         <v>74</v>
@@ -770,7 +808,7 @@
         <v>82</v>
       </c>
       <c r="W2" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -804,10 +842,10 @@
       <c r="I3" t="s">
         <v>71</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>46238</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46238</v>
       </c>
       <c r="L3">
@@ -816,17 +854,17 @@
       <c r="M3" t="s">
         <v>73</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <v>46269</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46269</v>
       </c>
       <c r="Q3">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R3">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S3" t="s">
         <v>74</v>
@@ -838,7 +876,7 @@
         <v>83</v>
       </c>
       <c r="W3" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -872,10 +910,10 @@
       <c r="I4" t="s">
         <v>71</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>46251</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46249</v>
       </c>
       <c r="L4">
@@ -884,17 +922,17 @@
       <c r="M4" t="s">
         <v>73</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="2">
         <v>46280</v>
       </c>
-      <c r="O4" s="1">
+      <c r="O4" s="2">
         <v>46280</v>
       </c>
       <c r="Q4">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="R4">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="S4" t="s">
         <v>74</v>
@@ -906,7 +944,7 @@
         <v>84</v>
       </c>
       <c r="W4" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -940,10 +978,10 @@
       <c r="I5" t="s">
         <v>71</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>46253</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46252</v>
       </c>
       <c r="L5">
@@ -952,14 +990,14 @@
       <c r="M5" t="s">
         <v>73</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <v>46283</v>
       </c>
       <c r="Q5">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="R5">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S5" t="s">
         <v>74</v>
@@ -968,7 +1006,7 @@
         <v>75</v>
       </c>
       <c r="W5" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1002,10 +1040,10 @@
       <c r="I6" t="s">
         <v>71</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>46252</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46253</v>
       </c>
       <c r="L6">
@@ -1014,17 +1052,17 @@
       <c r="M6" t="s">
         <v>73</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <v>46284</v>
       </c>
-      <c r="O6" s="1">
+      <c r="O6" s="2">
         <v>46265</v>
       </c>
       <c r="Q6">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="R6">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S6" t="s">
         <v>74</v>
@@ -1039,7 +1077,7 @@
         <v>85</v>
       </c>
       <c r="W6" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1073,10 +1111,10 @@
       <c r="I7" t="s">
         <v>71</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46254</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46255</v>
       </c>
       <c r="L7">
@@ -1085,17 +1123,17 @@
       <c r="M7" t="s">
         <v>73</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="2">
         <v>46286</v>
       </c>
-      <c r="O7" s="1">
+      <c r="O7" s="2">
         <v>46258</v>
       </c>
       <c r="Q7">
-        <v>-20</v>
+        <v>-19</v>
       </c>
       <c r="R7">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="S7" t="s">
         <v>74</v>
@@ -1110,7 +1148,7 @@
         <v>86</v>
       </c>
       <c r="W7" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1144,10 +1182,10 @@
       <c r="I8" t="s">
         <v>72</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46259</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46260</v>
       </c>
       <c r="L8">
@@ -1156,17 +1194,17 @@
       <c r="M8" t="s">
         <v>73</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="2">
         <v>46267</v>
       </c>
-      <c r="O8" s="1">
+      <c r="O8" s="2">
         <v>46262</v>
       </c>
       <c r="Q8">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S8" t="s">
         <v>75</v>
@@ -1181,7 +1219,7 @@
         <v>87</v>
       </c>
       <c r="W8" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1215,10 +1253,10 @@
       <c r="I9" t="s">
         <v>72</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46262</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46262</v>
       </c>
       <c r="L9">
@@ -1227,14 +1265,14 @@
       <c r="M9" t="s">
         <v>73</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>46269</v>
       </c>
       <c r="Q9">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S9" t="s">
         <v>74</v>
@@ -1242,8 +1280,11 @@
       <c r="T9" t="s">
         <v>74</v>
       </c>
+      <c r="V9" t="s">
+        <v>88</v>
+      </c>
       <c r="W9" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1277,10 +1318,10 @@
       <c r="I10" t="s">
         <v>71</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46262</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>46262</v>
       </c>
       <c r="L10">
@@ -1289,14 +1330,17 @@
       <c r="M10" t="s">
         <v>73</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
         <v>46293</v>
       </c>
+      <c r="O10" s="2">
+        <v>46293</v>
+      </c>
       <c r="Q10">
-        <v>-27</v>
+        <v>-26</v>
       </c>
       <c r="R10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S10" t="s">
         <v>74</v>
@@ -1305,10 +1349,10 @@
         <v>75</v>
       </c>
       <c r="V10" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="W10" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1342,10 +1386,10 @@
       <c r="I11" t="s">
         <v>72</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46265</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>46266</v>
       </c>
       <c r="L11">
@@ -1354,14 +1398,17 @@
       <c r="M11" t="s">
         <v>73</v>
       </c>
-      <c r="N11" s="1">
+      <c r="N11" s="2">
         <v>46273</v>
       </c>
+      <c r="O11" s="2">
+        <v>46267</v>
+      </c>
       <c r="Q11">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S11" t="s">
         <v>75</v>
@@ -1372,8 +1419,11 @@
       <c r="U11" t="s">
         <v>80</v>
       </c>
+      <c r="V11" t="s">
+        <v>90</v>
+      </c>
       <c r="W11" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1407,10 +1457,10 @@
       <c r="I12" t="s">
         <v>72</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>46265</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>46266</v>
       </c>
       <c r="L12">
@@ -1419,14 +1469,17 @@
       <c r="M12" t="s">
         <v>73</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="2">
         <v>46273</v>
       </c>
+      <c r="O12" s="2">
+        <v>46266</v>
+      </c>
       <c r="Q12">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S12" t="s">
         <v>75</v>
@@ -1437,8 +1490,11 @@
       <c r="U12" t="s">
         <v>81</v>
       </c>
+      <c r="V12" t="s">
+        <v>91</v>
+      </c>
       <c r="W12" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1472,10 +1528,10 @@
       <c r="I13" t="s">
         <v>71</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46265</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>46266</v>
       </c>
       <c r="L13">
@@ -1484,14 +1540,17 @@
       <c r="M13" t="s">
         <v>73</v>
       </c>
-      <c r="N13" s="1">
+      <c r="N13" s="2">
         <v>46297</v>
       </c>
+      <c r="O13" s="2">
+        <v>46297</v>
+      </c>
       <c r="Q13">
-        <v>-31</v>
+        <v>-30</v>
       </c>
       <c r="R13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S13" t="s">
         <v>75</v>
@@ -1499,8 +1558,11 @@
       <c r="T13" t="s">
         <v>74</v>
       </c>
+      <c r="V13" t="s">
+        <v>92</v>
+      </c>
       <c r="W13" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (02/09/2026 12:04)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="84">
   <si>
     <t>om_emg</t>
   </si>
@@ -130,9 +130,6 @@
     <t>313260018713</t>
   </si>
   <si>
-    <t>329260019286</t>
-  </si>
-  <si>
     <t>329260019288</t>
   </si>
   <si>
@@ -142,9 +139,6 @@
     <t>396260016605</t>
   </si>
   <si>
-    <t>396260016606</t>
-  </si>
-  <si>
     <t>690260002556</t>
   </si>
   <si>
@@ -175,9 +169,6 @@
     <t>2641011-5</t>
   </si>
   <si>
-    <t>030-18200</t>
-  </si>
-  <si>
     <t>C592001-0206</t>
   </si>
   <si>
@@ -208,9 +199,6 @@
     <t>AXLE-MAIN GEAR</t>
   </si>
   <si>
-    <t>MAIN WHEEL BRAKE</t>
-  </si>
-  <si>
     <t>WICK-STAT DISC</t>
   </si>
   <si>
@@ -223,12 +211,6 @@
     <t>Providência tomada</t>
   </si>
   <si>
-    <t>Expedido total</t>
-  </si>
-  <si>
-    <t>Aguardando solução</t>
-  </si>
-  <si>
     <t>ANCE</t>
   </si>
   <si>
@@ -253,15 +235,9 @@
     <t>Emergência transformada em ANCE em 24/08. Aguardaremos atendimento com item da Vee One. Ramon 24/08/26.</t>
   </si>
   <si>
-    <t>item será atendido com o estoque local pedido 18294676. Godoy 26/08. Emg é na verdade AIFP, corrigido na planilha de 28/08. Ramon 28/08/26.</t>
-  </si>
-  <si>
     <t>Cedeu o item para o 2739. Ramon 01/09/26</t>
   </si>
   <si>
-    <t>Cedeu o item para o 2733. Ramon 01/09/26. AWB 112755521406 - volume retirado na loja GOLLOG - BEL por Marlon bispo em 01/09. Godoy 02/09/26. Recibo 734/FAB/26 assinado em 01/09. Ramon 02/09/26.</t>
-  </si>
-  <si>
     <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Chegada GIG dia 15-08 (voo 4273). Entregue V1 JPA 17/08 - MATERIAL EM TRANSITO - RECIBO 722/FAB/26 awb 12754830370 DPE 28/08/2026 - entregue 29/08/2026</t>
   </si>
   <si>
@@ -277,9 +253,6 @@
     <t>Colocado pedido no fornecedor I823285 - entregue em Miami 21/08 - TEMOS 3 EA NO ESTOQUE DA BANT. Material seguiu via awb 12754249845. Recebido por Kleyton em 24/08. Atl Ges.</t>
   </si>
   <si>
-    <t>Enviado para o Operador em 27/08/26- AWB 127-5516 5121 - REZ - MATERIAL DISPONIVEL PRA RETIRADA DIA 28/08/2026</t>
-  </si>
-  <si>
     <t>EM REPARO NA WILLIAM, DPE (confirmado) dia 02/09/2026 - REZ</t>
   </si>
   <si>
@@ -287,9 +260,6 @@
   </si>
   <si>
     <t>material será atendido pelo item reparado no estoque V1 01/09/2026</t>
-  </si>
-  <si>
-    <t>Material enviado dia 31/08/2026 VIA AWB 12755521406 DPE 01/09/2026</t>
   </si>
   <si>
     <t>Não temos em estoque, podemos movimentar o estoque da FAB para atendimento? RC 01/09/2026</t>
@@ -305,16 +275,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -330,7 +292,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -338,30 +300,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -657,89 +601,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA13"/>
+  <dimension ref="A1:AA11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -754,39 +698,39 @@
         <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F2" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="G2">
         <v>2702</v>
       </c>
       <c r="H2" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="I2" t="s">
-        <v>71</v>
-      </c>
-      <c r="J2" s="2">
+        <v>65</v>
+      </c>
+      <c r="J2" s="1">
         <v>46212</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46212</v>
       </c>
       <c r="L2">
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>73</v>
-      </c>
-      <c r="N2" s="2">
+        <v>67</v>
+      </c>
+      <c r="N2" s="1">
         <v>46243</v>
       </c>
-      <c r="O2" s="2">
+      <c r="O2" s="1">
         <v>46263</v>
       </c>
       <c r="Q2">
@@ -796,19 +740,19 @@
         <v>55</v>
       </c>
       <c r="S2" t="s">
+        <v>68</v>
+      </c>
+      <c r="T2" t="s">
+        <v>69</v>
+      </c>
+      <c r="U2" t="s">
+        <v>70</v>
+      </c>
+      <c r="V2" t="s">
         <v>74</v>
       </c>
-      <c r="T2" t="s">
-        <v>75</v>
-      </c>
-      <c r="U2" t="s">
-        <v>76</v>
-      </c>
-      <c r="V2" t="s">
-        <v>82</v>
-      </c>
       <c r="W2" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -825,39 +769,39 @@
         <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E3" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F3" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="G3">
         <v>2733</v>
       </c>
       <c r="H3" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="I3" t="s">
-        <v>71</v>
-      </c>
-      <c r="J3" s="2">
+        <v>65</v>
+      </c>
+      <c r="J3" s="1">
         <v>46238</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46238</v>
       </c>
       <c r="L3">
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>73</v>
-      </c>
-      <c r="N3" s="2">
+        <v>67</v>
+      </c>
+      <c r="N3" s="1">
         <v>46269</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46269</v>
       </c>
       <c r="Q3">
@@ -867,16 +811,16 @@
         <v>29</v>
       </c>
       <c r="S3" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="T3" t="s">
+        <v>69</v>
+      </c>
+      <c r="V3" t="s">
         <v>75</v>
       </c>
-      <c r="V3" t="s">
+      <c r="W3" t="s">
         <v>83</v>
-      </c>
-      <c r="W3" t="s">
-        <v>93</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -893,39 +837,39 @@
         <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E4" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="F4" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="G4">
         <v>2741</v>
       </c>
       <c r="H4" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="I4" t="s">
-        <v>71</v>
-      </c>
-      <c r="J4" s="2">
+        <v>65</v>
+      </c>
+      <c r="J4" s="1">
         <v>46251</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46249</v>
       </c>
       <c r="L4">
         <v>2</v>
       </c>
       <c r="M4" t="s">
-        <v>73</v>
-      </c>
-      <c r="N4" s="2">
+        <v>67</v>
+      </c>
+      <c r="N4" s="1">
         <v>46280</v>
       </c>
-      <c r="O4" s="2">
+      <c r="O4" s="1">
         <v>46280</v>
       </c>
       <c r="Q4">
@@ -935,16 +879,16 @@
         <v>18</v>
       </c>
       <c r="S4" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="T4" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="V4" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="W4" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -961,36 +905,36 @@
         <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E5" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="F5" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G5">
         <v>2741</v>
       </c>
       <c r="H5" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="I5" t="s">
-        <v>71</v>
-      </c>
-      <c r="J5" s="2">
+        <v>65</v>
+      </c>
+      <c r="J5" s="1">
         <v>46253</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46252</v>
       </c>
       <c r="L5">
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>73</v>
-      </c>
-      <c r="N5" s="2">
+        <v>67</v>
+      </c>
+      <c r="N5" s="1">
         <v>46283</v>
       </c>
       <c r="Q5">
@@ -1000,13 +944,13 @@
         <v>15</v>
       </c>
       <c r="S5" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="T5" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="W5" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1023,39 +967,39 @@
         <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E6" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F6" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="G6">
         <v>2731</v>
       </c>
       <c r="H6" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="I6" t="s">
-        <v>71</v>
-      </c>
-      <c r="J6" s="2">
+        <v>65</v>
+      </c>
+      <c r="J6" s="1">
         <v>46252</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46253</v>
       </c>
       <c r="L6">
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>73</v>
-      </c>
-      <c r="N6" s="2">
+        <v>67</v>
+      </c>
+      <c r="N6" s="1">
         <v>46284</v>
       </c>
-      <c r="O6" s="2">
+      <c r="O6" s="1">
         <v>46265</v>
       </c>
       <c r="Q6">
@@ -1065,19 +1009,19 @@
         <v>14</v>
       </c>
       <c r="S6" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="T6" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="U6" t="s">
+        <v>71</v>
+      </c>
+      <c r="V6" t="s">
         <v>77</v>
       </c>
-      <c r="V6" t="s">
-        <v>85</v>
-      </c>
       <c r="W6" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1094,39 +1038,39 @@
         <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E7" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="F7" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="G7">
         <v>2737</v>
       </c>
       <c r="H7" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="I7" t="s">
-        <v>71</v>
-      </c>
-      <c r="J7" s="2">
+        <v>65</v>
+      </c>
+      <c r="J7" s="1">
         <v>46254</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>46255</v>
       </c>
       <c r="L7">
         <v>2</v>
       </c>
       <c r="M7" t="s">
-        <v>73</v>
-      </c>
-      <c r="N7" s="2">
+        <v>67</v>
+      </c>
+      <c r="N7" s="1">
         <v>46286</v>
       </c>
-      <c r="O7" s="2">
+      <c r="O7" s="1">
         <v>46258</v>
       </c>
       <c r="Q7">
@@ -1136,19 +1080,19 @@
         <v>12</v>
       </c>
       <c r="S7" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="T7" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="U7" t="s">
+        <v>72</v>
+      </c>
+      <c r="V7" t="s">
         <v>78</v>
       </c>
-      <c r="V7" t="s">
-        <v>86</v>
-      </c>
       <c r="W7" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1165,61 +1109,55 @@
         <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E8" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="F8" t="s">
+        <v>63</v>
+      </c>
+      <c r="G8">
+        <v>2721</v>
+      </c>
+      <c r="H8" t="s">
+        <v>64</v>
+      </c>
+      <c r="I8" t="s">
+        <v>66</v>
+      </c>
+      <c r="J8" s="1">
+        <v>46262</v>
+      </c>
+      <c r="K8" s="1">
+        <v>46262</v>
+      </c>
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8" t="s">
         <v>67</v>
       </c>
-      <c r="G8">
-        <v>2709</v>
-      </c>
-      <c r="H8" t="s">
-        <v>69</v>
-      </c>
-      <c r="I8" t="s">
-        <v>72</v>
-      </c>
-      <c r="J8" s="2">
-        <v>46259</v>
-      </c>
-      <c r="K8" s="2">
-        <v>46260</v>
-      </c>
-      <c r="L8">
-        <v>1</v>
-      </c>
-      <c r="M8" t="s">
-        <v>73</v>
-      </c>
-      <c r="N8" s="2">
-        <v>46267</v>
-      </c>
-      <c r="O8" s="2">
-        <v>46262</v>
+      <c r="N8" s="1">
+        <v>46269</v>
       </c>
       <c r="Q8">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="R8">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="S8" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="T8" t="s">
-        <v>74</v>
-      </c>
-      <c r="U8" t="s">
+        <v>68</v>
+      </c>
+      <c r="V8" t="s">
         <v>79</v>
       </c>
-      <c r="V8" t="s">
-        <v>87</v>
-      </c>
       <c r="W8" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1227,64 +1165,67 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9">
-        <v>329</v>
+        <v>396</v>
       </c>
       <c r="B9" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C9" t="s">
         <v>39</v>
       </c>
       <c r="D9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E9" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F9" t="s">
+        <v>62</v>
+      </c>
+      <c r="G9">
+        <v>2733</v>
+      </c>
+      <c r="H9" t="s">
+        <v>64</v>
+      </c>
+      <c r="I9" t="s">
+        <v>65</v>
+      </c>
+      <c r="J9" s="1">
+        <v>46262</v>
+      </c>
+      <c r="K9" s="1">
+        <v>46262</v>
+      </c>
+      <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9" t="s">
         <v>67</v>
       </c>
-      <c r="G9">
-        <v>2721</v>
-      </c>
-      <c r="H9" t="s">
-        <v>68</v>
-      </c>
-      <c r="I9" t="s">
-        <v>72</v>
-      </c>
-      <c r="J9" s="2">
-        <v>46262</v>
-      </c>
-      <c r="K9" s="2">
-        <v>46262</v>
-      </c>
-      <c r="L9">
-        <v>1</v>
-      </c>
-      <c r="M9" t="s">
-        <v>73</v>
-      </c>
-      <c r="N9" s="2">
-        <v>46269</v>
+      <c r="N9" s="1">
+        <v>46293</v>
+      </c>
+      <c r="O9" s="1">
+        <v>46293</v>
       </c>
       <c r="Q9">
-        <v>-2</v>
+        <v>-26</v>
       </c>
       <c r="R9">
         <v>5</v>
       </c>
       <c r="S9" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="T9" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="V9" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="W9" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1301,58 +1242,61 @@
         <v>40</v>
       </c>
       <c r="D10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F10" t="s">
+        <v>63</v>
+      </c>
+      <c r="G10">
+        <v>2731</v>
+      </c>
+      <c r="H10" t="s">
+        <v>64</v>
+      </c>
+      <c r="I10" t="s">
         <v>66</v>
       </c>
-      <c r="G10">
-        <v>2733</v>
-      </c>
-      <c r="H10" t="s">
-        <v>68</v>
-      </c>
-      <c r="I10" t="s">
-        <v>71</v>
-      </c>
-      <c r="J10" s="2">
-        <v>46262</v>
-      </c>
-      <c r="K10" s="2">
-        <v>46262</v>
+      <c r="J10" s="1">
+        <v>46265</v>
+      </c>
+      <c r="K10" s="1">
+        <v>46266</v>
       </c>
       <c r="L10">
         <v>1</v>
       </c>
       <c r="M10" t="s">
+        <v>67</v>
+      </c>
+      <c r="N10" s="1">
+        <v>46273</v>
+      </c>
+      <c r="O10" s="1">
+        <v>46267</v>
+      </c>
+      <c r="Q10">
+        <v>-6</v>
+      </c>
+      <c r="R10">
+        <v>1</v>
+      </c>
+      <c r="S10" t="s">
+        <v>69</v>
+      </c>
+      <c r="T10" t="s">
+        <v>69</v>
+      </c>
+      <c r="U10" t="s">
         <v>73</v>
       </c>
-      <c r="N10" s="2">
-        <v>46293</v>
-      </c>
-      <c r="O10" s="2">
-        <v>46293</v>
-      </c>
-      <c r="Q10">
-        <v>-26</v>
-      </c>
-      <c r="R10">
-        <v>5</v>
-      </c>
-      <c r="S10" t="s">
-        <v>74</v>
-      </c>
-      <c r="T10" t="s">
-        <v>75</v>
-      </c>
       <c r="V10" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="W10" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1360,211 +1304,69 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>396</v>
+        <v>690</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C11" t="s">
         <v>41</v>
       </c>
       <c r="D11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E11" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F11" t="s">
+        <v>62</v>
+      </c>
+      <c r="G11">
+        <v>2727</v>
+      </c>
+      <c r="H11" t="s">
+        <v>64</v>
+      </c>
+      <c r="I11" t="s">
+        <v>65</v>
+      </c>
+      <c r="J11" s="1">
+        <v>46265</v>
+      </c>
+      <c r="K11" s="1">
+        <v>46266</v>
+      </c>
+      <c r="L11">
+        <v>5</v>
+      </c>
+      <c r="M11" t="s">
         <v>67</v>
       </c>
-      <c r="G11">
-        <v>2731</v>
-      </c>
-      <c r="H11" t="s">
-        <v>70</v>
-      </c>
-      <c r="I11" t="s">
-        <v>72</v>
-      </c>
-      <c r="J11" s="2">
-        <v>46265</v>
-      </c>
-      <c r="K11" s="2">
-        <v>46266</v>
-      </c>
-      <c r="L11">
-        <v>1</v>
-      </c>
-      <c r="M11" t="s">
-        <v>73</v>
-      </c>
-      <c r="N11" s="2">
-        <v>46273</v>
-      </c>
-      <c r="O11" s="2">
-        <v>46267</v>
+      <c r="N11" s="1">
+        <v>46297</v>
+      </c>
+      <c r="O11" s="1">
+        <v>46297</v>
       </c>
       <c r="Q11">
-        <v>-6</v>
+        <v>-30</v>
       </c>
       <c r="R11">
         <v>1</v>
       </c>
       <c r="S11" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="T11" t="s">
-        <v>75</v>
-      </c>
-      <c r="U11" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="V11" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="W11" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="AA11" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:27">
-      <c r="A12">
-        <v>396</v>
-      </c>
-      <c r="B12" t="s">
-        <v>28</v>
-      </c>
-      <c r="C12" t="s">
-        <v>42</v>
-      </c>
-      <c r="D12" t="s">
-        <v>53</v>
-      </c>
-      <c r="E12" t="s">
-        <v>64</v>
-      </c>
-      <c r="F12" t="s">
-        <v>67</v>
-      </c>
-      <c r="G12">
-        <v>2731</v>
-      </c>
-      <c r="H12" t="s">
-        <v>70</v>
-      </c>
-      <c r="I12" t="s">
-        <v>72</v>
-      </c>
-      <c r="J12" s="2">
-        <v>46265</v>
-      </c>
-      <c r="K12" s="2">
-        <v>46266</v>
-      </c>
-      <c r="L12">
-        <v>1</v>
-      </c>
-      <c r="M12" t="s">
-        <v>73</v>
-      </c>
-      <c r="N12" s="2">
-        <v>46273</v>
-      </c>
-      <c r="O12" s="2">
-        <v>46266</v>
-      </c>
-      <c r="Q12">
-        <v>-6</v>
-      </c>
-      <c r="R12">
-        <v>1</v>
-      </c>
-      <c r="S12" t="s">
-        <v>75</v>
-      </c>
-      <c r="T12" t="s">
-        <v>75</v>
-      </c>
-      <c r="U12" t="s">
-        <v>81</v>
-      </c>
-      <c r="V12" t="s">
-        <v>91</v>
-      </c>
-      <c r="W12" t="s">
-        <v>93</v>
-      </c>
-      <c r="AA12" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:27">
-      <c r="A13">
-        <v>690</v>
-      </c>
-      <c r="B13" t="s">
-        <v>31</v>
-      </c>
-      <c r="C13" t="s">
-        <v>43</v>
-      </c>
-      <c r="D13" t="s">
-        <v>54</v>
-      </c>
-      <c r="E13" t="s">
-        <v>65</v>
-      </c>
-      <c r="F13" t="s">
-        <v>66</v>
-      </c>
-      <c r="G13">
-        <v>2727</v>
-      </c>
-      <c r="H13" t="s">
-        <v>70</v>
-      </c>
-      <c r="I13" t="s">
-        <v>71</v>
-      </c>
-      <c r="J13" s="2">
-        <v>46265</v>
-      </c>
-      <c r="K13" s="2">
-        <v>46266</v>
-      </c>
-      <c r="L13">
-        <v>5</v>
-      </c>
-      <c r="M13" t="s">
-        <v>73</v>
-      </c>
-      <c r="N13" s="2">
-        <v>46297</v>
-      </c>
-      <c r="O13" s="2">
-        <v>46297</v>
-      </c>
-      <c r="Q13">
-        <v>-30</v>
-      </c>
-      <c r="R13">
-        <v>1</v>
-      </c>
-      <c r="S13" t="s">
-        <v>75</v>
-      </c>
-      <c r="T13" t="s">
-        <v>74</v>
-      </c>
-      <c r="V13" t="s">
-        <v>92</v>
-      </c>
-      <c r="W13" t="s">
-        <v>93</v>
-      </c>
-      <c r="AA13" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (03/09/2026 11:59)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="81">
   <si>
     <t>om_emg</t>
   </si>
@@ -136,9 +136,6 @@
     <t>396260016603</t>
   </si>
   <si>
-    <t>396260016605</t>
-  </si>
-  <si>
     <t>690260002556</t>
   </si>
   <si>
@@ -166,9 +163,6 @@
     <t>OD1232-24MB</t>
   </si>
   <si>
-    <t>2641011-5</t>
-  </si>
-  <si>
     <t>C592001-0206</t>
   </si>
   <si>
@@ -196,9 +190,6 @@
     <t>DC FAN</t>
   </si>
   <si>
-    <t>AXLE-MAIN GEAR</t>
-  </si>
-  <si>
     <t>WICK-STAT DISC</t>
   </si>
   <si>
@@ -211,6 +202,9 @@
     <t>Providência tomada</t>
   </si>
   <si>
+    <t>Expedido total</t>
+  </si>
+  <si>
     <t>ANCE</t>
   </si>
   <si>
@@ -235,7 +229,7 @@
     <t>Emergência transformada em ANCE em 24/08. Aguardaremos atendimento com item da Vee One. Ramon 24/08/26.</t>
   </si>
   <si>
-    <t>Cedeu o item para o 2739. Ramon 01/09/26</t>
+    <t>Pedido será atendido pelo estoque FAB pedido n° 18353156- Godoy 02/09/2026.</t>
   </si>
   <si>
     <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Chegada GIG dia 15-08 (voo 4273). Entregue V1 JPA 17/08 - MATERIAL EM TRANSITO - RECIBO 722/FAB/26 awb 12754830370 DPE 28/08/2026 - entregue 29/08/2026</t>
@@ -257,9 +251,6 @@
   </si>
   <si>
     <t>Colocado pedido WB0003139756 - previsão de entrega em Miami 02/09</t>
-  </si>
-  <si>
-    <t>material será atendido pelo item reparado no estoque V1 01/09/2026</t>
   </si>
   <si>
     <t>Não temos em estoque, podemos movimentar o estoque da FAB para atendimento? RC 01/09/2026</t>
@@ -601,7 +592,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA11"/>
+  <dimension ref="A1:AA10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -698,22 +689,22 @@
         <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="G2">
         <v>2702</v>
       </c>
       <c r="H2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="I2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J2" s="1">
         <v>46212</v>
@@ -725,7 +716,7 @@
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="N2" s="1">
         <v>46243</v>
@@ -734,25 +725,25 @@
         <v>46263</v>
       </c>
       <c r="Q2">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="R2">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="S2" t="s">
+        <v>66</v>
+      </c>
+      <c r="T2" t="s">
+        <v>67</v>
+      </c>
+      <c r="U2" t="s">
         <v>68</v>
       </c>
-      <c r="T2" t="s">
-        <v>69</v>
-      </c>
-      <c r="U2" t="s">
-        <v>70</v>
-      </c>
       <c r="V2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="W2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -769,22 +760,22 @@
         <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="G3">
         <v>2733</v>
       </c>
       <c r="H3" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="I3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J3" s="1">
         <v>46238</v>
@@ -796,7 +787,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="N3" s="1">
         <v>46269</v>
@@ -805,22 +796,22 @@
         <v>46269</v>
       </c>
       <c r="Q3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R3">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="S3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="T3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="V3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="W3" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -837,22 +828,22 @@
         <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="G4">
         <v>2741</v>
       </c>
       <c r="H4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="I4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J4" s="1">
         <v>46251</v>
@@ -864,7 +855,7 @@
         <v>2</v>
       </c>
       <c r="M4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="N4" s="1">
         <v>46280</v>
@@ -873,22 +864,22 @@
         <v>46280</v>
       </c>
       <c r="Q4">
-        <v>-13</v>
+        <v>-12</v>
       </c>
       <c r="R4">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="S4" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="T4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="V4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="W4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -905,22 +896,22 @@
         <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F5" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="G5">
         <v>2741</v>
       </c>
       <c r="H5" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="I5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J5" s="1">
         <v>46253</v>
@@ -932,25 +923,25 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="N5" s="1">
         <v>46283</v>
       </c>
       <c r="Q5">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="R5">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="T5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="W5" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -967,22 +958,22 @@
         <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E6" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F6" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="G6">
         <v>2731</v>
       </c>
       <c r="H6" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="I6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J6" s="1">
         <v>46252</v>
@@ -994,7 +985,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="N6" s="1">
         <v>46284</v>
@@ -1003,25 +994,25 @@
         <v>46265</v>
       </c>
       <c r="Q6">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="R6">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="T6" t="s">
+        <v>67</v>
+      </c>
+      <c r="U6" t="s">
         <v>69</v>
       </c>
-      <c r="U6" t="s">
-        <v>71</v>
-      </c>
       <c r="V6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="W6" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1038,22 +1029,22 @@
         <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="G7">
         <v>2737</v>
       </c>
       <c r="H7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="I7" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J7" s="1">
         <v>46254</v>
@@ -1065,7 +1056,7 @@
         <v>2</v>
       </c>
       <c r="M7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="N7" s="1">
         <v>46286</v>
@@ -1074,25 +1065,25 @@
         <v>46258</v>
       </c>
       <c r="Q7">
-        <v>-19</v>
+        <v>-18</v>
       </c>
       <c r="R7">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S7" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="T7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="U7" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="V7" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="W7" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1109,22 +1100,22 @@
         <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E8" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F8" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="G8">
         <v>2721</v>
       </c>
       <c r="H8" t="s">
+        <v>61</v>
+      </c>
+      <c r="I8" t="s">
         <v>64</v>
-      </c>
-      <c r="I8" t="s">
-        <v>66</v>
       </c>
       <c r="J8" s="1">
         <v>46262</v>
@@ -1136,28 +1127,28 @@
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="N8" s="1">
         <v>46269</v>
       </c>
       <c r="Q8">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R8">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="T8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="V8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="W8" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1174,22 +1165,22 @@
         <v>39</v>
       </c>
       <c r="D9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F9" t="s">
         <v>59</v>
-      </c>
-      <c r="F9" t="s">
-        <v>62</v>
       </c>
       <c r="G9">
         <v>2733</v>
       </c>
       <c r="H9" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="I9" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J9" s="1">
         <v>46262</v>
@@ -1201,7 +1192,7 @@
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="N9" s="1">
         <v>46293</v>
@@ -1210,22 +1201,22 @@
         <v>46293</v>
       </c>
       <c r="Q9">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="R9">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S9" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="T9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="V9" t="s">
+        <v>78</v>
+      </c>
+      <c r="W9" t="s">
         <v>80</v>
-      </c>
-      <c r="W9" t="s">
-        <v>83</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1233,31 +1224,31 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>396</v>
+        <v>690</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C10" t="s">
         <v>40</v>
       </c>
       <c r="D10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E10" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F10" t="s">
+        <v>59</v>
+      </c>
+      <c r="G10">
+        <v>2727</v>
+      </c>
+      <c r="H10" t="s">
+        <v>62</v>
+      </c>
+      <c r="I10" t="s">
         <v>63</v>
-      </c>
-      <c r="G10">
-        <v>2731</v>
-      </c>
-      <c r="H10" t="s">
-        <v>64</v>
-      </c>
-      <c r="I10" t="s">
-        <v>66</v>
       </c>
       <c r="J10" s="1">
         <v>46265</v>
@@ -1266,107 +1257,39 @@
         <v>46266</v>
       </c>
       <c r="L10">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M10" t="s">
+        <v>65</v>
+      </c>
+      <c r="N10" s="1">
+        <v>46297</v>
+      </c>
+      <c r="O10" s="1">
+        <v>46297</v>
+      </c>
+      <c r="Q10">
+        <v>-29</v>
+      </c>
+      <c r="R10">
+        <v>2</v>
+      </c>
+      <c r="S10" t="s">
         <v>67</v>
       </c>
-      <c r="N10" s="1">
-        <v>46273</v>
-      </c>
-      <c r="O10" s="1">
-        <v>46267</v>
-      </c>
-      <c r="Q10">
-        <v>-6</v>
-      </c>
-      <c r="R10">
-        <v>1</v>
-      </c>
-      <c r="S10" t="s">
-        <v>69</v>
-      </c>
       <c r="T10" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="U10" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="V10" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="W10" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="AA10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:27">
-      <c r="A11">
-        <v>690</v>
-      </c>
-      <c r="B11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C11" t="s">
-        <v>41</v>
-      </c>
-      <c r="D11" t="s">
-        <v>51</v>
-      </c>
-      <c r="E11" t="s">
-        <v>61</v>
-      </c>
-      <c r="F11" t="s">
-        <v>62</v>
-      </c>
-      <c r="G11">
-        <v>2727</v>
-      </c>
-      <c r="H11" t="s">
-        <v>64</v>
-      </c>
-      <c r="I11" t="s">
-        <v>65</v>
-      </c>
-      <c r="J11" s="1">
-        <v>46265</v>
-      </c>
-      <c r="K11" s="1">
-        <v>46266</v>
-      </c>
-      <c r="L11">
-        <v>5</v>
-      </c>
-      <c r="M11" t="s">
-        <v>67</v>
-      </c>
-      <c r="N11" s="1">
-        <v>46297</v>
-      </c>
-      <c r="O11" s="1">
-        <v>46297</v>
-      </c>
-      <c r="Q11">
-        <v>-30</v>
-      </c>
-      <c r="R11">
-        <v>1</v>
-      </c>
-      <c r="S11" t="s">
-        <v>69</v>
-      </c>
-      <c r="T11" t="s">
-        <v>68</v>
-      </c>
-      <c r="V11" t="s">
-        <v>82</v>
-      </c>
-      <c r="W11" t="s">
-        <v>83</v>
-      </c>
-      <c r="AA11" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (03/09/2026 13:41)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -266,8 +266,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -283,7 +291,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -291,12 +299,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -596,85 +622,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -706,10 +732,10 @@
       <c r="I2" t="s">
         <v>63</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>46212</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46212</v>
       </c>
       <c r="L2">
@@ -718,10 +744,10 @@
       <c r="M2" t="s">
         <v>65</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <v>46243</v>
       </c>
-      <c r="O2" s="1">
+      <c r="O2" s="2">
         <v>46263</v>
       </c>
       <c r="Q2">
@@ -777,10 +803,10 @@
       <c r="I3" t="s">
         <v>63</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>46238</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46238</v>
       </c>
       <c r="L3">
@@ -789,10 +815,10 @@
       <c r="M3" t="s">
         <v>65</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <v>46269</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46269</v>
       </c>
       <c r="Q3">
@@ -845,10 +871,10 @@
       <c r="I4" t="s">
         <v>63</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>46251</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46249</v>
       </c>
       <c r="L4">
@@ -857,10 +883,10 @@
       <c r="M4" t="s">
         <v>65</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="2">
         <v>46280</v>
       </c>
-      <c r="O4" s="1">
+      <c r="O4" s="2">
         <v>46280</v>
       </c>
       <c r="Q4">
@@ -913,10 +939,10 @@
       <c r="I5" t="s">
         <v>63</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>46253</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46252</v>
       </c>
       <c r="L5">
@@ -925,7 +951,7 @@
       <c r="M5" t="s">
         <v>65</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <v>46283</v>
       </c>
       <c r="Q5">
@@ -975,10 +1001,10 @@
       <c r="I6" t="s">
         <v>63</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>46252</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46253</v>
       </c>
       <c r="L6">
@@ -987,10 +1013,10 @@
       <c r="M6" t="s">
         <v>65</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <v>46284</v>
       </c>
-      <c r="O6" s="1">
+      <c r="O6" s="2">
         <v>46265</v>
       </c>
       <c r="Q6">
@@ -1046,10 +1072,10 @@
       <c r="I7" t="s">
         <v>63</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46254</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46255</v>
       </c>
       <c r="L7">
@@ -1058,10 +1084,10 @@
       <c r="M7" t="s">
         <v>65</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="2">
         <v>46286</v>
       </c>
-      <c r="O7" s="1">
+      <c r="O7" s="2">
         <v>46258</v>
       </c>
       <c r="Q7">
@@ -1117,10 +1143,10 @@
       <c r="I8" t="s">
         <v>64</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46262</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46262</v>
       </c>
       <c r="L8">
@@ -1129,7 +1155,7 @@
       <c r="M8" t="s">
         <v>65</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="2">
         <v>46269</v>
       </c>
       <c r="Q8">
@@ -1182,10 +1208,10 @@
       <c r="I9" t="s">
         <v>63</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46262</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46262</v>
       </c>
       <c r="L9">
@@ -1194,10 +1220,10 @@
       <c r="M9" t="s">
         <v>65</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>46293</v>
       </c>
-      <c r="O9" s="1">
+      <c r="O9" s="2">
         <v>46293</v>
       </c>
       <c r="Q9">
@@ -1250,10 +1276,10 @@
       <c r="I10" t="s">
         <v>63</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46265</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>46266</v>
       </c>
       <c r="L10">
@@ -1262,10 +1288,10 @@
       <c r="M10" t="s">
         <v>65</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
         <v>46297</v>
       </c>
-      <c r="O10" s="1">
+      <c r="O10" s="2">
         <v>46297</v>
       </c>
       <c r="Q10">

</xml_diff>

<commit_message>
Atualização automática: emergencias (04/09/2026 11:55)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -266,16 +266,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -291,7 +283,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -299,30 +291,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -622,85 +596,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -732,10 +706,10 @@
       <c r="I2" t="s">
         <v>63</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>46212</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46212</v>
       </c>
       <c r="L2">
@@ -744,17 +718,17 @@
       <c r="M2" t="s">
         <v>65</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="1">
         <v>46243</v>
       </c>
-      <c r="O2" s="2">
+      <c r="O2" s="1">
         <v>46263</v>
       </c>
       <c r="Q2">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="R2">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="S2" t="s">
         <v>66</v>
@@ -803,10 +777,10 @@
       <c r="I3" t="s">
         <v>63</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>46238</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46238</v>
       </c>
       <c r="L3">
@@ -815,17 +789,17 @@
       <c r="M3" t="s">
         <v>65</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="1">
         <v>46269</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46269</v>
       </c>
       <c r="Q3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R3">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S3" t="s">
         <v>66</v>
@@ -871,10 +845,10 @@
       <c r="I4" t="s">
         <v>63</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>46251</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46249</v>
       </c>
       <c r="L4">
@@ -883,17 +857,17 @@
       <c r="M4" t="s">
         <v>65</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="1">
         <v>46280</v>
       </c>
-      <c r="O4" s="2">
+      <c r="O4" s="1">
         <v>46280</v>
       </c>
       <c r="Q4">
-        <v>-12</v>
+        <v>-11</v>
       </c>
       <c r="R4">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="S4" t="s">
         <v>66</v>
@@ -939,10 +913,10 @@
       <c r="I5" t="s">
         <v>63</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>46253</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46252</v>
       </c>
       <c r="L5">
@@ -951,14 +925,14 @@
       <c r="M5" t="s">
         <v>65</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="1">
         <v>46283</v>
       </c>
       <c r="Q5">
-        <v>-15</v>
+        <v>-14</v>
       </c>
       <c r="R5">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="S5" t="s">
         <v>66</v>
@@ -1001,10 +975,10 @@
       <c r="I6" t="s">
         <v>63</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>46252</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46253</v>
       </c>
       <c r="L6">
@@ -1013,17 +987,17 @@
       <c r="M6" t="s">
         <v>65</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="1">
         <v>46284</v>
       </c>
-      <c r="O6" s="2">
+      <c r="O6" s="1">
         <v>46265</v>
       </c>
       <c r="Q6">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="R6">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S6" t="s">
         <v>66</v>
@@ -1072,10 +1046,10 @@
       <c r="I7" t="s">
         <v>63</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46254</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>46255</v>
       </c>
       <c r="L7">
@@ -1084,17 +1058,17 @@
       <c r="M7" t="s">
         <v>65</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="1">
         <v>46286</v>
       </c>
-      <c r="O7" s="2">
+      <c r="O7" s="1">
         <v>46258</v>
       </c>
       <c r="Q7">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="R7">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S7" t="s">
         <v>66</v>
@@ -1143,10 +1117,10 @@
       <c r="I8" t="s">
         <v>64</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46262</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>46262</v>
       </c>
       <c r="L8">
@@ -1155,14 +1129,14 @@
       <c r="M8" t="s">
         <v>65</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="1">
         <v>46269</v>
       </c>
       <c r="Q8">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S8" t="s">
         <v>66</v>
@@ -1208,10 +1182,10 @@
       <c r="I9" t="s">
         <v>63</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46262</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>46262</v>
       </c>
       <c r="L9">
@@ -1220,17 +1194,17 @@
       <c r="M9" t="s">
         <v>65</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="1">
         <v>46293</v>
       </c>
-      <c r="O9" s="2">
+      <c r="O9" s="1">
         <v>46293</v>
       </c>
       <c r="Q9">
-        <v>-25</v>
+        <v>-24</v>
       </c>
       <c r="R9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S9" t="s">
         <v>66</v>
@@ -1276,10 +1250,10 @@
       <c r="I10" t="s">
         <v>63</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>46265</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>46266</v>
       </c>
       <c r="L10">
@@ -1288,17 +1262,17 @@
       <c r="M10" t="s">
         <v>65</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="1">
         <v>46297</v>
       </c>
-      <c r="O10" s="2">
+      <c r="O10" s="1">
         <v>46297</v>
       </c>
       <c r="Q10">
-        <v>-29</v>
+        <v>-28</v>
       </c>
       <c r="R10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S10" t="s">
         <v>67</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (07/09/2026 13:24)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -725,10 +725,10 @@
         <v>46263</v>
       </c>
       <c r="Q2">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="R2">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="S2" t="s">
         <v>66</v>
@@ -796,10 +796,10 @@
         <v>46269</v>
       </c>
       <c r="Q3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R3">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="S3" t="s">
         <v>66</v>
@@ -864,10 +864,10 @@
         <v>46280</v>
       </c>
       <c r="Q4">
-        <v>-11</v>
+        <v>-8</v>
       </c>
       <c r="R4">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="S4" t="s">
         <v>66</v>
@@ -929,10 +929,10 @@
         <v>46283</v>
       </c>
       <c r="Q5">
-        <v>-14</v>
+        <v>-11</v>
       </c>
       <c r="R5">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="S5" t="s">
         <v>66</v>
@@ -994,10 +994,10 @@
         <v>46265</v>
       </c>
       <c r="Q6">
-        <v>-15</v>
+        <v>-12</v>
       </c>
       <c r="R6">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="S6" t="s">
         <v>66</v>
@@ -1065,10 +1065,10 @@
         <v>46258</v>
       </c>
       <c r="Q7">
-        <v>-17</v>
+        <v>-14</v>
       </c>
       <c r="R7">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="S7" t="s">
         <v>66</v>
@@ -1133,10 +1133,10 @@
         <v>46269</v>
       </c>
       <c r="Q8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R8">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S8" t="s">
         <v>66</v>
@@ -1201,10 +1201,10 @@
         <v>46293</v>
       </c>
       <c r="Q9">
-        <v>-24</v>
+        <v>-21</v>
       </c>
       <c r="R9">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S9" t="s">
         <v>66</v>
@@ -1269,10 +1269,10 @@
         <v>46297</v>
       </c>
       <c r="Q10">
-        <v>-28</v>
+        <v>-25</v>
       </c>
       <c r="R10">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="S10" t="s">
         <v>67</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (08/09/2026 08:35)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -266,8 +266,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -283,7 +291,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -291,12 +299,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -596,85 +622,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -706,10 +732,10 @@
       <c r="I2" t="s">
         <v>63</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>46212</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46212</v>
       </c>
       <c r="L2">
@@ -718,17 +744,17 @@
       <c r="M2" t="s">
         <v>65</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <v>46243</v>
       </c>
-      <c r="O2" s="1">
+      <c r="O2" s="2">
         <v>46263</v>
       </c>
       <c r="Q2">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R2">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="S2" t="s">
         <v>66</v>
@@ -777,10 +803,10 @@
       <c r="I3" t="s">
         <v>63</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>46238</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46238</v>
       </c>
       <c r="L3">
@@ -789,17 +815,17 @@
       <c r="M3" t="s">
         <v>65</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <v>46269</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46269</v>
       </c>
       <c r="Q3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R3">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S3" t="s">
         <v>66</v>
@@ -845,10 +871,10 @@
       <c r="I4" t="s">
         <v>63</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>46251</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46249</v>
       </c>
       <c r="L4">
@@ -857,17 +883,17 @@
       <c r="M4" t="s">
         <v>65</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="2">
         <v>46280</v>
       </c>
-      <c r="O4" s="1">
+      <c r="O4" s="2">
         <v>46280</v>
       </c>
       <c r="Q4">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="R4">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="S4" t="s">
         <v>66</v>
@@ -913,10 +939,10 @@
       <c r="I5" t="s">
         <v>63</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>46253</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46252</v>
       </c>
       <c r="L5">
@@ -925,14 +951,14 @@
       <c r="M5" t="s">
         <v>65</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <v>46283</v>
       </c>
       <c r="Q5">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R5">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="S5" t="s">
         <v>66</v>
@@ -975,10 +1001,10 @@
       <c r="I6" t="s">
         <v>63</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>46252</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46253</v>
       </c>
       <c r="L6">
@@ -987,17 +1013,17 @@
       <c r="M6" t="s">
         <v>65</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <v>46284</v>
       </c>
-      <c r="O6" s="1">
+      <c r="O6" s="2">
         <v>46265</v>
       </c>
       <c r="Q6">
-        <v>-12</v>
+        <v>-11</v>
       </c>
       <c r="R6">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="S6" t="s">
         <v>66</v>
@@ -1046,10 +1072,10 @@
       <c r="I7" t="s">
         <v>63</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46254</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46255</v>
       </c>
       <c r="L7">
@@ -1058,17 +1084,17 @@
       <c r="M7" t="s">
         <v>65</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="2">
         <v>46286</v>
       </c>
-      <c r="O7" s="1">
+      <c r="O7" s="2">
         <v>46258</v>
       </c>
       <c r="Q7">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="R7">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="S7" t="s">
         <v>66</v>
@@ -1117,10 +1143,10 @@
       <c r="I8" t="s">
         <v>64</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46262</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46262</v>
       </c>
       <c r="L8">
@@ -1129,14 +1155,14 @@
       <c r="M8" t="s">
         <v>65</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="2">
         <v>46269</v>
       </c>
       <c r="Q8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R8">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S8" t="s">
         <v>66</v>
@@ -1182,10 +1208,10 @@
       <c r="I9" t="s">
         <v>63</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46262</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46262</v>
       </c>
       <c r="L9">
@@ -1194,17 +1220,17 @@
       <c r="M9" t="s">
         <v>65</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>46293</v>
       </c>
-      <c r="O9" s="1">
+      <c r="O9" s="2">
         <v>46293</v>
       </c>
       <c r="Q9">
-        <v>-21</v>
+        <v>-20</v>
       </c>
       <c r="R9">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S9" t="s">
         <v>66</v>
@@ -1250,10 +1276,10 @@
       <c r="I10" t="s">
         <v>63</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46265</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>46266</v>
       </c>
       <c r="L10">
@@ -1262,17 +1288,17 @@
       <c r="M10" t="s">
         <v>65</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
         <v>46297</v>
       </c>
-      <c r="O10" s="1">
+      <c r="O10" s="2">
         <v>46297</v>
       </c>
       <c r="Q10">
-        <v>-25</v>
+        <v>-24</v>
       </c>
       <c r="R10">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S10" t="s">
         <v>67</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (08/09/2026 11:30)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="88">
   <si>
     <t>om_emg</t>
   </si>
@@ -139,6 +139,9 @@
     <t>690260002556</t>
   </si>
   <si>
+    <t>313260018737</t>
+  </si>
+  <si>
     <t>030-1094-58</t>
   </si>
   <si>
@@ -166,6 +169,9 @@
     <t>C592001-0206</t>
   </si>
   <si>
+    <t>D210507</t>
+  </si>
+  <si>
     <t>CONNECTOR</t>
   </si>
   <si>
@@ -193,24 +199,36 @@
     <t>WICK-STAT DISC</t>
   </si>
   <si>
+    <t>GOVERNOR,OVERSPEED</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
     <t>T</t>
   </si>
   <si>
+    <t>R</t>
+  </si>
+  <si>
     <t>Providência tomada</t>
   </si>
   <si>
     <t>Expedido total</t>
   </si>
   <si>
+    <t>Aguardando solução</t>
+  </si>
+  <si>
     <t>ANCE</t>
   </si>
   <si>
     <t>AIFP</t>
   </si>
   <si>
+    <t>IPLR</t>
+  </si>
+  <si>
     <t>EA</t>
   </si>
   <si>
@@ -232,13 +250,16 @@
     <t>Pedido será atendido pelo estoque FAB pedido n° 18353156- Godoy 02/09/2026.</t>
   </si>
   <si>
+    <t>ITEM FOI REMOVIDO PARA ATENDER A ANV 2736 POR MOTIVO DE PANE. Godoy 08/09/26.</t>
+  </si>
+  <si>
     <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Chegada GIG dia 15-08 (voo 4273). Entregue V1 JPA 17/08 - MATERIAL EM TRANSITO - RECIBO 722/FAB/26 awb 12754830370 DPE 28/08/2026 - entregue 29/08/2026</t>
   </si>
   <si>
     <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
   </si>
   <si>
-    <t>Colocado pedido no fornecedor WAGA INTERNATIONAL INV26-00008 - tracking 876324334524 - previsão de entrega em Miami 31/08</t>
+    <t>Colocado pedido no fornecedor WAGA INTERNATIONAL INV26-00008 - tracking 876324334524 - aguardando voo cargueiro para o GIG</t>
   </si>
   <si>
     <t>Colocado pedido Textron WB0003128625 - tracking 535477333011 - previsão de entrega 25/08 V1 JPA - MATERIAL ENVIADO VIA RECIBO 726/FAB/26, AWB A SER GERADA PELA GOLLOG RC 25/08/2026 - AWB 12754866615 DPE 28/08/2026 - recebido dia 31/08/2026</t>
@@ -247,13 +268,13 @@
     <t>Colocado pedido no fornecedor I823285 - entregue em Miami 21/08 - TEMOS 3 EA NO ESTOQUE DA BANT. Material seguiu via awb 12754249845. Recebido por Kleyton em 24/08. Atl Ges.</t>
   </si>
   <si>
-    <t>EM REPARO NA WILLIAM, DPE (confirmado) dia 02/09/2026 - REZ</t>
-  </si>
-  <si>
-    <t>Colocado pedido WB0003139756 - previsão de entrega em Miami 02/09</t>
-  </si>
-  <si>
-    <t>Não temos em estoque, podemos movimentar o estoque da FAB para atendimento? RC 01/09/2026</t>
+    <t>Enviado para o Operador dia 03/09/26 - AWB 127-5593 2321- REZ</t>
+  </si>
+  <si>
+    <t>Colocado pedido IJ17699595 - previsão de chegada GIG 04/09</t>
+  </si>
+  <si>
+    <t>Enviado para o Operador dia 03/09/26 - AWB 127-5594 5035- REZ</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -618,7 +639,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA10"/>
+  <dimension ref="A1:AA11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -715,22 +736,22 @@
         <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G2">
         <v>2702</v>
       </c>
       <c r="H2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="I2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="J2" s="2">
         <v>46212</v>
@@ -742,7 +763,7 @@
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="N2" s="2">
         <v>46243</v>
@@ -757,19 +778,19 @@
         <v>61</v>
       </c>
       <c r="S2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="T2" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="U2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="V2" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="W2" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -786,22 +807,22 @@
         <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G3">
         <v>2733</v>
       </c>
       <c r="H3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="I3" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="J3" s="2">
         <v>46238</v>
@@ -813,7 +834,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="N3" s="2">
         <v>46269</v>
@@ -828,16 +849,16 @@
         <v>35</v>
       </c>
       <c r="S3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="T3" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="V3" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="W3" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -854,22 +875,22 @@
         <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F4" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G4">
         <v>2741</v>
       </c>
       <c r="H4" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="I4" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="J4" s="2">
         <v>46251</v>
@@ -881,7 +902,7 @@
         <v>2</v>
       </c>
       <c r="M4" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="N4" s="2">
         <v>46280</v>
@@ -896,16 +917,16 @@
         <v>24</v>
       </c>
       <c r="S4" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="T4" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="V4" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="W4" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -922,22 +943,22 @@
         <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F5" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="G5">
         <v>2741</v>
       </c>
       <c r="H5" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="I5" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="J5" s="2">
         <v>46253</v>
@@ -949,7 +970,7 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="N5" s="2">
         <v>46283</v>
@@ -961,13 +982,13 @@
         <v>21</v>
       </c>
       <c r="S5" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="T5" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="W5" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -984,22 +1005,22 @@
         <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F6" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G6">
         <v>2731</v>
       </c>
       <c r="H6" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="I6" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="J6" s="2">
         <v>46252</v>
@@ -1011,7 +1032,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="N6" s="2">
         <v>46284</v>
@@ -1026,19 +1047,19 @@
         <v>20</v>
       </c>
       <c r="S6" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="T6" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="U6" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="V6" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="W6" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1055,22 +1076,22 @@
         <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E7" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F7" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G7">
         <v>2737</v>
       </c>
       <c r="H7" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="I7" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="J7" s="2">
         <v>46254</v>
@@ -1082,7 +1103,7 @@
         <v>2</v>
       </c>
       <c r="M7" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="N7" s="2">
         <v>46286</v>
@@ -1097,19 +1118,19 @@
         <v>18</v>
       </c>
       <c r="S7" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="T7" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="U7" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="V7" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="W7" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1126,22 +1147,22 @@
         <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F8" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="G8">
         <v>2721</v>
       </c>
       <c r="H8" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="I8" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="J8" s="2">
         <v>46262</v>
@@ -1153,11 +1174,14 @@
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="N8" s="2">
         <v>46269</v>
       </c>
+      <c r="O8" s="2">
+        <v>46269</v>
+      </c>
       <c r="Q8">
         <v>4</v>
       </c>
@@ -1165,16 +1189,16 @@
         <v>11</v>
       </c>
       <c r="S8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="T8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="V8" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="W8" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1191,22 +1215,22 @@
         <v>39</v>
       </c>
       <c r="D9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F9" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G9">
         <v>2733</v>
       </c>
       <c r="H9" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="I9" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="J9" s="2">
         <v>46262</v>
@@ -1218,7 +1242,7 @@
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="N9" s="2">
         <v>46293</v>
@@ -1233,16 +1257,16 @@
         <v>11</v>
       </c>
       <c r="S9" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="T9" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="V9" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="W9" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1259,22 +1283,22 @@
         <v>40</v>
       </c>
       <c r="D10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E10" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F10" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G10">
         <v>2727</v>
       </c>
       <c r="H10" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I10" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="J10" s="2">
         <v>46265</v>
@@ -1286,7 +1310,7 @@
         <v>5</v>
       </c>
       <c r="M10" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="N10" s="2">
         <v>46297</v>
@@ -1301,21 +1325,86 @@
         <v>7</v>
       </c>
       <c r="S10" t="s">
+        <v>73</v>
+      </c>
+      <c r="T10" t="s">
+        <v>72</v>
+      </c>
+      <c r="U10" t="s">
+        <v>77</v>
+      </c>
+      <c r="V10" t="s">
+        <v>86</v>
+      </c>
+      <c r="W10" t="s">
+        <v>87</v>
+      </c>
+      <c r="AA10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27">
+      <c r="A11">
+        <v>313</v>
+      </c>
+      <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" t="s">
+        <v>51</v>
+      </c>
+      <c r="E11" t="s">
+        <v>61</v>
+      </c>
+      <c r="F11" t="s">
+        <v>64</v>
+      </c>
+      <c r="G11">
+        <v>2730</v>
+      </c>
+      <c r="H11" t="s">
         <v>67</v>
       </c>
-      <c r="T10" t="s">
-        <v>66</v>
-      </c>
-      <c r="U10" t="s">
+      <c r="I11" t="s">
+        <v>70</v>
+      </c>
+      <c r="J11" s="2">
+        <v>46269</v>
+      </c>
+      <c r="K11" s="2">
+        <v>46273</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11" t="s">
         <v>71</v>
       </c>
-      <c r="V10" t="s">
-        <v>79</v>
-      </c>
-      <c r="W10" t="s">
-        <v>80</v>
-      </c>
-      <c r="AA10" t="b">
+      <c r="N11" s="2">
+        <v>46284</v>
+      </c>
+      <c r="Q11">
+        <v>-11</v>
+      </c>
+      <c r="R11">
+        <v>0</v>
+      </c>
+      <c r="S11" t="s">
+        <v>73</v>
+      </c>
+      <c r="T11" t="s">
+        <v>73</v>
+      </c>
+      <c r="U11" t="s">
+        <v>78</v>
+      </c>
+      <c r="W11" t="s">
+        <v>87</v>
+      </c>
+      <c r="AA11" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (08/09/2026 12:03)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -287,16 +287,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -312,7 +304,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -320,30 +312,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -643,85 +617,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -753,10 +727,10 @@
       <c r="I2" t="s">
         <v>68</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>46212</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46212</v>
       </c>
       <c r="L2">
@@ -765,10 +739,10 @@
       <c r="M2" t="s">
         <v>71</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="1">
         <v>46243</v>
       </c>
-      <c r="O2" s="2">
+      <c r="O2" s="1">
         <v>46263</v>
       </c>
       <c r="Q2">
@@ -824,10 +798,10 @@
       <c r="I3" t="s">
         <v>68</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>46238</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46238</v>
       </c>
       <c r="L3">
@@ -836,10 +810,10 @@
       <c r="M3" t="s">
         <v>71</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="1">
         <v>46269</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46269</v>
       </c>
       <c r="Q3">
@@ -892,10 +866,10 @@
       <c r="I4" t="s">
         <v>68</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>46251</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46249</v>
       </c>
       <c r="L4">
@@ -904,10 +878,10 @@
       <c r="M4" t="s">
         <v>71</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="1">
         <v>46280</v>
       </c>
-      <c r="O4" s="2">
+      <c r="O4" s="1">
         <v>46280</v>
       </c>
       <c r="Q4">
@@ -960,10 +934,10 @@
       <c r="I5" t="s">
         <v>68</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>46253</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46252</v>
       </c>
       <c r="L5">
@@ -972,7 +946,7 @@
       <c r="M5" t="s">
         <v>71</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="1">
         <v>46283</v>
       </c>
       <c r="Q5">
@@ -1022,10 +996,10 @@
       <c r="I6" t="s">
         <v>68</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>46252</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46253</v>
       </c>
       <c r="L6">
@@ -1034,10 +1008,10 @@
       <c r="M6" t="s">
         <v>71</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="1">
         <v>46284</v>
       </c>
-      <c r="O6" s="2">
+      <c r="O6" s="1">
         <v>46265</v>
       </c>
       <c r="Q6">
@@ -1093,10 +1067,10 @@
       <c r="I7" t="s">
         <v>68</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46254</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>46255</v>
       </c>
       <c r="L7">
@@ -1105,10 +1079,10 @@
       <c r="M7" t="s">
         <v>71</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="1">
         <v>46286</v>
       </c>
-      <c r="O7" s="2">
+      <c r="O7" s="1">
         <v>46258</v>
       </c>
       <c r="Q7">
@@ -1164,10 +1138,10 @@
       <c r="I8" t="s">
         <v>69</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46262</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>46262</v>
       </c>
       <c r="L8">
@@ -1176,10 +1150,10 @@
       <c r="M8" t="s">
         <v>71</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="1">
         <v>46269</v>
       </c>
-      <c r="O8" s="2">
+      <c r="O8" s="1">
         <v>46269</v>
       </c>
       <c r="Q8">
@@ -1232,10 +1206,10 @@
       <c r="I9" t="s">
         <v>68</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46262</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>46262</v>
       </c>
       <c r="L9">
@@ -1244,10 +1218,10 @@
       <c r="M9" t="s">
         <v>71</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="1">
         <v>46293</v>
       </c>
-      <c r="O9" s="2">
+      <c r="O9" s="1">
         <v>46293</v>
       </c>
       <c r="Q9">
@@ -1300,10 +1274,10 @@
       <c r="I10" t="s">
         <v>68</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>46265</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>46266</v>
       </c>
       <c r="L10">
@@ -1312,10 +1286,10 @@
       <c r="M10" t="s">
         <v>71</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="1">
         <v>46297</v>
       </c>
-      <c r="O10" s="2">
+      <c r="O10" s="1">
         <v>46297</v>
       </c>
       <c r="Q10">
@@ -1371,10 +1345,10 @@
       <c r="I11" t="s">
         <v>70</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46269</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>46273</v>
       </c>
       <c r="L11">
@@ -1383,7 +1357,7 @@
       <c r="M11" t="s">
         <v>71</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11" s="1">
         <v>46284</v>
       </c>
       <c r="Q11">

</xml_diff>

<commit_message>
Atualização automática: emergencias (09/09/2026 12:05)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="87">
   <si>
     <t>om_emg</t>
   </si>
@@ -217,9 +217,6 @@
     <t>Expedido total</t>
   </si>
   <si>
-    <t>Aguardando solução</t>
-  </si>
-  <si>
     <t>ANCE</t>
   </si>
   <si>
@@ -238,10 +235,10 @@
     <t>Sim</t>
   </si>
   <si>
-    <t>AWB 12754830370 -  volume retirado na loja GOLLOG - NAT por Teodoro silva em 29/08. Godoy 01/09/26.</t>
-  </si>
-  <si>
-    <t>AWB 12754866615 -  volume retirado na loja GOLLOG - BEL por Marcos bispo em 31/08. Godoy 01/09/26.</t>
+    <t>AWB 12754830370 -  volume retirado na loja GOLLOG - NAT por Teodoro silva em 29/08. Godoy 01/09/26. V1 favor inserir o recibo na pasta do Drive. Godoy 09/09/26.</t>
+  </si>
+  <si>
+    <t>AWB 12754866615 -  volume retirado na loja GOLLOG - BEL por Marcos bispo em 31/08. Godoy 01/09/26.   V1 favor inserir o recibo na pasta do Drive. Godoy 09/09/26.</t>
   </si>
   <si>
     <t>Emergência transformada em ANCE em 24/08. Aguardaremos atendimento com item da Vee One. Ramon 24/08/26.</t>
@@ -259,7 +256,7 @@
     <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
   </si>
   <si>
-    <t>Colocado pedido no fornecedor WAGA INTERNATIONAL INV26-00008 - tracking 876324334524 - aguardando voo cargueiro para o GIG</t>
+    <t>Colocado pedido no fornecedor WAGA INTERNATIONAL INV26-00008 - tracking 876324334524 - previsão de chegada GIG 10/09</t>
   </si>
   <si>
     <t>Colocado pedido Textron WB0003128625 - tracking 535477333011 - previsão de entrega 25/08 V1 JPA - MATERIAL ENVIADO VIA RECIBO 726/FAB/26, AWB A SER GERADA PELA GOLLOG RC 25/08/2026 - AWB 12754866615 DPE 28/08/2026 - recebido dia 31/08/2026</t>
@@ -271,7 +268,7 @@
     <t>Enviado para o Operador dia 03/09/26 - AWB 127-5593 2321- REZ</t>
   </si>
   <si>
-    <t>Colocado pedido IJ17699595 - previsão de chegada GIG 04/09</t>
+    <t>Colocado pedido IJ17699595 - previsão de chegada GIG 04/09. Em desembaraço 08/09</t>
   </si>
   <si>
     <t>Enviado para o Operador dia 03/09/26 - AWB 127-5594 5035- REZ</t>
@@ -725,7 +722,7 @@
         <v>65</v>
       </c>
       <c r="I2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J2" s="1">
         <v>46212</v>
@@ -737,7 +734,7 @@
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N2" s="1">
         <v>46243</v>
@@ -746,25 +743,25 @@
         <v>46263</v>
       </c>
       <c r="Q2">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R2">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="S2" t="s">
+        <v>71</v>
+      </c>
+      <c r="T2" t="s">
         <v>72</v>
       </c>
-      <c r="T2" t="s">
+      <c r="U2" t="s">
         <v>73</v>
       </c>
-      <c r="U2" t="s">
-        <v>74</v>
-      </c>
       <c r="V2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="W2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -796,7 +793,7 @@
         <v>65</v>
       </c>
       <c r="I3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J3" s="1">
         <v>46238</v>
@@ -808,7 +805,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N3" s="1">
         <v>46269</v>
@@ -817,22 +814,22 @@
         <v>46269</v>
       </c>
       <c r="Q3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R3">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="S3" t="s">
+        <v>71</v>
+      </c>
+      <c r="T3" t="s">
         <v>72</v>
       </c>
-      <c r="T3" t="s">
-        <v>73</v>
-      </c>
       <c r="V3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="W3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -864,7 +861,7 @@
         <v>65</v>
       </c>
       <c r="I4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J4" s="1">
         <v>46251</v>
@@ -876,7 +873,7 @@
         <v>2</v>
       </c>
       <c r="M4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N4" s="1">
         <v>46280</v>
@@ -885,22 +882,22 @@
         <v>46280</v>
       </c>
       <c r="Q4">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R4">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="S4" t="s">
+        <v>71</v>
+      </c>
+      <c r="T4" t="s">
         <v>72</v>
       </c>
-      <c r="T4" t="s">
-        <v>73</v>
-      </c>
       <c r="V4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="W4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -932,7 +929,7 @@
         <v>65</v>
       </c>
       <c r="I5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J5" s="1">
         <v>46253</v>
@@ -944,25 +941,25 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N5" s="1">
         <v>46283</v>
       </c>
       <c r="Q5">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="R5">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S5" t="s">
+        <v>71</v>
+      </c>
+      <c r="T5" t="s">
         <v>72</v>
       </c>
-      <c r="T5" t="s">
-        <v>73</v>
-      </c>
       <c r="W5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -994,7 +991,7 @@
         <v>65</v>
       </c>
       <c r="I6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J6" s="1">
         <v>46252</v>
@@ -1006,7 +1003,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N6" s="1">
         <v>46284</v>
@@ -1015,25 +1012,25 @@
         <v>46265</v>
       </c>
       <c r="Q6">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R6">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="S6" t="s">
+        <v>71</v>
+      </c>
+      <c r="T6" t="s">
         <v>72</v>
       </c>
-      <c r="T6" t="s">
-        <v>73</v>
-      </c>
       <c r="U6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="V6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="W6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1065,7 +1062,7 @@
         <v>65</v>
       </c>
       <c r="I7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J7" s="1">
         <v>46254</v>
@@ -1077,7 +1074,7 @@
         <v>2</v>
       </c>
       <c r="M7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N7" s="1">
         <v>46286</v>
@@ -1086,25 +1083,25 @@
         <v>46258</v>
       </c>
       <c r="Q7">
-        <v>-13</v>
+        <v>-12</v>
       </c>
       <c r="R7">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="S7" t="s">
+        <v>71</v>
+      </c>
+      <c r="T7" t="s">
         <v>72</v>
       </c>
-      <c r="T7" t="s">
-        <v>73</v>
-      </c>
       <c r="U7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="V7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="W7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1136,7 +1133,7 @@
         <v>65</v>
       </c>
       <c r="I8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J8" s="1">
         <v>46262</v>
@@ -1148,7 +1145,7 @@
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N8" s="1">
         <v>46269</v>
@@ -1157,22 +1154,22 @@
         <v>46269</v>
       </c>
       <c r="Q8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R8">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="S8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="T8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="V8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="W8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1204,7 +1201,7 @@
         <v>65</v>
       </c>
       <c r="I9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J9" s="1">
         <v>46262</v>
@@ -1216,7 +1213,7 @@
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N9" s="1">
         <v>46293</v>
@@ -1225,22 +1222,22 @@
         <v>46293</v>
       </c>
       <c r="Q9">
-        <v>-20</v>
+        <v>-19</v>
       </c>
       <c r="R9">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="S9" t="s">
+        <v>71</v>
+      </c>
+      <c r="T9" t="s">
         <v>72</v>
       </c>
-      <c r="T9" t="s">
-        <v>73</v>
-      </c>
       <c r="V9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="W9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1272,7 +1269,7 @@
         <v>66</v>
       </c>
       <c r="I10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J10" s="1">
         <v>46265</v>
@@ -1284,7 +1281,7 @@
         <v>5</v>
       </c>
       <c r="M10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N10" s="1">
         <v>46297</v>
@@ -1293,25 +1290,25 @@
         <v>46297</v>
       </c>
       <c r="Q10">
-        <v>-24</v>
+        <v>-23</v>
       </c>
       <c r="R10">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="T10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="U10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="V10" t="s">
+        <v>85</v>
+      </c>
+      <c r="W10" t="s">
         <v>86</v>
-      </c>
-      <c r="W10" t="s">
-        <v>87</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1340,10 +1337,10 @@
         <v>2730</v>
       </c>
       <c r="H11" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="I11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J11" s="1">
         <v>46269</v>
@@ -1355,28 +1352,28 @@
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N11" s="1">
         <v>46284</v>
       </c>
       <c r="Q11">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="T11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="U11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="W11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (10/09/2026 11:57)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="85">
   <si>
     <t>om_emg</t>
   </si>
@@ -97,9 +97,6 @@
     <t>em_aberto</t>
   </si>
   <si>
-    <t>BANT</t>
-  </si>
-  <si>
     <t>BABE</t>
   </si>
   <si>
@@ -112,9 +109,6 @@
     <t>BACG</t>
   </si>
   <si>
-    <t>685260012350</t>
-  </si>
-  <si>
     <t>396260016580</t>
   </si>
   <si>
@@ -124,9 +118,6 @@
     <t>313260018708</t>
   </si>
   <si>
-    <t>396260016588</t>
-  </si>
-  <si>
     <t>313260018713</t>
   </si>
   <si>
@@ -142,7 +133,10 @@
     <t>313260018737</t>
   </si>
   <si>
-    <t>030-1094-58</t>
+    <t>690260002566</t>
+  </si>
+  <si>
+    <t>329260019291</t>
   </si>
   <si>
     <t>2601188-204</t>
@@ -154,9 +148,6 @@
     <t>2698010-7</t>
   </si>
   <si>
-    <t>0750220-1</t>
-  </si>
-  <si>
     <t>2115040-8</t>
   </si>
   <si>
@@ -172,7 +163,10 @@
     <t>D210507</t>
   </si>
   <si>
-    <t>CONNECTOR</t>
+    <t>HM-6C</t>
+  </si>
+  <si>
+    <t>3244897-4</t>
   </si>
   <si>
     <t>COMPRESSOR DRIVE ASS</t>
@@ -184,9 +178,6 @@
     <t>PASSENGER DOOR - LOW</t>
   </si>
   <si>
-    <t>BOLT,MACHINE</t>
-  </si>
-  <si>
     <t>CYLINDER GAS S</t>
   </si>
   <si>
@@ -202,6 +193,12 @@
     <t>GOVERNOR,OVERSPEED</t>
   </si>
   <si>
+    <t>BEARING,PLAIN,ROD EN</t>
+  </si>
+  <si>
+    <t>FUEL CONTROL UNIT</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -217,6 +214,9 @@
     <t>Expedido total</t>
   </si>
   <si>
+    <t>Aguardando solução</t>
+  </si>
+  <si>
     <t>ANCE</t>
   </si>
   <si>
@@ -235,12 +235,6 @@
     <t>Sim</t>
   </si>
   <si>
-    <t>AWB 12754830370 -  volume retirado na loja GOLLOG - NAT por Teodoro silva em 29/08. Godoy 01/09/26. V1 favor inserir o recibo na pasta do Drive. Godoy 09/09/26.</t>
-  </si>
-  <si>
-    <t>AWB 12754866615 -  volume retirado na loja GOLLOG - BEL por Marcos bispo em 31/08. Godoy 01/09/26.   V1 favor inserir o recibo na pasta do Drive. Godoy 09/09/26.</t>
-  </si>
-  <si>
     <t>Emergência transformada em ANCE em 24/08. Aguardaremos atendimento com item da Vee One. Ramon 24/08/26.</t>
   </si>
   <si>
@@ -250,7 +244,7 @@
     <t>ITEM FOI REMOVIDO PARA ATENDER A ANV 2736 POR MOTIVO DE PANE. Godoy 08/09/26.</t>
   </si>
   <si>
-    <t>Colocado pedido junto ao fornecedor LEGACY PARTS - tracking 1ZY85G530324002115 - entregue em Miami 11/08. Chegada GIG dia 15-08 (voo 4273). Entregue V1 JPA 17/08 - MATERIAL EM TRANSITO - RECIBO 722/FAB/26 awb 12754830370 DPE 28/08/2026 - entregue 29/08/2026</t>
+    <t>Pedido será atendido pelo estoque FAB pedido n° 18398885 - Godoy 02/09/2026.</t>
   </si>
   <si>
     <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
@@ -259,9 +253,6 @@
     <t>Colocado pedido no fornecedor WAGA INTERNATIONAL INV26-00008 - tracking 876324334524 - previsão de chegada GIG 10/09</t>
   </si>
   <si>
-    <t>Colocado pedido Textron WB0003128625 - tracking 535477333011 - previsão de entrega 25/08 V1 JPA - MATERIAL ENVIADO VIA RECIBO 726/FAB/26, AWB A SER GERADA PELA GOLLOG RC 25/08/2026 - AWB 12754866615 DPE 28/08/2026 - recebido dia 31/08/2026</t>
-  </si>
-  <si>
     <t>Colocado pedido no fornecedor I823285 - entregue em Miami 21/08 - TEMOS 3 EA NO ESTOQUE DA BANT. Material seguiu via awb 12754249845. Recebido por Kleyton em 24/08. Atl Ges.</t>
   </si>
   <si>
@@ -272,6 +263,9 @@
   </si>
   <si>
     <t>Enviado para o Operador dia 03/09/26 - AWB 127-5594 5035- REZ</t>
+  </si>
+  <si>
+    <t>MATERIAL ENVIADO VIA RECIBO 764/FAB/26 AWB 12756368406 DPE 12/09/2026</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -698,37 +692,37 @@
     </row>
     <row r="2" spans="1:27">
       <c r="A2">
-        <v>685</v>
+        <v>396</v>
       </c>
       <c r="B2" t="s">
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G2">
-        <v>2702</v>
+        <v>2733</v>
       </c>
       <c r="H2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I2" t="s">
         <v>67</v>
       </c>
       <c r="J2" s="1">
-        <v>46212</v>
+        <v>46238</v>
       </c>
       <c r="K2" s="1">
-        <v>46212</v>
+        <v>46238</v>
       </c>
       <c r="L2">
         <v>1</v>
@@ -737,16 +731,16 @@
         <v>70</v>
       </c>
       <c r="N2" s="1">
-        <v>46243</v>
+        <v>46269</v>
       </c>
       <c r="O2" s="1">
-        <v>46263</v>
+        <v>46269</v>
       </c>
       <c r="Q2">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="R2">
-        <v>62</v>
+        <v>37</v>
       </c>
       <c r="S2" t="s">
         <v>71</v>
@@ -754,14 +748,11 @@
       <c r="T2" t="s">
         <v>72</v>
       </c>
-      <c r="U2" t="s">
-        <v>73</v>
-      </c>
       <c r="V2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="W2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -769,55 +760,55 @@
     </row>
     <row r="3" spans="1:27">
       <c r="A3">
-        <v>396</v>
+        <v>313</v>
       </c>
       <c r="B3" t="s">
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G3">
-        <v>2733</v>
+        <v>2741</v>
       </c>
       <c r="H3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I3" t="s">
         <v>67</v>
       </c>
       <c r="J3" s="1">
-        <v>46238</v>
+        <v>46251</v>
       </c>
       <c r="K3" s="1">
-        <v>46238</v>
+        <v>46249</v>
       </c>
       <c r="L3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M3" t="s">
         <v>70</v>
       </c>
       <c r="N3" s="1">
-        <v>46269</v>
+        <v>46280</v>
       </c>
       <c r="O3" s="1">
-        <v>46269</v>
+        <v>46280</v>
       </c>
       <c r="Q3">
-        <v>5</v>
+        <v>-5</v>
       </c>
       <c r="R3">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="S3" t="s">
         <v>71</v>
@@ -826,10 +817,10 @@
         <v>72</v>
       </c>
       <c r="V3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="W3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -840,16 +831,16 @@
         <v>313</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F4" t="s">
         <v>62</v>
@@ -858,34 +849,31 @@
         <v>2741</v>
       </c>
       <c r="H4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I4" t="s">
         <v>67</v>
       </c>
       <c r="J4" s="1">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="K4" s="1">
-        <v>46249</v>
+        <v>46252</v>
       </c>
       <c r="L4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M4" t="s">
         <v>70</v>
       </c>
       <c r="N4" s="1">
-        <v>46280</v>
-      </c>
-      <c r="O4" s="1">
-        <v>46280</v>
+        <v>46283</v>
       </c>
       <c r="Q4">
-        <v>-6</v>
+        <v>-8</v>
       </c>
       <c r="R4">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S4" t="s">
         <v>71</v>
@@ -893,11 +881,8 @@
       <c r="T4" t="s">
         <v>72</v>
       </c>
-      <c r="V4" t="s">
-        <v>80</v>
-      </c>
       <c r="W4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -908,49 +893,52 @@
         <v>313</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G5">
-        <v>2741</v>
+        <v>2737</v>
       </c>
       <c r="H5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I5" t="s">
         <v>67</v>
       </c>
       <c r="J5" s="1">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="K5" s="1">
-        <v>46252</v>
+        <v>46255</v>
       </c>
       <c r="L5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M5" t="s">
         <v>70</v>
       </c>
       <c r="N5" s="1">
-        <v>46283</v>
+        <v>46286</v>
+      </c>
+      <c r="O5" s="1">
+        <v>46258</v>
       </c>
       <c r="Q5">
-        <v>-9</v>
+        <v>-11</v>
       </c>
       <c r="R5">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="S5" t="s">
         <v>71</v>
@@ -958,8 +946,14 @@
       <c r="T5" t="s">
         <v>72</v>
       </c>
+      <c r="U5" t="s">
+        <v>73</v>
+      </c>
+      <c r="V5" t="s">
+        <v>79</v>
+      </c>
       <c r="W5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -967,37 +961,37 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6">
-        <v>396</v>
+        <v>329</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F6" t="s">
         <v>62</v>
       </c>
       <c r="G6">
-        <v>2731</v>
+        <v>2721</v>
       </c>
       <c r="H6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="J6" s="1">
-        <v>46252</v>
+        <v>46262</v>
       </c>
       <c r="K6" s="1">
-        <v>46253</v>
+        <v>46262</v>
       </c>
       <c r="L6">
         <v>1</v>
@@ -1006,31 +1000,28 @@
         <v>70</v>
       </c>
       <c r="N6" s="1">
-        <v>46284</v>
+        <v>46269</v>
       </c>
       <c r="O6" s="1">
-        <v>46265</v>
+        <v>46269</v>
       </c>
       <c r="Q6">
-        <v>-10</v>
+        <v>6</v>
       </c>
       <c r="R6">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="S6" t="s">
         <v>71</v>
       </c>
       <c r="T6" t="s">
-        <v>72</v>
-      </c>
-      <c r="U6" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="V6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="W6" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1038,55 +1029,55 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>313</v>
+        <v>396</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G7">
-        <v>2737</v>
+        <v>2733</v>
       </c>
       <c r="H7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I7" t="s">
         <v>67</v>
       </c>
       <c r="J7" s="1">
-        <v>46254</v>
+        <v>46262</v>
       </c>
       <c r="K7" s="1">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="L7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M7" t="s">
         <v>70</v>
       </c>
       <c r="N7" s="1">
-        <v>46286</v>
+        <v>46293</v>
       </c>
       <c r="O7" s="1">
-        <v>46258</v>
+        <v>46293</v>
       </c>
       <c r="Q7">
-        <v>-12</v>
+        <v>-18</v>
       </c>
       <c r="R7">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="S7" t="s">
         <v>71</v>
@@ -1094,14 +1085,11 @@
       <c r="T7" t="s">
         <v>72</v>
       </c>
-      <c r="U7" t="s">
-        <v>75</v>
-      </c>
       <c r="V7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="W7" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1109,67 +1097,70 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>329</v>
+        <v>690</v>
       </c>
       <c r="B8" t="s">
         <v>30</v>
       </c>
       <c r="C8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G8">
-        <v>2721</v>
+        <v>2727</v>
       </c>
       <c r="H8" t="s">
         <v>65</v>
       </c>
       <c r="I8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J8" s="1">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="K8" s="1">
-        <v>46262</v>
+        <v>46266</v>
       </c>
       <c r="L8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M8" t="s">
         <v>70</v>
       </c>
       <c r="N8" s="1">
-        <v>46269</v>
+        <v>46297</v>
       </c>
       <c r="O8" s="1">
-        <v>46269</v>
+        <v>46297</v>
       </c>
       <c r="Q8">
-        <v>5</v>
+        <v>-22</v>
       </c>
       <c r="R8">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="S8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="T8" t="s">
         <v>71</v>
       </c>
+      <c r="U8" t="s">
+        <v>74</v>
+      </c>
       <c r="V8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="W8" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1177,37 +1168,37 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9">
-        <v>396</v>
+        <v>313</v>
       </c>
       <c r="B9" t="s">
         <v>28</v>
       </c>
       <c r="C9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G9">
-        <v>2733</v>
+        <v>2730</v>
       </c>
       <c r="H9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I9" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J9" s="1">
-        <v>46262</v>
+        <v>46269</v>
       </c>
       <c r="K9" s="1">
-        <v>46262</v>
+        <v>46273</v>
       </c>
       <c r="L9">
         <v>1</v>
@@ -1216,28 +1207,31 @@
         <v>70</v>
       </c>
       <c r="N9" s="1">
-        <v>46293</v>
+        <v>46284</v>
       </c>
       <c r="O9" s="1">
-        <v>46293</v>
+        <v>46277</v>
       </c>
       <c r="Q9">
-        <v>-19</v>
+        <v>-9</v>
       </c>
       <c r="R9">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="S9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="T9" t="s">
         <v>72</v>
       </c>
+      <c r="U9" t="s">
+        <v>75</v>
+      </c>
       <c r="V9" t="s">
+        <v>83</v>
+      </c>
+      <c r="W9" t="s">
         <v>84</v>
-      </c>
-      <c r="W9" t="s">
-        <v>86</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1248,52 +1242,49 @@
         <v>690</v>
       </c>
       <c r="B10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G10">
         <v>2727</v>
       </c>
       <c r="H10" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="J10" s="1">
-        <v>46265</v>
+        <v>46274</v>
       </c>
       <c r="K10" s="1">
-        <v>46266</v>
+        <v>46275</v>
       </c>
       <c r="L10">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M10" t="s">
         <v>70</v>
       </c>
       <c r="N10" s="1">
-        <v>46297</v>
-      </c>
-      <c r="O10" s="1">
-        <v>46297</v>
+        <v>46282</v>
       </c>
       <c r="Q10">
-        <v>-23</v>
+        <v>-7</v>
       </c>
       <c r="R10">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S10" t="s">
         <v>72</v>
@@ -1304,11 +1295,8 @@
       <c r="U10" t="s">
         <v>76</v>
       </c>
-      <c r="V10" t="s">
-        <v>85</v>
-      </c>
       <c r="W10" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1316,37 +1304,37 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B11" t="s">
         <v>29</v>
       </c>
       <c r="C11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G11">
-        <v>2730</v>
+        <v>2709</v>
       </c>
       <c r="H11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J11" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K11" s="1">
-        <v>46273</v>
+        <v>46275</v>
       </c>
       <c r="L11">
         <v>1</v>
@@ -1355,25 +1343,22 @@
         <v>70</v>
       </c>
       <c r="N11" s="1">
-        <v>46284</v>
+        <v>46282</v>
       </c>
       <c r="Q11">
-        <v>-10</v>
+        <v>-7</v>
       </c>
       <c r="R11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="T11" t="s">
-        <v>72</v>
-      </c>
-      <c r="U11" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="W11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (11/09/2026 11:58)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="101">
   <si>
     <t>om_emg</t>
   </si>
@@ -109,6 +109,9 @@
     <t>BACG</t>
   </si>
   <si>
+    <t>BANT</t>
+  </si>
+  <si>
     <t>396260016580</t>
   </si>
   <si>
@@ -139,6 +142,15 @@
     <t>329260019291</t>
   </si>
   <si>
+    <t>685260012774</t>
+  </si>
+  <si>
+    <t>685260012773</t>
+  </si>
+  <si>
+    <t>685260012775</t>
+  </si>
+  <si>
     <t>2601188-204</t>
   </si>
   <si>
@@ -169,6 +181,15 @@
     <t>3244897-4</t>
   </si>
   <si>
+    <t>S3465-2-0132</t>
+  </si>
+  <si>
+    <t>S3465-2-0146</t>
+  </si>
+  <si>
+    <t>060-0017-00</t>
+  </si>
+  <si>
     <t>COMPRESSOR DRIVE ASS</t>
   </si>
   <si>
@@ -199,6 +220,15 @@
     <t>FUEL CONTROL UNIT</t>
   </si>
   <si>
+    <t>HOSE ASSY BRAKE CYL</t>
+  </si>
+  <si>
+    <t>HOSE ASSY BRAK</t>
+  </si>
+  <si>
+    <t>FLIGHT DIR HOR</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -238,6 +268,9 @@
     <t>Emergência transformada em ANCE em 24/08. Aguardaremos atendimento com item da Vee One. Ramon 24/08/26.</t>
   </si>
   <si>
+    <t>AWB 127-5593 2321 -  volume retirado na loja GOLLOG - BSB por mateus em 10/09 - Godoy 10/09/2026.</t>
+  </si>
+  <si>
     <t>Pedido será atendido pelo estoque FAB pedido n° 18353156- Godoy 02/09/2026.</t>
   </si>
   <si>
@@ -247,10 +280,13 @@
     <t>Pedido será atendido pelo estoque FAB pedido n° 18398885 - Godoy 02/09/2026.</t>
   </si>
   <si>
+    <t>AWB 12756560825 - volume retirado na loja GOLLOG - BSB por Mateus Oliveira em 10/09. Godoy 10/09/26.</t>
+  </si>
+  <si>
     <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
   </si>
   <si>
-    <t>Colocado pedido no fornecedor WAGA INTERNATIONAL INV26-00008 - tracking 876324334524 - previsão de chegada GIG 10/09</t>
+    <t>Colocado pedido no fornecedor WAGA INTERNATIONAL INV26-00008 - tracking 876324334524 - previsão de chegada GIG 16/09</t>
   </si>
   <si>
     <t>Colocado pedido no fornecedor I823285 - entregue em Miami 21/08 - TEMOS 3 EA NO ESTOQUE DA BANT. Material seguiu via awb 12754249845. Recebido por Kleyton em 24/08. Atl Ges.</t>
@@ -259,13 +295,25 @@
     <t>Enviado para o Operador dia 03/09/26 - AWB 127-5593 2321- REZ</t>
   </si>
   <si>
-    <t>Colocado pedido IJ17699595 - previsão de chegada GIG 04/09. Em desembaraço 08/09</t>
-  </si>
-  <si>
-    <t>Enviado para o Operador dia 03/09/26 - AWB 127-5594 5035- REZ</t>
+    <t>Colocado pedido IJ17699595 - entregue V1 JPA 09/09. Em processo de envio para a base FAB.</t>
+  </si>
+  <si>
+    <t>Enviado para o Operador dia 03/09/26 - AWB 127-5594 5035- REZ - Material disponivel para coleta, em contato com a transportadora rc 10/09/2026</t>
   </si>
   <si>
     <t>MATERIAL ENVIADO VIA RECIBO 764/FAB/26 AWB 12756368406 DPE 12/09/2026</t>
+  </si>
+  <si>
+    <t>Será atendido via estoque FAB.</t>
+  </si>
+  <si>
+    <t>MATERIAL ENVIADO VIA RECIBO 769/FAB/26 AWB 12756560825 dpe 10/09/2026 - MATERIAL DISPONIVEL PARA RETIRADA DIA 10/09/2026 11:58 RC 10/09/2026</t>
+  </si>
+  <si>
+    <t>Colocado pedido WB0003149512 - envio direto para o Brasil</t>
+  </si>
+  <si>
+    <t>SERÁ ENVIADO DA BASE PAMALS</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -604,7 +652,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA11"/>
+  <dimension ref="A1:AA14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -698,25 +746,25 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E2" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="F2" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="G2">
         <v>2733</v>
       </c>
       <c r="H2" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="I2" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="J2" s="1">
         <v>46238</v>
@@ -728,7 +776,7 @@
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="N2" s="1">
         <v>46269</v>
@@ -737,22 +785,22 @@
         <v>46269</v>
       </c>
       <c r="Q2">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R2">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="S2" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="T2" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="V2" t="s">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="W2" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -766,25 +814,25 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E3" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="F3" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="G3">
         <v>2741</v>
       </c>
       <c r="H3" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="I3" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="J3" s="1">
         <v>46251</v>
@@ -796,7 +844,7 @@
         <v>2</v>
       </c>
       <c r="M3" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="N3" s="1">
         <v>46280</v>
@@ -805,22 +853,22 @@
         <v>46280</v>
       </c>
       <c r="Q3">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R3">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S3" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="T3" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="V3" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="W3" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -834,25 +882,25 @@
         <v>28</v>
       </c>
       <c r="C4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E4" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="F4" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="G4">
         <v>2741</v>
       </c>
       <c r="H4" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="I4" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="J4" s="1">
         <v>46253</v>
@@ -864,25 +912,25 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="N4" s="1">
         <v>46283</v>
       </c>
       <c r="Q4">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="R4">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="S4" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="T4" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="W4" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -896,25 +944,25 @@
         <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E5" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="F5" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="G5">
         <v>2737</v>
       </c>
       <c r="H5" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="I5" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="J5" s="1">
         <v>46254</v>
@@ -926,7 +974,7 @@
         <v>2</v>
       </c>
       <c r="M5" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="N5" s="1">
         <v>46286</v>
@@ -935,25 +983,25 @@
         <v>46258</v>
       </c>
       <c r="Q5">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R5">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="S5" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="T5" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="U5" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="V5" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="W5" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -967,25 +1015,25 @@
         <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E6" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="F6" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="G6">
         <v>2721</v>
       </c>
       <c r="H6" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="I6" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="J6" s="1">
         <v>46262</v>
@@ -997,7 +1045,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="N6" s="1">
         <v>46269</v>
@@ -1006,22 +1054,25 @@
         <v>46269</v>
       </c>
       <c r="Q6">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R6">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S6" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="T6" t="s">
-        <v>71</v>
+        <v>81</v>
+      </c>
+      <c r="U6" t="s">
+        <v>84</v>
       </c>
       <c r="V6" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="W6" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1035,25 +1086,25 @@
         <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E7" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="F7" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="G7">
         <v>2733</v>
       </c>
       <c r="H7" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="I7" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="J7" s="1">
         <v>46262</v>
@@ -1065,7 +1116,7 @@
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="N7" s="1">
         <v>46293</v>
@@ -1074,22 +1125,22 @@
         <v>46293</v>
       </c>
       <c r="Q7">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="R7">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S7" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="T7" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="V7" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="W7" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1103,25 +1154,25 @@
         <v>30</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E8" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="F8" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="G8">
         <v>2727</v>
       </c>
       <c r="H8" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="I8" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="J8" s="1">
         <v>46265</v>
@@ -1133,7 +1184,7 @@
         <v>5</v>
       </c>
       <c r="M8" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="N8" s="1">
         <v>46297</v>
@@ -1142,25 +1193,25 @@
         <v>46297</v>
       </c>
       <c r="Q8">
-        <v>-22</v>
+        <v>-21</v>
       </c>
       <c r="R8">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="S8" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="T8" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="U8" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="V8" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="W8" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1174,25 +1225,25 @@
         <v>28</v>
       </c>
       <c r="C9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D9" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E9" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="F9" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="G9">
         <v>2730</v>
       </c>
       <c r="H9" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="I9" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="J9" s="1">
         <v>46269</v>
@@ -1204,7 +1255,7 @@
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="N9" s="1">
         <v>46284</v>
@@ -1213,25 +1264,25 @@
         <v>46277</v>
       </c>
       <c r="Q9">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="R9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S9" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="T9" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="U9" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="V9" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="W9" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1245,25 +1296,25 @@
         <v>30</v>
       </c>
       <c r="C10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D10" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="E10" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="F10" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="G10">
         <v>2727</v>
       </c>
       <c r="H10" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="I10" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="J10" s="1">
         <v>46274</v>
@@ -1275,28 +1326,31 @@
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="N10" s="1">
         <v>46282</v>
       </c>
       <c r="Q10">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S10" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="T10" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="U10" t="s">
-        <v>76</v>
+        <v>87</v>
+      </c>
+      <c r="V10" t="s">
+        <v>96</v>
       </c>
       <c r="W10" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1310,25 +1364,25 @@
         <v>29</v>
       </c>
       <c r="C11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D11" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E11" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="F11" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="G11">
         <v>2709</v>
       </c>
       <c r="H11" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="I11" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="J11" s="1">
         <v>46274</v>
@@ -1340,27 +1394,237 @@
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="N11" s="1">
         <v>46282</v>
       </c>
+      <c r="O11" s="1">
+        <v>46275</v>
+      </c>
       <c r="Q11">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S11" t="s">
+        <v>81</v>
+      </c>
+      <c r="T11" t="s">
+        <v>81</v>
+      </c>
+      <c r="U11" t="s">
+        <v>88</v>
+      </c>
+      <c r="V11" t="s">
+        <v>97</v>
+      </c>
+      <c r="W11" t="s">
+        <v>100</v>
+      </c>
+      <c r="AA11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27">
+      <c r="A12">
+        <v>685</v>
+      </c>
+      <c r="B12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" t="s">
+        <v>55</v>
+      </c>
+      <c r="E12" t="s">
+        <v>68</v>
+      </c>
+      <c r="F12" t="s">
         <v>71</v>
       </c>
-      <c r="T11" t="s">
+      <c r="G12">
+        <v>2702</v>
+      </c>
+      <c r="H12" t="s">
+        <v>76</v>
+      </c>
+      <c r="I12" t="s">
+        <v>78</v>
+      </c>
+      <c r="J12" s="1">
+        <v>46275</v>
+      </c>
+      <c r="K12" s="1">
+        <v>46305</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12" t="s">
+        <v>80</v>
+      </c>
+      <c r="N12" s="1">
+        <v>46312</v>
+      </c>
+      <c r="O12" s="1">
+        <v>46282</v>
+      </c>
+      <c r="Q12">
+        <v>-36</v>
+      </c>
+      <c r="R12">
+        <v>-29</v>
+      </c>
+      <c r="S12" t="s">
+        <v>81</v>
+      </c>
+      <c r="T12" t="s">
+        <v>82</v>
+      </c>
+      <c r="V12" t="s">
+        <v>98</v>
+      </c>
+      <c r="W12" t="s">
+        <v>100</v>
+      </c>
+      <c r="AA12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27">
+      <c r="A13">
+        <v>685</v>
+      </c>
+      <c r="B13" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" t="s">
+        <v>56</v>
+      </c>
+      <c r="E13" t="s">
+        <v>69</v>
+      </c>
+      <c r="F13" t="s">
         <v>71</v>
       </c>
-      <c r="W11" t="s">
-        <v>84</v>
-      </c>
-      <c r="AA11" t="b">
+      <c r="G13">
+        <v>2702</v>
+      </c>
+      <c r="H13" t="s">
+        <v>76</v>
+      </c>
+      <c r="I13" t="s">
+        <v>78</v>
+      </c>
+      <c r="J13" s="1">
+        <v>46275</v>
+      </c>
+      <c r="K13" s="1">
+        <v>46305</v>
+      </c>
+      <c r="L13">
+        <v>1</v>
+      </c>
+      <c r="M13" t="s">
+        <v>80</v>
+      </c>
+      <c r="N13" s="1">
+        <v>46312</v>
+      </c>
+      <c r="O13" s="1">
+        <v>46282</v>
+      </c>
+      <c r="Q13">
+        <v>-36</v>
+      </c>
+      <c r="R13">
+        <v>-29</v>
+      </c>
+      <c r="S13" t="s">
+        <v>81</v>
+      </c>
+      <c r="T13" t="s">
+        <v>82</v>
+      </c>
+      <c r="V13" t="s">
+        <v>98</v>
+      </c>
+      <c r="W13" t="s">
+        <v>100</v>
+      </c>
+      <c r="AA13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:27">
+      <c r="A14">
+        <v>685</v>
+      </c>
+      <c r="B14" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" t="s">
+        <v>44</v>
+      </c>
+      <c r="D14" t="s">
+        <v>57</v>
+      </c>
+      <c r="E14" t="s">
+        <v>70</v>
+      </c>
+      <c r="F14" t="s">
+        <v>73</v>
+      </c>
+      <c r="G14">
+        <v>2729</v>
+      </c>
+      <c r="H14" t="s">
+        <v>76</v>
+      </c>
+      <c r="I14" t="s">
+        <v>79</v>
+      </c>
+      <c r="J14" s="1">
+        <v>46275</v>
+      </c>
+      <c r="K14" s="1">
+        <v>46305</v>
+      </c>
+      <c r="L14">
+        <v>1</v>
+      </c>
+      <c r="M14" t="s">
+        <v>80</v>
+      </c>
+      <c r="N14" s="1">
+        <v>46316</v>
+      </c>
+      <c r="Q14">
+        <v>-40</v>
+      </c>
+      <c r="R14">
+        <v>-29</v>
+      </c>
+      <c r="S14" t="s">
+        <v>81</v>
+      </c>
+      <c r="T14" t="s">
+        <v>82</v>
+      </c>
+      <c r="V14" t="s">
+        <v>99</v>
+      </c>
+      <c r="W14" t="s">
+        <v>100</v>
+      </c>
+      <c r="AA14" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>